<commit_message>
데이터 갱신: holdings,kr_etf (2026-10-12)
</commit_message>
<xml_diff>
--- a/downloads/schd_dividend_tracker.xlsx
+++ b/downloads/schd_dividend_tracker.xlsx
@@ -1265,22 +1265,22 @@
   <commentList>
     <comment ref="C6" authorId="0" shapeId="0">
       <text>
-        <t>총보수 0.01% + 기타비용 0.05% + 매매·중개수수료 0.0434% (KOFIA 2026-08-31)</t>
+        <t>총보수 0.01% + 기타비용 0.05% + 매매·중개수수료 0.0464% (KOFIA 2026-09-30)</t>
       </text>
     </comment>
     <comment ref="C7" authorId="0" shapeId="0">
       <text>
-        <t>총보수 0.01% + 기타비용 0.06% + 매매·중개수수료 0.0998% (KOFIA 2026-08-31)</t>
+        <t>총보수 0.01% + 기타비용 0.06% + 매매·중개수수료 0.1011% (KOFIA 2026-09-30)</t>
       </text>
     </comment>
     <comment ref="C8" authorId="0" shapeId="0">
       <text>
-        <t>총보수 0.01% + 기타비용 0.06% + 매매·중개수수료 0.0781% (KOFIA 2026-08-31)</t>
+        <t>총보수 0.01% + 기타비용 0.06% + 매매·중개수수료 0.0824% (KOFIA 2026-09-30)</t>
       </text>
     </comment>
     <comment ref="C9" authorId="0" shapeId="0">
       <text>
-        <t>총보수 0.0099% + 기타비용 0.08% + 매매·중개수수료 0.0934% (KOFIA 2026-08-31)</t>
+        <t>총보수 0.0099% + 기타비용 0.07% + 매매·중개수수료 0.0959% (KOFIA 2026-09-30)</t>
       </text>
     </comment>
   </commentList>
@@ -1724,7 +1724,7 @@
     <row r="3">
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>최종 갱신: 2026-10-10 · 반영 범위: 2012년 1분기 ~ 2026년 3분기 (배당락 2026-09-23) · GitHub Actions 자동 생성</t>
+          <t>최종 갱신: 2026-10-12 · 반영 범위: 2012년 1분기 ~ 2026년 3분기 (배당락 2026-09-23) · GitHub Actions 자동 생성</t>
         </is>
       </c>
     </row>
@@ -24842,7 +24842,7 @@
         </is>
       </c>
       <c r="C6" s="51" t="n">
-        <v>0.001034</v>
+        <v>0.001064</v>
       </c>
       <c r="D6" s="33" t="inlineStr">
         <is>
@@ -24882,7 +24882,7 @@
         </is>
       </c>
       <c r="C7" s="51" t="n">
-        <v>0.001698</v>
+        <v>0.001711</v>
       </c>
       <c r="D7" s="33" t="inlineStr">
         <is>
@@ -24922,7 +24922,7 @@
         </is>
       </c>
       <c r="C8" s="51" t="n">
-        <v>0.001481</v>
+        <v>0.001524</v>
       </c>
       <c r="D8" s="33" t="inlineStr">
         <is>
@@ -24962,7 +24962,7 @@
         </is>
       </c>
       <c r="C9" s="51" t="n">
-        <v>0.001834</v>
+        <v>0.001759</v>
       </c>
       <c r="D9" s="33" t="inlineStr">
         <is>
@@ -25040,7 +25040,7 @@
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>※ 국내 ETF 실부담비용 = 총보수 + 기타비용 + 매매·중개수수료(+판매수수료), 금융투자협회 공시 2026-08-31 기준. 셀 메모에 항목별 금액.</t>
+          <t>※ 국내 ETF 실부담비용 = 총보수 + 기타비용 + 매매·중개수수료(+판매수수료), 금융투자협회 공시 2026-09-30 기준. 셀 메모에 항목별 금액.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
데이터 갱신: holdings (2026-10-13)
</commit_message>
<xml_diff>
--- a/downloads/schd_dividend_tracker.xlsx
+++ b/downloads/schd_dividend_tracker.xlsx
@@ -1724,7 +1724,7 @@
     <row r="3">
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>최종 갱신: 2026-10-12 · 반영 범위: 2012년 1분기 ~ 2026년 3분기 (배당락 2026-09-23) · GitHub Actions 자동 생성</t>
+          <t>최종 갱신: 2026-10-13 · 반영 범위: 2012년 1분기 ~ 2026년 3분기 (배당락 2026-09-23) · GitHub Actions 자동 생성</t>
         </is>
       </c>
     </row>
@@ -26215,11 +26215,11 @@
         </is>
       </c>
       <c r="B2" s="49" t="n">
-        <v>46304</v>
+        <v>46307</v>
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>← 이 날 종가로 계산한 비중. 그날 공식 파일을 못 받아 Schwab 공식 보유종목 CSV(2026-10-08)의 보유 주식 수 × 종가로 계산했습니다.</t>
+          <t>← 이 날 종가로 계산한 비중. 그날 공식 파일을 못 받아 Schwab 공식 보유종목 CSV(2026-10-09)의 보유 주식 수 × 종가로 계산했습니다.</t>
         </is>
       </c>
     </row>
@@ -26316,7 +26316,7 @@
         </is>
       </c>
       <c r="I5" s="61" t="n">
-        <v>0.04686291</v>
+        <v>0.04621969</v>
       </c>
       <c r="J5" s="6" t="inlineStr">
         <is>
@@ -26370,25 +26370,25 @@
       </c>
       <c r="H6" s="6" t="inlineStr">
         <is>
-          <t>QCOM</t>
+          <t>PG</t>
         </is>
       </c>
       <c r="I6" s="61" t="n">
-        <v>0.04345508</v>
+        <v>0.04337427</v>
       </c>
       <c r="J6" s="6" t="inlineStr">
         <is>
-          <t>QUALCOMM</t>
+          <t>PROCTER &amp; GAMBLE</t>
         </is>
       </c>
       <c r="K6" s="6" t="inlineStr">
         <is>
-          <t>Information Technology</t>
+          <t>Consumer Staples</t>
         </is>
       </c>
       <c r="L6" s="6" t="inlineStr">
         <is>
-          <t>퀄컴</t>
+          <t>프록터앤드갬블</t>
         </is>
       </c>
       <c r="M6" s="7">
@@ -26428,25 +26428,25 @@
       </c>
       <c r="H7" s="6" t="inlineStr">
         <is>
-          <t>PG</t>
+          <t>QCOM</t>
         </is>
       </c>
       <c r="I7" s="61" t="n">
-        <v>0.04310645</v>
+        <v>0.04289955</v>
       </c>
       <c r="J7" s="6" t="inlineStr">
         <is>
-          <t>PROCTER &amp; GAMBLE</t>
+          <t>QUALCOMM</t>
         </is>
       </c>
       <c r="K7" s="6" t="inlineStr">
         <is>
-          <t>Consumer Staples</t>
+          <t>Information Technology</t>
         </is>
       </c>
       <c r="L7" s="6" t="inlineStr">
         <is>
-          <t>프록터앤드갬블</t>
+          <t>퀄컴</t>
         </is>
       </c>
       <c r="M7" s="7">
@@ -26486,25 +26486,25 @@
       </c>
       <c r="H8" s="6" t="inlineStr">
         <is>
-          <t>CVX</t>
+          <t>KO</t>
         </is>
       </c>
       <c r="I8" s="61" t="n">
-        <v>0.04212293</v>
+        <v>0.04253438</v>
       </c>
       <c r="J8" s="6" t="inlineStr">
         <is>
-          <t>CHEVRON</t>
+          <t>COCA-COLA</t>
         </is>
       </c>
       <c r="K8" s="6" t="inlineStr">
         <is>
-          <t>Energy</t>
+          <t>Consumer Staples</t>
         </is>
       </c>
       <c r="L8" s="6" t="inlineStr">
         <is>
-          <t>셰브론</t>
+          <t>코카콜라</t>
         </is>
       </c>
       <c r="M8" s="7">
@@ -26544,25 +26544,25 @@
       </c>
       <c r="H9" s="6" t="inlineStr">
         <is>
-          <t>KO</t>
+          <t>CVX</t>
         </is>
       </c>
       <c r="I9" s="61" t="n">
-        <v>0.04199263</v>
+        <v>0.04243566999999999</v>
       </c>
       <c r="J9" s="6" t="inlineStr">
         <is>
-          <t>COCA-COLA</t>
+          <t>CHEVRON</t>
         </is>
       </c>
       <c r="K9" s="6" t="inlineStr">
         <is>
-          <t>Consumer Staples</t>
+          <t>Energy</t>
         </is>
       </c>
       <c r="L9" s="6" t="inlineStr">
         <is>
-          <t>코카콜라</t>
+          <t>셰브론</t>
         </is>
       </c>
       <c r="M9" s="7">
@@ -26606,7 +26606,7 @@
         </is>
       </c>
       <c r="I10" s="61" t="n">
-        <v>0.04107964</v>
+        <v>0.04185615</v>
       </c>
       <c r="J10" s="6" t="inlineStr">
         <is>
@@ -26664,7 +26664,7 @@
         </is>
       </c>
       <c r="I11" s="61" t="n">
-        <v>0.04040699</v>
+        <v>0.04009386</v>
       </c>
       <c r="J11" s="6" t="inlineStr">
         <is>
@@ -26722,7 +26722,7 @@
         </is>
       </c>
       <c r="I12" s="61" t="n">
-        <v>0.03993899</v>
+        <v>0.03958902</v>
       </c>
       <c r="J12" s="6" t="inlineStr">
         <is>
@@ -26780,7 +26780,7 @@
         </is>
       </c>
       <c r="I13" s="61" t="n">
-        <v>0.03942468</v>
+        <v>0.03941473</v>
       </c>
       <c r="J13" s="6" t="inlineStr">
         <is>
@@ -26834,25 +26834,25 @@
       </c>
       <c r="H14" s="6" t="inlineStr">
         <is>
-          <t>HD</t>
+          <t>ABT</t>
         </is>
       </c>
       <c r="I14" s="61" t="n">
-        <v>0.03841367</v>
+        <v>0.0385271</v>
       </c>
       <c r="J14" s="6" t="inlineStr">
         <is>
-          <t>HOME DEPOT</t>
+          <t>ABBOTT LABORATORIES</t>
         </is>
       </c>
       <c r="K14" s="6" t="inlineStr">
         <is>
-          <t>Consumer Discretionary</t>
+          <t>Health Care</t>
         </is>
       </c>
       <c r="L14" s="6" t="inlineStr">
         <is>
-          <t>홈디포</t>
+          <t>애보트</t>
         </is>
       </c>
       <c r="M14" s="7">
@@ -26882,25 +26882,25 @@
       </c>
       <c r="H15" s="6" t="inlineStr">
         <is>
-          <t>ABT</t>
+          <t>HD</t>
         </is>
       </c>
       <c r="I15" s="61" t="n">
-        <v>0.03794233</v>
+        <v>0.03813983</v>
       </c>
       <c r="J15" s="6" t="inlineStr">
         <is>
-          <t>ABBOTT LABORATORIES</t>
+          <t>HOME DEPOT</t>
         </is>
       </c>
       <c r="K15" s="6" t="inlineStr">
         <is>
-          <t>Health Care</t>
+          <t>Consumer Discretionary</t>
         </is>
       </c>
       <c r="L15" s="6" t="inlineStr">
         <is>
-          <t>애보트</t>
+          <t>홈디포</t>
         </is>
       </c>
       <c r="M15" s="7">
@@ -26934,7 +26934,7 @@
         </is>
       </c>
       <c r="I16" s="61" t="n">
-        <v>0.0377258</v>
+        <v>0.03768319</v>
       </c>
       <c r="J16" s="6" t="inlineStr">
         <is>
@@ -26972,7 +26972,7 @@
         </is>
       </c>
       <c r="I17" s="61" t="n">
-        <v>0.03490183</v>
+        <v>0.03560754</v>
       </c>
       <c r="J17" s="6" t="inlineStr">
         <is>
@@ -27010,7 +27010,7 @@
         </is>
       </c>
       <c r="I18" s="61" t="n">
-        <v>0.03262227</v>
+        <v>0.03330342</v>
       </c>
       <c r="J18" s="6" t="inlineStr">
         <is>
@@ -27035,25 +27035,25 @@
     <row r="19">
       <c r="H19" s="6" t="inlineStr">
         <is>
-          <t>BMY</t>
+          <t>MO</t>
         </is>
       </c>
       <c r="I19" s="61" t="n">
-        <v>0.03079479</v>
+        <v>0.03030605</v>
       </c>
       <c r="J19" s="6" t="inlineStr">
         <is>
-          <t>BRISTOL MYERS SQUIBB</t>
+          <t>ALTRIA GROUP INC</t>
         </is>
       </c>
       <c r="K19" s="6" t="inlineStr">
         <is>
-          <t>Health Care</t>
+          <t>Consumer Staples</t>
         </is>
       </c>
       <c r="L19" s="6" t="inlineStr">
         <is>
-          <t>브리스톨마이어스스퀴브</t>
+          <t>알트리아</t>
         </is>
       </c>
       <c r="M19" s="7">
@@ -27069,25 +27069,25 @@
       </c>
       <c r="H20" s="6" t="inlineStr">
         <is>
-          <t>MO</t>
+          <t>BMY</t>
         </is>
       </c>
       <c r="I20" s="61" t="n">
-        <v>0.03051986</v>
+        <v>0.02979081</v>
       </c>
       <c r="J20" s="6" t="inlineStr">
         <is>
-          <t>ALTRIA GROUP INC</t>
+          <t>BRISTOL MYERS SQUIBB</t>
         </is>
       </c>
       <c r="K20" s="6" t="inlineStr">
         <is>
-          <t>Consumer Staples</t>
+          <t>Health Care</t>
         </is>
       </c>
       <c r="L20" s="6" t="inlineStr">
         <is>
-          <t>알트리아</t>
+          <t>브리스톨마이어스스퀴브</t>
         </is>
       </c>
       <c r="M20" s="7">
@@ -27112,7 +27112,7 @@
         </is>
       </c>
       <c r="I21" s="61" t="n">
-        <v>0.02743966</v>
+        <v>0.02755036</v>
       </c>
       <c r="J21" s="6" t="inlineStr">
         <is>
@@ -27150,7 +27150,7 @@
         </is>
       </c>
       <c r="I22" s="61" t="n">
-        <v>0.02639063</v>
+        <v>0.02633119</v>
       </c>
       <c r="J22" s="6" t="inlineStr">
         <is>
@@ -27188,7 +27188,7 @@
         </is>
       </c>
       <c r="I23" s="61" t="n">
-        <v>0.02187585</v>
+        <v>0.02182185</v>
       </c>
       <c r="J23" s="6" t="inlineStr">
         <is>
@@ -27226,7 +27226,7 @@
         </is>
       </c>
       <c r="I24" s="61" t="n">
-        <v>0.01981677</v>
+        <v>0.01999572</v>
       </c>
       <c r="J24" s="6" t="inlineStr">
         <is>
@@ -27264,7 +27264,7 @@
         </is>
       </c>
       <c r="I25" s="61" t="n">
-        <v>0.01864535</v>
+        <v>0.01853778</v>
       </c>
       <c r="J25" s="6" t="inlineStr">
         <is>
@@ -27302,7 +27302,7 @@
         </is>
       </c>
       <c r="I26" s="61" t="n">
-        <v>0.01852519</v>
+        <v>0.0183329</v>
       </c>
       <c r="J26" s="6" t="inlineStr">
         <is>
@@ -27340,7 +27340,7 @@
         </is>
       </c>
       <c r="I27" s="61" t="n">
-        <v>0.0180704</v>
+        <v>0.01809509</v>
       </c>
       <c r="J27" s="6" t="inlineStr">
         <is>
@@ -27378,7 +27378,7 @@
         </is>
       </c>
       <c r="I28" s="61" t="n">
-        <v>0.01779382</v>
+        <v>0.01767205</v>
       </c>
       <c r="J28" s="6" t="inlineStr">
         <is>
@@ -27416,7 +27416,7 @@
         </is>
       </c>
       <c r="I29" s="61" t="n">
-        <v>0.01484986</v>
+        <v>0.01496504</v>
       </c>
       <c r="J29" s="6" t="inlineStr">
         <is>
@@ -27454,7 +27454,7 @@
         </is>
       </c>
       <c r="I30" s="61" t="n">
-        <v>0.01443447</v>
+        <v>0.01469193</v>
       </c>
       <c r="J30" s="6" t="inlineStr">
         <is>
@@ -27488,7 +27488,7 @@
         </is>
       </c>
       <c r="I31" s="61" t="n">
-        <v>0.01353674</v>
+        <v>0.01364071</v>
       </c>
       <c r="J31" s="6" t="inlineStr">
         <is>
@@ -27513,7 +27513,7 @@
         </is>
       </c>
       <c r="I32" s="61" t="n">
-        <v>0.01215489</v>
+        <v>0.01190445</v>
       </c>
       <c r="J32" s="6" t="inlineStr">
         <is>
@@ -27543,7 +27543,7 @@
         </is>
       </c>
       <c r="I33" s="61" t="n">
-        <v>0.01171074</v>
+        <v>0.0116733</v>
       </c>
       <c r="J33" s="6" t="inlineStr">
         <is>
@@ -27568,7 +27568,7 @@
         </is>
       </c>
       <c r="I34" s="61" t="n">
-        <v>0.009818249999999999</v>
+        <v>0.00981695</v>
       </c>
       <c r="J34" s="6" t="inlineStr">
         <is>
@@ -27593,7 +27593,7 @@
         </is>
       </c>
       <c r="I35" s="61" t="n">
-        <v>0.00848757</v>
+        <v>0.00848407</v>
       </c>
       <c r="J35" s="6" t="inlineStr">
         <is>
@@ -27618,7 +27618,7 @@
         </is>
       </c>
       <c r="I36" s="61" t="n">
-        <v>0.00827607</v>
+        <v>0.00831993</v>
       </c>
       <c r="J36" s="6" t="inlineStr">
         <is>
@@ -27643,7 +27643,7 @@
         </is>
       </c>
       <c r="I37" s="61" t="n">
-        <v>0.00669426</v>
+        <v>0.006701970000000001</v>
       </c>
       <c r="J37" s="6" t="inlineStr">
         <is>
@@ -27668,7 +27668,7 @@
         </is>
       </c>
       <c r="I38" s="61" t="n">
-        <v>0.00639543</v>
+        <v>0.00643539</v>
       </c>
       <c r="J38" s="6" t="inlineStr">
         <is>
@@ -27693,7 +27693,7 @@
         </is>
       </c>
       <c r="I39" s="61" t="n">
-        <v>0.00607187</v>
+        <v>0.00607153</v>
       </c>
       <c r="J39" s="6" t="inlineStr">
         <is>
@@ -27718,7 +27718,7 @@
         </is>
       </c>
       <c r="I40" s="61" t="n">
-        <v>0.00587245</v>
+        <v>0.00590588</v>
       </c>
       <c r="J40" s="6" t="inlineStr">
         <is>
@@ -27743,7 +27743,7 @@
         </is>
       </c>
       <c r="I41" s="61" t="n">
-        <v>0.00572298</v>
+        <v>0.00574028</v>
       </c>
       <c r="J41" s="6" t="inlineStr">
         <is>
@@ -27768,7 +27768,7 @@
         </is>
       </c>
       <c r="I42" s="61" t="n">
-        <v>0.00572055</v>
+        <v>0.005618499999999999</v>
       </c>
       <c r="J42" s="6" t="inlineStr">
         <is>
@@ -27793,7 +27793,7 @@
         </is>
       </c>
       <c r="I43" s="61" t="n">
-        <v>0.00532826</v>
+        <v>0.00532189</v>
       </c>
       <c r="J43" s="6" t="inlineStr">
         <is>
@@ -27814,20 +27814,20 @@
     <row r="44">
       <c r="H44" s="6" t="inlineStr">
         <is>
-          <t>BR</t>
+          <t>DINO</t>
         </is>
       </c>
       <c r="I44" s="61" t="n">
-        <v>0.00481132</v>
+        <v>0.0048129</v>
       </c>
       <c r="J44" s="6" t="inlineStr">
         <is>
-          <t>BROADRIDGE FINANCIAL SOLUTIONS INC</t>
+          <t>HF SINCLAIR</t>
         </is>
       </c>
       <c r="K44" s="6" t="inlineStr">
         <is>
-          <t>Industrials</t>
+          <t>Energy</t>
         </is>
       </c>
       <c r="L44" s="6" t="inlineStr"/>
@@ -27839,20 +27839,20 @@
     <row r="45">
       <c r="H45" s="6" t="inlineStr">
         <is>
-          <t>DINO</t>
+          <t>BR</t>
         </is>
       </c>
       <c r="I45" s="61" t="n">
-        <v>0.00478645</v>
+        <v>0.00480721</v>
       </c>
       <c r="J45" s="6" t="inlineStr">
         <is>
-          <t>HF SINCLAIR</t>
+          <t>BROADRIDGE FINANCIAL SOLUTIONS INC</t>
         </is>
       </c>
       <c r="K45" s="6" t="inlineStr">
         <is>
-          <t>Energy</t>
+          <t>Industrials</t>
         </is>
       </c>
       <c r="L45" s="6" t="inlineStr"/>
@@ -27868,7 +27868,7 @@
         </is>
       </c>
       <c r="I46" s="61" t="n">
-        <v>0.00475361</v>
+        <v>0.00474319</v>
       </c>
       <c r="J46" s="6" t="inlineStr">
         <is>
@@ -27893,7 +27893,7 @@
         </is>
       </c>
       <c r="I47" s="61" t="n">
-        <v>0.00440205</v>
+        <v>0.00442888</v>
       </c>
       <c r="J47" s="6" t="inlineStr">
         <is>
@@ -27918,7 +27918,7 @@
         </is>
       </c>
       <c r="I48" s="61" t="n">
-        <v>0.00439755</v>
+        <v>0.0043629</v>
       </c>
       <c r="J48" s="6" t="inlineStr">
         <is>
@@ -27943,7 +27943,7 @@
         </is>
       </c>
       <c r="I49" s="61" t="n">
-        <v>0.00438552</v>
+        <v>0.00435788</v>
       </c>
       <c r="J49" s="6" t="inlineStr">
         <is>
@@ -27968,7 +27968,7 @@
         </is>
       </c>
       <c r="I50" s="61" t="n">
-        <v>0.00409683</v>
+        <v>0.00415646</v>
       </c>
       <c r="J50" s="6" t="inlineStr">
         <is>
@@ -27993,7 +27993,7 @@
         </is>
       </c>
       <c r="I51" s="61" t="n">
-        <v>0.00253814</v>
+        <v>0.00258126</v>
       </c>
       <c r="J51" s="6" t="inlineStr">
         <is>
@@ -28018,7 +28018,7 @@
         </is>
       </c>
       <c r="I52" s="61" t="n">
-        <v>0.00252111</v>
+        <v>0.00251795</v>
       </c>
       <c r="J52" s="6" t="inlineStr">
         <is>
@@ -28043,7 +28043,7 @@
         </is>
       </c>
       <c r="I53" s="61" t="n">
-        <v>0.00247576</v>
+        <v>0.00250375</v>
       </c>
       <c r="J53" s="6" t="inlineStr">
         <is>
@@ -28068,7 +28068,7 @@
         </is>
       </c>
       <c r="I54" s="61" t="n">
-        <v>0.00226879</v>
+        <v>0.00224197</v>
       </c>
       <c r="J54" s="6" t="inlineStr">
         <is>
@@ -28093,7 +28093,7 @@
         </is>
       </c>
       <c r="I55" s="61" t="n">
-        <v>0.00216306</v>
+        <v>0.00214089</v>
       </c>
       <c r="J55" s="6" t="inlineStr">
         <is>
@@ -28118,7 +28118,7 @@
         </is>
       </c>
       <c r="I56" s="61" t="n">
-        <v>0.00204651</v>
+        <v>0.00204087</v>
       </c>
       <c r="J56" s="6" t="inlineStr">
         <is>
@@ -28143,7 +28143,7 @@
         </is>
       </c>
       <c r="I57" s="61" t="n">
-        <v>0.0018663</v>
+        <v>0.00186367</v>
       </c>
       <c r="J57" s="6" t="inlineStr">
         <is>
@@ -28168,7 +28168,7 @@
         </is>
       </c>
       <c r="I58" s="61" t="n">
-        <v>0.00152055</v>
+        <v>0.00153021</v>
       </c>
       <c r="J58" s="6" t="inlineStr">
         <is>
@@ -28193,7 +28193,7 @@
         </is>
       </c>
       <c r="I59" s="61" t="n">
-        <v>0.00151452</v>
+        <v>0.00149316</v>
       </c>
       <c r="J59" s="6" t="inlineStr">
         <is>
@@ -28218,7 +28218,7 @@
         </is>
       </c>
       <c r="I60" s="61" t="n">
-        <v>0.00146504</v>
+        <v>0.00147345</v>
       </c>
       <c r="J60" s="6" t="inlineStr">
         <is>
@@ -28239,20 +28239,20 @@
     <row r="61">
       <c r="H61" s="6" t="inlineStr">
         <is>
-          <t>MTN</t>
+          <t>MUR</t>
         </is>
       </c>
       <c r="I61" s="61" t="n">
-        <v>0.00132875</v>
+        <v>0.00134565</v>
       </c>
       <c r="J61" s="6" t="inlineStr">
         <is>
-          <t>VAIL RESORTS</t>
+          <t>MURPHY OIL CORP</t>
         </is>
       </c>
       <c r="K61" s="6" t="inlineStr">
         <is>
-          <t>Consumer Discretionary</t>
+          <t>Energy</t>
         </is>
       </c>
       <c r="L61" s="6" t="inlineStr"/>
@@ -28264,20 +28264,20 @@
     <row r="62">
       <c r="H62" s="6" t="inlineStr">
         <is>
-          <t>MUR</t>
+          <t>MTN</t>
         </is>
       </c>
       <c r="I62" s="61" t="n">
-        <v>0.0013268</v>
+        <v>0.00132723</v>
       </c>
       <c r="J62" s="6" t="inlineStr">
         <is>
-          <t>MURPHY OIL CORP</t>
+          <t>VAIL RESORTS</t>
         </is>
       </c>
       <c r="K62" s="6" t="inlineStr">
         <is>
-          <t>Energy</t>
+          <t>Consumer Discretionary</t>
         </is>
       </c>
       <c r="L62" s="6" t="inlineStr"/>
@@ -28293,7 +28293,7 @@
         </is>
       </c>
       <c r="I63" s="61" t="n">
-        <v>0.0011899</v>
+        <v>0.00117918</v>
       </c>
       <c r="J63" s="6" t="inlineStr">
         <is>
@@ -28318,7 +28318,7 @@
         </is>
       </c>
       <c r="I64" s="61" t="n">
-        <v>0.00114609</v>
+        <v>0.00116572</v>
       </c>
       <c r="J64" s="6" t="inlineStr">
         <is>
@@ -28343,7 +28343,7 @@
         </is>
       </c>
       <c r="I65" s="61" t="n">
-        <v>0.00107629</v>
+        <v>0.0010776</v>
       </c>
       <c r="J65" s="6" t="inlineStr">
         <is>
@@ -28368,7 +28368,7 @@
         </is>
       </c>
       <c r="I66" s="61" t="n">
-        <v>0.00102357</v>
+        <v>0.00101182</v>
       </c>
       <c r="J66" s="6" t="inlineStr">
         <is>
@@ -28389,20 +28389,20 @@
     <row r="67">
       <c r="H67" s="6" t="inlineStr">
         <is>
-          <t>KFY</t>
+          <t>CWEN</t>
         </is>
       </c>
       <c r="I67" s="61" t="n">
-        <v>0.0009363900000000001</v>
+        <v>0.00093153</v>
       </c>
       <c r="J67" s="6" t="inlineStr">
         <is>
-          <t>KORN FERRY</t>
+          <t>CLEARWAY ENERGY INC CLASS C</t>
         </is>
       </c>
       <c r="K67" s="6" t="inlineStr">
         <is>
-          <t>Industrials</t>
+          <t>Utilities</t>
         </is>
       </c>
       <c r="L67" s="6" t="inlineStr"/>
@@ -28414,20 +28414,20 @@
     <row r="68">
       <c r="H68" s="6" t="inlineStr">
         <is>
-          <t>CWEN</t>
+          <t>KFY</t>
         </is>
       </c>
       <c r="I68" s="61" t="n">
-        <v>0.0009310200000000001</v>
+        <v>0.00092506</v>
       </c>
       <c r="J68" s="6" t="inlineStr">
         <is>
-          <t>CLEARWAY ENERGY INC CLASS C</t>
+          <t>KORN FERRY</t>
         </is>
       </c>
       <c r="K68" s="6" t="inlineStr">
         <is>
-          <t>Utilities</t>
+          <t>Industrials</t>
         </is>
       </c>
       <c r="L68" s="6" t="inlineStr"/>
@@ -28443,7 +28443,7 @@
         </is>
       </c>
       <c r="I69" s="61" t="n">
-        <v>0.00091457</v>
+        <v>0.00091434</v>
       </c>
       <c r="J69" s="6" t="inlineStr">
         <is>
@@ -28468,7 +28468,7 @@
         </is>
       </c>
       <c r="I70" s="61" t="n">
-        <v>0.00088438</v>
+        <v>0.0008758</v>
       </c>
       <c r="J70" s="6" t="inlineStr">
         <is>
@@ -28493,7 +28493,7 @@
         </is>
       </c>
       <c r="I71" s="61" t="n">
-        <v>0.00086883</v>
+        <v>0.0008741300000000001</v>
       </c>
       <c r="J71" s="6" t="inlineStr">
         <is>
@@ -28514,18 +28514,22 @@
     <row r="72">
       <c r="H72" s="6" t="inlineStr">
         <is>
-          <t>GVMXX</t>
+          <t>APAM</t>
         </is>
       </c>
       <c r="I72" s="61" t="n">
-        <v>0.00069814</v>
+        <v>0.0005806</v>
       </c>
       <c r="J72" s="6" t="inlineStr">
         <is>
-          <t>SSC GOVERNMENT MM GVMXX</t>
-        </is>
-      </c>
-      <c r="K72" s="6" t="inlineStr"/>
+          <t>ARTISAN PARTNERS ASSET MANAGEMENT</t>
+        </is>
+      </c>
+      <c r="K72" s="6" t="inlineStr">
+        <is>
+          <t>Financials</t>
+        </is>
+      </c>
       <c r="L72" s="6" t="inlineStr"/>
       <c r="M72" s="7">
         <f>IF(H72="","",IFERROR(VLOOKUP(K72,$P$5:$Q$15,2,FALSE),"현금·선물"))</f>
@@ -28535,15 +28539,15 @@
     <row r="73">
       <c r="H73" s="6" t="inlineStr">
         <is>
-          <t>APAM</t>
+          <t>BANR</t>
         </is>
       </c>
       <c r="I73" s="61" t="n">
-        <v>0.0006036699999999999</v>
+        <v>0.00057219</v>
       </c>
       <c r="J73" s="6" t="inlineStr">
         <is>
-          <t>ARTISAN PARTNERS ASSET MANAGEMENT</t>
+          <t>BANNER CORP</t>
         </is>
       </c>
       <c r="K73" s="6" t="inlineStr">
@@ -28560,15 +28564,15 @@
     <row r="74">
       <c r="H74" s="6" t="inlineStr">
         <is>
-          <t>BANR</t>
+          <t>OFG</t>
         </is>
       </c>
       <c r="I74" s="61" t="n">
-        <v>0.00057333</v>
+        <v>0.00054473</v>
       </c>
       <c r="J74" s="6" t="inlineStr">
         <is>
-          <t>BANNER CORP</t>
+          <t>OFG BANCORP</t>
         </is>
       </c>
       <c r="K74" s="6" t="inlineStr">
@@ -28585,20 +28589,20 @@
     <row r="75">
       <c r="H75" s="6" t="inlineStr">
         <is>
-          <t>OFG</t>
+          <t>IPAR</t>
         </is>
       </c>
       <c r="I75" s="61" t="n">
-        <v>0.00054572</v>
+        <v>0.0005197999999999999</v>
       </c>
       <c r="J75" s="6" t="inlineStr">
         <is>
-          <t>OFG BANCORP</t>
+          <t>INTERPARFUMS INC</t>
         </is>
       </c>
       <c r="K75" s="6" t="inlineStr">
         <is>
-          <t>Financials</t>
+          <t>Consumer Staples</t>
         </is>
       </c>
       <c r="L75" s="6" t="inlineStr"/>
@@ -28610,15 +28614,15 @@
     <row r="76">
       <c r="H76" s="6" t="inlineStr">
         <is>
-          <t>IPAR</t>
+          <t>MZTI</t>
         </is>
       </c>
       <c r="I76" s="61" t="n">
-        <v>0.0005233</v>
+        <v>0.0004995900000000001</v>
       </c>
       <c r="J76" s="6" t="inlineStr">
         <is>
-          <t>INTERPARFUMS INC</t>
+          <t>MARZETTI</t>
         </is>
       </c>
       <c r="K76" s="6" t="inlineStr">
@@ -28639,7 +28643,7 @@
         </is>
       </c>
       <c r="I77" s="61" t="n">
-        <v>0.0005022399999999999</v>
+        <v>0.00049819</v>
       </c>
       <c r="J77" s="6" t="inlineStr">
         <is>
@@ -28664,7 +28668,7 @@
         </is>
       </c>
       <c r="I78" s="61" t="n">
-        <v>0.0005004100000000001</v>
+        <v>0.0004946</v>
       </c>
       <c r="J78" s="6" t="inlineStr">
         <is>
@@ -28685,20 +28689,20 @@
     <row r="79">
       <c r="H79" s="6" t="inlineStr">
         <is>
-          <t>MZTI</t>
+          <t>WU</t>
         </is>
       </c>
       <c r="I79" s="61" t="n">
-        <v>0.00049391</v>
+        <v>0.00048395</v>
       </c>
       <c r="J79" s="6" t="inlineStr">
         <is>
-          <t>MARZETTI</t>
+          <t>WESTERN UNION</t>
         </is>
       </c>
       <c r="K79" s="6" t="inlineStr">
         <is>
-          <t>Consumer Staples</t>
+          <t>Financials</t>
         </is>
       </c>
       <c r="L79" s="6" t="inlineStr"/>
@@ -28710,15 +28714,15 @@
     <row r="80">
       <c r="H80" s="6" t="inlineStr">
         <is>
-          <t>WU</t>
+          <t>AGM</t>
         </is>
       </c>
       <c r="I80" s="61" t="n">
-        <v>0.00048848</v>
+        <v>0.00048145</v>
       </c>
       <c r="J80" s="6" t="inlineStr">
         <is>
-          <t>WESTERN UNION</t>
+          <t>FEDERAL AGRICULTURAL MORTGAGE NON</t>
         </is>
       </c>
       <c r="K80" s="6" t="inlineStr">
@@ -28735,15 +28739,15 @@
     <row r="81">
       <c r="H81" s="6" t="inlineStr">
         <is>
-          <t>AGM</t>
+          <t>GABC</t>
         </is>
       </c>
       <c r="I81" s="61" t="n">
-        <v>0.00048224</v>
+        <v>0.00046591</v>
       </c>
       <c r="J81" s="6" t="inlineStr">
         <is>
-          <t>FEDERAL AGRICULTURAL MORTGAGE NON</t>
+          <t>GERMAN AMERICAN BANCORP INC</t>
         </is>
       </c>
       <c r="K81" s="6" t="inlineStr">
@@ -28760,20 +28764,20 @@
     <row r="82">
       <c r="H82" s="6" t="inlineStr">
         <is>
-          <t>GABC</t>
+          <t>NSP</t>
         </is>
       </c>
       <c r="I82" s="61" t="n">
-        <v>0.00046319</v>
+        <v>0.00044001</v>
       </c>
       <c r="J82" s="6" t="inlineStr">
         <is>
-          <t>GERMAN AMERICAN BANCORP INC</t>
+          <t>INSPERITY</t>
         </is>
       </c>
       <c r="K82" s="6" t="inlineStr">
         <is>
-          <t>Financials</t>
+          <t>Industrials</t>
         </is>
       </c>
       <c r="L82" s="6" t="inlineStr"/>
@@ -28785,20 +28789,20 @@
     <row r="83">
       <c r="H83" s="6" t="inlineStr">
         <is>
-          <t>NSP</t>
+          <t>STBA</t>
         </is>
       </c>
       <c r="I83" s="61" t="n">
-        <v>0.00044532</v>
+        <v>0.0004335399999999999</v>
       </c>
       <c r="J83" s="6" t="inlineStr">
         <is>
-          <t>INSPERITY</t>
+          <t>S AND T BANCORP INC</t>
         </is>
       </c>
       <c r="K83" s="6" t="inlineStr">
         <is>
-          <t>Industrials</t>
+          <t>Financials</t>
         </is>
       </c>
       <c r="L83" s="6" t="inlineStr"/>
@@ -28810,15 +28814,15 @@
     <row r="84">
       <c r="H84" s="6" t="inlineStr">
         <is>
-          <t>STBA</t>
+          <t>NBHC</t>
         </is>
       </c>
       <c r="I84" s="61" t="n">
-        <v>0.00043367</v>
+        <v>0.00042875</v>
       </c>
       <c r="J84" s="6" t="inlineStr">
         <is>
-          <t>S AND T BANCORP INC</t>
+          <t>NATIONAL BANK HOLDINGS CORP CLASS</t>
         </is>
       </c>
       <c r="K84" s="6" t="inlineStr">
@@ -28835,15 +28839,15 @@
     <row r="85">
       <c r="H85" s="6" t="inlineStr">
         <is>
-          <t>NBHC</t>
+          <t>SRCE</t>
         </is>
       </c>
       <c r="I85" s="61" t="n">
-        <v>0.00043071</v>
+        <v>0.00038317</v>
       </c>
       <c r="J85" s="6" t="inlineStr">
         <is>
-          <t>NATIONAL BANK HOLDINGS CORP CLASS</t>
+          <t>1ST SOURCE</t>
         </is>
       </c>
       <c r="K85" s="6" t="inlineStr">
@@ -28860,15 +28864,15 @@
     <row r="86">
       <c r="H86" s="6" t="inlineStr">
         <is>
-          <t>SRCE</t>
+          <t>LKFN</t>
         </is>
       </c>
       <c r="I86" s="61" t="n">
-        <v>0.00038251</v>
+        <v>0.00036137</v>
       </c>
       <c r="J86" s="6" t="inlineStr">
         <is>
-          <t>1ST SOURCE</t>
+          <t>LAKELAND FINANCIAL CORP</t>
         </is>
       </c>
       <c r="K86" s="6" t="inlineStr">
@@ -28885,20 +28889,20 @@
     <row r="87">
       <c r="H87" s="6" t="inlineStr">
         <is>
-          <t>LKFN</t>
+          <t>BKE</t>
         </is>
       </c>
       <c r="I87" s="61" t="n">
-        <v>0.00036163</v>
+        <v>0.00034331</v>
       </c>
       <c r="J87" s="6" t="inlineStr">
         <is>
-          <t>LAKELAND FINANCIAL CORP</t>
+          <t>BUCKLE</t>
         </is>
       </c>
       <c r="K87" s="6" t="inlineStr">
         <is>
-          <t>Financials</t>
+          <t>Consumer Discretionary</t>
         </is>
       </c>
       <c r="L87" s="6" t="inlineStr"/>
@@ -28910,20 +28914,20 @@
     <row r="88">
       <c r="H88" s="6" t="inlineStr">
         <is>
-          <t>BKE</t>
+          <t>FLO</t>
         </is>
       </c>
       <c r="I88" s="61" t="n">
-        <v>0.00034677</v>
+        <v>0.00032477</v>
       </c>
       <c r="J88" s="6" t="inlineStr">
         <is>
-          <t>BUCKLE</t>
+          <t>FLOWERS FOODS INC</t>
         </is>
       </c>
       <c r="K88" s="6" t="inlineStr">
         <is>
-          <t>Consumer Discretionary</t>
+          <t>Consumer Staples</t>
         </is>
       </c>
       <c r="L88" s="6" t="inlineStr"/>
@@ -28935,20 +28939,20 @@
     <row r="89">
       <c r="H89" s="6" t="inlineStr">
         <is>
-          <t>FLO</t>
+          <t>PFBC</t>
         </is>
       </c>
       <c r="I89" s="61" t="n">
-        <v>0.00031481</v>
+        <v>0.00028576</v>
       </c>
       <c r="J89" s="6" t="inlineStr">
         <is>
-          <t>FLOWERS FOODS INC</t>
+          <t>PREFERRED BANK</t>
         </is>
       </c>
       <c r="K89" s="6" t="inlineStr">
         <is>
-          <t>Consumer Staples</t>
+          <t>Financials</t>
         </is>
       </c>
       <c r="L89" s="6" t="inlineStr"/>
@@ -28960,20 +28964,20 @@
     <row r="90">
       <c r="H90" s="6" t="inlineStr">
         <is>
-          <t>PFBC</t>
+          <t>WEN</t>
         </is>
       </c>
       <c r="I90" s="61" t="n">
-        <v>0.00028586</v>
+        <v>0.00025686</v>
       </c>
       <c r="J90" s="6" t="inlineStr">
         <is>
-          <t>PREFERRED BANK</t>
+          <t>WENDYS</t>
         </is>
       </c>
       <c r="K90" s="6" t="inlineStr">
         <is>
-          <t>Financials</t>
+          <t>Consumer Discretionary</t>
         </is>
       </c>
       <c r="L90" s="6" t="inlineStr"/>
@@ -28989,7 +28993,7 @@
         </is>
       </c>
       <c r="I91" s="61" t="n">
-        <v>0.00025597</v>
+        <v>0.0002567</v>
       </c>
       <c r="J91" s="6" t="inlineStr">
         <is>
@@ -29010,22 +29014,18 @@
     <row r="92">
       <c r="H92" s="6" t="inlineStr">
         <is>
-          <t>WEN</t>
+          <t>GVMXX</t>
         </is>
       </c>
       <c r="I92" s="61" t="n">
-        <v>0.00025556</v>
+        <v>0.00024435</v>
       </c>
       <c r="J92" s="6" t="inlineStr">
         <is>
-          <t>WENDYS</t>
-        </is>
-      </c>
-      <c r="K92" s="6" t="inlineStr">
-        <is>
-          <t>Consumer Discretionary</t>
-        </is>
-      </c>
+          <t>SSC GOVERNMENT MM GVMXX</t>
+        </is>
+      </c>
+      <c r="K92" s="6" t="inlineStr"/>
       <c r="L92" s="6" t="inlineStr"/>
       <c r="M92" s="7">
         <f>IF(H92="","",IFERROR(VLOOKUP(K92,$P$5:$Q$15,2,FALSE),"현금·선물"))</f>
@@ -29039,7 +29039,7 @@
         </is>
       </c>
       <c r="I93" s="61" t="n">
-        <v>0.00023346</v>
+        <v>0.00023328</v>
       </c>
       <c r="J93" s="6" t="inlineStr">
         <is>
@@ -29064,7 +29064,7 @@
         </is>
       </c>
       <c r="I94" s="61" t="n">
-        <v>0.00023183</v>
+        <v>0.00023229</v>
       </c>
       <c r="J94" s="6" t="inlineStr">
         <is>
@@ -29089,7 +29089,7 @@
         </is>
       </c>
       <c r="I95" s="61" t="n">
-        <v>0.00020811</v>
+        <v>0.00020862</v>
       </c>
       <c r="J95" s="6" t="inlineStr">
         <is>
@@ -29114,7 +29114,7 @@
         </is>
       </c>
       <c r="I96" s="61" t="n">
-        <v>0.00020509</v>
+        <v>0.00020236</v>
       </c>
       <c r="J96" s="6" t="inlineStr">
         <is>
@@ -29139,7 +29139,7 @@
         </is>
       </c>
       <c r="I97" s="61" t="n">
-        <v>0.00020096</v>
+        <v>0.0002006</v>
       </c>
       <c r="J97" s="6" t="inlineStr">
         <is>
@@ -29164,7 +29164,7 @@
         </is>
       </c>
       <c r="I98" s="61" t="n">
-        <v>0.00019848</v>
+        <v>0.00019921</v>
       </c>
       <c r="J98" s="6" t="inlineStr">
         <is>
@@ -29189,7 +29189,7 @@
         </is>
       </c>
       <c r="I99" s="61" t="n">
-        <v>0.00016827</v>
+        <v>0.00016796</v>
       </c>
       <c r="J99" s="6" t="inlineStr">
         <is>
@@ -29210,18 +29210,22 @@
     <row r="100">
       <c r="H100" s="6" t="inlineStr">
         <is>
-          <t>USD</t>
+          <t>EBF</t>
         </is>
       </c>
       <c r="I100" s="61" t="n">
-        <v>0.00013909</v>
+        <v>0.00013436</v>
       </c>
       <c r="J100" s="6" t="inlineStr">
         <is>
-          <t>US DOLLAR</t>
-        </is>
-      </c>
-      <c r="K100" s="6" t="inlineStr"/>
+          <t>ENNIS INC</t>
+        </is>
+      </c>
+      <c r="K100" s="6" t="inlineStr">
+        <is>
+          <t>Industrials</t>
+        </is>
+      </c>
       <c r="L100" s="6" t="inlineStr"/>
       <c r="M100" s="7">
         <f>IF(H100="","",IFERROR(VLOOKUP(K100,$P$5:$Q$15,2,FALSE),"현금·선물"))</f>
@@ -29231,22 +29235,18 @@
     <row r="101">
       <c r="H101" s="6" t="inlineStr">
         <is>
-          <t>EBF</t>
+          <t>USD</t>
         </is>
       </c>
       <c r="I101" s="61" t="n">
-        <v>0.00013509</v>
+        <v>0.00012374</v>
       </c>
       <c r="J101" s="6" t="inlineStr">
         <is>
-          <t>ENNIS INC</t>
-        </is>
-      </c>
-      <c r="K101" s="6" t="inlineStr">
-        <is>
-          <t>Industrials</t>
-        </is>
-      </c>
+          <t>US DOLLAR</t>
+        </is>
+      </c>
+      <c r="K101" s="6" t="inlineStr"/>
       <c r="L101" s="6" t="inlineStr"/>
       <c r="M101" s="7">
         <f>IF(H101="","",IFERROR(VLOOKUP(K101,$P$5:$Q$15,2,FALSE),"현금·선물"))</f>
@@ -29260,7 +29260,7 @@
         </is>
       </c>
       <c r="I102" s="61" t="n">
-        <v>0.00011563</v>
+        <v>0.00011731</v>
       </c>
       <c r="J102" s="6" t="inlineStr">
         <is>
@@ -29285,7 +29285,7 @@
         </is>
       </c>
       <c r="I103" s="61" t="n">
-        <v>0.00010387</v>
+        <v>0.00010297</v>
       </c>
       <c r="J103" s="6" t="inlineStr">
         <is>
@@ -29310,7 +29310,7 @@
         </is>
       </c>
       <c r="I104" s="61" t="n">
-        <v>9.005000000000001e-05</v>
+        <v>8.899e-05</v>
       </c>
       <c r="J104" s="6" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
데이터 갱신: holdings,kr_etf (2026-10-14)
</commit_message>
<xml_diff>
--- a/downloads/schd_dividend_tracker.xlsx
+++ b/downloads/schd_dividend_tracker.xlsx
@@ -1724,7 +1724,7 @@
     <row r="3">
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>최종 갱신: 2026-10-13 · 반영 범위: 2012년 1분기 ~ 2026년 3분기 (배당락 2026-09-23) · GitHub Actions 자동 생성</t>
+          <t>최종 갱신: 2026-10-14 · 반영 범위: 2012년 1분기 ~ 2026년 3분기 (배당락 2026-09-23) · GitHub Actions 자동 생성</t>
         </is>
       </c>
     </row>
@@ -20053,7 +20053,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F355"/>
+  <dimension ref="A1:F357"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -22808,22 +22808,22 @@
     <row r="131">
       <c r="A131" s="46" t="inlineStr">
         <is>
-          <t>489250</t>
+          <t>402970</t>
         </is>
       </c>
       <c r="B131" s="33" t="inlineStr">
         <is>
-          <t>KODEX 미국배당다우존스</t>
+          <t>ACE 미국배당다우존스</t>
         </is>
       </c>
       <c r="C131" s="26" t="n">
-        <v>45547</v>
+        <v>46309</v>
       </c>
       <c r="D131" s="47" t="n">
-        <v>30</v>
+        <v>38</v>
       </c>
       <c r="E131" s="48" t="n">
-        <v>0.002954</v>
+        <v>0.002624</v>
       </c>
     </row>
     <row r="132">
@@ -22838,13 +22838,13 @@
         </is>
       </c>
       <c r="C132" s="26" t="n">
-        <v>45579</v>
+        <v>45547</v>
       </c>
       <c r="D132" s="47" t="n">
-        <v>33</v>
+        <v>30</v>
       </c>
       <c r="E132" s="48" t="n">
-        <v>0.003148</v>
+        <v>0.002954</v>
       </c>
     </row>
     <row r="133">
@@ -22859,13 +22859,13 @@
         </is>
       </c>
       <c r="C133" s="26" t="n">
-        <v>45610</v>
+        <v>45579</v>
       </c>
       <c r="D133" s="47" t="n">
-        <v>28</v>
+        <v>33</v>
       </c>
       <c r="E133" s="48" t="n">
-        <v>0.002509</v>
+        <v>0.003148</v>
       </c>
     </row>
     <row r="134">
@@ -22880,13 +22880,13 @@
         </is>
       </c>
       <c r="C134" s="26" t="n">
-        <v>45638</v>
+        <v>45610</v>
       </c>
       <c r="D134" s="47" t="n">
-        <v>41</v>
+        <v>28</v>
       </c>
       <c r="E134" s="48" t="n">
-        <v>0.003647</v>
+        <v>0.002509</v>
       </c>
     </row>
     <row r="135">
@@ -22901,13 +22901,13 @@
         </is>
       </c>
       <c r="C135" s="26" t="n">
-        <v>45671</v>
+        <v>45638</v>
       </c>
       <c r="D135" s="47" t="n">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="E135" s="48" t="n">
-        <v>0.003659</v>
+        <v>0.003647</v>
       </c>
     </row>
     <row r="136">
@@ -22922,13 +22922,13 @@
         </is>
       </c>
       <c r="C136" s="26" t="n">
-        <v>45701</v>
+        <v>45671</v>
       </c>
       <c r="D136" s="47" t="n">
-        <v>32</v>
+        <v>40</v>
       </c>
       <c r="E136" s="48" t="n">
-        <v>0.002909</v>
+        <v>0.003659</v>
       </c>
     </row>
     <row r="137">
@@ -22943,13 +22943,13 @@
         </is>
       </c>
       <c r="C137" s="26" t="n">
-        <v>45729</v>
+        <v>45701</v>
       </c>
       <c r="D137" s="47" t="n">
-        <v>29</v>
+        <v>32</v>
       </c>
       <c r="E137" s="48" t="n">
-        <v>0.002634</v>
+        <v>0.002909</v>
       </c>
     </row>
     <row r="138">
@@ -22964,13 +22964,13 @@
         </is>
       </c>
       <c r="C138" s="26" t="n">
-        <v>45761</v>
+        <v>45729</v>
       </c>
       <c r="D138" s="47" t="n">
-        <v>34</v>
+        <v>29</v>
       </c>
       <c r="E138" s="48" t="n">
-        <v>0.003378</v>
+        <v>0.002634</v>
       </c>
     </row>
     <row r="139">
@@ -22985,13 +22985,13 @@
         </is>
       </c>
       <c r="C139" s="26" t="n">
-        <v>45791</v>
+        <v>45761</v>
       </c>
       <c r="D139" s="47" t="n">
-        <v>24</v>
+        <v>34</v>
       </c>
       <c r="E139" s="48" t="n">
-        <v>0.002356</v>
+        <v>0.003378</v>
       </c>
     </row>
     <row r="140">
@@ -23006,13 +23006,13 @@
         </is>
       </c>
       <c r="C140" s="26" t="n">
-        <v>45820</v>
+        <v>45791</v>
       </c>
       <c r="D140" s="47" t="n">
-        <v>30</v>
+        <v>24</v>
       </c>
       <c r="E140" s="48" t="n">
-        <v>0.00299</v>
+        <v>0.002356</v>
       </c>
     </row>
     <row r="141">
@@ -23027,13 +23027,13 @@
         </is>
       </c>
       <c r="C141" s="26" t="n">
-        <v>45852</v>
+        <v>45820</v>
       </c>
       <c r="D141" s="47" t="n">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="E141" s="48" t="n">
-        <v>0.003007</v>
+        <v>0.00299</v>
       </c>
     </row>
     <row r="142">
@@ -23048,13 +23048,13 @@
         </is>
       </c>
       <c r="C142" s="26" t="n">
-        <v>45882</v>
+        <v>45852</v>
       </c>
       <c r="D142" s="47" t="n">
-        <v>22</v>
+        <v>31</v>
       </c>
       <c r="E142" s="48" t="n">
-        <v>0.002165</v>
+        <v>0.003007</v>
       </c>
     </row>
     <row r="143">
@@ -23069,13 +23069,13 @@
         </is>
       </c>
       <c r="C143" s="26" t="n">
-        <v>45912</v>
+        <v>45882</v>
       </c>
       <c r="D143" s="47" t="n">
-        <v>28</v>
+        <v>22</v>
       </c>
       <c r="E143" s="48" t="n">
-        <v>0.002688</v>
+        <v>0.002165</v>
       </c>
     </row>
     <row r="144">
@@ -23090,13 +23090,13 @@
         </is>
       </c>
       <c r="C144" s="26" t="n">
-        <v>45944</v>
+        <v>45912</v>
       </c>
       <c r="D144" s="47" t="n">
-        <v>31</v>
+        <v>28</v>
       </c>
       <c r="E144" s="48" t="n">
-        <v>0.002989</v>
+        <v>0.002688</v>
       </c>
     </row>
     <row r="145">
@@ -23111,13 +23111,13 @@
         </is>
       </c>
       <c r="C145" s="26" t="n">
-        <v>45974</v>
+        <v>45944</v>
       </c>
       <c r="D145" s="47" t="n">
-        <v>21</v>
+        <v>31</v>
       </c>
       <c r="E145" s="48" t="n">
-        <v>0.001939</v>
+        <v>0.002989</v>
       </c>
     </row>
     <row r="146">
@@ -23132,13 +23132,13 @@
         </is>
       </c>
       <c r="C146" s="26" t="n">
-        <v>46003</v>
+        <v>45974</v>
       </c>
       <c r="D146" s="47" t="n">
-        <v>33</v>
+        <v>21</v>
       </c>
       <c r="E146" s="48" t="n">
-        <v>0.002966</v>
+        <v>0.001939</v>
       </c>
     </row>
     <row r="147">
@@ -23153,13 +23153,13 @@
         </is>
       </c>
       <c r="C147" s="26" t="n">
-        <v>46036</v>
+        <v>46003</v>
       </c>
       <c r="D147" s="47" t="n">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="E147" s="48" t="n">
-        <v>0.002964</v>
+        <v>0.002966</v>
       </c>
     </row>
     <row r="148">
@@ -23174,13 +23174,13 @@
         </is>
       </c>
       <c r="C148" s="26" t="n">
-        <v>46065</v>
+        <v>46036</v>
       </c>
       <c r="D148" s="47" t="n">
-        <v>28</v>
+        <v>34</v>
       </c>
       <c r="E148" s="48" t="n">
-        <v>0.00224</v>
+        <v>0.002964</v>
       </c>
     </row>
     <row r="149">
@@ -23195,13 +23195,13 @@
         </is>
       </c>
       <c r="C149" s="26" t="n">
-        <v>46093</v>
+        <v>46065</v>
       </c>
       <c r="D149" s="47" t="n">
-        <v>32</v>
+        <v>28</v>
       </c>
       <c r="E149" s="48" t="n">
-        <v>0.002589</v>
+        <v>0.00224</v>
       </c>
     </row>
     <row r="150">
@@ -23216,13 +23216,13 @@
         </is>
       </c>
       <c r="C150" s="26" t="n">
-        <v>46126</v>
+        <v>46093</v>
       </c>
       <c r="D150" s="47" t="n">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="E150" s="48" t="n">
-        <v>0.002645</v>
+        <v>0.002589</v>
       </c>
     </row>
     <row r="151">
@@ -23237,13 +23237,13 @@
         </is>
       </c>
       <c r="C151" s="26" t="n">
-        <v>46156</v>
+        <v>46126</v>
       </c>
       <c r="D151" s="47" t="n">
-        <v>26</v>
+        <v>33</v>
       </c>
       <c r="E151" s="48" t="n">
-        <v>0.002016</v>
+        <v>0.002645</v>
       </c>
     </row>
     <row r="152">
@@ -23258,13 +23258,13 @@
         </is>
       </c>
       <c r="C152" s="26" t="n">
-        <v>46185</v>
+        <v>46156</v>
       </c>
       <c r="D152" s="47" t="n">
-        <v>29</v>
+        <v>26</v>
       </c>
       <c r="E152" s="48" t="n">
-        <v>0.002161</v>
+        <v>0.002016</v>
       </c>
     </row>
     <row r="153">
@@ -23279,13 +23279,13 @@
         </is>
       </c>
       <c r="C153" s="26" t="n">
-        <v>46217</v>
+        <v>46185</v>
       </c>
       <c r="D153" s="47" t="n">
-        <v>40</v>
+        <v>29</v>
       </c>
       <c r="E153" s="48" t="n">
-        <v>0.003001</v>
+        <v>0.002161</v>
       </c>
     </row>
     <row r="154">
@@ -23300,13 +23300,13 @@
         </is>
       </c>
       <c r="C154" s="26" t="n">
-        <v>46247</v>
+        <v>46217</v>
       </c>
       <c r="D154" s="47" t="n">
-        <v>37</v>
+        <v>40</v>
       </c>
       <c r="E154" s="48" t="n">
-        <v>0.0028</v>
+        <v>0.003001</v>
       </c>
     </row>
     <row r="155">
@@ -23321,28 +23321,56 @@
         </is>
       </c>
       <c r="C155" s="26" t="n">
+        <v>46247</v>
+      </c>
+      <c r="D155" s="47" t="n">
+        <v>37</v>
+      </c>
+      <c r="E155" s="48" t="n">
+        <v>0.0028</v>
+      </c>
+    </row>
+    <row r="156">
+      <c r="A156" s="46" t="inlineStr">
+        <is>
+          <t>489250</t>
+        </is>
+      </c>
+      <c r="B156" s="33" t="inlineStr">
+        <is>
+          <t>KODEX 미국배당다우존스</t>
+        </is>
+      </c>
+      <c r="C156" s="26" t="n">
         <v>46279</v>
       </c>
-      <c r="D155" s="47" t="n">
+      <c r="D156" s="47" t="n">
         <v>24</v>
       </c>
-      <c r="E155" s="48" t="n">
+      <c r="E156" s="48" t="n">
         <v>0.001924</v>
       </c>
     </row>
-    <row r="156">
-      <c r="A156" s="46" t="n"/>
-      <c r="B156" s="33" t="n"/>
-      <c r="C156" s="26" t="n"/>
-      <c r="D156" s="47" t="n"/>
-      <c r="E156" s="48" t="n"/>
-    </row>
     <row r="157">
-      <c r="A157" s="46" t="n"/>
-      <c r="B157" s="33" t="n"/>
-      <c r="C157" s="26" t="n"/>
-      <c r="D157" s="47" t="n"/>
-      <c r="E157" s="48" t="n"/>
+      <c r="A157" s="46" t="inlineStr">
+        <is>
+          <t>489250</t>
+        </is>
+      </c>
+      <c r="B157" s="33" t="inlineStr">
+        <is>
+          <t>KODEX 미국배당다우존스</t>
+        </is>
+      </c>
+      <c r="C157" s="26" t="n">
+        <v>46309</v>
+      </c>
+      <c r="D157" s="47" t="n">
+        <v>37</v>
+      </c>
+      <c r="E157" s="48" t="n">
+        <v>0.003019</v>
+      </c>
     </row>
     <row r="158">
       <c r="A158" s="46" t="n"/>
@@ -24729,6 +24757,20 @@
       <c r="C355" s="26" t="n"/>
       <c r="D355" s="47" t="n"/>
       <c r="E355" s="48" t="n"/>
+    </row>
+    <row r="356">
+      <c r="A356" s="46" t="n"/>
+      <c r="B356" s="33" t="n"/>
+      <c r="C356" s="26" t="n"/>
+      <c r="D356" s="47" t="n"/>
+      <c r="E356" s="48" t="n"/>
+    </row>
+    <row r="357">
+      <c r="A357" s="46" t="n"/>
+      <c r="B357" s="33" t="n"/>
+      <c r="C357" s="26" t="n"/>
+      <c r="D357" s="47" t="n"/>
+      <c r="E357" s="48" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -24770,7 +24812,7 @@
         </is>
       </c>
       <c r="B3" s="49" t="n">
-        <v>46295</v>
+        <v>46326</v>
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
@@ -24850,23 +24892,23 @@
         </is>
       </c>
       <c r="E6" s="52">
-        <f>_xlfn.MAXIFS(국내SCHD형_분배!$C$2:$C$355,국내SCHD형_분배!$A$2:$A$355,$B6,국내SCHD형_분배!$C$2:$C$355,"&lt;="&amp;$B$3)</f>
+        <f>_xlfn.MAXIFS(국내SCHD형_분배!$C$2:$C$357,국내SCHD형_분배!$A$2:$A$357,$B6,국내SCHD형_분배!$C$2:$C$357,"&lt;="&amp;$B$3)</f>
         <v/>
       </c>
       <c r="F6" s="53">
-        <f>SUMIFS(국내SCHD형_분배!$D$2:$D$355,국내SCHD형_분배!$A$2:$A$355,$B6,국내SCHD형_분배!$C$2:$C$355,E6)</f>
+        <f>SUMIFS(국내SCHD형_분배!$D$2:$D$357,국내SCHD형_분배!$A$2:$A$357,$B6,국내SCHD형_분배!$C$2:$C$357,E6)</f>
         <v/>
       </c>
       <c r="G6" s="45">
-        <f>COUNTIFS(국내SCHD형_분배!$A$2:$A$355,$B6,국내SCHD형_분배!$C$2:$C$355,"&gt;"&amp;EDATE($B$3,-12),국내SCHD형_분배!$C$2:$C$355,"&lt;="&amp;$B$3)</f>
+        <f>COUNTIFS(국내SCHD형_분배!$A$2:$A$357,$B6,국내SCHD형_분배!$C$2:$C$357,"&gt;"&amp;EDATE($B$3,-12),국내SCHD형_분배!$C$2:$C$357,"&lt;="&amp;$B$3)</f>
         <v/>
       </c>
       <c r="H6" s="53">
-        <f>SUMIFS(국내SCHD형_분배!$D$2:$D$355,국내SCHD형_분배!$A$2:$A$355,$B6,국내SCHD형_분배!$C$2:$C$355,"&gt;"&amp;EDATE($B$3,-12),국내SCHD형_분배!$C$2:$C$355,"&lt;="&amp;$B$3)</f>
+        <f>SUMIFS(국내SCHD형_분배!$D$2:$D$357,국내SCHD형_분배!$A$2:$A$357,$B6,국내SCHD형_분배!$C$2:$C$357,"&gt;"&amp;EDATE($B$3,-12),국내SCHD형_분배!$C$2:$C$357,"&lt;="&amp;$B$3)</f>
         <v/>
       </c>
       <c r="I6" s="29">
-        <f>SUMIFS(국내SCHD형_분배!$E$2:$E$355,국내SCHD형_분배!$A$2:$A$355,$B6,국내SCHD형_분배!$C$2:$C$355,"&gt;"&amp;EDATE($B$3,-12),국내SCHD형_분배!$C$2:$C$355,"&lt;="&amp;$B$3)</f>
+        <f>SUMIFS(국내SCHD형_분배!$E$2:$E$357,국내SCHD형_분배!$A$2:$A$357,$B6,국내SCHD형_분배!$C$2:$C$357,"&gt;"&amp;EDATE($B$3,-12),국내SCHD형_분배!$C$2:$C$357,"&lt;="&amp;$B$3)</f>
         <v/>
       </c>
     </row>
@@ -24890,23 +24932,23 @@
         </is>
       </c>
       <c r="E7" s="52">
-        <f>_xlfn.MAXIFS(국내SCHD형_분배!$C$2:$C$355,국내SCHD형_분배!$A$2:$A$355,$B7,국내SCHD형_분배!$C$2:$C$355,"&lt;="&amp;$B$3)</f>
+        <f>_xlfn.MAXIFS(국내SCHD형_분배!$C$2:$C$357,국내SCHD형_분배!$A$2:$A$357,$B7,국내SCHD형_분배!$C$2:$C$357,"&lt;="&amp;$B$3)</f>
         <v/>
       </c>
       <c r="F7" s="53">
-        <f>SUMIFS(국내SCHD형_분배!$D$2:$D$355,국내SCHD형_분배!$A$2:$A$355,$B7,국내SCHD형_분배!$C$2:$C$355,E7)</f>
+        <f>SUMIFS(국내SCHD형_분배!$D$2:$D$357,국내SCHD형_분배!$A$2:$A$357,$B7,국내SCHD형_분배!$C$2:$C$357,E7)</f>
         <v/>
       </c>
       <c r="G7" s="45">
-        <f>COUNTIFS(국내SCHD형_분배!$A$2:$A$355,$B7,국내SCHD형_분배!$C$2:$C$355,"&gt;"&amp;EDATE($B$3,-12),국내SCHD형_분배!$C$2:$C$355,"&lt;="&amp;$B$3)</f>
+        <f>COUNTIFS(국내SCHD형_분배!$A$2:$A$357,$B7,국내SCHD형_분배!$C$2:$C$357,"&gt;"&amp;EDATE($B$3,-12),국내SCHD형_분배!$C$2:$C$357,"&lt;="&amp;$B$3)</f>
         <v/>
       </c>
       <c r="H7" s="53">
-        <f>SUMIFS(국내SCHD형_분배!$D$2:$D$355,국내SCHD형_분배!$A$2:$A$355,$B7,국내SCHD형_분배!$C$2:$C$355,"&gt;"&amp;EDATE($B$3,-12),국내SCHD형_분배!$C$2:$C$355,"&lt;="&amp;$B$3)</f>
+        <f>SUMIFS(국내SCHD형_분배!$D$2:$D$357,국내SCHD형_분배!$A$2:$A$357,$B7,국내SCHD형_분배!$C$2:$C$357,"&gt;"&amp;EDATE($B$3,-12),국내SCHD형_분배!$C$2:$C$357,"&lt;="&amp;$B$3)</f>
         <v/>
       </c>
       <c r="I7" s="29">
-        <f>SUMIFS(국내SCHD형_분배!$E$2:$E$355,국내SCHD형_분배!$A$2:$A$355,$B7,국내SCHD형_분배!$C$2:$C$355,"&gt;"&amp;EDATE($B$3,-12),국내SCHD형_분배!$C$2:$C$355,"&lt;="&amp;$B$3)</f>
+        <f>SUMIFS(국내SCHD형_분배!$E$2:$E$357,국내SCHD형_분배!$A$2:$A$357,$B7,국내SCHD형_분배!$C$2:$C$357,"&gt;"&amp;EDATE($B$3,-12),국내SCHD형_분배!$C$2:$C$357,"&lt;="&amp;$B$3)</f>
         <v/>
       </c>
     </row>
@@ -24930,23 +24972,23 @@
         </is>
       </c>
       <c r="E8" s="52">
-        <f>_xlfn.MAXIFS(국내SCHD형_분배!$C$2:$C$355,국내SCHD형_분배!$A$2:$A$355,$B8,국내SCHD형_분배!$C$2:$C$355,"&lt;="&amp;$B$3)</f>
+        <f>_xlfn.MAXIFS(국내SCHD형_분배!$C$2:$C$357,국내SCHD형_분배!$A$2:$A$357,$B8,국내SCHD형_분배!$C$2:$C$357,"&lt;="&amp;$B$3)</f>
         <v/>
       </c>
       <c r="F8" s="53">
-        <f>SUMIFS(국내SCHD형_분배!$D$2:$D$355,국내SCHD형_분배!$A$2:$A$355,$B8,국내SCHD형_분배!$C$2:$C$355,E8)</f>
+        <f>SUMIFS(국내SCHD형_분배!$D$2:$D$357,국내SCHD형_분배!$A$2:$A$357,$B8,국내SCHD형_분배!$C$2:$C$357,E8)</f>
         <v/>
       </c>
       <c r="G8" s="45">
-        <f>COUNTIFS(국내SCHD형_분배!$A$2:$A$355,$B8,국내SCHD형_분배!$C$2:$C$355,"&gt;"&amp;EDATE($B$3,-12),국내SCHD형_분배!$C$2:$C$355,"&lt;="&amp;$B$3)</f>
+        <f>COUNTIFS(국내SCHD형_분배!$A$2:$A$357,$B8,국내SCHD형_분배!$C$2:$C$357,"&gt;"&amp;EDATE($B$3,-12),국내SCHD형_분배!$C$2:$C$357,"&lt;="&amp;$B$3)</f>
         <v/>
       </c>
       <c r="H8" s="53">
-        <f>SUMIFS(국내SCHD형_분배!$D$2:$D$355,국내SCHD형_분배!$A$2:$A$355,$B8,국내SCHD형_분배!$C$2:$C$355,"&gt;"&amp;EDATE($B$3,-12),국내SCHD형_분배!$C$2:$C$355,"&lt;="&amp;$B$3)</f>
+        <f>SUMIFS(국내SCHD형_분배!$D$2:$D$357,국내SCHD형_분배!$A$2:$A$357,$B8,국내SCHD형_분배!$C$2:$C$357,"&gt;"&amp;EDATE($B$3,-12),국내SCHD형_분배!$C$2:$C$357,"&lt;="&amp;$B$3)</f>
         <v/>
       </c>
       <c r="I8" s="29">
-        <f>SUMIFS(국내SCHD형_분배!$E$2:$E$355,국내SCHD형_분배!$A$2:$A$355,$B8,국내SCHD형_분배!$C$2:$C$355,"&gt;"&amp;EDATE($B$3,-12),국내SCHD형_분배!$C$2:$C$355,"&lt;="&amp;$B$3)</f>
+        <f>SUMIFS(국내SCHD형_분배!$E$2:$E$357,국내SCHD형_분배!$A$2:$A$357,$B8,국내SCHD형_분배!$C$2:$C$357,"&gt;"&amp;EDATE($B$3,-12),국내SCHD형_분배!$C$2:$C$357,"&lt;="&amp;$B$3)</f>
         <v/>
       </c>
     </row>
@@ -24970,23 +25012,23 @@
         </is>
       </c>
       <c r="E9" s="52">
-        <f>_xlfn.MAXIFS(국내SCHD형_분배!$C$2:$C$355,국내SCHD형_분배!$A$2:$A$355,$B9,국내SCHD형_분배!$C$2:$C$355,"&lt;="&amp;$B$3)</f>
+        <f>_xlfn.MAXIFS(국내SCHD형_분배!$C$2:$C$357,국내SCHD형_분배!$A$2:$A$357,$B9,국내SCHD형_분배!$C$2:$C$357,"&lt;="&amp;$B$3)</f>
         <v/>
       </c>
       <c r="F9" s="53">
-        <f>SUMIFS(국내SCHD형_분배!$D$2:$D$355,국내SCHD형_분배!$A$2:$A$355,$B9,국내SCHD형_분배!$C$2:$C$355,E9)</f>
+        <f>SUMIFS(국내SCHD형_분배!$D$2:$D$357,국내SCHD형_분배!$A$2:$A$357,$B9,국내SCHD형_분배!$C$2:$C$357,E9)</f>
         <v/>
       </c>
       <c r="G9" s="45">
-        <f>COUNTIFS(국내SCHD형_분배!$A$2:$A$355,$B9,국내SCHD형_분배!$C$2:$C$355,"&gt;"&amp;EDATE($B$3,-12),국내SCHD형_분배!$C$2:$C$355,"&lt;="&amp;$B$3)</f>
+        <f>COUNTIFS(국내SCHD형_분배!$A$2:$A$357,$B9,국내SCHD형_분배!$C$2:$C$357,"&gt;"&amp;EDATE($B$3,-12),국내SCHD형_분배!$C$2:$C$357,"&lt;="&amp;$B$3)</f>
         <v/>
       </c>
       <c r="H9" s="53">
-        <f>SUMIFS(국내SCHD형_분배!$D$2:$D$355,국내SCHD형_분배!$A$2:$A$355,$B9,국내SCHD형_분배!$C$2:$C$355,"&gt;"&amp;EDATE($B$3,-12),국내SCHD형_분배!$C$2:$C$355,"&lt;="&amp;$B$3)</f>
+        <f>SUMIFS(국내SCHD형_분배!$D$2:$D$357,국내SCHD형_분배!$A$2:$A$357,$B9,국내SCHD형_분배!$C$2:$C$357,"&gt;"&amp;EDATE($B$3,-12),국내SCHD형_분배!$C$2:$C$357,"&lt;="&amp;$B$3)</f>
         <v/>
       </c>
       <c r="I9" s="29">
-        <f>SUMIFS(국내SCHD형_분배!$E$2:$E$355,국내SCHD형_분배!$A$2:$A$355,$B9,국내SCHD형_분배!$C$2:$C$355,"&gt;"&amp;EDATE($B$3,-12),국내SCHD형_분배!$C$2:$C$355,"&lt;="&amp;$B$3)</f>
+        <f>SUMIFS(국내SCHD형_분배!$E$2:$E$357,국내SCHD형_분배!$A$2:$A$357,$B9,국내SCHD형_분배!$C$2:$C$357,"&gt;"&amp;EDATE($B$3,-12),국내SCHD형_분배!$C$2:$C$357,"&lt;="&amp;$B$3)</f>
         <v/>
       </c>
     </row>
@@ -25121,19 +25163,19 @@
         <v/>
       </c>
       <c r="D17" s="53">
-        <f>IF(COUNTIFS(국내SCHD형_분배!$A$2:$A$355,"458730",국내SCHD형_분배!$C$2:$C$355,"&gt;="&amp;$B17,국내SCHD형_분배!$C$2:$C$355,"&lt;="&amp;$C17)=0,"",SUMIFS(국내SCHD형_분배!$D$2:$D$355,국내SCHD형_분배!$A$2:$A$355,"458730",국내SCHD형_분배!$C$2:$C$355,"&gt;="&amp;$B17,국내SCHD형_분배!$C$2:$C$355,"&lt;="&amp;$C17))</f>
+        <f>IF(COUNTIFS(국내SCHD형_분배!$A$2:$A$357,"458730",국내SCHD형_분배!$C$2:$C$357,"&gt;="&amp;$B17,국내SCHD형_분배!$C$2:$C$357,"&lt;="&amp;$C17)=0,"",SUMIFS(국내SCHD형_분배!$D$2:$D$357,국내SCHD형_분배!$A$2:$A$357,"458730",국내SCHD형_분배!$C$2:$C$357,"&gt;="&amp;$B17,국내SCHD형_분배!$C$2:$C$357,"&lt;="&amp;$C17))</f>
         <v/>
       </c>
       <c r="E17" s="53">
-        <f>IF(COUNTIFS(국내SCHD형_분배!$A$2:$A$355,"446720",국내SCHD형_분배!$C$2:$C$355,"&gt;="&amp;$B17,국내SCHD형_분배!$C$2:$C$355,"&lt;="&amp;$C17)=0,"",SUMIFS(국내SCHD형_분배!$D$2:$D$355,국내SCHD형_분배!$A$2:$A$355,"446720",국내SCHD형_분배!$C$2:$C$355,"&gt;="&amp;$B17,국내SCHD형_분배!$C$2:$C$355,"&lt;="&amp;$C17))</f>
+        <f>IF(COUNTIFS(국내SCHD형_분배!$A$2:$A$357,"446720",국내SCHD형_분배!$C$2:$C$357,"&gt;="&amp;$B17,국내SCHD형_분배!$C$2:$C$357,"&lt;="&amp;$C17)=0,"",SUMIFS(국내SCHD형_분배!$D$2:$D$357,국내SCHD형_분배!$A$2:$A$357,"446720",국내SCHD형_분배!$C$2:$C$357,"&gt;="&amp;$B17,국내SCHD형_분배!$C$2:$C$357,"&lt;="&amp;$C17))</f>
         <v/>
       </c>
       <c r="F17" s="53">
-        <f>IF(COUNTIFS(국내SCHD형_분배!$A$2:$A$355,"402970",국내SCHD형_분배!$C$2:$C$355,"&gt;="&amp;$B17,국내SCHD형_분배!$C$2:$C$355,"&lt;="&amp;$C17)=0,"",SUMIFS(국내SCHD형_분배!$D$2:$D$355,국내SCHD형_분배!$A$2:$A$355,"402970",국내SCHD형_분배!$C$2:$C$355,"&gt;="&amp;$B17,국내SCHD형_분배!$C$2:$C$355,"&lt;="&amp;$C17))</f>
+        <f>IF(COUNTIFS(국내SCHD형_분배!$A$2:$A$357,"402970",국내SCHD형_분배!$C$2:$C$357,"&gt;="&amp;$B17,국내SCHD형_분배!$C$2:$C$357,"&lt;="&amp;$C17)=0,"",SUMIFS(국내SCHD형_분배!$D$2:$D$357,국내SCHD형_분배!$A$2:$A$357,"402970",국내SCHD형_분배!$C$2:$C$357,"&gt;="&amp;$B17,국내SCHD형_분배!$C$2:$C$357,"&lt;="&amp;$C17))</f>
         <v/>
       </c>
       <c r="G17" s="53">
-        <f>IF(COUNTIFS(국내SCHD형_분배!$A$2:$A$355,"489250",국내SCHD형_분배!$C$2:$C$355,"&gt;="&amp;$B17,국내SCHD형_분배!$C$2:$C$355,"&lt;="&amp;$C17)=0,"",SUMIFS(국내SCHD형_분배!$D$2:$D$355,국내SCHD형_분배!$A$2:$A$355,"489250",국내SCHD형_분배!$C$2:$C$355,"&gt;="&amp;$B17,국내SCHD형_분배!$C$2:$C$355,"&lt;="&amp;$C17))</f>
+        <f>IF(COUNTIFS(국내SCHD형_분배!$A$2:$A$357,"489250",국내SCHD형_분배!$C$2:$C$357,"&gt;="&amp;$B17,국내SCHD형_분배!$C$2:$C$357,"&lt;="&amp;$C17)=0,"",SUMIFS(국내SCHD형_분배!$D$2:$D$357,국내SCHD형_분배!$A$2:$A$357,"489250",국내SCHD형_분배!$C$2:$C$357,"&gt;="&amp;$B17,국내SCHD형_분배!$C$2:$C$357,"&lt;="&amp;$C17))</f>
         <v/>
       </c>
       <c r="H17" s="28">
@@ -25159,19 +25201,19 @@
         <v/>
       </c>
       <c r="D18" s="53">
-        <f>IF(COUNTIFS(국내SCHD형_분배!$A$2:$A$355,"458730",국내SCHD형_분배!$C$2:$C$355,"&gt;="&amp;$B18,국내SCHD형_분배!$C$2:$C$355,"&lt;="&amp;$C18)=0,"",SUMIFS(국내SCHD형_분배!$D$2:$D$355,국내SCHD형_분배!$A$2:$A$355,"458730",국내SCHD형_분배!$C$2:$C$355,"&gt;="&amp;$B18,국내SCHD형_분배!$C$2:$C$355,"&lt;="&amp;$C18))</f>
+        <f>IF(COUNTIFS(국내SCHD형_분배!$A$2:$A$357,"458730",국내SCHD형_분배!$C$2:$C$357,"&gt;="&amp;$B18,국내SCHD형_분배!$C$2:$C$357,"&lt;="&amp;$C18)=0,"",SUMIFS(국내SCHD형_분배!$D$2:$D$357,국내SCHD형_분배!$A$2:$A$357,"458730",국내SCHD형_분배!$C$2:$C$357,"&gt;="&amp;$B18,국내SCHD형_분배!$C$2:$C$357,"&lt;="&amp;$C18))</f>
         <v/>
       </c>
       <c r="E18" s="53">
-        <f>IF(COUNTIFS(국내SCHD형_분배!$A$2:$A$355,"446720",국내SCHD형_분배!$C$2:$C$355,"&gt;="&amp;$B18,국내SCHD형_분배!$C$2:$C$355,"&lt;="&amp;$C18)=0,"",SUMIFS(국내SCHD형_분배!$D$2:$D$355,국내SCHD형_분배!$A$2:$A$355,"446720",국내SCHD형_분배!$C$2:$C$355,"&gt;="&amp;$B18,국내SCHD형_분배!$C$2:$C$355,"&lt;="&amp;$C18))</f>
+        <f>IF(COUNTIFS(국내SCHD형_분배!$A$2:$A$357,"446720",국내SCHD형_분배!$C$2:$C$357,"&gt;="&amp;$B18,국내SCHD형_분배!$C$2:$C$357,"&lt;="&amp;$C18)=0,"",SUMIFS(국내SCHD형_분배!$D$2:$D$357,국내SCHD형_분배!$A$2:$A$357,"446720",국내SCHD형_분배!$C$2:$C$357,"&gt;="&amp;$B18,국내SCHD형_분배!$C$2:$C$357,"&lt;="&amp;$C18))</f>
         <v/>
       </c>
       <c r="F18" s="53">
-        <f>IF(COUNTIFS(국내SCHD형_분배!$A$2:$A$355,"402970",국내SCHD형_분배!$C$2:$C$355,"&gt;="&amp;$B18,국내SCHD형_분배!$C$2:$C$355,"&lt;="&amp;$C18)=0,"",SUMIFS(국내SCHD형_분배!$D$2:$D$355,국내SCHD형_분배!$A$2:$A$355,"402970",국내SCHD형_분배!$C$2:$C$355,"&gt;="&amp;$B18,국내SCHD형_분배!$C$2:$C$355,"&lt;="&amp;$C18))</f>
+        <f>IF(COUNTIFS(국내SCHD형_분배!$A$2:$A$357,"402970",국내SCHD형_분배!$C$2:$C$357,"&gt;="&amp;$B18,국내SCHD형_분배!$C$2:$C$357,"&lt;="&amp;$C18)=0,"",SUMIFS(국내SCHD형_분배!$D$2:$D$357,국내SCHD형_분배!$A$2:$A$357,"402970",국내SCHD형_분배!$C$2:$C$357,"&gt;="&amp;$B18,국내SCHD형_분배!$C$2:$C$357,"&lt;="&amp;$C18))</f>
         <v/>
       </c>
       <c r="G18" s="53">
-        <f>IF(COUNTIFS(국내SCHD형_분배!$A$2:$A$355,"489250",국내SCHD형_분배!$C$2:$C$355,"&gt;="&amp;$B18,국내SCHD형_분배!$C$2:$C$355,"&lt;="&amp;$C18)=0,"",SUMIFS(국내SCHD형_분배!$D$2:$D$355,국내SCHD형_분배!$A$2:$A$355,"489250",국내SCHD형_분배!$C$2:$C$355,"&gt;="&amp;$B18,국내SCHD형_분배!$C$2:$C$355,"&lt;="&amp;$C18))</f>
+        <f>IF(COUNTIFS(국내SCHD형_분배!$A$2:$A$357,"489250",국내SCHD형_분배!$C$2:$C$357,"&gt;="&amp;$B18,국내SCHD형_분배!$C$2:$C$357,"&lt;="&amp;$C18)=0,"",SUMIFS(국내SCHD형_분배!$D$2:$D$357,국내SCHD형_분배!$A$2:$A$357,"489250",국내SCHD형_분배!$C$2:$C$357,"&gt;="&amp;$B18,국내SCHD형_분배!$C$2:$C$357,"&lt;="&amp;$C18))</f>
         <v/>
       </c>
       <c r="H18" s="28">
@@ -25197,19 +25239,19 @@
         <v/>
       </c>
       <c r="D19" s="53">
-        <f>IF(COUNTIFS(국내SCHD형_분배!$A$2:$A$355,"458730",국내SCHD형_분배!$C$2:$C$355,"&gt;="&amp;$B19,국내SCHD형_분배!$C$2:$C$355,"&lt;="&amp;$C19)=0,"",SUMIFS(국내SCHD형_분배!$D$2:$D$355,국내SCHD형_분배!$A$2:$A$355,"458730",국내SCHD형_분배!$C$2:$C$355,"&gt;="&amp;$B19,국내SCHD형_분배!$C$2:$C$355,"&lt;="&amp;$C19))</f>
+        <f>IF(COUNTIFS(국내SCHD형_분배!$A$2:$A$357,"458730",국내SCHD형_분배!$C$2:$C$357,"&gt;="&amp;$B19,국내SCHD형_분배!$C$2:$C$357,"&lt;="&amp;$C19)=0,"",SUMIFS(국내SCHD형_분배!$D$2:$D$357,국내SCHD형_분배!$A$2:$A$357,"458730",국내SCHD형_분배!$C$2:$C$357,"&gt;="&amp;$B19,국내SCHD형_분배!$C$2:$C$357,"&lt;="&amp;$C19))</f>
         <v/>
       </c>
       <c r="E19" s="53">
-        <f>IF(COUNTIFS(국내SCHD형_분배!$A$2:$A$355,"446720",국내SCHD형_분배!$C$2:$C$355,"&gt;="&amp;$B19,국내SCHD형_분배!$C$2:$C$355,"&lt;="&amp;$C19)=0,"",SUMIFS(국내SCHD형_분배!$D$2:$D$355,국내SCHD형_분배!$A$2:$A$355,"446720",국내SCHD형_분배!$C$2:$C$355,"&gt;="&amp;$B19,국내SCHD형_분배!$C$2:$C$355,"&lt;="&amp;$C19))</f>
+        <f>IF(COUNTIFS(국내SCHD형_분배!$A$2:$A$357,"446720",국내SCHD형_분배!$C$2:$C$357,"&gt;="&amp;$B19,국내SCHD형_분배!$C$2:$C$357,"&lt;="&amp;$C19)=0,"",SUMIFS(국내SCHD형_분배!$D$2:$D$357,국내SCHD형_분배!$A$2:$A$357,"446720",국내SCHD형_분배!$C$2:$C$357,"&gt;="&amp;$B19,국내SCHD형_분배!$C$2:$C$357,"&lt;="&amp;$C19))</f>
         <v/>
       </c>
       <c r="F19" s="53">
-        <f>IF(COUNTIFS(국내SCHD형_분배!$A$2:$A$355,"402970",국내SCHD형_분배!$C$2:$C$355,"&gt;="&amp;$B19,국내SCHD형_분배!$C$2:$C$355,"&lt;="&amp;$C19)=0,"",SUMIFS(국내SCHD형_분배!$D$2:$D$355,국내SCHD형_분배!$A$2:$A$355,"402970",국내SCHD형_분배!$C$2:$C$355,"&gt;="&amp;$B19,국내SCHD형_분배!$C$2:$C$355,"&lt;="&amp;$C19))</f>
+        <f>IF(COUNTIFS(국내SCHD형_분배!$A$2:$A$357,"402970",국내SCHD형_분배!$C$2:$C$357,"&gt;="&amp;$B19,국내SCHD형_분배!$C$2:$C$357,"&lt;="&amp;$C19)=0,"",SUMIFS(국내SCHD형_분배!$D$2:$D$357,국내SCHD형_분배!$A$2:$A$357,"402970",국내SCHD형_분배!$C$2:$C$357,"&gt;="&amp;$B19,국내SCHD형_분배!$C$2:$C$357,"&lt;="&amp;$C19))</f>
         <v/>
       </c>
       <c r="G19" s="53">
-        <f>IF(COUNTIFS(국내SCHD형_분배!$A$2:$A$355,"489250",국내SCHD형_분배!$C$2:$C$355,"&gt;="&amp;$B19,국내SCHD형_분배!$C$2:$C$355,"&lt;="&amp;$C19)=0,"",SUMIFS(국내SCHD형_분배!$D$2:$D$355,국내SCHD형_분배!$A$2:$A$355,"489250",국내SCHD형_분배!$C$2:$C$355,"&gt;="&amp;$B19,국내SCHD형_분배!$C$2:$C$355,"&lt;="&amp;$C19))</f>
+        <f>IF(COUNTIFS(국내SCHD형_분배!$A$2:$A$357,"489250",국내SCHD형_분배!$C$2:$C$357,"&gt;="&amp;$B19,국내SCHD형_분배!$C$2:$C$357,"&lt;="&amp;$C19)=0,"",SUMIFS(국내SCHD형_분배!$D$2:$D$357,국내SCHD형_분배!$A$2:$A$357,"489250",국내SCHD형_분배!$C$2:$C$357,"&gt;="&amp;$B19,국내SCHD형_분배!$C$2:$C$357,"&lt;="&amp;$C19))</f>
         <v/>
       </c>
       <c r="H19" s="28">
@@ -25235,19 +25277,19 @@
         <v/>
       </c>
       <c r="D20" s="53">
-        <f>IF(COUNTIFS(국내SCHD형_분배!$A$2:$A$355,"458730",국내SCHD형_분배!$C$2:$C$355,"&gt;="&amp;$B20,국내SCHD형_분배!$C$2:$C$355,"&lt;="&amp;$C20)=0,"",SUMIFS(국내SCHD형_분배!$D$2:$D$355,국내SCHD형_분배!$A$2:$A$355,"458730",국내SCHD형_분배!$C$2:$C$355,"&gt;="&amp;$B20,국내SCHD형_분배!$C$2:$C$355,"&lt;="&amp;$C20))</f>
+        <f>IF(COUNTIFS(국내SCHD형_분배!$A$2:$A$357,"458730",국내SCHD형_분배!$C$2:$C$357,"&gt;="&amp;$B20,국내SCHD형_분배!$C$2:$C$357,"&lt;="&amp;$C20)=0,"",SUMIFS(국내SCHD형_분배!$D$2:$D$357,국내SCHD형_분배!$A$2:$A$357,"458730",국내SCHD형_분배!$C$2:$C$357,"&gt;="&amp;$B20,국내SCHD형_분배!$C$2:$C$357,"&lt;="&amp;$C20))</f>
         <v/>
       </c>
       <c r="E20" s="53">
-        <f>IF(COUNTIFS(국내SCHD형_분배!$A$2:$A$355,"446720",국내SCHD형_분배!$C$2:$C$355,"&gt;="&amp;$B20,국내SCHD형_분배!$C$2:$C$355,"&lt;="&amp;$C20)=0,"",SUMIFS(국내SCHD형_분배!$D$2:$D$355,국내SCHD형_분배!$A$2:$A$355,"446720",국내SCHD형_분배!$C$2:$C$355,"&gt;="&amp;$B20,국내SCHD형_분배!$C$2:$C$355,"&lt;="&amp;$C20))</f>
+        <f>IF(COUNTIFS(국내SCHD형_분배!$A$2:$A$357,"446720",국내SCHD형_분배!$C$2:$C$357,"&gt;="&amp;$B20,국내SCHD형_분배!$C$2:$C$357,"&lt;="&amp;$C20)=0,"",SUMIFS(국내SCHD형_분배!$D$2:$D$357,국내SCHD형_분배!$A$2:$A$357,"446720",국내SCHD형_분배!$C$2:$C$357,"&gt;="&amp;$B20,국내SCHD형_분배!$C$2:$C$357,"&lt;="&amp;$C20))</f>
         <v/>
       </c>
       <c r="F20" s="53">
-        <f>IF(COUNTIFS(국내SCHD형_분배!$A$2:$A$355,"402970",국내SCHD형_분배!$C$2:$C$355,"&gt;="&amp;$B20,국내SCHD형_분배!$C$2:$C$355,"&lt;="&amp;$C20)=0,"",SUMIFS(국내SCHD형_분배!$D$2:$D$355,국내SCHD형_분배!$A$2:$A$355,"402970",국내SCHD형_분배!$C$2:$C$355,"&gt;="&amp;$B20,국내SCHD형_분배!$C$2:$C$355,"&lt;="&amp;$C20))</f>
+        <f>IF(COUNTIFS(국내SCHD형_분배!$A$2:$A$357,"402970",국내SCHD형_분배!$C$2:$C$357,"&gt;="&amp;$B20,국내SCHD형_분배!$C$2:$C$357,"&lt;="&amp;$C20)=0,"",SUMIFS(국내SCHD형_분배!$D$2:$D$357,국내SCHD형_분배!$A$2:$A$357,"402970",국내SCHD형_분배!$C$2:$C$357,"&gt;="&amp;$B20,국내SCHD형_분배!$C$2:$C$357,"&lt;="&amp;$C20))</f>
         <v/>
       </c>
       <c r="G20" s="53">
-        <f>IF(COUNTIFS(국내SCHD형_분배!$A$2:$A$355,"489250",국내SCHD형_분배!$C$2:$C$355,"&gt;="&amp;$B20,국내SCHD형_분배!$C$2:$C$355,"&lt;="&amp;$C20)=0,"",SUMIFS(국내SCHD형_분배!$D$2:$D$355,국내SCHD형_분배!$A$2:$A$355,"489250",국내SCHD형_분배!$C$2:$C$355,"&gt;="&amp;$B20,국내SCHD형_분배!$C$2:$C$355,"&lt;="&amp;$C20))</f>
+        <f>IF(COUNTIFS(국내SCHD형_분배!$A$2:$A$357,"489250",국내SCHD형_분배!$C$2:$C$357,"&gt;="&amp;$B20,국내SCHD형_분배!$C$2:$C$357,"&lt;="&amp;$C20)=0,"",SUMIFS(국내SCHD형_분배!$D$2:$D$357,국내SCHD형_분배!$A$2:$A$357,"489250",국내SCHD형_분배!$C$2:$C$357,"&gt;="&amp;$B20,국내SCHD형_분배!$C$2:$C$357,"&lt;="&amp;$C20))</f>
         <v/>
       </c>
       <c r="H20" s="28">
@@ -25273,19 +25315,19 @@
         <v/>
       </c>
       <c r="D21" s="53">
-        <f>IF(COUNTIFS(국내SCHD형_분배!$A$2:$A$355,"458730",국내SCHD형_분배!$C$2:$C$355,"&gt;="&amp;$B21,국내SCHD형_분배!$C$2:$C$355,"&lt;="&amp;$C21)=0,"",SUMIFS(국내SCHD형_분배!$D$2:$D$355,국내SCHD형_분배!$A$2:$A$355,"458730",국내SCHD형_분배!$C$2:$C$355,"&gt;="&amp;$B21,국내SCHD형_분배!$C$2:$C$355,"&lt;="&amp;$C21))</f>
+        <f>IF(COUNTIFS(국내SCHD형_분배!$A$2:$A$357,"458730",국내SCHD형_분배!$C$2:$C$357,"&gt;="&amp;$B21,국내SCHD형_분배!$C$2:$C$357,"&lt;="&amp;$C21)=0,"",SUMIFS(국내SCHD형_분배!$D$2:$D$357,국내SCHD형_분배!$A$2:$A$357,"458730",국내SCHD형_분배!$C$2:$C$357,"&gt;="&amp;$B21,국내SCHD형_분배!$C$2:$C$357,"&lt;="&amp;$C21))</f>
         <v/>
       </c>
       <c r="E21" s="53">
-        <f>IF(COUNTIFS(국내SCHD형_분배!$A$2:$A$355,"446720",국내SCHD형_분배!$C$2:$C$355,"&gt;="&amp;$B21,국내SCHD형_분배!$C$2:$C$355,"&lt;="&amp;$C21)=0,"",SUMIFS(국내SCHD형_분배!$D$2:$D$355,국내SCHD형_분배!$A$2:$A$355,"446720",국내SCHD형_분배!$C$2:$C$355,"&gt;="&amp;$B21,국내SCHD형_분배!$C$2:$C$355,"&lt;="&amp;$C21))</f>
+        <f>IF(COUNTIFS(국내SCHD형_분배!$A$2:$A$357,"446720",국내SCHD형_분배!$C$2:$C$357,"&gt;="&amp;$B21,국내SCHD형_분배!$C$2:$C$357,"&lt;="&amp;$C21)=0,"",SUMIFS(국내SCHD형_분배!$D$2:$D$357,국내SCHD형_분배!$A$2:$A$357,"446720",국내SCHD형_분배!$C$2:$C$357,"&gt;="&amp;$B21,국내SCHD형_분배!$C$2:$C$357,"&lt;="&amp;$C21))</f>
         <v/>
       </c>
       <c r="F21" s="53">
-        <f>IF(COUNTIFS(국내SCHD형_분배!$A$2:$A$355,"402970",국내SCHD형_분배!$C$2:$C$355,"&gt;="&amp;$B21,국내SCHD형_분배!$C$2:$C$355,"&lt;="&amp;$C21)=0,"",SUMIFS(국내SCHD형_분배!$D$2:$D$355,국내SCHD형_분배!$A$2:$A$355,"402970",국내SCHD형_분배!$C$2:$C$355,"&gt;="&amp;$B21,국내SCHD형_분배!$C$2:$C$355,"&lt;="&amp;$C21))</f>
+        <f>IF(COUNTIFS(국내SCHD형_분배!$A$2:$A$357,"402970",국내SCHD형_분배!$C$2:$C$357,"&gt;="&amp;$B21,국내SCHD형_분배!$C$2:$C$357,"&lt;="&amp;$C21)=0,"",SUMIFS(국내SCHD형_분배!$D$2:$D$357,국내SCHD형_분배!$A$2:$A$357,"402970",국내SCHD형_분배!$C$2:$C$357,"&gt;="&amp;$B21,국내SCHD형_분배!$C$2:$C$357,"&lt;="&amp;$C21))</f>
         <v/>
       </c>
       <c r="G21" s="53">
-        <f>IF(COUNTIFS(국내SCHD형_분배!$A$2:$A$355,"489250",국내SCHD형_분배!$C$2:$C$355,"&gt;="&amp;$B21,국내SCHD형_분배!$C$2:$C$355,"&lt;="&amp;$C21)=0,"",SUMIFS(국내SCHD형_분배!$D$2:$D$355,국내SCHD형_분배!$A$2:$A$355,"489250",국내SCHD형_분배!$C$2:$C$355,"&gt;="&amp;$B21,국내SCHD형_분배!$C$2:$C$355,"&lt;="&amp;$C21))</f>
+        <f>IF(COUNTIFS(국내SCHD형_분배!$A$2:$A$357,"489250",국내SCHD형_분배!$C$2:$C$357,"&gt;="&amp;$B21,국내SCHD형_분배!$C$2:$C$357,"&lt;="&amp;$C21)=0,"",SUMIFS(국내SCHD형_분배!$D$2:$D$357,국내SCHD형_분배!$A$2:$A$357,"489250",국내SCHD형_분배!$C$2:$C$357,"&gt;="&amp;$B21,국내SCHD형_분배!$C$2:$C$357,"&lt;="&amp;$C21))</f>
         <v/>
       </c>
       <c r="H21" s="28">
@@ -25311,19 +25353,19 @@
         <v/>
       </c>
       <c r="D22" s="53">
-        <f>IF(COUNTIFS(국내SCHD형_분배!$A$2:$A$355,"458730",국내SCHD형_분배!$C$2:$C$355,"&gt;="&amp;$B22,국내SCHD형_분배!$C$2:$C$355,"&lt;="&amp;$C22)=0,"",SUMIFS(국내SCHD형_분배!$D$2:$D$355,국내SCHD형_분배!$A$2:$A$355,"458730",국내SCHD형_분배!$C$2:$C$355,"&gt;="&amp;$B22,국내SCHD형_분배!$C$2:$C$355,"&lt;="&amp;$C22))</f>
+        <f>IF(COUNTIFS(국내SCHD형_분배!$A$2:$A$357,"458730",국내SCHD형_분배!$C$2:$C$357,"&gt;="&amp;$B22,국내SCHD형_분배!$C$2:$C$357,"&lt;="&amp;$C22)=0,"",SUMIFS(국내SCHD형_분배!$D$2:$D$357,국내SCHD형_분배!$A$2:$A$357,"458730",국내SCHD형_분배!$C$2:$C$357,"&gt;="&amp;$B22,국내SCHD형_분배!$C$2:$C$357,"&lt;="&amp;$C22))</f>
         <v/>
       </c>
       <c r="E22" s="53">
-        <f>IF(COUNTIFS(국내SCHD형_분배!$A$2:$A$355,"446720",국내SCHD형_분배!$C$2:$C$355,"&gt;="&amp;$B22,국내SCHD형_분배!$C$2:$C$355,"&lt;="&amp;$C22)=0,"",SUMIFS(국내SCHD형_분배!$D$2:$D$355,국내SCHD형_분배!$A$2:$A$355,"446720",국내SCHD형_분배!$C$2:$C$355,"&gt;="&amp;$B22,국내SCHD형_분배!$C$2:$C$355,"&lt;="&amp;$C22))</f>
+        <f>IF(COUNTIFS(국내SCHD형_분배!$A$2:$A$357,"446720",국내SCHD형_분배!$C$2:$C$357,"&gt;="&amp;$B22,국내SCHD형_분배!$C$2:$C$357,"&lt;="&amp;$C22)=0,"",SUMIFS(국내SCHD형_분배!$D$2:$D$357,국내SCHD형_분배!$A$2:$A$357,"446720",국내SCHD형_분배!$C$2:$C$357,"&gt;="&amp;$B22,국내SCHD형_분배!$C$2:$C$357,"&lt;="&amp;$C22))</f>
         <v/>
       </c>
       <c r="F22" s="53">
-        <f>IF(COUNTIFS(국내SCHD형_분배!$A$2:$A$355,"402970",국내SCHD형_분배!$C$2:$C$355,"&gt;="&amp;$B22,국내SCHD형_분배!$C$2:$C$355,"&lt;="&amp;$C22)=0,"",SUMIFS(국내SCHD형_분배!$D$2:$D$355,국내SCHD형_분배!$A$2:$A$355,"402970",국내SCHD형_분배!$C$2:$C$355,"&gt;="&amp;$B22,국내SCHD형_분배!$C$2:$C$355,"&lt;="&amp;$C22))</f>
+        <f>IF(COUNTIFS(국내SCHD형_분배!$A$2:$A$357,"402970",국내SCHD형_분배!$C$2:$C$357,"&gt;="&amp;$B22,국내SCHD형_분배!$C$2:$C$357,"&lt;="&amp;$C22)=0,"",SUMIFS(국내SCHD형_분배!$D$2:$D$357,국내SCHD형_분배!$A$2:$A$357,"402970",국내SCHD형_분배!$C$2:$C$357,"&gt;="&amp;$B22,국내SCHD형_분배!$C$2:$C$357,"&lt;="&amp;$C22))</f>
         <v/>
       </c>
       <c r="G22" s="53">
-        <f>IF(COUNTIFS(국내SCHD형_분배!$A$2:$A$355,"489250",국내SCHD형_분배!$C$2:$C$355,"&gt;="&amp;$B22,국내SCHD형_분배!$C$2:$C$355,"&lt;="&amp;$C22)=0,"",SUMIFS(국내SCHD형_분배!$D$2:$D$355,국내SCHD형_분배!$A$2:$A$355,"489250",국내SCHD형_분배!$C$2:$C$355,"&gt;="&amp;$B22,국내SCHD형_분배!$C$2:$C$355,"&lt;="&amp;$C22))</f>
+        <f>IF(COUNTIFS(국내SCHD형_분배!$A$2:$A$357,"489250",국내SCHD형_분배!$C$2:$C$357,"&gt;="&amp;$B22,국내SCHD형_분배!$C$2:$C$357,"&lt;="&amp;$C22)=0,"",SUMIFS(국내SCHD형_분배!$D$2:$D$357,국내SCHD형_분배!$A$2:$A$357,"489250",국내SCHD형_분배!$C$2:$C$357,"&gt;="&amp;$B22,국내SCHD형_분배!$C$2:$C$357,"&lt;="&amp;$C22))</f>
         <v/>
       </c>
       <c r="H22" s="28">
@@ -25349,19 +25391,19 @@
         <v/>
       </c>
       <c r="D23" s="53">
-        <f>IF(COUNTIFS(국내SCHD형_분배!$A$2:$A$355,"458730",국내SCHD형_분배!$C$2:$C$355,"&gt;="&amp;$B23,국내SCHD형_분배!$C$2:$C$355,"&lt;="&amp;$C23)=0,"",SUMIFS(국내SCHD형_분배!$D$2:$D$355,국내SCHD형_분배!$A$2:$A$355,"458730",국내SCHD형_분배!$C$2:$C$355,"&gt;="&amp;$B23,국내SCHD형_분배!$C$2:$C$355,"&lt;="&amp;$C23))</f>
+        <f>IF(COUNTIFS(국내SCHD형_분배!$A$2:$A$357,"458730",국내SCHD형_분배!$C$2:$C$357,"&gt;="&amp;$B23,국내SCHD형_분배!$C$2:$C$357,"&lt;="&amp;$C23)=0,"",SUMIFS(국내SCHD형_분배!$D$2:$D$357,국내SCHD형_분배!$A$2:$A$357,"458730",국내SCHD형_분배!$C$2:$C$357,"&gt;="&amp;$B23,국내SCHD형_분배!$C$2:$C$357,"&lt;="&amp;$C23))</f>
         <v/>
       </c>
       <c r="E23" s="53">
-        <f>IF(COUNTIFS(국내SCHD형_분배!$A$2:$A$355,"446720",국내SCHD형_분배!$C$2:$C$355,"&gt;="&amp;$B23,국내SCHD형_분배!$C$2:$C$355,"&lt;="&amp;$C23)=0,"",SUMIFS(국내SCHD형_분배!$D$2:$D$355,국내SCHD형_분배!$A$2:$A$355,"446720",국내SCHD형_분배!$C$2:$C$355,"&gt;="&amp;$B23,국내SCHD형_분배!$C$2:$C$355,"&lt;="&amp;$C23))</f>
+        <f>IF(COUNTIFS(국내SCHD형_분배!$A$2:$A$357,"446720",국내SCHD형_분배!$C$2:$C$357,"&gt;="&amp;$B23,국내SCHD형_분배!$C$2:$C$357,"&lt;="&amp;$C23)=0,"",SUMIFS(국내SCHD형_분배!$D$2:$D$357,국내SCHD형_분배!$A$2:$A$357,"446720",국내SCHD형_분배!$C$2:$C$357,"&gt;="&amp;$B23,국내SCHD형_분배!$C$2:$C$357,"&lt;="&amp;$C23))</f>
         <v/>
       </c>
       <c r="F23" s="53">
-        <f>IF(COUNTIFS(국내SCHD형_분배!$A$2:$A$355,"402970",국내SCHD형_분배!$C$2:$C$355,"&gt;="&amp;$B23,국내SCHD형_분배!$C$2:$C$355,"&lt;="&amp;$C23)=0,"",SUMIFS(국내SCHD형_분배!$D$2:$D$355,국내SCHD형_분배!$A$2:$A$355,"402970",국내SCHD형_분배!$C$2:$C$355,"&gt;="&amp;$B23,국내SCHD형_분배!$C$2:$C$355,"&lt;="&amp;$C23))</f>
+        <f>IF(COUNTIFS(국내SCHD형_분배!$A$2:$A$357,"402970",국내SCHD형_분배!$C$2:$C$357,"&gt;="&amp;$B23,국내SCHD형_분배!$C$2:$C$357,"&lt;="&amp;$C23)=0,"",SUMIFS(국내SCHD형_분배!$D$2:$D$357,국내SCHD형_분배!$A$2:$A$357,"402970",국내SCHD형_분배!$C$2:$C$357,"&gt;="&amp;$B23,국내SCHD형_분배!$C$2:$C$357,"&lt;="&amp;$C23))</f>
         <v/>
       </c>
       <c r="G23" s="53">
-        <f>IF(COUNTIFS(국내SCHD형_분배!$A$2:$A$355,"489250",국내SCHD형_분배!$C$2:$C$355,"&gt;="&amp;$B23,국내SCHD형_분배!$C$2:$C$355,"&lt;="&amp;$C23)=0,"",SUMIFS(국내SCHD형_분배!$D$2:$D$355,국내SCHD형_분배!$A$2:$A$355,"489250",국내SCHD형_분배!$C$2:$C$355,"&gt;="&amp;$B23,국내SCHD형_분배!$C$2:$C$355,"&lt;="&amp;$C23))</f>
+        <f>IF(COUNTIFS(국내SCHD형_분배!$A$2:$A$357,"489250",국내SCHD형_분배!$C$2:$C$357,"&gt;="&amp;$B23,국내SCHD형_분배!$C$2:$C$357,"&lt;="&amp;$C23)=0,"",SUMIFS(국내SCHD형_분배!$D$2:$D$357,국내SCHD형_분배!$A$2:$A$357,"489250",국내SCHD형_분배!$C$2:$C$357,"&gt;="&amp;$B23,국내SCHD형_분배!$C$2:$C$357,"&lt;="&amp;$C23))</f>
         <v/>
       </c>
       <c r="H23" s="28">
@@ -25387,19 +25429,19 @@
         <v/>
       </c>
       <c r="D24" s="53">
-        <f>IF(COUNTIFS(국내SCHD형_분배!$A$2:$A$355,"458730",국내SCHD형_분배!$C$2:$C$355,"&gt;="&amp;$B24,국내SCHD형_분배!$C$2:$C$355,"&lt;="&amp;$C24)=0,"",SUMIFS(국내SCHD형_분배!$D$2:$D$355,국내SCHD형_분배!$A$2:$A$355,"458730",국내SCHD형_분배!$C$2:$C$355,"&gt;="&amp;$B24,국내SCHD형_분배!$C$2:$C$355,"&lt;="&amp;$C24))</f>
+        <f>IF(COUNTIFS(국내SCHD형_분배!$A$2:$A$357,"458730",국내SCHD형_분배!$C$2:$C$357,"&gt;="&amp;$B24,국내SCHD형_분배!$C$2:$C$357,"&lt;="&amp;$C24)=0,"",SUMIFS(국내SCHD형_분배!$D$2:$D$357,국내SCHD형_분배!$A$2:$A$357,"458730",국내SCHD형_분배!$C$2:$C$357,"&gt;="&amp;$B24,국내SCHD형_분배!$C$2:$C$357,"&lt;="&amp;$C24))</f>
         <v/>
       </c>
       <c r="E24" s="53">
-        <f>IF(COUNTIFS(국내SCHD형_분배!$A$2:$A$355,"446720",국내SCHD형_분배!$C$2:$C$355,"&gt;="&amp;$B24,국내SCHD형_분배!$C$2:$C$355,"&lt;="&amp;$C24)=0,"",SUMIFS(국내SCHD형_분배!$D$2:$D$355,국내SCHD형_분배!$A$2:$A$355,"446720",국내SCHD형_분배!$C$2:$C$355,"&gt;="&amp;$B24,국내SCHD형_분배!$C$2:$C$355,"&lt;="&amp;$C24))</f>
+        <f>IF(COUNTIFS(국내SCHD형_분배!$A$2:$A$357,"446720",국내SCHD형_분배!$C$2:$C$357,"&gt;="&amp;$B24,국내SCHD형_분배!$C$2:$C$357,"&lt;="&amp;$C24)=0,"",SUMIFS(국내SCHD형_분배!$D$2:$D$357,국내SCHD형_분배!$A$2:$A$357,"446720",국내SCHD형_분배!$C$2:$C$357,"&gt;="&amp;$B24,국내SCHD형_분배!$C$2:$C$357,"&lt;="&amp;$C24))</f>
         <v/>
       </c>
       <c r="F24" s="53">
-        <f>IF(COUNTIFS(국내SCHD형_분배!$A$2:$A$355,"402970",국내SCHD형_분배!$C$2:$C$355,"&gt;="&amp;$B24,국내SCHD형_분배!$C$2:$C$355,"&lt;="&amp;$C24)=0,"",SUMIFS(국내SCHD형_분배!$D$2:$D$355,국내SCHD형_분배!$A$2:$A$355,"402970",국내SCHD형_분배!$C$2:$C$355,"&gt;="&amp;$B24,국내SCHD형_분배!$C$2:$C$355,"&lt;="&amp;$C24))</f>
+        <f>IF(COUNTIFS(국내SCHD형_분배!$A$2:$A$357,"402970",국내SCHD형_분배!$C$2:$C$357,"&gt;="&amp;$B24,국내SCHD형_분배!$C$2:$C$357,"&lt;="&amp;$C24)=0,"",SUMIFS(국내SCHD형_분배!$D$2:$D$357,국내SCHD형_분배!$A$2:$A$357,"402970",국내SCHD형_분배!$C$2:$C$357,"&gt;="&amp;$B24,국내SCHD형_분배!$C$2:$C$357,"&lt;="&amp;$C24))</f>
         <v/>
       </c>
       <c r="G24" s="53">
-        <f>IF(COUNTIFS(국내SCHD형_분배!$A$2:$A$355,"489250",국내SCHD형_분배!$C$2:$C$355,"&gt;="&amp;$B24,국내SCHD형_분배!$C$2:$C$355,"&lt;="&amp;$C24)=0,"",SUMIFS(국내SCHD형_분배!$D$2:$D$355,국내SCHD형_분배!$A$2:$A$355,"489250",국내SCHD형_분배!$C$2:$C$355,"&gt;="&amp;$B24,국내SCHD형_분배!$C$2:$C$355,"&lt;="&amp;$C24))</f>
+        <f>IF(COUNTIFS(국내SCHD형_분배!$A$2:$A$357,"489250",국내SCHD형_분배!$C$2:$C$357,"&gt;="&amp;$B24,국내SCHD형_분배!$C$2:$C$357,"&lt;="&amp;$C24)=0,"",SUMIFS(국내SCHD형_분배!$D$2:$D$357,국내SCHD형_분배!$A$2:$A$357,"489250",국내SCHD형_분배!$C$2:$C$357,"&gt;="&amp;$B24,국내SCHD형_분배!$C$2:$C$357,"&lt;="&amp;$C24))</f>
         <v/>
       </c>
       <c r="H24" s="28">
@@ -25425,19 +25467,19 @@
         <v/>
       </c>
       <c r="D25" s="53">
-        <f>IF(COUNTIFS(국내SCHD형_분배!$A$2:$A$355,"458730",국내SCHD형_분배!$C$2:$C$355,"&gt;="&amp;$B25,국내SCHD형_분배!$C$2:$C$355,"&lt;="&amp;$C25)=0,"",SUMIFS(국내SCHD형_분배!$D$2:$D$355,국내SCHD형_분배!$A$2:$A$355,"458730",국내SCHD형_분배!$C$2:$C$355,"&gt;="&amp;$B25,국내SCHD형_분배!$C$2:$C$355,"&lt;="&amp;$C25))</f>
+        <f>IF(COUNTIFS(국내SCHD형_분배!$A$2:$A$357,"458730",국내SCHD형_분배!$C$2:$C$357,"&gt;="&amp;$B25,국내SCHD형_분배!$C$2:$C$357,"&lt;="&amp;$C25)=0,"",SUMIFS(국내SCHD형_분배!$D$2:$D$357,국내SCHD형_분배!$A$2:$A$357,"458730",국내SCHD형_분배!$C$2:$C$357,"&gt;="&amp;$B25,국내SCHD형_분배!$C$2:$C$357,"&lt;="&amp;$C25))</f>
         <v/>
       </c>
       <c r="E25" s="53">
-        <f>IF(COUNTIFS(국내SCHD형_분배!$A$2:$A$355,"446720",국내SCHD형_분배!$C$2:$C$355,"&gt;="&amp;$B25,국내SCHD형_분배!$C$2:$C$355,"&lt;="&amp;$C25)=0,"",SUMIFS(국내SCHD형_분배!$D$2:$D$355,국내SCHD형_분배!$A$2:$A$355,"446720",국내SCHD형_분배!$C$2:$C$355,"&gt;="&amp;$B25,국내SCHD형_분배!$C$2:$C$355,"&lt;="&amp;$C25))</f>
+        <f>IF(COUNTIFS(국내SCHD형_분배!$A$2:$A$357,"446720",국내SCHD형_분배!$C$2:$C$357,"&gt;="&amp;$B25,국내SCHD형_분배!$C$2:$C$357,"&lt;="&amp;$C25)=0,"",SUMIFS(국내SCHD형_분배!$D$2:$D$357,국내SCHD형_분배!$A$2:$A$357,"446720",국내SCHD형_분배!$C$2:$C$357,"&gt;="&amp;$B25,국내SCHD형_분배!$C$2:$C$357,"&lt;="&amp;$C25))</f>
         <v/>
       </c>
       <c r="F25" s="53">
-        <f>IF(COUNTIFS(국내SCHD형_분배!$A$2:$A$355,"402970",국내SCHD형_분배!$C$2:$C$355,"&gt;="&amp;$B25,국내SCHD형_분배!$C$2:$C$355,"&lt;="&amp;$C25)=0,"",SUMIFS(국내SCHD형_분배!$D$2:$D$355,국내SCHD형_분배!$A$2:$A$355,"402970",국내SCHD형_분배!$C$2:$C$355,"&gt;="&amp;$B25,국내SCHD형_분배!$C$2:$C$355,"&lt;="&amp;$C25))</f>
+        <f>IF(COUNTIFS(국내SCHD형_분배!$A$2:$A$357,"402970",국내SCHD형_분배!$C$2:$C$357,"&gt;="&amp;$B25,국내SCHD형_분배!$C$2:$C$357,"&lt;="&amp;$C25)=0,"",SUMIFS(국내SCHD형_분배!$D$2:$D$357,국내SCHD형_분배!$A$2:$A$357,"402970",국내SCHD형_분배!$C$2:$C$357,"&gt;="&amp;$B25,국내SCHD형_분배!$C$2:$C$357,"&lt;="&amp;$C25))</f>
         <v/>
       </c>
       <c r="G25" s="53">
-        <f>IF(COUNTIFS(국내SCHD형_분배!$A$2:$A$355,"489250",국내SCHD형_분배!$C$2:$C$355,"&gt;="&amp;$B25,국내SCHD형_분배!$C$2:$C$355,"&lt;="&amp;$C25)=0,"",SUMIFS(국내SCHD형_분배!$D$2:$D$355,국내SCHD형_분배!$A$2:$A$355,"489250",국내SCHD형_분배!$C$2:$C$355,"&gt;="&amp;$B25,국내SCHD형_분배!$C$2:$C$355,"&lt;="&amp;$C25))</f>
+        <f>IF(COUNTIFS(국내SCHD형_분배!$A$2:$A$357,"489250",국내SCHD형_분배!$C$2:$C$357,"&gt;="&amp;$B25,국내SCHD형_분배!$C$2:$C$357,"&lt;="&amp;$C25)=0,"",SUMIFS(국내SCHD형_분배!$D$2:$D$357,국내SCHD형_분배!$A$2:$A$357,"489250",국내SCHD형_분배!$C$2:$C$357,"&gt;="&amp;$B25,국내SCHD형_분배!$C$2:$C$357,"&lt;="&amp;$C25))</f>
         <v/>
       </c>
       <c r="H25" s="28">
@@ -25463,19 +25505,19 @@
         <v/>
       </c>
       <c r="D26" s="53">
-        <f>IF(COUNTIFS(국내SCHD형_분배!$A$2:$A$355,"458730",국내SCHD형_분배!$C$2:$C$355,"&gt;="&amp;$B26,국내SCHD형_분배!$C$2:$C$355,"&lt;="&amp;$C26)=0,"",SUMIFS(국내SCHD형_분배!$D$2:$D$355,국내SCHD형_분배!$A$2:$A$355,"458730",국내SCHD형_분배!$C$2:$C$355,"&gt;="&amp;$B26,국내SCHD형_분배!$C$2:$C$355,"&lt;="&amp;$C26))</f>
+        <f>IF(COUNTIFS(국내SCHD형_분배!$A$2:$A$357,"458730",국내SCHD형_분배!$C$2:$C$357,"&gt;="&amp;$B26,국내SCHD형_분배!$C$2:$C$357,"&lt;="&amp;$C26)=0,"",SUMIFS(국내SCHD형_분배!$D$2:$D$357,국내SCHD형_분배!$A$2:$A$357,"458730",국내SCHD형_분배!$C$2:$C$357,"&gt;="&amp;$B26,국내SCHD형_분배!$C$2:$C$357,"&lt;="&amp;$C26))</f>
         <v/>
       </c>
       <c r="E26" s="53">
-        <f>IF(COUNTIFS(국내SCHD형_분배!$A$2:$A$355,"446720",국내SCHD형_분배!$C$2:$C$355,"&gt;="&amp;$B26,국내SCHD형_분배!$C$2:$C$355,"&lt;="&amp;$C26)=0,"",SUMIFS(국내SCHD형_분배!$D$2:$D$355,국내SCHD형_분배!$A$2:$A$355,"446720",국내SCHD형_분배!$C$2:$C$355,"&gt;="&amp;$B26,국내SCHD형_분배!$C$2:$C$355,"&lt;="&amp;$C26))</f>
+        <f>IF(COUNTIFS(국내SCHD형_분배!$A$2:$A$357,"446720",국내SCHD형_분배!$C$2:$C$357,"&gt;="&amp;$B26,국내SCHD형_분배!$C$2:$C$357,"&lt;="&amp;$C26)=0,"",SUMIFS(국내SCHD형_분배!$D$2:$D$357,국내SCHD형_분배!$A$2:$A$357,"446720",국내SCHD형_분배!$C$2:$C$357,"&gt;="&amp;$B26,국내SCHD형_분배!$C$2:$C$357,"&lt;="&amp;$C26))</f>
         <v/>
       </c>
       <c r="F26" s="53">
-        <f>IF(COUNTIFS(국내SCHD형_분배!$A$2:$A$355,"402970",국내SCHD형_분배!$C$2:$C$355,"&gt;="&amp;$B26,국내SCHD형_분배!$C$2:$C$355,"&lt;="&amp;$C26)=0,"",SUMIFS(국내SCHD형_분배!$D$2:$D$355,국내SCHD형_분배!$A$2:$A$355,"402970",국내SCHD형_분배!$C$2:$C$355,"&gt;="&amp;$B26,국내SCHD형_분배!$C$2:$C$355,"&lt;="&amp;$C26))</f>
+        <f>IF(COUNTIFS(국내SCHD형_분배!$A$2:$A$357,"402970",국내SCHD형_분배!$C$2:$C$357,"&gt;="&amp;$B26,국내SCHD형_분배!$C$2:$C$357,"&lt;="&amp;$C26)=0,"",SUMIFS(국내SCHD형_분배!$D$2:$D$357,국내SCHD형_분배!$A$2:$A$357,"402970",국내SCHD형_분배!$C$2:$C$357,"&gt;="&amp;$B26,국내SCHD형_분배!$C$2:$C$357,"&lt;="&amp;$C26))</f>
         <v/>
       </c>
       <c r="G26" s="53">
-        <f>IF(COUNTIFS(국내SCHD형_분배!$A$2:$A$355,"489250",국내SCHD형_분배!$C$2:$C$355,"&gt;="&amp;$B26,국내SCHD형_분배!$C$2:$C$355,"&lt;="&amp;$C26)=0,"",SUMIFS(국내SCHD형_분배!$D$2:$D$355,국내SCHD형_분배!$A$2:$A$355,"489250",국내SCHD형_분배!$C$2:$C$355,"&gt;="&amp;$B26,국내SCHD형_분배!$C$2:$C$355,"&lt;="&amp;$C26))</f>
+        <f>IF(COUNTIFS(국내SCHD형_분배!$A$2:$A$357,"489250",국내SCHD형_분배!$C$2:$C$357,"&gt;="&amp;$B26,국내SCHD형_분배!$C$2:$C$357,"&lt;="&amp;$C26)=0,"",SUMIFS(국내SCHD형_분배!$D$2:$D$357,국내SCHD형_분배!$A$2:$A$357,"489250",국내SCHD형_분배!$C$2:$C$357,"&gt;="&amp;$B26,국내SCHD형_분배!$C$2:$C$357,"&lt;="&amp;$C26))</f>
         <v/>
       </c>
       <c r="H26" s="28">
@@ -25501,19 +25543,19 @@
         <v/>
       </c>
       <c r="D27" s="53">
-        <f>IF(COUNTIFS(국내SCHD형_분배!$A$2:$A$355,"458730",국내SCHD형_분배!$C$2:$C$355,"&gt;="&amp;$B27,국내SCHD형_분배!$C$2:$C$355,"&lt;="&amp;$C27)=0,"",SUMIFS(국내SCHD형_분배!$D$2:$D$355,국내SCHD형_분배!$A$2:$A$355,"458730",국내SCHD형_분배!$C$2:$C$355,"&gt;="&amp;$B27,국내SCHD형_분배!$C$2:$C$355,"&lt;="&amp;$C27))</f>
+        <f>IF(COUNTIFS(국내SCHD형_분배!$A$2:$A$357,"458730",국내SCHD형_분배!$C$2:$C$357,"&gt;="&amp;$B27,국내SCHD형_분배!$C$2:$C$357,"&lt;="&amp;$C27)=0,"",SUMIFS(국내SCHD형_분배!$D$2:$D$357,국내SCHD형_분배!$A$2:$A$357,"458730",국내SCHD형_분배!$C$2:$C$357,"&gt;="&amp;$B27,국내SCHD형_분배!$C$2:$C$357,"&lt;="&amp;$C27))</f>
         <v/>
       </c>
       <c r="E27" s="53">
-        <f>IF(COUNTIFS(국내SCHD형_분배!$A$2:$A$355,"446720",국내SCHD형_분배!$C$2:$C$355,"&gt;="&amp;$B27,국내SCHD형_분배!$C$2:$C$355,"&lt;="&amp;$C27)=0,"",SUMIFS(국내SCHD형_분배!$D$2:$D$355,국내SCHD형_분배!$A$2:$A$355,"446720",국내SCHD형_분배!$C$2:$C$355,"&gt;="&amp;$B27,국내SCHD형_분배!$C$2:$C$355,"&lt;="&amp;$C27))</f>
+        <f>IF(COUNTIFS(국내SCHD형_분배!$A$2:$A$357,"446720",국내SCHD형_분배!$C$2:$C$357,"&gt;="&amp;$B27,국내SCHD형_분배!$C$2:$C$357,"&lt;="&amp;$C27)=0,"",SUMIFS(국내SCHD형_분배!$D$2:$D$357,국내SCHD형_분배!$A$2:$A$357,"446720",국내SCHD형_분배!$C$2:$C$357,"&gt;="&amp;$B27,국내SCHD형_분배!$C$2:$C$357,"&lt;="&amp;$C27))</f>
         <v/>
       </c>
       <c r="F27" s="53">
-        <f>IF(COUNTIFS(국내SCHD형_분배!$A$2:$A$355,"402970",국내SCHD형_분배!$C$2:$C$355,"&gt;="&amp;$B27,국내SCHD형_분배!$C$2:$C$355,"&lt;="&amp;$C27)=0,"",SUMIFS(국내SCHD형_분배!$D$2:$D$355,국내SCHD형_분배!$A$2:$A$355,"402970",국내SCHD형_분배!$C$2:$C$355,"&gt;="&amp;$B27,국내SCHD형_분배!$C$2:$C$355,"&lt;="&amp;$C27))</f>
+        <f>IF(COUNTIFS(국내SCHD형_분배!$A$2:$A$357,"402970",국내SCHD형_분배!$C$2:$C$357,"&gt;="&amp;$B27,국내SCHD형_분배!$C$2:$C$357,"&lt;="&amp;$C27)=0,"",SUMIFS(국내SCHD형_분배!$D$2:$D$357,국내SCHD형_분배!$A$2:$A$357,"402970",국내SCHD형_분배!$C$2:$C$357,"&gt;="&amp;$B27,국내SCHD형_분배!$C$2:$C$357,"&lt;="&amp;$C27))</f>
         <v/>
       </c>
       <c r="G27" s="53">
-        <f>IF(COUNTIFS(국내SCHD형_분배!$A$2:$A$355,"489250",국내SCHD형_분배!$C$2:$C$355,"&gt;="&amp;$B27,국내SCHD형_분배!$C$2:$C$355,"&lt;="&amp;$C27)=0,"",SUMIFS(국내SCHD형_분배!$D$2:$D$355,국내SCHD형_분배!$A$2:$A$355,"489250",국내SCHD형_분배!$C$2:$C$355,"&gt;="&amp;$B27,국내SCHD형_분배!$C$2:$C$355,"&lt;="&amp;$C27))</f>
+        <f>IF(COUNTIFS(국내SCHD형_분배!$A$2:$A$357,"489250",국내SCHD형_분배!$C$2:$C$357,"&gt;="&amp;$B27,국내SCHD형_분배!$C$2:$C$357,"&lt;="&amp;$C27)=0,"",SUMIFS(국내SCHD형_분배!$D$2:$D$357,국내SCHD형_분배!$A$2:$A$357,"489250",국내SCHD형_분배!$C$2:$C$357,"&gt;="&amp;$B27,국내SCHD형_분배!$C$2:$C$357,"&lt;="&amp;$C27))</f>
         <v/>
       </c>
       <c r="H27" s="28">
@@ -25539,19 +25581,19 @@
         <v/>
       </c>
       <c r="D28" s="53">
-        <f>IF(COUNTIFS(국내SCHD형_분배!$A$2:$A$355,"458730",국내SCHD형_분배!$C$2:$C$355,"&gt;="&amp;$B28,국내SCHD형_분배!$C$2:$C$355,"&lt;="&amp;$C28)=0,"",SUMIFS(국내SCHD형_분배!$D$2:$D$355,국내SCHD형_분배!$A$2:$A$355,"458730",국내SCHD형_분배!$C$2:$C$355,"&gt;="&amp;$B28,국내SCHD형_분배!$C$2:$C$355,"&lt;="&amp;$C28))</f>
+        <f>IF(COUNTIFS(국내SCHD형_분배!$A$2:$A$357,"458730",국내SCHD형_분배!$C$2:$C$357,"&gt;="&amp;$B28,국내SCHD형_분배!$C$2:$C$357,"&lt;="&amp;$C28)=0,"",SUMIFS(국내SCHD형_분배!$D$2:$D$357,국내SCHD형_분배!$A$2:$A$357,"458730",국내SCHD형_분배!$C$2:$C$357,"&gt;="&amp;$B28,국내SCHD형_분배!$C$2:$C$357,"&lt;="&amp;$C28))</f>
         <v/>
       </c>
       <c r="E28" s="53">
-        <f>IF(COUNTIFS(국내SCHD형_분배!$A$2:$A$355,"446720",국내SCHD형_분배!$C$2:$C$355,"&gt;="&amp;$B28,국내SCHD형_분배!$C$2:$C$355,"&lt;="&amp;$C28)=0,"",SUMIFS(국내SCHD형_분배!$D$2:$D$355,국내SCHD형_분배!$A$2:$A$355,"446720",국내SCHD형_분배!$C$2:$C$355,"&gt;="&amp;$B28,국내SCHD형_분배!$C$2:$C$355,"&lt;="&amp;$C28))</f>
+        <f>IF(COUNTIFS(국내SCHD형_분배!$A$2:$A$357,"446720",국내SCHD형_분배!$C$2:$C$357,"&gt;="&amp;$B28,국내SCHD형_분배!$C$2:$C$357,"&lt;="&amp;$C28)=0,"",SUMIFS(국내SCHD형_분배!$D$2:$D$357,국내SCHD형_분배!$A$2:$A$357,"446720",국내SCHD형_분배!$C$2:$C$357,"&gt;="&amp;$B28,국내SCHD형_분배!$C$2:$C$357,"&lt;="&amp;$C28))</f>
         <v/>
       </c>
       <c r="F28" s="53">
-        <f>IF(COUNTIFS(국내SCHD형_분배!$A$2:$A$355,"402970",국내SCHD형_분배!$C$2:$C$355,"&gt;="&amp;$B28,국내SCHD형_분배!$C$2:$C$355,"&lt;="&amp;$C28)=0,"",SUMIFS(국내SCHD형_분배!$D$2:$D$355,국내SCHD형_분배!$A$2:$A$355,"402970",국내SCHD형_분배!$C$2:$C$355,"&gt;="&amp;$B28,국내SCHD형_분배!$C$2:$C$355,"&lt;="&amp;$C28))</f>
+        <f>IF(COUNTIFS(국내SCHD형_분배!$A$2:$A$357,"402970",국내SCHD형_분배!$C$2:$C$357,"&gt;="&amp;$B28,국내SCHD형_분배!$C$2:$C$357,"&lt;="&amp;$C28)=0,"",SUMIFS(국내SCHD형_분배!$D$2:$D$357,국내SCHD형_분배!$A$2:$A$357,"402970",국내SCHD형_분배!$C$2:$C$357,"&gt;="&amp;$B28,국내SCHD형_분배!$C$2:$C$357,"&lt;="&amp;$C28))</f>
         <v/>
       </c>
       <c r="G28" s="53">
-        <f>IF(COUNTIFS(국내SCHD형_분배!$A$2:$A$355,"489250",국내SCHD형_분배!$C$2:$C$355,"&gt;="&amp;$B28,국내SCHD형_분배!$C$2:$C$355,"&lt;="&amp;$C28)=0,"",SUMIFS(국내SCHD형_분배!$D$2:$D$355,국내SCHD형_분배!$A$2:$A$355,"489250",국내SCHD형_분배!$C$2:$C$355,"&gt;="&amp;$B28,국내SCHD형_분배!$C$2:$C$355,"&lt;="&amp;$C28))</f>
+        <f>IF(COUNTIFS(국내SCHD형_분배!$A$2:$A$357,"489250",국내SCHD형_분배!$C$2:$C$357,"&gt;="&amp;$B28,국내SCHD형_분배!$C$2:$C$357,"&lt;="&amp;$C28)=0,"",SUMIFS(국내SCHD형_분배!$D$2:$D$357,국내SCHD형_분배!$A$2:$A$357,"489250",국내SCHD형_분배!$C$2:$C$357,"&gt;="&amp;$B28,국내SCHD형_분배!$C$2:$C$357,"&lt;="&amp;$C28))</f>
         <v/>
       </c>
       <c r="H28" s="28">
@@ -25577,19 +25619,19 @@
         <v/>
       </c>
       <c r="D29" s="53">
-        <f>IF(COUNTIFS(국내SCHD형_분배!$A$2:$A$355,"458730",국내SCHD형_분배!$C$2:$C$355,"&gt;="&amp;$B29,국내SCHD형_분배!$C$2:$C$355,"&lt;="&amp;$C29)=0,"",SUMIFS(국내SCHD형_분배!$D$2:$D$355,국내SCHD형_분배!$A$2:$A$355,"458730",국내SCHD형_분배!$C$2:$C$355,"&gt;="&amp;$B29,국내SCHD형_분배!$C$2:$C$355,"&lt;="&amp;$C29))</f>
+        <f>IF(COUNTIFS(국내SCHD형_분배!$A$2:$A$357,"458730",국내SCHD형_분배!$C$2:$C$357,"&gt;="&amp;$B29,국내SCHD형_분배!$C$2:$C$357,"&lt;="&amp;$C29)=0,"",SUMIFS(국내SCHD형_분배!$D$2:$D$357,국내SCHD형_분배!$A$2:$A$357,"458730",국내SCHD형_분배!$C$2:$C$357,"&gt;="&amp;$B29,국내SCHD형_분배!$C$2:$C$357,"&lt;="&amp;$C29))</f>
         <v/>
       </c>
       <c r="E29" s="53">
-        <f>IF(COUNTIFS(국내SCHD형_분배!$A$2:$A$355,"446720",국내SCHD형_분배!$C$2:$C$355,"&gt;="&amp;$B29,국내SCHD형_분배!$C$2:$C$355,"&lt;="&amp;$C29)=0,"",SUMIFS(국내SCHD형_분배!$D$2:$D$355,국내SCHD형_분배!$A$2:$A$355,"446720",국내SCHD형_분배!$C$2:$C$355,"&gt;="&amp;$B29,국내SCHD형_분배!$C$2:$C$355,"&lt;="&amp;$C29))</f>
+        <f>IF(COUNTIFS(국내SCHD형_분배!$A$2:$A$357,"446720",국내SCHD형_분배!$C$2:$C$357,"&gt;="&amp;$B29,국내SCHD형_분배!$C$2:$C$357,"&lt;="&amp;$C29)=0,"",SUMIFS(국내SCHD형_분배!$D$2:$D$357,국내SCHD형_분배!$A$2:$A$357,"446720",국내SCHD형_분배!$C$2:$C$357,"&gt;="&amp;$B29,국내SCHD형_분배!$C$2:$C$357,"&lt;="&amp;$C29))</f>
         <v/>
       </c>
       <c r="F29" s="53">
-        <f>IF(COUNTIFS(국내SCHD형_분배!$A$2:$A$355,"402970",국내SCHD형_분배!$C$2:$C$355,"&gt;="&amp;$B29,국내SCHD형_분배!$C$2:$C$355,"&lt;="&amp;$C29)=0,"",SUMIFS(국내SCHD형_분배!$D$2:$D$355,국내SCHD형_분배!$A$2:$A$355,"402970",국내SCHD형_분배!$C$2:$C$355,"&gt;="&amp;$B29,국내SCHD형_분배!$C$2:$C$355,"&lt;="&amp;$C29))</f>
+        <f>IF(COUNTIFS(국내SCHD형_분배!$A$2:$A$357,"402970",국내SCHD형_분배!$C$2:$C$357,"&gt;="&amp;$B29,국내SCHD형_분배!$C$2:$C$357,"&lt;="&amp;$C29)=0,"",SUMIFS(국내SCHD형_분배!$D$2:$D$357,국내SCHD형_분배!$A$2:$A$357,"402970",국내SCHD형_분배!$C$2:$C$357,"&gt;="&amp;$B29,국내SCHD형_분배!$C$2:$C$357,"&lt;="&amp;$C29))</f>
         <v/>
       </c>
       <c r="G29" s="53">
-        <f>IF(COUNTIFS(국내SCHD형_분배!$A$2:$A$355,"489250",국내SCHD형_분배!$C$2:$C$355,"&gt;="&amp;$B29,국내SCHD형_분배!$C$2:$C$355,"&lt;="&amp;$C29)=0,"",SUMIFS(국내SCHD형_분배!$D$2:$D$355,국내SCHD형_분배!$A$2:$A$355,"489250",국내SCHD형_분배!$C$2:$C$355,"&gt;="&amp;$B29,국내SCHD형_분배!$C$2:$C$355,"&lt;="&amp;$C29))</f>
+        <f>IF(COUNTIFS(국내SCHD형_분배!$A$2:$A$357,"489250",국내SCHD형_분배!$C$2:$C$357,"&gt;="&amp;$B29,국내SCHD형_분배!$C$2:$C$357,"&lt;="&amp;$C29)=0,"",SUMIFS(국내SCHD형_분배!$D$2:$D$357,국내SCHD형_분배!$A$2:$A$357,"489250",국내SCHD형_분배!$C$2:$C$357,"&gt;="&amp;$B29,국내SCHD형_분배!$C$2:$C$357,"&lt;="&amp;$C29))</f>
         <v/>
       </c>
       <c r="H29" s="28">
@@ -25615,19 +25657,19 @@
         <v/>
       </c>
       <c r="D30" s="53">
-        <f>IF(COUNTIFS(국내SCHD형_분배!$A$2:$A$355,"458730",국내SCHD형_분배!$C$2:$C$355,"&gt;="&amp;$B30,국내SCHD형_분배!$C$2:$C$355,"&lt;="&amp;$C30)=0,"",SUMIFS(국내SCHD형_분배!$D$2:$D$355,국내SCHD형_분배!$A$2:$A$355,"458730",국내SCHD형_분배!$C$2:$C$355,"&gt;="&amp;$B30,국내SCHD형_분배!$C$2:$C$355,"&lt;="&amp;$C30))</f>
+        <f>IF(COUNTIFS(국내SCHD형_분배!$A$2:$A$357,"458730",국내SCHD형_분배!$C$2:$C$357,"&gt;="&amp;$B30,국내SCHD형_분배!$C$2:$C$357,"&lt;="&amp;$C30)=0,"",SUMIFS(국내SCHD형_분배!$D$2:$D$357,국내SCHD형_분배!$A$2:$A$357,"458730",국내SCHD형_분배!$C$2:$C$357,"&gt;="&amp;$B30,국내SCHD형_분배!$C$2:$C$357,"&lt;="&amp;$C30))</f>
         <v/>
       </c>
       <c r="E30" s="53">
-        <f>IF(COUNTIFS(국내SCHD형_분배!$A$2:$A$355,"446720",국내SCHD형_분배!$C$2:$C$355,"&gt;="&amp;$B30,국내SCHD형_분배!$C$2:$C$355,"&lt;="&amp;$C30)=0,"",SUMIFS(국내SCHD형_분배!$D$2:$D$355,국내SCHD형_분배!$A$2:$A$355,"446720",국내SCHD형_분배!$C$2:$C$355,"&gt;="&amp;$B30,국내SCHD형_분배!$C$2:$C$355,"&lt;="&amp;$C30))</f>
+        <f>IF(COUNTIFS(국내SCHD형_분배!$A$2:$A$357,"446720",국내SCHD형_분배!$C$2:$C$357,"&gt;="&amp;$B30,국내SCHD형_분배!$C$2:$C$357,"&lt;="&amp;$C30)=0,"",SUMIFS(국내SCHD형_분배!$D$2:$D$357,국내SCHD형_분배!$A$2:$A$357,"446720",국내SCHD형_분배!$C$2:$C$357,"&gt;="&amp;$B30,국내SCHD형_분배!$C$2:$C$357,"&lt;="&amp;$C30))</f>
         <v/>
       </c>
       <c r="F30" s="53">
-        <f>IF(COUNTIFS(국내SCHD형_분배!$A$2:$A$355,"402970",국내SCHD형_분배!$C$2:$C$355,"&gt;="&amp;$B30,국내SCHD형_분배!$C$2:$C$355,"&lt;="&amp;$C30)=0,"",SUMIFS(국내SCHD형_분배!$D$2:$D$355,국내SCHD형_분배!$A$2:$A$355,"402970",국내SCHD형_분배!$C$2:$C$355,"&gt;="&amp;$B30,국내SCHD형_분배!$C$2:$C$355,"&lt;="&amp;$C30))</f>
+        <f>IF(COUNTIFS(국내SCHD형_분배!$A$2:$A$357,"402970",국내SCHD형_분배!$C$2:$C$357,"&gt;="&amp;$B30,국내SCHD형_분배!$C$2:$C$357,"&lt;="&amp;$C30)=0,"",SUMIFS(국내SCHD형_분배!$D$2:$D$357,국내SCHD형_분배!$A$2:$A$357,"402970",국내SCHD형_분배!$C$2:$C$357,"&gt;="&amp;$B30,국내SCHD형_분배!$C$2:$C$357,"&lt;="&amp;$C30))</f>
         <v/>
       </c>
       <c r="G30" s="53">
-        <f>IF(COUNTIFS(국내SCHD형_분배!$A$2:$A$355,"489250",국내SCHD형_분배!$C$2:$C$355,"&gt;="&amp;$B30,국내SCHD형_분배!$C$2:$C$355,"&lt;="&amp;$C30)=0,"",SUMIFS(국내SCHD형_분배!$D$2:$D$355,국내SCHD형_분배!$A$2:$A$355,"489250",국내SCHD형_분배!$C$2:$C$355,"&gt;="&amp;$B30,국내SCHD형_분배!$C$2:$C$355,"&lt;="&amp;$C30))</f>
+        <f>IF(COUNTIFS(국내SCHD형_분배!$A$2:$A$357,"489250",국내SCHD형_분배!$C$2:$C$357,"&gt;="&amp;$B30,국내SCHD형_분배!$C$2:$C$357,"&lt;="&amp;$C30)=0,"",SUMIFS(국내SCHD형_분배!$D$2:$D$357,국내SCHD형_분배!$A$2:$A$357,"489250",국내SCHD형_분배!$C$2:$C$357,"&gt;="&amp;$B30,국내SCHD형_분배!$C$2:$C$357,"&lt;="&amp;$C30))</f>
         <v/>
       </c>
       <c r="H30" s="28">
@@ -25653,19 +25695,19 @@
         <v/>
       </c>
       <c r="D31" s="53">
-        <f>IF(COUNTIFS(국내SCHD형_분배!$A$2:$A$355,"458730",국내SCHD형_분배!$C$2:$C$355,"&gt;="&amp;$B31,국내SCHD형_분배!$C$2:$C$355,"&lt;="&amp;$C31)=0,"",SUMIFS(국내SCHD형_분배!$D$2:$D$355,국내SCHD형_분배!$A$2:$A$355,"458730",국내SCHD형_분배!$C$2:$C$355,"&gt;="&amp;$B31,국내SCHD형_분배!$C$2:$C$355,"&lt;="&amp;$C31))</f>
+        <f>IF(COUNTIFS(국내SCHD형_분배!$A$2:$A$357,"458730",국내SCHD형_분배!$C$2:$C$357,"&gt;="&amp;$B31,국내SCHD형_분배!$C$2:$C$357,"&lt;="&amp;$C31)=0,"",SUMIFS(국내SCHD형_분배!$D$2:$D$357,국내SCHD형_분배!$A$2:$A$357,"458730",국내SCHD형_분배!$C$2:$C$357,"&gt;="&amp;$B31,국내SCHD형_분배!$C$2:$C$357,"&lt;="&amp;$C31))</f>
         <v/>
       </c>
       <c r="E31" s="53">
-        <f>IF(COUNTIFS(국내SCHD형_분배!$A$2:$A$355,"446720",국내SCHD형_분배!$C$2:$C$355,"&gt;="&amp;$B31,국내SCHD형_분배!$C$2:$C$355,"&lt;="&amp;$C31)=0,"",SUMIFS(국내SCHD형_분배!$D$2:$D$355,국내SCHD형_분배!$A$2:$A$355,"446720",국내SCHD형_분배!$C$2:$C$355,"&gt;="&amp;$B31,국내SCHD형_분배!$C$2:$C$355,"&lt;="&amp;$C31))</f>
+        <f>IF(COUNTIFS(국내SCHD형_분배!$A$2:$A$357,"446720",국내SCHD형_분배!$C$2:$C$357,"&gt;="&amp;$B31,국내SCHD형_분배!$C$2:$C$357,"&lt;="&amp;$C31)=0,"",SUMIFS(국내SCHD형_분배!$D$2:$D$357,국내SCHD형_분배!$A$2:$A$357,"446720",국내SCHD형_분배!$C$2:$C$357,"&gt;="&amp;$B31,국내SCHD형_분배!$C$2:$C$357,"&lt;="&amp;$C31))</f>
         <v/>
       </c>
       <c r="F31" s="53">
-        <f>IF(COUNTIFS(국내SCHD형_분배!$A$2:$A$355,"402970",국내SCHD형_분배!$C$2:$C$355,"&gt;="&amp;$B31,국내SCHD형_분배!$C$2:$C$355,"&lt;="&amp;$C31)=0,"",SUMIFS(국내SCHD형_분배!$D$2:$D$355,국내SCHD형_분배!$A$2:$A$355,"402970",국내SCHD형_분배!$C$2:$C$355,"&gt;="&amp;$B31,국내SCHD형_분배!$C$2:$C$355,"&lt;="&amp;$C31))</f>
+        <f>IF(COUNTIFS(국내SCHD형_분배!$A$2:$A$357,"402970",국내SCHD형_분배!$C$2:$C$357,"&gt;="&amp;$B31,국내SCHD형_분배!$C$2:$C$357,"&lt;="&amp;$C31)=0,"",SUMIFS(국내SCHD형_분배!$D$2:$D$357,국내SCHD형_분배!$A$2:$A$357,"402970",국내SCHD형_분배!$C$2:$C$357,"&gt;="&amp;$B31,국내SCHD형_분배!$C$2:$C$357,"&lt;="&amp;$C31))</f>
         <v/>
       </c>
       <c r="G31" s="53">
-        <f>IF(COUNTIFS(국내SCHD형_분배!$A$2:$A$355,"489250",국내SCHD형_분배!$C$2:$C$355,"&gt;="&amp;$B31,국내SCHD형_분배!$C$2:$C$355,"&lt;="&amp;$C31)=0,"",SUMIFS(국내SCHD형_분배!$D$2:$D$355,국내SCHD형_분배!$A$2:$A$355,"489250",국내SCHD형_분배!$C$2:$C$355,"&gt;="&amp;$B31,국내SCHD형_분배!$C$2:$C$355,"&lt;="&amp;$C31))</f>
+        <f>IF(COUNTIFS(국내SCHD형_분배!$A$2:$A$357,"489250",국내SCHD형_분배!$C$2:$C$357,"&gt;="&amp;$B31,국내SCHD형_분배!$C$2:$C$357,"&lt;="&amp;$C31)=0,"",SUMIFS(국내SCHD형_분배!$D$2:$D$357,국내SCHD형_분배!$A$2:$A$357,"489250",국내SCHD형_분배!$C$2:$C$357,"&gt;="&amp;$B31,국내SCHD형_분배!$C$2:$C$357,"&lt;="&amp;$C31))</f>
         <v/>
       </c>
       <c r="H31" s="28">
@@ -25691,19 +25733,19 @@
         <v/>
       </c>
       <c r="D32" s="53">
-        <f>IF(COUNTIFS(국내SCHD형_분배!$A$2:$A$355,"458730",국내SCHD형_분배!$C$2:$C$355,"&gt;="&amp;$B32,국내SCHD형_분배!$C$2:$C$355,"&lt;="&amp;$C32)=0,"",SUMIFS(국내SCHD형_분배!$D$2:$D$355,국내SCHD형_분배!$A$2:$A$355,"458730",국내SCHD형_분배!$C$2:$C$355,"&gt;="&amp;$B32,국내SCHD형_분배!$C$2:$C$355,"&lt;="&amp;$C32))</f>
+        <f>IF(COUNTIFS(국내SCHD형_분배!$A$2:$A$357,"458730",국내SCHD형_분배!$C$2:$C$357,"&gt;="&amp;$B32,국내SCHD형_분배!$C$2:$C$357,"&lt;="&amp;$C32)=0,"",SUMIFS(국내SCHD형_분배!$D$2:$D$357,국내SCHD형_분배!$A$2:$A$357,"458730",국내SCHD형_분배!$C$2:$C$357,"&gt;="&amp;$B32,국내SCHD형_분배!$C$2:$C$357,"&lt;="&amp;$C32))</f>
         <v/>
       </c>
       <c r="E32" s="53">
-        <f>IF(COUNTIFS(국내SCHD형_분배!$A$2:$A$355,"446720",국내SCHD형_분배!$C$2:$C$355,"&gt;="&amp;$B32,국내SCHD형_분배!$C$2:$C$355,"&lt;="&amp;$C32)=0,"",SUMIFS(국내SCHD형_분배!$D$2:$D$355,국내SCHD형_분배!$A$2:$A$355,"446720",국내SCHD형_분배!$C$2:$C$355,"&gt;="&amp;$B32,국내SCHD형_분배!$C$2:$C$355,"&lt;="&amp;$C32))</f>
+        <f>IF(COUNTIFS(국내SCHD형_분배!$A$2:$A$357,"446720",국내SCHD형_분배!$C$2:$C$357,"&gt;="&amp;$B32,국내SCHD형_분배!$C$2:$C$357,"&lt;="&amp;$C32)=0,"",SUMIFS(국내SCHD형_분배!$D$2:$D$357,국내SCHD형_분배!$A$2:$A$357,"446720",국내SCHD형_분배!$C$2:$C$357,"&gt;="&amp;$B32,국내SCHD형_분배!$C$2:$C$357,"&lt;="&amp;$C32))</f>
         <v/>
       </c>
       <c r="F32" s="53">
-        <f>IF(COUNTIFS(국내SCHD형_분배!$A$2:$A$355,"402970",국내SCHD형_분배!$C$2:$C$355,"&gt;="&amp;$B32,국내SCHD형_분배!$C$2:$C$355,"&lt;="&amp;$C32)=0,"",SUMIFS(국내SCHD형_분배!$D$2:$D$355,국내SCHD형_분배!$A$2:$A$355,"402970",국내SCHD형_분배!$C$2:$C$355,"&gt;="&amp;$B32,국내SCHD형_분배!$C$2:$C$355,"&lt;="&amp;$C32))</f>
+        <f>IF(COUNTIFS(국내SCHD형_분배!$A$2:$A$357,"402970",국내SCHD형_분배!$C$2:$C$357,"&gt;="&amp;$B32,국내SCHD형_분배!$C$2:$C$357,"&lt;="&amp;$C32)=0,"",SUMIFS(국내SCHD형_분배!$D$2:$D$357,국내SCHD형_분배!$A$2:$A$357,"402970",국내SCHD형_분배!$C$2:$C$357,"&gt;="&amp;$B32,국내SCHD형_분배!$C$2:$C$357,"&lt;="&amp;$C32))</f>
         <v/>
       </c>
       <c r="G32" s="53">
-        <f>IF(COUNTIFS(국내SCHD형_분배!$A$2:$A$355,"489250",국내SCHD형_분배!$C$2:$C$355,"&gt;="&amp;$B32,국내SCHD형_분배!$C$2:$C$355,"&lt;="&amp;$C32)=0,"",SUMIFS(국내SCHD형_분배!$D$2:$D$355,국내SCHD형_분배!$A$2:$A$355,"489250",국내SCHD형_분배!$C$2:$C$355,"&gt;="&amp;$B32,국내SCHD형_분배!$C$2:$C$355,"&lt;="&amp;$C32))</f>
+        <f>IF(COUNTIFS(국내SCHD형_분배!$A$2:$A$357,"489250",국내SCHD형_분배!$C$2:$C$357,"&gt;="&amp;$B32,국내SCHD형_분배!$C$2:$C$357,"&lt;="&amp;$C32)=0,"",SUMIFS(국내SCHD형_분배!$D$2:$D$357,국내SCHD형_분배!$A$2:$A$357,"489250",국내SCHD형_분배!$C$2:$C$357,"&gt;="&amp;$B32,국내SCHD형_분배!$C$2:$C$357,"&lt;="&amp;$C32))</f>
         <v/>
       </c>
       <c r="H32" s="28">
@@ -25729,19 +25771,19 @@
         <v/>
       </c>
       <c r="D33" s="53">
-        <f>IF(COUNTIFS(국내SCHD형_분배!$A$2:$A$355,"458730",국내SCHD형_분배!$C$2:$C$355,"&gt;="&amp;$B33,국내SCHD형_분배!$C$2:$C$355,"&lt;="&amp;$C33)=0,"",SUMIFS(국내SCHD형_분배!$D$2:$D$355,국내SCHD형_분배!$A$2:$A$355,"458730",국내SCHD형_분배!$C$2:$C$355,"&gt;="&amp;$B33,국내SCHD형_분배!$C$2:$C$355,"&lt;="&amp;$C33))</f>
+        <f>IF(COUNTIFS(국내SCHD형_분배!$A$2:$A$357,"458730",국내SCHD형_분배!$C$2:$C$357,"&gt;="&amp;$B33,국내SCHD형_분배!$C$2:$C$357,"&lt;="&amp;$C33)=0,"",SUMIFS(국내SCHD형_분배!$D$2:$D$357,국내SCHD형_분배!$A$2:$A$357,"458730",국내SCHD형_분배!$C$2:$C$357,"&gt;="&amp;$B33,국내SCHD형_분배!$C$2:$C$357,"&lt;="&amp;$C33))</f>
         <v/>
       </c>
       <c r="E33" s="53">
-        <f>IF(COUNTIFS(국내SCHD형_분배!$A$2:$A$355,"446720",국내SCHD형_분배!$C$2:$C$355,"&gt;="&amp;$B33,국내SCHD형_분배!$C$2:$C$355,"&lt;="&amp;$C33)=0,"",SUMIFS(국내SCHD형_분배!$D$2:$D$355,국내SCHD형_분배!$A$2:$A$355,"446720",국내SCHD형_분배!$C$2:$C$355,"&gt;="&amp;$B33,국내SCHD형_분배!$C$2:$C$355,"&lt;="&amp;$C33))</f>
+        <f>IF(COUNTIFS(국내SCHD형_분배!$A$2:$A$357,"446720",국내SCHD형_분배!$C$2:$C$357,"&gt;="&amp;$B33,국내SCHD형_분배!$C$2:$C$357,"&lt;="&amp;$C33)=0,"",SUMIFS(국내SCHD형_분배!$D$2:$D$357,국내SCHD형_분배!$A$2:$A$357,"446720",국내SCHD형_분배!$C$2:$C$357,"&gt;="&amp;$B33,국내SCHD형_분배!$C$2:$C$357,"&lt;="&amp;$C33))</f>
         <v/>
       </c>
       <c r="F33" s="53">
-        <f>IF(COUNTIFS(국내SCHD형_분배!$A$2:$A$355,"402970",국내SCHD형_분배!$C$2:$C$355,"&gt;="&amp;$B33,국내SCHD형_분배!$C$2:$C$355,"&lt;="&amp;$C33)=0,"",SUMIFS(국내SCHD형_분배!$D$2:$D$355,국내SCHD형_분배!$A$2:$A$355,"402970",국내SCHD형_분배!$C$2:$C$355,"&gt;="&amp;$B33,국내SCHD형_분배!$C$2:$C$355,"&lt;="&amp;$C33))</f>
+        <f>IF(COUNTIFS(국내SCHD형_분배!$A$2:$A$357,"402970",국내SCHD형_분배!$C$2:$C$357,"&gt;="&amp;$B33,국내SCHD형_분배!$C$2:$C$357,"&lt;="&amp;$C33)=0,"",SUMIFS(국내SCHD형_분배!$D$2:$D$357,국내SCHD형_분배!$A$2:$A$357,"402970",국내SCHD형_분배!$C$2:$C$357,"&gt;="&amp;$B33,국내SCHD형_분배!$C$2:$C$357,"&lt;="&amp;$C33))</f>
         <v/>
       </c>
       <c r="G33" s="53">
-        <f>IF(COUNTIFS(국내SCHD형_분배!$A$2:$A$355,"489250",국내SCHD형_분배!$C$2:$C$355,"&gt;="&amp;$B33,국내SCHD형_분배!$C$2:$C$355,"&lt;="&amp;$C33)=0,"",SUMIFS(국내SCHD형_분배!$D$2:$D$355,국내SCHD형_분배!$A$2:$A$355,"489250",국내SCHD형_분배!$C$2:$C$355,"&gt;="&amp;$B33,국내SCHD형_분배!$C$2:$C$355,"&lt;="&amp;$C33))</f>
+        <f>IF(COUNTIFS(국내SCHD형_분배!$A$2:$A$357,"489250",국내SCHD형_분배!$C$2:$C$357,"&gt;="&amp;$B33,국내SCHD형_분배!$C$2:$C$357,"&lt;="&amp;$C33)=0,"",SUMIFS(국내SCHD형_분배!$D$2:$D$357,국내SCHD형_분배!$A$2:$A$357,"489250",국내SCHD형_분배!$C$2:$C$357,"&gt;="&amp;$B33,국내SCHD형_분배!$C$2:$C$357,"&lt;="&amp;$C33))</f>
         <v/>
       </c>
       <c r="H33" s="28">
@@ -25767,19 +25809,19 @@
         <v/>
       </c>
       <c r="D34" s="53">
-        <f>IF(COUNTIFS(국내SCHD형_분배!$A$2:$A$355,"458730",국내SCHD형_분배!$C$2:$C$355,"&gt;="&amp;$B34,국내SCHD형_분배!$C$2:$C$355,"&lt;="&amp;$C34)=0,"",SUMIFS(국내SCHD형_분배!$D$2:$D$355,국내SCHD형_분배!$A$2:$A$355,"458730",국내SCHD형_분배!$C$2:$C$355,"&gt;="&amp;$B34,국내SCHD형_분배!$C$2:$C$355,"&lt;="&amp;$C34))</f>
+        <f>IF(COUNTIFS(국내SCHD형_분배!$A$2:$A$357,"458730",국내SCHD형_분배!$C$2:$C$357,"&gt;="&amp;$B34,국내SCHD형_분배!$C$2:$C$357,"&lt;="&amp;$C34)=0,"",SUMIFS(국내SCHD형_분배!$D$2:$D$357,국내SCHD형_분배!$A$2:$A$357,"458730",국내SCHD형_분배!$C$2:$C$357,"&gt;="&amp;$B34,국내SCHD형_분배!$C$2:$C$357,"&lt;="&amp;$C34))</f>
         <v/>
       </c>
       <c r="E34" s="53">
-        <f>IF(COUNTIFS(국내SCHD형_분배!$A$2:$A$355,"446720",국내SCHD형_분배!$C$2:$C$355,"&gt;="&amp;$B34,국내SCHD형_분배!$C$2:$C$355,"&lt;="&amp;$C34)=0,"",SUMIFS(국내SCHD형_분배!$D$2:$D$355,국내SCHD형_분배!$A$2:$A$355,"446720",국내SCHD형_분배!$C$2:$C$355,"&gt;="&amp;$B34,국내SCHD형_분배!$C$2:$C$355,"&lt;="&amp;$C34))</f>
+        <f>IF(COUNTIFS(국내SCHD형_분배!$A$2:$A$357,"446720",국내SCHD형_분배!$C$2:$C$357,"&gt;="&amp;$B34,국내SCHD형_분배!$C$2:$C$357,"&lt;="&amp;$C34)=0,"",SUMIFS(국내SCHD형_분배!$D$2:$D$357,국내SCHD형_분배!$A$2:$A$357,"446720",국내SCHD형_분배!$C$2:$C$357,"&gt;="&amp;$B34,국내SCHD형_분배!$C$2:$C$357,"&lt;="&amp;$C34))</f>
         <v/>
       </c>
       <c r="F34" s="53">
-        <f>IF(COUNTIFS(국내SCHD형_분배!$A$2:$A$355,"402970",국내SCHD형_분배!$C$2:$C$355,"&gt;="&amp;$B34,국내SCHD형_분배!$C$2:$C$355,"&lt;="&amp;$C34)=0,"",SUMIFS(국내SCHD형_분배!$D$2:$D$355,국내SCHD형_분배!$A$2:$A$355,"402970",국내SCHD형_분배!$C$2:$C$355,"&gt;="&amp;$B34,국내SCHD형_분배!$C$2:$C$355,"&lt;="&amp;$C34))</f>
+        <f>IF(COUNTIFS(국내SCHD형_분배!$A$2:$A$357,"402970",국내SCHD형_분배!$C$2:$C$357,"&gt;="&amp;$B34,국내SCHD형_분배!$C$2:$C$357,"&lt;="&amp;$C34)=0,"",SUMIFS(국내SCHD형_분배!$D$2:$D$357,국내SCHD형_분배!$A$2:$A$357,"402970",국내SCHD형_분배!$C$2:$C$357,"&gt;="&amp;$B34,국내SCHD형_분배!$C$2:$C$357,"&lt;="&amp;$C34))</f>
         <v/>
       </c>
       <c r="G34" s="53">
-        <f>IF(COUNTIFS(국내SCHD형_분배!$A$2:$A$355,"489250",국내SCHD형_분배!$C$2:$C$355,"&gt;="&amp;$B34,국내SCHD형_분배!$C$2:$C$355,"&lt;="&amp;$C34)=0,"",SUMIFS(국내SCHD형_분배!$D$2:$D$355,국내SCHD형_분배!$A$2:$A$355,"489250",국내SCHD형_분배!$C$2:$C$355,"&gt;="&amp;$B34,국내SCHD형_분배!$C$2:$C$355,"&lt;="&amp;$C34))</f>
+        <f>IF(COUNTIFS(국내SCHD형_분배!$A$2:$A$357,"489250",국내SCHD형_분배!$C$2:$C$357,"&gt;="&amp;$B34,국내SCHD형_분배!$C$2:$C$357,"&lt;="&amp;$C34)=0,"",SUMIFS(국내SCHD형_분배!$D$2:$D$357,국내SCHD형_분배!$A$2:$A$357,"489250",국내SCHD형_분배!$C$2:$C$357,"&gt;="&amp;$B34,국내SCHD형_분배!$C$2:$C$357,"&lt;="&amp;$C34))</f>
         <v/>
       </c>
       <c r="H34" s="28">
@@ -25805,19 +25847,19 @@
         <v/>
       </c>
       <c r="D35" s="53">
-        <f>IF(COUNTIFS(국내SCHD형_분배!$A$2:$A$355,"458730",국내SCHD형_분배!$C$2:$C$355,"&gt;="&amp;$B35,국내SCHD형_분배!$C$2:$C$355,"&lt;="&amp;$C35)=0,"",SUMIFS(국내SCHD형_분배!$D$2:$D$355,국내SCHD형_분배!$A$2:$A$355,"458730",국내SCHD형_분배!$C$2:$C$355,"&gt;="&amp;$B35,국내SCHD형_분배!$C$2:$C$355,"&lt;="&amp;$C35))</f>
+        <f>IF(COUNTIFS(국내SCHD형_분배!$A$2:$A$357,"458730",국내SCHD형_분배!$C$2:$C$357,"&gt;="&amp;$B35,국내SCHD형_분배!$C$2:$C$357,"&lt;="&amp;$C35)=0,"",SUMIFS(국내SCHD형_분배!$D$2:$D$357,국내SCHD형_분배!$A$2:$A$357,"458730",국내SCHD형_분배!$C$2:$C$357,"&gt;="&amp;$B35,국내SCHD형_분배!$C$2:$C$357,"&lt;="&amp;$C35))</f>
         <v/>
       </c>
       <c r="E35" s="53">
-        <f>IF(COUNTIFS(국내SCHD형_분배!$A$2:$A$355,"446720",국내SCHD형_분배!$C$2:$C$355,"&gt;="&amp;$B35,국내SCHD형_분배!$C$2:$C$355,"&lt;="&amp;$C35)=0,"",SUMIFS(국내SCHD형_분배!$D$2:$D$355,국내SCHD형_분배!$A$2:$A$355,"446720",국내SCHD형_분배!$C$2:$C$355,"&gt;="&amp;$B35,국내SCHD형_분배!$C$2:$C$355,"&lt;="&amp;$C35))</f>
+        <f>IF(COUNTIFS(국내SCHD형_분배!$A$2:$A$357,"446720",국내SCHD형_분배!$C$2:$C$357,"&gt;="&amp;$B35,국내SCHD형_분배!$C$2:$C$357,"&lt;="&amp;$C35)=0,"",SUMIFS(국내SCHD형_분배!$D$2:$D$357,국내SCHD형_분배!$A$2:$A$357,"446720",국내SCHD형_분배!$C$2:$C$357,"&gt;="&amp;$B35,국내SCHD형_분배!$C$2:$C$357,"&lt;="&amp;$C35))</f>
         <v/>
       </c>
       <c r="F35" s="53">
-        <f>IF(COUNTIFS(국내SCHD형_분배!$A$2:$A$355,"402970",국내SCHD형_분배!$C$2:$C$355,"&gt;="&amp;$B35,국내SCHD형_분배!$C$2:$C$355,"&lt;="&amp;$C35)=0,"",SUMIFS(국내SCHD형_분배!$D$2:$D$355,국내SCHD형_분배!$A$2:$A$355,"402970",국내SCHD형_분배!$C$2:$C$355,"&gt;="&amp;$B35,국내SCHD형_분배!$C$2:$C$355,"&lt;="&amp;$C35))</f>
+        <f>IF(COUNTIFS(국내SCHD형_분배!$A$2:$A$357,"402970",국내SCHD형_분배!$C$2:$C$357,"&gt;="&amp;$B35,국내SCHD형_분배!$C$2:$C$357,"&lt;="&amp;$C35)=0,"",SUMIFS(국내SCHD형_분배!$D$2:$D$357,국내SCHD형_분배!$A$2:$A$357,"402970",국내SCHD형_분배!$C$2:$C$357,"&gt;="&amp;$B35,국내SCHD형_분배!$C$2:$C$357,"&lt;="&amp;$C35))</f>
         <v/>
       </c>
       <c r="G35" s="53">
-        <f>IF(COUNTIFS(국내SCHD형_분배!$A$2:$A$355,"489250",국내SCHD형_분배!$C$2:$C$355,"&gt;="&amp;$B35,국내SCHD형_분배!$C$2:$C$355,"&lt;="&amp;$C35)=0,"",SUMIFS(국내SCHD형_분배!$D$2:$D$355,국내SCHD형_분배!$A$2:$A$355,"489250",국내SCHD형_분배!$C$2:$C$355,"&gt;="&amp;$B35,국내SCHD형_분배!$C$2:$C$355,"&lt;="&amp;$C35))</f>
+        <f>IF(COUNTIFS(국내SCHD형_분배!$A$2:$A$357,"489250",국내SCHD형_분배!$C$2:$C$357,"&gt;="&amp;$B35,국내SCHD형_분배!$C$2:$C$357,"&lt;="&amp;$C35)=0,"",SUMIFS(국내SCHD형_분배!$D$2:$D$357,국내SCHD형_분배!$A$2:$A$357,"489250",국내SCHD형_분배!$C$2:$C$357,"&gt;="&amp;$B35,국내SCHD형_분배!$C$2:$C$357,"&lt;="&amp;$C35))</f>
         <v/>
       </c>
       <c r="H35" s="28">
@@ -25843,19 +25885,19 @@
         <v/>
       </c>
       <c r="D36" s="53">
-        <f>IF(COUNTIFS(국내SCHD형_분배!$A$2:$A$355,"458730",국내SCHD형_분배!$C$2:$C$355,"&gt;="&amp;$B36,국내SCHD형_분배!$C$2:$C$355,"&lt;="&amp;$C36)=0,"",SUMIFS(국내SCHD형_분배!$D$2:$D$355,국내SCHD형_분배!$A$2:$A$355,"458730",국내SCHD형_분배!$C$2:$C$355,"&gt;="&amp;$B36,국내SCHD형_분배!$C$2:$C$355,"&lt;="&amp;$C36))</f>
+        <f>IF(COUNTIFS(국내SCHD형_분배!$A$2:$A$357,"458730",국내SCHD형_분배!$C$2:$C$357,"&gt;="&amp;$B36,국내SCHD형_분배!$C$2:$C$357,"&lt;="&amp;$C36)=0,"",SUMIFS(국내SCHD형_분배!$D$2:$D$357,국내SCHD형_분배!$A$2:$A$357,"458730",국내SCHD형_분배!$C$2:$C$357,"&gt;="&amp;$B36,국내SCHD형_분배!$C$2:$C$357,"&lt;="&amp;$C36))</f>
         <v/>
       </c>
       <c r="E36" s="53">
-        <f>IF(COUNTIFS(국내SCHD형_분배!$A$2:$A$355,"446720",국내SCHD형_분배!$C$2:$C$355,"&gt;="&amp;$B36,국내SCHD형_분배!$C$2:$C$355,"&lt;="&amp;$C36)=0,"",SUMIFS(국내SCHD형_분배!$D$2:$D$355,국내SCHD형_분배!$A$2:$A$355,"446720",국내SCHD형_분배!$C$2:$C$355,"&gt;="&amp;$B36,국내SCHD형_분배!$C$2:$C$355,"&lt;="&amp;$C36))</f>
+        <f>IF(COUNTIFS(국내SCHD형_분배!$A$2:$A$357,"446720",국내SCHD형_분배!$C$2:$C$357,"&gt;="&amp;$B36,국내SCHD형_분배!$C$2:$C$357,"&lt;="&amp;$C36)=0,"",SUMIFS(국내SCHD형_분배!$D$2:$D$357,국내SCHD형_분배!$A$2:$A$357,"446720",국내SCHD형_분배!$C$2:$C$357,"&gt;="&amp;$B36,국내SCHD형_분배!$C$2:$C$357,"&lt;="&amp;$C36))</f>
         <v/>
       </c>
       <c r="F36" s="53">
-        <f>IF(COUNTIFS(국내SCHD형_분배!$A$2:$A$355,"402970",국내SCHD형_분배!$C$2:$C$355,"&gt;="&amp;$B36,국내SCHD형_분배!$C$2:$C$355,"&lt;="&amp;$C36)=0,"",SUMIFS(국내SCHD형_분배!$D$2:$D$355,국내SCHD형_분배!$A$2:$A$355,"402970",국내SCHD형_분배!$C$2:$C$355,"&gt;="&amp;$B36,국내SCHD형_분배!$C$2:$C$355,"&lt;="&amp;$C36))</f>
+        <f>IF(COUNTIFS(국내SCHD형_분배!$A$2:$A$357,"402970",국내SCHD형_분배!$C$2:$C$357,"&gt;="&amp;$B36,국내SCHD형_분배!$C$2:$C$357,"&lt;="&amp;$C36)=0,"",SUMIFS(국내SCHD형_분배!$D$2:$D$357,국내SCHD형_분배!$A$2:$A$357,"402970",국내SCHD형_분배!$C$2:$C$357,"&gt;="&amp;$B36,국내SCHD형_분배!$C$2:$C$357,"&lt;="&amp;$C36))</f>
         <v/>
       </c>
       <c r="G36" s="53">
-        <f>IF(COUNTIFS(국내SCHD형_분배!$A$2:$A$355,"489250",국내SCHD형_분배!$C$2:$C$355,"&gt;="&amp;$B36,국내SCHD형_분배!$C$2:$C$355,"&lt;="&amp;$C36)=0,"",SUMIFS(국내SCHD형_분배!$D$2:$D$355,국내SCHD형_분배!$A$2:$A$355,"489250",국내SCHD형_분배!$C$2:$C$355,"&gt;="&amp;$B36,국내SCHD형_분배!$C$2:$C$355,"&lt;="&amp;$C36))</f>
+        <f>IF(COUNTIFS(국내SCHD형_분배!$A$2:$A$357,"489250",국내SCHD형_분배!$C$2:$C$357,"&gt;="&amp;$B36,국내SCHD형_분배!$C$2:$C$357,"&lt;="&amp;$C36)=0,"",SUMIFS(국내SCHD형_분배!$D$2:$D$357,국내SCHD형_분배!$A$2:$A$357,"489250",국내SCHD형_분배!$C$2:$C$357,"&gt;="&amp;$B36,국내SCHD형_분배!$C$2:$C$357,"&lt;="&amp;$C36))</f>
         <v/>
       </c>
       <c r="H36" s="28">
@@ -25881,19 +25923,19 @@
         <v/>
       </c>
       <c r="D37" s="53">
-        <f>IF(COUNTIFS(국내SCHD형_분배!$A$2:$A$355,"458730",국내SCHD형_분배!$C$2:$C$355,"&gt;="&amp;$B37,국내SCHD형_분배!$C$2:$C$355,"&lt;="&amp;$C37)=0,"",SUMIFS(국내SCHD형_분배!$D$2:$D$355,국내SCHD형_분배!$A$2:$A$355,"458730",국내SCHD형_분배!$C$2:$C$355,"&gt;="&amp;$B37,국내SCHD형_분배!$C$2:$C$355,"&lt;="&amp;$C37))</f>
+        <f>IF(COUNTIFS(국내SCHD형_분배!$A$2:$A$357,"458730",국내SCHD형_분배!$C$2:$C$357,"&gt;="&amp;$B37,국내SCHD형_분배!$C$2:$C$357,"&lt;="&amp;$C37)=0,"",SUMIFS(국내SCHD형_분배!$D$2:$D$357,국내SCHD형_분배!$A$2:$A$357,"458730",국내SCHD형_분배!$C$2:$C$357,"&gt;="&amp;$B37,국내SCHD형_분배!$C$2:$C$357,"&lt;="&amp;$C37))</f>
         <v/>
       </c>
       <c r="E37" s="53">
-        <f>IF(COUNTIFS(국내SCHD형_분배!$A$2:$A$355,"446720",국내SCHD형_분배!$C$2:$C$355,"&gt;="&amp;$B37,국내SCHD형_분배!$C$2:$C$355,"&lt;="&amp;$C37)=0,"",SUMIFS(국내SCHD형_분배!$D$2:$D$355,국내SCHD형_분배!$A$2:$A$355,"446720",국내SCHD형_분배!$C$2:$C$355,"&gt;="&amp;$B37,국내SCHD형_분배!$C$2:$C$355,"&lt;="&amp;$C37))</f>
+        <f>IF(COUNTIFS(국내SCHD형_분배!$A$2:$A$357,"446720",국내SCHD형_분배!$C$2:$C$357,"&gt;="&amp;$B37,국내SCHD형_분배!$C$2:$C$357,"&lt;="&amp;$C37)=0,"",SUMIFS(국내SCHD형_분배!$D$2:$D$357,국내SCHD형_분배!$A$2:$A$357,"446720",국내SCHD형_분배!$C$2:$C$357,"&gt;="&amp;$B37,국내SCHD형_분배!$C$2:$C$357,"&lt;="&amp;$C37))</f>
         <v/>
       </c>
       <c r="F37" s="53">
-        <f>IF(COUNTIFS(국내SCHD형_분배!$A$2:$A$355,"402970",국내SCHD형_분배!$C$2:$C$355,"&gt;="&amp;$B37,국내SCHD형_분배!$C$2:$C$355,"&lt;="&amp;$C37)=0,"",SUMIFS(국내SCHD형_분배!$D$2:$D$355,국내SCHD형_분배!$A$2:$A$355,"402970",국내SCHD형_분배!$C$2:$C$355,"&gt;="&amp;$B37,국내SCHD형_분배!$C$2:$C$355,"&lt;="&amp;$C37))</f>
+        <f>IF(COUNTIFS(국내SCHD형_분배!$A$2:$A$357,"402970",국내SCHD형_분배!$C$2:$C$357,"&gt;="&amp;$B37,국내SCHD형_분배!$C$2:$C$357,"&lt;="&amp;$C37)=0,"",SUMIFS(국내SCHD형_분배!$D$2:$D$357,국내SCHD형_분배!$A$2:$A$357,"402970",국내SCHD형_분배!$C$2:$C$357,"&gt;="&amp;$B37,국내SCHD형_분배!$C$2:$C$357,"&lt;="&amp;$C37))</f>
         <v/>
       </c>
       <c r="G37" s="53">
-        <f>IF(COUNTIFS(국내SCHD형_분배!$A$2:$A$355,"489250",국내SCHD형_분배!$C$2:$C$355,"&gt;="&amp;$B37,국내SCHD형_분배!$C$2:$C$355,"&lt;="&amp;$C37)=0,"",SUMIFS(국내SCHD형_분배!$D$2:$D$355,국내SCHD형_분배!$A$2:$A$355,"489250",국내SCHD형_분배!$C$2:$C$355,"&gt;="&amp;$B37,국내SCHD형_분배!$C$2:$C$355,"&lt;="&amp;$C37))</f>
+        <f>IF(COUNTIFS(국내SCHD형_분배!$A$2:$A$357,"489250",국내SCHD형_분배!$C$2:$C$357,"&gt;="&amp;$B37,국내SCHD형_분배!$C$2:$C$357,"&lt;="&amp;$C37)=0,"",SUMIFS(국내SCHD형_분배!$D$2:$D$357,국내SCHD형_분배!$A$2:$A$357,"489250",국내SCHD형_분배!$C$2:$C$357,"&gt;="&amp;$B37,국내SCHD형_분배!$C$2:$C$357,"&lt;="&amp;$C37))</f>
         <v/>
       </c>
       <c r="H37" s="28">
@@ -25919,19 +25961,19 @@
         <v/>
       </c>
       <c r="D38" s="53">
-        <f>IF(COUNTIFS(국내SCHD형_분배!$A$2:$A$355,"458730",국내SCHD형_분배!$C$2:$C$355,"&gt;="&amp;$B38,국내SCHD형_분배!$C$2:$C$355,"&lt;="&amp;$C38)=0,"",SUMIFS(국내SCHD형_분배!$D$2:$D$355,국내SCHD형_분배!$A$2:$A$355,"458730",국내SCHD형_분배!$C$2:$C$355,"&gt;="&amp;$B38,국내SCHD형_분배!$C$2:$C$355,"&lt;="&amp;$C38))</f>
+        <f>IF(COUNTIFS(국내SCHD형_분배!$A$2:$A$357,"458730",국내SCHD형_분배!$C$2:$C$357,"&gt;="&amp;$B38,국내SCHD형_분배!$C$2:$C$357,"&lt;="&amp;$C38)=0,"",SUMIFS(국내SCHD형_분배!$D$2:$D$357,국내SCHD형_분배!$A$2:$A$357,"458730",국내SCHD형_분배!$C$2:$C$357,"&gt;="&amp;$B38,국내SCHD형_분배!$C$2:$C$357,"&lt;="&amp;$C38))</f>
         <v/>
       </c>
       <c r="E38" s="53">
-        <f>IF(COUNTIFS(국내SCHD형_분배!$A$2:$A$355,"446720",국내SCHD형_분배!$C$2:$C$355,"&gt;="&amp;$B38,국내SCHD형_분배!$C$2:$C$355,"&lt;="&amp;$C38)=0,"",SUMIFS(국내SCHD형_분배!$D$2:$D$355,국내SCHD형_분배!$A$2:$A$355,"446720",국내SCHD형_분배!$C$2:$C$355,"&gt;="&amp;$B38,국내SCHD형_분배!$C$2:$C$355,"&lt;="&amp;$C38))</f>
+        <f>IF(COUNTIFS(국내SCHD형_분배!$A$2:$A$357,"446720",국내SCHD형_분배!$C$2:$C$357,"&gt;="&amp;$B38,국내SCHD형_분배!$C$2:$C$357,"&lt;="&amp;$C38)=0,"",SUMIFS(국내SCHD형_분배!$D$2:$D$357,국내SCHD형_분배!$A$2:$A$357,"446720",국내SCHD형_분배!$C$2:$C$357,"&gt;="&amp;$B38,국내SCHD형_분배!$C$2:$C$357,"&lt;="&amp;$C38))</f>
         <v/>
       </c>
       <c r="F38" s="53">
-        <f>IF(COUNTIFS(국내SCHD형_분배!$A$2:$A$355,"402970",국내SCHD형_분배!$C$2:$C$355,"&gt;="&amp;$B38,국내SCHD형_분배!$C$2:$C$355,"&lt;="&amp;$C38)=0,"",SUMIFS(국내SCHD형_분배!$D$2:$D$355,국내SCHD형_분배!$A$2:$A$355,"402970",국내SCHD형_분배!$C$2:$C$355,"&gt;="&amp;$B38,국내SCHD형_분배!$C$2:$C$355,"&lt;="&amp;$C38))</f>
+        <f>IF(COUNTIFS(국내SCHD형_분배!$A$2:$A$357,"402970",국내SCHD형_분배!$C$2:$C$357,"&gt;="&amp;$B38,국내SCHD형_분배!$C$2:$C$357,"&lt;="&amp;$C38)=0,"",SUMIFS(국내SCHD형_분배!$D$2:$D$357,국내SCHD형_분배!$A$2:$A$357,"402970",국내SCHD형_분배!$C$2:$C$357,"&gt;="&amp;$B38,국내SCHD형_분배!$C$2:$C$357,"&lt;="&amp;$C38))</f>
         <v/>
       </c>
       <c r="G38" s="53">
-        <f>IF(COUNTIFS(국내SCHD형_분배!$A$2:$A$355,"489250",국내SCHD형_분배!$C$2:$C$355,"&gt;="&amp;$B38,국내SCHD형_분배!$C$2:$C$355,"&lt;="&amp;$C38)=0,"",SUMIFS(국내SCHD형_분배!$D$2:$D$355,국내SCHD형_분배!$A$2:$A$355,"489250",국내SCHD형_분배!$C$2:$C$355,"&gt;="&amp;$B38,국내SCHD형_분배!$C$2:$C$355,"&lt;="&amp;$C38))</f>
+        <f>IF(COUNTIFS(국내SCHD형_분배!$A$2:$A$357,"489250",국내SCHD형_분배!$C$2:$C$357,"&gt;="&amp;$B38,국내SCHD형_분배!$C$2:$C$357,"&lt;="&amp;$C38)=0,"",SUMIFS(국내SCHD형_분배!$D$2:$D$357,국내SCHD형_분배!$A$2:$A$357,"489250",국내SCHD형_분배!$C$2:$C$357,"&gt;="&amp;$B38,국내SCHD형_분배!$C$2:$C$357,"&lt;="&amp;$C38))</f>
         <v/>
       </c>
       <c r="H38" s="28">
@@ -25957,19 +25999,19 @@
         <v/>
       </c>
       <c r="D39" s="53">
-        <f>IF(COUNTIFS(국내SCHD형_분배!$A$2:$A$355,"458730",국내SCHD형_분배!$C$2:$C$355,"&gt;="&amp;$B39,국내SCHD형_분배!$C$2:$C$355,"&lt;="&amp;$C39)=0,"",SUMIFS(국내SCHD형_분배!$D$2:$D$355,국내SCHD형_분배!$A$2:$A$355,"458730",국내SCHD형_분배!$C$2:$C$355,"&gt;="&amp;$B39,국내SCHD형_분배!$C$2:$C$355,"&lt;="&amp;$C39))</f>
+        <f>IF(COUNTIFS(국내SCHD형_분배!$A$2:$A$357,"458730",국내SCHD형_분배!$C$2:$C$357,"&gt;="&amp;$B39,국내SCHD형_분배!$C$2:$C$357,"&lt;="&amp;$C39)=0,"",SUMIFS(국내SCHD형_분배!$D$2:$D$357,국내SCHD형_분배!$A$2:$A$357,"458730",국내SCHD형_분배!$C$2:$C$357,"&gt;="&amp;$B39,국내SCHD형_분배!$C$2:$C$357,"&lt;="&amp;$C39))</f>
         <v/>
       </c>
       <c r="E39" s="53">
-        <f>IF(COUNTIFS(국내SCHD형_분배!$A$2:$A$355,"446720",국내SCHD형_분배!$C$2:$C$355,"&gt;="&amp;$B39,국내SCHD형_분배!$C$2:$C$355,"&lt;="&amp;$C39)=0,"",SUMIFS(국내SCHD형_분배!$D$2:$D$355,국내SCHD형_분배!$A$2:$A$355,"446720",국내SCHD형_분배!$C$2:$C$355,"&gt;="&amp;$B39,국내SCHD형_분배!$C$2:$C$355,"&lt;="&amp;$C39))</f>
+        <f>IF(COUNTIFS(국내SCHD형_분배!$A$2:$A$357,"446720",국내SCHD형_분배!$C$2:$C$357,"&gt;="&amp;$B39,국내SCHD형_분배!$C$2:$C$357,"&lt;="&amp;$C39)=0,"",SUMIFS(국내SCHD형_분배!$D$2:$D$357,국내SCHD형_분배!$A$2:$A$357,"446720",국내SCHD형_분배!$C$2:$C$357,"&gt;="&amp;$B39,국내SCHD형_분배!$C$2:$C$357,"&lt;="&amp;$C39))</f>
         <v/>
       </c>
       <c r="F39" s="53">
-        <f>IF(COUNTIFS(국내SCHD형_분배!$A$2:$A$355,"402970",국내SCHD형_분배!$C$2:$C$355,"&gt;="&amp;$B39,국내SCHD형_분배!$C$2:$C$355,"&lt;="&amp;$C39)=0,"",SUMIFS(국내SCHD형_분배!$D$2:$D$355,국내SCHD형_분배!$A$2:$A$355,"402970",국내SCHD형_분배!$C$2:$C$355,"&gt;="&amp;$B39,국내SCHD형_분배!$C$2:$C$355,"&lt;="&amp;$C39))</f>
+        <f>IF(COUNTIFS(국내SCHD형_분배!$A$2:$A$357,"402970",국내SCHD형_분배!$C$2:$C$357,"&gt;="&amp;$B39,국내SCHD형_분배!$C$2:$C$357,"&lt;="&amp;$C39)=0,"",SUMIFS(국내SCHD형_분배!$D$2:$D$357,국내SCHD형_분배!$A$2:$A$357,"402970",국내SCHD형_분배!$C$2:$C$357,"&gt;="&amp;$B39,국내SCHD형_분배!$C$2:$C$357,"&lt;="&amp;$C39))</f>
         <v/>
       </c>
       <c r="G39" s="53">
-        <f>IF(COUNTIFS(국내SCHD형_분배!$A$2:$A$355,"489250",국내SCHD형_분배!$C$2:$C$355,"&gt;="&amp;$B39,국내SCHD형_분배!$C$2:$C$355,"&lt;="&amp;$C39)=0,"",SUMIFS(국내SCHD형_분배!$D$2:$D$355,국내SCHD형_분배!$A$2:$A$355,"489250",국내SCHD형_분배!$C$2:$C$355,"&gt;="&amp;$B39,국내SCHD형_분배!$C$2:$C$355,"&lt;="&amp;$C39))</f>
+        <f>IF(COUNTIFS(국내SCHD형_분배!$A$2:$A$357,"489250",국내SCHD형_분배!$C$2:$C$357,"&gt;="&amp;$B39,국내SCHD형_분배!$C$2:$C$357,"&lt;="&amp;$C39)=0,"",SUMIFS(국내SCHD형_분배!$D$2:$D$357,국내SCHD형_분배!$A$2:$A$357,"489250",국내SCHD형_분배!$C$2:$C$357,"&gt;="&amp;$B39,국내SCHD형_분배!$C$2:$C$357,"&lt;="&amp;$C39))</f>
         <v/>
       </c>
       <c r="H39" s="28">
@@ -25995,19 +26037,19 @@
         <v/>
       </c>
       <c r="D40" s="53">
-        <f>IF(COUNTIFS(국내SCHD형_분배!$A$2:$A$355,"458730",국내SCHD형_분배!$C$2:$C$355,"&gt;="&amp;$B40,국내SCHD형_분배!$C$2:$C$355,"&lt;="&amp;$C40)=0,"",SUMIFS(국내SCHD형_분배!$D$2:$D$355,국내SCHD형_분배!$A$2:$A$355,"458730",국내SCHD형_분배!$C$2:$C$355,"&gt;="&amp;$B40,국내SCHD형_분배!$C$2:$C$355,"&lt;="&amp;$C40))</f>
+        <f>IF(COUNTIFS(국내SCHD형_분배!$A$2:$A$357,"458730",국내SCHD형_분배!$C$2:$C$357,"&gt;="&amp;$B40,국내SCHD형_분배!$C$2:$C$357,"&lt;="&amp;$C40)=0,"",SUMIFS(국내SCHD형_분배!$D$2:$D$357,국내SCHD형_분배!$A$2:$A$357,"458730",국내SCHD형_분배!$C$2:$C$357,"&gt;="&amp;$B40,국내SCHD형_분배!$C$2:$C$357,"&lt;="&amp;$C40))</f>
         <v/>
       </c>
       <c r="E40" s="53">
-        <f>IF(COUNTIFS(국내SCHD형_분배!$A$2:$A$355,"446720",국내SCHD형_분배!$C$2:$C$355,"&gt;="&amp;$B40,국내SCHD형_분배!$C$2:$C$355,"&lt;="&amp;$C40)=0,"",SUMIFS(국내SCHD형_분배!$D$2:$D$355,국내SCHD형_분배!$A$2:$A$355,"446720",국내SCHD형_분배!$C$2:$C$355,"&gt;="&amp;$B40,국내SCHD형_분배!$C$2:$C$355,"&lt;="&amp;$C40))</f>
+        <f>IF(COUNTIFS(국내SCHD형_분배!$A$2:$A$357,"446720",국내SCHD형_분배!$C$2:$C$357,"&gt;="&amp;$B40,국내SCHD형_분배!$C$2:$C$357,"&lt;="&amp;$C40)=0,"",SUMIFS(국내SCHD형_분배!$D$2:$D$357,국내SCHD형_분배!$A$2:$A$357,"446720",국내SCHD형_분배!$C$2:$C$357,"&gt;="&amp;$B40,국내SCHD형_분배!$C$2:$C$357,"&lt;="&amp;$C40))</f>
         <v/>
       </c>
       <c r="F40" s="53">
-        <f>IF(COUNTIFS(국내SCHD형_분배!$A$2:$A$355,"402970",국내SCHD형_분배!$C$2:$C$355,"&gt;="&amp;$B40,국내SCHD형_분배!$C$2:$C$355,"&lt;="&amp;$C40)=0,"",SUMIFS(국내SCHD형_분배!$D$2:$D$355,국내SCHD형_분배!$A$2:$A$355,"402970",국내SCHD형_분배!$C$2:$C$355,"&gt;="&amp;$B40,국내SCHD형_분배!$C$2:$C$355,"&lt;="&amp;$C40))</f>
+        <f>IF(COUNTIFS(국내SCHD형_분배!$A$2:$A$357,"402970",국내SCHD형_분배!$C$2:$C$357,"&gt;="&amp;$B40,국내SCHD형_분배!$C$2:$C$357,"&lt;="&amp;$C40)=0,"",SUMIFS(국내SCHD형_분배!$D$2:$D$357,국내SCHD형_분배!$A$2:$A$357,"402970",국내SCHD형_분배!$C$2:$C$357,"&gt;="&amp;$B40,국내SCHD형_분배!$C$2:$C$357,"&lt;="&amp;$C40))</f>
         <v/>
       </c>
       <c r="G40" s="53">
-        <f>IF(COUNTIFS(국내SCHD형_분배!$A$2:$A$355,"489250",국내SCHD형_분배!$C$2:$C$355,"&gt;="&amp;$B40,국내SCHD형_분배!$C$2:$C$355,"&lt;="&amp;$C40)=0,"",SUMIFS(국내SCHD형_분배!$D$2:$D$355,국내SCHD형_분배!$A$2:$A$355,"489250",국내SCHD형_분배!$C$2:$C$355,"&gt;="&amp;$B40,국내SCHD형_분배!$C$2:$C$355,"&lt;="&amp;$C40))</f>
+        <f>IF(COUNTIFS(국내SCHD형_분배!$A$2:$A$357,"489250",국내SCHD형_분배!$C$2:$C$357,"&gt;="&amp;$B40,국내SCHD형_분배!$C$2:$C$357,"&lt;="&amp;$C40)=0,"",SUMIFS(국내SCHD형_분배!$D$2:$D$357,국내SCHD형_분배!$A$2:$A$357,"489250",국내SCHD형_분배!$C$2:$C$357,"&gt;="&amp;$B40,국내SCHD형_분배!$C$2:$C$357,"&lt;="&amp;$C40))</f>
         <v/>
       </c>
       <c r="H40" s="28">
@@ -26033,19 +26075,19 @@
         <v/>
       </c>
       <c r="D41" s="53">
-        <f>IF(COUNTIFS(국내SCHD형_분배!$A$2:$A$355,"458730",국내SCHD형_분배!$C$2:$C$355,"&gt;="&amp;$B41,국내SCHD형_분배!$C$2:$C$355,"&lt;="&amp;$C41)=0,"",SUMIFS(국내SCHD형_분배!$D$2:$D$355,국내SCHD형_분배!$A$2:$A$355,"458730",국내SCHD형_분배!$C$2:$C$355,"&gt;="&amp;$B41,국내SCHD형_분배!$C$2:$C$355,"&lt;="&amp;$C41))</f>
+        <f>IF(COUNTIFS(국내SCHD형_분배!$A$2:$A$357,"458730",국내SCHD형_분배!$C$2:$C$357,"&gt;="&amp;$B41,국내SCHD형_분배!$C$2:$C$357,"&lt;="&amp;$C41)=0,"",SUMIFS(국내SCHD형_분배!$D$2:$D$357,국내SCHD형_분배!$A$2:$A$357,"458730",국내SCHD형_분배!$C$2:$C$357,"&gt;="&amp;$B41,국내SCHD형_분배!$C$2:$C$357,"&lt;="&amp;$C41))</f>
         <v/>
       </c>
       <c r="E41" s="53">
-        <f>IF(COUNTIFS(국내SCHD형_분배!$A$2:$A$355,"446720",국내SCHD형_분배!$C$2:$C$355,"&gt;="&amp;$B41,국내SCHD형_분배!$C$2:$C$355,"&lt;="&amp;$C41)=0,"",SUMIFS(국내SCHD형_분배!$D$2:$D$355,국내SCHD형_분배!$A$2:$A$355,"446720",국내SCHD형_분배!$C$2:$C$355,"&gt;="&amp;$B41,국내SCHD형_분배!$C$2:$C$355,"&lt;="&amp;$C41))</f>
+        <f>IF(COUNTIFS(국내SCHD형_분배!$A$2:$A$357,"446720",국내SCHD형_분배!$C$2:$C$357,"&gt;="&amp;$B41,국내SCHD형_분배!$C$2:$C$357,"&lt;="&amp;$C41)=0,"",SUMIFS(국내SCHD형_분배!$D$2:$D$357,국내SCHD형_분배!$A$2:$A$357,"446720",국내SCHD형_분배!$C$2:$C$357,"&gt;="&amp;$B41,국내SCHD형_분배!$C$2:$C$357,"&lt;="&amp;$C41))</f>
         <v/>
       </c>
       <c r="F41" s="53">
-        <f>IF(COUNTIFS(국내SCHD형_분배!$A$2:$A$355,"402970",국내SCHD형_분배!$C$2:$C$355,"&gt;="&amp;$B41,국내SCHD형_분배!$C$2:$C$355,"&lt;="&amp;$C41)=0,"",SUMIFS(국내SCHD형_분배!$D$2:$D$355,국내SCHD형_분배!$A$2:$A$355,"402970",국내SCHD형_분배!$C$2:$C$355,"&gt;="&amp;$B41,국내SCHD형_분배!$C$2:$C$355,"&lt;="&amp;$C41))</f>
+        <f>IF(COUNTIFS(국내SCHD형_분배!$A$2:$A$357,"402970",국내SCHD형_분배!$C$2:$C$357,"&gt;="&amp;$B41,국내SCHD형_분배!$C$2:$C$357,"&lt;="&amp;$C41)=0,"",SUMIFS(국내SCHD형_분배!$D$2:$D$357,국내SCHD형_분배!$A$2:$A$357,"402970",국내SCHD형_분배!$C$2:$C$357,"&gt;="&amp;$B41,국내SCHD형_분배!$C$2:$C$357,"&lt;="&amp;$C41))</f>
         <v/>
       </c>
       <c r="G41" s="53">
-        <f>IF(COUNTIFS(국내SCHD형_분배!$A$2:$A$355,"489250",국내SCHD형_분배!$C$2:$C$355,"&gt;="&amp;$B41,국내SCHD형_분배!$C$2:$C$355,"&lt;="&amp;$C41)=0,"",SUMIFS(국내SCHD형_분배!$D$2:$D$355,국내SCHD형_분배!$A$2:$A$355,"489250",국내SCHD형_분배!$C$2:$C$355,"&gt;="&amp;$B41,국내SCHD형_분배!$C$2:$C$355,"&lt;="&amp;$C41))</f>
+        <f>IF(COUNTIFS(국내SCHD형_분배!$A$2:$A$357,"489250",국내SCHD형_분배!$C$2:$C$357,"&gt;="&amp;$B41,국내SCHD형_분배!$C$2:$C$357,"&lt;="&amp;$C41)=0,"",SUMIFS(국내SCHD형_분배!$D$2:$D$357,국내SCHD형_분배!$A$2:$A$357,"489250",국내SCHD형_분배!$C$2:$C$357,"&gt;="&amp;$B41,국내SCHD형_분배!$C$2:$C$357,"&lt;="&amp;$C41))</f>
         <v/>
       </c>
       <c r="H41" s="28">
@@ -26071,19 +26113,19 @@
         <v/>
       </c>
       <c r="D42" s="53">
-        <f>IF(COUNTIFS(국내SCHD형_분배!$A$2:$A$355,"458730",국내SCHD형_분배!$C$2:$C$355,"&gt;="&amp;$B42,국내SCHD형_분배!$C$2:$C$355,"&lt;="&amp;$C42)=0,"",SUMIFS(국내SCHD형_분배!$D$2:$D$355,국내SCHD형_분배!$A$2:$A$355,"458730",국내SCHD형_분배!$C$2:$C$355,"&gt;="&amp;$B42,국내SCHD형_분배!$C$2:$C$355,"&lt;="&amp;$C42))</f>
+        <f>IF(COUNTIFS(국내SCHD형_분배!$A$2:$A$357,"458730",국내SCHD형_분배!$C$2:$C$357,"&gt;="&amp;$B42,국내SCHD형_분배!$C$2:$C$357,"&lt;="&amp;$C42)=0,"",SUMIFS(국내SCHD형_분배!$D$2:$D$357,국내SCHD형_분배!$A$2:$A$357,"458730",국내SCHD형_분배!$C$2:$C$357,"&gt;="&amp;$B42,국내SCHD형_분배!$C$2:$C$357,"&lt;="&amp;$C42))</f>
         <v/>
       </c>
       <c r="E42" s="53">
-        <f>IF(COUNTIFS(국내SCHD형_분배!$A$2:$A$355,"446720",국내SCHD형_분배!$C$2:$C$355,"&gt;="&amp;$B42,국내SCHD형_분배!$C$2:$C$355,"&lt;="&amp;$C42)=0,"",SUMIFS(국내SCHD형_분배!$D$2:$D$355,국내SCHD형_분배!$A$2:$A$355,"446720",국내SCHD형_분배!$C$2:$C$355,"&gt;="&amp;$B42,국내SCHD형_분배!$C$2:$C$355,"&lt;="&amp;$C42))</f>
+        <f>IF(COUNTIFS(국내SCHD형_분배!$A$2:$A$357,"446720",국내SCHD형_분배!$C$2:$C$357,"&gt;="&amp;$B42,국내SCHD형_분배!$C$2:$C$357,"&lt;="&amp;$C42)=0,"",SUMIFS(국내SCHD형_분배!$D$2:$D$357,국내SCHD형_분배!$A$2:$A$357,"446720",국내SCHD형_분배!$C$2:$C$357,"&gt;="&amp;$B42,국내SCHD형_분배!$C$2:$C$357,"&lt;="&amp;$C42))</f>
         <v/>
       </c>
       <c r="F42" s="53">
-        <f>IF(COUNTIFS(국내SCHD형_분배!$A$2:$A$355,"402970",국내SCHD형_분배!$C$2:$C$355,"&gt;="&amp;$B42,국내SCHD형_분배!$C$2:$C$355,"&lt;="&amp;$C42)=0,"",SUMIFS(국내SCHD형_분배!$D$2:$D$355,국내SCHD형_분배!$A$2:$A$355,"402970",국내SCHD형_분배!$C$2:$C$355,"&gt;="&amp;$B42,국내SCHD형_분배!$C$2:$C$355,"&lt;="&amp;$C42))</f>
+        <f>IF(COUNTIFS(국내SCHD형_분배!$A$2:$A$357,"402970",국내SCHD형_분배!$C$2:$C$357,"&gt;="&amp;$B42,국내SCHD형_분배!$C$2:$C$357,"&lt;="&amp;$C42)=0,"",SUMIFS(국내SCHD형_분배!$D$2:$D$357,국내SCHD형_분배!$A$2:$A$357,"402970",국내SCHD형_분배!$C$2:$C$357,"&gt;="&amp;$B42,국내SCHD형_분배!$C$2:$C$357,"&lt;="&amp;$C42))</f>
         <v/>
       </c>
       <c r="G42" s="53">
-        <f>IF(COUNTIFS(국내SCHD형_분배!$A$2:$A$355,"489250",국내SCHD형_분배!$C$2:$C$355,"&gt;="&amp;$B42,국내SCHD형_분배!$C$2:$C$355,"&lt;="&amp;$C42)=0,"",SUMIFS(국내SCHD형_분배!$D$2:$D$355,국내SCHD형_분배!$A$2:$A$355,"489250",국내SCHD형_분배!$C$2:$C$355,"&gt;="&amp;$B42,국내SCHD형_분배!$C$2:$C$355,"&lt;="&amp;$C42))</f>
+        <f>IF(COUNTIFS(국내SCHD형_분배!$A$2:$A$357,"489250",국내SCHD형_분배!$C$2:$C$357,"&gt;="&amp;$B42,국내SCHD형_분배!$C$2:$C$357,"&lt;="&amp;$C42)=0,"",SUMIFS(국내SCHD형_분배!$D$2:$D$357,국내SCHD형_분배!$A$2:$A$357,"489250",국내SCHD형_분배!$C$2:$C$357,"&gt;="&amp;$B42,국내SCHD형_분배!$C$2:$C$357,"&lt;="&amp;$C42))</f>
         <v/>
       </c>
       <c r="H42" s="28">
@@ -26109,19 +26151,19 @@
         <v/>
       </c>
       <c r="D43" s="53">
-        <f>IF(COUNTIFS(국내SCHD형_분배!$A$2:$A$355,"458730",국내SCHD형_분배!$C$2:$C$355,"&gt;="&amp;$B43,국내SCHD형_분배!$C$2:$C$355,"&lt;="&amp;$C43)=0,"",SUMIFS(국내SCHD형_분배!$D$2:$D$355,국내SCHD형_분배!$A$2:$A$355,"458730",국내SCHD형_분배!$C$2:$C$355,"&gt;="&amp;$B43,국내SCHD형_분배!$C$2:$C$355,"&lt;="&amp;$C43))</f>
+        <f>IF(COUNTIFS(국내SCHD형_분배!$A$2:$A$357,"458730",국내SCHD형_분배!$C$2:$C$357,"&gt;="&amp;$B43,국내SCHD형_분배!$C$2:$C$357,"&lt;="&amp;$C43)=0,"",SUMIFS(국내SCHD형_분배!$D$2:$D$357,국내SCHD형_분배!$A$2:$A$357,"458730",국내SCHD형_분배!$C$2:$C$357,"&gt;="&amp;$B43,국내SCHD형_분배!$C$2:$C$357,"&lt;="&amp;$C43))</f>
         <v/>
       </c>
       <c r="E43" s="53">
-        <f>IF(COUNTIFS(국내SCHD형_분배!$A$2:$A$355,"446720",국내SCHD형_분배!$C$2:$C$355,"&gt;="&amp;$B43,국내SCHD형_분배!$C$2:$C$355,"&lt;="&amp;$C43)=0,"",SUMIFS(국내SCHD형_분배!$D$2:$D$355,국내SCHD형_분배!$A$2:$A$355,"446720",국내SCHD형_분배!$C$2:$C$355,"&gt;="&amp;$B43,국내SCHD형_분배!$C$2:$C$355,"&lt;="&amp;$C43))</f>
+        <f>IF(COUNTIFS(국내SCHD형_분배!$A$2:$A$357,"446720",국내SCHD형_분배!$C$2:$C$357,"&gt;="&amp;$B43,국내SCHD형_분배!$C$2:$C$357,"&lt;="&amp;$C43)=0,"",SUMIFS(국내SCHD형_분배!$D$2:$D$357,국내SCHD형_분배!$A$2:$A$357,"446720",국내SCHD형_분배!$C$2:$C$357,"&gt;="&amp;$B43,국내SCHD형_분배!$C$2:$C$357,"&lt;="&amp;$C43))</f>
         <v/>
       </c>
       <c r="F43" s="53">
-        <f>IF(COUNTIFS(국내SCHD형_분배!$A$2:$A$355,"402970",국내SCHD형_분배!$C$2:$C$355,"&gt;="&amp;$B43,국내SCHD형_분배!$C$2:$C$355,"&lt;="&amp;$C43)=0,"",SUMIFS(국내SCHD형_분배!$D$2:$D$355,국내SCHD형_분배!$A$2:$A$355,"402970",국내SCHD형_분배!$C$2:$C$355,"&gt;="&amp;$B43,국내SCHD형_분배!$C$2:$C$355,"&lt;="&amp;$C43))</f>
+        <f>IF(COUNTIFS(국내SCHD형_분배!$A$2:$A$357,"402970",국내SCHD형_분배!$C$2:$C$357,"&gt;="&amp;$B43,국내SCHD형_분배!$C$2:$C$357,"&lt;="&amp;$C43)=0,"",SUMIFS(국내SCHD형_분배!$D$2:$D$357,국내SCHD형_분배!$A$2:$A$357,"402970",국내SCHD형_분배!$C$2:$C$357,"&gt;="&amp;$B43,국내SCHD형_분배!$C$2:$C$357,"&lt;="&amp;$C43))</f>
         <v/>
       </c>
       <c r="G43" s="53">
-        <f>IF(COUNTIFS(국내SCHD형_분배!$A$2:$A$355,"489250",국내SCHD형_분배!$C$2:$C$355,"&gt;="&amp;$B43,국내SCHD형_분배!$C$2:$C$355,"&lt;="&amp;$C43)=0,"",SUMIFS(국내SCHD형_분배!$D$2:$D$355,국내SCHD형_분배!$A$2:$A$355,"489250",국내SCHD형_분배!$C$2:$C$355,"&gt;="&amp;$B43,국내SCHD형_분배!$C$2:$C$355,"&lt;="&amp;$C43))</f>
+        <f>IF(COUNTIFS(국내SCHD형_분배!$A$2:$A$357,"489250",국내SCHD형_분배!$C$2:$C$357,"&gt;="&amp;$B43,국내SCHD형_분배!$C$2:$C$357,"&lt;="&amp;$C43)=0,"",SUMIFS(국내SCHD형_분배!$D$2:$D$357,국내SCHD형_분배!$A$2:$A$357,"489250",국내SCHD형_분배!$C$2:$C$357,"&gt;="&amp;$B43,국내SCHD형_분배!$C$2:$C$357,"&lt;="&amp;$C43))</f>
         <v/>
       </c>
       <c r="H43" s="28">
@@ -26147,19 +26189,19 @@
         <v/>
       </c>
       <c r="D44" s="53">
-        <f>IF(COUNTIFS(국내SCHD형_분배!$A$2:$A$355,"458730",국내SCHD형_분배!$C$2:$C$355,"&gt;="&amp;$B44,국내SCHD형_분배!$C$2:$C$355,"&lt;="&amp;$C44)=0,"",SUMIFS(국내SCHD형_분배!$D$2:$D$355,국내SCHD형_분배!$A$2:$A$355,"458730",국내SCHD형_분배!$C$2:$C$355,"&gt;="&amp;$B44,국내SCHD형_분배!$C$2:$C$355,"&lt;="&amp;$C44))</f>
+        <f>IF(COUNTIFS(국내SCHD형_분배!$A$2:$A$357,"458730",국내SCHD형_분배!$C$2:$C$357,"&gt;="&amp;$B44,국내SCHD형_분배!$C$2:$C$357,"&lt;="&amp;$C44)=0,"",SUMIFS(국내SCHD형_분배!$D$2:$D$357,국내SCHD형_분배!$A$2:$A$357,"458730",국내SCHD형_분배!$C$2:$C$357,"&gt;="&amp;$B44,국내SCHD형_분배!$C$2:$C$357,"&lt;="&amp;$C44))</f>
         <v/>
       </c>
       <c r="E44" s="53">
-        <f>IF(COUNTIFS(국내SCHD형_분배!$A$2:$A$355,"446720",국내SCHD형_분배!$C$2:$C$355,"&gt;="&amp;$B44,국내SCHD형_분배!$C$2:$C$355,"&lt;="&amp;$C44)=0,"",SUMIFS(국내SCHD형_분배!$D$2:$D$355,국내SCHD형_분배!$A$2:$A$355,"446720",국내SCHD형_분배!$C$2:$C$355,"&gt;="&amp;$B44,국내SCHD형_분배!$C$2:$C$355,"&lt;="&amp;$C44))</f>
+        <f>IF(COUNTIFS(국내SCHD형_분배!$A$2:$A$357,"446720",국내SCHD형_분배!$C$2:$C$357,"&gt;="&amp;$B44,국내SCHD형_분배!$C$2:$C$357,"&lt;="&amp;$C44)=0,"",SUMIFS(국내SCHD형_분배!$D$2:$D$357,국내SCHD형_분배!$A$2:$A$357,"446720",국내SCHD형_분배!$C$2:$C$357,"&gt;="&amp;$B44,국내SCHD형_분배!$C$2:$C$357,"&lt;="&amp;$C44))</f>
         <v/>
       </c>
       <c r="F44" s="53">
-        <f>IF(COUNTIFS(국내SCHD형_분배!$A$2:$A$355,"402970",국내SCHD형_분배!$C$2:$C$355,"&gt;="&amp;$B44,국내SCHD형_분배!$C$2:$C$355,"&lt;="&amp;$C44)=0,"",SUMIFS(국내SCHD형_분배!$D$2:$D$355,국내SCHD형_분배!$A$2:$A$355,"402970",국내SCHD형_분배!$C$2:$C$355,"&gt;="&amp;$B44,국내SCHD형_분배!$C$2:$C$355,"&lt;="&amp;$C44))</f>
+        <f>IF(COUNTIFS(국내SCHD형_분배!$A$2:$A$357,"402970",국내SCHD형_분배!$C$2:$C$357,"&gt;="&amp;$B44,국내SCHD형_분배!$C$2:$C$357,"&lt;="&amp;$C44)=0,"",SUMIFS(국내SCHD형_분배!$D$2:$D$357,국내SCHD형_분배!$A$2:$A$357,"402970",국내SCHD형_분배!$C$2:$C$357,"&gt;="&amp;$B44,국내SCHD형_분배!$C$2:$C$357,"&lt;="&amp;$C44))</f>
         <v/>
       </c>
       <c r="G44" s="53">
-        <f>IF(COUNTIFS(국내SCHD형_분배!$A$2:$A$355,"489250",국내SCHD형_분배!$C$2:$C$355,"&gt;="&amp;$B44,국내SCHD형_분배!$C$2:$C$355,"&lt;="&amp;$C44)=0,"",SUMIFS(국내SCHD형_분배!$D$2:$D$355,국내SCHD형_분배!$A$2:$A$355,"489250",국내SCHD형_분배!$C$2:$C$355,"&gt;="&amp;$B44,국내SCHD형_분배!$C$2:$C$355,"&lt;="&amp;$C44))</f>
+        <f>IF(COUNTIFS(국내SCHD형_분배!$A$2:$A$357,"489250",국내SCHD형_분배!$C$2:$C$357,"&gt;="&amp;$B44,국내SCHD형_분배!$C$2:$C$357,"&lt;="&amp;$C44)=0,"",SUMIFS(국내SCHD형_분배!$D$2:$D$357,국내SCHD형_분배!$A$2:$A$357,"489250",국내SCHD형_분배!$C$2:$C$357,"&gt;="&amp;$B44,국내SCHD형_분배!$C$2:$C$357,"&lt;="&amp;$C44))</f>
         <v/>
       </c>
       <c r="H44" s="28">
@@ -26215,11 +26257,11 @@
         </is>
       </c>
       <c r="B2" s="49" t="n">
-        <v>46307</v>
+        <v>46308</v>
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>← 이 날 종가로 계산한 비중. 그날 공식 파일을 못 받아 Schwab 공식 보유종목 CSV(2026-10-09)의 보유 주식 수 × 종가로 계산했습니다.</t>
+          <t>← 이 날 종가로 계산한 비중. 그날 공식 파일을 못 받아 Schwab 공식 보유종목 CSV(2026-10-12)의 보유 주식 수 × 종가로 계산했습니다.</t>
         </is>
       </c>
     </row>
@@ -26316,7 +26358,7 @@
         </is>
       </c>
       <c r="I5" s="61" t="n">
-        <v>0.04621969</v>
+        <v>0.04708691</v>
       </c>
       <c r="J5" s="6" t="inlineStr">
         <is>
@@ -26370,25 +26412,25 @@
       </c>
       <c r="H6" s="6" t="inlineStr">
         <is>
-          <t>PG</t>
+          <t>QCOM</t>
         </is>
       </c>
       <c r="I6" s="61" t="n">
-        <v>0.04337427</v>
+        <v>0.04337273</v>
       </c>
       <c r="J6" s="6" t="inlineStr">
         <is>
-          <t>PROCTER &amp; GAMBLE</t>
+          <t>QUALCOMM</t>
         </is>
       </c>
       <c r="K6" s="6" t="inlineStr">
         <is>
-          <t>Consumer Staples</t>
+          <t>Information Technology</t>
         </is>
       </c>
       <c r="L6" s="6" t="inlineStr">
         <is>
-          <t>프록터앤드갬블</t>
+          <t>퀄컴</t>
         </is>
       </c>
       <c r="M6" s="7">
@@ -26428,25 +26470,25 @@
       </c>
       <c r="H7" s="6" t="inlineStr">
         <is>
-          <t>QCOM</t>
+          <t>PG</t>
         </is>
       </c>
       <c r="I7" s="61" t="n">
-        <v>0.04289955</v>
+        <v>0.04320501</v>
       </c>
       <c r="J7" s="6" t="inlineStr">
         <is>
-          <t>QUALCOMM</t>
+          <t>PROCTER &amp; GAMBLE</t>
         </is>
       </c>
       <c r="K7" s="6" t="inlineStr">
         <is>
-          <t>Information Technology</t>
+          <t>Consumer Staples</t>
         </is>
       </c>
       <c r="L7" s="6" t="inlineStr">
         <is>
-          <t>퀄컴</t>
+          <t>프록터앤드갬블</t>
         </is>
       </c>
       <c r="M7" s="7">
@@ -26486,25 +26528,25 @@
       </c>
       <c r="H8" s="6" t="inlineStr">
         <is>
-          <t>KO</t>
+          <t>CVX</t>
         </is>
       </c>
       <c r="I8" s="61" t="n">
-        <v>0.04253438</v>
+        <v>0.0428515</v>
       </c>
       <c r="J8" s="6" t="inlineStr">
         <is>
-          <t>COCA-COLA</t>
+          <t>CHEVRON</t>
         </is>
       </c>
       <c r="K8" s="6" t="inlineStr">
         <is>
-          <t>Consumer Staples</t>
+          <t>Energy</t>
         </is>
       </c>
       <c r="L8" s="6" t="inlineStr">
         <is>
-          <t>코카콜라</t>
+          <t>셰브론</t>
         </is>
       </c>
       <c r="M8" s="7">
@@ -26544,15 +26586,15 @@
       </c>
       <c r="H9" s="6" t="inlineStr">
         <is>
-          <t>CVX</t>
+          <t>COP</t>
         </is>
       </c>
       <c r="I9" s="61" t="n">
-        <v>0.04243566999999999</v>
+        <v>0.04274977</v>
       </c>
       <c r="J9" s="6" t="inlineStr">
         <is>
-          <t>CHEVRON</t>
+          <t>CONOCOPHILLIPS</t>
         </is>
       </c>
       <c r="K9" s="6" t="inlineStr">
@@ -26562,7 +26604,7 @@
       </c>
       <c r="L9" s="6" t="inlineStr">
         <is>
-          <t>셰브론</t>
+          <t>코노코필립스</t>
         </is>
       </c>
       <c r="M9" s="7">
@@ -26602,25 +26644,25 @@
       </c>
       <c r="H10" s="6" t="inlineStr">
         <is>
-          <t>COP</t>
+          <t>KO</t>
         </is>
       </c>
       <c r="I10" s="61" t="n">
-        <v>0.04185615</v>
+        <v>0.04256384</v>
       </c>
       <c r="J10" s="6" t="inlineStr">
         <is>
-          <t>CONOCOPHILLIPS</t>
+          <t>COCA-COLA</t>
         </is>
       </c>
       <c r="K10" s="6" t="inlineStr">
         <is>
-          <t>Energy</t>
+          <t>Consumer Staples</t>
         </is>
       </c>
       <c r="L10" s="6" t="inlineStr">
         <is>
-          <t>코노코필립스</t>
+          <t>코카콜라</t>
         </is>
       </c>
       <c r="M10" s="7">
@@ -26660,15 +26702,15 @@
       </c>
       <c r="H11" s="6" t="inlineStr">
         <is>
-          <t>MRK</t>
+          <t>UNH</t>
         </is>
       </c>
       <c r="I11" s="61" t="n">
-        <v>0.04009386</v>
+        <v>0.0393964</v>
       </c>
       <c r="J11" s="6" t="inlineStr">
         <is>
-          <t>MERCK &amp; CO INC</t>
+          <t>UNITEDHEALTH GROUP</t>
         </is>
       </c>
       <c r="K11" s="6" t="inlineStr">
@@ -26678,7 +26720,7 @@
       </c>
       <c r="L11" s="6" t="inlineStr">
         <is>
-          <t>머크</t>
+          <t>유나이티드헬스</t>
         </is>
       </c>
       <c r="M11" s="7">
@@ -26718,15 +26760,15 @@
       </c>
       <c r="H12" s="6" t="inlineStr">
         <is>
-          <t>UNH</t>
+          <t>MRK</t>
         </is>
       </c>
       <c r="I12" s="61" t="n">
-        <v>0.03958902</v>
+        <v>0.03902534</v>
       </c>
       <c r="J12" s="6" t="inlineStr">
         <is>
-          <t>UNITEDHEALTH GROUP</t>
+          <t>MERCK &amp; CO INC</t>
         </is>
       </c>
       <c r="K12" s="6" t="inlineStr">
@@ -26736,7 +26778,7 @@
       </c>
       <c r="L12" s="6" t="inlineStr">
         <is>
-          <t>유나이티드헬스</t>
+          <t>머크</t>
         </is>
       </c>
       <c r="M12" s="7">
@@ -26780,7 +26822,7 @@
         </is>
       </c>
       <c r="I13" s="61" t="n">
-        <v>0.03941473</v>
+        <v>0.03885666</v>
       </c>
       <c r="J13" s="6" t="inlineStr">
         <is>
@@ -26838,7 +26880,7 @@
         </is>
       </c>
       <c r="I14" s="61" t="n">
-        <v>0.0385271</v>
+        <v>0.03871495</v>
       </c>
       <c r="J14" s="6" t="inlineStr">
         <is>
@@ -26886,7 +26928,7 @@
         </is>
       </c>
       <c r="I15" s="61" t="n">
-        <v>0.03813983</v>
+        <v>0.03846246</v>
       </c>
       <c r="J15" s="6" t="inlineStr">
         <is>
@@ -26934,7 +26976,7 @@
         </is>
       </c>
       <c r="I16" s="61" t="n">
-        <v>0.03768319</v>
+        <v>0.03775924</v>
       </c>
       <c r="J16" s="6" t="inlineStr">
         <is>
@@ -26972,7 +27014,7 @@
         </is>
       </c>
       <c r="I17" s="61" t="n">
-        <v>0.03560754</v>
+        <v>0.03612815</v>
       </c>
       <c r="J17" s="6" t="inlineStr">
         <is>
@@ -27010,7 +27052,7 @@
         </is>
       </c>
       <c r="I18" s="61" t="n">
-        <v>0.03330342</v>
+        <v>0.03300566</v>
       </c>
       <c r="J18" s="6" t="inlineStr">
         <is>
@@ -27039,7 +27081,7 @@
         </is>
       </c>
       <c r="I19" s="61" t="n">
-        <v>0.03030605</v>
+        <v>0.03017718</v>
       </c>
       <c r="J19" s="6" t="inlineStr">
         <is>
@@ -27073,7 +27115,7 @@
         </is>
       </c>
       <c r="I20" s="61" t="n">
-        <v>0.02979081</v>
+        <v>0.02923612</v>
       </c>
       <c r="J20" s="6" t="inlineStr">
         <is>
@@ -27112,7 +27154,7 @@
         </is>
       </c>
       <c r="I21" s="61" t="n">
-        <v>0.02755036</v>
+        <v>0.02768124</v>
       </c>
       <c r="J21" s="6" t="inlineStr">
         <is>
@@ -27150,7 +27192,7 @@
         </is>
       </c>
       <c r="I22" s="61" t="n">
-        <v>0.02633119</v>
+        <v>0.02585262</v>
       </c>
       <c r="J22" s="6" t="inlineStr">
         <is>
@@ -27188,7 +27230,7 @@
         </is>
       </c>
       <c r="I23" s="61" t="n">
-        <v>0.02182185</v>
+        <v>0.02084944</v>
       </c>
       <c r="J23" s="6" t="inlineStr">
         <is>
@@ -27226,7 +27268,7 @@
         </is>
       </c>
       <c r="I24" s="61" t="n">
-        <v>0.01999572</v>
+        <v>0.02029086</v>
       </c>
       <c r="J24" s="6" t="inlineStr">
         <is>
@@ -27264,7 +27306,7 @@
         </is>
       </c>
       <c r="I25" s="61" t="n">
-        <v>0.01853778</v>
+        <v>0.01866352</v>
       </c>
       <c r="J25" s="6" t="inlineStr">
         <is>
@@ -27302,7 +27344,7 @@
         </is>
       </c>
       <c r="I26" s="61" t="n">
-        <v>0.0183329</v>
+        <v>0.01828045</v>
       </c>
       <c r="J26" s="6" t="inlineStr">
         <is>
@@ -27340,7 +27382,7 @@
         </is>
       </c>
       <c r="I27" s="61" t="n">
-        <v>0.01809509</v>
+        <v>0.01793923</v>
       </c>
       <c r="J27" s="6" t="inlineStr">
         <is>
@@ -27378,7 +27420,7 @@
         </is>
       </c>
       <c r="I28" s="61" t="n">
-        <v>0.01767205</v>
+        <v>0.01743452</v>
       </c>
       <c r="J28" s="6" t="inlineStr">
         <is>
@@ -27416,7 +27458,7 @@
         </is>
       </c>
       <c r="I29" s="61" t="n">
-        <v>0.01496504</v>
+        <v>0.01490483</v>
       </c>
       <c r="J29" s="6" t="inlineStr">
         <is>
@@ -27454,7 +27496,7 @@
         </is>
       </c>
       <c r="I30" s="61" t="n">
-        <v>0.01469193</v>
+        <v>0.01486642</v>
       </c>
       <c r="J30" s="6" t="inlineStr">
         <is>
@@ -27488,7 +27530,7 @@
         </is>
       </c>
       <c r="I31" s="61" t="n">
-        <v>0.01364071</v>
+        <v>0.01394894</v>
       </c>
       <c r="J31" s="6" t="inlineStr">
         <is>
@@ -27513,7 +27555,7 @@
         </is>
       </c>
       <c r="I32" s="61" t="n">
-        <v>0.01190445</v>
+        <v>0.01196931</v>
       </c>
       <c r="J32" s="6" t="inlineStr">
         <is>
@@ -27543,7 +27585,7 @@
         </is>
       </c>
       <c r="I33" s="61" t="n">
-        <v>0.0116733</v>
+        <v>0.01150248</v>
       </c>
       <c r="J33" s="6" t="inlineStr">
         <is>
@@ -27568,7 +27610,7 @@
         </is>
       </c>
       <c r="I34" s="61" t="n">
-        <v>0.00981695</v>
+        <v>0.01012723</v>
       </c>
       <c r="J34" s="6" t="inlineStr">
         <is>
@@ -27593,7 +27635,7 @@
         </is>
       </c>
       <c r="I35" s="61" t="n">
-        <v>0.00848407</v>
+        <v>0.008589940000000001</v>
       </c>
       <c r="J35" s="6" t="inlineStr">
         <is>
@@ -27618,7 +27660,7 @@
         </is>
       </c>
       <c r="I36" s="61" t="n">
-        <v>0.00831993</v>
+        <v>0.008255780000000001</v>
       </c>
       <c r="J36" s="6" t="inlineStr">
         <is>
@@ -27643,7 +27685,7 @@
         </is>
       </c>
       <c r="I37" s="61" t="n">
-        <v>0.006701970000000001</v>
+        <v>0.00653969</v>
       </c>
       <c r="J37" s="6" t="inlineStr">
         <is>
@@ -27668,7 +27710,7 @@
         </is>
       </c>
       <c r="I38" s="61" t="n">
-        <v>0.00643539</v>
+        <v>0.00642043</v>
       </c>
       <c r="J38" s="6" t="inlineStr">
         <is>
@@ -27693,7 +27735,7 @@
         </is>
       </c>
       <c r="I39" s="61" t="n">
-        <v>0.00607153</v>
+        <v>0.006024939999999999</v>
       </c>
       <c r="J39" s="6" t="inlineStr">
         <is>
@@ -27714,20 +27756,20 @@
     <row r="40">
       <c r="H40" s="6" t="inlineStr">
         <is>
-          <t>RF</t>
+          <t>DRI</t>
         </is>
       </c>
       <c r="I40" s="61" t="n">
-        <v>0.00590588</v>
+        <v>0.005895559999999999</v>
       </c>
       <c r="J40" s="6" t="inlineStr">
         <is>
-          <t>REGIONS FINANCIAL</t>
+          <t>DARDEN RESTAURANTS INC</t>
         </is>
       </c>
       <c r="K40" s="6" t="inlineStr">
         <is>
-          <t>Financials</t>
+          <t>Consumer Discretionary</t>
         </is>
       </c>
       <c r="L40" s="6" t="inlineStr"/>
@@ -27739,20 +27781,20 @@
     <row r="41">
       <c r="H41" s="6" t="inlineStr">
         <is>
-          <t>DRI</t>
+          <t>RF</t>
         </is>
       </c>
       <c r="I41" s="61" t="n">
-        <v>0.00574028</v>
+        <v>0.00581152</v>
       </c>
       <c r="J41" s="6" t="inlineStr">
         <is>
-          <t>DARDEN RESTAURANTS INC</t>
+          <t>REGIONS FINANCIAL</t>
         </is>
       </c>
       <c r="K41" s="6" t="inlineStr">
         <is>
-          <t>Consumer Discretionary</t>
+          <t>Financials</t>
         </is>
       </c>
       <c r="L41" s="6" t="inlineStr"/>
@@ -27768,7 +27810,7 @@
         </is>
       </c>
       <c r="I42" s="61" t="n">
-        <v>0.005618499999999999</v>
+        <v>0.005462320000000001</v>
       </c>
       <c r="J42" s="6" t="inlineStr">
         <is>
@@ -27793,7 +27835,7 @@
         </is>
       </c>
       <c r="I43" s="61" t="n">
-        <v>0.00532189</v>
+        <v>0.00529678</v>
       </c>
       <c r="J43" s="6" t="inlineStr">
         <is>
@@ -27818,7 +27860,7 @@
         </is>
       </c>
       <c r="I44" s="61" t="n">
-        <v>0.0048129</v>
+        <v>0.00500685</v>
       </c>
       <c r="J44" s="6" t="inlineStr">
         <is>
@@ -27843,7 +27885,7 @@
         </is>
       </c>
       <c r="I45" s="61" t="n">
-        <v>0.00480721</v>
+        <v>0.00485186</v>
       </c>
       <c r="J45" s="6" t="inlineStr">
         <is>
@@ -27868,7 +27910,7 @@
         </is>
       </c>
       <c r="I46" s="61" t="n">
-        <v>0.00474319</v>
+        <v>0.00475145</v>
       </c>
       <c r="J46" s="6" t="inlineStr">
         <is>
@@ -27889,20 +27931,20 @@
     <row r="47">
       <c r="H47" s="6" t="inlineStr">
         <is>
-          <t>GIS</t>
+          <t>BBY</t>
         </is>
       </c>
       <c r="I47" s="61" t="n">
-        <v>0.00442888</v>
+        <v>0.00439892</v>
       </c>
       <c r="J47" s="6" t="inlineStr">
         <is>
-          <t>GENERAL MILLS INC</t>
+          <t>BEST BUY</t>
         </is>
       </c>
       <c r="K47" s="6" t="inlineStr">
         <is>
-          <t>Consumer Staples</t>
+          <t>Consumer Discretionary</t>
         </is>
       </c>
       <c r="L47" s="6" t="inlineStr"/>
@@ -27914,20 +27956,20 @@
     <row r="48">
       <c r="H48" s="6" t="inlineStr">
         <is>
-          <t>BBY</t>
+          <t>EWBC</t>
         </is>
       </c>
       <c r="I48" s="61" t="n">
-        <v>0.0043629</v>
+        <v>0.00432773</v>
       </c>
       <c r="J48" s="6" t="inlineStr">
         <is>
-          <t>BEST BUY</t>
+          <t>EAST WEST BANCORP</t>
         </is>
       </c>
       <c r="K48" s="6" t="inlineStr">
         <is>
-          <t>Consumer Discretionary</t>
+          <t>Financials</t>
         </is>
       </c>
       <c r="L48" s="6" t="inlineStr"/>
@@ -27939,20 +27981,20 @@
     <row r="49">
       <c r="H49" s="6" t="inlineStr">
         <is>
-          <t>EWBC</t>
+          <t>GIS</t>
         </is>
       </c>
       <c r="I49" s="61" t="n">
-        <v>0.00435788</v>
+        <v>0.00429871</v>
       </c>
       <c r="J49" s="6" t="inlineStr">
         <is>
-          <t>EAST WEST BANCORP</t>
+          <t>GENERAL MILLS INC</t>
         </is>
       </c>
       <c r="K49" s="6" t="inlineStr">
         <is>
-          <t>Financials</t>
+          <t>Consumer Staples</t>
         </is>
       </c>
       <c r="L49" s="6" t="inlineStr"/>
@@ -27968,7 +28010,7 @@
         </is>
       </c>
       <c r="I50" s="61" t="n">
-        <v>0.00415646</v>
+        <v>0.00424809</v>
       </c>
       <c r="J50" s="6" t="inlineStr">
         <is>
@@ -27993,7 +28035,7 @@
         </is>
       </c>
       <c r="I51" s="61" t="n">
-        <v>0.00258126</v>
+        <v>0.00262032</v>
       </c>
       <c r="J51" s="6" t="inlineStr">
         <is>
@@ -28018,7 +28060,7 @@
         </is>
       </c>
       <c r="I52" s="61" t="n">
-        <v>0.00251795</v>
+        <v>0.00252232</v>
       </c>
       <c r="J52" s="6" t="inlineStr">
         <is>
@@ -28043,7 +28085,7 @@
         </is>
       </c>
       <c r="I53" s="61" t="n">
-        <v>0.00250375</v>
+        <v>0.00251094</v>
       </c>
       <c r="J53" s="6" t="inlineStr">
         <is>
@@ -28068,7 +28110,7 @@
         </is>
       </c>
       <c r="I54" s="61" t="n">
-        <v>0.00224197</v>
+        <v>0.00219546</v>
       </c>
       <c r="J54" s="6" t="inlineStr">
         <is>
@@ -28093,7 +28135,7 @@
         </is>
       </c>
       <c r="I55" s="61" t="n">
-        <v>0.00214089</v>
+        <v>0.00213924</v>
       </c>
       <c r="J55" s="6" t="inlineStr">
         <is>
@@ -28118,7 +28160,7 @@
         </is>
       </c>
       <c r="I56" s="61" t="n">
-        <v>0.00204087</v>
+        <v>0.00201503</v>
       </c>
       <c r="J56" s="6" t="inlineStr">
         <is>
@@ -28143,7 +28185,7 @@
         </is>
       </c>
       <c r="I57" s="61" t="n">
-        <v>0.00186367</v>
+        <v>0.00191453</v>
       </c>
       <c r="J57" s="6" t="inlineStr">
         <is>
@@ -28164,20 +28206,20 @@
     <row r="58">
       <c r="H58" s="6" t="inlineStr">
         <is>
-          <t>M</t>
+          <t>MSM</t>
         </is>
       </c>
       <c r="I58" s="61" t="n">
-        <v>0.00153021</v>
+        <v>0.00152937</v>
       </c>
       <c r="J58" s="6" t="inlineStr">
         <is>
-          <t>MACYS INC</t>
+          <t>MSC INDUSTRIAL CLASS A</t>
         </is>
       </c>
       <c r="K58" s="6" t="inlineStr">
         <is>
-          <t>Consumer Discretionary</t>
+          <t>Industrials</t>
         </is>
       </c>
       <c r="L58" s="6" t="inlineStr"/>
@@ -28189,20 +28231,20 @@
     <row r="59">
       <c r="H59" s="6" t="inlineStr">
         <is>
-          <t>MSM</t>
+          <t>M</t>
         </is>
       </c>
       <c r="I59" s="61" t="n">
-        <v>0.00149316</v>
+        <v>0.00150924</v>
       </c>
       <c r="J59" s="6" t="inlineStr">
         <is>
-          <t>MSC INDUSTRIAL CLASS A</t>
+          <t>MACYS INC</t>
         </is>
       </c>
       <c r="K59" s="6" t="inlineStr">
         <is>
-          <t>Industrials</t>
+          <t>Consumer Discretionary</t>
         </is>
       </c>
       <c r="L59" s="6" t="inlineStr"/>
@@ -28218,7 +28260,7 @@
         </is>
       </c>
       <c r="I60" s="61" t="n">
-        <v>0.00147345</v>
+        <v>0.00150688</v>
       </c>
       <c r="J60" s="6" t="inlineStr">
         <is>
@@ -28239,20 +28281,20 @@
     <row r="61">
       <c r="H61" s="6" t="inlineStr">
         <is>
-          <t>MUR</t>
+          <t>MTN</t>
         </is>
       </c>
       <c r="I61" s="61" t="n">
-        <v>0.00134565</v>
+        <v>0.00137352</v>
       </c>
       <c r="J61" s="6" t="inlineStr">
         <is>
-          <t>MURPHY OIL CORP</t>
+          <t>VAIL RESORTS</t>
         </is>
       </c>
       <c r="K61" s="6" t="inlineStr">
         <is>
-          <t>Energy</t>
+          <t>Consumer Discretionary</t>
         </is>
       </c>
       <c r="L61" s="6" t="inlineStr"/>
@@ -28264,20 +28306,20 @@
     <row r="62">
       <c r="H62" s="6" t="inlineStr">
         <is>
-          <t>MTN</t>
+          <t>MUR</t>
         </is>
       </c>
       <c r="I62" s="61" t="n">
-        <v>0.00132723</v>
+        <v>0.0013302</v>
       </c>
       <c r="J62" s="6" t="inlineStr">
         <is>
-          <t>VAIL RESORTS</t>
+          <t>MURPHY OIL CORP</t>
         </is>
       </c>
       <c r="K62" s="6" t="inlineStr">
         <is>
-          <t>Consumer Discretionary</t>
+          <t>Energy</t>
         </is>
       </c>
       <c r="L62" s="6" t="inlineStr"/>
@@ -28293,7 +28335,7 @@
         </is>
       </c>
       <c r="I63" s="61" t="n">
-        <v>0.00117918</v>
+        <v>0.00117587</v>
       </c>
       <c r="J63" s="6" t="inlineStr">
         <is>
@@ -28318,7 +28360,7 @@
         </is>
       </c>
       <c r="I64" s="61" t="n">
-        <v>0.00116572</v>
+        <v>0.00115621</v>
       </c>
       <c r="J64" s="6" t="inlineStr">
         <is>
@@ -28343,7 +28385,7 @@
         </is>
       </c>
       <c r="I65" s="61" t="n">
-        <v>0.0010776</v>
+        <v>0.00105213</v>
       </c>
       <c r="J65" s="6" t="inlineStr">
         <is>
@@ -28368,7 +28410,7 @@
         </is>
       </c>
       <c r="I66" s="61" t="n">
-        <v>0.00101182</v>
+        <v>0.0009912600000000001</v>
       </c>
       <c r="J66" s="6" t="inlineStr">
         <is>
@@ -28389,20 +28431,20 @@
     <row r="67">
       <c r="H67" s="6" t="inlineStr">
         <is>
-          <t>CWEN</t>
+          <t>KFY</t>
         </is>
       </c>
       <c r="I67" s="61" t="n">
-        <v>0.00093153</v>
+        <v>0.00093461</v>
       </c>
       <c r="J67" s="6" t="inlineStr">
         <is>
-          <t>CLEARWAY ENERGY INC CLASS C</t>
+          <t>KORN FERRY</t>
         </is>
       </c>
       <c r="K67" s="6" t="inlineStr">
         <is>
-          <t>Utilities</t>
+          <t>Industrials</t>
         </is>
       </c>
       <c r="L67" s="6" t="inlineStr"/>
@@ -28414,20 +28456,20 @@
     <row r="68">
       <c r="H68" s="6" t="inlineStr">
         <is>
-          <t>KFY</t>
+          <t>CWEN</t>
         </is>
       </c>
       <c r="I68" s="61" t="n">
-        <v>0.00092506</v>
+        <v>0.0009285499999999999</v>
       </c>
       <c r="J68" s="6" t="inlineStr">
         <is>
-          <t>KORN FERRY</t>
+          <t>CLEARWAY ENERGY INC CLASS C</t>
         </is>
       </c>
       <c r="K68" s="6" t="inlineStr">
         <is>
-          <t>Industrials</t>
+          <t>Utilities</t>
         </is>
       </c>
       <c r="L68" s="6" t="inlineStr"/>
@@ -28443,7 +28485,7 @@
         </is>
       </c>
       <c r="I69" s="61" t="n">
-        <v>0.00091434</v>
+        <v>0.00090456</v>
       </c>
       <c r="J69" s="6" t="inlineStr">
         <is>
@@ -28464,20 +28506,20 @@
     <row r="70">
       <c r="H70" s="6" t="inlineStr">
         <is>
-          <t>PAG</t>
+          <t>RHI</t>
         </is>
       </c>
       <c r="I70" s="61" t="n">
-        <v>0.0008758</v>
+        <v>0.00088303</v>
       </c>
       <c r="J70" s="6" t="inlineStr">
         <is>
-          <t>PENSKE AUTOMOTIVE GROUP VOTING INC</t>
+          <t>ROBERT HALF INC</t>
         </is>
       </c>
       <c r="K70" s="6" t="inlineStr">
         <is>
-          <t>Consumer Discretionary</t>
+          <t>Industrials</t>
         </is>
       </c>
       <c r="L70" s="6" t="inlineStr"/>
@@ -28489,20 +28531,20 @@
     <row r="71">
       <c r="H71" s="6" t="inlineStr">
         <is>
-          <t>RHI</t>
+          <t>PAG</t>
         </is>
       </c>
       <c r="I71" s="61" t="n">
-        <v>0.0008741300000000001</v>
+        <v>0.00087774</v>
       </c>
       <c r="J71" s="6" t="inlineStr">
         <is>
-          <t>ROBERT HALF INC</t>
+          <t>PENSKE AUTOMOTIVE GROUP VOTING INC</t>
         </is>
       </c>
       <c r="K71" s="6" t="inlineStr">
         <is>
-          <t>Industrials</t>
+          <t>Consumer Discretionary</t>
         </is>
       </c>
       <c r="L71" s="6" t="inlineStr"/>
@@ -28514,15 +28556,15 @@
     <row r="72">
       <c r="H72" s="6" t="inlineStr">
         <is>
-          <t>APAM</t>
+          <t>BANR</t>
         </is>
       </c>
       <c r="I72" s="61" t="n">
-        <v>0.0005806</v>
+        <v>0.00056875</v>
       </c>
       <c r="J72" s="6" t="inlineStr">
         <is>
-          <t>ARTISAN PARTNERS ASSET MANAGEMENT</t>
+          <t>BANNER CORP</t>
         </is>
       </c>
       <c r="K72" s="6" t="inlineStr">
@@ -28539,15 +28581,15 @@
     <row r="73">
       <c r="H73" s="6" t="inlineStr">
         <is>
-          <t>BANR</t>
+          <t>APAM</t>
         </is>
       </c>
       <c r="I73" s="61" t="n">
-        <v>0.00057219</v>
+        <v>0.00055786</v>
       </c>
       <c r="J73" s="6" t="inlineStr">
         <is>
-          <t>BANNER CORP</t>
+          <t>ARTISAN PARTNERS ASSET MANAGEMENT</t>
         </is>
       </c>
       <c r="K73" s="6" t="inlineStr">
@@ -28568,7 +28610,7 @@
         </is>
       </c>
       <c r="I74" s="61" t="n">
-        <v>0.00054473</v>
+        <v>0.0005433700000000001</v>
       </c>
       <c r="J74" s="6" t="inlineStr">
         <is>
@@ -28593,7 +28635,7 @@
         </is>
       </c>
       <c r="I75" s="61" t="n">
-        <v>0.0005197999999999999</v>
+        <v>0.00052626</v>
       </c>
       <c r="J75" s="6" t="inlineStr">
         <is>
@@ -28618,7 +28660,7 @@
         </is>
       </c>
       <c r="I76" s="61" t="n">
-        <v>0.0004995900000000001</v>
+        <v>0.00049683</v>
       </c>
       <c r="J76" s="6" t="inlineStr">
         <is>
@@ -28643,7 +28685,7 @@
         </is>
       </c>
       <c r="I77" s="61" t="n">
-        <v>0.00049819</v>
+        <v>0.0004948600000000001</v>
       </c>
       <c r="J77" s="6" t="inlineStr">
         <is>
@@ -28668,7 +28710,7 @@
         </is>
       </c>
       <c r="I78" s="61" t="n">
-        <v>0.0004946</v>
+        <v>0.0004922300000000001</v>
       </c>
       <c r="J78" s="6" t="inlineStr">
         <is>
@@ -28689,15 +28731,15 @@
     <row r="79">
       <c r="H79" s="6" t="inlineStr">
         <is>
-          <t>WU</t>
+          <t>AGM</t>
         </is>
       </c>
       <c r="I79" s="61" t="n">
-        <v>0.00048395</v>
+        <v>0.00048252</v>
       </c>
       <c r="J79" s="6" t="inlineStr">
         <is>
-          <t>WESTERN UNION</t>
+          <t>FEDERAL AGRICULTURAL MORTGAGE NON</t>
         </is>
       </c>
       <c r="K79" s="6" t="inlineStr">
@@ -28714,15 +28756,15 @@
     <row r="80">
       <c r="H80" s="6" t="inlineStr">
         <is>
-          <t>AGM</t>
+          <t>WU</t>
         </is>
       </c>
       <c r="I80" s="61" t="n">
-        <v>0.00048145</v>
+        <v>0.00048178</v>
       </c>
       <c r="J80" s="6" t="inlineStr">
         <is>
-          <t>FEDERAL AGRICULTURAL MORTGAGE NON</t>
+          <t>WESTERN UNION</t>
         </is>
       </c>
       <c r="K80" s="6" t="inlineStr">
@@ -28743,7 +28785,7 @@
         </is>
       </c>
       <c r="I81" s="61" t="n">
-        <v>0.00046591</v>
+        <v>0.0004638</v>
       </c>
       <c r="J81" s="6" t="inlineStr">
         <is>
@@ -28768,7 +28810,7 @@
         </is>
       </c>
       <c r="I82" s="61" t="n">
-        <v>0.00044001</v>
+        <v>0.00044671</v>
       </c>
       <c r="J82" s="6" t="inlineStr">
         <is>
@@ -28793,7 +28835,7 @@
         </is>
       </c>
       <c r="I83" s="61" t="n">
-        <v>0.0004335399999999999</v>
+        <v>0.00042943</v>
       </c>
       <c r="J83" s="6" t="inlineStr">
         <is>
@@ -28818,7 +28860,7 @@
         </is>
       </c>
       <c r="I84" s="61" t="n">
-        <v>0.00042875</v>
+        <v>0.000422</v>
       </c>
       <c r="J84" s="6" t="inlineStr">
         <is>
@@ -28843,7 +28885,7 @@
         </is>
       </c>
       <c r="I85" s="61" t="n">
-        <v>0.00038317</v>
+        <v>0.00037917</v>
       </c>
       <c r="J85" s="6" t="inlineStr">
         <is>
@@ -28868,7 +28910,7 @@
         </is>
       </c>
       <c r="I86" s="61" t="n">
-        <v>0.00036137</v>
+        <v>0.000358</v>
       </c>
       <c r="J86" s="6" t="inlineStr">
         <is>
@@ -28893,7 +28935,7 @@
         </is>
       </c>
       <c r="I87" s="61" t="n">
-        <v>0.00034331</v>
+        <v>0.00034581</v>
       </c>
       <c r="J87" s="6" t="inlineStr">
         <is>
@@ -28918,7 +28960,7 @@
         </is>
       </c>
       <c r="I88" s="61" t="n">
-        <v>0.00032477</v>
+        <v>0.00032008</v>
       </c>
       <c r="J88" s="6" t="inlineStr">
         <is>
@@ -28943,7 +28985,7 @@
         </is>
       </c>
       <c r="I89" s="61" t="n">
-        <v>0.00028576</v>
+        <v>0.00028273</v>
       </c>
       <c r="J89" s="6" t="inlineStr">
         <is>
@@ -28968,7 +29010,7 @@
         </is>
       </c>
       <c r="I90" s="61" t="n">
-        <v>0.00025686</v>
+        <v>0.00025775</v>
       </c>
       <c r="J90" s="6" t="inlineStr">
         <is>
@@ -28993,7 +29035,7 @@
         </is>
       </c>
       <c r="I91" s="61" t="n">
-        <v>0.0002567</v>
+        <v>0.00025635</v>
       </c>
       <c r="J91" s="6" t="inlineStr">
         <is>
@@ -29018,7 +29060,7 @@
         </is>
       </c>
       <c r="I92" s="61" t="n">
-        <v>0.00024435</v>
+        <v>0.00024348</v>
       </c>
       <c r="J92" s="6" t="inlineStr">
         <is>
@@ -29039,7 +29081,7 @@
         </is>
       </c>
       <c r="I93" s="61" t="n">
-        <v>0.00023328</v>
+        <v>0.00023104</v>
       </c>
       <c r="J93" s="6" t="inlineStr">
         <is>
@@ -29064,7 +29106,7 @@
         </is>
       </c>
       <c r="I94" s="61" t="n">
-        <v>0.00023229</v>
+        <v>0.00023021</v>
       </c>
       <c r="J94" s="6" t="inlineStr">
         <is>
@@ -29089,7 +29131,7 @@
         </is>
       </c>
       <c r="I95" s="61" t="n">
-        <v>0.00020862</v>
+        <v>0.00020731</v>
       </c>
       <c r="J95" s="6" t="inlineStr">
         <is>
@@ -29110,15 +29152,15 @@
     <row r="96">
       <c r="H96" s="6" t="inlineStr">
         <is>
-          <t>VRTS</t>
+          <t>THFF</t>
         </is>
       </c>
       <c r="I96" s="61" t="n">
-        <v>0.00020236</v>
+        <v>0.00019795</v>
       </c>
       <c r="J96" s="6" t="inlineStr">
         <is>
-          <t>VIRTUS INVESTMENT PARTNERS</t>
+          <t>FIRST FINANCIAL CORPORATION CORP</t>
         </is>
       </c>
       <c r="K96" s="6" t="inlineStr">
@@ -29135,15 +29177,15 @@
     <row r="97">
       <c r="H97" s="6" t="inlineStr">
         <is>
-          <t>IBCP</t>
+          <t>VRTS</t>
         </is>
       </c>
       <c r="I97" s="61" t="n">
-        <v>0.0002006</v>
+        <v>0.00019782</v>
       </c>
       <c r="J97" s="6" t="inlineStr">
         <is>
-          <t>INDEPENDENT BANK CORP</t>
+          <t>VIRTUS INVESTMENT PARTNERS</t>
         </is>
       </c>
       <c r="K97" s="6" t="inlineStr">
@@ -29160,15 +29202,15 @@
     <row r="98">
       <c r="H98" s="6" t="inlineStr">
         <is>
-          <t>THFF</t>
+          <t>IBCP</t>
         </is>
       </c>
       <c r="I98" s="61" t="n">
-        <v>0.00019921</v>
+        <v>0.00019772</v>
       </c>
       <c r="J98" s="6" t="inlineStr">
         <is>
-          <t>FIRST FINANCIAL CORPORATION CORP</t>
+          <t>INDEPENDENT BANK CORP</t>
         </is>
       </c>
       <c r="K98" s="6" t="inlineStr">
@@ -29189,7 +29231,7 @@
         </is>
       </c>
       <c r="I99" s="61" t="n">
-        <v>0.00016796</v>
+        <v>0.0001667</v>
       </c>
       <c r="J99" s="6" t="inlineStr">
         <is>
@@ -29214,7 +29256,7 @@
         </is>
       </c>
       <c r="I100" s="61" t="n">
-        <v>0.00013436</v>
+        <v>0.00013458</v>
       </c>
       <c r="J100" s="6" t="inlineStr">
         <is>
@@ -29239,7 +29281,7 @@
         </is>
       </c>
       <c r="I101" s="61" t="n">
-        <v>0.00012374</v>
+        <v>0.0001233</v>
       </c>
       <c r="J101" s="6" t="inlineStr">
         <is>
@@ -29260,7 +29302,7 @@
         </is>
       </c>
       <c r="I102" s="61" t="n">
-        <v>0.00011731</v>
+        <v>0.00011551</v>
       </c>
       <c r="J102" s="6" t="inlineStr">
         <is>
@@ -29285,7 +29327,7 @@
         </is>
       </c>
       <c r="I103" s="61" t="n">
-        <v>0.00010297</v>
+        <v>0.00010322</v>
       </c>
       <c r="J103" s="6" t="inlineStr">
         <is>
@@ -29310,7 +29352,7 @@
         </is>
       </c>
       <c r="I104" s="61" t="n">
-        <v>8.899e-05</v>
+        <v>9.028e-05</v>
       </c>
       <c r="J104" s="6" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
데이터 갱신: holdings,official,prices (2026-10-15)
</commit_message>
<xml_diff>
--- a/downloads/schd_dividend_tracker.xlsx
+++ b/downloads/schd_dividend_tracker.xlsx
@@ -1724,7 +1724,7 @@
     <row r="3">
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>최종 갱신: 2026-10-14 · 반영 범위: 2012년 1분기 ~ 2026년 3분기 (배당락 2026-09-23) · GitHub Actions 자동 생성</t>
+          <t>최종 갱신: 2026-10-15 · 반영 범위: 2012년 1분기 ~ 2026년 3분기 (배당락 2026-09-23) · GitHub Actions 자동 생성</t>
         </is>
       </c>
     </row>
@@ -5818,7 +5818,7 @@
       </c>
       <c r="H1" s="2" t="inlineStr">
         <is>
-          <t>출처: Yahoo Finance (종가: 주식분할 반영·배당 미조정 / adj: 배당 재투자 반영 수정주가) · 기준일 2026-10-08 · 3:1 분할(2024-10-11) 반영 가격</t>
+          <t>출처: Yahoo Finance (종가: 주식분할 반영·배당 미조정 / adj: 배당 재투자 반영 수정주가) · 기준일 2026-10-14 · 3:1 분할(2024-10-11) 반영 가격</t>
         </is>
       </c>
     </row>
@@ -6243,7 +6243,7 @@
         <v>10.9</v>
       </c>
       <c r="D22" s="77" t="n">
-        <v>7.1037</v>
+        <v>7.1038</v>
       </c>
       <c r="E22" s="58">
         <f>C22/C10-1</f>
@@ -7179,7 +7179,7 @@
         <v>14.1033</v>
       </c>
       <c r="D61" s="77" t="n">
-        <v>10.0736</v>
+        <v>10.0735</v>
       </c>
       <c r="E61" s="58">
         <f>C61/C49-1</f>
@@ -7995,7 +7995,7 @@
         <v>17.9833</v>
       </c>
       <c r="D95" s="77" t="n">
-        <v>13.9255</v>
+        <v>13.9254</v>
       </c>
       <c r="E95" s="58">
         <f>C95/C83-1</f>
@@ -8067,7 +8067,7 @@
         <v>18.5067</v>
       </c>
       <c r="D98" s="77" t="n">
-        <v>14.4594</v>
+        <v>14.4593</v>
       </c>
       <c r="E98" s="58">
         <f>C98/C86-1</f>
@@ -8187,7 +8187,7 @@
         <v>14.9933</v>
       </c>
       <c r="D103" s="77" t="n">
-        <v>11.9339</v>
+        <v>11.9338</v>
       </c>
       <c r="E103" s="58">
         <f>C103/C91-1</f>
@@ -10077,13 +10077,13 @@
         </is>
       </c>
       <c r="B182" s="56" t="n">
-        <v>46303</v>
+        <v>46309</v>
       </c>
       <c r="C182" s="76" t="n">
-        <v>33.15</v>
+        <v>33.71</v>
       </c>
       <c r="D182" s="77" t="n">
-        <v>33.15</v>
+        <v>33.71</v>
       </c>
       <c r="E182" s="58">
         <f>C182/C170-1</f>
@@ -11996,11 +11996,11 @@
         </is>
       </c>
       <c r="B34" s="19" t="n">
-        <v>0.0337</v>
+        <v>0.033</v>
       </c>
       <c r="C34" s="2" t="inlineStr">
         <is>
-          <t>2026-10-07 기준 · 최근 30일 순투자수익(보수 차감) 연 환산</t>
+          <t>2026-10-13 기준 · 최근 30일 순투자수익(보수 차감) 연 환산</t>
         </is>
       </c>
     </row>
@@ -12011,11 +12011,11 @@
         </is>
       </c>
       <c r="B35" s="19" t="n">
-        <v>0.03</v>
+        <v>0.0324</v>
       </c>
       <c r="C35" s="2" t="inlineStr">
         <is>
-          <t>2026-08-31 기준 · 최근 12개월 분배금 ÷ 기준일 NAV</t>
+          <t>2026-09-30 기준 · 최근 12개월 분배금 ÷ 기준일 NAV</t>
         </is>
       </c>
     </row>
@@ -26257,11 +26257,11 @@
         </is>
       </c>
       <c r="B2" s="49" t="n">
-        <v>46308</v>
+        <v>46309</v>
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>← 이 날 종가로 계산한 비중. 그날 공식 파일을 못 받아 Schwab 공식 보유종목 CSV(2026-10-12)의 보유 주식 수 × 종가로 계산했습니다.</t>
+          <t>← 이 날 종가로 계산한 비중. 그날 공식 파일을 못 받아 Schwab 공식 보유종목 CSV(2026-10-13)의 보유 주식 수 × 종가로 계산했습니다.</t>
         </is>
       </c>
     </row>
@@ -26358,7 +26358,7 @@
         </is>
       </c>
       <c r="I5" s="61" t="n">
-        <v>0.04708691</v>
+        <v>0.04543222</v>
       </c>
       <c r="J5" s="6" t="inlineStr">
         <is>
@@ -26412,25 +26412,25 @@
       </c>
       <c r="H6" s="6" t="inlineStr">
         <is>
-          <t>QCOM</t>
+          <t>PG</t>
         </is>
       </c>
       <c r="I6" s="61" t="n">
-        <v>0.04337273</v>
+        <v>0.04373126</v>
       </c>
       <c r="J6" s="6" t="inlineStr">
         <is>
-          <t>QUALCOMM</t>
+          <t>PROCTER &amp; GAMBLE</t>
         </is>
       </c>
       <c r="K6" s="6" t="inlineStr">
         <is>
-          <t>Information Technology</t>
+          <t>Consumer Staples</t>
         </is>
       </c>
       <c r="L6" s="6" t="inlineStr">
         <is>
-          <t>퀄컴</t>
+          <t>프록터앤드갬블</t>
         </is>
       </c>
       <c r="M6" s="7">
@@ -26470,25 +26470,25 @@
       </c>
       <c r="H7" s="6" t="inlineStr">
         <is>
-          <t>PG</t>
+          <t>CVX</t>
         </is>
       </c>
       <c r="I7" s="61" t="n">
-        <v>0.04320501</v>
+        <v>0.04324578</v>
       </c>
       <c r="J7" s="6" t="inlineStr">
         <is>
-          <t>PROCTER &amp; GAMBLE</t>
+          <t>CHEVRON</t>
         </is>
       </c>
       <c r="K7" s="6" t="inlineStr">
         <is>
-          <t>Consumer Staples</t>
+          <t>Energy</t>
         </is>
       </c>
       <c r="L7" s="6" t="inlineStr">
         <is>
-          <t>프록터앤드갬블</t>
+          <t>셰브론</t>
         </is>
       </c>
       <c r="M7" s="7">
@@ -26528,25 +26528,25 @@
       </c>
       <c r="H8" s="6" t="inlineStr">
         <is>
-          <t>CVX</t>
+          <t>KO</t>
         </is>
       </c>
       <c r="I8" s="61" t="n">
-        <v>0.0428515</v>
+        <v>0.04290234</v>
       </c>
       <c r="J8" s="6" t="inlineStr">
         <is>
-          <t>CHEVRON</t>
+          <t>COCA-COLA</t>
         </is>
       </c>
       <c r="K8" s="6" t="inlineStr">
         <is>
-          <t>Energy</t>
+          <t>Consumer Staples</t>
         </is>
       </c>
       <c r="L8" s="6" t="inlineStr">
         <is>
-          <t>셰브론</t>
+          <t>코카콜라</t>
         </is>
       </c>
       <c r="M8" s="7">
@@ -26590,7 +26590,7 @@
         </is>
       </c>
       <c r="I9" s="61" t="n">
-        <v>0.04274977</v>
+        <v>0.04273807</v>
       </c>
       <c r="J9" s="6" t="inlineStr">
         <is>
@@ -26644,25 +26644,25 @@
       </c>
       <c r="H10" s="6" t="inlineStr">
         <is>
-          <t>KO</t>
+          <t>QCOM</t>
         </is>
       </c>
       <c r="I10" s="61" t="n">
-        <v>0.04256384</v>
+        <v>0.04189318</v>
       </c>
       <c r="J10" s="6" t="inlineStr">
         <is>
-          <t>COCA-COLA</t>
+          <t>QUALCOMM</t>
         </is>
       </c>
       <c r="K10" s="6" t="inlineStr">
         <is>
-          <t>Consumer Staples</t>
+          <t>Information Technology</t>
         </is>
       </c>
       <c r="L10" s="6" t="inlineStr">
         <is>
-          <t>코카콜라</t>
+          <t>퀄컴</t>
         </is>
       </c>
       <c r="M10" s="7">
@@ -26706,7 +26706,7 @@
         </is>
       </c>
       <c r="I11" s="61" t="n">
-        <v>0.0393964</v>
+        <v>0.04083037</v>
       </c>
       <c r="J11" s="6" t="inlineStr">
         <is>
@@ -26764,7 +26764,7 @@
         </is>
       </c>
       <c r="I12" s="61" t="n">
-        <v>0.03902534</v>
+        <v>0.04008606999999999</v>
       </c>
       <c r="J12" s="6" t="inlineStr">
         <is>
@@ -26822,7 +26822,7 @@
         </is>
       </c>
       <c r="I13" s="61" t="n">
-        <v>0.03885666</v>
+        <v>0.03968896</v>
       </c>
       <c r="J13" s="6" t="inlineStr">
         <is>
@@ -26880,7 +26880,7 @@
         </is>
       </c>
       <c r="I14" s="61" t="n">
-        <v>0.03871495</v>
+        <v>0.03844721</v>
       </c>
       <c r="J14" s="6" t="inlineStr">
         <is>
@@ -26928,7 +26928,7 @@
         </is>
       </c>
       <c r="I15" s="61" t="n">
-        <v>0.03846246</v>
+        <v>0.03826877</v>
       </c>
       <c r="J15" s="6" t="inlineStr">
         <is>
@@ -26976,7 +26976,7 @@
         </is>
       </c>
       <c r="I16" s="61" t="n">
-        <v>0.03775924</v>
+        <v>0.03794526</v>
       </c>
       <c r="J16" s="6" t="inlineStr">
         <is>
@@ -27014,7 +27014,7 @@
         </is>
       </c>
       <c r="I17" s="61" t="n">
-        <v>0.03612815</v>
+        <v>0.03648387</v>
       </c>
       <c r="J17" s="6" t="inlineStr">
         <is>
@@ -27052,7 +27052,7 @@
         </is>
       </c>
       <c r="I18" s="61" t="n">
-        <v>0.03300566</v>
+        <v>0.03287692</v>
       </c>
       <c r="J18" s="6" t="inlineStr">
         <is>
@@ -27081,7 +27081,7 @@
         </is>
       </c>
       <c r="I19" s="61" t="n">
-        <v>0.03017718</v>
+        <v>0.03051891</v>
       </c>
       <c r="J19" s="6" t="inlineStr">
         <is>
@@ -27115,7 +27115,7 @@
         </is>
       </c>
       <c r="I20" s="61" t="n">
-        <v>0.02923612</v>
+        <v>0.03026495</v>
       </c>
       <c r="J20" s="6" t="inlineStr">
         <is>
@@ -27154,7 +27154,7 @@
         </is>
       </c>
       <c r="I21" s="61" t="n">
-        <v>0.02768124</v>
+        <v>0.02783255</v>
       </c>
       <c r="J21" s="6" t="inlineStr">
         <is>
@@ -27192,7 +27192,7 @@
         </is>
       </c>
       <c r="I22" s="61" t="n">
-        <v>0.02585262</v>
+        <v>0.02650835</v>
       </c>
       <c r="J22" s="6" t="inlineStr">
         <is>
@@ -27226,25 +27226,25 @@
       </c>
       <c r="H23" s="6" t="inlineStr">
         <is>
-          <t>BX</t>
+          <t>EOG</t>
         </is>
       </c>
       <c r="I23" s="61" t="n">
-        <v>0.02084944</v>
+        <v>0.02021378</v>
       </c>
       <c r="J23" s="6" t="inlineStr">
         <is>
-          <t>BLACKSTONE</t>
+          <t>EOG RESOURCES</t>
         </is>
       </c>
       <c r="K23" s="6" t="inlineStr">
         <is>
-          <t>Financials</t>
+          <t>Energy</t>
         </is>
       </c>
       <c r="L23" s="6" t="inlineStr">
         <is>
-          <t>블랙스톤</t>
+          <t>EOG 리소시스</t>
         </is>
       </c>
       <c r="M23" s="7">
@@ -27264,25 +27264,25 @@
       </c>
       <c r="H24" s="6" t="inlineStr">
         <is>
-          <t>EOG</t>
+          <t>BX</t>
         </is>
       </c>
       <c r="I24" s="61" t="n">
-        <v>0.02029086</v>
+        <v>0.01992557</v>
       </c>
       <c r="J24" s="6" t="inlineStr">
         <is>
-          <t>EOG RESOURCES</t>
+          <t>BLACKSTONE</t>
         </is>
       </c>
       <c r="K24" s="6" t="inlineStr">
         <is>
-          <t>Energy</t>
+          <t>Financials</t>
         </is>
       </c>
       <c r="L24" s="6" t="inlineStr">
         <is>
-          <t>EOG 리소시스</t>
+          <t>블랙스톤</t>
         </is>
       </c>
       <c r="M24" s="7">
@@ -27306,7 +27306,7 @@
         </is>
       </c>
       <c r="I25" s="61" t="n">
-        <v>0.01866352</v>
+        <v>0.01862003</v>
       </c>
       <c r="J25" s="6" t="inlineStr">
         <is>
@@ -27344,7 +27344,7 @@
         </is>
       </c>
       <c r="I26" s="61" t="n">
-        <v>0.01828045</v>
+        <v>0.01799412</v>
       </c>
       <c r="J26" s="6" t="inlineStr">
         <is>
@@ -27382,7 +27382,7 @@
         </is>
       </c>
       <c r="I27" s="61" t="n">
-        <v>0.01793923</v>
+        <v>0.0179383</v>
       </c>
       <c r="J27" s="6" t="inlineStr">
         <is>
@@ -27420,7 +27420,7 @@
         </is>
       </c>
       <c r="I28" s="61" t="n">
-        <v>0.01743452</v>
+        <v>0.01763029</v>
       </c>
       <c r="J28" s="6" t="inlineStr">
         <is>
@@ -27458,7 +27458,7 @@
         </is>
       </c>
       <c r="I29" s="61" t="n">
-        <v>0.01490483</v>
+        <v>0.01491347</v>
       </c>
       <c r="J29" s="6" t="inlineStr">
         <is>
@@ -27496,7 +27496,7 @@
         </is>
       </c>
       <c r="I30" s="61" t="n">
-        <v>0.01486642</v>
+        <v>0.01448985</v>
       </c>
       <c r="J30" s="6" t="inlineStr">
         <is>
@@ -27530,7 +27530,7 @@
         </is>
       </c>
       <c r="I31" s="61" t="n">
-        <v>0.01394894</v>
+        <v>0.01372431</v>
       </c>
       <c r="J31" s="6" t="inlineStr">
         <is>
@@ -27555,7 +27555,7 @@
         </is>
       </c>
       <c r="I32" s="61" t="n">
-        <v>0.01196931</v>
+        <v>0.01179604</v>
       </c>
       <c r="J32" s="6" t="inlineStr">
         <is>
@@ -27585,7 +27585,7 @@
         </is>
       </c>
       <c r="I33" s="61" t="n">
-        <v>0.01150248</v>
+        <v>0.01125153</v>
       </c>
       <c r="J33" s="6" t="inlineStr">
         <is>
@@ -27610,7 +27610,7 @@
         </is>
       </c>
       <c r="I34" s="61" t="n">
-        <v>0.01012723</v>
+        <v>0.01007502</v>
       </c>
       <c r="J34" s="6" t="inlineStr">
         <is>
@@ -27635,7 +27635,7 @@
         </is>
       </c>
       <c r="I35" s="61" t="n">
-        <v>0.008589940000000001</v>
+        <v>0.008670310000000001</v>
       </c>
       <c r="J35" s="6" t="inlineStr">
         <is>
@@ -27660,7 +27660,7 @@
         </is>
       </c>
       <c r="I36" s="61" t="n">
-        <v>0.008255780000000001</v>
+        <v>0.008263100000000001</v>
       </c>
       <c r="J36" s="6" t="inlineStr">
         <is>
@@ -27681,15 +27681,15 @@
     <row r="37">
       <c r="H37" s="6" t="inlineStr">
         <is>
-          <t>ARES</t>
+          <t>CINF</t>
         </is>
       </c>
       <c r="I37" s="61" t="n">
-        <v>0.00653969</v>
+        <v>0.00639322</v>
       </c>
       <c r="J37" s="6" t="inlineStr">
         <is>
-          <t>ARES MANAGEMENT CLASS A</t>
+          <t>CINCINNATI FINANCIAL</t>
         </is>
       </c>
       <c r="K37" s="6" t="inlineStr">
@@ -27706,15 +27706,15 @@
     <row r="38">
       <c r="H38" s="6" t="inlineStr">
         <is>
-          <t>CINF</t>
+          <t>ARES</t>
         </is>
       </c>
       <c r="I38" s="61" t="n">
-        <v>0.00642043</v>
+        <v>0.00629656</v>
       </c>
       <c r="J38" s="6" t="inlineStr">
         <is>
-          <t>CINCINNATI FINANCIAL</t>
+          <t>ARES MANAGEMENT CLASS A</t>
         </is>
       </c>
       <c r="K38" s="6" t="inlineStr">
@@ -27735,7 +27735,7 @@
         </is>
       </c>
       <c r="I39" s="61" t="n">
-        <v>0.006024939999999999</v>
+        <v>0.00600621</v>
       </c>
       <c r="J39" s="6" t="inlineStr">
         <is>
@@ -27760,7 +27760,7 @@
         </is>
       </c>
       <c r="I40" s="61" t="n">
-        <v>0.005895559999999999</v>
+        <v>0.00591714</v>
       </c>
       <c r="J40" s="6" t="inlineStr">
         <is>
@@ -27785,7 +27785,7 @@
         </is>
       </c>
       <c r="I41" s="61" t="n">
-        <v>0.00581152</v>
+        <v>0.0057256</v>
       </c>
       <c r="J41" s="6" t="inlineStr">
         <is>
@@ -27810,7 +27810,7 @@
         </is>
       </c>
       <c r="I42" s="61" t="n">
-        <v>0.005462320000000001</v>
+        <v>0.00531119</v>
       </c>
       <c r="J42" s="6" t="inlineStr">
         <is>
@@ -27835,7 +27835,7 @@
         </is>
       </c>
       <c r="I43" s="61" t="n">
-        <v>0.00529678</v>
+        <v>0.00522323</v>
       </c>
       <c r="J43" s="6" t="inlineStr">
         <is>
@@ -27860,7 +27860,7 @@
         </is>
       </c>
       <c r="I44" s="61" t="n">
-        <v>0.00500685</v>
+        <v>0.00493398</v>
       </c>
       <c r="J44" s="6" t="inlineStr">
         <is>
@@ -27885,7 +27885,7 @@
         </is>
       </c>
       <c r="I45" s="61" t="n">
-        <v>0.00485186</v>
+        <v>0.00479629</v>
       </c>
       <c r="J45" s="6" t="inlineStr">
         <is>
@@ -27910,7 +27910,7 @@
         </is>
       </c>
       <c r="I46" s="61" t="n">
-        <v>0.00475145</v>
+        <v>0.00469995</v>
       </c>
       <c r="J46" s="6" t="inlineStr">
         <is>
@@ -27935,7 +27935,7 @@
         </is>
       </c>
       <c r="I47" s="61" t="n">
-        <v>0.00439892</v>
+        <v>0.00440964</v>
       </c>
       <c r="J47" s="6" t="inlineStr">
         <is>
@@ -27956,20 +27956,20 @@
     <row r="48">
       <c r="H48" s="6" t="inlineStr">
         <is>
-          <t>EWBC</t>
+          <t>GIS</t>
         </is>
       </c>
       <c r="I48" s="61" t="n">
-        <v>0.00432773</v>
+        <v>0.00429147</v>
       </c>
       <c r="J48" s="6" t="inlineStr">
         <is>
-          <t>EAST WEST BANCORP</t>
+          <t>GENERAL MILLS INC</t>
         </is>
       </c>
       <c r="K48" s="6" t="inlineStr">
         <is>
-          <t>Financials</t>
+          <t>Consumer Staples</t>
         </is>
       </c>
       <c r="L48" s="6" t="inlineStr"/>
@@ -27981,20 +27981,20 @@
     <row r="49">
       <c r="H49" s="6" t="inlineStr">
         <is>
-          <t>GIS</t>
+          <t>EWBC</t>
         </is>
       </c>
       <c r="I49" s="61" t="n">
-        <v>0.00429871</v>
+        <v>0.00426734</v>
       </c>
       <c r="J49" s="6" t="inlineStr">
         <is>
-          <t>GENERAL MILLS INC</t>
+          <t>EAST WEST BANCORP</t>
         </is>
       </c>
       <c r="K49" s="6" t="inlineStr">
         <is>
-          <t>Consumer Staples</t>
+          <t>Financials</t>
         </is>
       </c>
       <c r="L49" s="6" t="inlineStr"/>
@@ -28010,7 +28010,7 @@
         </is>
       </c>
       <c r="I50" s="61" t="n">
-        <v>0.00424809</v>
+        <v>0.00414792</v>
       </c>
       <c r="J50" s="6" t="inlineStr">
         <is>
@@ -28035,7 +28035,7 @@
         </is>
       </c>
       <c r="I51" s="61" t="n">
-        <v>0.00262032</v>
+        <v>0.00262495</v>
       </c>
       <c r="J51" s="6" t="inlineStr">
         <is>
@@ -28056,15 +28056,15 @@
     <row r="52">
       <c r="H52" s="6" t="inlineStr">
         <is>
-          <t>FNF</t>
+          <t>AFG</t>
         </is>
       </c>
       <c r="I52" s="61" t="n">
-        <v>0.00252232</v>
+        <v>0.00250235</v>
       </c>
       <c r="J52" s="6" t="inlineStr">
         <is>
-          <t>FIDELITY NATIONAL FINANCIAL INC</t>
+          <t>AMERICAN FINANCIAL GROUP</t>
         </is>
       </c>
       <c r="K52" s="6" t="inlineStr">
@@ -28081,15 +28081,15 @@
     <row r="53">
       <c r="H53" s="6" t="inlineStr">
         <is>
-          <t>AFG</t>
+          <t>FNF</t>
         </is>
       </c>
       <c r="I53" s="61" t="n">
-        <v>0.00251094</v>
+        <v>0.00249803</v>
       </c>
       <c r="J53" s="6" t="inlineStr">
         <is>
-          <t>AMERICAN FINANCIAL GROUP</t>
+          <t>FIDELITY NATIONAL FINANCIAL INC</t>
         </is>
       </c>
       <c r="K53" s="6" t="inlineStr">
@@ -28110,7 +28110,7 @@
         </is>
       </c>
       <c r="I54" s="61" t="n">
-        <v>0.00219546</v>
+        <v>0.00215943</v>
       </c>
       <c r="J54" s="6" t="inlineStr">
         <is>
@@ -28135,7 +28135,7 @@
         </is>
       </c>
       <c r="I55" s="61" t="n">
-        <v>0.00213924</v>
+        <v>0.00213145</v>
       </c>
       <c r="J55" s="6" t="inlineStr">
         <is>
@@ -28160,7 +28160,7 @@
         </is>
       </c>
       <c r="I56" s="61" t="n">
-        <v>0.00201503</v>
+        <v>0.00197997</v>
       </c>
       <c r="J56" s="6" t="inlineStr">
         <is>
@@ -28185,7 +28185,7 @@
         </is>
       </c>
       <c r="I57" s="61" t="n">
-        <v>0.00191453</v>
+        <v>0.00189248</v>
       </c>
       <c r="J57" s="6" t="inlineStr">
         <is>
@@ -28210,7 +28210,7 @@
         </is>
       </c>
       <c r="I58" s="61" t="n">
-        <v>0.00152937</v>
+        <v>0.00151817</v>
       </c>
       <c r="J58" s="6" t="inlineStr">
         <is>
@@ -28235,7 +28235,7 @@
         </is>
       </c>
       <c r="I59" s="61" t="n">
-        <v>0.00150924</v>
+        <v>0.00148962</v>
       </c>
       <c r="J59" s="6" t="inlineStr">
         <is>
@@ -28260,7 +28260,7 @@
         </is>
       </c>
       <c r="I60" s="61" t="n">
-        <v>0.00150688</v>
+        <v>0.00148646</v>
       </c>
       <c r="J60" s="6" t="inlineStr">
         <is>
@@ -28285,7 +28285,7 @@
         </is>
       </c>
       <c r="I61" s="61" t="n">
-        <v>0.00137352</v>
+        <v>0.00133141</v>
       </c>
       <c r="J61" s="6" t="inlineStr">
         <is>
@@ -28310,11 +28310,11 @@
         </is>
       </c>
       <c r="I62" s="61" t="n">
-        <v>0.0013302</v>
+        <v>0.00132548</v>
       </c>
       <c r="J62" s="6" t="inlineStr">
         <is>
-          <t>MURPHY OIL CORP</t>
+          <t>MURPHY OIL</t>
         </is>
       </c>
       <c r="K62" s="6" t="inlineStr">
@@ -28335,7 +28335,7 @@
         </is>
       </c>
       <c r="I63" s="61" t="n">
-        <v>0.00117587</v>
+        <v>0.00116183</v>
       </c>
       <c r="J63" s="6" t="inlineStr">
         <is>
@@ -28360,7 +28360,7 @@
         </is>
       </c>
       <c r="I64" s="61" t="n">
-        <v>0.00115621</v>
+        <v>0.00114039</v>
       </c>
       <c r="J64" s="6" t="inlineStr">
         <is>
@@ -28385,7 +28385,7 @@
         </is>
       </c>
       <c r="I65" s="61" t="n">
-        <v>0.00105213</v>
+        <v>0.00100205</v>
       </c>
       <c r="J65" s="6" t="inlineStr">
         <is>
@@ -28410,7 +28410,7 @@
         </is>
       </c>
       <c r="I66" s="61" t="n">
-        <v>0.0009912600000000001</v>
+        <v>0.0009784500000000001</v>
       </c>
       <c r="J66" s="6" t="inlineStr">
         <is>
@@ -28435,7 +28435,7 @@
         </is>
       </c>
       <c r="I67" s="61" t="n">
-        <v>0.00093461</v>
+        <v>0.00091228</v>
       </c>
       <c r="J67" s="6" t="inlineStr">
         <is>
@@ -28460,7 +28460,7 @@
         </is>
       </c>
       <c r="I68" s="61" t="n">
-        <v>0.0009285499999999999</v>
+        <v>0.00089414</v>
       </c>
       <c r="J68" s="6" t="inlineStr">
         <is>
@@ -28485,7 +28485,7 @@
         </is>
       </c>
       <c r="I69" s="61" t="n">
-        <v>0.00090456</v>
+        <v>0.00088975</v>
       </c>
       <c r="J69" s="6" t="inlineStr">
         <is>
@@ -28510,7 +28510,7 @@
         </is>
       </c>
       <c r="I70" s="61" t="n">
-        <v>0.00088303</v>
+        <v>0.00087711</v>
       </c>
       <c r="J70" s="6" t="inlineStr">
         <is>
@@ -28535,7 +28535,7 @@
         </is>
       </c>
       <c r="I71" s="61" t="n">
-        <v>0.00087774</v>
+        <v>0.00086469</v>
       </c>
       <c r="J71" s="6" t="inlineStr">
         <is>
@@ -28560,7 +28560,7 @@
         </is>
       </c>
       <c r="I72" s="61" t="n">
-        <v>0.00056875</v>
+        <v>0.00056073</v>
       </c>
       <c r="J72" s="6" t="inlineStr">
         <is>
@@ -28585,7 +28585,7 @@
         </is>
       </c>
       <c r="I73" s="61" t="n">
-        <v>0.00055786</v>
+        <v>0.00056072</v>
       </c>
       <c r="J73" s="6" t="inlineStr">
         <is>
@@ -28610,7 +28610,7 @@
         </is>
       </c>
       <c r="I74" s="61" t="n">
-        <v>0.0005433700000000001</v>
+        <v>0.00053834</v>
       </c>
       <c r="J74" s="6" t="inlineStr">
         <is>
@@ -28635,7 +28635,7 @@
         </is>
       </c>
       <c r="I75" s="61" t="n">
-        <v>0.00052626</v>
+        <v>0.00052264</v>
       </c>
       <c r="J75" s="6" t="inlineStr">
         <is>
@@ -28660,7 +28660,7 @@
         </is>
       </c>
       <c r="I76" s="61" t="n">
-        <v>0.00049683</v>
+        <v>0.0004929299999999999</v>
       </c>
       <c r="J76" s="6" t="inlineStr">
         <is>
@@ -28685,7 +28685,7 @@
         </is>
       </c>
       <c r="I77" s="61" t="n">
-        <v>0.0004948600000000001</v>
+        <v>0.00049172</v>
       </c>
       <c r="J77" s="6" t="inlineStr">
         <is>
@@ -28706,15 +28706,15 @@
     <row r="78">
       <c r="H78" s="6" t="inlineStr">
         <is>
-          <t>CNS</t>
+          <t>AGM</t>
         </is>
       </c>
       <c r="I78" s="61" t="n">
-        <v>0.0004922300000000001</v>
+        <v>0.00047649</v>
       </c>
       <c r="J78" s="6" t="inlineStr">
         <is>
-          <t>COHEN &amp; STEERS INC</t>
+          <t>FEDERAL AGRICULTURAL MORTGAGE NON</t>
         </is>
       </c>
       <c r="K78" s="6" t="inlineStr">
@@ -28731,15 +28731,15 @@
     <row r="79">
       <c r="H79" s="6" t="inlineStr">
         <is>
-          <t>AGM</t>
+          <t>WU</t>
         </is>
       </c>
       <c r="I79" s="61" t="n">
-        <v>0.00048252</v>
+        <v>0.00047286</v>
       </c>
       <c r="J79" s="6" t="inlineStr">
         <is>
-          <t>FEDERAL AGRICULTURAL MORTGAGE NON</t>
+          <t>WESTERN UNION</t>
         </is>
       </c>
       <c r="K79" s="6" t="inlineStr">
@@ -28756,15 +28756,15 @@
     <row r="80">
       <c r="H80" s="6" t="inlineStr">
         <is>
-          <t>WU</t>
+          <t>CNS</t>
         </is>
       </c>
       <c r="I80" s="61" t="n">
-        <v>0.00048178</v>
+        <v>0.00046962</v>
       </c>
       <c r="J80" s="6" t="inlineStr">
         <is>
-          <t>WESTERN UNION</t>
+          <t>COHEN &amp; STEERS INC</t>
         </is>
       </c>
       <c r="K80" s="6" t="inlineStr">
@@ -28785,7 +28785,7 @@
         </is>
       </c>
       <c r="I81" s="61" t="n">
-        <v>0.0004638</v>
+        <v>0.00045944</v>
       </c>
       <c r="J81" s="6" t="inlineStr">
         <is>
@@ -28810,7 +28810,7 @@
         </is>
       </c>
       <c r="I82" s="61" t="n">
-        <v>0.00044671</v>
+        <v>0.00044368</v>
       </c>
       <c r="J82" s="6" t="inlineStr">
         <is>
@@ -28835,7 +28835,7 @@
         </is>
       </c>
       <c r="I83" s="61" t="n">
-        <v>0.00042943</v>
+        <v>0.00042389</v>
       </c>
       <c r="J83" s="6" t="inlineStr">
         <is>
@@ -28860,7 +28860,7 @@
         </is>
       </c>
       <c r="I84" s="61" t="n">
-        <v>0.000422</v>
+        <v>0.00041283</v>
       </c>
       <c r="J84" s="6" t="inlineStr">
         <is>
@@ -28885,7 +28885,7 @@
         </is>
       </c>
       <c r="I85" s="61" t="n">
-        <v>0.00037917</v>
+        <v>0.00037643</v>
       </c>
       <c r="J85" s="6" t="inlineStr">
         <is>
@@ -28910,7 +28910,7 @@
         </is>
       </c>
       <c r="I86" s="61" t="n">
-        <v>0.000358</v>
+        <v>0.0003552</v>
       </c>
       <c r="J86" s="6" t="inlineStr">
         <is>
@@ -28935,7 +28935,7 @@
         </is>
       </c>
       <c r="I87" s="61" t="n">
-        <v>0.00034581</v>
+        <v>0.00034336</v>
       </c>
       <c r="J87" s="6" t="inlineStr">
         <is>
@@ -28960,7 +28960,7 @@
         </is>
       </c>
       <c r="I88" s="61" t="n">
-        <v>0.00032008</v>
+        <v>0.00031676</v>
       </c>
       <c r="J88" s="6" t="inlineStr">
         <is>
@@ -28985,7 +28985,7 @@
         </is>
       </c>
       <c r="I89" s="61" t="n">
-        <v>0.00028273</v>
+        <v>0.00027823</v>
       </c>
       <c r="J89" s="6" t="inlineStr">
         <is>
@@ -29006,22 +29006,18 @@
     <row r="90">
       <c r="H90" s="6" t="inlineStr">
         <is>
-          <t>WEN</t>
+          <t>GVMXX</t>
         </is>
       </c>
       <c r="I90" s="61" t="n">
-        <v>0.00025775</v>
+        <v>0.00026386</v>
       </c>
       <c r="J90" s="6" t="inlineStr">
         <is>
-          <t>WENDYS</t>
-        </is>
-      </c>
-      <c r="K90" s="6" t="inlineStr">
-        <is>
-          <t>Consumer Discretionary</t>
-        </is>
-      </c>
+          <t>SSC GOVERNMENT MM GVMXX</t>
+        </is>
+      </c>
+      <c r="K90" s="6" t="inlineStr"/>
       <c r="L90" s="6" t="inlineStr"/>
       <c r="M90" s="7">
         <f>IF(H90="","",IFERROR(VLOOKUP(K90,$P$5:$Q$15,2,FALSE),"현금·선물"))</f>
@@ -29031,20 +29027,20 @@
     <row r="91">
       <c r="H91" s="6" t="inlineStr">
         <is>
-          <t>CNA</t>
+          <t>WEN</t>
         </is>
       </c>
       <c r="I91" s="61" t="n">
-        <v>0.00025635</v>
+        <v>0.00025869</v>
       </c>
       <c r="J91" s="6" t="inlineStr">
         <is>
-          <t>CNA FINANCIAL CORP</t>
+          <t>WENDYS</t>
         </is>
       </c>
       <c r="K91" s="6" t="inlineStr">
         <is>
-          <t>Financials</t>
+          <t>Consumer Discretionary</t>
         </is>
       </c>
       <c r="L91" s="6" t="inlineStr"/>
@@ -29056,18 +29052,22 @@
     <row r="92">
       <c r="H92" s="6" t="inlineStr">
         <is>
-          <t>GVMXX</t>
+          <t>CNA</t>
         </is>
       </c>
       <c r="I92" s="61" t="n">
-        <v>0.00024348</v>
+        <v>0.00025645</v>
       </c>
       <c r="J92" s="6" t="inlineStr">
         <is>
-          <t>SSC GOVERNMENT MM GVMXX</t>
-        </is>
-      </c>
-      <c r="K92" s="6" t="inlineStr"/>
+          <t>CNA FINANCIAL CORP</t>
+        </is>
+      </c>
+      <c r="K92" s="6" t="inlineStr">
+        <is>
+          <t>Financials</t>
+        </is>
+      </c>
       <c r="L92" s="6" t="inlineStr"/>
       <c r="M92" s="7">
         <f>IF(H92="","",IFERROR(VLOOKUP(K92,$P$5:$Q$15,2,FALSE),"현금·선물"))</f>
@@ -29081,7 +29081,7 @@
         </is>
       </c>
       <c r="I93" s="61" t="n">
-        <v>0.00023104</v>
+        <v>0.00022735</v>
       </c>
       <c r="J93" s="6" t="inlineStr">
         <is>
@@ -29106,7 +29106,7 @@
         </is>
       </c>
       <c r="I94" s="61" t="n">
-        <v>0.00023021</v>
+        <v>0.00022486</v>
       </c>
       <c r="J94" s="6" t="inlineStr">
         <is>
@@ -29131,7 +29131,7 @@
         </is>
       </c>
       <c r="I95" s="61" t="n">
-        <v>0.00020731</v>
+        <v>0.00020461</v>
       </c>
       <c r="J95" s="6" t="inlineStr">
         <is>
@@ -29156,7 +29156,7 @@
         </is>
       </c>
       <c r="I96" s="61" t="n">
-        <v>0.00019795</v>
+        <v>0.0001949</v>
       </c>
       <c r="J96" s="6" t="inlineStr">
         <is>
@@ -29177,15 +29177,15 @@
     <row r="97">
       <c r="H97" s="6" t="inlineStr">
         <is>
-          <t>VRTS</t>
+          <t>IBCP</t>
         </is>
       </c>
       <c r="I97" s="61" t="n">
-        <v>0.00019782</v>
+        <v>0.00019338</v>
       </c>
       <c r="J97" s="6" t="inlineStr">
         <is>
-          <t>VIRTUS INVESTMENT PARTNERS</t>
+          <t>INDEPENDENT BANK CORP</t>
         </is>
       </c>
       <c r="K97" s="6" t="inlineStr">
@@ -29202,15 +29202,15 @@
     <row r="98">
       <c r="H98" s="6" t="inlineStr">
         <is>
-          <t>IBCP</t>
+          <t>VRTS</t>
         </is>
       </c>
       <c r="I98" s="61" t="n">
-        <v>0.00019772</v>
+        <v>0.00018735</v>
       </c>
       <c r="J98" s="6" t="inlineStr">
         <is>
-          <t>INDEPENDENT BANK CORP</t>
+          <t>VIRTUS INVESTMENT PARTNERS</t>
         </is>
       </c>
       <c r="K98" s="6" t="inlineStr">
@@ -29231,7 +29231,7 @@
         </is>
       </c>
       <c r="I99" s="61" t="n">
-        <v>0.0001667</v>
+        <v>0.00016664</v>
       </c>
       <c r="J99" s="6" t="inlineStr">
         <is>
@@ -29256,7 +29256,7 @@
         </is>
       </c>
       <c r="I100" s="61" t="n">
-        <v>0.00013458</v>
+        <v>0.00013372</v>
       </c>
       <c r="J100" s="6" t="inlineStr">
         <is>
@@ -29277,18 +29277,22 @@
     <row r="101">
       <c r="H101" s="6" t="inlineStr">
         <is>
-          <t>USD</t>
+          <t>AMSF</t>
         </is>
       </c>
       <c r="I101" s="61" t="n">
-        <v>0.0001233</v>
+        <v>0.00011426</v>
       </c>
       <c r="J101" s="6" t="inlineStr">
         <is>
-          <t>US DOLLAR</t>
-        </is>
-      </c>
-      <c r="K101" s="6" t="inlineStr"/>
+          <t>AMERISAFE INC</t>
+        </is>
+      </c>
+      <c r="K101" s="6" t="inlineStr">
+        <is>
+          <t>Financials</t>
+        </is>
+      </c>
       <c r="L101" s="6" t="inlineStr"/>
       <c r="M101" s="7">
         <f>IF(H101="","",IFERROR(VLOOKUP(K101,$P$5:$Q$15,2,FALSE),"현금·선물"))</f>
@@ -29298,22 +29302,18 @@
     <row r="102">
       <c r="H102" s="6" t="inlineStr">
         <is>
-          <t>AMSF</t>
+          <t>USD</t>
         </is>
       </c>
       <c r="I102" s="61" t="n">
-        <v>0.00011551</v>
+        <v>0.00010633</v>
       </c>
       <c r="J102" s="6" t="inlineStr">
         <is>
-          <t>AMERISAFE INC</t>
-        </is>
-      </c>
-      <c r="K102" s="6" t="inlineStr">
-        <is>
-          <t>Financials</t>
-        </is>
-      </c>
+          <t>US DOLLAR</t>
+        </is>
+      </c>
+      <c r="K102" s="6" t="inlineStr"/>
       <c r="L102" s="6" t="inlineStr"/>
       <c r="M102" s="7">
         <f>IF(H102="","",IFERROR(VLOOKUP(K102,$P$5:$Q$15,2,FALSE),"현금·선물"))</f>
@@ -29327,7 +29327,7 @@
         </is>
       </c>
       <c r="I103" s="61" t="n">
-        <v>0.00010322</v>
+        <v>0.0001003</v>
       </c>
       <c r="J103" s="6" t="inlineStr">
         <is>
@@ -29352,7 +29352,7 @@
         </is>
       </c>
       <c r="I104" s="61" t="n">
-        <v>9.028e-05</v>
+        <v>9.043999999999999e-05</v>
       </c>
       <c r="J104" s="6" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
데이터 갱신: holdings (2026-10-16)
</commit_message>
<xml_diff>
--- a/downloads/schd_dividend_tracker.xlsx
+++ b/downloads/schd_dividend_tracker.xlsx
@@ -1724,7 +1724,7 @@
     <row r="3">
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>최종 갱신: 2026-10-15 · 반영 범위: 2012년 1분기 ~ 2026년 3분기 (배당락 2026-09-23) · GitHub Actions 자동 생성</t>
+          <t>최종 갱신: 2026-10-16 · 반영 범위: 2012년 1분기 ~ 2026년 3분기 (배당락 2026-09-23) · GitHub Actions 자동 생성</t>
         </is>
       </c>
     </row>
@@ -26257,11 +26257,11 @@
         </is>
       </c>
       <c r="B2" s="49" t="n">
-        <v>46309</v>
+        <v>46310</v>
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>← 이 날 종가로 계산한 비중. 그날 공식 파일을 못 받아 Schwab 공식 보유종목 CSV(2026-10-13)의 보유 주식 수 × 종가로 계산했습니다.</t>
+          <t>← 이 날 종가로 계산한 비중. 그날 공식 파일을 못 받아 Schwab 공식 보유종목 CSV(2026-10-14)의 보유 주식 수 × 종가로 계산했습니다.</t>
         </is>
       </c>
     </row>
@@ -26358,7 +26358,7 @@
         </is>
       </c>
       <c r="I5" s="61" t="n">
-        <v>0.04543222</v>
+        <v>0.04468937999999999</v>
       </c>
       <c r="J5" s="6" t="inlineStr">
         <is>
@@ -26416,7 +26416,7 @@
         </is>
       </c>
       <c r="I6" s="61" t="n">
-        <v>0.04373126</v>
+        <v>0.04340403</v>
       </c>
       <c r="J6" s="6" t="inlineStr">
         <is>
@@ -26470,25 +26470,25 @@
       </c>
       <c r="H7" s="6" t="inlineStr">
         <is>
-          <t>CVX</t>
+          <t>QCOM</t>
         </is>
       </c>
       <c r="I7" s="61" t="n">
-        <v>0.04324578</v>
+        <v>0.04282148</v>
       </c>
       <c r="J7" s="6" t="inlineStr">
         <is>
-          <t>CHEVRON</t>
+          <t>QUALCOMM</t>
         </is>
       </c>
       <c r="K7" s="6" t="inlineStr">
         <is>
-          <t>Energy</t>
+          <t>Information Technology</t>
         </is>
       </c>
       <c r="L7" s="6" t="inlineStr">
         <is>
-          <t>셰브론</t>
+          <t>퀄컴</t>
         </is>
       </c>
       <c r="M7" s="7">
@@ -26532,7 +26532,7 @@
         </is>
       </c>
       <c r="I8" s="61" t="n">
-        <v>0.04290234</v>
+        <v>0.04253392</v>
       </c>
       <c r="J8" s="6" t="inlineStr">
         <is>
@@ -26586,15 +26586,15 @@
       </c>
       <c r="H9" s="6" t="inlineStr">
         <is>
-          <t>COP</t>
+          <t>CVX</t>
         </is>
       </c>
       <c r="I9" s="61" t="n">
-        <v>0.04273807</v>
+        <v>0.0422479</v>
       </c>
       <c r="J9" s="6" t="inlineStr">
         <is>
-          <t>CONOCOPHILLIPS</t>
+          <t>CHEVRON</t>
         </is>
       </c>
       <c r="K9" s="6" t="inlineStr">
@@ -26604,7 +26604,7 @@
       </c>
       <c r="L9" s="6" t="inlineStr">
         <is>
-          <t>코노코필립스</t>
+          <t>셰브론</t>
         </is>
       </c>
       <c r="M9" s="7">
@@ -26644,25 +26644,25 @@
       </c>
       <c r="H10" s="6" t="inlineStr">
         <is>
-          <t>QCOM</t>
+          <t>COP</t>
         </is>
       </c>
       <c r="I10" s="61" t="n">
-        <v>0.04189318</v>
+        <v>0.04208859</v>
       </c>
       <c r="J10" s="6" t="inlineStr">
         <is>
-          <t>QUALCOMM</t>
+          <t>CONOCOPHILLIPS</t>
         </is>
       </c>
       <c r="K10" s="6" t="inlineStr">
         <is>
-          <t>Information Technology</t>
+          <t>Energy</t>
         </is>
       </c>
       <c r="L10" s="6" t="inlineStr">
         <is>
-          <t>퀄컴</t>
+          <t>코노코필립스</t>
         </is>
       </c>
       <c r="M10" s="7">
@@ -26706,7 +26706,7 @@
         </is>
       </c>
       <c r="I11" s="61" t="n">
-        <v>0.04083037</v>
+        <v>0.04151081</v>
       </c>
       <c r="J11" s="6" t="inlineStr">
         <is>
@@ -26760,15 +26760,15 @@
       </c>
       <c r="H12" s="6" t="inlineStr">
         <is>
-          <t>MRK</t>
+          <t>AMGN</t>
         </is>
       </c>
       <c r="I12" s="61" t="n">
-        <v>0.04008606999999999</v>
+        <v>0.03998357</v>
       </c>
       <c r="J12" s="6" t="inlineStr">
         <is>
-          <t>MERCK &amp; CO INC</t>
+          <t>AMGEN INC</t>
         </is>
       </c>
       <c r="K12" s="6" t="inlineStr">
@@ -26778,7 +26778,7 @@
       </c>
       <c r="L12" s="6" t="inlineStr">
         <is>
-          <t>머크</t>
+          <t>암젠</t>
         </is>
       </c>
       <c r="M12" s="7">
@@ -26818,25 +26818,25 @@
       </c>
       <c r="H13" s="6" t="inlineStr">
         <is>
-          <t>AMGN</t>
+          <t>HD</t>
         </is>
       </c>
       <c r="I13" s="61" t="n">
-        <v>0.03968896</v>
+        <v>0.03947982</v>
       </c>
       <c r="J13" s="6" t="inlineStr">
         <is>
-          <t>AMGEN INC</t>
+          <t>HOME DEPOT</t>
         </is>
       </c>
       <c r="K13" s="6" t="inlineStr">
         <is>
-          <t>Health Care</t>
+          <t>Consumer Discretionary</t>
         </is>
       </c>
       <c r="L13" s="6" t="inlineStr">
         <is>
-          <t>암젠</t>
+          <t>홈디포</t>
         </is>
       </c>
       <c r="M13" s="7">
@@ -26876,15 +26876,15 @@
       </c>
       <c r="H14" s="6" t="inlineStr">
         <is>
-          <t>ABT</t>
+          <t>MRK</t>
         </is>
       </c>
       <c r="I14" s="61" t="n">
-        <v>0.03844721</v>
+        <v>0.0390603</v>
       </c>
       <c r="J14" s="6" t="inlineStr">
         <is>
-          <t>ABBOTT LABORATORIES</t>
+          <t>MERCK &amp; CO INC</t>
         </is>
       </c>
       <c r="K14" s="6" t="inlineStr">
@@ -26894,7 +26894,7 @@
       </c>
       <c r="L14" s="6" t="inlineStr">
         <is>
-          <t>애보트</t>
+          <t>머크</t>
         </is>
       </c>
       <c r="M14" s="7">
@@ -26924,25 +26924,25 @@
       </c>
       <c r="H15" s="6" t="inlineStr">
         <is>
-          <t>HD</t>
+          <t>ABT</t>
         </is>
       </c>
       <c r="I15" s="61" t="n">
-        <v>0.03826877</v>
+        <v>0.03865739</v>
       </c>
       <c r="J15" s="6" t="inlineStr">
         <is>
-          <t>HOME DEPOT</t>
+          <t>ABBOTT LABORATORIES</t>
         </is>
       </c>
       <c r="K15" s="6" t="inlineStr">
         <is>
-          <t>Consumer Discretionary</t>
+          <t>Health Care</t>
         </is>
       </c>
       <c r="L15" s="6" t="inlineStr">
         <is>
-          <t>홈디포</t>
+          <t>애보트</t>
         </is>
       </c>
       <c r="M15" s="7">
@@ -26976,7 +26976,7 @@
         </is>
       </c>
       <c r="I16" s="61" t="n">
-        <v>0.03794526</v>
+        <v>0.03727104000000001</v>
       </c>
       <c r="J16" s="6" t="inlineStr">
         <is>
@@ -27014,7 +27014,7 @@
         </is>
       </c>
       <c r="I17" s="61" t="n">
-        <v>0.03648387</v>
+        <v>0.03606784</v>
       </c>
       <c r="J17" s="6" t="inlineStr">
         <is>
@@ -27052,7 +27052,7 @@
         </is>
       </c>
       <c r="I18" s="61" t="n">
-        <v>0.03287692</v>
+        <v>0.03402327</v>
       </c>
       <c r="J18" s="6" t="inlineStr">
         <is>
@@ -27077,25 +27077,25 @@
     <row r="19">
       <c r="H19" s="6" t="inlineStr">
         <is>
-          <t>MO</t>
+          <t>BMY</t>
         </is>
       </c>
       <c r="I19" s="61" t="n">
-        <v>0.03051891</v>
+        <v>0.03058469</v>
       </c>
       <c r="J19" s="6" t="inlineStr">
         <is>
-          <t>ALTRIA GROUP INC</t>
+          <t>BRISTOL MYERS SQUIBB</t>
         </is>
       </c>
       <c r="K19" s="6" t="inlineStr">
         <is>
-          <t>Consumer Staples</t>
+          <t>Health Care</t>
         </is>
       </c>
       <c r="L19" s="6" t="inlineStr">
         <is>
-          <t>알트리아</t>
+          <t>브리스톨마이어스스퀴브</t>
         </is>
       </c>
       <c r="M19" s="7">
@@ -27111,25 +27111,25 @@
       </c>
       <c r="H20" s="6" t="inlineStr">
         <is>
-          <t>BMY</t>
+          <t>MO</t>
         </is>
       </c>
       <c r="I20" s="61" t="n">
-        <v>0.03026495</v>
+        <v>0.03047754</v>
       </c>
       <c r="J20" s="6" t="inlineStr">
         <is>
-          <t>BRISTOL MYERS SQUIBB</t>
+          <t>ALTRIA GROUP INC</t>
         </is>
       </c>
       <c r="K20" s="6" t="inlineStr">
         <is>
-          <t>Health Care</t>
+          <t>Consumer Staples</t>
         </is>
       </c>
       <c r="L20" s="6" t="inlineStr">
         <is>
-          <t>브리스톨마이어스스퀴브</t>
+          <t>알트리아</t>
         </is>
       </c>
       <c r="M20" s="7">
@@ -27154,7 +27154,7 @@
         </is>
       </c>
       <c r="I21" s="61" t="n">
-        <v>0.02783255</v>
+        <v>0.02805097</v>
       </c>
       <c r="J21" s="6" t="inlineStr">
         <is>
@@ -27192,7 +27192,7 @@
         </is>
       </c>
       <c r="I22" s="61" t="n">
-        <v>0.02650835</v>
+        <v>0.02674044</v>
       </c>
       <c r="J22" s="6" t="inlineStr">
         <is>
@@ -27226,25 +27226,25 @@
       </c>
       <c r="H23" s="6" t="inlineStr">
         <is>
-          <t>EOG</t>
+          <t>BX</t>
         </is>
       </c>
       <c r="I23" s="61" t="n">
-        <v>0.02021378</v>
+        <v>0.020262</v>
       </c>
       <c r="J23" s="6" t="inlineStr">
         <is>
-          <t>EOG RESOURCES</t>
+          <t>BLACKSTONE</t>
         </is>
       </c>
       <c r="K23" s="6" t="inlineStr">
         <is>
-          <t>Energy</t>
+          <t>Financials</t>
         </is>
       </c>
       <c r="L23" s="6" t="inlineStr">
         <is>
-          <t>EOG 리소시스</t>
+          <t>블랙스톤</t>
         </is>
       </c>
       <c r="M23" s="7">
@@ -27264,25 +27264,25 @@
       </c>
       <c r="H24" s="6" t="inlineStr">
         <is>
-          <t>BX</t>
+          <t>EOG</t>
         </is>
       </c>
       <c r="I24" s="61" t="n">
-        <v>0.01992557</v>
+        <v>0.01978869</v>
       </c>
       <c r="J24" s="6" t="inlineStr">
         <is>
-          <t>BLACKSTONE</t>
+          <t>EOG RESOURCES</t>
         </is>
       </c>
       <c r="K24" s="6" t="inlineStr">
         <is>
-          <t>Financials</t>
+          <t>Energy</t>
         </is>
       </c>
       <c r="L24" s="6" t="inlineStr">
         <is>
-          <t>블랙스톤</t>
+          <t>EOG 리소시스</t>
         </is>
       </c>
       <c r="M24" s="7">
@@ -27306,7 +27306,7 @@
         </is>
       </c>
       <c r="I25" s="61" t="n">
-        <v>0.01862003</v>
+        <v>0.01904589</v>
       </c>
       <c r="J25" s="6" t="inlineStr">
         <is>
@@ -27340,25 +27340,25 @@
       </c>
       <c r="H26" s="6" t="inlineStr">
         <is>
-          <t>SLB</t>
+          <t>UPS</t>
         </is>
       </c>
       <c r="I26" s="61" t="n">
-        <v>0.01799412</v>
+        <v>0.01812146</v>
       </c>
       <c r="J26" s="6" t="inlineStr">
         <is>
-          <t>SLB</t>
+          <t>UNITED PARCEL SERVICE INC CLASS B</t>
         </is>
       </c>
       <c r="K26" s="6" t="inlineStr">
         <is>
-          <t>Energy</t>
+          <t>Industrials</t>
         </is>
       </c>
       <c r="L26" s="6" t="inlineStr">
         <is>
-          <t>SLB</t>
+          <t>UPS</t>
         </is>
       </c>
       <c r="M26" s="7">
@@ -27378,25 +27378,25 @@
       </c>
       <c r="H27" s="6" t="inlineStr">
         <is>
-          <t>UPS</t>
+          <t>SLB</t>
         </is>
       </c>
       <c r="I27" s="61" t="n">
-        <v>0.0179383</v>
+        <v>0.01774558</v>
       </c>
       <c r="J27" s="6" t="inlineStr">
         <is>
-          <t>UNITED PARCEL SERVICE INC CLASS B</t>
+          <t>SLB</t>
         </is>
       </c>
       <c r="K27" s="6" t="inlineStr">
         <is>
-          <t>Industrials</t>
+          <t>Energy</t>
         </is>
       </c>
       <c r="L27" s="6" t="inlineStr">
         <is>
-          <t>UPS</t>
+          <t>SLB</t>
         </is>
       </c>
       <c r="M27" s="7">
@@ -27420,7 +27420,7 @@
         </is>
       </c>
       <c r="I28" s="61" t="n">
-        <v>0.01763029</v>
+        <v>0.0175853</v>
       </c>
       <c r="J28" s="6" t="inlineStr">
         <is>
@@ -27458,7 +27458,7 @@
         </is>
       </c>
       <c r="I29" s="61" t="n">
-        <v>0.01491347</v>
+        <v>0.01429052</v>
       </c>
       <c r="J29" s="6" t="inlineStr">
         <is>
@@ -27496,7 +27496,7 @@
         </is>
       </c>
       <c r="I30" s="61" t="n">
-        <v>0.01448985</v>
+        <v>0.01412538</v>
       </c>
       <c r="J30" s="6" t="inlineStr">
         <is>
@@ -27530,7 +27530,7 @@
         </is>
       </c>
       <c r="I31" s="61" t="n">
-        <v>0.01372431</v>
+        <v>0.01338901</v>
       </c>
       <c r="J31" s="6" t="inlineStr">
         <is>
@@ -27555,7 +27555,7 @@
         </is>
       </c>
       <c r="I32" s="61" t="n">
-        <v>0.01179604</v>
+        <v>0.01191851</v>
       </c>
       <c r="J32" s="6" t="inlineStr">
         <is>
@@ -27585,7 +27585,7 @@
         </is>
       </c>
       <c r="I33" s="61" t="n">
-        <v>0.01125153</v>
+        <v>0.01128739</v>
       </c>
       <c r="J33" s="6" t="inlineStr">
         <is>
@@ -27610,7 +27610,7 @@
         </is>
       </c>
       <c r="I34" s="61" t="n">
-        <v>0.01007502</v>
+        <v>0.00988002</v>
       </c>
       <c r="J34" s="6" t="inlineStr">
         <is>
@@ -27635,7 +27635,7 @@
         </is>
       </c>
       <c r="I35" s="61" t="n">
-        <v>0.008670310000000001</v>
+        <v>0.00876598</v>
       </c>
       <c r="J35" s="6" t="inlineStr">
         <is>
@@ -27660,7 +27660,7 @@
         </is>
       </c>
       <c r="I36" s="61" t="n">
-        <v>0.008263100000000001</v>
+        <v>0.00855563</v>
       </c>
       <c r="J36" s="6" t="inlineStr">
         <is>
@@ -27685,7 +27685,7 @@
         </is>
       </c>
       <c r="I37" s="61" t="n">
-        <v>0.00639322</v>
+        <v>0.00634401</v>
       </c>
       <c r="J37" s="6" t="inlineStr">
         <is>
@@ -27710,7 +27710,7 @@
         </is>
       </c>
       <c r="I38" s="61" t="n">
-        <v>0.00629656</v>
+        <v>0.006312809999999999</v>
       </c>
       <c r="J38" s="6" t="inlineStr">
         <is>
@@ -27735,7 +27735,7 @@
         </is>
       </c>
       <c r="I39" s="61" t="n">
-        <v>0.00600621</v>
+        <v>0.00610059</v>
       </c>
       <c r="J39" s="6" t="inlineStr">
         <is>
@@ -27760,7 +27760,7 @@
         </is>
       </c>
       <c r="I40" s="61" t="n">
-        <v>0.00591714</v>
+        <v>0.00601476</v>
       </c>
       <c r="J40" s="6" t="inlineStr">
         <is>
@@ -27785,7 +27785,7 @@
         </is>
       </c>
       <c r="I41" s="61" t="n">
-        <v>0.0057256</v>
+        <v>0.005751309999999999</v>
       </c>
       <c r="J41" s="6" t="inlineStr">
         <is>
@@ -27810,7 +27810,7 @@
         </is>
       </c>
       <c r="I42" s="61" t="n">
-        <v>0.00531119</v>
+        <v>0.00534525</v>
       </c>
       <c r="J42" s="6" t="inlineStr">
         <is>
@@ -27835,7 +27835,7 @@
         </is>
       </c>
       <c r="I43" s="61" t="n">
-        <v>0.00522323</v>
+        <v>0.00524784</v>
       </c>
       <c r="J43" s="6" t="inlineStr">
         <is>
@@ -27856,20 +27856,20 @@
     <row r="44">
       <c r="H44" s="6" t="inlineStr">
         <is>
-          <t>DINO</t>
+          <t>BR</t>
         </is>
       </c>
       <c r="I44" s="61" t="n">
-        <v>0.00493398</v>
+        <v>0.00490861</v>
       </c>
       <c r="J44" s="6" t="inlineStr">
         <is>
-          <t>HF SINCLAIR</t>
+          <t>BROADRIDGE FINANCIAL SOLUTIONS INC</t>
         </is>
       </c>
       <c r="K44" s="6" t="inlineStr">
         <is>
-          <t>Energy</t>
+          <t>Industrials</t>
         </is>
       </c>
       <c r="L44" s="6" t="inlineStr"/>
@@ -27881,20 +27881,20 @@
     <row r="45">
       <c r="H45" s="6" t="inlineStr">
         <is>
-          <t>BR</t>
+          <t>DINO</t>
         </is>
       </c>
       <c r="I45" s="61" t="n">
-        <v>0.00479629</v>
+        <v>0.00476564</v>
       </c>
       <c r="J45" s="6" t="inlineStr">
         <is>
-          <t>BROADRIDGE FINANCIAL SOLUTIONS INC</t>
+          <t>HF SINCLAIR</t>
         </is>
       </c>
       <c r="K45" s="6" t="inlineStr">
         <is>
-          <t>Industrials</t>
+          <t>Energy</t>
         </is>
       </c>
       <c r="L45" s="6" t="inlineStr"/>
@@ -27910,7 +27910,7 @@
         </is>
       </c>
       <c r="I46" s="61" t="n">
-        <v>0.00469995</v>
+        <v>0.00467906</v>
       </c>
       <c r="J46" s="6" t="inlineStr">
         <is>
@@ -27935,7 +27935,7 @@
         </is>
       </c>
       <c r="I47" s="61" t="n">
-        <v>0.00440964</v>
+        <v>0.00460948</v>
       </c>
       <c r="J47" s="6" t="inlineStr">
         <is>
@@ -27960,7 +27960,7 @@
         </is>
       </c>
       <c r="I48" s="61" t="n">
-        <v>0.00429147</v>
+        <v>0.00434622</v>
       </c>
       <c r="J48" s="6" t="inlineStr">
         <is>
@@ -27985,7 +27985,7 @@
         </is>
       </c>
       <c r="I49" s="61" t="n">
-        <v>0.00426734</v>
+        <v>0.00427679</v>
       </c>
       <c r="J49" s="6" t="inlineStr">
         <is>
@@ -28010,7 +28010,7 @@
         </is>
       </c>
       <c r="I50" s="61" t="n">
-        <v>0.00414792</v>
+        <v>0.00409034</v>
       </c>
       <c r="J50" s="6" t="inlineStr">
         <is>
@@ -28035,7 +28035,7 @@
         </is>
       </c>
       <c r="I51" s="61" t="n">
-        <v>0.00262495</v>
+        <v>0.00263491</v>
       </c>
       <c r="J51" s="6" t="inlineStr">
         <is>
@@ -28056,15 +28056,15 @@
     <row r="52">
       <c r="H52" s="6" t="inlineStr">
         <is>
-          <t>AFG</t>
+          <t>FNF</t>
         </is>
       </c>
       <c r="I52" s="61" t="n">
-        <v>0.00250235</v>
+        <v>0.00249708</v>
       </c>
       <c r="J52" s="6" t="inlineStr">
         <is>
-          <t>AMERICAN FINANCIAL GROUP</t>
+          <t>FIDELITY NATIONAL FINANCIAL INC</t>
         </is>
       </c>
       <c r="K52" s="6" t="inlineStr">
@@ -28081,15 +28081,15 @@
     <row r="53">
       <c r="H53" s="6" t="inlineStr">
         <is>
-          <t>FNF</t>
+          <t>AFG</t>
         </is>
       </c>
       <c r="I53" s="61" t="n">
-        <v>0.00249803</v>
+        <v>0.00247659</v>
       </c>
       <c r="J53" s="6" t="inlineStr">
         <is>
-          <t>FIDELITY NATIONAL FINANCIAL INC</t>
+          <t>AMERICAN FINANCIAL GROUP</t>
         </is>
       </c>
       <c r="K53" s="6" t="inlineStr">
@@ -28110,7 +28110,7 @@
         </is>
       </c>
       <c r="I54" s="61" t="n">
-        <v>0.00215943</v>
+        <v>0.00221391</v>
       </c>
       <c r="J54" s="6" t="inlineStr">
         <is>
@@ -28135,7 +28135,7 @@
         </is>
       </c>
       <c r="I55" s="61" t="n">
-        <v>0.00213145</v>
+        <v>0.00212235</v>
       </c>
       <c r="J55" s="6" t="inlineStr">
         <is>
@@ -28160,7 +28160,7 @@
         </is>
       </c>
       <c r="I56" s="61" t="n">
-        <v>0.00197997</v>
+        <v>0.00200018</v>
       </c>
       <c r="J56" s="6" t="inlineStr">
         <is>
@@ -28185,7 +28185,7 @@
         </is>
       </c>
       <c r="I57" s="61" t="n">
-        <v>0.00189248</v>
+        <v>0.00190962</v>
       </c>
       <c r="J57" s="6" t="inlineStr">
         <is>
@@ -28206,20 +28206,20 @@
     <row r="58">
       <c r="H58" s="6" t="inlineStr">
         <is>
-          <t>MSM</t>
+          <t>M</t>
         </is>
       </c>
       <c r="I58" s="61" t="n">
-        <v>0.00151817</v>
+        <v>0.00157333</v>
       </c>
       <c r="J58" s="6" t="inlineStr">
         <is>
-          <t>MSC INDUSTRIAL CLASS A</t>
+          <t>MACYS INC</t>
         </is>
       </c>
       <c r="K58" s="6" t="inlineStr">
         <is>
-          <t>Industrials</t>
+          <t>Consumer Discretionary</t>
         </is>
       </c>
       <c r="L58" s="6" t="inlineStr"/>
@@ -28231,20 +28231,20 @@
     <row r="59">
       <c r="H59" s="6" t="inlineStr">
         <is>
-          <t>M</t>
+          <t>ERIE</t>
         </is>
       </c>
       <c r="I59" s="61" t="n">
-        <v>0.00148962</v>
+        <v>0.00152493</v>
       </c>
       <c r="J59" s="6" t="inlineStr">
         <is>
-          <t>MACYS INC</t>
+          <t>ERIE INDEMNITY CLASS A</t>
         </is>
       </c>
       <c r="K59" s="6" t="inlineStr">
         <is>
-          <t>Consumer Discretionary</t>
+          <t>Financials</t>
         </is>
       </c>
       <c r="L59" s="6" t="inlineStr"/>
@@ -28256,20 +28256,20 @@
     <row r="60">
       <c r="H60" s="6" t="inlineStr">
         <is>
-          <t>ERIE</t>
+          <t>MSM</t>
         </is>
       </c>
       <c r="I60" s="61" t="n">
-        <v>0.00148646</v>
+        <v>0.00148023</v>
       </c>
       <c r="J60" s="6" t="inlineStr">
         <is>
-          <t>ERIE INDEMNITY CLASS A</t>
+          <t>MSC INDUSTRIAL CLASS A</t>
         </is>
       </c>
       <c r="K60" s="6" t="inlineStr">
         <is>
-          <t>Financials</t>
+          <t>Industrials</t>
         </is>
       </c>
       <c r="L60" s="6" t="inlineStr"/>
@@ -28285,7 +28285,7 @@
         </is>
       </c>
       <c r="I61" s="61" t="n">
-        <v>0.00133141</v>
+        <v>0.00134771</v>
       </c>
       <c r="J61" s="6" t="inlineStr">
         <is>
@@ -28310,7 +28310,7 @@
         </is>
       </c>
       <c r="I62" s="61" t="n">
-        <v>0.00132548</v>
+        <v>0.00132896</v>
       </c>
       <c r="J62" s="6" t="inlineStr">
         <is>
@@ -28335,7 +28335,7 @@
         </is>
       </c>
       <c r="I63" s="61" t="n">
-        <v>0.00116183</v>
+        <v>0.0011802</v>
       </c>
       <c r="J63" s="6" t="inlineStr">
         <is>
@@ -28360,7 +28360,7 @@
         </is>
       </c>
       <c r="I64" s="61" t="n">
-        <v>0.00114039</v>
+        <v>0.00115072</v>
       </c>
       <c r="J64" s="6" t="inlineStr">
         <is>
@@ -28385,7 +28385,7 @@
         </is>
       </c>
       <c r="I65" s="61" t="n">
-        <v>0.00100205</v>
+        <v>0.00101025</v>
       </c>
       <c r="J65" s="6" t="inlineStr">
         <is>
@@ -28410,7 +28410,7 @@
         </is>
       </c>
       <c r="I66" s="61" t="n">
-        <v>0.0009784500000000001</v>
+        <v>0.0009951999999999999</v>
       </c>
       <c r="J66" s="6" t="inlineStr">
         <is>
@@ -28431,20 +28431,20 @@
     <row r="67">
       <c r="H67" s="6" t="inlineStr">
         <is>
-          <t>KFY</t>
+          <t>PAG</t>
         </is>
       </c>
       <c r="I67" s="61" t="n">
-        <v>0.00091228</v>
+        <v>0.00093075</v>
       </c>
       <c r="J67" s="6" t="inlineStr">
         <is>
-          <t>KORN FERRY</t>
+          <t>PENSKE AUTOMOTIVE GROUP VOTING INC</t>
         </is>
       </c>
       <c r="K67" s="6" t="inlineStr">
         <is>
-          <t>Industrials</t>
+          <t>Consumer Discretionary</t>
         </is>
       </c>
       <c r="L67" s="6" t="inlineStr"/>
@@ -28456,20 +28456,20 @@
     <row r="68">
       <c r="H68" s="6" t="inlineStr">
         <is>
-          <t>CWEN</t>
+          <t>KFY</t>
         </is>
       </c>
       <c r="I68" s="61" t="n">
-        <v>0.00089414</v>
+        <v>0.00092899</v>
       </c>
       <c r="J68" s="6" t="inlineStr">
         <is>
-          <t>CLEARWAY ENERGY INC CLASS C</t>
+          <t>KORN FERRY</t>
         </is>
       </c>
       <c r="K68" s="6" t="inlineStr">
         <is>
-          <t>Utilities</t>
+          <t>Industrials</t>
         </is>
       </c>
       <c r="L68" s="6" t="inlineStr"/>
@@ -28485,7 +28485,7 @@
         </is>
       </c>
       <c r="I69" s="61" t="n">
-        <v>0.00088975</v>
+        <v>0.00089978</v>
       </c>
       <c r="J69" s="6" t="inlineStr">
         <is>
@@ -28506,20 +28506,20 @@
     <row r="70">
       <c r="H70" s="6" t="inlineStr">
         <is>
-          <t>RHI</t>
+          <t>CWEN</t>
         </is>
       </c>
       <c r="I70" s="61" t="n">
-        <v>0.00087711</v>
+        <v>0.00089479</v>
       </c>
       <c r="J70" s="6" t="inlineStr">
         <is>
-          <t>ROBERT HALF INC</t>
+          <t>CLEARWAY ENERGY INC CLASS C</t>
         </is>
       </c>
       <c r="K70" s="6" t="inlineStr">
         <is>
-          <t>Industrials</t>
+          <t>Utilities</t>
         </is>
       </c>
       <c r="L70" s="6" t="inlineStr"/>
@@ -28531,20 +28531,20 @@
     <row r="71">
       <c r="H71" s="6" t="inlineStr">
         <is>
-          <t>PAG</t>
+          <t>RHI</t>
         </is>
       </c>
       <c r="I71" s="61" t="n">
-        <v>0.00086469</v>
+        <v>0.00085287</v>
       </c>
       <c r="J71" s="6" t="inlineStr">
         <is>
-          <t>PENSKE AUTOMOTIVE GROUP VOTING INC</t>
+          <t>ROBERT HALF INC</t>
         </is>
       </c>
       <c r="K71" s="6" t="inlineStr">
         <is>
-          <t>Consumer Discretionary</t>
+          <t>Industrials</t>
         </is>
       </c>
       <c r="L71" s="6" t="inlineStr"/>
@@ -28556,15 +28556,15 @@
     <row r="72">
       <c r="H72" s="6" t="inlineStr">
         <is>
-          <t>BANR</t>
+          <t>APAM</t>
         </is>
       </c>
       <c r="I72" s="61" t="n">
-        <v>0.00056073</v>
+        <v>0.00057239</v>
       </c>
       <c r="J72" s="6" t="inlineStr">
         <is>
-          <t>BANNER CORP</t>
+          <t>ARTISAN PARTNERS ASSET MANAGEMENT</t>
         </is>
       </c>
       <c r="K72" s="6" t="inlineStr">
@@ -28581,15 +28581,15 @@
     <row r="73">
       <c r="H73" s="6" t="inlineStr">
         <is>
-          <t>APAM</t>
+          <t>BANR</t>
         </is>
       </c>
       <c r="I73" s="61" t="n">
-        <v>0.00056072</v>
+        <v>0.00056285</v>
       </c>
       <c r="J73" s="6" t="inlineStr">
         <is>
-          <t>ARTISAN PARTNERS ASSET MANAGEMENT</t>
+          <t>BANNER CORP</t>
         </is>
       </c>
       <c r="K73" s="6" t="inlineStr">
@@ -28610,7 +28610,7 @@
         </is>
       </c>
       <c r="I74" s="61" t="n">
-        <v>0.00053834</v>
+        <v>0.00054509</v>
       </c>
       <c r="J74" s="6" t="inlineStr">
         <is>
@@ -28635,7 +28635,7 @@
         </is>
       </c>
       <c r="I75" s="61" t="n">
-        <v>0.00052264</v>
+        <v>0.0005197800000000001</v>
       </c>
       <c r="J75" s="6" t="inlineStr">
         <is>
@@ -28660,7 +28660,7 @@
         </is>
       </c>
       <c r="I76" s="61" t="n">
-        <v>0.0004929299999999999</v>
+        <v>0.00049706</v>
       </c>
       <c r="J76" s="6" t="inlineStr">
         <is>
@@ -28685,7 +28685,7 @@
         </is>
       </c>
       <c r="I77" s="61" t="n">
-        <v>0.00049172</v>
+        <v>0.00048956</v>
       </c>
       <c r="J77" s="6" t="inlineStr">
         <is>
@@ -28706,15 +28706,15 @@
     <row r="78">
       <c r="H78" s="6" t="inlineStr">
         <is>
-          <t>AGM</t>
+          <t>CNS</t>
         </is>
       </c>
       <c r="I78" s="61" t="n">
-        <v>0.00047649</v>
+        <v>0.00048258</v>
       </c>
       <c r="J78" s="6" t="inlineStr">
         <is>
-          <t>FEDERAL AGRICULTURAL MORTGAGE NON</t>
+          <t>COHEN &amp; STEERS INC</t>
         </is>
       </c>
       <c r="K78" s="6" t="inlineStr">
@@ -28735,7 +28735,7 @@
         </is>
       </c>
       <c r="I79" s="61" t="n">
-        <v>0.00047286</v>
+        <v>0.0004816</v>
       </c>
       <c r="J79" s="6" t="inlineStr">
         <is>
@@ -28756,15 +28756,15 @@
     <row r="80">
       <c r="H80" s="6" t="inlineStr">
         <is>
-          <t>CNS</t>
+          <t>AGM</t>
         </is>
       </c>
       <c r="I80" s="61" t="n">
-        <v>0.00046962</v>
+        <v>0.0004767699999999999</v>
       </c>
       <c r="J80" s="6" t="inlineStr">
         <is>
-          <t>COHEN &amp; STEERS INC</t>
+          <t>FEDERAL AGRICULTURAL MORTGAGE NON</t>
         </is>
       </c>
       <c r="K80" s="6" t="inlineStr">
@@ -28785,7 +28785,7 @@
         </is>
       </c>
       <c r="I81" s="61" t="n">
-        <v>0.00045944</v>
+        <v>0.0004612900000000001</v>
       </c>
       <c r="J81" s="6" t="inlineStr">
         <is>
@@ -28810,7 +28810,7 @@
         </is>
       </c>
       <c r="I82" s="61" t="n">
-        <v>0.00044368</v>
+        <v>0.00044961</v>
       </c>
       <c r="J82" s="6" t="inlineStr">
         <is>
@@ -28835,7 +28835,7 @@
         </is>
       </c>
       <c r="I83" s="61" t="n">
-        <v>0.00042389</v>
+        <v>0.00042413</v>
       </c>
       <c r="J83" s="6" t="inlineStr">
         <is>
@@ -28860,7 +28860,7 @@
         </is>
       </c>
       <c r="I84" s="61" t="n">
-        <v>0.00041283</v>
+        <v>0.0004150100000000001</v>
       </c>
       <c r="J84" s="6" t="inlineStr">
         <is>
@@ -28885,7 +28885,7 @@
         </is>
       </c>
       <c r="I85" s="61" t="n">
-        <v>0.00037643</v>
+        <v>0.00037781</v>
       </c>
       <c r="J85" s="6" t="inlineStr">
         <is>
@@ -28910,7 +28910,7 @@
         </is>
       </c>
       <c r="I86" s="61" t="n">
-        <v>0.0003552</v>
+        <v>0.00035679</v>
       </c>
       <c r="J86" s="6" t="inlineStr">
         <is>
@@ -28935,7 +28935,7 @@
         </is>
       </c>
       <c r="I87" s="61" t="n">
-        <v>0.00034336</v>
+        <v>0.00035411</v>
       </c>
       <c r="J87" s="6" t="inlineStr">
         <is>
@@ -28960,7 +28960,7 @@
         </is>
       </c>
       <c r="I88" s="61" t="n">
-        <v>0.00031676</v>
+        <v>0.00032116</v>
       </c>
       <c r="J88" s="6" t="inlineStr">
         <is>
@@ -28985,7 +28985,7 @@
         </is>
       </c>
       <c r="I89" s="61" t="n">
-        <v>0.00027823</v>
+        <v>0.00027948</v>
       </c>
       <c r="J89" s="6" t="inlineStr">
         <is>
@@ -29006,18 +29006,22 @@
     <row r="90">
       <c r="H90" s="6" t="inlineStr">
         <is>
-          <t>GVMXX</t>
+          <t>WEN</t>
         </is>
       </c>
       <c r="I90" s="61" t="n">
-        <v>0.00026386</v>
+        <v>0.00026618</v>
       </c>
       <c r="J90" s="6" t="inlineStr">
         <is>
-          <t>SSC GOVERNMENT MM GVMXX</t>
-        </is>
-      </c>
-      <c r="K90" s="6" t="inlineStr"/>
+          <t>WENDYS</t>
+        </is>
+      </c>
+      <c r="K90" s="6" t="inlineStr">
+        <is>
+          <t>Consumer Discretionary</t>
+        </is>
+      </c>
       <c r="L90" s="6" t="inlineStr"/>
       <c r="M90" s="7">
         <f>IF(H90="","",IFERROR(VLOOKUP(K90,$P$5:$Q$15,2,FALSE),"현금·선물"))</f>
@@ -29027,22 +29031,18 @@
     <row r="91">
       <c r="H91" s="6" t="inlineStr">
         <is>
-          <t>WEN</t>
+          <t>GVMXX</t>
         </is>
       </c>
       <c r="I91" s="61" t="n">
-        <v>0.00025869</v>
+        <v>0.00025601</v>
       </c>
       <c r="J91" s="6" t="inlineStr">
         <is>
-          <t>WENDYS</t>
-        </is>
-      </c>
-      <c r="K91" s="6" t="inlineStr">
-        <is>
-          <t>Consumer Discretionary</t>
-        </is>
-      </c>
+          <t>SSC GOVERNMENT MM GVMXX</t>
+        </is>
+      </c>
+      <c r="K91" s="6" t="inlineStr"/>
       <c r="L91" s="6" t="inlineStr"/>
       <c r="M91" s="7">
         <f>IF(H91="","",IFERROR(VLOOKUP(K91,$P$5:$Q$15,2,FALSE),"현금·선물"))</f>
@@ -29056,7 +29056,7 @@
         </is>
       </c>
       <c r="I92" s="61" t="n">
-        <v>0.00025645</v>
+        <v>0.00025402</v>
       </c>
       <c r="J92" s="6" t="inlineStr">
         <is>
@@ -29081,7 +29081,7 @@
         </is>
       </c>
       <c r="I93" s="61" t="n">
-        <v>0.00022735</v>
+        <v>0.00022923</v>
       </c>
       <c r="J93" s="6" t="inlineStr">
         <is>
@@ -29106,7 +29106,7 @@
         </is>
       </c>
       <c r="I94" s="61" t="n">
-        <v>0.00022486</v>
+        <v>0.00022568</v>
       </c>
       <c r="J94" s="6" t="inlineStr">
         <is>
@@ -29131,7 +29131,7 @@
         </is>
       </c>
       <c r="I95" s="61" t="n">
-        <v>0.00020461</v>
+        <v>0.00020443</v>
       </c>
       <c r="J95" s="6" t="inlineStr">
         <is>
@@ -29156,7 +29156,7 @@
         </is>
       </c>
       <c r="I96" s="61" t="n">
-        <v>0.0001949</v>
+        <v>0.00019465</v>
       </c>
       <c r="J96" s="6" t="inlineStr">
         <is>
@@ -29181,7 +29181,7 @@
         </is>
       </c>
       <c r="I97" s="61" t="n">
-        <v>0.00019338</v>
+        <v>0.00019417</v>
       </c>
       <c r="J97" s="6" t="inlineStr">
         <is>
@@ -29206,7 +29206,7 @@
         </is>
       </c>
       <c r="I98" s="61" t="n">
-        <v>0.00018735</v>
+        <v>0.00018591</v>
       </c>
       <c r="J98" s="6" t="inlineStr">
         <is>
@@ -29231,7 +29231,7 @@
         </is>
       </c>
       <c r="I99" s="61" t="n">
-        <v>0.00016664</v>
+        <v>0.00016554</v>
       </c>
       <c r="J99" s="6" t="inlineStr">
         <is>
@@ -29256,7 +29256,7 @@
         </is>
       </c>
       <c r="I100" s="61" t="n">
-        <v>0.00013372</v>
+        <v>0.00013261</v>
       </c>
       <c r="J100" s="6" t="inlineStr">
         <is>
@@ -29281,7 +29281,7 @@
         </is>
       </c>
       <c r="I101" s="61" t="n">
-        <v>0.00011426</v>
+        <v>0.00011484</v>
       </c>
       <c r="J101" s="6" t="inlineStr">
         <is>
@@ -29306,7 +29306,7 @@
         </is>
       </c>
       <c r="I102" s="61" t="n">
-        <v>0.00010633</v>
+        <v>0.00011285</v>
       </c>
       <c r="J102" s="6" t="inlineStr">
         <is>
@@ -29327,7 +29327,7 @@
         </is>
       </c>
       <c r="I103" s="61" t="n">
-        <v>0.0001003</v>
+        <v>0.00010068</v>
       </c>
       <c r="J103" s="6" t="inlineStr">
         <is>
@@ -29352,7 +29352,7 @@
         </is>
       </c>
       <c r="I104" s="61" t="n">
-        <v>9.043999999999999e-05</v>
+        <v>9.577e-05</v>
       </c>
       <c r="J104" s="6" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
데이터 갱신: holdings (2026-10-17)
</commit_message>
<xml_diff>
--- a/downloads/schd_dividend_tracker.xlsx
+++ b/downloads/schd_dividend_tracker.xlsx
@@ -1724,7 +1724,7 @@
     <row r="3">
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>최종 갱신: 2026-10-16 · 반영 범위: 2012년 1분기 ~ 2026년 3분기 (배당락 2026-09-23) · GitHub Actions 자동 생성</t>
+          <t>최종 갱신: 2026-10-17 · 반영 범위: 2012년 1분기 ~ 2026년 3분기 (배당락 2026-09-23) · GitHub Actions 자동 생성</t>
         </is>
       </c>
     </row>
@@ -26261,7 +26261,7 @@
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>← 이 날 종가로 계산한 비중. 그날 공식 파일을 못 받아 Schwab 공식 보유종목 CSV(2026-10-14)의 보유 주식 수 × 종가로 계산했습니다.</t>
+          <t>← Schwab 공식 보유종목 CSV 기준일. 매일 자동으로 최신 파일을 받습니다.</t>
         </is>
       </c>
     </row>
@@ -26358,7 +26358,7 @@
         </is>
       </c>
       <c r="I5" s="61" t="n">
-        <v>0.04468937999999999</v>
+        <v>0.04468282000000001</v>
       </c>
       <c r="J5" s="6" t="inlineStr">
         <is>
@@ -26416,7 +26416,7 @@
         </is>
       </c>
       <c r="I6" s="61" t="n">
-        <v>0.04340403</v>
+        <v>0.04339762999999999</v>
       </c>
       <c r="J6" s="6" t="inlineStr">
         <is>
@@ -26474,7 +26474,7 @@
         </is>
       </c>
       <c r="I7" s="61" t="n">
-        <v>0.04282148</v>
+        <v>0.04281518</v>
       </c>
       <c r="J7" s="6" t="inlineStr">
         <is>
@@ -26532,7 +26532,7 @@
         </is>
       </c>
       <c r="I8" s="61" t="n">
-        <v>0.04253392</v>
+        <v>0.04252766</v>
       </c>
       <c r="J8" s="6" t="inlineStr">
         <is>
@@ -26590,7 +26590,7 @@
         </is>
       </c>
       <c r="I9" s="61" t="n">
-        <v>0.0422479</v>
+        <v>0.0422417</v>
       </c>
       <c r="J9" s="6" t="inlineStr">
         <is>
@@ -26648,7 +26648,7 @@
         </is>
       </c>
       <c r="I10" s="61" t="n">
-        <v>0.04208859</v>
+        <v>0.0420824</v>
       </c>
       <c r="J10" s="6" t="inlineStr">
         <is>
@@ -26706,7 +26706,7 @@
         </is>
       </c>
       <c r="I11" s="61" t="n">
-        <v>0.04151081</v>
+        <v>0.04150475</v>
       </c>
       <c r="J11" s="6" t="inlineStr">
         <is>
@@ -26764,7 +26764,7 @@
         </is>
       </c>
       <c r="I12" s="61" t="n">
-        <v>0.03998357</v>
+        <v>0.03997775</v>
       </c>
       <c r="J12" s="6" t="inlineStr">
         <is>
@@ -26822,7 +26822,7 @@
         </is>
       </c>
       <c r="I13" s="61" t="n">
-        <v>0.03947982</v>
+        <v>0.03947407</v>
       </c>
       <c r="J13" s="6" t="inlineStr">
         <is>
@@ -26880,7 +26880,7 @@
         </is>
       </c>
       <c r="I14" s="61" t="n">
-        <v>0.0390603</v>
+        <v>0.03905457</v>
       </c>
       <c r="J14" s="6" t="inlineStr">
         <is>
@@ -26928,7 +26928,7 @@
         </is>
       </c>
       <c r="I15" s="61" t="n">
-        <v>0.03865739</v>
+        <v>0.0386517</v>
       </c>
       <c r="J15" s="6" t="inlineStr">
         <is>
@@ -26976,7 +26976,7 @@
         </is>
       </c>
       <c r="I16" s="61" t="n">
-        <v>0.03727104000000001</v>
+        <v>0.03726557</v>
       </c>
       <c r="J16" s="6" t="inlineStr">
         <is>
@@ -27014,7 +27014,7 @@
         </is>
       </c>
       <c r="I17" s="61" t="n">
-        <v>0.03606784</v>
+        <v>0.03606252</v>
       </c>
       <c r="J17" s="6" t="inlineStr">
         <is>
@@ -27052,7 +27052,7 @@
         </is>
       </c>
       <c r="I18" s="61" t="n">
-        <v>0.03402327</v>
+        <v>0.03401827</v>
       </c>
       <c r="J18" s="6" t="inlineStr">
         <is>
@@ -27081,7 +27081,7 @@
         </is>
       </c>
       <c r="I19" s="61" t="n">
-        <v>0.03058469</v>
+        <v>0.03058018</v>
       </c>
       <c r="J19" s="6" t="inlineStr">
         <is>
@@ -27115,7 +27115,7 @@
         </is>
       </c>
       <c r="I20" s="61" t="n">
-        <v>0.03047754</v>
+        <v>0.03047305</v>
       </c>
       <c r="J20" s="6" t="inlineStr">
         <is>
@@ -27154,7 +27154,7 @@
         </is>
       </c>
       <c r="I21" s="61" t="n">
-        <v>0.02805097</v>
+        <v>0.02804684</v>
       </c>
       <c r="J21" s="6" t="inlineStr">
         <is>
@@ -27192,7 +27192,7 @@
         </is>
       </c>
       <c r="I22" s="61" t="n">
-        <v>0.02674044</v>
+        <v>0.02673655</v>
       </c>
       <c r="J22" s="6" t="inlineStr">
         <is>
@@ -27230,7 +27230,7 @@
         </is>
       </c>
       <c r="I23" s="61" t="n">
-        <v>0.020262</v>
+        <v>0.02025903</v>
       </c>
       <c r="J23" s="6" t="inlineStr">
         <is>
@@ -27268,7 +27268,7 @@
         </is>
       </c>
       <c r="I24" s="61" t="n">
-        <v>0.01978869</v>
+        <v>0.01978579</v>
       </c>
       <c r="J24" s="6" t="inlineStr">
         <is>
@@ -27306,7 +27306,7 @@
         </is>
       </c>
       <c r="I25" s="61" t="n">
-        <v>0.01904589</v>
+        <v>0.01904309</v>
       </c>
       <c r="J25" s="6" t="inlineStr">
         <is>
@@ -27344,7 +27344,7 @@
         </is>
       </c>
       <c r="I26" s="61" t="n">
-        <v>0.01812146</v>
+        <v>0.01811879</v>
       </c>
       <c r="J26" s="6" t="inlineStr">
         <is>
@@ -27382,7 +27382,7 @@
         </is>
       </c>
       <c r="I27" s="61" t="n">
-        <v>0.01774558</v>
+        <v>0.01774296</v>
       </c>
       <c r="J27" s="6" t="inlineStr">
         <is>
@@ -27420,7 +27420,7 @@
         </is>
       </c>
       <c r="I28" s="61" t="n">
-        <v>0.0175853</v>
+        <v>0.01758271</v>
       </c>
       <c r="J28" s="6" t="inlineStr">
         <is>
@@ -27458,7 +27458,7 @@
         </is>
       </c>
       <c r="I29" s="61" t="n">
-        <v>0.01429052</v>
+        <v>0.01428842</v>
       </c>
       <c r="J29" s="6" t="inlineStr">
         <is>
@@ -27496,7 +27496,7 @@
         </is>
       </c>
       <c r="I30" s="61" t="n">
-        <v>0.01412538</v>
+        <v>0.0141233</v>
       </c>
       <c r="J30" s="6" t="inlineStr">
         <is>
@@ -27530,7 +27530,7 @@
         </is>
       </c>
       <c r="I31" s="61" t="n">
-        <v>0.01338901</v>
+        <v>0.01338705</v>
       </c>
       <c r="J31" s="6" t="inlineStr">
         <is>
@@ -27555,7 +27555,7 @@
         </is>
       </c>
       <c r="I32" s="61" t="n">
-        <v>0.01191851</v>
+        <v>0.01191675</v>
       </c>
       <c r="J32" s="6" t="inlineStr">
         <is>
@@ -27585,7 +27585,7 @@
         </is>
       </c>
       <c r="I33" s="61" t="n">
-        <v>0.01128739</v>
+        <v>0.01128573</v>
       </c>
       <c r="J33" s="6" t="inlineStr">
         <is>
@@ -27610,7 +27610,7 @@
         </is>
       </c>
       <c r="I34" s="61" t="n">
-        <v>0.00988002</v>
+        <v>0.00987858</v>
       </c>
       <c r="J34" s="6" t="inlineStr">
         <is>
@@ -27635,7 +27635,7 @@
         </is>
       </c>
       <c r="I35" s="61" t="n">
-        <v>0.00876598</v>
+        <v>0.0087647</v>
       </c>
       <c r="J35" s="6" t="inlineStr">
         <is>
@@ -27660,7 +27660,7 @@
         </is>
       </c>
       <c r="I36" s="61" t="n">
-        <v>0.00855563</v>
+        <v>0.00855439</v>
       </c>
       <c r="J36" s="6" t="inlineStr">
         <is>
@@ -27685,7 +27685,7 @@
         </is>
       </c>
       <c r="I37" s="61" t="n">
-        <v>0.00634401</v>
+        <v>0.00634309</v>
       </c>
       <c r="J37" s="6" t="inlineStr">
         <is>
@@ -27710,7 +27710,7 @@
         </is>
       </c>
       <c r="I38" s="61" t="n">
-        <v>0.006312809999999999</v>
+        <v>0.00631188</v>
       </c>
       <c r="J38" s="6" t="inlineStr">
         <is>
@@ -27735,7 +27735,7 @@
         </is>
       </c>
       <c r="I39" s="61" t="n">
-        <v>0.00610059</v>
+        <v>0.00609971</v>
       </c>
       <c r="J39" s="6" t="inlineStr">
         <is>
@@ -27760,7 +27760,7 @@
         </is>
       </c>
       <c r="I40" s="61" t="n">
-        <v>0.00601476</v>
+        <v>0.00601391</v>
       </c>
       <c r="J40" s="6" t="inlineStr">
         <is>
@@ -27785,7 +27785,7 @@
         </is>
       </c>
       <c r="I41" s="61" t="n">
-        <v>0.005751309999999999</v>
+        <v>0.00575046</v>
       </c>
       <c r="J41" s="6" t="inlineStr">
         <is>
@@ -27810,7 +27810,7 @@
         </is>
       </c>
       <c r="I42" s="61" t="n">
-        <v>0.00534525</v>
+        <v>0.00534448</v>
       </c>
       <c r="J42" s="6" t="inlineStr">
         <is>
@@ -27835,7 +27835,7 @@
         </is>
       </c>
       <c r="I43" s="61" t="n">
-        <v>0.00524784</v>
+        <v>0.005247089999999999</v>
       </c>
       <c r="J43" s="6" t="inlineStr">
         <is>
@@ -27860,7 +27860,7 @@
         </is>
       </c>
       <c r="I44" s="61" t="n">
-        <v>0.00490861</v>
+        <v>0.00490793</v>
       </c>
       <c r="J44" s="6" t="inlineStr">
         <is>
@@ -27885,7 +27885,7 @@
         </is>
       </c>
       <c r="I45" s="61" t="n">
-        <v>0.00476564</v>
+        <v>0.00476494</v>
       </c>
       <c r="J45" s="6" t="inlineStr">
         <is>
@@ -27910,7 +27910,7 @@
         </is>
       </c>
       <c r="I46" s="61" t="n">
-        <v>0.00467906</v>
+        <v>0.00467843</v>
       </c>
       <c r="J46" s="6" t="inlineStr">
         <is>
@@ -27935,7 +27935,7 @@
         </is>
       </c>
       <c r="I47" s="61" t="n">
-        <v>0.00460948</v>
+        <v>0.00460881</v>
       </c>
       <c r="J47" s="6" t="inlineStr">
         <is>
@@ -27960,7 +27960,7 @@
         </is>
       </c>
       <c r="I48" s="61" t="n">
-        <v>0.00434622</v>
+        <v>0.00434558</v>
       </c>
       <c r="J48" s="6" t="inlineStr">
         <is>
@@ -27985,7 +27985,7 @@
         </is>
       </c>
       <c r="I49" s="61" t="n">
-        <v>0.00427679</v>
+        <v>0.00427618</v>
       </c>
       <c r="J49" s="6" t="inlineStr">
         <is>
@@ -28010,7 +28010,7 @@
         </is>
       </c>
       <c r="I50" s="61" t="n">
-        <v>0.00409034</v>
+        <v>0.00408974</v>
       </c>
       <c r="J50" s="6" t="inlineStr">
         <is>
@@ -28035,7 +28035,7 @@
         </is>
       </c>
       <c r="I51" s="61" t="n">
-        <v>0.00263491</v>
+        <v>0.00263459</v>
       </c>
       <c r="J51" s="6" t="inlineStr">
         <is>
@@ -28060,7 +28060,7 @@
         </is>
       </c>
       <c r="I52" s="61" t="n">
-        <v>0.00249708</v>
+        <v>0.00249672</v>
       </c>
       <c r="J52" s="6" t="inlineStr">
         <is>
@@ -28085,7 +28085,7 @@
         </is>
       </c>
       <c r="I53" s="61" t="n">
-        <v>0.00247659</v>
+        <v>0.00247625</v>
       </c>
       <c r="J53" s="6" t="inlineStr">
         <is>
@@ -28110,7 +28110,7 @@
         </is>
       </c>
       <c r="I54" s="61" t="n">
-        <v>0.00221391</v>
+        <v>0.00221359</v>
       </c>
       <c r="J54" s="6" t="inlineStr">
         <is>
@@ -28135,7 +28135,7 @@
         </is>
       </c>
       <c r="I55" s="61" t="n">
-        <v>0.00212235</v>
+        <v>0.00212205</v>
       </c>
       <c r="J55" s="6" t="inlineStr">
         <is>
@@ -28160,7 +28160,7 @@
         </is>
       </c>
       <c r="I56" s="61" t="n">
-        <v>0.00200018</v>
+        <v>0.00199989</v>
       </c>
       <c r="J56" s="6" t="inlineStr">
         <is>
@@ -28185,7 +28185,7 @@
         </is>
       </c>
       <c r="I57" s="61" t="n">
-        <v>0.00190962</v>
+        <v>0.00190934</v>
       </c>
       <c r="J57" s="6" t="inlineStr">
         <is>
@@ -28210,7 +28210,7 @@
         </is>
       </c>
       <c r="I58" s="61" t="n">
-        <v>0.00157333</v>
+        <v>0.0015731</v>
       </c>
       <c r="J58" s="6" t="inlineStr">
         <is>
@@ -28235,7 +28235,7 @@
         </is>
       </c>
       <c r="I59" s="61" t="n">
-        <v>0.00152493</v>
+        <v>0.00152475</v>
       </c>
       <c r="J59" s="6" t="inlineStr">
         <is>
@@ -28260,7 +28260,7 @@
         </is>
       </c>
       <c r="I60" s="61" t="n">
-        <v>0.00148023</v>
+        <v>0.00148002</v>
       </c>
       <c r="J60" s="6" t="inlineStr">
         <is>
@@ -28285,7 +28285,7 @@
         </is>
       </c>
       <c r="I61" s="61" t="n">
-        <v>0.00134771</v>
+        <v>0.00134755</v>
       </c>
       <c r="J61" s="6" t="inlineStr">
         <is>
@@ -28310,7 +28310,7 @@
         </is>
       </c>
       <c r="I62" s="61" t="n">
-        <v>0.00132896</v>
+        <v>0.00132877</v>
       </c>
       <c r="J62" s="6" t="inlineStr">
         <is>
@@ -28335,7 +28335,7 @@
         </is>
       </c>
       <c r="I63" s="61" t="n">
-        <v>0.0011802</v>
+        <v>0.00118004</v>
       </c>
       <c r="J63" s="6" t="inlineStr">
         <is>
@@ -28360,7 +28360,7 @@
         </is>
       </c>
       <c r="I64" s="61" t="n">
-        <v>0.00115072</v>
+        <v>0.00115056</v>
       </c>
       <c r="J64" s="6" t="inlineStr">
         <is>
@@ -28385,7 +28385,7 @@
         </is>
       </c>
       <c r="I65" s="61" t="n">
-        <v>0.00101025</v>
+        <v>0.0010101</v>
       </c>
       <c r="J65" s="6" t="inlineStr">
         <is>
@@ -28410,7 +28410,7 @@
         </is>
       </c>
       <c r="I66" s="61" t="n">
-        <v>0.0009951999999999999</v>
+        <v>0.00099507</v>
       </c>
       <c r="J66" s="6" t="inlineStr">
         <is>
@@ -28435,7 +28435,7 @@
         </is>
       </c>
       <c r="I67" s="61" t="n">
-        <v>0.00093075</v>
+        <v>0.0009306399999999999</v>
       </c>
       <c r="J67" s="6" t="inlineStr">
         <is>
@@ -28460,7 +28460,7 @@
         </is>
       </c>
       <c r="I68" s="61" t="n">
-        <v>0.00092899</v>
+        <v>0.00092886</v>
       </c>
       <c r="J68" s="6" t="inlineStr">
         <is>
@@ -28485,7 +28485,7 @@
         </is>
       </c>
       <c r="I69" s="61" t="n">
-        <v>0.00089978</v>
+        <v>0.00089965</v>
       </c>
       <c r="J69" s="6" t="inlineStr">
         <is>
@@ -28510,7 +28510,7 @@
         </is>
       </c>
       <c r="I70" s="61" t="n">
-        <v>0.00089479</v>
+        <v>0.00089466</v>
       </c>
       <c r="J70" s="6" t="inlineStr">
         <is>
@@ -28535,7 +28535,7 @@
         </is>
       </c>
       <c r="I71" s="61" t="n">
-        <v>0.00085287</v>
+        <v>0.0008527400000000001</v>
       </c>
       <c r="J71" s="6" t="inlineStr">
         <is>
@@ -28560,7 +28560,7 @@
         </is>
       </c>
       <c r="I72" s="61" t="n">
-        <v>0.00057239</v>
+        <v>0.0005723099999999999</v>
       </c>
       <c r="J72" s="6" t="inlineStr">
         <is>
@@ -28585,7 +28585,7 @@
         </is>
       </c>
       <c r="I73" s="61" t="n">
-        <v>0.00056285</v>
+        <v>0.00056277</v>
       </c>
       <c r="J73" s="6" t="inlineStr">
         <is>
@@ -28610,7 +28610,7 @@
         </is>
       </c>
       <c r="I74" s="61" t="n">
-        <v>0.00054509</v>
+        <v>0.00054501</v>
       </c>
       <c r="J74" s="6" t="inlineStr">
         <is>
@@ -28635,7 +28635,7 @@
         </is>
       </c>
       <c r="I75" s="61" t="n">
-        <v>0.0005197800000000001</v>
+        <v>0.00051972</v>
       </c>
       <c r="J75" s="6" t="inlineStr">
         <is>
@@ -28660,7 +28660,7 @@
         </is>
       </c>
       <c r="I76" s="61" t="n">
-        <v>0.00049706</v>
+        <v>0.00049699</v>
       </c>
       <c r="J76" s="6" t="inlineStr">
         <is>
@@ -28685,7 +28685,7 @@
         </is>
       </c>
       <c r="I77" s="61" t="n">
-        <v>0.00048956</v>
+        <v>0.00048952</v>
       </c>
       <c r="J77" s="6" t="inlineStr">
         <is>
@@ -28710,7 +28710,7 @@
         </is>
       </c>
       <c r="I78" s="61" t="n">
-        <v>0.00048258</v>
+        <v>0.00048252</v>
       </c>
       <c r="J78" s="6" t="inlineStr">
         <is>
@@ -28735,7 +28735,7 @@
         </is>
       </c>
       <c r="I79" s="61" t="n">
-        <v>0.0004816</v>
+        <v>0.00048153</v>
       </c>
       <c r="J79" s="6" t="inlineStr">
         <is>
@@ -28760,7 +28760,7 @@
         </is>
       </c>
       <c r="I80" s="61" t="n">
-        <v>0.0004767699999999999</v>
+        <v>0.00047674</v>
       </c>
       <c r="J80" s="6" t="inlineStr">
         <is>
@@ -28785,7 +28785,7 @@
         </is>
       </c>
       <c r="I81" s="61" t="n">
-        <v>0.0004612900000000001</v>
+        <v>0.00046123</v>
       </c>
       <c r="J81" s="6" t="inlineStr">
         <is>
@@ -28810,7 +28810,7 @@
         </is>
       </c>
       <c r="I82" s="61" t="n">
-        <v>0.00044961</v>
+        <v>0.00044955</v>
       </c>
       <c r="J82" s="6" t="inlineStr">
         <is>
@@ -28835,7 +28835,7 @@
         </is>
       </c>
       <c r="I83" s="61" t="n">
-        <v>0.00042413</v>
+        <v>0.00042408</v>
       </c>
       <c r="J83" s="6" t="inlineStr">
         <is>
@@ -28860,7 +28860,7 @@
         </is>
       </c>
       <c r="I84" s="61" t="n">
-        <v>0.0004150100000000001</v>
+        <v>0.00041495</v>
       </c>
       <c r="J84" s="6" t="inlineStr">
         <is>
@@ -28881,22 +28881,18 @@
     <row r="85">
       <c r="H85" s="6" t="inlineStr">
         <is>
-          <t>SRCE</t>
+          <t>GVMXX</t>
         </is>
       </c>
       <c r="I85" s="61" t="n">
-        <v>0.00037781</v>
+        <v>0.00039536</v>
       </c>
       <c r="J85" s="6" t="inlineStr">
         <is>
-          <t>1ST SOURCE</t>
-        </is>
-      </c>
-      <c r="K85" s="6" t="inlineStr">
-        <is>
-          <t>Financials</t>
-        </is>
-      </c>
+          <t>SSC GOVERNMENT MM GVMXX</t>
+        </is>
+      </c>
+      <c r="K85" s="6" t="inlineStr"/>
       <c r="L85" s="6" t="inlineStr"/>
       <c r="M85" s="7">
         <f>IF(H85="","",IFERROR(VLOOKUP(K85,$P$5:$Q$15,2,FALSE),"현금·선물"))</f>
@@ -28906,15 +28902,15 @@
     <row r="86">
       <c r="H86" s="6" t="inlineStr">
         <is>
-          <t>LKFN</t>
+          <t>SRCE</t>
         </is>
       </c>
       <c r="I86" s="61" t="n">
-        <v>0.00035679</v>
+        <v>0.00037776</v>
       </c>
       <c r="J86" s="6" t="inlineStr">
         <is>
-          <t>LAKELAND FINANCIAL CORP</t>
+          <t>1ST SOURCE</t>
         </is>
       </c>
       <c r="K86" s="6" t="inlineStr">
@@ -28931,20 +28927,20 @@
     <row r="87">
       <c r="H87" s="6" t="inlineStr">
         <is>
-          <t>BKE</t>
+          <t>LKFN</t>
         </is>
       </c>
       <c r="I87" s="61" t="n">
-        <v>0.00035411</v>
+        <v>0.00035674</v>
       </c>
       <c r="J87" s="6" t="inlineStr">
         <is>
-          <t>BUCKLE</t>
+          <t>LAKELAND FINANCIAL CORP</t>
         </is>
       </c>
       <c r="K87" s="6" t="inlineStr">
         <is>
-          <t>Consumer Discretionary</t>
+          <t>Financials</t>
         </is>
       </c>
       <c r="L87" s="6" t="inlineStr"/>
@@ -28956,20 +28952,20 @@
     <row r="88">
       <c r="H88" s="6" t="inlineStr">
         <is>
-          <t>FLO</t>
+          <t>BKE</t>
         </is>
       </c>
       <c r="I88" s="61" t="n">
-        <v>0.00032116</v>
+        <v>0.00035406</v>
       </c>
       <c r="J88" s="6" t="inlineStr">
         <is>
-          <t>FLOWERS FOODS INC</t>
+          <t>BUCKLE</t>
         </is>
       </c>
       <c r="K88" s="6" t="inlineStr">
         <is>
-          <t>Consumer Staples</t>
+          <t>Consumer Discretionary</t>
         </is>
       </c>
       <c r="L88" s="6" t="inlineStr"/>
@@ -28981,20 +28977,20 @@
     <row r="89">
       <c r="H89" s="6" t="inlineStr">
         <is>
-          <t>PFBC</t>
+          <t>FLO</t>
         </is>
       </c>
       <c r="I89" s="61" t="n">
-        <v>0.00027948</v>
+        <v>0.00032111</v>
       </c>
       <c r="J89" s="6" t="inlineStr">
         <is>
-          <t>PREFERRED BANK</t>
+          <t>FLOWERS FOODS INC</t>
         </is>
       </c>
       <c r="K89" s="6" t="inlineStr">
         <is>
-          <t>Financials</t>
+          <t>Consumer Staples</t>
         </is>
       </c>
       <c r="L89" s="6" t="inlineStr"/>
@@ -29006,20 +29002,20 @@
     <row r="90">
       <c r="H90" s="6" t="inlineStr">
         <is>
-          <t>WEN</t>
+          <t>PFBC</t>
         </is>
       </c>
       <c r="I90" s="61" t="n">
-        <v>0.00026618</v>
+        <v>0.00027945</v>
       </c>
       <c r="J90" s="6" t="inlineStr">
         <is>
-          <t>WENDYS</t>
+          <t>PREFERRED BANK</t>
         </is>
       </c>
       <c r="K90" s="6" t="inlineStr">
         <is>
-          <t>Consumer Discretionary</t>
+          <t>Financials</t>
         </is>
       </c>
       <c r="L90" s="6" t="inlineStr"/>
@@ -29031,18 +29027,22 @@
     <row r="91">
       <c r="H91" s="6" t="inlineStr">
         <is>
-          <t>GVMXX</t>
+          <t>WEN</t>
         </is>
       </c>
       <c r="I91" s="61" t="n">
-        <v>0.00025601</v>
+        <v>0.00026614</v>
       </c>
       <c r="J91" s="6" t="inlineStr">
         <is>
-          <t>SSC GOVERNMENT MM GVMXX</t>
-        </is>
-      </c>
-      <c r="K91" s="6" t="inlineStr"/>
+          <t>WENDYS</t>
+        </is>
+      </c>
+      <c r="K91" s="6" t="inlineStr">
+        <is>
+          <t>Consumer Discretionary</t>
+        </is>
+      </c>
       <c r="L91" s="6" t="inlineStr"/>
       <c r="M91" s="7">
         <f>IF(H91="","",IFERROR(VLOOKUP(K91,$P$5:$Q$15,2,FALSE),"현금·선물"))</f>
@@ -29056,7 +29056,7 @@
         </is>
       </c>
       <c r="I92" s="61" t="n">
-        <v>0.00025402</v>
+        <v>0.00025398</v>
       </c>
       <c r="J92" s="6" t="inlineStr">
         <is>
@@ -29081,7 +29081,7 @@
         </is>
       </c>
       <c r="I93" s="61" t="n">
-        <v>0.00022923</v>
+        <v>0.0002292</v>
       </c>
       <c r="J93" s="6" t="inlineStr">
         <is>
@@ -29106,7 +29106,7 @@
         </is>
       </c>
       <c r="I94" s="61" t="n">
-        <v>0.00022568</v>
+        <v>0.00022565</v>
       </c>
       <c r="J94" s="6" t="inlineStr">
         <is>
@@ -29131,7 +29131,7 @@
         </is>
       </c>
       <c r="I95" s="61" t="n">
-        <v>0.00020443</v>
+        <v>0.00020441</v>
       </c>
       <c r="J95" s="6" t="inlineStr">
         <is>
@@ -29156,7 +29156,7 @@
         </is>
       </c>
       <c r="I96" s="61" t="n">
-        <v>0.00019465</v>
+        <v>0.00019463</v>
       </c>
       <c r="J96" s="6" t="inlineStr">
         <is>
@@ -29181,7 +29181,7 @@
         </is>
       </c>
       <c r="I97" s="61" t="n">
-        <v>0.00019417</v>
+        <v>0.00019415</v>
       </c>
       <c r="J97" s="6" t="inlineStr">
         <is>
@@ -29206,7 +29206,7 @@
         </is>
       </c>
       <c r="I98" s="61" t="n">
-        <v>0.00018591</v>
+        <v>0.0001859</v>
       </c>
       <c r="J98" s="6" t="inlineStr">
         <is>
@@ -29231,7 +29231,7 @@
         </is>
       </c>
       <c r="I99" s="61" t="n">
-        <v>0.00016554</v>
+        <v>0.00016553</v>
       </c>
       <c r="J99" s="6" t="inlineStr">
         <is>
@@ -29256,7 +29256,7 @@
         </is>
       </c>
       <c r="I100" s="61" t="n">
-        <v>0.00013261</v>
+        <v>0.00013259</v>
       </c>
       <c r="J100" s="6" t="inlineStr">
         <is>
@@ -29277,22 +29277,18 @@
     <row r="101">
       <c r="H101" s="6" t="inlineStr">
         <is>
-          <t>AMSF</t>
+          <t>USD</t>
         </is>
       </c>
       <c r="I101" s="61" t="n">
-        <v>0.00011484</v>
+        <v>0.00011947</v>
       </c>
       <c r="J101" s="6" t="inlineStr">
         <is>
-          <t>AMERISAFE INC</t>
-        </is>
-      </c>
-      <c r="K101" s="6" t="inlineStr">
-        <is>
-          <t>Financials</t>
-        </is>
-      </c>
+          <t>US DOLLAR</t>
+        </is>
+      </c>
+      <c r="K101" s="6" t="inlineStr"/>
       <c r="L101" s="6" t="inlineStr"/>
       <c r="M101" s="7">
         <f>IF(H101="","",IFERROR(VLOOKUP(K101,$P$5:$Q$15,2,FALSE),"현금·선물"))</f>
@@ -29302,18 +29298,22 @@
     <row r="102">
       <c r="H102" s="6" t="inlineStr">
         <is>
-          <t>USD</t>
+          <t>AMSF</t>
         </is>
       </c>
       <c r="I102" s="61" t="n">
-        <v>0.00011285</v>
+        <v>0.00011483</v>
       </c>
       <c r="J102" s="6" t="inlineStr">
         <is>
-          <t>US DOLLAR</t>
-        </is>
-      </c>
-      <c r="K102" s="6" t="inlineStr"/>
+          <t>AMERISAFE INC</t>
+        </is>
+      </c>
+      <c r="K102" s="6" t="inlineStr">
+        <is>
+          <t>Financials</t>
+        </is>
+      </c>
       <c r="L102" s="6" t="inlineStr"/>
       <c r="M102" s="7">
         <f>IF(H102="","",IFERROR(VLOOKUP(K102,$P$5:$Q$15,2,FALSE),"현금·선물"))</f>
@@ -29327,7 +29327,7 @@
         </is>
       </c>
       <c r="I103" s="61" t="n">
-        <v>0.00010068</v>
+        <v>0.00010067</v>
       </c>
       <c r="J103" s="6" t="inlineStr">
         <is>
@@ -29352,7 +29352,7 @@
         </is>
       </c>
       <c r="I104" s="61" t="n">
-        <v>9.577e-05</v>
+        <v>9.575999999999999e-05</v>
       </c>
       <c r="J104" s="6" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
데이터 갱신: holdings (2026-10-18)
</commit_message>
<xml_diff>
--- a/downloads/schd_dividend_tracker.xlsx
+++ b/downloads/schd_dividend_tracker.xlsx
@@ -1724,7 +1724,7 @@
     <row r="3">
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>최종 갱신: 2026-10-17 · 반영 범위: 2012년 1분기 ~ 2026년 3분기 (배당락 2026-09-23) · GitHub Actions 자동 생성</t>
+          <t>최종 갱신: 2026-10-18 · 반영 범위: 2012년 1분기 ~ 2026년 3분기 (배당락 2026-09-23) · GitHub Actions 자동 생성</t>
         </is>
       </c>
     </row>
@@ -26257,11 +26257,11 @@
         </is>
       </c>
       <c r="B2" s="49" t="n">
-        <v>46310</v>
+        <v>46311</v>
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>← Schwab 공식 보유종목 CSV 기준일. 매일 자동으로 최신 파일을 받습니다.</t>
+          <t>← 이 날 종가로 계산한 비중. 그날 공식 파일을 못 받아 Schwab 공식 보유종목 CSV(2026-10-15)의 보유 주식 수 × 종가로 계산했습니다.</t>
         </is>
       </c>
     </row>
@@ -26358,7 +26358,7 @@
         </is>
       </c>
       <c r="I5" s="61" t="n">
-        <v>0.04468282000000001</v>
+        <v>0.04393346</v>
       </c>
       <c r="J5" s="6" t="inlineStr">
         <is>
@@ -26416,7 +26416,7 @@
         </is>
       </c>
       <c r="I6" s="61" t="n">
-        <v>0.04339762999999999</v>
+        <v>0.04369979</v>
       </c>
       <c r="J6" s="6" t="inlineStr">
         <is>
@@ -26470,25 +26470,25 @@
       </c>
       <c r="H7" s="6" t="inlineStr">
         <is>
-          <t>QCOM</t>
+          <t>COP</t>
         </is>
       </c>
       <c r="I7" s="61" t="n">
-        <v>0.04281518</v>
+        <v>0.04318054</v>
       </c>
       <c r="J7" s="6" t="inlineStr">
         <is>
-          <t>QUALCOMM</t>
+          <t>CONOCOPHILLIPS</t>
         </is>
       </c>
       <c r="K7" s="6" t="inlineStr">
         <is>
-          <t>Information Technology</t>
+          <t>Energy</t>
         </is>
       </c>
       <c r="L7" s="6" t="inlineStr">
         <is>
-          <t>퀄컴</t>
+          <t>코노코필립스</t>
         </is>
       </c>
       <c r="M7" s="7">
@@ -26532,7 +26532,7 @@
         </is>
       </c>
       <c r="I8" s="61" t="n">
-        <v>0.04252766</v>
+        <v>0.04308552</v>
       </c>
       <c r="J8" s="6" t="inlineStr">
         <is>
@@ -26590,7 +26590,7 @@
         </is>
       </c>
       <c r="I9" s="61" t="n">
-        <v>0.0422417</v>
+        <v>0.04301387</v>
       </c>
       <c r="J9" s="6" t="inlineStr">
         <is>
@@ -26644,25 +26644,25 @@
       </c>
       <c r="H10" s="6" t="inlineStr">
         <is>
-          <t>COP</t>
+          <t>QCOM</t>
         </is>
       </c>
       <c r="I10" s="61" t="n">
-        <v>0.0420824</v>
+        <v>0.04100069000000001</v>
       </c>
       <c r="J10" s="6" t="inlineStr">
         <is>
-          <t>CONOCOPHILLIPS</t>
+          <t>QUALCOMM</t>
         </is>
       </c>
       <c r="K10" s="6" t="inlineStr">
         <is>
-          <t>Energy</t>
+          <t>Information Technology</t>
         </is>
       </c>
       <c r="L10" s="6" t="inlineStr">
         <is>
-          <t>코노코필립스</t>
+          <t>퀄컴</t>
         </is>
       </c>
       <c r="M10" s="7">
@@ -26706,7 +26706,7 @@
         </is>
       </c>
       <c r="I11" s="61" t="n">
-        <v>0.04150475</v>
+        <v>0.04066751</v>
       </c>
       <c r="J11" s="6" t="inlineStr">
         <is>
@@ -26764,7 +26764,7 @@
         </is>
       </c>
       <c r="I12" s="61" t="n">
-        <v>0.03997775</v>
+        <v>0.03954183</v>
       </c>
       <c r="J12" s="6" t="inlineStr">
         <is>
@@ -26822,7 +26822,7 @@
         </is>
       </c>
       <c r="I13" s="61" t="n">
-        <v>0.03947407</v>
+        <v>0.03935936</v>
       </c>
       <c r="J13" s="6" t="inlineStr">
         <is>
@@ -26880,7 +26880,7 @@
         </is>
       </c>
       <c r="I14" s="61" t="n">
-        <v>0.03905457</v>
+        <v>0.03896919</v>
       </c>
       <c r="J14" s="6" t="inlineStr">
         <is>
@@ -26928,7 +26928,7 @@
         </is>
       </c>
       <c r="I15" s="61" t="n">
-        <v>0.0386517</v>
+        <v>0.03844334</v>
       </c>
       <c r="J15" s="6" t="inlineStr">
         <is>
@@ -26976,7 +26976,7 @@
         </is>
       </c>
       <c r="I16" s="61" t="n">
-        <v>0.03726557</v>
+        <v>0.03788657</v>
       </c>
       <c r="J16" s="6" t="inlineStr">
         <is>
@@ -27014,7 +27014,7 @@
         </is>
       </c>
       <c r="I17" s="61" t="n">
-        <v>0.03606252</v>
+        <v>0.03611073</v>
       </c>
       <c r="J17" s="6" t="inlineStr">
         <is>
@@ -27052,7 +27052,7 @@
         </is>
       </c>
       <c r="I18" s="61" t="n">
-        <v>0.03401827</v>
+        <v>0.03448176</v>
       </c>
       <c r="J18" s="6" t="inlineStr">
         <is>
@@ -27077,25 +27077,25 @@
     <row r="19">
       <c r="H19" s="6" t="inlineStr">
         <is>
-          <t>BMY</t>
+          <t>MO</t>
         </is>
       </c>
       <c r="I19" s="61" t="n">
-        <v>0.03058018</v>
+        <v>0.03076834</v>
       </c>
       <c r="J19" s="6" t="inlineStr">
         <is>
-          <t>BRISTOL MYERS SQUIBB</t>
+          <t>ALTRIA GROUP INC</t>
         </is>
       </c>
       <c r="K19" s="6" t="inlineStr">
         <is>
-          <t>Health Care</t>
+          <t>Consumer Staples</t>
         </is>
       </c>
       <c r="L19" s="6" t="inlineStr">
         <is>
-          <t>브리스톨마이어스스퀴브</t>
+          <t>알트리아</t>
         </is>
       </c>
       <c r="M19" s="7">
@@ -27111,25 +27111,25 @@
       </c>
       <c r="H20" s="6" t="inlineStr">
         <is>
-          <t>MO</t>
+          <t>BMY</t>
         </is>
       </c>
       <c r="I20" s="61" t="n">
-        <v>0.03047305</v>
+        <v>0.0299435</v>
       </c>
       <c r="J20" s="6" t="inlineStr">
         <is>
-          <t>ALTRIA GROUP INC</t>
+          <t>BRISTOL MYERS SQUIBB</t>
         </is>
       </c>
       <c r="K20" s="6" t="inlineStr">
         <is>
-          <t>Consumer Staples</t>
+          <t>Health Care</t>
         </is>
       </c>
       <c r="L20" s="6" t="inlineStr">
         <is>
-          <t>알트리아</t>
+          <t>브리스톨마이어스스퀴브</t>
         </is>
       </c>
       <c r="M20" s="7">
@@ -27154,7 +27154,7 @@
         </is>
       </c>
       <c r="I21" s="61" t="n">
-        <v>0.02804684</v>
+        <v>0.02815654</v>
       </c>
       <c r="J21" s="6" t="inlineStr">
         <is>
@@ -27192,7 +27192,7 @@
         </is>
       </c>
       <c r="I22" s="61" t="n">
-        <v>0.02673655</v>
+        <v>0.02750829</v>
       </c>
       <c r="J22" s="6" t="inlineStr">
         <is>
@@ -27226,25 +27226,25 @@
       </c>
       <c r="H23" s="6" t="inlineStr">
         <is>
-          <t>BX</t>
+          <t>EOG</t>
         </is>
       </c>
       <c r="I23" s="61" t="n">
-        <v>0.02025903</v>
+        <v>0.02033334</v>
       </c>
       <c r="J23" s="6" t="inlineStr">
         <is>
-          <t>BLACKSTONE</t>
+          <t>EOG RESOURCES</t>
         </is>
       </c>
       <c r="K23" s="6" t="inlineStr">
         <is>
-          <t>Financials</t>
+          <t>Energy</t>
         </is>
       </c>
       <c r="L23" s="6" t="inlineStr">
         <is>
-          <t>블랙스톤</t>
+          <t>EOG 리소시스</t>
         </is>
       </c>
       <c r="M23" s="7">
@@ -27264,25 +27264,25 @@
       </c>
       <c r="H24" s="6" t="inlineStr">
         <is>
-          <t>EOG</t>
+          <t>BX</t>
         </is>
       </c>
       <c r="I24" s="61" t="n">
-        <v>0.01978579</v>
+        <v>0.01963252</v>
       </c>
       <c r="J24" s="6" t="inlineStr">
         <is>
-          <t>EOG RESOURCES</t>
+          <t>BLACKSTONE</t>
         </is>
       </c>
       <c r="K24" s="6" t="inlineStr">
         <is>
-          <t>Energy</t>
+          <t>Financials</t>
         </is>
       </c>
       <c r="L24" s="6" t="inlineStr">
         <is>
-          <t>EOG 리소시스</t>
+          <t>블랙스톤</t>
         </is>
       </c>
       <c r="M24" s="7">
@@ -27306,7 +27306,7 @@
         </is>
       </c>
       <c r="I25" s="61" t="n">
-        <v>0.01904309</v>
+        <v>0.01901539</v>
       </c>
       <c r="J25" s="6" t="inlineStr">
         <is>
@@ -27340,25 +27340,25 @@
       </c>
       <c r="H26" s="6" t="inlineStr">
         <is>
-          <t>UPS</t>
+          <t>SLB</t>
         </is>
       </c>
       <c r="I26" s="61" t="n">
-        <v>0.01811879</v>
+        <v>0.01802343</v>
       </c>
       <c r="J26" s="6" t="inlineStr">
         <is>
-          <t>UNITED PARCEL SERVICE INC CLASS B</t>
+          <t>SLB</t>
         </is>
       </c>
       <c r="K26" s="6" t="inlineStr">
         <is>
-          <t>Industrials</t>
+          <t>Energy</t>
         </is>
       </c>
       <c r="L26" s="6" t="inlineStr">
         <is>
-          <t>UPS</t>
+          <t>SLB</t>
         </is>
       </c>
       <c r="M26" s="7">
@@ -27378,25 +27378,25 @@
       </c>
       <c r="H27" s="6" t="inlineStr">
         <is>
-          <t>SLB</t>
+          <t>UPS</t>
         </is>
       </c>
       <c r="I27" s="61" t="n">
-        <v>0.01774296</v>
+        <v>0.0179207</v>
       </c>
       <c r="J27" s="6" t="inlineStr">
         <is>
-          <t>SLB</t>
+          <t>UNITED PARCEL SERVICE INC CLASS B</t>
         </is>
       </c>
       <c r="K27" s="6" t="inlineStr">
         <is>
-          <t>Energy</t>
+          <t>Industrials</t>
         </is>
       </c>
       <c r="L27" s="6" t="inlineStr">
         <is>
-          <t>SLB</t>
+          <t>UPS</t>
         </is>
       </c>
       <c r="M27" s="7">
@@ -27420,7 +27420,7 @@
         </is>
       </c>
       <c r="I28" s="61" t="n">
-        <v>0.01758271</v>
+        <v>0.01718883</v>
       </c>
       <c r="J28" s="6" t="inlineStr">
         <is>
@@ -27454,27 +27454,23 @@
       </c>
       <c r="H29" s="6" t="inlineStr">
         <is>
-          <t>FAST</t>
+          <t>OKE</t>
         </is>
       </c>
       <c r="I29" s="61" t="n">
-        <v>0.01428842</v>
+        <v>0.01443041</v>
       </c>
       <c r="J29" s="6" t="inlineStr">
         <is>
-          <t>FASTENAL</t>
+          <t>ONEOK</t>
         </is>
       </c>
       <c r="K29" s="6" t="inlineStr">
         <is>
-          <t>Industrials</t>
-        </is>
-      </c>
-      <c r="L29" s="6" t="inlineStr">
-        <is>
-          <t>패스널</t>
-        </is>
-      </c>
+          <t>Energy</t>
+        </is>
+      </c>
+      <c r="L29" s="6" t="inlineStr"/>
       <c r="M29" s="7">
         <f>IF(H29="","",IFERROR(VLOOKUP(K29,$P$5:$Q$15,2,FALSE),"현금·선물"))</f>
         <v/>
@@ -27492,23 +27488,27 @@
       </c>
       <c r="H30" s="6" t="inlineStr">
         <is>
-          <t>OKE</t>
+          <t>FAST</t>
         </is>
       </c>
       <c r="I30" s="61" t="n">
-        <v>0.0141233</v>
+        <v>0.01436311</v>
       </c>
       <c r="J30" s="6" t="inlineStr">
         <is>
-          <t>ONEOK</t>
+          <t>FASTENAL</t>
         </is>
       </c>
       <c r="K30" s="6" t="inlineStr">
         <is>
-          <t>Energy</t>
-        </is>
-      </c>
-      <c r="L30" s="6" t="inlineStr"/>
+          <t>Industrials</t>
+        </is>
+      </c>
+      <c r="L30" s="6" t="inlineStr">
+        <is>
+          <t>패스널</t>
+        </is>
+      </c>
       <c r="M30" s="7">
         <f>IF(H30="","",IFERROR(VLOOKUP(K30,$P$5:$Q$15,2,FALSE),"현금·선물"))</f>
         <v/>
@@ -27530,7 +27530,7 @@
         </is>
       </c>
       <c r="I31" s="61" t="n">
-        <v>0.01338705</v>
+        <v>0.01369032</v>
       </c>
       <c r="J31" s="6" t="inlineStr">
         <is>
@@ -27555,7 +27555,7 @@
         </is>
       </c>
       <c r="I32" s="61" t="n">
-        <v>0.01191675</v>
+        <v>0.01194409</v>
       </c>
       <c r="J32" s="6" t="inlineStr">
         <is>
@@ -27585,7 +27585,7 @@
         </is>
       </c>
       <c r="I33" s="61" t="n">
-        <v>0.01128573</v>
+        <v>0.01120687</v>
       </c>
       <c r="J33" s="6" t="inlineStr">
         <is>
@@ -27610,7 +27610,7 @@
         </is>
       </c>
       <c r="I34" s="61" t="n">
-        <v>0.00987858</v>
+        <v>0.00976781</v>
       </c>
       <c r="J34" s="6" t="inlineStr">
         <is>
@@ -27635,7 +27635,7 @@
         </is>
       </c>
       <c r="I35" s="61" t="n">
-        <v>0.0087647</v>
+        <v>0.00876676</v>
       </c>
       <c r="J35" s="6" t="inlineStr">
         <is>
@@ -27660,7 +27660,7 @@
         </is>
       </c>
       <c r="I36" s="61" t="n">
-        <v>0.00855439</v>
+        <v>0.008613619999999999</v>
       </c>
       <c r="J36" s="6" t="inlineStr">
         <is>
@@ -27685,7 +27685,7 @@
         </is>
       </c>
       <c r="I37" s="61" t="n">
-        <v>0.00634309</v>
+        <v>0.00644801</v>
       </c>
       <c r="J37" s="6" t="inlineStr">
         <is>
@@ -27710,7 +27710,7 @@
         </is>
       </c>
       <c r="I38" s="61" t="n">
-        <v>0.00631188</v>
+        <v>0.006168590000000001</v>
       </c>
       <c r="J38" s="6" t="inlineStr">
         <is>
@@ -27735,7 +27735,7 @@
         </is>
       </c>
       <c r="I39" s="61" t="n">
-        <v>0.00609971</v>
+        <v>0.00613186</v>
       </c>
       <c r="J39" s="6" t="inlineStr">
         <is>
@@ -27760,7 +27760,7 @@
         </is>
       </c>
       <c r="I40" s="61" t="n">
-        <v>0.00601391</v>
+        <v>0.00602634</v>
       </c>
       <c r="J40" s="6" t="inlineStr">
         <is>
@@ -27785,7 +27785,7 @@
         </is>
       </c>
       <c r="I41" s="61" t="n">
-        <v>0.00575046</v>
+        <v>0.00573727</v>
       </c>
       <c r="J41" s="6" t="inlineStr">
         <is>
@@ -27810,7 +27810,7 @@
         </is>
       </c>
       <c r="I42" s="61" t="n">
-        <v>0.00534448</v>
+        <v>0.005284100000000001</v>
       </c>
       <c r="J42" s="6" t="inlineStr">
         <is>
@@ -27835,7 +27835,7 @@
         </is>
       </c>
       <c r="I43" s="61" t="n">
-        <v>0.005247089999999999</v>
+        <v>0.00520119</v>
       </c>
       <c r="J43" s="6" t="inlineStr">
         <is>
@@ -27860,7 +27860,7 @@
         </is>
       </c>
       <c r="I44" s="61" t="n">
-        <v>0.00490793</v>
+        <v>0.00489968</v>
       </c>
       <c r="J44" s="6" t="inlineStr">
         <is>
@@ -27885,7 +27885,7 @@
         </is>
       </c>
       <c r="I45" s="61" t="n">
-        <v>0.00476494</v>
+        <v>0.00475214</v>
       </c>
       <c r="J45" s="6" t="inlineStr">
         <is>
@@ -27910,7 +27910,7 @@
         </is>
       </c>
       <c r="I46" s="61" t="n">
-        <v>0.00467843</v>
+        <v>0.0046609</v>
       </c>
       <c r="J46" s="6" t="inlineStr">
         <is>
@@ -27935,7 +27935,7 @@
         </is>
       </c>
       <c r="I47" s="61" t="n">
-        <v>0.00460881</v>
+        <v>0.00449997</v>
       </c>
       <c r="J47" s="6" t="inlineStr">
         <is>
@@ -27960,7 +27960,7 @@
         </is>
       </c>
       <c r="I48" s="61" t="n">
-        <v>0.00434558</v>
+        <v>0.0043463</v>
       </c>
       <c r="J48" s="6" t="inlineStr">
         <is>
@@ -27985,7 +27985,7 @@
         </is>
       </c>
       <c r="I49" s="61" t="n">
-        <v>0.00427618</v>
+        <v>0.00426545</v>
       </c>
       <c r="J49" s="6" t="inlineStr">
         <is>
@@ -28010,7 +28010,7 @@
         </is>
       </c>
       <c r="I50" s="61" t="n">
-        <v>0.00408974</v>
+        <v>0.00422458</v>
       </c>
       <c r="J50" s="6" t="inlineStr">
         <is>
@@ -28035,7 +28035,7 @@
         </is>
       </c>
       <c r="I51" s="61" t="n">
-        <v>0.00263459</v>
+        <v>0.00258379</v>
       </c>
       <c r="J51" s="6" t="inlineStr">
         <is>
@@ -28056,15 +28056,15 @@
     <row r="52">
       <c r="H52" s="6" t="inlineStr">
         <is>
-          <t>FNF</t>
+          <t>AFG</t>
         </is>
       </c>
       <c r="I52" s="61" t="n">
-        <v>0.00249672</v>
+        <v>0.00251532</v>
       </c>
       <c r="J52" s="6" t="inlineStr">
         <is>
-          <t>FIDELITY NATIONAL FINANCIAL INC</t>
+          <t>AMERICAN FINANCIAL GROUP</t>
         </is>
       </c>
       <c r="K52" s="6" t="inlineStr">
@@ -28081,15 +28081,15 @@
     <row r="53">
       <c r="H53" s="6" t="inlineStr">
         <is>
-          <t>AFG</t>
+          <t>FNF</t>
         </is>
       </c>
       <c r="I53" s="61" t="n">
-        <v>0.00247625</v>
+        <v>0.0025014</v>
       </c>
       <c r="J53" s="6" t="inlineStr">
         <is>
-          <t>AMERICAN FINANCIAL GROUP</t>
+          <t>FIDELITY NATIONAL FINANCIAL INC</t>
         </is>
       </c>
       <c r="K53" s="6" t="inlineStr">
@@ -28110,7 +28110,7 @@
         </is>
       </c>
       <c r="I54" s="61" t="n">
-        <v>0.00221359</v>
+        <v>0.00219017</v>
       </c>
       <c r="J54" s="6" t="inlineStr">
         <is>
@@ -28135,7 +28135,7 @@
         </is>
       </c>
       <c r="I55" s="61" t="n">
-        <v>0.00212205</v>
+        <v>0.00216031</v>
       </c>
       <c r="J55" s="6" t="inlineStr">
         <is>
@@ -28160,7 +28160,7 @@
         </is>
       </c>
       <c r="I56" s="61" t="n">
-        <v>0.00199989</v>
+        <v>0.00197196</v>
       </c>
       <c r="J56" s="6" t="inlineStr">
         <is>
@@ -28185,7 +28185,7 @@
         </is>
       </c>
       <c r="I57" s="61" t="n">
-        <v>0.00190934</v>
+        <v>0.00189573</v>
       </c>
       <c r="J57" s="6" t="inlineStr">
         <is>
@@ -28210,7 +28210,7 @@
         </is>
       </c>
       <c r="I58" s="61" t="n">
-        <v>0.0015731</v>
+        <v>0.00154731</v>
       </c>
       <c r="J58" s="6" t="inlineStr">
         <is>
@@ -28235,7 +28235,7 @@
         </is>
       </c>
       <c r="I59" s="61" t="n">
-        <v>0.00152475</v>
+        <v>0.00154533</v>
       </c>
       <c r="J59" s="6" t="inlineStr">
         <is>
@@ -28260,7 +28260,7 @@
         </is>
       </c>
       <c r="I60" s="61" t="n">
-        <v>0.00148002</v>
+        <v>0.0014655</v>
       </c>
       <c r="J60" s="6" t="inlineStr">
         <is>
@@ -28281,20 +28281,20 @@
     <row r="61">
       <c r="H61" s="6" t="inlineStr">
         <is>
-          <t>MTN</t>
+          <t>MUR</t>
         </is>
       </c>
       <c r="I61" s="61" t="n">
-        <v>0.00134755</v>
+        <v>0.00138152</v>
       </c>
       <c r="J61" s="6" t="inlineStr">
         <is>
-          <t>VAIL RESORTS</t>
+          <t>MURPHY OIL</t>
         </is>
       </c>
       <c r="K61" s="6" t="inlineStr">
         <is>
-          <t>Consumer Discretionary</t>
+          <t>Energy</t>
         </is>
       </c>
       <c r="L61" s="6" t="inlineStr"/>
@@ -28306,20 +28306,20 @@
     <row r="62">
       <c r="H62" s="6" t="inlineStr">
         <is>
-          <t>MUR</t>
+          <t>MTN</t>
         </is>
       </c>
       <c r="I62" s="61" t="n">
-        <v>0.00132877</v>
+        <v>0.00132055</v>
       </c>
       <c r="J62" s="6" t="inlineStr">
         <is>
-          <t>MURPHY OIL</t>
+          <t>VAIL RESORTS</t>
         </is>
       </c>
       <c r="K62" s="6" t="inlineStr">
         <is>
-          <t>Energy</t>
+          <t>Consumer Discretionary</t>
         </is>
       </c>
       <c r="L62" s="6" t="inlineStr"/>
@@ -28335,7 +28335,7 @@
         </is>
       </c>
       <c r="I63" s="61" t="n">
-        <v>0.00118004</v>
+        <v>0.0011709</v>
       </c>
       <c r="J63" s="6" t="inlineStr">
         <is>
@@ -28360,7 +28360,7 @@
         </is>
       </c>
       <c r="I64" s="61" t="n">
-        <v>0.00115056</v>
+        <v>0.00114904</v>
       </c>
       <c r="J64" s="6" t="inlineStr">
         <is>
@@ -28385,7 +28385,7 @@
         </is>
       </c>
       <c r="I65" s="61" t="n">
-        <v>0.0010101</v>
+        <v>0.00098869</v>
       </c>
       <c r="J65" s="6" t="inlineStr">
         <is>
@@ -28410,7 +28410,7 @@
         </is>
       </c>
       <c r="I66" s="61" t="n">
-        <v>0.00099507</v>
+        <v>0.00097828</v>
       </c>
       <c r="J66" s="6" t="inlineStr">
         <is>
@@ -28435,7 +28435,7 @@
         </is>
       </c>
       <c r="I67" s="61" t="n">
-        <v>0.0009306399999999999</v>
+        <v>0.0009256000000000001</v>
       </c>
       <c r="J67" s="6" t="inlineStr">
         <is>
@@ -28460,7 +28460,7 @@
         </is>
       </c>
       <c r="I68" s="61" t="n">
-        <v>0.00092886</v>
+        <v>0.0009221300000000001</v>
       </c>
       <c r="J68" s="6" t="inlineStr">
         <is>
@@ -28485,7 +28485,7 @@
         </is>
       </c>
       <c r="I69" s="61" t="n">
-        <v>0.00089965</v>
+        <v>0.00089464</v>
       </c>
       <c r="J69" s="6" t="inlineStr">
         <is>
@@ -28510,7 +28510,7 @@
         </is>
       </c>
       <c r="I70" s="61" t="n">
-        <v>0.00089466</v>
+        <v>0.0008871700000000001</v>
       </c>
       <c r="J70" s="6" t="inlineStr">
         <is>
@@ -28535,7 +28535,7 @@
         </is>
       </c>
       <c r="I71" s="61" t="n">
-        <v>0.0008527400000000001</v>
+        <v>0.00081987</v>
       </c>
       <c r="J71" s="6" t="inlineStr">
         <is>
@@ -28556,15 +28556,15 @@
     <row r="72">
       <c r="H72" s="6" t="inlineStr">
         <is>
-          <t>APAM</t>
+          <t>BANR</t>
         </is>
       </c>
       <c r="I72" s="61" t="n">
-        <v>0.0005723099999999999</v>
+        <v>0.0005605299999999999</v>
       </c>
       <c r="J72" s="6" t="inlineStr">
         <is>
-          <t>ARTISAN PARTNERS ASSET MANAGEMENT</t>
+          <t>BANNER CORP</t>
         </is>
       </c>
       <c r="K72" s="6" t="inlineStr">
@@ -28581,15 +28581,15 @@
     <row r="73">
       <c r="H73" s="6" t="inlineStr">
         <is>
-          <t>BANR</t>
+          <t>APAM</t>
         </is>
       </c>
       <c r="I73" s="61" t="n">
-        <v>0.00056277</v>
+        <v>0.00055993</v>
       </c>
       <c r="J73" s="6" t="inlineStr">
         <is>
-          <t>BANNER CORP</t>
+          <t>ARTISAN PARTNERS ASSET MANAGEMENT</t>
         </is>
       </c>
       <c r="K73" s="6" t="inlineStr">
@@ -28610,7 +28610,7 @@
         </is>
       </c>
       <c r="I74" s="61" t="n">
-        <v>0.00054501</v>
+        <v>0.00054628</v>
       </c>
       <c r="J74" s="6" t="inlineStr">
         <is>
@@ -28635,7 +28635,7 @@
         </is>
       </c>
       <c r="I75" s="61" t="n">
-        <v>0.00051972</v>
+        <v>0.00051849</v>
       </c>
       <c r="J75" s="6" t="inlineStr">
         <is>
@@ -28660,7 +28660,7 @@
         </is>
       </c>
       <c r="I76" s="61" t="n">
-        <v>0.00049699</v>
+        <v>0.00049944</v>
       </c>
       <c r="J76" s="6" t="inlineStr">
         <is>
@@ -28685,7 +28685,7 @@
         </is>
       </c>
       <c r="I77" s="61" t="n">
-        <v>0.00048952</v>
+        <v>0.00048849</v>
       </c>
       <c r="J77" s="6" t="inlineStr">
         <is>
@@ -28710,7 +28710,7 @@
         </is>
       </c>
       <c r="I78" s="61" t="n">
-        <v>0.00048252</v>
+        <v>0.00048348</v>
       </c>
       <c r="J78" s="6" t="inlineStr">
         <is>
@@ -28735,7 +28735,7 @@
         </is>
       </c>
       <c r="I79" s="61" t="n">
-        <v>0.00048153</v>
+        <v>0.00047337</v>
       </c>
       <c r="J79" s="6" t="inlineStr">
         <is>
@@ -28760,7 +28760,7 @@
         </is>
       </c>
       <c r="I80" s="61" t="n">
-        <v>0.00047674</v>
+        <v>0.00046806</v>
       </c>
       <c r="J80" s="6" t="inlineStr">
         <is>
@@ -28785,7 +28785,7 @@
         </is>
       </c>
       <c r="I81" s="61" t="n">
-        <v>0.00046123</v>
+        <v>0.00046152</v>
       </c>
       <c r="J81" s="6" t="inlineStr">
         <is>
@@ -28810,7 +28810,7 @@
         </is>
       </c>
       <c r="I82" s="61" t="n">
-        <v>0.00044955</v>
+        <v>0.00045132</v>
       </c>
       <c r="J82" s="6" t="inlineStr">
         <is>
@@ -28835,7 +28835,7 @@
         </is>
       </c>
       <c r="I83" s="61" t="n">
-        <v>0.00042408</v>
+        <v>0.00042364</v>
       </c>
       <c r="J83" s="6" t="inlineStr">
         <is>
@@ -28860,7 +28860,7 @@
         </is>
       </c>
       <c r="I84" s="61" t="n">
-        <v>0.00041495</v>
+        <v>0.00041385</v>
       </c>
       <c r="J84" s="6" t="inlineStr">
         <is>
@@ -28885,7 +28885,7 @@
         </is>
       </c>
       <c r="I85" s="61" t="n">
-        <v>0.00039536</v>
+        <v>0.00039244</v>
       </c>
       <c r="J85" s="6" t="inlineStr">
         <is>
@@ -28906,7 +28906,7 @@
         </is>
       </c>
       <c r="I86" s="61" t="n">
-        <v>0.00037776</v>
+        <v>0.00037642</v>
       </c>
       <c r="J86" s="6" t="inlineStr">
         <is>
@@ -28931,7 +28931,7 @@
         </is>
       </c>
       <c r="I87" s="61" t="n">
-        <v>0.00035674</v>
+        <v>0.00035466</v>
       </c>
       <c r="J87" s="6" t="inlineStr">
         <is>
@@ -28956,7 +28956,7 @@
         </is>
       </c>
       <c r="I88" s="61" t="n">
-        <v>0.00035406</v>
+        <v>0.00035092</v>
       </c>
       <c r="J88" s="6" t="inlineStr">
         <is>
@@ -28981,7 +28981,7 @@
         </is>
       </c>
       <c r="I89" s="61" t="n">
-        <v>0.00032111</v>
+        <v>0.00031822</v>
       </c>
       <c r="J89" s="6" t="inlineStr">
         <is>
@@ -29006,7 +29006,7 @@
         </is>
       </c>
       <c r="I90" s="61" t="n">
-        <v>0.00027945</v>
+        <v>0.00027958</v>
       </c>
       <c r="J90" s="6" t="inlineStr">
         <is>
@@ -29031,7 +29031,7 @@
         </is>
       </c>
       <c r="I91" s="61" t="n">
-        <v>0.00026614</v>
+        <v>0.00026418</v>
       </c>
       <c r="J91" s="6" t="inlineStr">
         <is>
@@ -29056,7 +29056,7 @@
         </is>
       </c>
       <c r="I92" s="61" t="n">
-        <v>0.00025398</v>
+        <v>0.00025525</v>
       </c>
       <c r="J92" s="6" t="inlineStr">
         <is>
@@ -29081,7 +29081,7 @@
         </is>
       </c>
       <c r="I93" s="61" t="n">
-        <v>0.0002292</v>
+        <v>0.0002299</v>
       </c>
       <c r="J93" s="6" t="inlineStr">
         <is>
@@ -29106,7 +29106,7 @@
         </is>
       </c>
       <c r="I94" s="61" t="n">
-        <v>0.00022565</v>
+        <v>0.00022529</v>
       </c>
       <c r="J94" s="6" t="inlineStr">
         <is>
@@ -29131,7 +29131,7 @@
         </is>
       </c>
       <c r="I95" s="61" t="n">
-        <v>0.00020441</v>
+        <v>0.00020373</v>
       </c>
       <c r="J95" s="6" t="inlineStr">
         <is>
@@ -29152,15 +29152,15 @@
     <row r="96">
       <c r="H96" s="6" t="inlineStr">
         <is>
-          <t>THFF</t>
+          <t>IBCP</t>
         </is>
       </c>
       <c r="I96" s="61" t="n">
-        <v>0.00019463</v>
+        <v>0.00019441</v>
       </c>
       <c r="J96" s="6" t="inlineStr">
         <is>
-          <t>FIRST FINANCIAL CORPORATION CORP</t>
+          <t>INDEPENDENT BANK CORP</t>
         </is>
       </c>
       <c r="K96" s="6" t="inlineStr">
@@ -29177,15 +29177,15 @@
     <row r="97">
       <c r="H97" s="6" t="inlineStr">
         <is>
-          <t>IBCP</t>
+          <t>THFF</t>
         </is>
       </c>
       <c r="I97" s="61" t="n">
-        <v>0.00019415</v>
+        <v>0.0001943</v>
       </c>
       <c r="J97" s="6" t="inlineStr">
         <is>
-          <t>INDEPENDENT BANK CORP</t>
+          <t>FIRST FINANCIAL CORPORATION CORP</t>
         </is>
       </c>
       <c r="K97" s="6" t="inlineStr">
@@ -29206,7 +29206,7 @@
         </is>
       </c>
       <c r="I98" s="61" t="n">
-        <v>0.0001859</v>
+        <v>0.00018458</v>
       </c>
       <c r="J98" s="6" t="inlineStr">
         <is>
@@ -29231,7 +29231,7 @@
         </is>
       </c>
       <c r="I99" s="61" t="n">
-        <v>0.00016553</v>
+        <v>0.00016498</v>
       </c>
       <c r="J99" s="6" t="inlineStr">
         <is>
@@ -29256,7 +29256,7 @@
         </is>
       </c>
       <c r="I100" s="61" t="n">
-        <v>0.00013259</v>
+        <v>0.00013126</v>
       </c>
       <c r="J100" s="6" t="inlineStr">
         <is>
@@ -29281,7 +29281,7 @@
         </is>
       </c>
       <c r="I101" s="61" t="n">
-        <v>0.00011947</v>
+        <v>0.00011859</v>
       </c>
       <c r="J101" s="6" t="inlineStr">
         <is>
@@ -29302,7 +29302,7 @@
         </is>
       </c>
       <c r="I102" s="61" t="n">
-        <v>0.00011483</v>
+        <v>0.00011494</v>
       </c>
       <c r="J102" s="6" t="inlineStr">
         <is>
@@ -29327,7 +29327,7 @@
         </is>
       </c>
       <c r="I103" s="61" t="n">
-        <v>0.00010067</v>
+        <v>9.831e-05</v>
       </c>
       <c r="J103" s="6" t="inlineStr">
         <is>
@@ -29352,7 +29352,7 @@
         </is>
       </c>
       <c r="I104" s="61" t="n">
-        <v>9.575999999999999e-05</v>
+        <v>9.007e-05</v>
       </c>
       <c r="J104" s="6" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
데이터 갱신: holdings (2026-10-20)
</commit_message>
<xml_diff>
--- a/downloads/schd_dividend_tracker.xlsx
+++ b/downloads/schd_dividend_tracker.xlsx
@@ -1724,7 +1724,7 @@
     <row r="3">
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>최종 갱신: 2026-10-18 · 반영 범위: 2012년 1분기 ~ 2026년 3분기 (배당락 2026-09-23) · GitHub Actions 자동 생성</t>
+          <t>최종 갱신: 2026-10-20 · 반영 범위: 2012년 1분기 ~ 2026년 3분기 (배당락 2026-09-23) · GitHub Actions 자동 생성</t>
         </is>
       </c>
     </row>
@@ -26257,11 +26257,11 @@
         </is>
       </c>
       <c r="B2" s="49" t="n">
-        <v>46311</v>
+        <v>46314</v>
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>← 이 날 종가로 계산한 비중. 그날 공식 파일을 못 받아 Schwab 공식 보유종목 CSV(2026-10-15)의 보유 주식 수 × 종가로 계산했습니다.</t>
+          <t>← 이 날 종가로 계산한 비중. 그날 공식 파일을 못 받아 Schwab 공식 보유종목 CSV(2026-10-16)의 보유 주식 수 × 종가로 계산했습니다.</t>
         </is>
       </c>
     </row>
@@ -26358,7 +26358,7 @@
         </is>
       </c>
       <c r="I5" s="61" t="n">
-        <v>0.04393346</v>
+        <v>0.04404334000000001</v>
       </c>
       <c r="J5" s="6" t="inlineStr">
         <is>
@@ -26416,7 +26416,7 @@
         </is>
       </c>
       <c r="I6" s="61" t="n">
-        <v>0.04369979</v>
+        <v>0.04340455000000001</v>
       </c>
       <c r="J6" s="6" t="inlineStr">
         <is>
@@ -26470,15 +26470,15 @@
       </c>
       <c r="H7" s="6" t="inlineStr">
         <is>
-          <t>COP</t>
+          <t>CVX</t>
         </is>
       </c>
       <c r="I7" s="61" t="n">
-        <v>0.04318054</v>
+        <v>0.04305399000000001</v>
       </c>
       <c r="J7" s="6" t="inlineStr">
         <is>
-          <t>CONOCOPHILLIPS</t>
+          <t>CHEVRON</t>
         </is>
       </c>
       <c r="K7" s="6" t="inlineStr">
@@ -26488,7 +26488,7 @@
       </c>
       <c r="L7" s="6" t="inlineStr">
         <is>
-          <t>코노코필립스</t>
+          <t>셰브론</t>
         </is>
       </c>
       <c r="M7" s="7">
@@ -26532,7 +26532,7 @@
         </is>
       </c>
       <c r="I8" s="61" t="n">
-        <v>0.04308552</v>
+        <v>0.04302386</v>
       </c>
       <c r="J8" s="6" t="inlineStr">
         <is>
@@ -26586,15 +26586,15 @@
       </c>
       <c r="H9" s="6" t="inlineStr">
         <is>
-          <t>CVX</t>
+          <t>COP</t>
         </is>
       </c>
       <c r="I9" s="61" t="n">
-        <v>0.04301387</v>
+        <v>0.04296461</v>
       </c>
       <c r="J9" s="6" t="inlineStr">
         <is>
-          <t>CHEVRON</t>
+          <t>CONOCOPHILLIPS</t>
         </is>
       </c>
       <c r="K9" s="6" t="inlineStr">
@@ -26604,7 +26604,7 @@
       </c>
       <c r="L9" s="6" t="inlineStr">
         <is>
-          <t>셰브론</t>
+          <t>코노코필립스</t>
         </is>
       </c>
       <c r="M9" s="7">
@@ -26648,7 +26648,7 @@
         </is>
       </c>
       <c r="I10" s="61" t="n">
-        <v>0.04100069000000001</v>
+        <v>0.0414919</v>
       </c>
       <c r="J10" s="6" t="inlineStr">
         <is>
@@ -26706,7 +26706,7 @@
         </is>
       </c>
       <c r="I11" s="61" t="n">
-        <v>0.04066751</v>
+        <v>0.04137204</v>
       </c>
       <c r="J11" s="6" t="inlineStr">
         <is>
@@ -26760,25 +26760,25 @@
       </c>
       <c r="H12" s="6" t="inlineStr">
         <is>
-          <t>AMGN</t>
+          <t>HD</t>
         </is>
       </c>
       <c r="I12" s="61" t="n">
-        <v>0.03954183</v>
+        <v>0.03953678</v>
       </c>
       <c r="J12" s="6" t="inlineStr">
         <is>
-          <t>AMGEN INC</t>
+          <t>HOME DEPOT</t>
         </is>
       </c>
       <c r="K12" s="6" t="inlineStr">
         <is>
-          <t>Health Care</t>
+          <t>Consumer Discretionary</t>
         </is>
       </c>
       <c r="L12" s="6" t="inlineStr">
         <is>
-          <t>암젠</t>
+          <t>홈디포</t>
         </is>
       </c>
       <c r="M12" s="7">
@@ -26818,25 +26818,25 @@
       </c>
       <c r="H13" s="6" t="inlineStr">
         <is>
-          <t>HD</t>
+          <t>AMGN</t>
         </is>
       </c>
       <c r="I13" s="61" t="n">
-        <v>0.03935936</v>
+        <v>0.03899518</v>
       </c>
       <c r="J13" s="6" t="inlineStr">
         <is>
-          <t>HOME DEPOT</t>
+          <t>AMGEN INC</t>
         </is>
       </c>
       <c r="K13" s="6" t="inlineStr">
         <is>
-          <t>Consumer Discretionary</t>
+          <t>Health Care</t>
         </is>
       </c>
       <c r="L13" s="6" t="inlineStr">
         <is>
-          <t>홈디포</t>
+          <t>암젠</t>
         </is>
       </c>
       <c r="M13" s="7">
@@ -26876,25 +26876,25 @@
       </c>
       <c r="H14" s="6" t="inlineStr">
         <is>
-          <t>MRK</t>
+          <t>PEP</t>
         </is>
       </c>
       <c r="I14" s="61" t="n">
-        <v>0.03896919</v>
+        <v>0.03862823</v>
       </c>
       <c r="J14" s="6" t="inlineStr">
         <is>
-          <t>MERCK &amp; CO INC</t>
+          <t>PEPSICO</t>
         </is>
       </c>
       <c r="K14" s="6" t="inlineStr">
         <is>
-          <t>Health Care</t>
+          <t>Consumer Staples</t>
         </is>
       </c>
       <c r="L14" s="6" t="inlineStr">
         <is>
-          <t>머크</t>
+          <t>펩시코</t>
         </is>
       </c>
       <c r="M14" s="7">
@@ -26924,15 +26924,15 @@
       </c>
       <c r="H15" s="6" t="inlineStr">
         <is>
-          <t>ABT</t>
+          <t>MRK</t>
         </is>
       </c>
       <c r="I15" s="61" t="n">
-        <v>0.03844334</v>
+        <v>0.0384916</v>
       </c>
       <c r="J15" s="6" t="inlineStr">
         <is>
-          <t>ABBOTT LABORATORIES</t>
+          <t>MERCK &amp; CO INC</t>
         </is>
       </c>
       <c r="K15" s="6" t="inlineStr">
@@ -26942,7 +26942,7 @@
       </c>
       <c r="L15" s="6" t="inlineStr">
         <is>
-          <t>애보트</t>
+          <t>머크</t>
         </is>
       </c>
       <c r="M15" s="7">
@@ -26972,25 +26972,25 @@
       </c>
       <c r="H16" s="6" t="inlineStr">
         <is>
-          <t>PEP</t>
+          <t>ABT</t>
         </is>
       </c>
       <c r="I16" s="61" t="n">
-        <v>0.03788657</v>
+        <v>0.03828023</v>
       </c>
       <c r="J16" s="6" t="inlineStr">
         <is>
-          <t>PEPSICO</t>
+          <t>ABBOTT LABORATORIES</t>
         </is>
       </c>
       <c r="K16" s="6" t="inlineStr">
         <is>
-          <t>Consumer Staples</t>
+          <t>Health Care</t>
         </is>
       </c>
       <c r="L16" s="6" t="inlineStr">
         <is>
-          <t>펩시코</t>
+          <t>애보트</t>
         </is>
       </c>
       <c r="M16" s="7">
@@ -27014,7 +27014,7 @@
         </is>
       </c>
       <c r="I17" s="61" t="n">
-        <v>0.03611073</v>
+        <v>0.03572645</v>
       </c>
       <c r="J17" s="6" t="inlineStr">
         <is>
@@ -27052,7 +27052,7 @@
         </is>
       </c>
       <c r="I18" s="61" t="n">
-        <v>0.03448176</v>
+        <v>0.03570178</v>
       </c>
       <c r="J18" s="6" t="inlineStr">
         <is>
@@ -27081,7 +27081,7 @@
         </is>
       </c>
       <c r="I19" s="61" t="n">
-        <v>0.03076834</v>
+        <v>0.03046279</v>
       </c>
       <c r="J19" s="6" t="inlineStr">
         <is>
@@ -27115,7 +27115,7 @@
         </is>
       </c>
       <c r="I20" s="61" t="n">
-        <v>0.0299435</v>
+        <v>0.02959153</v>
       </c>
       <c r="J20" s="6" t="inlineStr">
         <is>
@@ -27154,7 +27154,7 @@
         </is>
       </c>
       <c r="I21" s="61" t="n">
-        <v>0.02815654</v>
+        <v>0.02807779</v>
       </c>
       <c r="J21" s="6" t="inlineStr">
         <is>
@@ -27192,7 +27192,7 @@
         </is>
       </c>
       <c r="I22" s="61" t="n">
-        <v>0.02750829</v>
+        <v>0.02741694</v>
       </c>
       <c r="J22" s="6" t="inlineStr">
         <is>
@@ -27230,7 +27230,7 @@
         </is>
       </c>
       <c r="I23" s="61" t="n">
-        <v>0.02033334</v>
+        <v>0.02036204</v>
       </c>
       <c r="J23" s="6" t="inlineStr">
         <is>
@@ -27268,7 +27268,7 @@
         </is>
       </c>
       <c r="I24" s="61" t="n">
-        <v>0.01963252</v>
+        <v>0.01979386</v>
       </c>
       <c r="J24" s="6" t="inlineStr">
         <is>
@@ -27306,7 +27306,7 @@
         </is>
       </c>
       <c r="I25" s="61" t="n">
-        <v>0.01901539</v>
+        <v>0.01908574</v>
       </c>
       <c r="J25" s="6" t="inlineStr">
         <is>
@@ -27340,25 +27340,25 @@
       </c>
       <c r="H26" s="6" t="inlineStr">
         <is>
-          <t>SLB</t>
+          <t>UPS</t>
         </is>
       </c>
       <c r="I26" s="61" t="n">
-        <v>0.01802343</v>
+        <v>0.01798331</v>
       </c>
       <c r="J26" s="6" t="inlineStr">
         <is>
-          <t>SLB</t>
+          <t>UNITED PARCEL SERVICE INC CLASS B</t>
         </is>
       </c>
       <c r="K26" s="6" t="inlineStr">
         <is>
-          <t>Energy</t>
+          <t>Industrials</t>
         </is>
       </c>
       <c r="L26" s="6" t="inlineStr">
         <is>
-          <t>SLB</t>
+          <t>UPS</t>
         </is>
       </c>
       <c r="M26" s="7">
@@ -27378,25 +27378,25 @@
       </c>
       <c r="H27" s="6" t="inlineStr">
         <is>
-          <t>UPS</t>
+          <t>SLB</t>
         </is>
       </c>
       <c r="I27" s="61" t="n">
-        <v>0.0179207</v>
+        <v>0.01794027</v>
       </c>
       <c r="J27" s="6" t="inlineStr">
         <is>
-          <t>UNITED PARCEL SERVICE INC CLASS B</t>
+          <t>SLB</t>
         </is>
       </c>
       <c r="K27" s="6" t="inlineStr">
         <is>
-          <t>Industrials</t>
+          <t>Energy</t>
         </is>
       </c>
       <c r="L27" s="6" t="inlineStr">
         <is>
-          <t>UPS</t>
+          <t>SLB</t>
         </is>
       </c>
       <c r="M27" s="7">
@@ -27420,7 +27420,7 @@
         </is>
       </c>
       <c r="I28" s="61" t="n">
-        <v>0.01718883</v>
+        <v>0.01714394</v>
       </c>
       <c r="J28" s="6" t="inlineStr">
         <is>
@@ -27454,23 +27454,27 @@
       </c>
       <c r="H29" s="6" t="inlineStr">
         <is>
-          <t>OKE</t>
+          <t>FAST</t>
         </is>
       </c>
       <c r="I29" s="61" t="n">
-        <v>0.01443041</v>
+        <v>0.01441625</v>
       </c>
       <c r="J29" s="6" t="inlineStr">
         <is>
-          <t>ONEOK</t>
+          <t>FASTENAL</t>
         </is>
       </c>
       <c r="K29" s="6" t="inlineStr">
         <is>
-          <t>Energy</t>
-        </is>
-      </c>
-      <c r="L29" s="6" t="inlineStr"/>
+          <t>Industrials</t>
+        </is>
+      </c>
+      <c r="L29" s="6" t="inlineStr">
+        <is>
+          <t>패스널</t>
+        </is>
+      </c>
       <c r="M29" s="7">
         <f>IF(H29="","",IFERROR(VLOOKUP(K29,$P$5:$Q$15,2,FALSE),"현금·선물"))</f>
         <v/>
@@ -27488,27 +27492,23 @@
       </c>
       <c r="H30" s="6" t="inlineStr">
         <is>
-          <t>FAST</t>
+          <t>OKE</t>
         </is>
       </c>
       <c r="I30" s="61" t="n">
-        <v>0.01436311</v>
+        <v>0.01434565</v>
       </c>
       <c r="J30" s="6" t="inlineStr">
         <is>
-          <t>FASTENAL</t>
+          <t>ONEOK</t>
         </is>
       </c>
       <c r="K30" s="6" t="inlineStr">
         <is>
-          <t>Industrials</t>
-        </is>
-      </c>
-      <c r="L30" s="6" t="inlineStr">
-        <is>
-          <t>패스널</t>
-        </is>
-      </c>
+          <t>Energy</t>
+        </is>
+      </c>
+      <c r="L30" s="6" t="inlineStr"/>
       <c r="M30" s="7">
         <f>IF(H30="","",IFERROR(VLOOKUP(K30,$P$5:$Q$15,2,FALSE),"현금·선물"))</f>
         <v/>
@@ -27530,7 +27530,7 @@
         </is>
       </c>
       <c r="I31" s="61" t="n">
-        <v>0.01369032</v>
+        <v>0.01379243</v>
       </c>
       <c r="J31" s="6" t="inlineStr">
         <is>
@@ -27555,7 +27555,7 @@
         </is>
       </c>
       <c r="I32" s="61" t="n">
-        <v>0.01194409</v>
+        <v>0.01174717</v>
       </c>
       <c r="J32" s="6" t="inlineStr">
         <is>
@@ -27585,7 +27585,7 @@
         </is>
       </c>
       <c r="I33" s="61" t="n">
-        <v>0.01120687</v>
+        <v>0.01127959</v>
       </c>
       <c r="J33" s="6" t="inlineStr">
         <is>
@@ -27610,7 +27610,7 @@
         </is>
       </c>
       <c r="I34" s="61" t="n">
-        <v>0.00976781</v>
+        <v>0.009554709999999999</v>
       </c>
       <c r="J34" s="6" t="inlineStr">
         <is>
@@ -27635,7 +27635,7 @@
         </is>
       </c>
       <c r="I35" s="61" t="n">
-        <v>0.00876676</v>
+        <v>0.008729799999999999</v>
       </c>
       <c r="J35" s="6" t="inlineStr">
         <is>
@@ -27660,7 +27660,7 @@
         </is>
       </c>
       <c r="I36" s="61" t="n">
-        <v>0.008613619999999999</v>
+        <v>0.00863236</v>
       </c>
       <c r="J36" s="6" t="inlineStr">
         <is>
@@ -27685,7 +27685,7 @@
         </is>
       </c>
       <c r="I37" s="61" t="n">
-        <v>0.00644801</v>
+        <v>0.00642043</v>
       </c>
       <c r="J37" s="6" t="inlineStr">
         <is>
@@ -27710,7 +27710,7 @@
         </is>
       </c>
       <c r="I38" s="61" t="n">
-        <v>0.006168590000000001</v>
+        <v>0.00623166</v>
       </c>
       <c r="J38" s="6" t="inlineStr">
         <is>
@@ -27731,20 +27731,20 @@
     <row r="39">
       <c r="H39" s="6" t="inlineStr">
         <is>
-          <t>HSY</t>
+          <t>DRI</t>
         </is>
       </c>
       <c r="I39" s="61" t="n">
-        <v>0.00613186</v>
+        <v>0.006045500000000001</v>
       </c>
       <c r="J39" s="6" t="inlineStr">
         <is>
-          <t>HERSHEY FOODS</t>
+          <t>DARDEN RESTAURANTS INC</t>
         </is>
       </c>
       <c r="K39" s="6" t="inlineStr">
         <is>
-          <t>Consumer Staples</t>
+          <t>Consumer Discretionary</t>
         </is>
       </c>
       <c r="L39" s="6" t="inlineStr"/>
@@ -27756,20 +27756,20 @@
     <row r="40">
       <c r="H40" s="6" t="inlineStr">
         <is>
-          <t>DRI</t>
+          <t>HSY</t>
         </is>
       </c>
       <c r="I40" s="61" t="n">
-        <v>0.00602634</v>
+        <v>0.00601652</v>
       </c>
       <c r="J40" s="6" t="inlineStr">
         <is>
-          <t>DARDEN RESTAURANTS INC</t>
+          <t>HERSHEY FOODS</t>
         </is>
       </c>
       <c r="K40" s="6" t="inlineStr">
         <is>
-          <t>Consumer Discretionary</t>
+          <t>Consumer Staples</t>
         </is>
       </c>
       <c r="L40" s="6" t="inlineStr"/>
@@ -27785,7 +27785,7 @@
         </is>
       </c>
       <c r="I41" s="61" t="n">
-        <v>0.00573727</v>
+        <v>0.005706050000000001</v>
       </c>
       <c r="J41" s="6" t="inlineStr">
         <is>
@@ -27810,7 +27810,7 @@
         </is>
       </c>
       <c r="I42" s="61" t="n">
-        <v>0.005284100000000001</v>
+        <v>0.00525792</v>
       </c>
       <c r="J42" s="6" t="inlineStr">
         <is>
@@ -27835,7 +27835,7 @@
         </is>
       </c>
       <c r="I43" s="61" t="n">
-        <v>0.00520119</v>
+        <v>0.005126840000000001</v>
       </c>
       <c r="J43" s="6" t="inlineStr">
         <is>
@@ -27860,7 +27860,7 @@
         </is>
       </c>
       <c r="I44" s="61" t="n">
-        <v>0.00489968</v>
+        <v>0.00491802</v>
       </c>
       <c r="J44" s="6" t="inlineStr">
         <is>
@@ -27885,7 +27885,7 @@
         </is>
       </c>
       <c r="I45" s="61" t="n">
-        <v>0.00475214</v>
+        <v>0.00473661</v>
       </c>
       <c r="J45" s="6" t="inlineStr">
         <is>
@@ -27910,7 +27910,7 @@
         </is>
       </c>
       <c r="I46" s="61" t="n">
-        <v>0.0046609</v>
+        <v>0.00464773</v>
       </c>
       <c r="J46" s="6" t="inlineStr">
         <is>
@@ -27935,7 +27935,7 @@
         </is>
       </c>
       <c r="I47" s="61" t="n">
-        <v>0.00449997</v>
+        <v>0.00444347</v>
       </c>
       <c r="J47" s="6" t="inlineStr">
         <is>
@@ -27956,20 +27956,20 @@
     <row r="48">
       <c r="H48" s="6" t="inlineStr">
         <is>
-          <t>GIS</t>
+          <t>APA</t>
         </is>
       </c>
       <c r="I48" s="61" t="n">
-        <v>0.0043463</v>
+        <v>0.00429283</v>
       </c>
       <c r="J48" s="6" t="inlineStr">
         <is>
-          <t>GENERAL MILLS INC</t>
+          <t>APA</t>
         </is>
       </c>
       <c r="K48" s="6" t="inlineStr">
         <is>
-          <t>Consumer Staples</t>
+          <t>Energy</t>
         </is>
       </c>
       <c r="L48" s="6" t="inlineStr"/>
@@ -27981,20 +27981,20 @@
     <row r="49">
       <c r="H49" s="6" t="inlineStr">
         <is>
-          <t>EWBC</t>
+          <t>GIS</t>
         </is>
       </c>
       <c r="I49" s="61" t="n">
-        <v>0.00426545</v>
+        <v>0.00428863</v>
       </c>
       <c r="J49" s="6" t="inlineStr">
         <is>
-          <t>EAST WEST BANCORP</t>
+          <t>GENERAL MILLS INC</t>
         </is>
       </c>
       <c r="K49" s="6" t="inlineStr">
         <is>
-          <t>Financials</t>
+          <t>Consumer Staples</t>
         </is>
       </c>
       <c r="L49" s="6" t="inlineStr"/>
@@ -28006,20 +28006,20 @@
     <row r="50">
       <c r="H50" s="6" t="inlineStr">
         <is>
-          <t>APA</t>
+          <t>EWBC</t>
         </is>
       </c>
       <c r="I50" s="61" t="n">
-        <v>0.00422458</v>
+        <v>0.00423464</v>
       </c>
       <c r="J50" s="6" t="inlineStr">
         <is>
-          <t>APA</t>
+          <t>EAST WEST BANCORP</t>
         </is>
       </c>
       <c r="K50" s="6" t="inlineStr">
         <is>
-          <t>Energy</t>
+          <t>Financials</t>
         </is>
       </c>
       <c r="L50" s="6" t="inlineStr"/>
@@ -28035,7 +28035,7 @@
         </is>
       </c>
       <c r="I51" s="61" t="n">
-        <v>0.00258379</v>
+        <v>0.0025765</v>
       </c>
       <c r="J51" s="6" t="inlineStr">
         <is>
@@ -28060,7 +28060,7 @@
         </is>
       </c>
       <c r="I52" s="61" t="n">
-        <v>0.00251532</v>
+        <v>0.0025068</v>
       </c>
       <c r="J52" s="6" t="inlineStr">
         <is>
@@ -28085,7 +28085,7 @@
         </is>
       </c>
       <c r="I53" s="61" t="n">
-        <v>0.0025014</v>
+        <v>0.00249122</v>
       </c>
       <c r="J53" s="6" t="inlineStr">
         <is>
@@ -28110,7 +28110,7 @@
         </is>
       </c>
       <c r="I54" s="61" t="n">
-        <v>0.00219017</v>
+        <v>0.00219234</v>
       </c>
       <c r="J54" s="6" t="inlineStr">
         <is>
@@ -28135,7 +28135,7 @@
         </is>
       </c>
       <c r="I55" s="61" t="n">
-        <v>0.00216031</v>
+        <v>0.00214697</v>
       </c>
       <c r="J55" s="6" t="inlineStr">
         <is>
@@ -28160,7 +28160,7 @@
         </is>
       </c>
       <c r="I56" s="61" t="n">
-        <v>0.00197196</v>
+        <v>0.00197159</v>
       </c>
       <c r="J56" s="6" t="inlineStr">
         <is>
@@ -28185,7 +28185,7 @@
         </is>
       </c>
       <c r="I57" s="61" t="n">
-        <v>0.00189573</v>
+        <v>0.00191095</v>
       </c>
       <c r="J57" s="6" t="inlineStr">
         <is>
@@ -28206,20 +28206,20 @@
     <row r="58">
       <c r="H58" s="6" t="inlineStr">
         <is>
-          <t>M</t>
+          <t>ERIE</t>
         </is>
       </c>
       <c r="I58" s="61" t="n">
-        <v>0.00154731</v>
+        <v>0.00154167</v>
       </c>
       <c r="J58" s="6" t="inlineStr">
         <is>
-          <t>MACYS INC</t>
+          <t>ERIE INDEMNITY CLASS A</t>
         </is>
       </c>
       <c r="K58" s="6" t="inlineStr">
         <is>
-          <t>Consumer Discretionary</t>
+          <t>Financials</t>
         </is>
       </c>
       <c r="L58" s="6" t="inlineStr"/>
@@ -28231,20 +28231,20 @@
     <row r="59">
       <c r="H59" s="6" t="inlineStr">
         <is>
-          <t>ERIE</t>
+          <t>M</t>
         </is>
       </c>
       <c r="I59" s="61" t="n">
-        <v>0.00154533</v>
+        <v>0.00152714</v>
       </c>
       <c r="J59" s="6" t="inlineStr">
         <is>
-          <t>ERIE INDEMNITY CLASS A</t>
+          <t>MACYS INC</t>
         </is>
       </c>
       <c r="K59" s="6" t="inlineStr">
         <is>
-          <t>Financials</t>
+          <t>Consumer Discretionary</t>
         </is>
       </c>
       <c r="L59" s="6" t="inlineStr"/>
@@ -28260,7 +28260,7 @@
         </is>
       </c>
       <c r="I60" s="61" t="n">
-        <v>0.0014655</v>
+        <v>0.00144688</v>
       </c>
       <c r="J60" s="6" t="inlineStr">
         <is>
@@ -28285,7 +28285,7 @@
         </is>
       </c>
       <c r="I61" s="61" t="n">
-        <v>0.00138152</v>
+        <v>0.00141319</v>
       </c>
       <c r="J61" s="6" t="inlineStr">
         <is>
@@ -28310,7 +28310,7 @@
         </is>
       </c>
       <c r="I62" s="61" t="n">
-        <v>0.00132055</v>
+        <v>0.00132502</v>
       </c>
       <c r="J62" s="6" t="inlineStr">
         <is>
@@ -28335,7 +28335,7 @@
         </is>
       </c>
       <c r="I63" s="61" t="n">
-        <v>0.0011709</v>
+        <v>0.00118386</v>
       </c>
       <c r="J63" s="6" t="inlineStr">
         <is>
@@ -28360,7 +28360,7 @@
         </is>
       </c>
       <c r="I64" s="61" t="n">
-        <v>0.00114904</v>
+        <v>0.00113003</v>
       </c>
       <c r="J64" s="6" t="inlineStr">
         <is>
@@ -28381,15 +28381,15 @@
     <row r="65">
       <c r="H65" s="6" t="inlineStr">
         <is>
-          <t>MC</t>
+          <t>FHI</t>
         </is>
       </c>
       <c r="I65" s="61" t="n">
-        <v>0.00098869</v>
+        <v>0.00096994</v>
       </c>
       <c r="J65" s="6" t="inlineStr">
         <is>
-          <t>MOELIS CLASS A</t>
+          <t>FEDERATED HERMES INC CLASS B</t>
         </is>
       </c>
       <c r="K65" s="6" t="inlineStr">
@@ -28406,15 +28406,15 @@
     <row r="66">
       <c r="H66" s="6" t="inlineStr">
         <is>
-          <t>FHI</t>
+          <t>MC</t>
         </is>
       </c>
       <c r="I66" s="61" t="n">
-        <v>0.00097828</v>
+        <v>0.00096542</v>
       </c>
       <c r="J66" s="6" t="inlineStr">
         <is>
-          <t>FEDERATED HERMES INC CLASS B</t>
+          <t>MOELIS CLASS A</t>
         </is>
       </c>
       <c r="K66" s="6" t="inlineStr">
@@ -28435,7 +28435,7 @@
         </is>
       </c>
       <c r="I67" s="61" t="n">
-        <v>0.0009256000000000001</v>
+        <v>0.0009271500000000001</v>
       </c>
       <c r="J67" s="6" t="inlineStr">
         <is>
@@ -28460,7 +28460,7 @@
         </is>
       </c>
       <c r="I68" s="61" t="n">
-        <v>0.0009221300000000001</v>
+        <v>0.00091108</v>
       </c>
       <c r="J68" s="6" t="inlineStr">
         <is>
@@ -28485,7 +28485,7 @@
         </is>
       </c>
       <c r="I69" s="61" t="n">
-        <v>0.00089464</v>
+        <v>0.00089713</v>
       </c>
       <c r="J69" s="6" t="inlineStr">
         <is>
@@ -28510,7 +28510,7 @@
         </is>
       </c>
       <c r="I70" s="61" t="n">
-        <v>0.0008871700000000001</v>
+        <v>0.00087914</v>
       </c>
       <c r="J70" s="6" t="inlineStr">
         <is>
@@ -28535,7 +28535,7 @@
         </is>
       </c>
       <c r="I71" s="61" t="n">
-        <v>0.00081987</v>
+        <v>0.0008120299999999999</v>
       </c>
       <c r="J71" s="6" t="inlineStr">
         <is>
@@ -28560,7 +28560,7 @@
         </is>
       </c>
       <c r="I72" s="61" t="n">
-        <v>0.0005605299999999999</v>
+        <v>0.00055785</v>
       </c>
       <c r="J72" s="6" t="inlineStr">
         <is>
@@ -28585,7 +28585,7 @@
         </is>
       </c>
       <c r="I73" s="61" t="n">
-        <v>0.00055993</v>
+        <v>0.00055747</v>
       </c>
       <c r="J73" s="6" t="inlineStr">
         <is>
@@ -28610,7 +28610,7 @@
         </is>
       </c>
       <c r="I74" s="61" t="n">
-        <v>0.00054628</v>
+        <v>0.0005436</v>
       </c>
       <c r="J74" s="6" t="inlineStr">
         <is>
@@ -28635,7 +28635,7 @@
         </is>
       </c>
       <c r="I75" s="61" t="n">
-        <v>0.00051849</v>
+        <v>0.0005161500000000001</v>
       </c>
       <c r="J75" s="6" t="inlineStr">
         <is>
@@ -28660,7 +28660,7 @@
         </is>
       </c>
       <c r="I76" s="61" t="n">
-        <v>0.00049944</v>
+        <v>0.00050315</v>
       </c>
       <c r="J76" s="6" t="inlineStr">
         <is>
@@ -28685,7 +28685,7 @@
         </is>
       </c>
       <c r="I77" s="61" t="n">
-        <v>0.00048849</v>
+        <v>0.00048714</v>
       </c>
       <c r="J77" s="6" t="inlineStr">
         <is>
@@ -28710,7 +28710,7 @@
         </is>
       </c>
       <c r="I78" s="61" t="n">
-        <v>0.00048348</v>
+        <v>0.00047667</v>
       </c>
       <c r="J78" s="6" t="inlineStr">
         <is>
@@ -28735,7 +28735,7 @@
         </is>
       </c>
       <c r="I79" s="61" t="n">
-        <v>0.00047337</v>
+        <v>0.00047435</v>
       </c>
       <c r="J79" s="6" t="inlineStr">
         <is>
@@ -28756,15 +28756,15 @@
     <row r="80">
       <c r="H80" s="6" t="inlineStr">
         <is>
-          <t>AGM</t>
+          <t>GABC</t>
         </is>
       </c>
       <c r="I80" s="61" t="n">
-        <v>0.00046806</v>
+        <v>0.00046024</v>
       </c>
       <c r="J80" s="6" t="inlineStr">
         <is>
-          <t>FEDERAL AGRICULTURAL MORTGAGE NON</t>
+          <t>GERMAN AMERICAN BANCORP INC</t>
         </is>
       </c>
       <c r="K80" s="6" t="inlineStr">
@@ -28781,15 +28781,15 @@
     <row r="81">
       <c r="H81" s="6" t="inlineStr">
         <is>
-          <t>GABC</t>
+          <t>AGM</t>
         </is>
       </c>
       <c r="I81" s="61" t="n">
-        <v>0.00046152</v>
+        <v>0.00045899</v>
       </c>
       <c r="J81" s="6" t="inlineStr">
         <is>
-          <t>GERMAN AMERICAN BANCORP INC</t>
+          <t>FEDERAL AGRICULTURAL MORTGAGE NON</t>
         </is>
       </c>
       <c r="K81" s="6" t="inlineStr">
@@ -28810,7 +28810,7 @@
         </is>
       </c>
       <c r="I82" s="61" t="n">
-        <v>0.00045132</v>
+        <v>0.00043236</v>
       </c>
       <c r="J82" s="6" t="inlineStr">
         <is>
@@ -28835,7 +28835,7 @@
         </is>
       </c>
       <c r="I83" s="61" t="n">
-        <v>0.00042364</v>
+        <v>0.00042214</v>
       </c>
       <c r="J83" s="6" t="inlineStr">
         <is>
@@ -28860,7 +28860,7 @@
         </is>
       </c>
       <c r="I84" s="61" t="n">
-        <v>0.00041385</v>
+        <v>0.00041077</v>
       </c>
       <c r="J84" s="6" t="inlineStr">
         <is>
@@ -28885,7 +28885,7 @@
         </is>
       </c>
       <c r="I85" s="61" t="n">
-        <v>0.00039244</v>
+        <v>0.00040583</v>
       </c>
       <c r="J85" s="6" t="inlineStr">
         <is>
@@ -28906,7 +28906,7 @@
         </is>
       </c>
       <c r="I86" s="61" t="n">
-        <v>0.00037642</v>
+        <v>0.00037481</v>
       </c>
       <c r="J86" s="6" t="inlineStr">
         <is>
@@ -28927,20 +28927,20 @@
     <row r="87">
       <c r="H87" s="6" t="inlineStr">
         <is>
-          <t>LKFN</t>
+          <t>BKE</t>
         </is>
       </c>
       <c r="I87" s="61" t="n">
-        <v>0.00035466</v>
+        <v>0.00035561</v>
       </c>
       <c r="J87" s="6" t="inlineStr">
         <is>
-          <t>LAKELAND FINANCIAL CORP</t>
+          <t>BUCKLE</t>
         </is>
       </c>
       <c r="K87" s="6" t="inlineStr">
         <is>
-          <t>Financials</t>
+          <t>Consumer Discretionary</t>
         </is>
       </c>
       <c r="L87" s="6" t="inlineStr"/>
@@ -28952,20 +28952,20 @@
     <row r="88">
       <c r="H88" s="6" t="inlineStr">
         <is>
-          <t>BKE</t>
+          <t>LKFN</t>
         </is>
       </c>
       <c r="I88" s="61" t="n">
-        <v>0.00035092</v>
+        <v>0.00035326</v>
       </c>
       <c r="J88" s="6" t="inlineStr">
         <is>
-          <t>BUCKLE</t>
+          <t>LAKELAND FINANCIAL CORP</t>
         </is>
       </c>
       <c r="K88" s="6" t="inlineStr">
         <is>
-          <t>Consumer Discretionary</t>
+          <t>Financials</t>
         </is>
       </c>
       <c r="L88" s="6" t="inlineStr"/>
@@ -28981,7 +28981,7 @@
         </is>
       </c>
       <c r="I89" s="61" t="n">
-        <v>0.00031822</v>
+        <v>0.0003126</v>
       </c>
       <c r="J89" s="6" t="inlineStr">
         <is>
@@ -29006,7 +29006,7 @@
         </is>
       </c>
       <c r="I90" s="61" t="n">
-        <v>0.00027958</v>
+        <v>0.00027839</v>
       </c>
       <c r="J90" s="6" t="inlineStr">
         <is>
@@ -29031,7 +29031,7 @@
         </is>
       </c>
       <c r="I91" s="61" t="n">
-        <v>0.00026418</v>
+        <v>0.00026436</v>
       </c>
       <c r="J91" s="6" t="inlineStr">
         <is>
@@ -29056,7 +29056,7 @@
         </is>
       </c>
       <c r="I92" s="61" t="n">
-        <v>0.00025525</v>
+        <v>0.00025582</v>
       </c>
       <c r="J92" s="6" t="inlineStr">
         <is>
@@ -29081,7 +29081,7 @@
         </is>
       </c>
       <c r="I93" s="61" t="n">
-        <v>0.0002299</v>
+        <v>0.00022948</v>
       </c>
       <c r="J93" s="6" t="inlineStr">
         <is>
@@ -29106,7 +29106,7 @@
         </is>
       </c>
       <c r="I94" s="61" t="n">
-        <v>0.00022529</v>
+        <v>0.0002251</v>
       </c>
       <c r="J94" s="6" t="inlineStr">
         <is>
@@ -29131,7 +29131,7 @@
         </is>
       </c>
       <c r="I95" s="61" t="n">
-        <v>0.00020373</v>
+        <v>0.00020276</v>
       </c>
       <c r="J95" s="6" t="inlineStr">
         <is>
@@ -29156,7 +29156,7 @@
         </is>
       </c>
       <c r="I96" s="61" t="n">
-        <v>0.00019441</v>
+        <v>0.00019517</v>
       </c>
       <c r="J96" s="6" t="inlineStr">
         <is>
@@ -29181,7 +29181,7 @@
         </is>
       </c>
       <c r="I97" s="61" t="n">
-        <v>0.0001943</v>
+        <v>0.00019455</v>
       </c>
       <c r="J97" s="6" t="inlineStr">
         <is>
@@ -29206,7 +29206,7 @@
         </is>
       </c>
       <c r="I98" s="61" t="n">
-        <v>0.00018458</v>
+        <v>0.00017741</v>
       </c>
       <c r="J98" s="6" t="inlineStr">
         <is>
@@ -29231,7 +29231,7 @@
         </is>
       </c>
       <c r="I99" s="61" t="n">
-        <v>0.00016498</v>
+        <v>0.00016406</v>
       </c>
       <c r="J99" s="6" t="inlineStr">
         <is>
@@ -29256,7 +29256,7 @@
         </is>
       </c>
       <c r="I100" s="61" t="n">
-        <v>0.00013126</v>
+        <v>0.00013139</v>
       </c>
       <c r="J100" s="6" t="inlineStr">
         <is>
@@ -29277,18 +29277,22 @@
     <row r="101">
       <c r="H101" s="6" t="inlineStr">
         <is>
-          <t>USD</t>
+          <t>AMSF</t>
         </is>
       </c>
       <c r="I101" s="61" t="n">
-        <v>0.00011859</v>
+        <v>0.00011576</v>
       </c>
       <c r="J101" s="6" t="inlineStr">
         <is>
-          <t>US DOLLAR</t>
-        </is>
-      </c>
-      <c r="K101" s="6" t="inlineStr"/>
+          <t>AMERISAFE INC</t>
+        </is>
+      </c>
+      <c r="K101" s="6" t="inlineStr">
+        <is>
+          <t>Financials</t>
+        </is>
+      </c>
       <c r="L101" s="6" t="inlineStr"/>
       <c r="M101" s="7">
         <f>IF(H101="","",IFERROR(VLOOKUP(K101,$P$5:$Q$15,2,FALSE),"현금·선물"))</f>
@@ -29298,22 +29302,18 @@
     <row r="102">
       <c r="H102" s="6" t="inlineStr">
         <is>
-          <t>AMSF</t>
+          <t>USD</t>
         </is>
       </c>
       <c r="I102" s="61" t="n">
-        <v>0.00011494</v>
+        <v>0.00011066</v>
       </c>
       <c r="J102" s="6" t="inlineStr">
         <is>
-          <t>AMERISAFE INC</t>
-        </is>
-      </c>
-      <c r="K102" s="6" t="inlineStr">
-        <is>
-          <t>Financials</t>
-        </is>
-      </c>
+          <t>US DOLLAR</t>
+        </is>
+      </c>
+      <c r="K102" s="6" t="inlineStr"/>
       <c r="L102" s="6" t="inlineStr"/>
       <c r="M102" s="7">
         <f>IF(H102="","",IFERROR(VLOOKUP(K102,$P$5:$Q$15,2,FALSE),"현금·선물"))</f>
@@ -29327,7 +29327,7 @@
         </is>
       </c>
       <c r="I103" s="61" t="n">
-        <v>9.831e-05</v>
+        <v>9.738999999999999e-05</v>
       </c>
       <c r="J103" s="6" t="inlineStr">
         <is>
@@ -29352,7 +29352,7 @@
         </is>
       </c>
       <c r="I104" s="61" t="n">
-        <v>9.007e-05</v>
+        <v>9.112000000000001e-05</v>
       </c>
       <c r="J104" s="6" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
데이터 갱신: holdings,prices (2026-10-21)
</commit_message>
<xml_diff>
--- a/downloads/schd_dividend_tracker.xlsx
+++ b/downloads/schd_dividend_tracker.xlsx
@@ -1724,7 +1724,7 @@
     <row r="3">
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>최종 갱신: 2026-10-20 · 반영 범위: 2012년 1분기 ~ 2026년 3분기 (배당락 2026-09-23) · GitHub Actions 자동 생성</t>
+          <t>최종 갱신: 2026-10-21 · 반영 범위: 2012년 1분기 ~ 2026년 3분기 (배당락 2026-09-23) · GitHub Actions 자동 생성</t>
         </is>
       </c>
     </row>
@@ -5818,7 +5818,7 @@
       </c>
       <c r="H1" s="2" t="inlineStr">
         <is>
-          <t>출처: Yahoo Finance (종가: 주식분할 반영·배당 미조정 / adj: 배당 재투자 반영 수정주가) · 기준일 2026-10-14 · 3:1 분할(2024-10-11) 반영 가격</t>
+          <t>출처: Yahoo Finance (종가: 주식분할 반영·배당 미조정 / adj: 배당 재투자 반영 수정주가) · 기준일 2026-10-20 · 3:1 분할(2024-10-11) 반영 가격</t>
         </is>
       </c>
     </row>
@@ -6243,7 +6243,7 @@
         <v>10.9</v>
       </c>
       <c r="D22" s="77" t="n">
-        <v>7.1038</v>
+        <v>7.1037</v>
       </c>
       <c r="E22" s="58">
         <f>C22/C10-1</f>
@@ -7491,7 +7491,7 @@
         <v>16.1633</v>
       </c>
       <c r="D74" s="77" t="n">
-        <v>11.9069</v>
+        <v>11.9068</v>
       </c>
       <c r="E74" s="58">
         <f>C74/C62-1</f>
@@ -7995,7 +7995,7 @@
         <v>17.9833</v>
       </c>
       <c r="D95" s="77" t="n">
-        <v>13.9254</v>
+        <v>13.9255</v>
       </c>
       <c r="E95" s="58">
         <f>C95/C83-1</f>
@@ -9555,7 +9555,7 @@
         <v>27.32</v>
       </c>
       <c r="D160" s="77" t="n">
-        <v>25.6579</v>
+        <v>25.658</v>
       </c>
       <c r="E160" s="58">
         <f>C160/C148-1</f>
@@ -10077,13 +10077,13 @@
         </is>
       </c>
       <c r="B182" s="56" t="n">
-        <v>46309</v>
+        <v>46315</v>
       </c>
       <c r="C182" s="76" t="n">
-        <v>33.71</v>
+        <v>34.69</v>
       </c>
       <c r="D182" s="77" t="n">
-        <v>33.71</v>
+        <v>34.69</v>
       </c>
       <c r="E182" s="58">
         <f>C182/C170-1</f>
@@ -26257,11 +26257,11 @@
         </is>
       </c>
       <c r="B2" s="49" t="n">
-        <v>46314</v>
+        <v>46315</v>
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>← 이 날 종가로 계산한 비중. 그날 공식 파일을 못 받아 Schwab 공식 보유종목 CSV(2026-10-16)의 보유 주식 수 × 종가로 계산했습니다.</t>
+          <t>← 이 날 종가로 계산한 비중. 그날 공식 파일을 못 받아 Schwab 공식 보유종목 CSV(2026-10-19)의 보유 주식 수 × 종가로 계산했습니다.</t>
         </is>
       </c>
     </row>
@@ -26358,11 +26358,11 @@
         </is>
       </c>
       <c r="I5" s="61" t="n">
-        <v>0.04404334000000001</v>
+        <v>0.0437362</v>
       </c>
       <c r="J5" s="6" t="inlineStr">
         <is>
-          <t>TEXAS INSTRUMENT INC</t>
+          <t>TEXAS INSTRUMENT</t>
         </is>
       </c>
       <c r="K5" s="6" t="inlineStr">
@@ -26416,7 +26416,7 @@
         </is>
       </c>
       <c r="I6" s="61" t="n">
-        <v>0.04340455000000001</v>
+        <v>0.04329193</v>
       </c>
       <c r="J6" s="6" t="inlineStr">
         <is>
@@ -26474,7 +26474,7 @@
         </is>
       </c>
       <c r="I7" s="61" t="n">
-        <v>0.04305399000000001</v>
+        <v>0.04275667</v>
       </c>
       <c r="J7" s="6" t="inlineStr">
         <is>
@@ -26528,25 +26528,25 @@
       </c>
       <c r="H8" s="6" t="inlineStr">
         <is>
-          <t>KO</t>
+          <t>COP</t>
         </is>
       </c>
       <c r="I8" s="61" t="n">
-        <v>0.04302386</v>
+        <v>0.04262202</v>
       </c>
       <c r="J8" s="6" t="inlineStr">
         <is>
-          <t>COCA-COLA</t>
+          <t>CONOCOPHILLIPS</t>
         </is>
       </c>
       <c r="K8" s="6" t="inlineStr">
         <is>
-          <t>Consumer Staples</t>
+          <t>Energy</t>
         </is>
       </c>
       <c r="L8" s="6" t="inlineStr">
         <is>
-          <t>코카콜라</t>
+          <t>코노코필립스</t>
         </is>
       </c>
       <c r="M8" s="7">
@@ -26586,25 +26586,25 @@
       </c>
       <c r="H9" s="6" t="inlineStr">
         <is>
-          <t>COP</t>
+          <t>KO</t>
         </is>
       </c>
       <c r="I9" s="61" t="n">
-        <v>0.04296461</v>
+        <v>0.04250498</v>
       </c>
       <c r="J9" s="6" t="inlineStr">
         <is>
-          <t>CONOCOPHILLIPS</t>
+          <t>COCA-COLA</t>
         </is>
       </c>
       <c r="K9" s="6" t="inlineStr">
         <is>
-          <t>Energy</t>
+          <t>Consumer Staples</t>
         </is>
       </c>
       <c r="L9" s="6" t="inlineStr">
         <is>
-          <t>코노코필립스</t>
+          <t>코카콜라</t>
         </is>
       </c>
       <c r="M9" s="7">
@@ -26644,25 +26644,25 @@
       </c>
       <c r="H10" s="6" t="inlineStr">
         <is>
-          <t>QCOM</t>
+          <t>UNH</t>
         </is>
       </c>
       <c r="I10" s="61" t="n">
-        <v>0.0414919</v>
+        <v>0.04208503</v>
       </c>
       <c r="J10" s="6" t="inlineStr">
         <is>
-          <t>QUALCOMM</t>
+          <t>UNITEDHEALTH GROUP</t>
         </is>
       </c>
       <c r="K10" s="6" t="inlineStr">
         <is>
-          <t>Information Technology</t>
+          <t>Health Care</t>
         </is>
       </c>
       <c r="L10" s="6" t="inlineStr">
         <is>
-          <t>퀄컴</t>
+          <t>유나이티드헬스</t>
         </is>
       </c>
       <c r="M10" s="7">
@@ -26702,25 +26702,25 @@
       </c>
       <c r="H11" s="6" t="inlineStr">
         <is>
-          <t>UNH</t>
+          <t>QCOM</t>
         </is>
       </c>
       <c r="I11" s="61" t="n">
-        <v>0.04137204</v>
+        <v>0.04147538</v>
       </c>
       <c r="J11" s="6" t="inlineStr">
         <is>
-          <t>UNITEDHEALTH GROUP</t>
+          <t>QUALCOMM</t>
         </is>
       </c>
       <c r="K11" s="6" t="inlineStr">
         <is>
-          <t>Health Care</t>
+          <t>Information Technology</t>
         </is>
       </c>
       <c r="L11" s="6" t="inlineStr">
         <is>
-          <t>유나이티드헬스</t>
+          <t>퀄컴</t>
         </is>
       </c>
       <c r="M11" s="7">
@@ -26760,25 +26760,25 @@
       </c>
       <c r="H12" s="6" t="inlineStr">
         <is>
-          <t>HD</t>
+          <t>AMGN</t>
         </is>
       </c>
       <c r="I12" s="61" t="n">
-        <v>0.03953678</v>
+        <v>0.03976414</v>
       </c>
       <c r="J12" s="6" t="inlineStr">
         <is>
-          <t>HOME DEPOT</t>
+          <t>AMGEN INC</t>
         </is>
       </c>
       <c r="K12" s="6" t="inlineStr">
         <is>
-          <t>Consumer Discretionary</t>
+          <t>Health Care</t>
         </is>
       </c>
       <c r="L12" s="6" t="inlineStr">
         <is>
-          <t>홈디포</t>
+          <t>암젠</t>
         </is>
       </c>
       <c r="M12" s="7">
@@ -26818,25 +26818,25 @@
       </c>
       <c r="H13" s="6" t="inlineStr">
         <is>
-          <t>AMGN</t>
+          <t>HD</t>
         </is>
       </c>
       <c r="I13" s="61" t="n">
-        <v>0.03899518</v>
+        <v>0.03968929</v>
       </c>
       <c r="J13" s="6" t="inlineStr">
         <is>
-          <t>AMGEN INC</t>
+          <t>HOME DEPOT</t>
         </is>
       </c>
       <c r="K13" s="6" t="inlineStr">
         <is>
-          <t>Health Care</t>
+          <t>Consumer Discretionary</t>
         </is>
       </c>
       <c r="L13" s="6" t="inlineStr">
         <is>
-          <t>암젠</t>
+          <t>홈디포</t>
         </is>
       </c>
       <c r="M13" s="7">
@@ -26876,25 +26876,25 @@
       </c>
       <c r="H14" s="6" t="inlineStr">
         <is>
-          <t>PEP</t>
+          <t>MRK</t>
         </is>
       </c>
       <c r="I14" s="61" t="n">
-        <v>0.03862823</v>
+        <v>0.03923437</v>
       </c>
       <c r="J14" s="6" t="inlineStr">
         <is>
-          <t>PEPSICO</t>
+          <t>MERCK &amp; CO INC</t>
         </is>
       </c>
       <c r="K14" s="6" t="inlineStr">
         <is>
-          <t>Consumer Staples</t>
+          <t>Health Care</t>
         </is>
       </c>
       <c r="L14" s="6" t="inlineStr">
         <is>
-          <t>펩시코</t>
+          <t>머크</t>
         </is>
       </c>
       <c r="M14" s="7">
@@ -26924,25 +26924,25 @@
       </c>
       <c r="H15" s="6" t="inlineStr">
         <is>
-          <t>MRK</t>
+          <t>PEP</t>
         </is>
       </c>
       <c r="I15" s="61" t="n">
-        <v>0.0384916</v>
+        <v>0.03826222</v>
       </c>
       <c r="J15" s="6" t="inlineStr">
         <is>
-          <t>MERCK &amp; CO INC</t>
+          <t>PEPSICO</t>
         </is>
       </c>
       <c r="K15" s="6" t="inlineStr">
         <is>
-          <t>Health Care</t>
+          <t>Consumer Staples</t>
         </is>
       </c>
       <c r="L15" s="6" t="inlineStr">
         <is>
-          <t>머크</t>
+          <t>펩시코</t>
         </is>
       </c>
       <c r="M15" s="7">
@@ -26976,7 +26976,7 @@
         </is>
       </c>
       <c r="I16" s="61" t="n">
-        <v>0.03828023</v>
+        <v>0.03720558</v>
       </c>
       <c r="J16" s="6" t="inlineStr">
         <is>
@@ -27014,7 +27014,7 @@
         </is>
       </c>
       <c r="I17" s="61" t="n">
-        <v>0.03572645</v>
+        <v>0.03558074</v>
       </c>
       <c r="J17" s="6" t="inlineStr">
         <is>
@@ -27052,7 +27052,7 @@
         </is>
       </c>
       <c r="I18" s="61" t="n">
-        <v>0.03570178</v>
+        <v>0.03557055</v>
       </c>
       <c r="J18" s="6" t="inlineStr">
         <is>
@@ -27077,25 +27077,25 @@
     <row r="19">
       <c r="H19" s="6" t="inlineStr">
         <is>
-          <t>MO</t>
+          <t>BMY</t>
         </is>
       </c>
       <c r="I19" s="61" t="n">
-        <v>0.03046279</v>
+        <v>0.03062798</v>
       </c>
       <c r="J19" s="6" t="inlineStr">
         <is>
-          <t>ALTRIA GROUP INC</t>
+          <t>BRISTOL MYERS SQUIBB</t>
         </is>
       </c>
       <c r="K19" s="6" t="inlineStr">
         <is>
-          <t>Consumer Staples</t>
+          <t>Health Care</t>
         </is>
       </c>
       <c r="L19" s="6" t="inlineStr">
         <is>
-          <t>알트리아</t>
+          <t>브리스톨마이어스스퀴브</t>
         </is>
       </c>
       <c r="M19" s="7">
@@ -27111,25 +27111,25 @@
       </c>
       <c r="H20" s="6" t="inlineStr">
         <is>
-          <t>BMY</t>
+          <t>MO</t>
         </is>
       </c>
       <c r="I20" s="61" t="n">
-        <v>0.02959153</v>
+        <v>0.03029613</v>
       </c>
       <c r="J20" s="6" t="inlineStr">
         <is>
-          <t>BRISTOL MYERS SQUIBB</t>
+          <t>ALTRIA GROUP INC</t>
         </is>
       </c>
       <c r="K20" s="6" t="inlineStr">
         <is>
-          <t>Health Care</t>
+          <t>Consumer Staples</t>
         </is>
       </c>
       <c r="L20" s="6" t="inlineStr">
         <is>
-          <t>브리스톨마이어스스퀴브</t>
+          <t>알트리아</t>
         </is>
       </c>
       <c r="M20" s="7">
@@ -27154,7 +27154,7 @@
         </is>
       </c>
       <c r="I21" s="61" t="n">
-        <v>0.02807779</v>
+        <v>0.02827079</v>
       </c>
       <c r="J21" s="6" t="inlineStr">
         <is>
@@ -27192,7 +27192,7 @@
         </is>
       </c>
       <c r="I22" s="61" t="n">
-        <v>0.02741694</v>
+        <v>0.02708957</v>
       </c>
       <c r="J22" s="6" t="inlineStr">
         <is>
@@ -27230,7 +27230,7 @@
         </is>
       </c>
       <c r="I23" s="61" t="n">
-        <v>0.02036204</v>
+        <v>0.02013451</v>
       </c>
       <c r="J23" s="6" t="inlineStr">
         <is>
@@ -27268,7 +27268,7 @@
         </is>
       </c>
       <c r="I24" s="61" t="n">
-        <v>0.01979386</v>
+        <v>0.02013349</v>
       </c>
       <c r="J24" s="6" t="inlineStr">
         <is>
@@ -27306,7 +27306,7 @@
         </is>
       </c>
       <c r="I25" s="61" t="n">
-        <v>0.01908574</v>
+        <v>0.01923721</v>
       </c>
       <c r="J25" s="6" t="inlineStr">
         <is>
@@ -27340,25 +27340,25 @@
       </c>
       <c r="H26" s="6" t="inlineStr">
         <is>
-          <t>UPS</t>
+          <t>SLB</t>
         </is>
       </c>
       <c r="I26" s="61" t="n">
-        <v>0.01798331</v>
+        <v>0.01803174</v>
       </c>
       <c r="J26" s="6" t="inlineStr">
         <is>
-          <t>UNITED PARCEL SERVICE INC CLASS B</t>
+          <t>SLB</t>
         </is>
       </c>
       <c r="K26" s="6" t="inlineStr">
         <is>
-          <t>Industrials</t>
+          <t>Energy</t>
         </is>
       </c>
       <c r="L26" s="6" t="inlineStr">
         <is>
-          <t>UPS</t>
+          <t>SLB</t>
         </is>
       </c>
       <c r="M26" s="7">
@@ -27378,25 +27378,25 @@
       </c>
       <c r="H27" s="6" t="inlineStr">
         <is>
-          <t>SLB</t>
+          <t>UPS</t>
         </is>
       </c>
       <c r="I27" s="61" t="n">
-        <v>0.01794027</v>
+        <v>0.01794622</v>
       </c>
       <c r="J27" s="6" t="inlineStr">
         <is>
-          <t>SLB</t>
+          <t>UNITED PARCEL SERVICE INC CLASS B</t>
         </is>
       </c>
       <c r="K27" s="6" t="inlineStr">
         <is>
-          <t>Energy</t>
+          <t>Industrials</t>
         </is>
       </c>
       <c r="L27" s="6" t="inlineStr">
         <is>
-          <t>SLB</t>
+          <t>UPS</t>
         </is>
       </c>
       <c r="M27" s="7">
@@ -27420,7 +27420,7 @@
         </is>
       </c>
       <c r="I28" s="61" t="n">
-        <v>0.01714394</v>
+        <v>0.01700291</v>
       </c>
       <c r="J28" s="6" t="inlineStr">
         <is>
@@ -27458,7 +27458,7 @@
         </is>
       </c>
       <c r="I29" s="61" t="n">
-        <v>0.01441625</v>
+        <v>0.01440745</v>
       </c>
       <c r="J29" s="6" t="inlineStr">
         <is>
@@ -27496,7 +27496,7 @@
         </is>
       </c>
       <c r="I30" s="61" t="n">
-        <v>0.01434565</v>
+        <v>0.01422793</v>
       </c>
       <c r="J30" s="6" t="inlineStr">
         <is>
@@ -27530,7 +27530,7 @@
         </is>
       </c>
       <c r="I31" s="61" t="n">
-        <v>0.01379243</v>
+        <v>0.01347148</v>
       </c>
       <c r="J31" s="6" t="inlineStr">
         <is>
@@ -27555,7 +27555,7 @@
         </is>
       </c>
       <c r="I32" s="61" t="n">
-        <v>0.01174717</v>
+        <v>0.01156825</v>
       </c>
       <c r="J32" s="6" t="inlineStr">
         <is>
@@ -27585,7 +27585,7 @@
         </is>
       </c>
       <c r="I33" s="61" t="n">
-        <v>0.01127959</v>
+        <v>0.01155408</v>
       </c>
       <c r="J33" s="6" t="inlineStr">
         <is>
@@ -27610,7 +27610,7 @@
         </is>
       </c>
       <c r="I34" s="61" t="n">
-        <v>0.009554709999999999</v>
+        <v>0.009426520000000001</v>
       </c>
       <c r="J34" s="6" t="inlineStr">
         <is>
@@ -27635,7 +27635,7 @@
         </is>
       </c>
       <c r="I35" s="61" t="n">
-        <v>0.008729799999999999</v>
+        <v>0.00876353</v>
       </c>
       <c r="J35" s="6" t="inlineStr">
         <is>
@@ -27660,7 +27660,7 @@
         </is>
       </c>
       <c r="I36" s="61" t="n">
-        <v>0.00863236</v>
+        <v>0.008757869999999999</v>
       </c>
       <c r="J36" s="6" t="inlineStr">
         <is>
@@ -27685,7 +27685,7 @@
         </is>
       </c>
       <c r="I37" s="61" t="n">
-        <v>0.00642043</v>
+        <v>0.00641953</v>
       </c>
       <c r="J37" s="6" t="inlineStr">
         <is>
@@ -27710,7 +27710,7 @@
         </is>
       </c>
       <c r="I38" s="61" t="n">
-        <v>0.00623166</v>
+        <v>0.006331</v>
       </c>
       <c r="J38" s="6" t="inlineStr">
         <is>
@@ -27731,20 +27731,20 @@
     <row r="39">
       <c r="H39" s="6" t="inlineStr">
         <is>
-          <t>DRI</t>
+          <t>HSY</t>
         </is>
       </c>
       <c r="I39" s="61" t="n">
-        <v>0.006045500000000001</v>
+        <v>0.00603122</v>
       </c>
       <c r="J39" s="6" t="inlineStr">
         <is>
-          <t>DARDEN RESTAURANTS INC</t>
+          <t>HERSHEY FOODS</t>
         </is>
       </c>
       <c r="K39" s="6" t="inlineStr">
         <is>
-          <t>Consumer Discretionary</t>
+          <t>Consumer Staples</t>
         </is>
       </c>
       <c r="L39" s="6" t="inlineStr"/>
@@ -27756,20 +27756,20 @@
     <row r="40">
       <c r="H40" s="6" t="inlineStr">
         <is>
-          <t>HSY</t>
+          <t>DRI</t>
         </is>
       </c>
       <c r="I40" s="61" t="n">
-        <v>0.00601652</v>
+        <v>0.0060163</v>
       </c>
       <c r="J40" s="6" t="inlineStr">
         <is>
-          <t>HERSHEY FOODS</t>
+          <t>DARDEN RESTAURANTS INC</t>
         </is>
       </c>
       <c r="K40" s="6" t="inlineStr">
         <is>
-          <t>Consumer Staples</t>
+          <t>Consumer Discretionary</t>
         </is>
       </c>
       <c r="L40" s="6" t="inlineStr"/>
@@ -27785,7 +27785,7 @@
         </is>
       </c>
       <c r="I41" s="61" t="n">
-        <v>0.005706050000000001</v>
+        <v>0.00576763</v>
       </c>
       <c r="J41" s="6" t="inlineStr">
         <is>
@@ -27810,7 +27810,7 @@
         </is>
       </c>
       <c r="I42" s="61" t="n">
-        <v>0.00525792</v>
+        <v>0.00529584</v>
       </c>
       <c r="J42" s="6" t="inlineStr">
         <is>
@@ -27835,7 +27835,7 @@
         </is>
       </c>
       <c r="I43" s="61" t="n">
-        <v>0.005126840000000001</v>
+        <v>0.005112299999999999</v>
       </c>
       <c r="J43" s="6" t="inlineStr">
         <is>
@@ -27860,7 +27860,7 @@
         </is>
       </c>
       <c r="I44" s="61" t="n">
-        <v>0.00491802</v>
+        <v>0.00498997</v>
       </c>
       <c r="J44" s="6" t="inlineStr">
         <is>
@@ -27885,7 +27885,7 @@
         </is>
       </c>
       <c r="I45" s="61" t="n">
-        <v>0.00473661</v>
+        <v>0.00470943</v>
       </c>
       <c r="J45" s="6" t="inlineStr">
         <is>
@@ -27910,7 +27910,7 @@
         </is>
       </c>
       <c r="I46" s="61" t="n">
-        <v>0.00464773</v>
+        <v>0.00460754</v>
       </c>
       <c r="J46" s="6" t="inlineStr">
         <is>
@@ -27935,7 +27935,7 @@
         </is>
       </c>
       <c r="I47" s="61" t="n">
-        <v>0.00444347</v>
+        <v>0.00451944</v>
       </c>
       <c r="J47" s="6" t="inlineStr">
         <is>
@@ -27956,20 +27956,20 @@
     <row r="48">
       <c r="H48" s="6" t="inlineStr">
         <is>
-          <t>APA</t>
+          <t>GIS</t>
         </is>
       </c>
       <c r="I48" s="61" t="n">
-        <v>0.00429283</v>
+        <v>0.00434551</v>
       </c>
       <c r="J48" s="6" t="inlineStr">
         <is>
-          <t>APA</t>
+          <t>GENERAL MILLS INC</t>
         </is>
       </c>
       <c r="K48" s="6" t="inlineStr">
         <is>
-          <t>Energy</t>
+          <t>Consumer Staples</t>
         </is>
       </c>
       <c r="L48" s="6" t="inlineStr"/>
@@ -27981,20 +27981,20 @@
     <row r="49">
       <c r="H49" s="6" t="inlineStr">
         <is>
-          <t>GIS</t>
+          <t>EWBC</t>
         </is>
       </c>
       <c r="I49" s="61" t="n">
-        <v>0.00428863</v>
+        <v>0.00427266</v>
       </c>
       <c r="J49" s="6" t="inlineStr">
         <is>
-          <t>GENERAL MILLS INC</t>
+          <t>EAST WEST BANCORP</t>
         </is>
       </c>
       <c r="K49" s="6" t="inlineStr">
         <is>
-          <t>Consumer Staples</t>
+          <t>Financials</t>
         </is>
       </c>
       <c r="L49" s="6" t="inlineStr"/>
@@ -28006,20 +28006,20 @@
     <row r="50">
       <c r="H50" s="6" t="inlineStr">
         <is>
-          <t>EWBC</t>
+          <t>APA</t>
         </is>
       </c>
       <c r="I50" s="61" t="n">
-        <v>0.00423464</v>
+        <v>0.00424979</v>
       </c>
       <c r="J50" s="6" t="inlineStr">
         <is>
-          <t>EAST WEST BANCORP</t>
+          <t>APA</t>
         </is>
       </c>
       <c r="K50" s="6" t="inlineStr">
         <is>
-          <t>Financials</t>
+          <t>Energy</t>
         </is>
       </c>
       <c r="L50" s="6" t="inlineStr"/>
@@ -28035,7 +28035,7 @@
         </is>
       </c>
       <c r="I51" s="61" t="n">
-        <v>0.0025765</v>
+        <v>0.00261124</v>
       </c>
       <c r="J51" s="6" t="inlineStr">
         <is>
@@ -28056,15 +28056,15 @@
     <row r="52">
       <c r="H52" s="6" t="inlineStr">
         <is>
-          <t>AFG</t>
+          <t>FNF</t>
         </is>
       </c>
       <c r="I52" s="61" t="n">
-        <v>0.0025068</v>
+        <v>0.00250636</v>
       </c>
       <c r="J52" s="6" t="inlineStr">
         <is>
-          <t>AMERICAN FINANCIAL GROUP</t>
+          <t>FIDELITY NATIONAL FINANCIAL INC</t>
         </is>
       </c>
       <c r="K52" s="6" t="inlineStr">
@@ -28081,15 +28081,15 @@
     <row r="53">
       <c r="H53" s="6" t="inlineStr">
         <is>
-          <t>FNF</t>
+          <t>AFG</t>
         </is>
       </c>
       <c r="I53" s="61" t="n">
-        <v>0.00249122</v>
+        <v>0.00249401</v>
       </c>
       <c r="J53" s="6" t="inlineStr">
         <is>
-          <t>FIDELITY NATIONAL FINANCIAL INC</t>
+          <t>AMERICAN FINANCIAL GROUP</t>
         </is>
       </c>
       <c r="K53" s="6" t="inlineStr">
@@ -28110,7 +28110,7 @@
         </is>
       </c>
       <c r="I54" s="61" t="n">
-        <v>0.00219234</v>
+        <v>0.00219085</v>
       </c>
       <c r="J54" s="6" t="inlineStr">
         <is>
@@ -28135,7 +28135,7 @@
         </is>
       </c>
       <c r="I55" s="61" t="n">
-        <v>0.00214697</v>
+        <v>0.00214161</v>
       </c>
       <c r="J55" s="6" t="inlineStr">
         <is>
@@ -28160,7 +28160,7 @@
         </is>
       </c>
       <c r="I56" s="61" t="n">
-        <v>0.00197159</v>
+        <v>0.00199168</v>
       </c>
       <c r="J56" s="6" t="inlineStr">
         <is>
@@ -28185,7 +28185,7 @@
         </is>
       </c>
       <c r="I57" s="61" t="n">
-        <v>0.00191095</v>
+        <v>0.00189993</v>
       </c>
       <c r="J57" s="6" t="inlineStr">
         <is>
@@ -28210,7 +28210,7 @@
         </is>
       </c>
       <c r="I58" s="61" t="n">
-        <v>0.00154167</v>
+        <v>0.00154497</v>
       </c>
       <c r="J58" s="6" t="inlineStr">
         <is>
@@ -28235,11 +28235,11 @@
         </is>
       </c>
       <c r="I59" s="61" t="n">
-        <v>0.00152714</v>
+        <v>0.00149545</v>
       </c>
       <c r="J59" s="6" t="inlineStr">
         <is>
-          <t>MACYS INC</t>
+          <t>MACYS</t>
         </is>
       </c>
       <c r="K59" s="6" t="inlineStr">
@@ -28260,7 +28260,7 @@
         </is>
       </c>
       <c r="I60" s="61" t="n">
-        <v>0.00144688</v>
+        <v>0.00144259</v>
       </c>
       <c r="J60" s="6" t="inlineStr">
         <is>
@@ -28285,7 +28285,7 @@
         </is>
       </c>
       <c r="I61" s="61" t="n">
-        <v>0.00141319</v>
+        <v>0.00141312</v>
       </c>
       <c r="J61" s="6" t="inlineStr">
         <is>
@@ -28310,7 +28310,7 @@
         </is>
       </c>
       <c r="I62" s="61" t="n">
-        <v>0.00132502</v>
+        <v>0.00131177</v>
       </c>
       <c r="J62" s="6" t="inlineStr">
         <is>
@@ -28335,7 +28335,7 @@
         </is>
       </c>
       <c r="I63" s="61" t="n">
-        <v>0.00118386</v>
+        <v>0.00119145</v>
       </c>
       <c r="J63" s="6" t="inlineStr">
         <is>
@@ -28360,7 +28360,7 @@
         </is>
       </c>
       <c r="I64" s="61" t="n">
-        <v>0.00113003</v>
+        <v>0.00113949</v>
       </c>
       <c r="J64" s="6" t="inlineStr">
         <is>
@@ -28385,7 +28385,7 @@
         </is>
       </c>
       <c r="I65" s="61" t="n">
-        <v>0.00096994</v>
+        <v>0.00096997</v>
       </c>
       <c r="J65" s="6" t="inlineStr">
         <is>
@@ -28410,7 +28410,7 @@
         </is>
       </c>
       <c r="I66" s="61" t="n">
-        <v>0.00096542</v>
+        <v>0.00096707</v>
       </c>
       <c r="J66" s="6" t="inlineStr">
         <is>
@@ -28435,7 +28435,7 @@
         </is>
       </c>
       <c r="I67" s="61" t="n">
-        <v>0.0009271500000000001</v>
+        <v>0.0009162900000000001</v>
       </c>
       <c r="J67" s="6" t="inlineStr">
         <is>
@@ -28460,7 +28460,7 @@
         </is>
       </c>
       <c r="I68" s="61" t="n">
-        <v>0.00091108</v>
+        <v>0.0009137699999999999</v>
       </c>
       <c r="J68" s="6" t="inlineStr">
         <is>
@@ -28485,7 +28485,7 @@
         </is>
       </c>
       <c r="I69" s="61" t="n">
-        <v>0.00089713</v>
+        <v>0.00089821</v>
       </c>
       <c r="J69" s="6" t="inlineStr">
         <is>
@@ -28510,7 +28510,7 @@
         </is>
       </c>
       <c r="I70" s="61" t="n">
-        <v>0.00087914</v>
+        <v>0.00088813</v>
       </c>
       <c r="J70" s="6" t="inlineStr">
         <is>
@@ -28535,7 +28535,7 @@
         </is>
       </c>
       <c r="I71" s="61" t="n">
-        <v>0.0008120299999999999</v>
+        <v>0.00082553</v>
       </c>
       <c r="J71" s="6" t="inlineStr">
         <is>
@@ -28556,15 +28556,15 @@
     <row r="72">
       <c r="H72" s="6" t="inlineStr">
         <is>
-          <t>BANR</t>
+          <t>APAM</t>
         </is>
       </c>
       <c r="I72" s="61" t="n">
-        <v>0.00055785</v>
+        <v>0.0005663</v>
       </c>
       <c r="J72" s="6" t="inlineStr">
         <is>
-          <t>BANNER CORP</t>
+          <t>ARTISAN PARTNERS ASSET MANAGEMENT</t>
         </is>
       </c>
       <c r="K72" s="6" t="inlineStr">
@@ -28581,15 +28581,15 @@
     <row r="73">
       <c r="H73" s="6" t="inlineStr">
         <is>
-          <t>APAM</t>
+          <t>BANR</t>
         </is>
       </c>
       <c r="I73" s="61" t="n">
-        <v>0.00055747</v>
+        <v>0.00056032</v>
       </c>
       <c r="J73" s="6" t="inlineStr">
         <is>
-          <t>ARTISAN PARTNERS ASSET MANAGEMENT</t>
+          <t>BANNER CORP</t>
         </is>
       </c>
       <c r="K73" s="6" t="inlineStr">
@@ -28610,7 +28610,7 @@
         </is>
       </c>
       <c r="I74" s="61" t="n">
-        <v>0.0005436</v>
+        <v>0.0005444299999999999</v>
       </c>
       <c r="J74" s="6" t="inlineStr">
         <is>
@@ -28635,7 +28635,7 @@
         </is>
       </c>
       <c r="I75" s="61" t="n">
-        <v>0.0005161500000000001</v>
+        <v>0.00051459</v>
       </c>
       <c r="J75" s="6" t="inlineStr">
         <is>
@@ -28660,7 +28660,7 @@
         </is>
       </c>
       <c r="I76" s="61" t="n">
-        <v>0.00050315</v>
+        <v>0.00050215</v>
       </c>
       <c r="J76" s="6" t="inlineStr">
         <is>
@@ -28681,15 +28681,15 @@
     <row r="77">
       <c r="H77" s="6" t="inlineStr">
         <is>
-          <t>CHCO</t>
+          <t>CNS</t>
         </is>
       </c>
       <c r="I77" s="61" t="n">
-        <v>0.00048714</v>
+        <v>0.00049549</v>
       </c>
       <c r="J77" s="6" t="inlineStr">
         <is>
-          <t>CITY HOLDING</t>
+          <t>COHEN &amp; STEERS INC</t>
         </is>
       </c>
       <c r="K77" s="6" t="inlineStr">
@@ -28706,15 +28706,15 @@
     <row r="78">
       <c r="H78" s="6" t="inlineStr">
         <is>
-          <t>CNS</t>
+          <t>CHCO</t>
         </is>
       </c>
       <c r="I78" s="61" t="n">
-        <v>0.00047667</v>
+        <v>0.00048529</v>
       </c>
       <c r="J78" s="6" t="inlineStr">
         <is>
-          <t>COHEN &amp; STEERS INC</t>
+          <t>CITY HOLDING</t>
         </is>
       </c>
       <c r="K78" s="6" t="inlineStr">
@@ -28735,7 +28735,7 @@
         </is>
       </c>
       <c r="I79" s="61" t="n">
-        <v>0.00047435</v>
+        <v>0.00047208</v>
       </c>
       <c r="J79" s="6" t="inlineStr">
         <is>
@@ -28760,7 +28760,7 @@
         </is>
       </c>
       <c r="I80" s="61" t="n">
-        <v>0.00046024</v>
+        <v>0.00046119</v>
       </c>
       <c r="J80" s="6" t="inlineStr">
         <is>
@@ -28785,7 +28785,7 @@
         </is>
       </c>
       <c r="I81" s="61" t="n">
-        <v>0.00045899</v>
+        <v>0.00045641</v>
       </c>
       <c r="J81" s="6" t="inlineStr">
         <is>
@@ -28810,7 +28810,7 @@
         </is>
       </c>
       <c r="I82" s="61" t="n">
-        <v>0.00043236</v>
+        <v>0.00043535</v>
       </c>
       <c r="J82" s="6" t="inlineStr">
         <is>
@@ -28835,7 +28835,7 @@
         </is>
       </c>
       <c r="I83" s="61" t="n">
-        <v>0.00042214</v>
+        <v>0.00042315</v>
       </c>
       <c r="J83" s="6" t="inlineStr">
         <is>
@@ -28860,7 +28860,7 @@
         </is>
       </c>
       <c r="I84" s="61" t="n">
-        <v>0.00041077</v>
+        <v>0.00041123</v>
       </c>
       <c r="J84" s="6" t="inlineStr">
         <is>
@@ -28885,7 +28885,7 @@
         </is>
       </c>
       <c r="I85" s="61" t="n">
-        <v>0.00040583</v>
+        <v>0.00038781</v>
       </c>
       <c r="J85" s="6" t="inlineStr">
         <is>
@@ -28906,7 +28906,7 @@
         </is>
       </c>
       <c r="I86" s="61" t="n">
-        <v>0.00037481</v>
+        <v>0.00037497</v>
       </c>
       <c r="J86" s="6" t="inlineStr">
         <is>
@@ -28927,20 +28927,20 @@
     <row r="87">
       <c r="H87" s="6" t="inlineStr">
         <is>
-          <t>BKE</t>
+          <t>LKFN</t>
         </is>
       </c>
       <c r="I87" s="61" t="n">
-        <v>0.00035561</v>
+        <v>0.00035496</v>
       </c>
       <c r="J87" s="6" t="inlineStr">
         <is>
-          <t>BUCKLE</t>
+          <t>LAKELAND FINANCIAL CORP</t>
         </is>
       </c>
       <c r="K87" s="6" t="inlineStr">
         <is>
-          <t>Consumer Discretionary</t>
+          <t>Financials</t>
         </is>
       </c>
       <c r="L87" s="6" t="inlineStr"/>
@@ -28952,20 +28952,20 @@
     <row r="88">
       <c r="H88" s="6" t="inlineStr">
         <is>
-          <t>LKFN</t>
+          <t>BKE</t>
         </is>
       </c>
       <c r="I88" s="61" t="n">
-        <v>0.00035326</v>
+        <v>0.00034819</v>
       </c>
       <c r="J88" s="6" t="inlineStr">
         <is>
-          <t>LAKELAND FINANCIAL CORP</t>
+          <t>BUCKLE</t>
         </is>
       </c>
       <c r="K88" s="6" t="inlineStr">
         <is>
-          <t>Financials</t>
+          <t>Consumer Discretionary</t>
         </is>
       </c>
       <c r="L88" s="6" t="inlineStr"/>
@@ -28981,7 +28981,7 @@
         </is>
       </c>
       <c r="I89" s="61" t="n">
-        <v>0.0003126</v>
+        <v>0.00030963</v>
       </c>
       <c r="J89" s="6" t="inlineStr">
         <is>
@@ -29006,7 +29006,7 @@
         </is>
       </c>
       <c r="I90" s="61" t="n">
-        <v>0.00027839</v>
+        <v>0.00027876</v>
       </c>
       <c r="J90" s="6" t="inlineStr">
         <is>
@@ -29027,20 +29027,20 @@
     <row r="91">
       <c r="H91" s="6" t="inlineStr">
         <is>
-          <t>WEN</t>
+          <t>CNA</t>
         </is>
       </c>
       <c r="I91" s="61" t="n">
-        <v>0.00026436</v>
+        <v>0.00025555</v>
       </c>
       <c r="J91" s="6" t="inlineStr">
         <is>
-          <t>WENDYS</t>
+          <t>CNA FINANCIAL CORP</t>
         </is>
       </c>
       <c r="K91" s="6" t="inlineStr">
         <is>
-          <t>Consumer Discretionary</t>
+          <t>Financials</t>
         </is>
       </c>
       <c r="L91" s="6" t="inlineStr"/>
@@ -29052,20 +29052,20 @@
     <row r="92">
       <c r="H92" s="6" t="inlineStr">
         <is>
-          <t>CNA</t>
+          <t>WEN</t>
         </is>
       </c>
       <c r="I92" s="61" t="n">
-        <v>0.00025582</v>
+        <v>0.00025473</v>
       </c>
       <c r="J92" s="6" t="inlineStr">
         <is>
-          <t>CNA FINANCIAL CORP</t>
+          <t>WENDYS</t>
         </is>
       </c>
       <c r="K92" s="6" t="inlineStr">
         <is>
-          <t>Financials</t>
+          <t>Consumer Discretionary</t>
         </is>
       </c>
       <c r="L92" s="6" t="inlineStr"/>
@@ -29081,7 +29081,7 @@
         </is>
       </c>
       <c r="I93" s="61" t="n">
-        <v>0.00022948</v>
+        <v>0.00022989</v>
       </c>
       <c r="J93" s="6" t="inlineStr">
         <is>
@@ -29106,7 +29106,7 @@
         </is>
       </c>
       <c r="I94" s="61" t="n">
-        <v>0.0002251</v>
+        <v>0.00022572</v>
       </c>
       <c r="J94" s="6" t="inlineStr">
         <is>
@@ -29131,7 +29131,7 @@
         </is>
       </c>
       <c r="I95" s="61" t="n">
-        <v>0.00020276</v>
+        <v>0.00020398</v>
       </c>
       <c r="J95" s="6" t="inlineStr">
         <is>
@@ -29156,7 +29156,7 @@
         </is>
       </c>
       <c r="I96" s="61" t="n">
-        <v>0.00019517</v>
+        <v>0.00019656</v>
       </c>
       <c r="J96" s="6" t="inlineStr">
         <is>
@@ -29181,7 +29181,7 @@
         </is>
       </c>
       <c r="I97" s="61" t="n">
-        <v>0.00019455</v>
+        <v>0.00019476</v>
       </c>
       <c r="J97" s="6" t="inlineStr">
         <is>
@@ -29206,7 +29206,7 @@
         </is>
       </c>
       <c r="I98" s="61" t="n">
-        <v>0.00017741</v>
+        <v>0.00017857</v>
       </c>
       <c r="J98" s="6" t="inlineStr">
         <is>
@@ -29231,7 +29231,7 @@
         </is>
       </c>
       <c r="I99" s="61" t="n">
-        <v>0.00016406</v>
+        <v>0.00016453</v>
       </c>
       <c r="J99" s="6" t="inlineStr">
         <is>
@@ -29256,7 +29256,7 @@
         </is>
       </c>
       <c r="I100" s="61" t="n">
-        <v>0.00013139</v>
+        <v>0.00013087</v>
       </c>
       <c r="J100" s="6" t="inlineStr">
         <is>
@@ -29277,22 +29277,18 @@
     <row r="101">
       <c r="H101" s="6" t="inlineStr">
         <is>
-          <t>AMSF</t>
+          <t>USD</t>
         </is>
       </c>
       <c r="I101" s="61" t="n">
-        <v>0.00011576</v>
+        <v>0.00013085</v>
       </c>
       <c r="J101" s="6" t="inlineStr">
         <is>
-          <t>AMERISAFE INC</t>
-        </is>
-      </c>
-      <c r="K101" s="6" t="inlineStr">
-        <is>
-          <t>Financials</t>
-        </is>
-      </c>
+          <t>US DOLLAR</t>
+        </is>
+      </c>
+      <c r="K101" s="6" t="inlineStr"/>
       <c r="L101" s="6" t="inlineStr"/>
       <c r="M101" s="7">
         <f>IF(H101="","",IFERROR(VLOOKUP(K101,$P$5:$Q$15,2,FALSE),"현금·선물"))</f>
@@ -29302,18 +29298,22 @@
     <row r="102">
       <c r="H102" s="6" t="inlineStr">
         <is>
-          <t>USD</t>
+          <t>AMSF</t>
         </is>
       </c>
       <c r="I102" s="61" t="n">
-        <v>0.00011066</v>
+        <v>0.00011431</v>
       </c>
       <c r="J102" s="6" t="inlineStr">
         <is>
-          <t>US DOLLAR</t>
-        </is>
-      </c>
-      <c r="K102" s="6" t="inlineStr"/>
+          <t>AMERISAFE INC</t>
+        </is>
+      </c>
+      <c r="K102" s="6" t="inlineStr">
+        <is>
+          <t>Financials</t>
+        </is>
+      </c>
       <c r="L102" s="6" t="inlineStr"/>
       <c r="M102" s="7">
         <f>IF(H102="","",IFERROR(VLOOKUP(K102,$P$5:$Q$15,2,FALSE),"현금·선물"))</f>
@@ -29327,7 +29327,7 @@
         </is>
       </c>
       <c r="I103" s="61" t="n">
-        <v>9.738999999999999e-05</v>
+        <v>9.802999999999999e-05</v>
       </c>
       <c r="J103" s="6" t="inlineStr">
         <is>
@@ -29352,7 +29352,7 @@
         </is>
       </c>
       <c r="I104" s="61" t="n">
-        <v>9.112000000000001e-05</v>
+        <v>9.091e-05</v>
       </c>
       <c r="J104" s="6" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
데이터 갱신: holdings,official (2026-10-22)
</commit_message>
<xml_diff>
--- a/downloads/schd_dividend_tracker.xlsx
+++ b/downloads/schd_dividend_tracker.xlsx
@@ -1724,7 +1724,7 @@
     <row r="3">
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>최종 갱신: 2026-10-21 · 반영 범위: 2012년 1분기 ~ 2026년 3분기 (배당락 2026-09-23) · GitHub Actions 자동 생성</t>
+          <t>최종 갱신: 2026-10-22 · 반영 범위: 2012년 1분기 ~ 2026년 3분기 (배당락 2026-09-23) · GitHub Actions 자동 생성</t>
         </is>
       </c>
     </row>
@@ -11996,11 +11996,11 @@
         </is>
       </c>
       <c r="B34" s="19" t="n">
-        <v>0.033</v>
+        <v>0.0318</v>
       </c>
       <c r="C34" s="2" t="inlineStr">
         <is>
-          <t>2026-10-13 기준 · 최근 30일 순투자수익(보수 차감) 연 환산</t>
+          <t>2026-10-20 기준 · 최근 30일 순투자수익(보수 차감) 연 환산</t>
         </is>
       </c>
     </row>
@@ -26257,11 +26257,11 @@
         </is>
       </c>
       <c r="B2" s="49" t="n">
-        <v>46315</v>
+        <v>46316</v>
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>← 이 날 종가로 계산한 비중. 그날 공식 파일을 못 받아 Schwab 공식 보유종목 CSV(2026-10-19)의 보유 주식 수 × 종가로 계산했습니다.</t>
+          <t>← 이 날 종가로 계산한 비중. 그날 공식 파일을 못 받아 Schwab 공식 보유종목 CSV(2026-10-20)의 보유 주식 수 × 종가로 계산했습니다.</t>
         </is>
       </c>
     </row>
@@ -26358,7 +26358,7 @@
         </is>
       </c>
       <c r="I5" s="61" t="n">
-        <v>0.0437362</v>
+        <v>0.04485776</v>
       </c>
       <c r="J5" s="6" t="inlineStr">
         <is>
@@ -26412,25 +26412,25 @@
       </c>
       <c r="H6" s="6" t="inlineStr">
         <is>
-          <t>PG</t>
+          <t>CVX</t>
         </is>
       </c>
       <c r="I6" s="61" t="n">
-        <v>0.04329193</v>
+        <v>0.04299757</v>
       </c>
       <c r="J6" s="6" t="inlineStr">
         <is>
-          <t>PROCTER &amp; GAMBLE</t>
+          <t>CHEVRON</t>
         </is>
       </c>
       <c r="K6" s="6" t="inlineStr">
         <is>
-          <t>Consumer Staples</t>
+          <t>Energy</t>
         </is>
       </c>
       <c r="L6" s="6" t="inlineStr">
         <is>
-          <t>프록터앤드갬블</t>
+          <t>셰브론</t>
         </is>
       </c>
       <c r="M6" s="7">
@@ -26470,25 +26470,25 @@
       </c>
       <c r="H7" s="6" t="inlineStr">
         <is>
-          <t>CVX</t>
+          <t>PG</t>
         </is>
       </c>
       <c r="I7" s="61" t="n">
-        <v>0.04275667</v>
+        <v>0.042656</v>
       </c>
       <c r="J7" s="6" t="inlineStr">
         <is>
-          <t>CHEVRON</t>
+          <t>PROCTER &amp; GAMBLE</t>
         </is>
       </c>
       <c r="K7" s="6" t="inlineStr">
         <is>
-          <t>Energy</t>
+          <t>Consumer Staples</t>
         </is>
       </c>
       <c r="L7" s="6" t="inlineStr">
         <is>
-          <t>셰브론</t>
+          <t>프록터앤드갬블</t>
         </is>
       </c>
       <c r="M7" s="7">
@@ -26532,7 +26532,7 @@
         </is>
       </c>
       <c r="I8" s="61" t="n">
-        <v>0.04262202</v>
+        <v>0.04257815</v>
       </c>
       <c r="J8" s="6" t="inlineStr">
         <is>
@@ -26590,7 +26590,7 @@
         </is>
       </c>
       <c r="I9" s="61" t="n">
-        <v>0.04250498</v>
+        <v>0.04217424</v>
       </c>
       <c r="J9" s="6" t="inlineStr">
         <is>
@@ -26644,25 +26644,25 @@
       </c>
       <c r="H10" s="6" t="inlineStr">
         <is>
-          <t>UNH</t>
+          <t>QCOM</t>
         </is>
       </c>
       <c r="I10" s="61" t="n">
-        <v>0.04208503</v>
+        <v>0.04204388</v>
       </c>
       <c r="J10" s="6" t="inlineStr">
         <is>
-          <t>UNITEDHEALTH GROUP</t>
+          <t>QUALCOMM</t>
         </is>
       </c>
       <c r="K10" s="6" t="inlineStr">
         <is>
-          <t>Health Care</t>
+          <t>Information Technology</t>
         </is>
       </c>
       <c r="L10" s="6" t="inlineStr">
         <is>
-          <t>유나이티드헬스</t>
+          <t>퀄컴</t>
         </is>
       </c>
       <c r="M10" s="7">
@@ -26702,25 +26702,25 @@
       </c>
       <c r="H11" s="6" t="inlineStr">
         <is>
-          <t>QCOM</t>
+          <t>UNH</t>
         </is>
       </c>
       <c r="I11" s="61" t="n">
-        <v>0.04147538</v>
+        <v>0.04189536999999999</v>
       </c>
       <c r="J11" s="6" t="inlineStr">
         <is>
-          <t>QUALCOMM</t>
+          <t>UNITEDHEALTH GROUP</t>
         </is>
       </c>
       <c r="K11" s="6" t="inlineStr">
         <is>
-          <t>Information Technology</t>
+          <t>Health Care</t>
         </is>
       </c>
       <c r="L11" s="6" t="inlineStr">
         <is>
-          <t>퀄컴</t>
+          <t>유나이티드헬스</t>
         </is>
       </c>
       <c r="M11" s="7">
@@ -26764,7 +26764,7 @@
         </is>
       </c>
       <c r="I12" s="61" t="n">
-        <v>0.03976414</v>
+        <v>0.03974505</v>
       </c>
       <c r="J12" s="6" t="inlineStr">
         <is>
@@ -26818,25 +26818,25 @@
       </c>
       <c r="H13" s="6" t="inlineStr">
         <is>
-          <t>HD</t>
+          <t>MRK</t>
         </is>
       </c>
       <c r="I13" s="61" t="n">
-        <v>0.03968929</v>
+        <v>0.03968767</v>
       </c>
       <c r="J13" s="6" t="inlineStr">
         <is>
-          <t>HOME DEPOT</t>
+          <t>MERCK &amp; CO INC</t>
         </is>
       </c>
       <c r="K13" s="6" t="inlineStr">
         <is>
-          <t>Consumer Discretionary</t>
+          <t>Health Care</t>
         </is>
       </c>
       <c r="L13" s="6" t="inlineStr">
         <is>
-          <t>홈디포</t>
+          <t>머크</t>
         </is>
       </c>
       <c r="M13" s="7">
@@ -26876,25 +26876,25 @@
       </c>
       <c r="H14" s="6" t="inlineStr">
         <is>
-          <t>MRK</t>
+          <t>HD</t>
         </is>
       </c>
       <c r="I14" s="61" t="n">
-        <v>0.03923437</v>
+        <v>0.03960226</v>
       </c>
       <c r="J14" s="6" t="inlineStr">
         <is>
-          <t>MERCK &amp; CO INC</t>
+          <t>HOME DEPOT</t>
         </is>
       </c>
       <c r="K14" s="6" t="inlineStr">
         <is>
-          <t>Health Care</t>
+          <t>Consumer Discretionary</t>
         </is>
       </c>
       <c r="L14" s="6" t="inlineStr">
         <is>
-          <t>머크</t>
+          <t>홈디포</t>
         </is>
       </c>
       <c r="M14" s="7">
@@ -26928,7 +26928,7 @@
         </is>
       </c>
       <c r="I15" s="61" t="n">
-        <v>0.03826222</v>
+        <v>0.03849057</v>
       </c>
       <c r="J15" s="6" t="inlineStr">
         <is>
@@ -26976,7 +26976,7 @@
         </is>
       </c>
       <c r="I16" s="61" t="n">
-        <v>0.03720558</v>
+        <v>0.03653357</v>
       </c>
       <c r="J16" s="6" t="inlineStr">
         <is>
@@ -27010,25 +27010,25 @@
       </c>
       <c r="H17" s="6" t="inlineStr">
         <is>
-          <t>VZ</t>
+          <t>ACN</t>
         </is>
       </c>
       <c r="I17" s="61" t="n">
-        <v>0.03558074</v>
+        <v>0.03577195</v>
       </c>
       <c r="J17" s="6" t="inlineStr">
         <is>
-          <t>VERIZON COMMUNICATIONS INC</t>
+          <t>ACCENTURE PLC CLASS A</t>
         </is>
       </c>
       <c r="K17" s="6" t="inlineStr">
         <is>
-          <t>Communication Services</t>
+          <t>Information Technology</t>
         </is>
       </c>
       <c r="L17" s="6" t="inlineStr">
         <is>
-          <t>버라이즌</t>
+          <t>액센츄어</t>
         </is>
       </c>
       <c r="M17" s="7">
@@ -27048,25 +27048,25 @@
       </c>
       <c r="H18" s="6" t="inlineStr">
         <is>
-          <t>ACN</t>
+          <t>VZ</t>
         </is>
       </c>
       <c r="I18" s="61" t="n">
-        <v>0.03557055</v>
+        <v>0.03482887</v>
       </c>
       <c r="J18" s="6" t="inlineStr">
         <is>
-          <t>ACCENTURE PLC CLASS A</t>
+          <t>VERIZON COMMUNICATIONS INC</t>
         </is>
       </c>
       <c r="K18" s="6" t="inlineStr">
         <is>
-          <t>Information Technology</t>
+          <t>Communication Services</t>
         </is>
       </c>
       <c r="L18" s="6" t="inlineStr">
         <is>
-          <t>액센츄어</t>
+          <t>버라이즌</t>
         </is>
       </c>
       <c r="M18" s="7">
@@ -27081,7 +27081,7 @@
         </is>
       </c>
       <c r="I19" s="61" t="n">
-        <v>0.03062798</v>
+        <v>0.03037695</v>
       </c>
       <c r="J19" s="6" t="inlineStr">
         <is>
@@ -27115,7 +27115,7 @@
         </is>
       </c>
       <c r="I20" s="61" t="n">
-        <v>0.03029613</v>
+        <v>0.02999405</v>
       </c>
       <c r="J20" s="6" t="inlineStr">
         <is>
@@ -27154,7 +27154,7 @@
         </is>
       </c>
       <c r="I21" s="61" t="n">
-        <v>0.02827079</v>
+        <v>0.02846511</v>
       </c>
       <c r="J21" s="6" t="inlineStr">
         <is>
@@ -27192,11 +27192,11 @@
         </is>
       </c>
       <c r="I22" s="61" t="n">
-        <v>0.02708957</v>
+        <v>0.02725198</v>
       </c>
       <c r="J22" s="6" t="inlineStr">
         <is>
-          <t>LOCKHEED MARTIN CORP</t>
+          <t>LOCKHEED MARTIN</t>
         </is>
       </c>
       <c r="K22" s="6" t="inlineStr">
@@ -27230,7 +27230,7 @@
         </is>
       </c>
       <c r="I23" s="61" t="n">
-        <v>0.02013451</v>
+        <v>0.02014859</v>
       </c>
       <c r="J23" s="6" t="inlineStr">
         <is>
@@ -27268,7 +27268,7 @@
         </is>
       </c>
       <c r="I24" s="61" t="n">
-        <v>0.02013349</v>
+        <v>0.02001077</v>
       </c>
       <c r="J24" s="6" t="inlineStr">
         <is>
@@ -27306,7 +27306,7 @@
         </is>
       </c>
       <c r="I25" s="61" t="n">
-        <v>0.01923721</v>
+        <v>0.01901324</v>
       </c>
       <c r="J25" s="6" t="inlineStr">
         <is>
@@ -27344,7 +27344,7 @@
         </is>
       </c>
       <c r="I26" s="61" t="n">
-        <v>0.01803174</v>
+        <v>0.01845224</v>
       </c>
       <c r="J26" s="6" t="inlineStr">
         <is>
@@ -27382,7 +27382,7 @@
         </is>
       </c>
       <c r="I27" s="61" t="n">
-        <v>0.01794622</v>
+        <v>0.01815364</v>
       </c>
       <c r="J27" s="6" t="inlineStr">
         <is>
@@ -27420,7 +27420,7 @@
         </is>
       </c>
       <c r="I28" s="61" t="n">
-        <v>0.01700291</v>
+        <v>0.01683904</v>
       </c>
       <c r="J28" s="6" t="inlineStr">
         <is>
@@ -27458,7 +27458,7 @@
         </is>
       </c>
       <c r="I29" s="61" t="n">
-        <v>0.01440745</v>
+        <v>0.0146548</v>
       </c>
       <c r="J29" s="6" t="inlineStr">
         <is>
@@ -27496,7 +27496,7 @@
         </is>
       </c>
       <c r="I30" s="61" t="n">
-        <v>0.01422793</v>
+        <v>0.01428201</v>
       </c>
       <c r="J30" s="6" t="inlineStr">
         <is>
@@ -27530,7 +27530,7 @@
         </is>
       </c>
       <c r="I31" s="61" t="n">
-        <v>0.01347148</v>
+        <v>0.01334698</v>
       </c>
       <c r="J31" s="6" t="inlineStr">
         <is>
@@ -27551,20 +27551,20 @@
     <row r="32">
       <c r="H32" s="6" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>FITB</t>
         </is>
       </c>
       <c r="I32" s="61" t="n">
-        <v>0.01156825</v>
+        <v>0.01165263</v>
       </c>
       <c r="J32" s="6" t="inlineStr">
         <is>
-          <t>FORD MOTOR</t>
+          <t>FIFTH THIRD BANCORP</t>
         </is>
       </c>
       <c r="K32" s="6" t="inlineStr">
         <is>
-          <t>Consumer Discretionary</t>
+          <t>Financials</t>
         </is>
       </c>
       <c r="L32" s="6" t="inlineStr"/>
@@ -27581,20 +27581,20 @@
       </c>
       <c r="H33" s="6" t="inlineStr">
         <is>
-          <t>FITB</t>
+          <t>F</t>
         </is>
       </c>
       <c r="I33" s="61" t="n">
-        <v>0.01155408</v>
+        <v>0.01134031</v>
       </c>
       <c r="J33" s="6" t="inlineStr">
         <is>
-          <t>FIFTH THIRD BANCORP</t>
+          <t>FORD MOTOR</t>
         </is>
       </c>
       <c r="K33" s="6" t="inlineStr">
         <is>
-          <t>Financials</t>
+          <t>Consumer Discretionary</t>
         </is>
       </c>
       <c r="L33" s="6" t="inlineStr"/>
@@ -27610,7 +27610,7 @@
         </is>
       </c>
       <c r="I34" s="61" t="n">
-        <v>0.009426520000000001</v>
+        <v>0.009305909999999999</v>
       </c>
       <c r="J34" s="6" t="inlineStr">
         <is>
@@ -27635,7 +27635,7 @@
         </is>
       </c>
       <c r="I35" s="61" t="n">
-        <v>0.00876353</v>
+        <v>0.008761970000000001</v>
       </c>
       <c r="J35" s="6" t="inlineStr">
         <is>
@@ -27660,7 +27660,7 @@
         </is>
       </c>
       <c r="I36" s="61" t="n">
-        <v>0.008757869999999999</v>
+        <v>0.00862889</v>
       </c>
       <c r="J36" s="6" t="inlineStr">
         <is>
@@ -27685,7 +27685,7 @@
         </is>
       </c>
       <c r="I37" s="61" t="n">
-        <v>0.00641953</v>
+        <v>0.00648346</v>
       </c>
       <c r="J37" s="6" t="inlineStr">
         <is>
@@ -27710,7 +27710,7 @@
         </is>
       </c>
       <c r="I38" s="61" t="n">
-        <v>0.006331</v>
+        <v>0.00637586</v>
       </c>
       <c r="J38" s="6" t="inlineStr">
         <is>
@@ -27735,7 +27735,7 @@
         </is>
       </c>
       <c r="I39" s="61" t="n">
-        <v>0.00603122</v>
+        <v>0.005973549999999999</v>
       </c>
       <c r="J39" s="6" t="inlineStr">
         <is>
@@ -27760,7 +27760,7 @@
         </is>
       </c>
       <c r="I40" s="61" t="n">
-        <v>0.0060163</v>
+        <v>0.00592575</v>
       </c>
       <c r="J40" s="6" t="inlineStr">
         <is>
@@ -27785,7 +27785,7 @@
         </is>
       </c>
       <c r="I41" s="61" t="n">
-        <v>0.00576763</v>
+        <v>0.00581422</v>
       </c>
       <c r="J41" s="6" t="inlineStr">
         <is>
@@ -27810,7 +27810,7 @@
         </is>
       </c>
       <c r="I42" s="61" t="n">
-        <v>0.00529584</v>
+        <v>0.00536073</v>
       </c>
       <c r="J42" s="6" t="inlineStr">
         <is>
@@ -27835,7 +27835,7 @@
         </is>
       </c>
       <c r="I43" s="61" t="n">
-        <v>0.005112299999999999</v>
+        <v>0.005140519999999999</v>
       </c>
       <c r="J43" s="6" t="inlineStr">
         <is>
@@ -27860,7 +27860,7 @@
         </is>
       </c>
       <c r="I44" s="61" t="n">
-        <v>0.00498997</v>
+        <v>0.00494746</v>
       </c>
       <c r="J44" s="6" t="inlineStr">
         <is>
@@ -27885,7 +27885,7 @@
         </is>
       </c>
       <c r="I45" s="61" t="n">
-        <v>0.00470943</v>
+        <v>0.0047234</v>
       </c>
       <c r="J45" s="6" t="inlineStr">
         <is>
@@ -27910,7 +27910,7 @@
         </is>
       </c>
       <c r="I46" s="61" t="n">
-        <v>0.00460754</v>
+        <v>0.004642879999999999</v>
       </c>
       <c r="J46" s="6" t="inlineStr">
         <is>
@@ -27935,7 +27935,7 @@
         </is>
       </c>
       <c r="I47" s="61" t="n">
-        <v>0.00451944</v>
+        <v>0.00453454</v>
       </c>
       <c r="J47" s="6" t="inlineStr">
         <is>
@@ -27956,20 +27956,20 @@
     <row r="48">
       <c r="H48" s="6" t="inlineStr">
         <is>
-          <t>GIS</t>
+          <t>EWBC</t>
         </is>
       </c>
       <c r="I48" s="61" t="n">
-        <v>0.00434551</v>
+        <v>0.00438045</v>
       </c>
       <c r="J48" s="6" t="inlineStr">
         <is>
-          <t>GENERAL MILLS INC</t>
+          <t>EAST WEST BANCORP</t>
         </is>
       </c>
       <c r="K48" s="6" t="inlineStr">
         <is>
-          <t>Consumer Staples</t>
+          <t>Financials</t>
         </is>
       </c>
       <c r="L48" s="6" t="inlineStr"/>
@@ -27981,20 +27981,20 @@
     <row r="49">
       <c r="H49" s="6" t="inlineStr">
         <is>
-          <t>EWBC</t>
+          <t>GIS</t>
         </is>
       </c>
       <c r="I49" s="61" t="n">
-        <v>0.00427266</v>
+        <v>0.00423748</v>
       </c>
       <c r="J49" s="6" t="inlineStr">
         <is>
-          <t>EAST WEST BANCORP</t>
+          <t>GENERAL MILLS INC</t>
         </is>
       </c>
       <c r="K49" s="6" t="inlineStr">
         <is>
-          <t>Financials</t>
+          <t>Consumer Staples</t>
         </is>
       </c>
       <c r="L49" s="6" t="inlineStr"/>
@@ -28010,7 +28010,7 @@
         </is>
       </c>
       <c r="I50" s="61" t="n">
-        <v>0.00424979</v>
+        <v>0.00423056</v>
       </c>
       <c r="J50" s="6" t="inlineStr">
         <is>
@@ -28035,7 +28035,7 @@
         </is>
       </c>
       <c r="I51" s="61" t="n">
-        <v>0.00261124</v>
+        <v>0.00264098</v>
       </c>
       <c r="J51" s="6" t="inlineStr">
         <is>
@@ -28060,7 +28060,7 @@
         </is>
       </c>
       <c r="I52" s="61" t="n">
-        <v>0.00250636</v>
+        <v>0.00251603</v>
       </c>
       <c r="J52" s="6" t="inlineStr">
         <is>
@@ -28085,7 +28085,7 @@
         </is>
       </c>
       <c r="I53" s="61" t="n">
-        <v>0.00249401</v>
+        <v>0.00250354</v>
       </c>
       <c r="J53" s="6" t="inlineStr">
         <is>
@@ -28110,7 +28110,7 @@
         </is>
       </c>
       <c r="I54" s="61" t="n">
-        <v>0.00219085</v>
+        <v>0.00219483</v>
       </c>
       <c r="J54" s="6" t="inlineStr">
         <is>
@@ -28135,7 +28135,7 @@
         </is>
       </c>
       <c r="I55" s="61" t="n">
-        <v>0.00214161</v>
+        <v>0.00216782</v>
       </c>
       <c r="J55" s="6" t="inlineStr">
         <is>
@@ -28160,7 +28160,7 @@
         </is>
       </c>
       <c r="I56" s="61" t="n">
-        <v>0.00199168</v>
+        <v>0.00200789</v>
       </c>
       <c r="J56" s="6" t="inlineStr">
         <is>
@@ -28185,7 +28185,7 @@
         </is>
       </c>
       <c r="I57" s="61" t="n">
-        <v>0.00189993</v>
+        <v>0.00187926</v>
       </c>
       <c r="J57" s="6" t="inlineStr">
         <is>
@@ -28210,7 +28210,7 @@
         </is>
       </c>
       <c r="I58" s="61" t="n">
-        <v>0.00154497</v>
+        <v>0.00153483</v>
       </c>
       <c r="J58" s="6" t="inlineStr">
         <is>
@@ -28235,7 +28235,7 @@
         </is>
       </c>
       <c r="I59" s="61" t="n">
-        <v>0.00149545</v>
+        <v>0.00149806</v>
       </c>
       <c r="J59" s="6" t="inlineStr">
         <is>
@@ -28260,7 +28260,7 @@
         </is>
       </c>
       <c r="I60" s="61" t="n">
-        <v>0.00144259</v>
+        <v>0.00148054</v>
       </c>
       <c r="J60" s="6" t="inlineStr">
         <is>
@@ -28285,7 +28285,7 @@
         </is>
       </c>
       <c r="I61" s="61" t="n">
-        <v>0.00141312</v>
+        <v>0.0014101</v>
       </c>
       <c r="J61" s="6" t="inlineStr">
         <is>
@@ -28310,7 +28310,7 @@
         </is>
       </c>
       <c r="I62" s="61" t="n">
-        <v>0.00131177</v>
+        <v>0.00127473</v>
       </c>
       <c r="J62" s="6" t="inlineStr">
         <is>
@@ -28331,20 +28331,20 @@
     <row r="63">
       <c r="H63" s="6" t="inlineStr">
         <is>
-          <t>NXST</t>
+          <t>OZK</t>
         </is>
       </c>
       <c r="I63" s="61" t="n">
-        <v>0.00119145</v>
+        <v>0.00118818</v>
       </c>
       <c r="J63" s="6" t="inlineStr">
         <is>
-          <t>NEXSTAR MEDIA GROUP INC</t>
+          <t>BANK OZK</t>
         </is>
       </c>
       <c r="K63" s="6" t="inlineStr">
         <is>
-          <t>Communication Services</t>
+          <t>Financials</t>
         </is>
       </c>
       <c r="L63" s="6" t="inlineStr"/>
@@ -28356,20 +28356,20 @@
     <row r="64">
       <c r="H64" s="6" t="inlineStr">
         <is>
-          <t>OZK</t>
+          <t>NXST</t>
         </is>
       </c>
       <c r="I64" s="61" t="n">
-        <v>0.00113949</v>
+        <v>0.00116287</v>
       </c>
       <c r="J64" s="6" t="inlineStr">
         <is>
-          <t>BANK OZK</t>
+          <t>NEXSTAR MEDIA GROUP INC</t>
         </is>
       </c>
       <c r="K64" s="6" t="inlineStr">
         <is>
-          <t>Financials</t>
+          <t>Communication Services</t>
         </is>
       </c>
       <c r="L64" s="6" t="inlineStr"/>
@@ -28385,7 +28385,7 @@
         </is>
       </c>
       <c r="I65" s="61" t="n">
-        <v>0.00096997</v>
+        <v>0.0009725399999999999</v>
       </c>
       <c r="J65" s="6" t="inlineStr">
         <is>
@@ -28410,7 +28410,7 @@
         </is>
       </c>
       <c r="I66" s="61" t="n">
-        <v>0.00096707</v>
+        <v>0.00095373</v>
       </c>
       <c r="J66" s="6" t="inlineStr">
         <is>
@@ -28431,20 +28431,20 @@
     <row r="67">
       <c r="H67" s="6" t="inlineStr">
         <is>
-          <t>PAG</t>
+          <t>CWEN</t>
         </is>
       </c>
       <c r="I67" s="61" t="n">
-        <v>0.0009162900000000001</v>
+        <v>0.00092919</v>
       </c>
       <c r="J67" s="6" t="inlineStr">
         <is>
-          <t>PENSKE AUTOMOTIVE GROUP VOTING INC</t>
+          <t>CLEARWAY ENERGY INC CLASS C</t>
         </is>
       </c>
       <c r="K67" s="6" t="inlineStr">
         <is>
-          <t>Consumer Discretionary</t>
+          <t>Utilities</t>
         </is>
       </c>
       <c r="L67" s="6" t="inlineStr"/>
@@ -28456,20 +28456,20 @@
     <row r="68">
       <c r="H68" s="6" t="inlineStr">
         <is>
-          <t>KFY</t>
+          <t>PAG</t>
         </is>
       </c>
       <c r="I68" s="61" t="n">
-        <v>0.0009137699999999999</v>
+        <v>0.00091621</v>
       </c>
       <c r="J68" s="6" t="inlineStr">
         <is>
-          <t>KORN FERRY</t>
+          <t>PENSKE AUTOMOTIVE GROUP VOTING INC</t>
         </is>
       </c>
       <c r="K68" s="6" t="inlineStr">
         <is>
-          <t>Industrials</t>
+          <t>Consumer Discretionary</t>
         </is>
       </c>
       <c r="L68" s="6" t="inlineStr"/>
@@ -28481,20 +28481,20 @@
     <row r="69">
       <c r="H69" s="6" t="inlineStr">
         <is>
-          <t>CVBF</t>
+          <t>KFY</t>
         </is>
       </c>
       <c r="I69" s="61" t="n">
-        <v>0.00089821</v>
+        <v>0.0009149500000000001</v>
       </c>
       <c r="J69" s="6" t="inlineStr">
         <is>
-          <t>CVB FINANCIAL CORP</t>
+          <t>KORN FERRY</t>
         </is>
       </c>
       <c r="K69" s="6" t="inlineStr">
         <is>
-          <t>Financials</t>
+          <t>Industrials</t>
         </is>
       </c>
       <c r="L69" s="6" t="inlineStr"/>
@@ -28506,20 +28506,20 @@
     <row r="70">
       <c r="H70" s="6" t="inlineStr">
         <is>
-          <t>CWEN</t>
+          <t>CVBF</t>
         </is>
       </c>
       <c r="I70" s="61" t="n">
-        <v>0.00088813</v>
+        <v>0.00090226</v>
       </c>
       <c r="J70" s="6" t="inlineStr">
         <is>
-          <t>CLEARWAY ENERGY INC CLASS C</t>
+          <t>CVB FINANCIAL CORP</t>
         </is>
       </c>
       <c r="K70" s="6" t="inlineStr">
         <is>
-          <t>Utilities</t>
+          <t>Financials</t>
         </is>
       </c>
       <c r="L70" s="6" t="inlineStr"/>
@@ -28535,7 +28535,7 @@
         </is>
       </c>
       <c r="I71" s="61" t="n">
-        <v>0.00082553</v>
+        <v>0.00084555</v>
       </c>
       <c r="J71" s="6" t="inlineStr">
         <is>
@@ -28560,7 +28560,7 @@
         </is>
       </c>
       <c r="I72" s="61" t="n">
-        <v>0.0005663</v>
+        <v>0.00056972</v>
       </c>
       <c r="J72" s="6" t="inlineStr">
         <is>
@@ -28585,7 +28585,7 @@
         </is>
       </c>
       <c r="I73" s="61" t="n">
-        <v>0.00056032</v>
+        <v>0.0005598199999999999</v>
       </c>
       <c r="J73" s="6" t="inlineStr">
         <is>
@@ -28610,7 +28610,7 @@
         </is>
       </c>
       <c r="I74" s="61" t="n">
-        <v>0.0005444299999999999</v>
+        <v>0.0005196900000000001</v>
       </c>
       <c r="J74" s="6" t="inlineStr">
         <is>
@@ -28635,7 +28635,7 @@
         </is>
       </c>
       <c r="I75" s="61" t="n">
-        <v>0.00051459</v>
+        <v>0.00050302</v>
       </c>
       <c r="J75" s="6" t="inlineStr">
         <is>
@@ -28660,7 +28660,7 @@
         </is>
       </c>
       <c r="I76" s="61" t="n">
-        <v>0.00050215</v>
+        <v>0.00049936</v>
       </c>
       <c r="J76" s="6" t="inlineStr">
         <is>
@@ -28685,7 +28685,7 @@
         </is>
       </c>
       <c r="I77" s="61" t="n">
-        <v>0.00049549</v>
+        <v>0.00048373</v>
       </c>
       <c r="J77" s="6" t="inlineStr">
         <is>
@@ -28710,7 +28710,7 @@
         </is>
       </c>
       <c r="I78" s="61" t="n">
-        <v>0.00048529</v>
+        <v>0.0004815</v>
       </c>
       <c r="J78" s="6" t="inlineStr">
         <is>
@@ -28735,7 +28735,7 @@
         </is>
       </c>
       <c r="I79" s="61" t="n">
-        <v>0.00047208</v>
+        <v>0.00047554</v>
       </c>
       <c r="J79" s="6" t="inlineStr">
         <is>
@@ -28760,7 +28760,7 @@
         </is>
       </c>
       <c r="I80" s="61" t="n">
-        <v>0.00046119</v>
+        <v>0.00045774</v>
       </c>
       <c r="J80" s="6" t="inlineStr">
         <is>
@@ -28785,7 +28785,7 @@
         </is>
       </c>
       <c r="I81" s="61" t="n">
-        <v>0.00045641</v>
+        <v>0.00045368</v>
       </c>
       <c r="J81" s="6" t="inlineStr">
         <is>
@@ -28810,7 +28810,7 @@
         </is>
       </c>
       <c r="I82" s="61" t="n">
-        <v>0.00043535</v>
+        <v>0.00043713</v>
       </c>
       <c r="J82" s="6" t="inlineStr">
         <is>
@@ -28835,7 +28835,7 @@
         </is>
       </c>
       <c r="I83" s="61" t="n">
-        <v>0.00042315</v>
+        <v>0.00042025</v>
       </c>
       <c r="J83" s="6" t="inlineStr">
         <is>
@@ -28856,22 +28856,18 @@
     <row r="84">
       <c r="H84" s="6" t="inlineStr">
         <is>
-          <t>NBHC</t>
+          <t>GVMXX</t>
         </is>
       </c>
       <c r="I84" s="61" t="n">
-        <v>0.00041123</v>
+        <v>0.00041188</v>
       </c>
       <c r="J84" s="6" t="inlineStr">
         <is>
-          <t>NATIONAL BANK HOLDINGS CORP CLASS</t>
-        </is>
-      </c>
-      <c r="K84" s="6" t="inlineStr">
-        <is>
-          <t>Financials</t>
-        </is>
-      </c>
+          <t>SSC GOVERNMENT MM GVMXX</t>
+        </is>
+      </c>
+      <c r="K84" s="6" t="inlineStr"/>
       <c r="L84" s="6" t="inlineStr"/>
       <c r="M84" s="7">
         <f>IF(H84="","",IFERROR(VLOOKUP(K84,$P$5:$Q$15,2,FALSE),"현금·선물"))</f>
@@ -28881,18 +28877,22 @@
     <row r="85">
       <c r="H85" s="6" t="inlineStr">
         <is>
-          <t>GVMXX</t>
+          <t>NBHC</t>
         </is>
       </c>
       <c r="I85" s="61" t="n">
-        <v>0.00038781</v>
+        <v>0.00041158</v>
       </c>
       <c r="J85" s="6" t="inlineStr">
         <is>
-          <t>SSC GOVERNMENT MM GVMXX</t>
-        </is>
-      </c>
-      <c r="K85" s="6" t="inlineStr"/>
+          <t>NATIONAL BANK HOLDINGS CORP CLASS</t>
+        </is>
+      </c>
+      <c r="K85" s="6" t="inlineStr">
+        <is>
+          <t>Financials</t>
+        </is>
+      </c>
       <c r="L85" s="6" t="inlineStr"/>
       <c r="M85" s="7">
         <f>IF(H85="","",IFERROR(VLOOKUP(K85,$P$5:$Q$15,2,FALSE),"현금·선물"))</f>
@@ -28906,7 +28906,7 @@
         </is>
       </c>
       <c r="I86" s="61" t="n">
-        <v>0.00037497</v>
+        <v>0.00037281</v>
       </c>
       <c r="J86" s="6" t="inlineStr">
         <is>
@@ -28931,7 +28931,7 @@
         </is>
       </c>
       <c r="I87" s="61" t="n">
-        <v>0.00035496</v>
+        <v>0.00035181</v>
       </c>
       <c r="J87" s="6" t="inlineStr">
         <is>
@@ -28956,7 +28956,7 @@
         </is>
       </c>
       <c r="I88" s="61" t="n">
-        <v>0.00034819</v>
+        <v>0.00034437</v>
       </c>
       <c r="J88" s="6" t="inlineStr">
         <is>
@@ -28981,7 +28981,7 @@
         </is>
       </c>
       <c r="I89" s="61" t="n">
-        <v>0.00030963</v>
+        <v>0.00030009</v>
       </c>
       <c r="J89" s="6" t="inlineStr">
         <is>
@@ -29006,7 +29006,7 @@
         </is>
       </c>
       <c r="I90" s="61" t="n">
-        <v>0.00027876</v>
+        <v>0.00027976</v>
       </c>
       <c r="J90" s="6" t="inlineStr">
         <is>
@@ -29031,7 +29031,7 @@
         </is>
       </c>
       <c r="I91" s="61" t="n">
-        <v>0.00025555</v>
+        <v>0.00025535</v>
       </c>
       <c r="J91" s="6" t="inlineStr">
         <is>
@@ -29056,7 +29056,7 @@
         </is>
       </c>
       <c r="I92" s="61" t="n">
-        <v>0.00025473</v>
+        <v>0.00024557</v>
       </c>
       <c r="J92" s="6" t="inlineStr">
         <is>
@@ -29081,7 +29081,7 @@
         </is>
       </c>
       <c r="I93" s="61" t="n">
-        <v>0.00022989</v>
+        <v>0.00023034</v>
       </c>
       <c r="J93" s="6" t="inlineStr">
         <is>
@@ -29106,7 +29106,7 @@
         </is>
       </c>
       <c r="I94" s="61" t="n">
-        <v>0.00022572</v>
+        <v>0.00022613</v>
       </c>
       <c r="J94" s="6" t="inlineStr">
         <is>
@@ -29131,7 +29131,7 @@
         </is>
       </c>
       <c r="I95" s="61" t="n">
-        <v>0.00020398</v>
+        <v>0.00020799</v>
       </c>
       <c r="J95" s="6" t="inlineStr">
         <is>
@@ -29156,7 +29156,7 @@
         </is>
       </c>
       <c r="I96" s="61" t="n">
-        <v>0.00019656</v>
+        <v>0.00019489</v>
       </c>
       <c r="J96" s="6" t="inlineStr">
         <is>
@@ -29181,7 +29181,7 @@
         </is>
       </c>
       <c r="I97" s="61" t="n">
-        <v>0.00019476</v>
+        <v>0.00019378</v>
       </c>
       <c r="J97" s="6" t="inlineStr">
         <is>
@@ -29206,7 +29206,7 @@
         </is>
       </c>
       <c r="I98" s="61" t="n">
-        <v>0.00017857</v>
+        <v>0.00017768</v>
       </c>
       <c r="J98" s="6" t="inlineStr">
         <is>
@@ -29231,7 +29231,7 @@
         </is>
       </c>
       <c r="I99" s="61" t="n">
-        <v>0.00016453</v>
+        <v>0.00016509</v>
       </c>
       <c r="J99" s="6" t="inlineStr">
         <is>
@@ -29252,22 +29252,18 @@
     <row r="100">
       <c r="H100" s="6" t="inlineStr">
         <is>
-          <t>EBF</t>
+          <t>USD</t>
         </is>
       </c>
       <c r="I100" s="61" t="n">
-        <v>0.00013087</v>
+        <v>0.00013204</v>
       </c>
       <c r="J100" s="6" t="inlineStr">
         <is>
-          <t>ENNIS INC</t>
-        </is>
-      </c>
-      <c r="K100" s="6" t="inlineStr">
-        <is>
-          <t>Industrials</t>
-        </is>
-      </c>
+          <t>US DOLLAR</t>
+        </is>
+      </c>
+      <c r="K100" s="6" t="inlineStr"/>
       <c r="L100" s="6" t="inlineStr"/>
       <c r="M100" s="7">
         <f>IF(H100="","",IFERROR(VLOOKUP(K100,$P$5:$Q$15,2,FALSE),"현금·선물"))</f>
@@ -29277,18 +29273,22 @@
     <row r="101">
       <c r="H101" s="6" t="inlineStr">
         <is>
-          <t>USD</t>
+          <t>EBF</t>
         </is>
       </c>
       <c r="I101" s="61" t="n">
-        <v>0.00013085</v>
+        <v>0.00013122</v>
       </c>
       <c r="J101" s="6" t="inlineStr">
         <is>
-          <t>US DOLLAR</t>
-        </is>
-      </c>
-      <c r="K101" s="6" t="inlineStr"/>
+          <t>ENNIS INC</t>
+        </is>
+      </c>
+      <c r="K101" s="6" t="inlineStr">
+        <is>
+          <t>Industrials</t>
+        </is>
+      </c>
       <c r="L101" s="6" t="inlineStr"/>
       <c r="M101" s="7">
         <f>IF(H101="","",IFERROR(VLOOKUP(K101,$P$5:$Q$15,2,FALSE),"현금·선물"))</f>
@@ -29302,7 +29302,7 @@
         </is>
       </c>
       <c r="I102" s="61" t="n">
-        <v>0.00011431</v>
+        <v>0.00011517</v>
       </c>
       <c r="J102" s="6" t="inlineStr">
         <is>
@@ -29327,7 +29327,7 @@
         </is>
       </c>
       <c r="I103" s="61" t="n">
-        <v>9.802999999999999e-05</v>
+        <v>9.625999999999999e-05</v>
       </c>
       <c r="J103" s="6" t="inlineStr">
         <is>
@@ -29352,7 +29352,7 @@
         </is>
       </c>
       <c r="I104" s="61" t="n">
-        <v>9.091e-05</v>
+        <v>8.805e-05</v>
       </c>
       <c r="J104" s="6" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
데이터 갱신: holdings (2026-10-23)
</commit_message>
<xml_diff>
--- a/downloads/schd_dividend_tracker.xlsx
+++ b/downloads/schd_dividend_tracker.xlsx
@@ -1724,7 +1724,7 @@
     <row r="3">
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>최종 갱신: 2026-10-22 · 반영 범위: 2012년 1분기 ~ 2026년 3분기 (배당락 2026-09-23) · GitHub Actions 자동 생성</t>
+          <t>최종 갱신: 2026-10-23 · 반영 범위: 2012년 1분기 ~ 2026년 3분기 (배당락 2026-09-23) · GitHub Actions 자동 생성</t>
         </is>
       </c>
     </row>
@@ -26257,11 +26257,11 @@
         </is>
       </c>
       <c r="B2" s="49" t="n">
-        <v>46316</v>
+        <v>46317</v>
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>← 이 날 종가로 계산한 비중. 그날 공식 파일을 못 받아 Schwab 공식 보유종목 CSV(2026-10-20)의 보유 주식 수 × 종가로 계산했습니다.</t>
+          <t>← 이 날 종가로 계산한 비중. 그날 공식 파일을 못 받아 Schwab 공식 보유종목 CSV(2026-10-21)의 보유 주식 수 × 종가로 계산했습니다.</t>
         </is>
       </c>
     </row>
@@ -26354,25 +26354,25 @@
       </c>
       <c r="H5" s="6" t="inlineStr">
         <is>
-          <t>TXN</t>
+          <t>PG</t>
         </is>
       </c>
       <c r="I5" s="61" t="n">
-        <v>0.04485776</v>
+        <v>0.0440797</v>
       </c>
       <c r="J5" s="6" t="inlineStr">
         <is>
-          <t>TEXAS INSTRUMENT</t>
+          <t>PROCTER &amp; GAMBLE</t>
         </is>
       </c>
       <c r="K5" s="6" t="inlineStr">
         <is>
-          <t>Information Technology</t>
+          <t>Consumer Staples</t>
         </is>
       </c>
       <c r="L5" s="6" t="inlineStr">
         <is>
-          <t>텍사스 인스트루먼트</t>
+          <t>프록터앤드갬블</t>
         </is>
       </c>
       <c r="M5" s="7">
@@ -26412,25 +26412,25 @@
       </c>
       <c r="H6" s="6" t="inlineStr">
         <is>
-          <t>CVX</t>
+          <t>TXN</t>
         </is>
       </c>
       <c r="I6" s="61" t="n">
-        <v>0.04299757</v>
+        <v>0.04311106</v>
       </c>
       <c r="J6" s="6" t="inlineStr">
         <is>
-          <t>CHEVRON</t>
+          <t>TEXAS INSTRUMENT</t>
         </is>
       </c>
       <c r="K6" s="6" t="inlineStr">
         <is>
-          <t>Energy</t>
+          <t>Information Technology</t>
         </is>
       </c>
       <c r="L6" s="6" t="inlineStr">
         <is>
-          <t>셰브론</t>
+          <t>텍사스 인스트루먼트</t>
         </is>
       </c>
       <c r="M6" s="7">
@@ -26470,15 +26470,15 @@
       </c>
       <c r="H7" s="6" t="inlineStr">
         <is>
-          <t>PG</t>
+          <t>KO</t>
         </is>
       </c>
       <c r="I7" s="61" t="n">
-        <v>0.042656</v>
+        <v>0.04246364</v>
       </c>
       <c r="J7" s="6" t="inlineStr">
         <is>
-          <t>PROCTER &amp; GAMBLE</t>
+          <t>COCA-COLA</t>
         </is>
       </c>
       <c r="K7" s="6" t="inlineStr">
@@ -26488,7 +26488,7 @@
       </c>
       <c r="L7" s="6" t="inlineStr">
         <is>
-          <t>프록터앤드갬블</t>
+          <t>코카콜라</t>
         </is>
       </c>
       <c r="M7" s="7">
@@ -26528,15 +26528,15 @@
       </c>
       <c r="H8" s="6" t="inlineStr">
         <is>
-          <t>COP</t>
+          <t>CVX</t>
         </is>
       </c>
       <c r="I8" s="61" t="n">
-        <v>0.04257815</v>
+        <v>0.04206611</v>
       </c>
       <c r="J8" s="6" t="inlineStr">
         <is>
-          <t>CONOCOPHILLIPS</t>
+          <t>CHEVRON</t>
         </is>
       </c>
       <c r="K8" s="6" t="inlineStr">
@@ -26546,7 +26546,7 @@
       </c>
       <c r="L8" s="6" t="inlineStr">
         <is>
-          <t>코노코필립스</t>
+          <t>셰브론</t>
         </is>
       </c>
       <c r="M8" s="7">
@@ -26586,25 +26586,25 @@
       </c>
       <c r="H9" s="6" t="inlineStr">
         <is>
-          <t>KO</t>
+          <t>UNH</t>
         </is>
       </c>
       <c r="I9" s="61" t="n">
-        <v>0.04217424</v>
+        <v>0.04179048</v>
       </c>
       <c r="J9" s="6" t="inlineStr">
         <is>
-          <t>COCA-COLA</t>
+          <t>UNITEDHEALTH GROUP</t>
         </is>
       </c>
       <c r="K9" s="6" t="inlineStr">
         <is>
-          <t>Consumer Staples</t>
+          <t>Health Care</t>
         </is>
       </c>
       <c r="L9" s="6" t="inlineStr">
         <is>
-          <t>코카콜라</t>
+          <t>유나이티드헬스</t>
         </is>
       </c>
       <c r="M9" s="7">
@@ -26644,25 +26644,25 @@
       </c>
       <c r="H10" s="6" t="inlineStr">
         <is>
-          <t>QCOM</t>
+          <t>COP</t>
         </is>
       </c>
       <c r="I10" s="61" t="n">
-        <v>0.04204388</v>
+        <v>0.04166280000000001</v>
       </c>
       <c r="J10" s="6" t="inlineStr">
         <is>
-          <t>QUALCOMM</t>
+          <t>CONOCOPHILLIPS</t>
         </is>
       </c>
       <c r="K10" s="6" t="inlineStr">
         <is>
-          <t>Information Technology</t>
+          <t>Energy</t>
         </is>
       </c>
       <c r="L10" s="6" t="inlineStr">
         <is>
-          <t>퀄컴</t>
+          <t>코노코필립스</t>
         </is>
       </c>
       <c r="M10" s="7">
@@ -26702,25 +26702,25 @@
       </c>
       <c r="H11" s="6" t="inlineStr">
         <is>
-          <t>UNH</t>
+          <t>HD</t>
         </is>
       </c>
       <c r="I11" s="61" t="n">
-        <v>0.04189536999999999</v>
+        <v>0.04043819</v>
       </c>
       <c r="J11" s="6" t="inlineStr">
         <is>
-          <t>UNITEDHEALTH GROUP</t>
+          <t>HOME DEPOT</t>
         </is>
       </c>
       <c r="K11" s="6" t="inlineStr">
         <is>
-          <t>Health Care</t>
+          <t>Consumer Discretionary</t>
         </is>
       </c>
       <c r="L11" s="6" t="inlineStr">
         <is>
-          <t>유나이티드헬스</t>
+          <t>홈디포</t>
         </is>
       </c>
       <c r="M11" s="7">
@@ -26760,25 +26760,25 @@
       </c>
       <c r="H12" s="6" t="inlineStr">
         <is>
-          <t>AMGN</t>
+          <t>QCOM</t>
         </is>
       </c>
       <c r="I12" s="61" t="n">
-        <v>0.03974505</v>
+        <v>0.03996504</v>
       </c>
       <c r="J12" s="6" t="inlineStr">
         <is>
-          <t>AMGEN INC</t>
+          <t>QUALCOMM</t>
         </is>
       </c>
       <c r="K12" s="6" t="inlineStr">
         <is>
-          <t>Health Care</t>
+          <t>Information Technology</t>
         </is>
       </c>
       <c r="L12" s="6" t="inlineStr">
         <is>
-          <t>암젠</t>
+          <t>퀄컴</t>
         </is>
       </c>
       <c r="M12" s="7">
@@ -26818,15 +26818,15 @@
       </c>
       <c r="H13" s="6" t="inlineStr">
         <is>
-          <t>MRK</t>
+          <t>AMGN</t>
         </is>
       </c>
       <c r="I13" s="61" t="n">
-        <v>0.03968767</v>
+        <v>0.03969446</v>
       </c>
       <c r="J13" s="6" t="inlineStr">
         <is>
-          <t>MERCK &amp; CO INC</t>
+          <t>AMGEN INC</t>
         </is>
       </c>
       <c r="K13" s="6" t="inlineStr">
@@ -26836,7 +26836,7 @@
       </c>
       <c r="L13" s="6" t="inlineStr">
         <is>
-          <t>머크</t>
+          <t>암젠</t>
         </is>
       </c>
       <c r="M13" s="7">
@@ -26876,25 +26876,25 @@
       </c>
       <c r="H14" s="6" t="inlineStr">
         <is>
-          <t>HD</t>
+          <t>PEP</t>
         </is>
       </c>
       <c r="I14" s="61" t="n">
-        <v>0.03960226</v>
+        <v>0.03882847</v>
       </c>
       <c r="J14" s="6" t="inlineStr">
         <is>
-          <t>HOME DEPOT</t>
+          <t>PEPSICO</t>
         </is>
       </c>
       <c r="K14" s="6" t="inlineStr">
         <is>
-          <t>Consumer Discretionary</t>
+          <t>Consumer Staples</t>
         </is>
       </c>
       <c r="L14" s="6" t="inlineStr">
         <is>
-          <t>홈디포</t>
+          <t>펩시코</t>
         </is>
       </c>
       <c r="M14" s="7">
@@ -26924,25 +26924,25 @@
       </c>
       <c r="H15" s="6" t="inlineStr">
         <is>
-          <t>PEP</t>
+          <t>MRK</t>
         </is>
       </c>
       <c r="I15" s="61" t="n">
-        <v>0.03849057</v>
+        <v>0.03816085</v>
       </c>
       <c r="J15" s="6" t="inlineStr">
         <is>
-          <t>PEPSICO</t>
+          <t>MERCK &amp; CO INC</t>
         </is>
       </c>
       <c r="K15" s="6" t="inlineStr">
         <is>
-          <t>Consumer Staples</t>
+          <t>Health Care</t>
         </is>
       </c>
       <c r="L15" s="6" t="inlineStr">
         <is>
-          <t>펩시코</t>
+          <t>머크</t>
         </is>
       </c>
       <c r="M15" s="7">
@@ -26972,25 +26972,25 @@
       </c>
       <c r="H16" s="6" t="inlineStr">
         <is>
-          <t>ABT</t>
+          <t>ACN</t>
         </is>
       </c>
       <c r="I16" s="61" t="n">
-        <v>0.03653357</v>
+        <v>0.03770554</v>
       </c>
       <c r="J16" s="6" t="inlineStr">
         <is>
-          <t>ABBOTT LABORATORIES</t>
+          <t>ACCENTURE PLC CLASS A</t>
         </is>
       </c>
       <c r="K16" s="6" t="inlineStr">
         <is>
-          <t>Health Care</t>
+          <t>Information Technology</t>
         </is>
       </c>
       <c r="L16" s="6" t="inlineStr">
         <is>
-          <t>애보트</t>
+          <t>액센츄어</t>
         </is>
       </c>
       <c r="M16" s="7">
@@ -27010,25 +27010,25 @@
       </c>
       <c r="H17" s="6" t="inlineStr">
         <is>
-          <t>ACN</t>
+          <t>ABT</t>
         </is>
       </c>
       <c r="I17" s="61" t="n">
-        <v>0.03577195</v>
+        <v>0.03646952000000001</v>
       </c>
       <c r="J17" s="6" t="inlineStr">
         <is>
-          <t>ACCENTURE PLC CLASS A</t>
+          <t>ABBOTT LABORATORIES</t>
         </is>
       </c>
       <c r="K17" s="6" t="inlineStr">
         <is>
-          <t>Information Technology</t>
+          <t>Health Care</t>
         </is>
       </c>
       <c r="L17" s="6" t="inlineStr">
         <is>
-          <t>액센츄어</t>
+          <t>애보트</t>
         </is>
       </c>
       <c r="M17" s="7">
@@ -27052,7 +27052,7 @@
         </is>
       </c>
       <c r="I18" s="61" t="n">
-        <v>0.03482887</v>
+        <v>0.03537294</v>
       </c>
       <c r="J18" s="6" t="inlineStr">
         <is>
@@ -27081,7 +27081,7 @@
         </is>
       </c>
       <c r="I19" s="61" t="n">
-        <v>0.03037695</v>
+        <v>0.03064662</v>
       </c>
       <c r="J19" s="6" t="inlineStr">
         <is>
@@ -27115,7 +27115,7 @@
         </is>
       </c>
       <c r="I20" s="61" t="n">
-        <v>0.02999405</v>
+        <v>0.03024801</v>
       </c>
       <c r="J20" s="6" t="inlineStr">
         <is>
@@ -27154,7 +27154,7 @@
         </is>
       </c>
       <c r="I21" s="61" t="n">
-        <v>0.02846511</v>
+        <v>0.0291323</v>
       </c>
       <c r="J21" s="6" t="inlineStr">
         <is>
@@ -27192,7 +27192,7 @@
         </is>
       </c>
       <c r="I22" s="61" t="n">
-        <v>0.02725198</v>
+        <v>0.02853046</v>
       </c>
       <c r="J22" s="6" t="inlineStr">
         <is>
@@ -27226,25 +27226,25 @@
       </c>
       <c r="H23" s="6" t="inlineStr">
         <is>
-          <t>EOG</t>
+          <t>BX</t>
         </is>
       </c>
       <c r="I23" s="61" t="n">
-        <v>0.02014859</v>
+        <v>0.02122686</v>
       </c>
       <c r="J23" s="6" t="inlineStr">
         <is>
-          <t>EOG RESOURCES</t>
+          <t>BLACKSTONE</t>
         </is>
       </c>
       <c r="K23" s="6" t="inlineStr">
         <is>
-          <t>Energy</t>
+          <t>Financials</t>
         </is>
       </c>
       <c r="L23" s="6" t="inlineStr">
         <is>
-          <t>EOG 리소시스</t>
+          <t>블랙스톤</t>
         </is>
       </c>
       <c r="M23" s="7">
@@ -27264,25 +27264,25 @@
       </c>
       <c r="H24" s="6" t="inlineStr">
         <is>
-          <t>BX</t>
+          <t>EOG</t>
         </is>
       </c>
       <c r="I24" s="61" t="n">
-        <v>0.02001077</v>
+        <v>0.01973078</v>
       </c>
       <c r="J24" s="6" t="inlineStr">
         <is>
-          <t>BLACKSTONE</t>
+          <t>EOG RESOURCES</t>
         </is>
       </c>
       <c r="K24" s="6" t="inlineStr">
         <is>
-          <t>Financials</t>
+          <t>Energy</t>
         </is>
       </c>
       <c r="L24" s="6" t="inlineStr">
         <is>
-          <t>블랙스톤</t>
+          <t>EOG 리소시스</t>
         </is>
       </c>
       <c r="M24" s="7">
@@ -27306,7 +27306,7 @@
         </is>
       </c>
       <c r="I25" s="61" t="n">
-        <v>0.01901324</v>
+        <v>0.01925016</v>
       </c>
       <c r="J25" s="6" t="inlineStr">
         <is>
@@ -27340,25 +27340,25 @@
       </c>
       <c r="H26" s="6" t="inlineStr">
         <is>
-          <t>SLB</t>
+          <t>UPS</t>
         </is>
       </c>
       <c r="I26" s="61" t="n">
-        <v>0.01845224</v>
+        <v>0.01811623</v>
       </c>
       <c r="J26" s="6" t="inlineStr">
         <is>
-          <t>SLB</t>
+          <t>UNITED PARCEL SERVICE INC CLASS B</t>
         </is>
       </c>
       <c r="K26" s="6" t="inlineStr">
         <is>
-          <t>Energy</t>
+          <t>Industrials</t>
         </is>
       </c>
       <c r="L26" s="6" t="inlineStr">
         <is>
-          <t>SLB</t>
+          <t>UPS</t>
         </is>
       </c>
       <c r="M26" s="7">
@@ -27378,25 +27378,25 @@
       </c>
       <c r="H27" s="6" t="inlineStr">
         <is>
-          <t>UPS</t>
+          <t>SLB</t>
         </is>
       </c>
       <c r="I27" s="61" t="n">
-        <v>0.01815364</v>
+        <v>0.01751269</v>
       </c>
       <c r="J27" s="6" t="inlineStr">
         <is>
-          <t>UNITED PARCEL SERVICE INC CLASS B</t>
+          <t>SLB</t>
         </is>
       </c>
       <c r="K27" s="6" t="inlineStr">
         <is>
-          <t>Industrials</t>
+          <t>Energy</t>
         </is>
       </c>
       <c r="L27" s="6" t="inlineStr">
         <is>
-          <t>UPS</t>
+          <t>SLB</t>
         </is>
       </c>
       <c r="M27" s="7">
@@ -27420,7 +27420,7 @@
         </is>
       </c>
       <c r="I28" s="61" t="n">
-        <v>0.01683904</v>
+        <v>0.01710133</v>
       </c>
       <c r="J28" s="6" t="inlineStr">
         <is>
@@ -27458,7 +27458,7 @@
         </is>
       </c>
       <c r="I29" s="61" t="n">
-        <v>0.0146548</v>
+        <v>0.01440925</v>
       </c>
       <c r="J29" s="6" t="inlineStr">
         <is>
@@ -27496,7 +27496,7 @@
         </is>
       </c>
       <c r="I30" s="61" t="n">
-        <v>0.01428201</v>
+        <v>0.01409591</v>
       </c>
       <c r="J30" s="6" t="inlineStr">
         <is>
@@ -27530,7 +27530,7 @@
         </is>
       </c>
       <c r="I31" s="61" t="n">
-        <v>0.01334698</v>
+        <v>0.01288287</v>
       </c>
       <c r="J31" s="6" t="inlineStr">
         <is>
@@ -27555,7 +27555,7 @@
         </is>
       </c>
       <c r="I32" s="61" t="n">
-        <v>0.01165263</v>
+        <v>0.01149595</v>
       </c>
       <c r="J32" s="6" t="inlineStr">
         <is>
@@ -27585,7 +27585,7 @@
         </is>
       </c>
       <c r="I33" s="61" t="n">
-        <v>0.01134031</v>
+        <v>0.01113688</v>
       </c>
       <c r="J33" s="6" t="inlineStr">
         <is>
@@ -27610,7 +27610,7 @@
         </is>
       </c>
       <c r="I34" s="61" t="n">
-        <v>0.009305909999999999</v>
+        <v>0.00916341</v>
       </c>
       <c r="J34" s="6" t="inlineStr">
         <is>
@@ -27635,7 +27635,7 @@
         </is>
       </c>
       <c r="I35" s="61" t="n">
-        <v>0.008761970000000001</v>
+        <v>0.009056920000000001</v>
       </c>
       <c r="J35" s="6" t="inlineStr">
         <is>
@@ -27660,7 +27660,7 @@
         </is>
       </c>
       <c r="I36" s="61" t="n">
-        <v>0.00862889</v>
+        <v>0.008895480000000001</v>
       </c>
       <c r="J36" s="6" t="inlineStr">
         <is>
@@ -27681,15 +27681,15 @@
     <row r="37">
       <c r="H37" s="6" t="inlineStr">
         <is>
-          <t>CINF</t>
+          <t>ARES</t>
         </is>
       </c>
       <c r="I37" s="61" t="n">
-        <v>0.00648346</v>
+        <v>0.00659729</v>
       </c>
       <c r="J37" s="6" t="inlineStr">
         <is>
-          <t>CINCINNATI FINANCIAL</t>
+          <t>ARES MANAGEMENT CLASS A</t>
         </is>
       </c>
       <c r="K37" s="6" t="inlineStr">
@@ -27706,15 +27706,15 @@
     <row r="38">
       <c r="H38" s="6" t="inlineStr">
         <is>
-          <t>ARES</t>
+          <t>CINF</t>
         </is>
       </c>
       <c r="I38" s="61" t="n">
-        <v>0.00637586</v>
+        <v>0.00648337</v>
       </c>
       <c r="J38" s="6" t="inlineStr">
         <is>
-          <t>ARES MANAGEMENT CLASS A</t>
+          <t>CINCINNATI FINANCIAL</t>
         </is>
       </c>
       <c r="K38" s="6" t="inlineStr">
@@ -27735,7 +27735,7 @@
         </is>
       </c>
       <c r="I39" s="61" t="n">
-        <v>0.005973549999999999</v>
+        <v>0.00611947</v>
       </c>
       <c r="J39" s="6" t="inlineStr">
         <is>
@@ -27760,7 +27760,7 @@
         </is>
       </c>
       <c r="I40" s="61" t="n">
-        <v>0.00592575</v>
+        <v>0.00588202</v>
       </c>
       <c r="J40" s="6" t="inlineStr">
         <is>
@@ -27785,7 +27785,7 @@
         </is>
       </c>
       <c r="I41" s="61" t="n">
-        <v>0.00581422</v>
+        <v>0.00576179</v>
       </c>
       <c r="J41" s="6" t="inlineStr">
         <is>
@@ -27810,7 +27810,7 @@
         </is>
       </c>
       <c r="I42" s="61" t="n">
-        <v>0.00536073</v>
+        <v>0.005254999999999999</v>
       </c>
       <c r="J42" s="6" t="inlineStr">
         <is>
@@ -27835,7 +27835,7 @@
         </is>
       </c>
       <c r="I43" s="61" t="n">
-        <v>0.005140519999999999</v>
+        <v>0.0051088</v>
       </c>
       <c r="J43" s="6" t="inlineStr">
         <is>
@@ -27860,7 +27860,7 @@
         </is>
       </c>
       <c r="I44" s="61" t="n">
-        <v>0.00494746</v>
+        <v>0.00505467</v>
       </c>
       <c r="J44" s="6" t="inlineStr">
         <is>
@@ -27881,20 +27881,20 @@
     <row r="45">
       <c r="H45" s="6" t="inlineStr">
         <is>
-          <t>DINO</t>
+          <t>BBY</t>
         </is>
       </c>
       <c r="I45" s="61" t="n">
-        <v>0.0047234</v>
+        <v>0.00470751</v>
       </c>
       <c r="J45" s="6" t="inlineStr">
         <is>
-          <t>HF SINCLAIR</t>
+          <t>BEST BUY</t>
         </is>
       </c>
       <c r="K45" s="6" t="inlineStr">
         <is>
-          <t>Energy</t>
+          <t>Consumer Discretionary</t>
         </is>
       </c>
       <c r="L45" s="6" t="inlineStr"/>
@@ -27906,20 +27906,20 @@
     <row r="46">
       <c r="H46" s="6" t="inlineStr">
         <is>
-          <t>SNA</t>
+          <t>DINO</t>
         </is>
       </c>
       <c r="I46" s="61" t="n">
-        <v>0.004642879999999999</v>
+        <v>0.004503480000000001</v>
       </c>
       <c r="J46" s="6" t="inlineStr">
         <is>
-          <t>SNAP ON INC</t>
+          <t>HF SINCLAIR</t>
         </is>
       </c>
       <c r="K46" s="6" t="inlineStr">
         <is>
-          <t>Industrials</t>
+          <t>Energy</t>
         </is>
       </c>
       <c r="L46" s="6" t="inlineStr"/>
@@ -27931,20 +27931,20 @@
     <row r="47">
       <c r="H47" s="6" t="inlineStr">
         <is>
-          <t>BBY</t>
+          <t>GIS</t>
         </is>
       </c>
       <c r="I47" s="61" t="n">
-        <v>0.00453454</v>
+        <v>0.00447987</v>
       </c>
       <c r="J47" s="6" t="inlineStr">
         <is>
-          <t>BEST BUY</t>
+          <t>GENERAL MILLS INC</t>
         </is>
       </c>
       <c r="K47" s="6" t="inlineStr">
         <is>
-          <t>Consumer Discretionary</t>
+          <t>Consumer Staples</t>
         </is>
       </c>
       <c r="L47" s="6" t="inlineStr"/>
@@ -27956,20 +27956,20 @@
     <row r="48">
       <c r="H48" s="6" t="inlineStr">
         <is>
-          <t>EWBC</t>
+          <t>SNA</t>
         </is>
       </c>
       <c r="I48" s="61" t="n">
-        <v>0.00438045</v>
+        <v>0.004390740000000001</v>
       </c>
       <c r="J48" s="6" t="inlineStr">
         <is>
-          <t>EAST WEST BANCORP</t>
+          <t>SNAP ON INC</t>
         </is>
       </c>
       <c r="K48" s="6" t="inlineStr">
         <is>
-          <t>Financials</t>
+          <t>Industrials</t>
         </is>
       </c>
       <c r="L48" s="6" t="inlineStr"/>
@@ -27981,20 +27981,20 @@
     <row r="49">
       <c r="H49" s="6" t="inlineStr">
         <is>
-          <t>GIS</t>
+          <t>EWBC</t>
         </is>
       </c>
       <c r="I49" s="61" t="n">
-        <v>0.00423748</v>
+        <v>0.00432851</v>
       </c>
       <c r="J49" s="6" t="inlineStr">
         <is>
-          <t>GENERAL MILLS INC</t>
+          <t>EAST WEST BANCORP</t>
         </is>
       </c>
       <c r="K49" s="6" t="inlineStr">
         <is>
-          <t>Consumer Staples</t>
+          <t>Financials</t>
         </is>
       </c>
       <c r="L49" s="6" t="inlineStr"/>
@@ -28010,7 +28010,7 @@
         </is>
       </c>
       <c r="I50" s="61" t="n">
-        <v>0.00423056</v>
+        <v>0.00412488</v>
       </c>
       <c r="J50" s="6" t="inlineStr">
         <is>
@@ -28035,7 +28035,7 @@
         </is>
       </c>
       <c r="I51" s="61" t="n">
-        <v>0.00264098</v>
+        <v>0.00277119</v>
       </c>
       <c r="J51" s="6" t="inlineStr">
         <is>
@@ -28056,15 +28056,15 @@
     <row r="52">
       <c r="H52" s="6" t="inlineStr">
         <is>
-          <t>FNF</t>
+          <t>AFG</t>
         </is>
       </c>
       <c r="I52" s="61" t="n">
-        <v>0.00251603</v>
+        <v>0.00251216</v>
       </c>
       <c r="J52" s="6" t="inlineStr">
         <is>
-          <t>FIDELITY NATIONAL FINANCIAL INC</t>
+          <t>AMERICAN FINANCIAL GROUP</t>
         </is>
       </c>
       <c r="K52" s="6" t="inlineStr">
@@ -28081,15 +28081,15 @@
     <row r="53">
       <c r="H53" s="6" t="inlineStr">
         <is>
-          <t>AFG</t>
+          <t>FNF</t>
         </is>
       </c>
       <c r="I53" s="61" t="n">
-        <v>0.00250354</v>
+        <v>0.00250869</v>
       </c>
       <c r="J53" s="6" t="inlineStr">
         <is>
-          <t>AMERICAN FINANCIAL GROUP</t>
+          <t>FIDELITY NATIONAL FINANCIAL INC</t>
         </is>
       </c>
       <c r="K53" s="6" t="inlineStr">
@@ -28110,7 +28110,7 @@
         </is>
       </c>
       <c r="I54" s="61" t="n">
-        <v>0.00219483</v>
+        <v>0.00224926</v>
       </c>
       <c r="J54" s="6" t="inlineStr">
         <is>
@@ -28135,7 +28135,7 @@
         </is>
       </c>
       <c r="I55" s="61" t="n">
-        <v>0.00216782</v>
+        <v>0.00211915</v>
       </c>
       <c r="J55" s="6" t="inlineStr">
         <is>
@@ -28160,7 +28160,7 @@
         </is>
       </c>
       <c r="I56" s="61" t="n">
-        <v>0.00200789</v>
+        <v>0.00201168</v>
       </c>
       <c r="J56" s="6" t="inlineStr">
         <is>
@@ -28185,7 +28185,7 @@
         </is>
       </c>
       <c r="I57" s="61" t="n">
-        <v>0.00187926</v>
+        <v>0.001886</v>
       </c>
       <c r="J57" s="6" t="inlineStr">
         <is>
@@ -28210,7 +28210,7 @@
         </is>
       </c>
       <c r="I58" s="61" t="n">
-        <v>0.00153483</v>
+        <v>0.0015801</v>
       </c>
       <c r="J58" s="6" t="inlineStr">
         <is>
@@ -28235,7 +28235,7 @@
         </is>
       </c>
       <c r="I59" s="61" t="n">
-        <v>0.00149806</v>
+        <v>0.00151255</v>
       </c>
       <c r="J59" s="6" t="inlineStr">
         <is>
@@ -28256,20 +28256,20 @@
     <row r="60">
       <c r="H60" s="6" t="inlineStr">
         <is>
-          <t>MSM</t>
+          <t>MUR</t>
         </is>
       </c>
       <c r="I60" s="61" t="n">
-        <v>0.00148054</v>
+        <v>0.00136119</v>
       </c>
       <c r="J60" s="6" t="inlineStr">
         <is>
-          <t>MSC INDUSTRIAL CLASS A</t>
+          <t>MURPHY OIL</t>
         </is>
       </c>
       <c r="K60" s="6" t="inlineStr">
         <is>
-          <t>Industrials</t>
+          <t>Energy</t>
         </is>
       </c>
       <c r="L60" s="6" t="inlineStr"/>
@@ -28281,20 +28281,20 @@
     <row r="61">
       <c r="H61" s="6" t="inlineStr">
         <is>
-          <t>MUR</t>
+          <t>MTN</t>
         </is>
       </c>
       <c r="I61" s="61" t="n">
-        <v>0.0014101</v>
+        <v>0.00125791</v>
       </c>
       <c r="J61" s="6" t="inlineStr">
         <is>
-          <t>MURPHY OIL</t>
+          <t>VAIL RESORTS</t>
         </is>
       </c>
       <c r="K61" s="6" t="inlineStr">
         <is>
-          <t>Energy</t>
+          <t>Consumer Discretionary</t>
         </is>
       </c>
       <c r="L61" s="6" t="inlineStr"/>
@@ -28306,20 +28306,20 @@
     <row r="62">
       <c r="H62" s="6" t="inlineStr">
         <is>
-          <t>MTN</t>
+          <t>MSM</t>
         </is>
       </c>
       <c r="I62" s="61" t="n">
-        <v>0.00127473</v>
+        <v>0.00122662</v>
       </c>
       <c r="J62" s="6" t="inlineStr">
         <is>
-          <t>VAIL RESORTS</t>
+          <t>MSC INDUSTRIAL CLASS A</t>
         </is>
       </c>
       <c r="K62" s="6" t="inlineStr">
         <is>
-          <t>Consumer Discretionary</t>
+          <t>Industrials</t>
         </is>
       </c>
       <c r="L62" s="6" t="inlineStr"/>
@@ -28335,7 +28335,7 @@
         </is>
       </c>
       <c r="I63" s="61" t="n">
-        <v>0.00118818</v>
+        <v>0.00120113</v>
       </c>
       <c r="J63" s="6" t="inlineStr">
         <is>
@@ -28360,7 +28360,7 @@
         </is>
       </c>
       <c r="I64" s="61" t="n">
-        <v>0.00116287</v>
+        <v>0.0011653</v>
       </c>
       <c r="J64" s="6" t="inlineStr">
         <is>
@@ -28385,7 +28385,7 @@
         </is>
       </c>
       <c r="I65" s="61" t="n">
-        <v>0.0009725399999999999</v>
+        <v>0.0009790199999999999</v>
       </c>
       <c r="J65" s="6" t="inlineStr">
         <is>
@@ -28410,7 +28410,7 @@
         </is>
       </c>
       <c r="I66" s="61" t="n">
-        <v>0.00095373</v>
+        <v>0.00096866</v>
       </c>
       <c r="J66" s="6" t="inlineStr">
         <is>
@@ -28431,20 +28431,20 @@
     <row r="67">
       <c r="H67" s="6" t="inlineStr">
         <is>
-          <t>CWEN</t>
+          <t>KFY</t>
         </is>
       </c>
       <c r="I67" s="61" t="n">
-        <v>0.00092919</v>
+        <v>0.0009356799999999999</v>
       </c>
       <c r="J67" s="6" t="inlineStr">
         <is>
-          <t>CLEARWAY ENERGY INC CLASS C</t>
+          <t>KORN FERRY</t>
         </is>
       </c>
       <c r="K67" s="6" t="inlineStr">
         <is>
-          <t>Utilities</t>
+          <t>Industrials</t>
         </is>
       </c>
       <c r="L67" s="6" t="inlineStr"/>
@@ -28456,20 +28456,20 @@
     <row r="68">
       <c r="H68" s="6" t="inlineStr">
         <is>
-          <t>PAG</t>
+          <t>CVBF</t>
         </is>
       </c>
       <c r="I68" s="61" t="n">
-        <v>0.00091621</v>
+        <v>0.00091526</v>
       </c>
       <c r="J68" s="6" t="inlineStr">
         <is>
-          <t>PENSKE AUTOMOTIVE GROUP VOTING INC</t>
+          <t>CVB FINANCIAL CORP</t>
         </is>
       </c>
       <c r="K68" s="6" t="inlineStr">
         <is>
-          <t>Consumer Discretionary</t>
+          <t>Financials</t>
         </is>
       </c>
       <c r="L68" s="6" t="inlineStr"/>
@@ -28481,20 +28481,20 @@
     <row r="69">
       <c r="H69" s="6" t="inlineStr">
         <is>
-          <t>KFY</t>
+          <t>CWEN</t>
         </is>
       </c>
       <c r="I69" s="61" t="n">
-        <v>0.0009149500000000001</v>
+        <v>0.00090426</v>
       </c>
       <c r="J69" s="6" t="inlineStr">
         <is>
-          <t>KORN FERRY</t>
+          <t>CLEARWAY ENERGY INC CLASS C</t>
         </is>
       </c>
       <c r="K69" s="6" t="inlineStr">
         <is>
-          <t>Industrials</t>
+          <t>Utilities</t>
         </is>
       </c>
       <c r="L69" s="6" t="inlineStr"/>
@@ -28506,20 +28506,20 @@
     <row r="70">
       <c r="H70" s="6" t="inlineStr">
         <is>
-          <t>CVBF</t>
+          <t>RHI</t>
         </is>
       </c>
       <c r="I70" s="61" t="n">
-        <v>0.00090226</v>
+        <v>0.0009002200000000001</v>
       </c>
       <c r="J70" s="6" t="inlineStr">
         <is>
-          <t>CVB FINANCIAL CORP</t>
+          <t>ROBERT HALF INC</t>
         </is>
       </c>
       <c r="K70" s="6" t="inlineStr">
         <is>
-          <t>Financials</t>
+          <t>Industrials</t>
         </is>
       </c>
       <c r="L70" s="6" t="inlineStr"/>
@@ -28531,20 +28531,20 @@
     <row r="71">
       <c r="H71" s="6" t="inlineStr">
         <is>
-          <t>RHI</t>
+          <t>PAG</t>
         </is>
       </c>
       <c r="I71" s="61" t="n">
-        <v>0.00084555</v>
+        <v>0.00089693</v>
       </c>
       <c r="J71" s="6" t="inlineStr">
         <is>
-          <t>ROBERT HALF INC</t>
+          <t>PENSKE AUTOMOTIVE GROUP VOTING INC</t>
         </is>
       </c>
       <c r="K71" s="6" t="inlineStr">
         <is>
-          <t>Industrials</t>
+          <t>Consumer Discretionary</t>
         </is>
       </c>
       <c r="L71" s="6" t="inlineStr"/>
@@ -28560,7 +28560,7 @@
         </is>
       </c>
       <c r="I72" s="61" t="n">
-        <v>0.00056972</v>
+        <v>0.00057898</v>
       </c>
       <c r="J72" s="6" t="inlineStr">
         <is>
@@ -28585,7 +28585,7 @@
         </is>
       </c>
       <c r="I73" s="61" t="n">
-        <v>0.0005598199999999999</v>
+        <v>0.00056443</v>
       </c>
       <c r="J73" s="6" t="inlineStr">
         <is>
@@ -28606,20 +28606,20 @@
     <row r="74">
       <c r="H74" s="6" t="inlineStr">
         <is>
-          <t>OFG</t>
+          <t>MZTI</t>
         </is>
       </c>
       <c r="I74" s="61" t="n">
-        <v>0.0005196900000000001</v>
+        <v>0.00052122</v>
       </c>
       <c r="J74" s="6" t="inlineStr">
         <is>
-          <t>OFG BANCORP</t>
+          <t>MARZETTI</t>
         </is>
       </c>
       <c r="K74" s="6" t="inlineStr">
         <is>
-          <t>Financials</t>
+          <t>Consumer Staples</t>
         </is>
       </c>
       <c r="L74" s="6" t="inlineStr"/>
@@ -28631,20 +28631,20 @@
     <row r="75">
       <c r="H75" s="6" t="inlineStr">
         <is>
-          <t>IPAR</t>
+          <t>OFG</t>
         </is>
       </c>
       <c r="I75" s="61" t="n">
-        <v>0.00050302</v>
+        <v>0.00051729</v>
       </c>
       <c r="J75" s="6" t="inlineStr">
         <is>
-          <t>INTERPARFUMS INC</t>
+          <t>OFG BANCORP</t>
         </is>
       </c>
       <c r="K75" s="6" t="inlineStr">
         <is>
-          <t>Consumer Staples</t>
+          <t>Financials</t>
         </is>
       </c>
       <c r="L75" s="6" t="inlineStr"/>
@@ -28656,15 +28656,15 @@
     <row r="76">
       <c r="H76" s="6" t="inlineStr">
         <is>
-          <t>MZTI</t>
+          <t>IPAR</t>
         </is>
       </c>
       <c r="I76" s="61" t="n">
-        <v>0.00049936</v>
+        <v>0.00050476</v>
       </c>
       <c r="J76" s="6" t="inlineStr">
         <is>
-          <t>MARZETTI</t>
+          <t>INTERPARFUMS INC</t>
         </is>
       </c>
       <c r="K76" s="6" t="inlineStr">
@@ -28685,7 +28685,7 @@
         </is>
       </c>
       <c r="I77" s="61" t="n">
-        <v>0.00048373</v>
+        <v>0.0004856</v>
       </c>
       <c r="J77" s="6" t="inlineStr">
         <is>
@@ -28710,7 +28710,7 @@
         </is>
       </c>
       <c r="I78" s="61" t="n">
-        <v>0.0004815</v>
+        <v>0.0004796099999999999</v>
       </c>
       <c r="J78" s="6" t="inlineStr">
         <is>
@@ -28735,7 +28735,7 @@
         </is>
       </c>
       <c r="I79" s="61" t="n">
-        <v>0.00047554</v>
+        <v>0.00047885</v>
       </c>
       <c r="J79" s="6" t="inlineStr">
         <is>
@@ -28760,7 +28760,7 @@
         </is>
       </c>
       <c r="I80" s="61" t="n">
-        <v>0.00045774</v>
+        <v>0.00045857</v>
       </c>
       <c r="J80" s="6" t="inlineStr">
         <is>
@@ -28781,20 +28781,20 @@
     <row r="81">
       <c r="H81" s="6" t="inlineStr">
         <is>
-          <t>AGM</t>
+          <t>NSP</t>
         </is>
       </c>
       <c r="I81" s="61" t="n">
-        <v>0.00045368</v>
+        <v>0.00045599</v>
       </c>
       <c r="J81" s="6" t="inlineStr">
         <is>
-          <t>FEDERAL AGRICULTURAL MORTGAGE NON</t>
+          <t>INSPERITY</t>
         </is>
       </c>
       <c r="K81" s="6" t="inlineStr">
         <is>
-          <t>Financials</t>
+          <t>Industrials</t>
         </is>
       </c>
       <c r="L81" s="6" t="inlineStr"/>
@@ -28806,20 +28806,20 @@
     <row r="82">
       <c r="H82" s="6" t="inlineStr">
         <is>
-          <t>NSP</t>
+          <t>AGM</t>
         </is>
       </c>
       <c r="I82" s="61" t="n">
-        <v>0.00043713</v>
+        <v>0.00044824</v>
       </c>
       <c r="J82" s="6" t="inlineStr">
         <is>
-          <t>INSPERITY</t>
+          <t>FEDERAL AGRICULTURAL MORTGAGE NON</t>
         </is>
       </c>
       <c r="K82" s="6" t="inlineStr">
         <is>
-          <t>Industrials</t>
+          <t>Financials</t>
         </is>
       </c>
       <c r="L82" s="6" t="inlineStr"/>
@@ -28831,22 +28831,18 @@
     <row r="83">
       <c r="H83" s="6" t="inlineStr">
         <is>
-          <t>STBA</t>
+          <t>GVMXX</t>
         </is>
       </c>
       <c r="I83" s="61" t="n">
-        <v>0.00042025</v>
+        <v>0.00043447</v>
       </c>
       <c r="J83" s="6" t="inlineStr">
         <is>
-          <t>S AND T BANCORP INC</t>
-        </is>
-      </c>
-      <c r="K83" s="6" t="inlineStr">
-        <is>
-          <t>Financials</t>
-        </is>
-      </c>
+          <t>SSC GOVERNMENT MM GVMXX</t>
+        </is>
+      </c>
+      <c r="K83" s="6" t="inlineStr"/>
       <c r="L83" s="6" t="inlineStr"/>
       <c r="M83" s="7">
         <f>IF(H83="","",IFERROR(VLOOKUP(K83,$P$5:$Q$15,2,FALSE),"현금·선물"))</f>
@@ -28856,18 +28852,22 @@
     <row r="84">
       <c r="H84" s="6" t="inlineStr">
         <is>
-          <t>GVMXX</t>
+          <t>STBA</t>
         </is>
       </c>
       <c r="I84" s="61" t="n">
-        <v>0.00041188</v>
+        <v>0.00042703</v>
       </c>
       <c r="J84" s="6" t="inlineStr">
         <is>
-          <t>SSC GOVERNMENT MM GVMXX</t>
-        </is>
-      </c>
-      <c r="K84" s="6" t="inlineStr"/>
+          <t>S AND T BANCORP INC</t>
+        </is>
+      </c>
+      <c r="K84" s="6" t="inlineStr">
+        <is>
+          <t>Financials</t>
+        </is>
+      </c>
       <c r="L84" s="6" t="inlineStr"/>
       <c r="M84" s="7">
         <f>IF(H84="","",IFERROR(VLOOKUP(K84,$P$5:$Q$15,2,FALSE),"현금·선물"))</f>
@@ -28881,7 +28881,7 @@
         </is>
       </c>
       <c r="I85" s="61" t="n">
-        <v>0.00041158</v>
+        <v>0.00041268</v>
       </c>
       <c r="J85" s="6" t="inlineStr">
         <is>
@@ -28906,7 +28906,7 @@
         </is>
       </c>
       <c r="I86" s="61" t="n">
-        <v>0.00037281</v>
+        <v>0.00037069</v>
       </c>
       <c r="J86" s="6" t="inlineStr">
         <is>
@@ -28931,7 +28931,7 @@
         </is>
       </c>
       <c r="I87" s="61" t="n">
-        <v>0.00035181</v>
+        <v>0.00035239</v>
       </c>
       <c r="J87" s="6" t="inlineStr">
         <is>
@@ -28956,7 +28956,7 @@
         </is>
       </c>
       <c r="I88" s="61" t="n">
-        <v>0.00034437</v>
+        <v>0.00034771</v>
       </c>
       <c r="J88" s="6" t="inlineStr">
         <is>
@@ -28981,7 +28981,7 @@
         </is>
       </c>
       <c r="I89" s="61" t="n">
-        <v>0.00030009</v>
+        <v>0.00032456</v>
       </c>
       <c r="J89" s="6" t="inlineStr">
         <is>
@@ -29006,7 +29006,7 @@
         </is>
       </c>
       <c r="I90" s="61" t="n">
-        <v>0.00027976</v>
+        <v>0.00028219</v>
       </c>
       <c r="J90" s="6" t="inlineStr">
         <is>
@@ -29031,7 +29031,7 @@
         </is>
       </c>
       <c r="I91" s="61" t="n">
-        <v>0.00025535</v>
+        <v>0.00025546</v>
       </c>
       <c r="J91" s="6" t="inlineStr">
         <is>
@@ -29056,7 +29056,7 @@
         </is>
       </c>
       <c r="I92" s="61" t="n">
-        <v>0.00024557</v>
+        <v>0.00025145</v>
       </c>
       <c r="J92" s="6" t="inlineStr">
         <is>
@@ -29081,7 +29081,7 @@
         </is>
       </c>
       <c r="I93" s="61" t="n">
-        <v>0.00023034</v>
+        <v>0.00023099</v>
       </c>
       <c r="J93" s="6" t="inlineStr">
         <is>
@@ -29106,7 +29106,7 @@
         </is>
       </c>
       <c r="I94" s="61" t="n">
-        <v>0.00022613</v>
+        <v>0.00022652</v>
       </c>
       <c r="J94" s="6" t="inlineStr">
         <is>
@@ -29131,7 +29131,7 @@
         </is>
       </c>
       <c r="I95" s="61" t="n">
-        <v>0.00020799</v>
+        <v>0.00021034</v>
       </c>
       <c r="J95" s="6" t="inlineStr">
         <is>
@@ -29156,7 +29156,7 @@
         </is>
       </c>
       <c r="I96" s="61" t="n">
-        <v>0.00019489</v>
+        <v>0.00019589</v>
       </c>
       <c r="J96" s="6" t="inlineStr">
         <is>
@@ -29181,7 +29181,7 @@
         </is>
       </c>
       <c r="I97" s="61" t="n">
-        <v>0.00019378</v>
+        <v>0.00019368</v>
       </c>
       <c r="J97" s="6" t="inlineStr">
         <is>
@@ -29206,7 +29206,7 @@
         </is>
       </c>
       <c r="I98" s="61" t="n">
-        <v>0.00017768</v>
+        <v>0.00017816</v>
       </c>
       <c r="J98" s="6" t="inlineStr">
         <is>
@@ -29231,7 +29231,7 @@
         </is>
       </c>
       <c r="I99" s="61" t="n">
-        <v>0.00016509</v>
+        <v>0.00016466</v>
       </c>
       <c r="J99" s="6" t="inlineStr">
         <is>
@@ -29252,18 +29252,22 @@
     <row r="100">
       <c r="H100" s="6" t="inlineStr">
         <is>
-          <t>USD</t>
+          <t>EBF</t>
         </is>
       </c>
       <c r="I100" s="61" t="n">
-        <v>0.00013204</v>
+        <v>0.0001306</v>
       </c>
       <c r="J100" s="6" t="inlineStr">
         <is>
-          <t>US DOLLAR</t>
-        </is>
-      </c>
-      <c r="K100" s="6" t="inlineStr"/>
+          <t>ENNIS INC</t>
+        </is>
+      </c>
+      <c r="K100" s="6" t="inlineStr">
+        <is>
+          <t>Industrials</t>
+        </is>
+      </c>
       <c r="L100" s="6" t="inlineStr"/>
       <c r="M100" s="7">
         <f>IF(H100="","",IFERROR(VLOOKUP(K100,$P$5:$Q$15,2,FALSE),"현금·선물"))</f>
@@ -29273,20 +29277,20 @@
     <row r="101">
       <c r="H101" s="6" t="inlineStr">
         <is>
-          <t>EBF</t>
+          <t>AMSF</t>
         </is>
       </c>
       <c r="I101" s="61" t="n">
-        <v>0.00013122</v>
+        <v>0.00011739</v>
       </c>
       <c r="J101" s="6" t="inlineStr">
         <is>
-          <t>ENNIS INC</t>
+          <t>AMERISAFE INC</t>
         </is>
       </c>
       <c r="K101" s="6" t="inlineStr">
         <is>
-          <t>Industrials</t>
+          <t>Financials</t>
         </is>
       </c>
       <c r="L101" s="6" t="inlineStr"/>
@@ -29298,22 +29302,18 @@
     <row r="102">
       <c r="H102" s="6" t="inlineStr">
         <is>
-          <t>AMSF</t>
+          <t>USD</t>
         </is>
       </c>
       <c r="I102" s="61" t="n">
-        <v>0.00011517</v>
+        <v>0.0001055</v>
       </c>
       <c r="J102" s="6" t="inlineStr">
         <is>
-          <t>AMERISAFE INC</t>
-        </is>
-      </c>
-      <c r="K102" s="6" t="inlineStr">
-        <is>
-          <t>Financials</t>
-        </is>
-      </c>
+          <t>US DOLLAR</t>
+        </is>
+      </c>
+      <c r="K102" s="6" t="inlineStr"/>
       <c r="L102" s="6" t="inlineStr"/>
       <c r="M102" s="7">
         <f>IF(H102="","",IFERROR(VLOOKUP(K102,$P$5:$Q$15,2,FALSE),"현금·선물"))</f>
@@ -29327,7 +29327,7 @@
         </is>
       </c>
       <c r="I103" s="61" t="n">
-        <v>9.625999999999999e-05</v>
+        <v>9.903000000000001e-05</v>
       </c>
       <c r="J103" s="6" t="inlineStr">
         <is>
@@ -29352,7 +29352,7 @@
         </is>
       </c>
       <c r="I104" s="61" t="n">
-        <v>8.805e-05</v>
+        <v>9.377000000000001e-05</v>
       </c>
       <c r="J104" s="6" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
데이터 갱신: holdings (2026-10-24)
</commit_message>
<xml_diff>
--- a/downloads/schd_dividend_tracker.xlsx
+++ b/downloads/schd_dividend_tracker.xlsx
@@ -1724,7 +1724,7 @@
     <row r="3">
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>최종 갱신: 2026-10-23 · 반영 범위: 2012년 1분기 ~ 2026년 3분기 (배당락 2026-09-23) · GitHub Actions 자동 생성</t>
+          <t>최종 갱신: 2026-10-24 · 반영 범위: 2012년 1분기 ~ 2026년 3분기 (배당락 2026-09-23) · GitHub Actions 자동 생성</t>
         </is>
       </c>
     </row>
@@ -26257,11 +26257,11 @@
         </is>
       </c>
       <c r="B2" s="49" t="n">
-        <v>46317</v>
+        <v>46318</v>
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>← 이 날 종가로 계산한 비중. 그날 공식 파일을 못 받아 Schwab 공식 보유종목 CSV(2026-10-21)의 보유 주식 수 × 종가로 계산했습니다.</t>
+          <t>← 이 날 종가로 계산한 비중. 그날 공식 파일을 못 받아 Schwab 공식 보유종목 CSV(2026-10-22)의 보유 주식 수 × 종가로 계산했습니다.</t>
         </is>
       </c>
     </row>
@@ -26354,25 +26354,25 @@
       </c>
       <c r="H5" s="6" t="inlineStr">
         <is>
-          <t>PG</t>
+          <t>TXN</t>
         </is>
       </c>
       <c r="I5" s="61" t="n">
-        <v>0.0440797</v>
+        <v>0.04408678</v>
       </c>
       <c r="J5" s="6" t="inlineStr">
         <is>
-          <t>PROCTER &amp; GAMBLE</t>
+          <t>TEXAS INSTRUMENT</t>
         </is>
       </c>
       <c r="K5" s="6" t="inlineStr">
         <is>
-          <t>Consumer Staples</t>
+          <t>Information Technology</t>
         </is>
       </c>
       <c r="L5" s="6" t="inlineStr">
         <is>
-          <t>프록터앤드갬블</t>
+          <t>텍사스 인스트루먼트</t>
         </is>
       </c>
       <c r="M5" s="7">
@@ -26412,25 +26412,25 @@
       </c>
       <c r="H6" s="6" t="inlineStr">
         <is>
-          <t>TXN</t>
+          <t>CVX</t>
         </is>
       </c>
       <c r="I6" s="61" t="n">
-        <v>0.04311106</v>
+        <v>0.04345056999999999</v>
       </c>
       <c r="J6" s="6" t="inlineStr">
         <is>
-          <t>TEXAS INSTRUMENT</t>
+          <t>CHEVRON</t>
         </is>
       </c>
       <c r="K6" s="6" t="inlineStr">
         <is>
-          <t>Information Technology</t>
+          <t>Energy</t>
         </is>
       </c>
       <c r="L6" s="6" t="inlineStr">
         <is>
-          <t>텍사스 인스트루먼트</t>
+          <t>셰브론</t>
         </is>
       </c>
       <c r="M6" s="7">
@@ -26470,25 +26470,25 @@
       </c>
       <c r="H7" s="6" t="inlineStr">
         <is>
-          <t>KO</t>
+          <t>COP</t>
         </is>
       </c>
       <c r="I7" s="61" t="n">
-        <v>0.04246364</v>
+        <v>0.04331401999999999</v>
       </c>
       <c r="J7" s="6" t="inlineStr">
         <is>
-          <t>COCA-COLA</t>
+          <t>CONOCOPHILLIPS</t>
         </is>
       </c>
       <c r="K7" s="6" t="inlineStr">
         <is>
-          <t>Consumer Staples</t>
+          <t>Energy</t>
         </is>
       </c>
       <c r="L7" s="6" t="inlineStr">
         <is>
-          <t>코카콜라</t>
+          <t>코노코필립스</t>
         </is>
       </c>
       <c r="M7" s="7">
@@ -26528,25 +26528,25 @@
       </c>
       <c r="H8" s="6" t="inlineStr">
         <is>
-          <t>CVX</t>
+          <t>PG</t>
         </is>
       </c>
       <c r="I8" s="61" t="n">
-        <v>0.04206611</v>
+        <v>0.04303422</v>
       </c>
       <c r="J8" s="6" t="inlineStr">
         <is>
-          <t>CHEVRON</t>
+          <t>PROCTER &amp; GAMBLE</t>
         </is>
       </c>
       <c r="K8" s="6" t="inlineStr">
         <is>
-          <t>Energy</t>
+          <t>Consumer Staples</t>
         </is>
       </c>
       <c r="L8" s="6" t="inlineStr">
         <is>
-          <t>셰브론</t>
+          <t>프록터앤드갬블</t>
         </is>
       </c>
       <c r="M8" s="7">
@@ -26586,25 +26586,25 @@
       </c>
       <c r="H9" s="6" t="inlineStr">
         <is>
-          <t>UNH</t>
+          <t>KO</t>
         </is>
       </c>
       <c r="I9" s="61" t="n">
-        <v>0.04179048</v>
+        <v>0.04145703</v>
       </c>
       <c r="J9" s="6" t="inlineStr">
         <is>
-          <t>UNITEDHEALTH GROUP</t>
+          <t>COCA-COLA</t>
         </is>
       </c>
       <c r="K9" s="6" t="inlineStr">
         <is>
-          <t>Health Care</t>
+          <t>Consumer Staples</t>
         </is>
       </c>
       <c r="L9" s="6" t="inlineStr">
         <is>
-          <t>유나이티드헬스</t>
+          <t>코카콜라</t>
         </is>
       </c>
       <c r="M9" s="7">
@@ -26644,25 +26644,25 @@
       </c>
       <c r="H10" s="6" t="inlineStr">
         <is>
-          <t>COP</t>
+          <t>UNH</t>
         </is>
       </c>
       <c r="I10" s="61" t="n">
-        <v>0.04166280000000001</v>
+        <v>0.04127694</v>
       </c>
       <c r="J10" s="6" t="inlineStr">
         <is>
-          <t>CONOCOPHILLIPS</t>
+          <t>UNITEDHEALTH GROUP</t>
         </is>
       </c>
       <c r="K10" s="6" t="inlineStr">
         <is>
-          <t>Energy</t>
+          <t>Health Care</t>
         </is>
       </c>
       <c r="L10" s="6" t="inlineStr">
         <is>
-          <t>코노코필립스</t>
+          <t>유나이티드헬스</t>
         </is>
       </c>
       <c r="M10" s="7">
@@ -26702,25 +26702,25 @@
       </c>
       <c r="H11" s="6" t="inlineStr">
         <is>
-          <t>HD</t>
+          <t>QCOM</t>
         </is>
       </c>
       <c r="I11" s="61" t="n">
-        <v>0.04043819</v>
+        <v>0.04083957</v>
       </c>
       <c r="J11" s="6" t="inlineStr">
         <is>
-          <t>HOME DEPOT</t>
+          <t>QUALCOMM</t>
         </is>
       </c>
       <c r="K11" s="6" t="inlineStr">
         <is>
-          <t>Consumer Discretionary</t>
+          <t>Information Technology</t>
         </is>
       </c>
       <c r="L11" s="6" t="inlineStr">
         <is>
-          <t>홈디포</t>
+          <t>퀄컴</t>
         </is>
       </c>
       <c r="M11" s="7">
@@ -26760,25 +26760,25 @@
       </c>
       <c r="H12" s="6" t="inlineStr">
         <is>
-          <t>QCOM</t>
+          <t>HD</t>
         </is>
       </c>
       <c r="I12" s="61" t="n">
-        <v>0.03996504</v>
+        <v>0.03962082</v>
       </c>
       <c r="J12" s="6" t="inlineStr">
         <is>
-          <t>QUALCOMM</t>
+          <t>HOME DEPOT</t>
         </is>
       </c>
       <c r="K12" s="6" t="inlineStr">
         <is>
-          <t>Information Technology</t>
+          <t>Consumer Discretionary</t>
         </is>
       </c>
       <c r="L12" s="6" t="inlineStr">
         <is>
-          <t>퀄컴</t>
+          <t>홈디포</t>
         </is>
       </c>
       <c r="M12" s="7">
@@ -26822,7 +26822,7 @@
         </is>
       </c>
       <c r="I13" s="61" t="n">
-        <v>0.03969446</v>
+        <v>0.03913819</v>
       </c>
       <c r="J13" s="6" t="inlineStr">
         <is>
@@ -26880,7 +26880,7 @@
         </is>
       </c>
       <c r="I14" s="61" t="n">
-        <v>0.03882847</v>
+        <v>0.03812414</v>
       </c>
       <c r="J14" s="6" t="inlineStr">
         <is>
@@ -26928,7 +26928,7 @@
         </is>
       </c>
       <c r="I15" s="61" t="n">
-        <v>0.03816085</v>
+        <v>0.0378005</v>
       </c>
       <c r="J15" s="6" t="inlineStr">
         <is>
@@ -26972,25 +26972,25 @@
       </c>
       <c r="H16" s="6" t="inlineStr">
         <is>
-          <t>ACN</t>
+          <t>ABT</t>
         </is>
       </c>
       <c r="I16" s="61" t="n">
-        <v>0.03770554</v>
+        <v>0.0370401</v>
       </c>
       <c r="J16" s="6" t="inlineStr">
         <is>
-          <t>ACCENTURE PLC CLASS A</t>
+          <t>ABBOTT LABORATORIES</t>
         </is>
       </c>
       <c r="K16" s="6" t="inlineStr">
         <is>
-          <t>Information Technology</t>
+          <t>Health Care</t>
         </is>
       </c>
       <c r="L16" s="6" t="inlineStr">
         <is>
-          <t>액센츄어</t>
+          <t>애보트</t>
         </is>
       </c>
       <c r="M16" s="7">
@@ -27010,25 +27010,25 @@
       </c>
       <c r="H17" s="6" t="inlineStr">
         <is>
-          <t>ABT</t>
+          <t>ACN</t>
         </is>
       </c>
       <c r="I17" s="61" t="n">
-        <v>0.03646952000000001</v>
+        <v>0.03648506</v>
       </c>
       <c r="J17" s="6" t="inlineStr">
         <is>
-          <t>ABBOTT LABORATORIES</t>
+          <t>ACCENTURE PLC CLASS A</t>
         </is>
       </c>
       <c r="K17" s="6" t="inlineStr">
         <is>
-          <t>Health Care</t>
+          <t>Information Technology</t>
         </is>
       </c>
       <c r="L17" s="6" t="inlineStr">
         <is>
-          <t>애보트</t>
+          <t>액센츄어</t>
         </is>
       </c>
       <c r="M17" s="7">
@@ -27052,7 +27052,7 @@
         </is>
       </c>
       <c r="I18" s="61" t="n">
-        <v>0.03537294</v>
+        <v>0.03508982</v>
       </c>
       <c r="J18" s="6" t="inlineStr">
         <is>
@@ -27081,7 +27081,7 @@
         </is>
       </c>
       <c r="I19" s="61" t="n">
-        <v>0.03064662</v>
+        <v>0.03002656</v>
       </c>
       <c r="J19" s="6" t="inlineStr">
         <is>
@@ -27115,7 +27115,7 @@
         </is>
       </c>
       <c r="I20" s="61" t="n">
-        <v>0.03024801</v>
+        <v>0.02966608</v>
       </c>
       <c r="J20" s="6" t="inlineStr">
         <is>
@@ -27150,15 +27150,15 @@
       </c>
       <c r="H21" s="6" t="inlineStr">
         <is>
-          <t>ADP</t>
+          <t>LMT</t>
         </is>
       </c>
       <c r="I21" s="61" t="n">
-        <v>0.0291323</v>
+        <v>0.02933715</v>
       </c>
       <c r="J21" s="6" t="inlineStr">
         <is>
-          <t>AUTOMATIC DATA PROCESSING INC</t>
+          <t>LOCKHEED MARTIN</t>
         </is>
       </c>
       <c r="K21" s="6" t="inlineStr">
@@ -27168,7 +27168,7 @@
       </c>
       <c r="L21" s="6" t="inlineStr">
         <is>
-          <t>ADP</t>
+          <t>록히드마틴</t>
         </is>
       </c>
       <c r="M21" s="7">
@@ -27188,15 +27188,15 @@
       </c>
       <c r="H22" s="6" t="inlineStr">
         <is>
-          <t>LMT</t>
+          <t>ADP</t>
         </is>
       </c>
       <c r="I22" s="61" t="n">
-        <v>0.02853046</v>
+        <v>0.02888952</v>
       </c>
       <c r="J22" s="6" t="inlineStr">
         <is>
-          <t>LOCKHEED MARTIN</t>
+          <t>AUTOMATIC DATA PROCESSING INC</t>
         </is>
       </c>
       <c r="K22" s="6" t="inlineStr">
@@ -27206,7 +27206,7 @@
       </c>
       <c r="L22" s="6" t="inlineStr">
         <is>
-          <t>록히드마틴</t>
+          <t>ADP</t>
         </is>
       </c>
       <c r="M22" s="7">
@@ -27230,7 +27230,7 @@
         </is>
       </c>
       <c r="I23" s="61" t="n">
-        <v>0.02122686</v>
+        <v>0.02117156</v>
       </c>
       <c r="J23" s="6" t="inlineStr">
         <is>
@@ -27268,7 +27268,7 @@
         </is>
       </c>
       <c r="I24" s="61" t="n">
-        <v>0.01973078</v>
+        <v>0.02044531</v>
       </c>
       <c r="J24" s="6" t="inlineStr">
         <is>
@@ -27306,7 +27306,7 @@
         </is>
       </c>
       <c r="I25" s="61" t="n">
-        <v>0.01925016</v>
+        <v>0.01920005</v>
       </c>
       <c r="J25" s="6" t="inlineStr">
         <is>
@@ -27340,25 +27340,25 @@
       </c>
       <c r="H26" s="6" t="inlineStr">
         <is>
-          <t>UPS</t>
+          <t>SLB</t>
         </is>
       </c>
       <c r="I26" s="61" t="n">
-        <v>0.01811623</v>
+        <v>0.01882809</v>
       </c>
       <c r="J26" s="6" t="inlineStr">
         <is>
-          <t>UNITED PARCEL SERVICE INC CLASS B</t>
+          <t>SLB</t>
         </is>
       </c>
       <c r="K26" s="6" t="inlineStr">
         <is>
-          <t>Industrials</t>
+          <t>Energy</t>
         </is>
       </c>
       <c r="L26" s="6" t="inlineStr">
         <is>
-          <t>UPS</t>
+          <t>SLB</t>
         </is>
       </c>
       <c r="M26" s="7">
@@ -27378,25 +27378,25 @@
       </c>
       <c r="H27" s="6" t="inlineStr">
         <is>
-          <t>SLB</t>
+          <t>UPS</t>
         </is>
       </c>
       <c r="I27" s="61" t="n">
-        <v>0.01751269</v>
+        <v>0.01810611</v>
       </c>
       <c r="J27" s="6" t="inlineStr">
         <is>
-          <t>SLB</t>
+          <t>UNITED PARCEL SERVICE INC CLASS B</t>
         </is>
       </c>
       <c r="K27" s="6" t="inlineStr">
         <is>
-          <t>Energy</t>
+          <t>Industrials</t>
         </is>
       </c>
       <c r="L27" s="6" t="inlineStr">
         <is>
-          <t>SLB</t>
+          <t>UPS</t>
         </is>
       </c>
       <c r="M27" s="7">
@@ -27420,7 +27420,7 @@
         </is>
       </c>
       <c r="I28" s="61" t="n">
-        <v>0.01710133</v>
+        <v>0.0165886</v>
       </c>
       <c r="J28" s="6" t="inlineStr">
         <is>
@@ -27454,27 +27454,23 @@
       </c>
       <c r="H29" s="6" t="inlineStr">
         <is>
-          <t>FAST</t>
+          <t>OKE</t>
         </is>
       </c>
       <c r="I29" s="61" t="n">
-        <v>0.01440925</v>
+        <v>0.01444304</v>
       </c>
       <c r="J29" s="6" t="inlineStr">
         <is>
-          <t>FASTENAL</t>
+          <t>ONEOK</t>
         </is>
       </c>
       <c r="K29" s="6" t="inlineStr">
         <is>
-          <t>Industrials</t>
-        </is>
-      </c>
-      <c r="L29" s="6" t="inlineStr">
-        <is>
-          <t>패스널</t>
-        </is>
-      </c>
+          <t>Energy</t>
+        </is>
+      </c>
+      <c r="L29" s="6" t="inlineStr"/>
       <c r="M29" s="7">
         <f>IF(H29="","",IFERROR(VLOOKUP(K29,$P$5:$Q$15,2,FALSE),"현금·선물"))</f>
         <v/>
@@ -27492,23 +27488,27 @@
       </c>
       <c r="H30" s="6" t="inlineStr">
         <is>
-          <t>OKE</t>
+          <t>FAST</t>
         </is>
       </c>
       <c r="I30" s="61" t="n">
-        <v>0.01409591</v>
+        <v>0.01424178</v>
       </c>
       <c r="J30" s="6" t="inlineStr">
         <is>
-          <t>ONEOK</t>
+          <t>FASTENAL</t>
         </is>
       </c>
       <c r="K30" s="6" t="inlineStr">
         <is>
-          <t>Energy</t>
-        </is>
-      </c>
-      <c r="L30" s="6" t="inlineStr"/>
+          <t>Industrials</t>
+        </is>
+      </c>
+      <c r="L30" s="6" t="inlineStr">
+        <is>
+          <t>패스널</t>
+        </is>
+      </c>
       <c r="M30" s="7">
         <f>IF(H30="","",IFERROR(VLOOKUP(K30,$P$5:$Q$15,2,FALSE),"현금·선물"))</f>
         <v/>
@@ -27530,7 +27530,7 @@
         </is>
       </c>
       <c r="I31" s="61" t="n">
-        <v>0.01288287</v>
+        <v>0.0135155</v>
       </c>
       <c r="J31" s="6" t="inlineStr">
         <is>
@@ -27555,7 +27555,7 @@
         </is>
       </c>
       <c r="I32" s="61" t="n">
-        <v>0.01149595</v>
+        <v>0.01148761</v>
       </c>
       <c r="J32" s="6" t="inlineStr">
         <is>
@@ -27585,7 +27585,7 @@
         </is>
       </c>
       <c r="I33" s="61" t="n">
-        <v>0.01113688</v>
+        <v>0.01086293</v>
       </c>
       <c r="J33" s="6" t="inlineStr">
         <is>
@@ -27610,7 +27610,7 @@
         </is>
       </c>
       <c r="I34" s="61" t="n">
-        <v>0.00916341</v>
+        <v>0.009234529999999999</v>
       </c>
       <c r="J34" s="6" t="inlineStr">
         <is>
@@ -27635,7 +27635,7 @@
         </is>
       </c>
       <c r="I35" s="61" t="n">
-        <v>0.009056920000000001</v>
+        <v>0.00903411</v>
       </c>
       <c r="J35" s="6" t="inlineStr">
         <is>
@@ -27660,7 +27660,7 @@
         </is>
       </c>
       <c r="I36" s="61" t="n">
-        <v>0.008895480000000001</v>
+        <v>0.008758409999999999</v>
       </c>
       <c r="J36" s="6" t="inlineStr">
         <is>
@@ -27685,7 +27685,7 @@
         </is>
       </c>
       <c r="I37" s="61" t="n">
-        <v>0.00659729</v>
+        <v>0.00653687</v>
       </c>
       <c r="J37" s="6" t="inlineStr">
         <is>
@@ -27710,7 +27710,7 @@
         </is>
       </c>
       <c r="I38" s="61" t="n">
-        <v>0.00648337</v>
+        <v>0.00646902</v>
       </c>
       <c r="J38" s="6" t="inlineStr">
         <is>
@@ -27735,7 +27735,7 @@
         </is>
       </c>
       <c r="I39" s="61" t="n">
-        <v>0.00611947</v>
+        <v>0.00593399</v>
       </c>
       <c r="J39" s="6" t="inlineStr">
         <is>
@@ -27756,20 +27756,20 @@
     <row r="40">
       <c r="H40" s="6" t="inlineStr">
         <is>
-          <t>DRI</t>
+          <t>RF</t>
         </is>
       </c>
       <c r="I40" s="61" t="n">
-        <v>0.00588202</v>
+        <v>0.00579904</v>
       </c>
       <c r="J40" s="6" t="inlineStr">
         <is>
-          <t>DARDEN RESTAURANTS INC</t>
+          <t>REGIONS FINANCIAL</t>
         </is>
       </c>
       <c r="K40" s="6" t="inlineStr">
         <is>
-          <t>Consumer Discretionary</t>
+          <t>Financials</t>
         </is>
       </c>
       <c r="L40" s="6" t="inlineStr"/>
@@ -27781,20 +27781,20 @@
     <row r="41">
       <c r="H41" s="6" t="inlineStr">
         <is>
-          <t>RF</t>
+          <t>DRI</t>
         </is>
       </c>
       <c r="I41" s="61" t="n">
-        <v>0.00576179</v>
+        <v>0.00576538</v>
       </c>
       <c r="J41" s="6" t="inlineStr">
         <is>
-          <t>REGIONS FINANCIAL</t>
+          <t>DARDEN RESTAURANTS INC</t>
         </is>
       </c>
       <c r="K41" s="6" t="inlineStr">
         <is>
-          <t>Financials</t>
+          <t>Consumer Discretionary</t>
         </is>
       </c>
       <c r="L41" s="6" t="inlineStr"/>
@@ -27810,7 +27810,7 @@
         </is>
       </c>
       <c r="I42" s="61" t="n">
-        <v>0.005254999999999999</v>
+        <v>0.0053142</v>
       </c>
       <c r="J42" s="6" t="inlineStr">
         <is>
@@ -27835,7 +27835,7 @@
         </is>
       </c>
       <c r="I43" s="61" t="n">
-        <v>0.0051088</v>
+        <v>0.00505742</v>
       </c>
       <c r="J43" s="6" t="inlineStr">
         <is>
@@ -27860,7 +27860,7 @@
         </is>
       </c>
       <c r="I44" s="61" t="n">
-        <v>0.00505467</v>
+        <v>0.00499736</v>
       </c>
       <c r="J44" s="6" t="inlineStr">
         <is>
@@ -27885,7 +27885,7 @@
         </is>
       </c>
       <c r="I45" s="61" t="n">
-        <v>0.00470751</v>
+        <v>0.00472818</v>
       </c>
       <c r="J45" s="6" t="inlineStr">
         <is>
@@ -27910,7 +27910,7 @@
         </is>
       </c>
       <c r="I46" s="61" t="n">
-        <v>0.004503480000000001</v>
+        <v>0.00449705</v>
       </c>
       <c r="J46" s="6" t="inlineStr">
         <is>
@@ -27931,20 +27931,20 @@
     <row r="47">
       <c r="H47" s="6" t="inlineStr">
         <is>
-          <t>GIS</t>
+          <t>SNA</t>
         </is>
       </c>
       <c r="I47" s="61" t="n">
-        <v>0.00447987</v>
+        <v>0.00441511</v>
       </c>
       <c r="J47" s="6" t="inlineStr">
         <is>
-          <t>GENERAL MILLS INC</t>
+          <t>SNAP ON INC</t>
         </is>
       </c>
       <c r="K47" s="6" t="inlineStr">
         <is>
-          <t>Consumer Staples</t>
+          <t>Industrials</t>
         </is>
       </c>
       <c r="L47" s="6" t="inlineStr"/>
@@ -27956,20 +27956,20 @@
     <row r="48">
       <c r="H48" s="6" t="inlineStr">
         <is>
-          <t>SNA</t>
+          <t>GIS</t>
         </is>
       </c>
       <c r="I48" s="61" t="n">
-        <v>0.004390740000000001</v>
+        <v>0.00439673</v>
       </c>
       <c r="J48" s="6" t="inlineStr">
         <is>
-          <t>SNAP ON INC</t>
+          <t>GENERAL MILLS INC</t>
         </is>
       </c>
       <c r="K48" s="6" t="inlineStr">
         <is>
-          <t>Industrials</t>
+          <t>Consumer Staples</t>
         </is>
       </c>
       <c r="L48" s="6" t="inlineStr"/>
@@ -27981,20 +27981,20 @@
     <row r="49">
       <c r="H49" s="6" t="inlineStr">
         <is>
-          <t>EWBC</t>
+          <t>APA</t>
         </is>
       </c>
       <c r="I49" s="61" t="n">
-        <v>0.00432851</v>
+        <v>0.0043474</v>
       </c>
       <c r="J49" s="6" t="inlineStr">
         <is>
-          <t>EAST WEST BANCORP</t>
+          <t>APA</t>
         </is>
       </c>
       <c r="K49" s="6" t="inlineStr">
         <is>
-          <t>Financials</t>
+          <t>Energy</t>
         </is>
       </c>
       <c r="L49" s="6" t="inlineStr"/>
@@ -28006,20 +28006,20 @@
     <row r="50">
       <c r="H50" s="6" t="inlineStr">
         <is>
-          <t>APA</t>
+          <t>EWBC</t>
         </is>
       </c>
       <c r="I50" s="61" t="n">
-        <v>0.00412488</v>
+        <v>0.00429793</v>
       </c>
       <c r="J50" s="6" t="inlineStr">
         <is>
-          <t>APA</t>
+          <t>EAST WEST BANCORP</t>
         </is>
       </c>
       <c r="K50" s="6" t="inlineStr">
         <is>
-          <t>Energy</t>
+          <t>Financials</t>
         </is>
       </c>
       <c r="L50" s="6" t="inlineStr"/>
@@ -28035,7 +28035,7 @@
         </is>
       </c>
       <c r="I51" s="61" t="n">
-        <v>0.00277119</v>
+        <v>0.00274762</v>
       </c>
       <c r="J51" s="6" t="inlineStr">
         <is>
@@ -28060,7 +28060,7 @@
         </is>
       </c>
       <c r="I52" s="61" t="n">
-        <v>0.00251216</v>
+        <v>0.00247547</v>
       </c>
       <c r="J52" s="6" t="inlineStr">
         <is>
@@ -28085,7 +28085,7 @@
         </is>
       </c>
       <c r="I53" s="61" t="n">
-        <v>0.00250869</v>
+        <v>0.00246148</v>
       </c>
       <c r="J53" s="6" t="inlineStr">
         <is>
@@ -28110,7 +28110,7 @@
         </is>
       </c>
       <c r="I54" s="61" t="n">
-        <v>0.00224926</v>
+        <v>0.00225104</v>
       </c>
       <c r="J54" s="6" t="inlineStr">
         <is>
@@ -28131,15 +28131,15 @@
     <row r="55">
       <c r="H55" s="6" t="inlineStr">
         <is>
-          <t>ORI</t>
+          <t>COLB</t>
         </is>
       </c>
       <c r="I55" s="61" t="n">
-        <v>0.00211915</v>
+        <v>0.00208524</v>
       </c>
       <c r="J55" s="6" t="inlineStr">
         <is>
-          <t>OLD REPUBLIC INTERNATIONAL</t>
+          <t>COLUMBIA BANKING SYSTEM INC</t>
         </is>
       </c>
       <c r="K55" s="6" t="inlineStr">
@@ -28156,15 +28156,15 @@
     <row r="56">
       <c r="H56" s="6" t="inlineStr">
         <is>
-          <t>COLB</t>
+          <t>ORI</t>
         </is>
       </c>
       <c r="I56" s="61" t="n">
-        <v>0.00201168</v>
+        <v>0.00206549</v>
       </c>
       <c r="J56" s="6" t="inlineStr">
         <is>
-          <t>COLUMBIA BANKING SYSTEM INC</t>
+          <t>OLD REPUBLIC INTERNATIONAL</t>
         </is>
       </c>
       <c r="K56" s="6" t="inlineStr">
@@ -28185,7 +28185,7 @@
         </is>
       </c>
       <c r="I57" s="61" t="n">
-        <v>0.001886</v>
+        <v>0.00182647</v>
       </c>
       <c r="J57" s="6" t="inlineStr">
         <is>
@@ -28210,7 +28210,7 @@
         </is>
       </c>
       <c r="I58" s="61" t="n">
-        <v>0.0015801</v>
+        <v>0.00156608</v>
       </c>
       <c r="J58" s="6" t="inlineStr">
         <is>
@@ -28235,7 +28235,7 @@
         </is>
       </c>
       <c r="I59" s="61" t="n">
-        <v>0.00151255</v>
+        <v>0.00151419</v>
       </c>
       <c r="J59" s="6" t="inlineStr">
         <is>
@@ -28260,7 +28260,7 @@
         </is>
       </c>
       <c r="I60" s="61" t="n">
-        <v>0.00136119</v>
+        <v>0.00143015</v>
       </c>
       <c r="J60" s="6" t="inlineStr">
         <is>
@@ -28285,7 +28285,7 @@
         </is>
       </c>
       <c r="I61" s="61" t="n">
-        <v>0.00125791</v>
+        <v>0.00124874</v>
       </c>
       <c r="J61" s="6" t="inlineStr">
         <is>
@@ -28310,7 +28310,7 @@
         </is>
       </c>
       <c r="I62" s="61" t="n">
-        <v>0.00122662</v>
+        <v>0.00124717</v>
       </c>
       <c r="J62" s="6" t="inlineStr">
         <is>
@@ -28335,7 +28335,7 @@
         </is>
       </c>
       <c r="I63" s="61" t="n">
-        <v>0.00120113</v>
+        <v>0.00122874</v>
       </c>
       <c r="J63" s="6" t="inlineStr">
         <is>
@@ -28360,7 +28360,7 @@
         </is>
       </c>
       <c r="I64" s="61" t="n">
-        <v>0.0011653</v>
+        <v>0.00116009</v>
       </c>
       <c r="J64" s="6" t="inlineStr">
         <is>
@@ -28381,20 +28381,20 @@
     <row r="65">
       <c r="H65" s="6" t="inlineStr">
         <is>
-          <t>FHI</t>
+          <t>RHI</t>
         </is>
       </c>
       <c r="I65" s="61" t="n">
-        <v>0.0009790199999999999</v>
+        <v>0.00110026</v>
       </c>
       <c r="J65" s="6" t="inlineStr">
         <is>
-          <t>FEDERATED HERMES INC CLASS B</t>
+          <t>ROBERT HALF INC</t>
         </is>
       </c>
       <c r="K65" s="6" t="inlineStr">
         <is>
-          <t>Financials</t>
+          <t>Industrials</t>
         </is>
       </c>
       <c r="L65" s="6" t="inlineStr"/>
@@ -28406,15 +28406,15 @@
     <row r="66">
       <c r="H66" s="6" t="inlineStr">
         <is>
-          <t>MC</t>
+          <t>FHI</t>
         </is>
       </c>
       <c r="I66" s="61" t="n">
-        <v>0.00096866</v>
+        <v>0.0009682499999999999</v>
       </c>
       <c r="J66" s="6" t="inlineStr">
         <is>
-          <t>MOELIS CLASS A</t>
+          <t>FEDERATED HERMES INC CLASS B</t>
         </is>
       </c>
       <c r="K66" s="6" t="inlineStr">
@@ -28435,7 +28435,7 @@
         </is>
       </c>
       <c r="I67" s="61" t="n">
-        <v>0.0009356799999999999</v>
+        <v>0.0009633899999999999</v>
       </c>
       <c r="J67" s="6" t="inlineStr">
         <is>
@@ -28456,15 +28456,15 @@
     <row r="68">
       <c r="H68" s="6" t="inlineStr">
         <is>
-          <t>CVBF</t>
+          <t>MC</t>
         </is>
       </c>
       <c r="I68" s="61" t="n">
-        <v>0.00091526</v>
+        <v>0.00096317</v>
       </c>
       <c r="J68" s="6" t="inlineStr">
         <is>
-          <t>CVB FINANCIAL CORP</t>
+          <t>MOELIS CLASS A</t>
         </is>
       </c>
       <c r="K68" s="6" t="inlineStr">
@@ -28481,20 +28481,20 @@
     <row r="69">
       <c r="H69" s="6" t="inlineStr">
         <is>
-          <t>CWEN</t>
+          <t>CVBF</t>
         </is>
       </c>
       <c r="I69" s="61" t="n">
-        <v>0.00090426</v>
+        <v>0.00091373</v>
       </c>
       <c r="J69" s="6" t="inlineStr">
         <is>
-          <t>CLEARWAY ENERGY INC CLASS C</t>
+          <t>CVB FINANCIAL CORP</t>
         </is>
       </c>
       <c r="K69" s="6" t="inlineStr">
         <is>
-          <t>Utilities</t>
+          <t>Financials</t>
         </is>
       </c>
       <c r="L69" s="6" t="inlineStr"/>
@@ -28506,20 +28506,20 @@
     <row r="70">
       <c r="H70" s="6" t="inlineStr">
         <is>
-          <t>RHI</t>
+          <t>PAG</t>
         </is>
       </c>
       <c r="I70" s="61" t="n">
-        <v>0.0009002200000000001</v>
+        <v>0.00090142</v>
       </c>
       <c r="J70" s="6" t="inlineStr">
         <is>
-          <t>ROBERT HALF INC</t>
+          <t>PENSKE AUTOMOTIVE GROUP VOTING INC</t>
         </is>
       </c>
       <c r="K70" s="6" t="inlineStr">
         <is>
-          <t>Industrials</t>
+          <t>Consumer Discretionary</t>
         </is>
       </c>
       <c r="L70" s="6" t="inlineStr"/>
@@ -28531,20 +28531,20 @@
     <row r="71">
       <c r="H71" s="6" t="inlineStr">
         <is>
-          <t>PAG</t>
+          <t>CWEN</t>
         </is>
       </c>
       <c r="I71" s="61" t="n">
-        <v>0.00089693</v>
+        <v>0.0008986199999999999</v>
       </c>
       <c r="J71" s="6" t="inlineStr">
         <is>
-          <t>PENSKE AUTOMOTIVE GROUP VOTING INC</t>
+          <t>CLEARWAY ENERGY INC CLASS C</t>
         </is>
       </c>
       <c r="K71" s="6" t="inlineStr">
         <is>
-          <t>Consumer Discretionary</t>
+          <t>Utilities</t>
         </is>
       </c>
       <c r="L71" s="6" t="inlineStr"/>
@@ -28556,15 +28556,15 @@
     <row r="72">
       <c r="H72" s="6" t="inlineStr">
         <is>
-          <t>APAM</t>
+          <t>BANR</t>
         </is>
       </c>
       <c r="I72" s="61" t="n">
-        <v>0.00057898</v>
+        <v>0.0005681400000000001</v>
       </c>
       <c r="J72" s="6" t="inlineStr">
         <is>
-          <t>ARTISAN PARTNERS ASSET MANAGEMENT</t>
+          <t>BANNER CORP</t>
         </is>
       </c>
       <c r="K72" s="6" t="inlineStr">
@@ -28581,15 +28581,15 @@
     <row r="73">
       <c r="H73" s="6" t="inlineStr">
         <is>
-          <t>BANR</t>
+          <t>APAM</t>
         </is>
       </c>
       <c r="I73" s="61" t="n">
-        <v>0.00056443</v>
+        <v>0.00056726</v>
       </c>
       <c r="J73" s="6" t="inlineStr">
         <is>
-          <t>BANNER CORP</t>
+          <t>ARTISAN PARTNERS ASSET MANAGEMENT</t>
         </is>
       </c>
       <c r="K73" s="6" t="inlineStr">
@@ -28606,20 +28606,20 @@
     <row r="74">
       <c r="H74" s="6" t="inlineStr">
         <is>
-          <t>MZTI</t>
+          <t>OFG</t>
         </is>
       </c>
       <c r="I74" s="61" t="n">
-        <v>0.00052122</v>
+        <v>0.00051843</v>
       </c>
       <c r="J74" s="6" t="inlineStr">
         <is>
-          <t>MARZETTI</t>
+          <t>OFG BANCORP</t>
         </is>
       </c>
       <c r="K74" s="6" t="inlineStr">
         <is>
-          <t>Consumer Staples</t>
+          <t>Financials</t>
         </is>
       </c>
       <c r="L74" s="6" t="inlineStr"/>
@@ -28631,20 +28631,20 @@
     <row r="75">
       <c r="H75" s="6" t="inlineStr">
         <is>
-          <t>OFG</t>
+          <t>MZTI</t>
         </is>
       </c>
       <c r="I75" s="61" t="n">
-        <v>0.00051729</v>
+        <v>0.0005083900000000001</v>
       </c>
       <c r="J75" s="6" t="inlineStr">
         <is>
-          <t>OFG BANCORP</t>
+          <t>MARZETTI</t>
         </is>
       </c>
       <c r="K75" s="6" t="inlineStr">
         <is>
-          <t>Financials</t>
+          <t>Consumer Staples</t>
         </is>
       </c>
       <c r="L75" s="6" t="inlineStr"/>
@@ -28660,7 +28660,7 @@
         </is>
       </c>
       <c r="I76" s="61" t="n">
-        <v>0.00050476</v>
+        <v>0.00050305</v>
       </c>
       <c r="J76" s="6" t="inlineStr">
         <is>
@@ -28685,7 +28685,7 @@
         </is>
       </c>
       <c r="I77" s="61" t="n">
-        <v>0.0004856</v>
+        <v>0.00048028</v>
       </c>
       <c r="J77" s="6" t="inlineStr">
         <is>
@@ -28710,7 +28710,7 @@
         </is>
       </c>
       <c r="I78" s="61" t="n">
-        <v>0.0004796099999999999</v>
+        <v>0.00047681</v>
       </c>
       <c r="J78" s="6" t="inlineStr">
         <is>
@@ -28735,7 +28735,7 @@
         </is>
       </c>
       <c r="I79" s="61" t="n">
-        <v>0.00047885</v>
+        <v>0.00047403</v>
       </c>
       <c r="J79" s="6" t="inlineStr">
         <is>
@@ -28756,20 +28756,20 @@
     <row r="80">
       <c r="H80" s="6" t="inlineStr">
         <is>
-          <t>GABC</t>
+          <t>NSP</t>
         </is>
       </c>
       <c r="I80" s="61" t="n">
-        <v>0.00045857</v>
+        <v>0.00046603</v>
       </c>
       <c r="J80" s="6" t="inlineStr">
         <is>
-          <t>GERMAN AMERICAN BANCORP INC</t>
+          <t>INSPERITY</t>
         </is>
       </c>
       <c r="K80" s="6" t="inlineStr">
         <is>
-          <t>Financials</t>
+          <t>Industrials</t>
         </is>
       </c>
       <c r="L80" s="6" t="inlineStr"/>
@@ -28781,20 +28781,20 @@
     <row r="81">
       <c r="H81" s="6" t="inlineStr">
         <is>
-          <t>NSP</t>
+          <t>GABC</t>
         </is>
       </c>
       <c r="I81" s="61" t="n">
-        <v>0.00045599</v>
+        <v>0.00045787</v>
       </c>
       <c r="J81" s="6" t="inlineStr">
         <is>
-          <t>INSPERITY</t>
+          <t>GERMAN AMERICAN BANCORP INC</t>
         </is>
       </c>
       <c r="K81" s="6" t="inlineStr">
         <is>
-          <t>Industrials</t>
+          <t>Financials</t>
         </is>
       </c>
       <c r="L81" s="6" t="inlineStr"/>
@@ -28806,22 +28806,18 @@
     <row r="82">
       <c r="H82" s="6" t="inlineStr">
         <is>
-          <t>AGM</t>
+          <t>GVMXX</t>
         </is>
       </c>
       <c r="I82" s="61" t="n">
-        <v>0.00044824</v>
+        <v>0.00045314</v>
       </c>
       <c r="J82" s="6" t="inlineStr">
         <is>
-          <t>FEDERAL AGRICULTURAL MORTGAGE NON</t>
-        </is>
-      </c>
-      <c r="K82" s="6" t="inlineStr">
-        <is>
-          <t>Financials</t>
-        </is>
-      </c>
+          <t>SSC GOVERNMENT MM GVMXX</t>
+        </is>
+      </c>
+      <c r="K82" s="6" t="inlineStr"/>
       <c r="L82" s="6" t="inlineStr"/>
       <c r="M82" s="7">
         <f>IF(H82="","",IFERROR(VLOOKUP(K82,$P$5:$Q$15,2,FALSE),"현금·선물"))</f>
@@ -28831,18 +28827,22 @@
     <row r="83">
       <c r="H83" s="6" t="inlineStr">
         <is>
-          <t>GVMXX</t>
+          <t>AGM</t>
         </is>
       </c>
       <c r="I83" s="61" t="n">
-        <v>0.00043447</v>
+        <v>0.000446</v>
       </c>
       <c r="J83" s="6" t="inlineStr">
         <is>
-          <t>SSC GOVERNMENT MM GVMXX</t>
-        </is>
-      </c>
-      <c r="K83" s="6" t="inlineStr"/>
+          <t>FEDERAL AGRICULTURAL MORTGAGE NON</t>
+        </is>
+      </c>
+      <c r="K83" s="6" t="inlineStr">
+        <is>
+          <t>Financials</t>
+        </is>
+      </c>
       <c r="L83" s="6" t="inlineStr"/>
       <c r="M83" s="7">
         <f>IF(H83="","",IFERROR(VLOOKUP(K83,$P$5:$Q$15,2,FALSE),"현금·선물"))</f>
@@ -28856,7 +28856,7 @@
         </is>
       </c>
       <c r="I84" s="61" t="n">
-        <v>0.00042703</v>
+        <v>0.0004269499999999999</v>
       </c>
       <c r="J84" s="6" t="inlineStr">
         <is>
@@ -28881,7 +28881,7 @@
         </is>
       </c>
       <c r="I85" s="61" t="n">
-        <v>0.00041268</v>
+        <v>0.00041346</v>
       </c>
       <c r="J85" s="6" t="inlineStr">
         <is>
@@ -28906,7 +28906,7 @@
         </is>
       </c>
       <c r="I86" s="61" t="n">
-        <v>0.00037069</v>
+        <v>0.00037262</v>
       </c>
       <c r="J86" s="6" t="inlineStr">
         <is>
@@ -28931,7 +28931,7 @@
         </is>
       </c>
       <c r="I87" s="61" t="n">
-        <v>0.00035239</v>
+        <v>0.00034789</v>
       </c>
       <c r="J87" s="6" t="inlineStr">
         <is>
@@ -28956,7 +28956,7 @@
         </is>
       </c>
       <c r="I88" s="61" t="n">
-        <v>0.00034771</v>
+        <v>0.00034218</v>
       </c>
       <c r="J88" s="6" t="inlineStr">
         <is>
@@ -28981,7 +28981,7 @@
         </is>
       </c>
       <c r="I89" s="61" t="n">
-        <v>0.00032456</v>
+        <v>0.00031215</v>
       </c>
       <c r="J89" s="6" t="inlineStr">
         <is>
@@ -29006,7 +29006,7 @@
         </is>
       </c>
       <c r="I90" s="61" t="n">
-        <v>0.00028219</v>
+        <v>0.00027834</v>
       </c>
       <c r="J90" s="6" t="inlineStr">
         <is>
@@ -29031,7 +29031,7 @@
         </is>
       </c>
       <c r="I91" s="61" t="n">
-        <v>0.00025546</v>
+        <v>0.00025134</v>
       </c>
       <c r="J91" s="6" t="inlineStr">
         <is>
@@ -29056,7 +29056,7 @@
         </is>
       </c>
       <c r="I92" s="61" t="n">
-        <v>0.00025145</v>
+        <v>0.000239</v>
       </c>
       <c r="J92" s="6" t="inlineStr">
         <is>
@@ -29081,7 +29081,7 @@
         </is>
       </c>
       <c r="I93" s="61" t="n">
-        <v>0.00023099</v>
+        <v>0.00023141</v>
       </c>
       <c r="J93" s="6" t="inlineStr">
         <is>
@@ -29106,7 +29106,7 @@
         </is>
       </c>
       <c r="I94" s="61" t="n">
-        <v>0.00022652</v>
+        <v>0.00022679</v>
       </c>
       <c r="J94" s="6" t="inlineStr">
         <is>
@@ -29131,7 +29131,7 @@
         </is>
       </c>
       <c r="I95" s="61" t="n">
-        <v>0.00021034</v>
+        <v>0.00021104</v>
       </c>
       <c r="J95" s="6" t="inlineStr">
         <is>
@@ -29156,7 +29156,7 @@
         </is>
       </c>
       <c r="I96" s="61" t="n">
-        <v>0.00019589</v>
+        <v>0.00019677</v>
       </c>
       <c r="J96" s="6" t="inlineStr">
         <is>
@@ -29181,7 +29181,7 @@
         </is>
       </c>
       <c r="I97" s="61" t="n">
-        <v>0.00019368</v>
+        <v>0.00019569</v>
       </c>
       <c r="J97" s="6" t="inlineStr">
         <is>
@@ -29206,7 +29206,7 @@
         </is>
       </c>
       <c r="I98" s="61" t="n">
-        <v>0.00017816</v>
+        <v>0.00017441</v>
       </c>
       <c r="J98" s="6" t="inlineStr">
         <is>
@@ -29231,7 +29231,7 @@
         </is>
       </c>
       <c r="I99" s="61" t="n">
-        <v>0.00016466</v>
+        <v>0.00016544</v>
       </c>
       <c r="J99" s="6" t="inlineStr">
         <is>
@@ -29256,7 +29256,7 @@
         </is>
       </c>
       <c r="I100" s="61" t="n">
-        <v>0.0001306</v>
+        <v>0.00012952</v>
       </c>
       <c r="J100" s="6" t="inlineStr">
         <is>
@@ -29281,7 +29281,7 @@
         </is>
       </c>
       <c r="I101" s="61" t="n">
-        <v>0.00011739</v>
+        <v>0.00011666</v>
       </c>
       <c r="J101" s="6" t="inlineStr">
         <is>
@@ -29302,18 +29302,22 @@
     <row r="102">
       <c r="H102" s="6" t="inlineStr">
         <is>
-          <t>USD</t>
+          <t>ETD</t>
         </is>
       </c>
       <c r="I102" s="61" t="n">
-        <v>0.0001055</v>
+        <v>9.779e-05</v>
       </c>
       <c r="J102" s="6" t="inlineStr">
         <is>
-          <t>US DOLLAR</t>
-        </is>
-      </c>
-      <c r="K102" s="6" t="inlineStr"/>
+          <t>ETHAN ALLEN INTERIORS</t>
+        </is>
+      </c>
+      <c r="K102" s="6" t="inlineStr">
+        <is>
+          <t>Consumer Discretionary</t>
+        </is>
+      </c>
       <c r="L102" s="6" t="inlineStr"/>
       <c r="M102" s="7">
         <f>IF(H102="","",IFERROR(VLOOKUP(K102,$P$5:$Q$15,2,FALSE),"현금·선물"))</f>
@@ -29323,15 +29327,15 @@
     <row r="103">
       <c r="H103" s="6" t="inlineStr">
         <is>
-          <t>ETD</t>
+          <t>OXM</t>
         </is>
       </c>
       <c r="I103" s="61" t="n">
-        <v>9.903000000000001e-05</v>
+        <v>9.221e-05</v>
       </c>
       <c r="J103" s="6" t="inlineStr">
         <is>
-          <t>ETHAN ALLEN INTERIORS</t>
+          <t>OXFORD INDUSTRIES INC</t>
         </is>
       </c>
       <c r="K103" s="6" t="inlineStr">
@@ -29348,22 +29352,18 @@
     <row r="104">
       <c r="H104" s="6" t="inlineStr">
         <is>
-          <t>OXM</t>
+          <t>USD</t>
         </is>
       </c>
       <c r="I104" s="61" t="n">
-        <v>9.377000000000001e-05</v>
+        <v>9.174e-05</v>
       </c>
       <c r="J104" s="6" t="inlineStr">
         <is>
-          <t>OXFORD INDUSTRIES INC</t>
-        </is>
-      </c>
-      <c r="K104" s="6" t="inlineStr">
-        <is>
-          <t>Consumer Discretionary</t>
-        </is>
-      </c>
+          <t>US DOLLAR</t>
+        </is>
+      </c>
+      <c r="K104" s="6" t="inlineStr"/>
       <c r="L104" s="6" t="inlineStr"/>
       <c r="M104" s="7">
         <f>IF(H104="","",IFERROR(VLOOKUP(K104,$P$5:$Q$15,2,FALSE),"현금·선물"))</f>

</xml_diff>

<commit_message>
데이터 갱신: holdings,prices (2026-10-27)
</commit_message>
<xml_diff>
--- a/downloads/schd_dividend_tracker.xlsx
+++ b/downloads/schd_dividend_tracker.xlsx
@@ -1724,7 +1724,7 @@
     <row r="3">
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>최종 갱신: 2026-10-24 · 반영 범위: 2012년 1분기 ~ 2026년 3분기 (배당락 2026-09-23) · GitHub Actions 자동 생성</t>
+          <t>최종 갱신: 2026-10-27 · 반영 범위: 2012년 1분기 ~ 2026년 3분기 (배당락 2026-09-23) · GitHub Actions 자동 생성</t>
         </is>
       </c>
     </row>
@@ -5818,7 +5818,7 @@
       </c>
       <c r="H1" s="2" t="inlineStr">
         <is>
-          <t>출처: Yahoo Finance (종가: 주식분할 반영·배당 미조정 / adj: 배당 재투자 반영 수정주가) · 기준일 2026-10-20 · 3:1 분할(2024-10-11) 반영 가격</t>
+          <t>출처: Yahoo Finance (종가: 주식분할 반영·배당 미조정 / adj: 배당 재투자 반영 수정주가) · 기준일 2026-10-26 · 3:1 분할(2024-10-11) 반영 가격</t>
         </is>
       </c>
     </row>
@@ -6627,7 +6627,7 @@
         <v>13.1067</v>
       </c>
       <c r="D38" s="77" t="n">
-        <v>8.8355</v>
+        <v>8.835599999999999</v>
       </c>
       <c r="E38" s="58">
         <f>C38/C26-1</f>
@@ -7995,7 +7995,7 @@
         <v>17.9833</v>
       </c>
       <c r="D95" s="77" t="n">
-        <v>13.9255</v>
+        <v>13.9254</v>
       </c>
       <c r="E95" s="58">
         <f>C95/C83-1</f>
@@ -9123,7 +9123,7 @@
         <v>24.2067</v>
       </c>
       <c r="D142" s="77" t="n">
-        <v>21.5029</v>
+        <v>21.503</v>
       </c>
       <c r="E142" s="58">
         <f>C142/C130-1</f>
@@ -9555,7 +9555,7 @@
         <v>27.32</v>
       </c>
       <c r="D160" s="77" t="n">
-        <v>25.658</v>
+        <v>25.6579</v>
       </c>
       <c r="E160" s="58">
         <f>C160/C148-1</f>
@@ -9651,7 +9651,7 @@
         <v>25.82</v>
       </c>
       <c r="D164" s="77" t="n">
-        <v>24.468</v>
+        <v>24.4681</v>
       </c>
       <c r="E164" s="58">
         <f>C164/C152-1</f>
@@ -10077,13 +10077,13 @@
         </is>
       </c>
       <c r="B182" s="56" t="n">
-        <v>46315</v>
+        <v>46321</v>
       </c>
       <c r="C182" s="76" t="n">
-        <v>34.69</v>
+        <v>35.3</v>
       </c>
       <c r="D182" s="77" t="n">
-        <v>34.69</v>
+        <v>35.3</v>
       </c>
       <c r="E182" s="58">
         <f>C182/C170-1</f>
@@ -26257,11 +26257,11 @@
         </is>
       </c>
       <c r="B2" s="49" t="n">
-        <v>46318</v>
+        <v>46321</v>
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>← 이 날 종가로 계산한 비중. 그날 공식 파일을 못 받아 Schwab 공식 보유종목 CSV(2026-10-22)의 보유 주식 수 × 종가로 계산했습니다.</t>
+          <t>← 이 날 종가로 계산한 비중. 그날 공식 파일을 못 받아 Schwab 공식 보유종목 CSV(2026-10-23)의 보유 주식 수 × 종가로 계산했습니다.</t>
         </is>
       </c>
     </row>
@@ -26358,7 +26358,7 @@
         </is>
       </c>
       <c r="I5" s="61" t="n">
-        <v>0.04408678</v>
+        <v>0.046169</v>
       </c>
       <c r="J5" s="6" t="inlineStr">
         <is>
@@ -26412,15 +26412,15 @@
       </c>
       <c r="H6" s="6" t="inlineStr">
         <is>
-          <t>CVX</t>
+          <t>COP</t>
         </is>
       </c>
       <c r="I6" s="61" t="n">
-        <v>0.04345056999999999</v>
+        <v>0.04348015</v>
       </c>
       <c r="J6" s="6" t="inlineStr">
         <is>
-          <t>CHEVRON</t>
+          <t>CONOCOPHILLIPS</t>
         </is>
       </c>
       <c r="K6" s="6" t="inlineStr">
@@ -26430,7 +26430,7 @@
       </c>
       <c r="L6" s="6" t="inlineStr">
         <is>
-          <t>셰브론</t>
+          <t>코노코필립스</t>
         </is>
       </c>
       <c r="M6" s="7">
@@ -26470,15 +26470,15 @@
       </c>
       <c r="H7" s="6" t="inlineStr">
         <is>
-          <t>COP</t>
+          <t>CVX</t>
         </is>
       </c>
       <c r="I7" s="61" t="n">
-        <v>0.04331401999999999</v>
+        <v>0.04322924</v>
       </c>
       <c r="J7" s="6" t="inlineStr">
         <is>
-          <t>CONOCOPHILLIPS</t>
+          <t>CHEVRON</t>
         </is>
       </c>
       <c r="K7" s="6" t="inlineStr">
@@ -26488,7 +26488,7 @@
       </c>
       <c r="L7" s="6" t="inlineStr">
         <is>
-          <t>코노코필립스</t>
+          <t>셰브론</t>
         </is>
       </c>
       <c r="M7" s="7">
@@ -26532,7 +26532,7 @@
         </is>
       </c>
       <c r="I8" s="61" t="n">
-        <v>0.04303422</v>
+        <v>0.04274261</v>
       </c>
       <c r="J8" s="6" t="inlineStr">
         <is>
@@ -26586,25 +26586,25 @@
       </c>
       <c r="H9" s="6" t="inlineStr">
         <is>
-          <t>KO</t>
+          <t>QCOM</t>
         </is>
       </c>
       <c r="I9" s="61" t="n">
-        <v>0.04145703</v>
+        <v>0.04169852</v>
       </c>
       <c r="J9" s="6" t="inlineStr">
         <is>
-          <t>COCA-COLA</t>
+          <t>QUALCOMM</t>
         </is>
       </c>
       <c r="K9" s="6" t="inlineStr">
         <is>
-          <t>Consumer Staples</t>
+          <t>Information Technology</t>
         </is>
       </c>
       <c r="L9" s="6" t="inlineStr">
         <is>
-          <t>코카콜라</t>
+          <t>퀄컴</t>
         </is>
       </c>
       <c r="M9" s="7">
@@ -26644,25 +26644,25 @@
       </c>
       <c r="H10" s="6" t="inlineStr">
         <is>
-          <t>UNH</t>
+          <t>KO</t>
         </is>
       </c>
       <c r="I10" s="61" t="n">
-        <v>0.04127694</v>
+        <v>0.04145483</v>
       </c>
       <c r="J10" s="6" t="inlineStr">
         <is>
-          <t>UNITEDHEALTH GROUP</t>
+          <t>COCA-COLA</t>
         </is>
       </c>
       <c r="K10" s="6" t="inlineStr">
         <is>
-          <t>Health Care</t>
+          <t>Consumer Staples</t>
         </is>
       </c>
       <c r="L10" s="6" t="inlineStr">
         <is>
-          <t>유나이티드헬스</t>
+          <t>코카콜라</t>
         </is>
       </c>
       <c r="M10" s="7">
@@ -26702,25 +26702,25 @@
       </c>
       <c r="H11" s="6" t="inlineStr">
         <is>
-          <t>QCOM</t>
+          <t>UNH</t>
         </is>
       </c>
       <c r="I11" s="61" t="n">
-        <v>0.04083957</v>
+        <v>0.04054933</v>
       </c>
       <c r="J11" s="6" t="inlineStr">
         <is>
-          <t>QUALCOMM</t>
+          <t>UNITEDHEALTH GROUP</t>
         </is>
       </c>
       <c r="K11" s="6" t="inlineStr">
         <is>
-          <t>Information Technology</t>
+          <t>Health Care</t>
         </is>
       </c>
       <c r="L11" s="6" t="inlineStr">
         <is>
-          <t>퀄컴</t>
+          <t>유나이티드헬스</t>
         </is>
       </c>
       <c r="M11" s="7">
@@ -26760,25 +26760,25 @@
       </c>
       <c r="H12" s="6" t="inlineStr">
         <is>
-          <t>HD</t>
+          <t>AMGN</t>
         </is>
       </c>
       <c r="I12" s="61" t="n">
-        <v>0.03962082</v>
+        <v>0.03961854</v>
       </c>
       <c r="J12" s="6" t="inlineStr">
         <is>
-          <t>HOME DEPOT</t>
+          <t>AMGEN INC</t>
         </is>
       </c>
       <c r="K12" s="6" t="inlineStr">
         <is>
-          <t>Consumer Discretionary</t>
+          <t>Health Care</t>
         </is>
       </c>
       <c r="L12" s="6" t="inlineStr">
         <is>
-          <t>홈디포</t>
+          <t>암젠</t>
         </is>
       </c>
       <c r="M12" s="7">
@@ -26818,25 +26818,25 @@
       </c>
       <c r="H13" s="6" t="inlineStr">
         <is>
-          <t>AMGN</t>
+          <t>HD</t>
         </is>
       </c>
       <c r="I13" s="61" t="n">
-        <v>0.03913819</v>
+        <v>0.03956699</v>
       </c>
       <c r="J13" s="6" t="inlineStr">
         <is>
-          <t>AMGEN INC</t>
+          <t>HOME DEPOT</t>
         </is>
       </c>
       <c r="K13" s="6" t="inlineStr">
         <is>
-          <t>Health Care</t>
+          <t>Consumer Discretionary</t>
         </is>
       </c>
       <c r="L13" s="6" t="inlineStr">
         <is>
-          <t>암젠</t>
+          <t>홈디포</t>
         </is>
       </c>
       <c r="M13" s="7">
@@ -26880,7 +26880,7 @@
         </is>
       </c>
       <c r="I14" s="61" t="n">
-        <v>0.03812414</v>
+        <v>0.03803909</v>
       </c>
       <c r="J14" s="6" t="inlineStr">
         <is>
@@ -26924,15 +26924,15 @@
       </c>
       <c r="H15" s="6" t="inlineStr">
         <is>
-          <t>MRK</t>
+          <t>ABT</t>
         </is>
       </c>
       <c r="I15" s="61" t="n">
-        <v>0.0378005</v>
+        <v>0.03746365</v>
       </c>
       <c r="J15" s="6" t="inlineStr">
         <is>
-          <t>MERCK &amp; CO INC</t>
+          <t>ABBOTT LABORATORIES</t>
         </is>
       </c>
       <c r="K15" s="6" t="inlineStr">
@@ -26942,7 +26942,7 @@
       </c>
       <c r="L15" s="6" t="inlineStr">
         <is>
-          <t>머크</t>
+          <t>애보트</t>
         </is>
       </c>
       <c r="M15" s="7">
@@ -26972,15 +26972,15 @@
       </c>
       <c r="H16" s="6" t="inlineStr">
         <is>
-          <t>ABT</t>
+          <t>MRK</t>
         </is>
       </c>
       <c r="I16" s="61" t="n">
-        <v>0.0370401</v>
+        <v>0.03658987</v>
       </c>
       <c r="J16" s="6" t="inlineStr">
         <is>
-          <t>ABBOTT LABORATORIES</t>
+          <t>MERCK &amp; CO INC</t>
         </is>
       </c>
       <c r="K16" s="6" t="inlineStr">
@@ -26990,7 +26990,7 @@
       </c>
       <c r="L16" s="6" t="inlineStr">
         <is>
-          <t>애보트</t>
+          <t>머크</t>
         </is>
       </c>
       <c r="M16" s="7">
@@ -27014,7 +27014,7 @@
         </is>
       </c>
       <c r="I17" s="61" t="n">
-        <v>0.03648506</v>
+        <v>0.0361739</v>
       </c>
       <c r="J17" s="6" t="inlineStr">
         <is>
@@ -27052,7 +27052,7 @@
         </is>
       </c>
       <c r="I18" s="61" t="n">
-        <v>0.03508982</v>
+        <v>0.03386601</v>
       </c>
       <c r="J18" s="6" t="inlineStr">
         <is>
@@ -27077,25 +27077,25 @@
     <row r="19">
       <c r="H19" s="6" t="inlineStr">
         <is>
-          <t>BMY</t>
+          <t>LMT</t>
         </is>
       </c>
       <c r="I19" s="61" t="n">
-        <v>0.03002656</v>
+        <v>0.03084485</v>
       </c>
       <c r="J19" s="6" t="inlineStr">
         <is>
-          <t>BRISTOL MYERS SQUIBB</t>
+          <t>LOCKHEED MARTIN</t>
         </is>
       </c>
       <c r="K19" s="6" t="inlineStr">
         <is>
-          <t>Health Care</t>
+          <t>Industrials</t>
         </is>
       </c>
       <c r="L19" s="6" t="inlineStr">
         <is>
-          <t>브리스톨마이어스스퀴브</t>
+          <t>록히드마틴</t>
         </is>
       </c>
       <c r="M19" s="7">
@@ -27111,25 +27111,25 @@
       </c>
       <c r="H20" s="6" t="inlineStr">
         <is>
-          <t>MO</t>
+          <t>BMY</t>
         </is>
       </c>
       <c r="I20" s="61" t="n">
-        <v>0.02966608</v>
+        <v>0.03009173</v>
       </c>
       <c r="J20" s="6" t="inlineStr">
         <is>
-          <t>ALTRIA GROUP INC</t>
+          <t>BRISTOL MYERS SQUIBB</t>
         </is>
       </c>
       <c r="K20" s="6" t="inlineStr">
         <is>
-          <t>Consumer Staples</t>
+          <t>Health Care</t>
         </is>
       </c>
       <c r="L20" s="6" t="inlineStr">
         <is>
-          <t>알트리아</t>
+          <t>브리스톨마이어스스퀴브</t>
         </is>
       </c>
       <c r="M20" s="7">
@@ -27150,25 +27150,25 @@
       </c>
       <c r="H21" s="6" t="inlineStr">
         <is>
-          <t>LMT</t>
+          <t>MO</t>
         </is>
       </c>
       <c r="I21" s="61" t="n">
-        <v>0.02933715</v>
+        <v>0.02939226</v>
       </c>
       <c r="J21" s="6" t="inlineStr">
         <is>
-          <t>LOCKHEED MARTIN</t>
+          <t>ALTRIA GROUP INC</t>
         </is>
       </c>
       <c r="K21" s="6" t="inlineStr">
         <is>
-          <t>Industrials</t>
+          <t>Consumer Staples</t>
         </is>
       </c>
       <c r="L21" s="6" t="inlineStr">
         <is>
-          <t>록히드마틴</t>
+          <t>알트리아</t>
         </is>
       </c>
       <c r="M21" s="7">
@@ -27192,7 +27192,7 @@
         </is>
       </c>
       <c r="I22" s="61" t="n">
-        <v>0.02888952</v>
+        <v>0.02860236</v>
       </c>
       <c r="J22" s="6" t="inlineStr">
         <is>
@@ -27230,7 +27230,7 @@
         </is>
       </c>
       <c r="I23" s="61" t="n">
-        <v>0.02117156</v>
+        <v>0.02136829</v>
       </c>
       <c r="J23" s="6" t="inlineStr">
         <is>
@@ -27268,7 +27268,7 @@
         </is>
       </c>
       <c r="I24" s="61" t="n">
-        <v>0.02044531</v>
+        <v>0.02052788</v>
       </c>
       <c r="J24" s="6" t="inlineStr">
         <is>
@@ -27302,25 +27302,25 @@
       </c>
       <c r="H25" s="6" t="inlineStr">
         <is>
-          <t>CMCSA</t>
+          <t>SLB</t>
         </is>
       </c>
       <c r="I25" s="61" t="n">
-        <v>0.01920005</v>
+        <v>0.01883623</v>
       </c>
       <c r="J25" s="6" t="inlineStr">
         <is>
-          <t>COMCAST CLASS A</t>
+          <t>SLB</t>
         </is>
       </c>
       <c r="K25" s="6" t="inlineStr">
         <is>
-          <t>Communication Services</t>
+          <t>Energy</t>
         </is>
       </c>
       <c r="L25" s="6" t="inlineStr">
         <is>
-          <t>컴캐스트</t>
+          <t>SLB</t>
         </is>
       </c>
       <c r="M25" s="7">
@@ -27340,25 +27340,25 @@
       </c>
       <c r="H26" s="6" t="inlineStr">
         <is>
-          <t>SLB</t>
+          <t>CMCSA</t>
         </is>
       </c>
       <c r="I26" s="61" t="n">
-        <v>0.01882809</v>
+        <v>0.01865952</v>
       </c>
       <c r="J26" s="6" t="inlineStr">
         <is>
-          <t>SLB</t>
+          <t>COMCAST CLASS A</t>
         </is>
       </c>
       <c r="K26" s="6" t="inlineStr">
         <is>
-          <t>Energy</t>
+          <t>Communication Services</t>
         </is>
       </c>
       <c r="L26" s="6" t="inlineStr">
         <is>
-          <t>SLB</t>
+          <t>컴캐스트</t>
         </is>
       </c>
       <c r="M26" s="7">
@@ -27382,7 +27382,7 @@
         </is>
       </c>
       <c r="I27" s="61" t="n">
-        <v>0.01810611</v>
+        <v>0.01797452</v>
       </c>
       <c r="J27" s="6" t="inlineStr">
         <is>
@@ -27420,7 +27420,7 @@
         </is>
       </c>
       <c r="I28" s="61" t="n">
-        <v>0.0165886</v>
+        <v>0.01613016</v>
       </c>
       <c r="J28" s="6" t="inlineStr">
         <is>
@@ -27458,7 +27458,7 @@
         </is>
       </c>
       <c r="I29" s="61" t="n">
-        <v>0.01444304</v>
+        <v>0.01452372</v>
       </c>
       <c r="J29" s="6" t="inlineStr">
         <is>
@@ -27492,7 +27492,7 @@
         </is>
       </c>
       <c r="I30" s="61" t="n">
-        <v>0.01424178</v>
+        <v>0.01439619</v>
       </c>
       <c r="J30" s="6" t="inlineStr">
         <is>
@@ -27530,7 +27530,7 @@
         </is>
       </c>
       <c r="I31" s="61" t="n">
-        <v>0.0135155</v>
+        <v>0.01358198</v>
       </c>
       <c r="J31" s="6" t="inlineStr">
         <is>
@@ -27555,7 +27555,7 @@
         </is>
       </c>
       <c r="I32" s="61" t="n">
-        <v>0.01148761</v>
+        <v>0.01151425</v>
       </c>
       <c r="J32" s="6" t="inlineStr">
         <is>
@@ -27585,7 +27585,7 @@
         </is>
       </c>
       <c r="I33" s="61" t="n">
-        <v>0.01086293</v>
+        <v>0.01084481</v>
       </c>
       <c r="J33" s="6" t="inlineStr">
         <is>
@@ -27610,7 +27610,7 @@
         </is>
       </c>
       <c r="I34" s="61" t="n">
-        <v>0.009234529999999999</v>
+        <v>0.00910477</v>
       </c>
       <c r="J34" s="6" t="inlineStr">
         <is>
@@ -27635,7 +27635,7 @@
         </is>
       </c>
       <c r="I35" s="61" t="n">
-        <v>0.00903411</v>
+        <v>0.008855439999999999</v>
       </c>
       <c r="J35" s="6" t="inlineStr">
         <is>
@@ -27660,7 +27660,7 @@
         </is>
       </c>
       <c r="I36" s="61" t="n">
-        <v>0.008758409999999999</v>
+        <v>0.00871745</v>
       </c>
       <c r="J36" s="6" t="inlineStr">
         <is>
@@ -27685,7 +27685,7 @@
         </is>
       </c>
       <c r="I37" s="61" t="n">
-        <v>0.00653687</v>
+        <v>0.006526499999999999</v>
       </c>
       <c r="J37" s="6" t="inlineStr">
         <is>
@@ -27710,7 +27710,7 @@
         </is>
       </c>
       <c r="I38" s="61" t="n">
-        <v>0.00646902</v>
+        <v>0.00650634</v>
       </c>
       <c r="J38" s="6" t="inlineStr">
         <is>
@@ -27735,7 +27735,7 @@
         </is>
       </c>
       <c r="I39" s="61" t="n">
-        <v>0.00593399</v>
+        <v>0.005884899999999999</v>
       </c>
       <c r="J39" s="6" t="inlineStr">
         <is>
@@ -27760,7 +27760,7 @@
         </is>
       </c>
       <c r="I40" s="61" t="n">
-        <v>0.00579904</v>
+        <v>0.00582788</v>
       </c>
       <c r="J40" s="6" t="inlineStr">
         <is>
@@ -27785,7 +27785,7 @@
         </is>
       </c>
       <c r="I41" s="61" t="n">
-        <v>0.00576538</v>
+        <v>0.00578861</v>
       </c>
       <c r="J41" s="6" t="inlineStr">
         <is>
@@ -27810,7 +27810,7 @@
         </is>
       </c>
       <c r="I42" s="61" t="n">
-        <v>0.0053142</v>
+        <v>0.00527821</v>
       </c>
       <c r="J42" s="6" t="inlineStr">
         <is>
@@ -27835,7 +27835,7 @@
         </is>
       </c>
       <c r="I43" s="61" t="n">
-        <v>0.00505742</v>
+        <v>0.00513027</v>
       </c>
       <c r="J43" s="6" t="inlineStr">
         <is>
@@ -27860,7 +27860,7 @@
         </is>
       </c>
       <c r="I44" s="61" t="n">
-        <v>0.00499736</v>
+        <v>0.00493773</v>
       </c>
       <c r="J44" s="6" t="inlineStr">
         <is>
@@ -27885,7 +27885,7 @@
         </is>
       </c>
       <c r="I45" s="61" t="n">
-        <v>0.00472818</v>
+        <v>0.00463751</v>
       </c>
       <c r="J45" s="6" t="inlineStr">
         <is>
@@ -27910,7 +27910,7 @@
         </is>
       </c>
       <c r="I46" s="61" t="n">
-        <v>0.00449705</v>
+        <v>0.00463001</v>
       </c>
       <c r="J46" s="6" t="inlineStr">
         <is>
@@ -27935,7 +27935,7 @@
         </is>
       </c>
       <c r="I47" s="61" t="n">
-        <v>0.00441511</v>
+        <v>0.00442571</v>
       </c>
       <c r="J47" s="6" t="inlineStr">
         <is>
@@ -27956,20 +27956,20 @@
     <row r="48">
       <c r="H48" s="6" t="inlineStr">
         <is>
-          <t>GIS</t>
+          <t>APA</t>
         </is>
       </c>
       <c r="I48" s="61" t="n">
-        <v>0.00439673</v>
+        <v>0.00432752</v>
       </c>
       <c r="J48" s="6" t="inlineStr">
         <is>
-          <t>GENERAL MILLS INC</t>
+          <t>APA</t>
         </is>
       </c>
       <c r="K48" s="6" t="inlineStr">
         <is>
-          <t>Consumer Staples</t>
+          <t>Energy</t>
         </is>
       </c>
       <c r="L48" s="6" t="inlineStr"/>
@@ -27981,20 +27981,20 @@
     <row r="49">
       <c r="H49" s="6" t="inlineStr">
         <is>
-          <t>APA</t>
+          <t>EWBC</t>
         </is>
       </c>
       <c r="I49" s="61" t="n">
-        <v>0.0043474</v>
+        <v>0.00431709</v>
       </c>
       <c r="J49" s="6" t="inlineStr">
         <is>
-          <t>APA</t>
+          <t>EAST WEST BANCORP</t>
         </is>
       </c>
       <c r="K49" s="6" t="inlineStr">
         <is>
-          <t>Energy</t>
+          <t>Financials</t>
         </is>
       </c>
       <c r="L49" s="6" t="inlineStr"/>
@@ -28006,20 +28006,20 @@
     <row r="50">
       <c r="H50" s="6" t="inlineStr">
         <is>
-          <t>EWBC</t>
+          <t>GIS</t>
         </is>
       </c>
       <c r="I50" s="61" t="n">
-        <v>0.00429793</v>
+        <v>0.00430873</v>
       </c>
       <c r="J50" s="6" t="inlineStr">
         <is>
-          <t>EAST WEST BANCORP</t>
+          <t>GENERAL MILLS INC</t>
         </is>
       </c>
       <c r="K50" s="6" t="inlineStr">
         <is>
-          <t>Financials</t>
+          <t>Consumer Staples</t>
         </is>
       </c>
       <c r="L50" s="6" t="inlineStr"/>
@@ -28035,7 +28035,7 @@
         </is>
       </c>
       <c r="I51" s="61" t="n">
-        <v>0.00274762</v>
+        <v>0.0025973</v>
       </c>
       <c r="J51" s="6" t="inlineStr">
         <is>
@@ -28060,7 +28060,7 @@
         </is>
       </c>
       <c r="I52" s="61" t="n">
-        <v>0.00247547</v>
+        <v>0.00247497</v>
       </c>
       <c r="J52" s="6" t="inlineStr">
         <is>
@@ -28085,7 +28085,7 @@
         </is>
       </c>
       <c r="I53" s="61" t="n">
-        <v>0.00246148</v>
+        <v>0.00243118</v>
       </c>
       <c r="J53" s="6" t="inlineStr">
         <is>
@@ -28110,7 +28110,7 @@
         </is>
       </c>
       <c r="I54" s="61" t="n">
-        <v>0.00225104</v>
+        <v>0.00239598</v>
       </c>
       <c r="J54" s="6" t="inlineStr">
         <is>
@@ -28135,7 +28135,7 @@
         </is>
       </c>
       <c r="I55" s="61" t="n">
-        <v>0.00208524</v>
+        <v>0.00209885</v>
       </c>
       <c r="J55" s="6" t="inlineStr">
         <is>
@@ -28160,7 +28160,7 @@
         </is>
       </c>
       <c r="I56" s="61" t="n">
-        <v>0.00206549</v>
+        <v>0.00204011</v>
       </c>
       <c r="J56" s="6" t="inlineStr">
         <is>
@@ -28185,7 +28185,7 @@
         </is>
       </c>
       <c r="I57" s="61" t="n">
-        <v>0.00182647</v>
+        <v>0.00183693</v>
       </c>
       <c r="J57" s="6" t="inlineStr">
         <is>
@@ -28210,7 +28210,7 @@
         </is>
       </c>
       <c r="I58" s="61" t="n">
-        <v>0.00156608</v>
+        <v>0.00155222</v>
       </c>
       <c r="J58" s="6" t="inlineStr">
         <is>
@@ -28235,7 +28235,7 @@
         </is>
       </c>
       <c r="I59" s="61" t="n">
-        <v>0.00151419</v>
+        <v>0.00148222</v>
       </c>
       <c r="J59" s="6" t="inlineStr">
         <is>
@@ -28260,7 +28260,7 @@
         </is>
       </c>
       <c r="I60" s="61" t="n">
-        <v>0.00143015</v>
+        <v>0.00142633</v>
       </c>
       <c r="J60" s="6" t="inlineStr">
         <is>
@@ -28281,20 +28281,20 @@
     <row r="61">
       <c r="H61" s="6" t="inlineStr">
         <is>
-          <t>MTN</t>
+          <t>MSM</t>
         </is>
       </c>
       <c r="I61" s="61" t="n">
-        <v>0.00124874</v>
+        <v>0.00130045</v>
       </c>
       <c r="J61" s="6" t="inlineStr">
         <is>
-          <t>VAIL RESORTS</t>
+          <t>MSC INDUSTRIAL CLASS A</t>
         </is>
       </c>
       <c r="K61" s="6" t="inlineStr">
         <is>
-          <t>Consumer Discretionary</t>
+          <t>Industrials</t>
         </is>
       </c>
       <c r="L61" s="6" t="inlineStr"/>
@@ -28306,20 +28306,20 @@
     <row r="62">
       <c r="H62" s="6" t="inlineStr">
         <is>
-          <t>MSM</t>
+          <t>MTN</t>
         </is>
       </c>
       <c r="I62" s="61" t="n">
-        <v>0.00124717</v>
+        <v>0.00127277</v>
       </c>
       <c r="J62" s="6" t="inlineStr">
         <is>
-          <t>MSC INDUSTRIAL CLASS A</t>
+          <t>VAIL RESORTS</t>
         </is>
       </c>
       <c r="K62" s="6" t="inlineStr">
         <is>
-          <t>Industrials</t>
+          <t>Consumer Discretionary</t>
         </is>
       </c>
       <c r="L62" s="6" t="inlineStr"/>
@@ -28335,7 +28335,7 @@
         </is>
       </c>
       <c r="I63" s="61" t="n">
-        <v>0.00122874</v>
+        <v>0.0012227</v>
       </c>
       <c r="J63" s="6" t="inlineStr">
         <is>
@@ -28360,7 +28360,7 @@
         </is>
       </c>
       <c r="I64" s="61" t="n">
-        <v>0.00116009</v>
+        <v>0.00114217</v>
       </c>
       <c r="J64" s="6" t="inlineStr">
         <is>
@@ -28385,7 +28385,7 @@
         </is>
       </c>
       <c r="I65" s="61" t="n">
-        <v>0.00110026</v>
+        <v>0.00107896</v>
       </c>
       <c r="J65" s="6" t="inlineStr">
         <is>
@@ -28406,15 +28406,15 @@
     <row r="66">
       <c r="H66" s="6" t="inlineStr">
         <is>
-          <t>FHI</t>
+          <t>MC</t>
         </is>
       </c>
       <c r="I66" s="61" t="n">
-        <v>0.0009682499999999999</v>
+        <v>0.00097594</v>
       </c>
       <c r="J66" s="6" t="inlineStr">
         <is>
-          <t>FEDERATED HERMES INC CLASS B</t>
+          <t>MOELIS CLASS A</t>
         </is>
       </c>
       <c r="K66" s="6" t="inlineStr">
@@ -28431,20 +28431,20 @@
     <row r="67">
       <c r="H67" s="6" t="inlineStr">
         <is>
-          <t>KFY</t>
+          <t>FHI</t>
         </is>
       </c>
       <c r="I67" s="61" t="n">
-        <v>0.0009633899999999999</v>
+        <v>0.0009702900000000001</v>
       </c>
       <c r="J67" s="6" t="inlineStr">
         <is>
-          <t>KORN FERRY</t>
+          <t>FEDERATED HERMES INC CLASS B</t>
         </is>
       </c>
       <c r="K67" s="6" t="inlineStr">
         <is>
-          <t>Industrials</t>
+          <t>Financials</t>
         </is>
       </c>
       <c r="L67" s="6" t="inlineStr"/>
@@ -28456,20 +28456,20 @@
     <row r="68">
       <c r="H68" s="6" t="inlineStr">
         <is>
-          <t>MC</t>
+          <t>KFY</t>
         </is>
       </c>
       <c r="I68" s="61" t="n">
-        <v>0.00096317</v>
+        <v>0.0009701600000000001</v>
       </c>
       <c r="J68" s="6" t="inlineStr">
         <is>
-          <t>MOELIS CLASS A</t>
+          <t>KORN FERRY</t>
         </is>
       </c>
       <c r="K68" s="6" t="inlineStr">
         <is>
-          <t>Financials</t>
+          <t>Industrials</t>
         </is>
       </c>
       <c r="L68" s="6" t="inlineStr"/>
@@ -28485,7 +28485,7 @@
         </is>
       </c>
       <c r="I69" s="61" t="n">
-        <v>0.00091373</v>
+        <v>0.00091338</v>
       </c>
       <c r="J69" s="6" t="inlineStr">
         <is>
@@ -28506,20 +28506,20 @@
     <row r="70">
       <c r="H70" s="6" t="inlineStr">
         <is>
-          <t>PAG</t>
+          <t>CWEN</t>
         </is>
       </c>
       <c r="I70" s="61" t="n">
-        <v>0.00090142</v>
+        <v>0.00090731</v>
       </c>
       <c r="J70" s="6" t="inlineStr">
         <is>
-          <t>PENSKE AUTOMOTIVE GROUP VOTING INC</t>
+          <t>CLEARWAY ENERGY INC CLASS C</t>
         </is>
       </c>
       <c r="K70" s="6" t="inlineStr">
         <is>
-          <t>Consumer Discretionary</t>
+          <t>Utilities</t>
         </is>
       </c>
       <c r="L70" s="6" t="inlineStr"/>
@@ -28531,20 +28531,20 @@
     <row r="71">
       <c r="H71" s="6" t="inlineStr">
         <is>
-          <t>CWEN</t>
+          <t>PAG</t>
         </is>
       </c>
       <c r="I71" s="61" t="n">
-        <v>0.0008986199999999999</v>
+        <v>0.00090034</v>
       </c>
       <c r="J71" s="6" t="inlineStr">
         <is>
-          <t>CLEARWAY ENERGY INC CLASS C</t>
+          <t>PENSKE AUTOMOTIVE GROUP VOTING INC</t>
         </is>
       </c>
       <c r="K71" s="6" t="inlineStr">
         <is>
-          <t>Utilities</t>
+          <t>Consumer Discretionary</t>
         </is>
       </c>
       <c r="L71" s="6" t="inlineStr"/>
@@ -28560,7 +28560,7 @@
         </is>
       </c>
       <c r="I72" s="61" t="n">
-        <v>0.0005681400000000001</v>
+        <v>0.00056977</v>
       </c>
       <c r="J72" s="6" t="inlineStr">
         <is>
@@ -28585,7 +28585,7 @@
         </is>
       </c>
       <c r="I73" s="61" t="n">
-        <v>0.00056726</v>
+        <v>0.00056338</v>
       </c>
       <c r="J73" s="6" t="inlineStr">
         <is>
@@ -28610,7 +28610,7 @@
         </is>
       </c>
       <c r="I74" s="61" t="n">
-        <v>0.00051843</v>
+        <v>0.00052084</v>
       </c>
       <c r="J74" s="6" t="inlineStr">
         <is>
@@ -28635,7 +28635,7 @@
         </is>
       </c>
       <c r="I75" s="61" t="n">
-        <v>0.0005083900000000001</v>
+        <v>0.00050793</v>
       </c>
       <c r="J75" s="6" t="inlineStr">
         <is>
@@ -28660,7 +28660,7 @@
         </is>
       </c>
       <c r="I76" s="61" t="n">
-        <v>0.00050305</v>
+        <v>0.0005036</v>
       </c>
       <c r="J76" s="6" t="inlineStr">
         <is>
@@ -28685,7 +28685,7 @@
         </is>
       </c>
       <c r="I77" s="61" t="n">
-        <v>0.00048028</v>
+        <v>0.00048119</v>
       </c>
       <c r="J77" s="6" t="inlineStr">
         <is>
@@ -28710,7 +28710,7 @@
         </is>
       </c>
       <c r="I78" s="61" t="n">
-        <v>0.00047681</v>
+        <v>0.00047939</v>
       </c>
       <c r="J78" s="6" t="inlineStr">
         <is>
@@ -28731,22 +28731,18 @@
     <row r="79">
       <c r="H79" s="6" t="inlineStr">
         <is>
-          <t>WU</t>
+          <t>GVMXX</t>
         </is>
       </c>
       <c r="I79" s="61" t="n">
-        <v>0.00047403</v>
+        <v>0.00047706</v>
       </c>
       <c r="J79" s="6" t="inlineStr">
         <is>
-          <t>WESTERN UNION</t>
-        </is>
-      </c>
-      <c r="K79" s="6" t="inlineStr">
-        <is>
-          <t>Financials</t>
-        </is>
-      </c>
+          <t>SSC GOVERNMENT MM GVMXX</t>
+        </is>
+      </c>
+      <c r="K79" s="6" t="inlineStr"/>
       <c r="L79" s="6" t="inlineStr"/>
       <c r="M79" s="7">
         <f>IF(H79="","",IFERROR(VLOOKUP(K79,$P$5:$Q$15,2,FALSE),"현금·선물"))</f>
@@ -28756,20 +28752,20 @@
     <row r="80">
       <c r="H80" s="6" t="inlineStr">
         <is>
-          <t>NSP</t>
+          <t>WU</t>
         </is>
       </c>
       <c r="I80" s="61" t="n">
-        <v>0.00046603</v>
+        <v>0.00046433</v>
       </c>
       <c r="J80" s="6" t="inlineStr">
         <is>
-          <t>INSPERITY</t>
+          <t>WESTERN UNION</t>
         </is>
       </c>
       <c r="K80" s="6" t="inlineStr">
         <is>
-          <t>Industrials</t>
+          <t>Financials</t>
         </is>
       </c>
       <c r="L80" s="6" t="inlineStr"/>
@@ -28781,20 +28777,20 @@
     <row r="81">
       <c r="H81" s="6" t="inlineStr">
         <is>
-          <t>GABC</t>
+          <t>NSP</t>
         </is>
       </c>
       <c r="I81" s="61" t="n">
-        <v>0.00045787</v>
+        <v>0.00046177</v>
       </c>
       <c r="J81" s="6" t="inlineStr">
         <is>
-          <t>GERMAN AMERICAN BANCORP INC</t>
+          <t>INSPERITY</t>
         </is>
       </c>
       <c r="K81" s="6" t="inlineStr">
         <is>
-          <t>Financials</t>
+          <t>Industrials</t>
         </is>
       </c>
       <c r="L81" s="6" t="inlineStr"/>
@@ -28806,18 +28802,22 @@
     <row r="82">
       <c r="H82" s="6" t="inlineStr">
         <is>
-          <t>GVMXX</t>
+          <t>GABC</t>
         </is>
       </c>
       <c r="I82" s="61" t="n">
-        <v>0.00045314</v>
+        <v>0.00046028</v>
       </c>
       <c r="J82" s="6" t="inlineStr">
         <is>
-          <t>SSC GOVERNMENT MM GVMXX</t>
-        </is>
-      </c>
-      <c r="K82" s="6" t="inlineStr"/>
+          <t>GERMAN AMERICAN BANCORP INC</t>
+        </is>
+      </c>
+      <c r="K82" s="6" t="inlineStr">
+        <is>
+          <t>Financials</t>
+        </is>
+      </c>
       <c r="L82" s="6" t="inlineStr"/>
       <c r="M82" s="7">
         <f>IF(H82="","",IFERROR(VLOOKUP(K82,$P$5:$Q$15,2,FALSE),"현금·선물"))</f>
@@ -28831,7 +28831,7 @@
         </is>
       </c>
       <c r="I83" s="61" t="n">
-        <v>0.000446</v>
+        <v>0.00044801</v>
       </c>
       <c r="J83" s="6" t="inlineStr">
         <is>
@@ -28856,7 +28856,7 @@
         </is>
       </c>
       <c r="I84" s="61" t="n">
-        <v>0.0004269499999999999</v>
+        <v>0.00043115</v>
       </c>
       <c r="J84" s="6" t="inlineStr">
         <is>
@@ -28881,7 +28881,7 @@
         </is>
       </c>
       <c r="I85" s="61" t="n">
-        <v>0.00041346</v>
+        <v>0.00041527</v>
       </c>
       <c r="J85" s="6" t="inlineStr">
         <is>
@@ -28906,7 +28906,7 @@
         </is>
       </c>
       <c r="I86" s="61" t="n">
-        <v>0.00037262</v>
+        <v>0.00037503</v>
       </c>
       <c r="J86" s="6" t="inlineStr">
         <is>
@@ -28931,7 +28931,7 @@
         </is>
       </c>
       <c r="I87" s="61" t="n">
-        <v>0.00034789</v>
+        <v>0.0003644399999999999</v>
       </c>
       <c r="J87" s="6" t="inlineStr">
         <is>
@@ -28956,7 +28956,7 @@
         </is>
       </c>
       <c r="I88" s="61" t="n">
-        <v>0.00034218</v>
+        <v>0.00034244</v>
       </c>
       <c r="J88" s="6" t="inlineStr">
         <is>
@@ -28981,7 +28981,7 @@
         </is>
       </c>
       <c r="I89" s="61" t="n">
-        <v>0.00031215</v>
+        <v>0.00031166</v>
       </c>
       <c r="J89" s="6" t="inlineStr">
         <is>
@@ -29006,7 +29006,7 @@
         </is>
       </c>
       <c r="I90" s="61" t="n">
-        <v>0.00027834</v>
+        <v>0.00027665</v>
       </c>
       <c r="J90" s="6" t="inlineStr">
         <is>
@@ -29031,7 +29031,7 @@
         </is>
       </c>
       <c r="I91" s="61" t="n">
-        <v>0.00025134</v>
+        <v>0.00025171</v>
       </c>
       <c r="J91" s="6" t="inlineStr">
         <is>
@@ -29056,7 +29056,7 @@
         </is>
       </c>
       <c r="I92" s="61" t="n">
-        <v>0.000239</v>
+        <v>0.00023786</v>
       </c>
       <c r="J92" s="6" t="inlineStr">
         <is>
@@ -29081,7 +29081,7 @@
         </is>
       </c>
       <c r="I93" s="61" t="n">
-        <v>0.00023141</v>
+        <v>0.00023164</v>
       </c>
       <c r="J93" s="6" t="inlineStr">
         <is>
@@ -29106,7 +29106,7 @@
         </is>
       </c>
       <c r="I94" s="61" t="n">
-        <v>0.00022679</v>
+        <v>0.00022693</v>
       </c>
       <c r="J94" s="6" t="inlineStr">
         <is>
@@ -29131,7 +29131,7 @@
         </is>
       </c>
       <c r="I95" s="61" t="n">
-        <v>0.00021104</v>
+        <v>0.00021275</v>
       </c>
       <c r="J95" s="6" t="inlineStr">
         <is>
@@ -29156,7 +29156,7 @@
         </is>
       </c>
       <c r="I96" s="61" t="n">
-        <v>0.00019677</v>
+        <v>0.00019693</v>
       </c>
       <c r="J96" s="6" t="inlineStr">
         <is>
@@ -29181,7 +29181,7 @@
         </is>
       </c>
       <c r="I97" s="61" t="n">
-        <v>0.00019569</v>
+        <v>0.00019513</v>
       </c>
       <c r="J97" s="6" t="inlineStr">
         <is>
@@ -29206,7 +29206,7 @@
         </is>
       </c>
       <c r="I98" s="61" t="n">
-        <v>0.00017441</v>
+        <v>0.00017381</v>
       </c>
       <c r="J98" s="6" t="inlineStr">
         <is>
@@ -29231,7 +29231,7 @@
         </is>
       </c>
       <c r="I99" s="61" t="n">
-        <v>0.00016544</v>
+        <v>0.00016662</v>
       </c>
       <c r="J99" s="6" t="inlineStr">
         <is>
@@ -29256,7 +29256,7 @@
         </is>
       </c>
       <c r="I100" s="61" t="n">
-        <v>0.00012952</v>
+        <v>0.00012907</v>
       </c>
       <c r="J100" s="6" t="inlineStr">
         <is>
@@ -29281,7 +29281,7 @@
         </is>
       </c>
       <c r="I101" s="61" t="n">
-        <v>0.00011666</v>
+        <v>0.00011629</v>
       </c>
       <c r="J101" s="6" t="inlineStr">
         <is>
@@ -29306,7 +29306,7 @@
         </is>
       </c>
       <c r="I102" s="61" t="n">
-        <v>9.779e-05</v>
+        <v>9.601999999999999e-05</v>
       </c>
       <c r="J102" s="6" t="inlineStr">
         <is>
@@ -29327,22 +29327,18 @@
     <row r="103">
       <c r="H103" s="6" t="inlineStr">
         <is>
-          <t>OXM</t>
+          <t>USD</t>
         </is>
       </c>
       <c r="I103" s="61" t="n">
-        <v>9.221e-05</v>
+        <v>9.407999999999999e-05</v>
       </c>
       <c r="J103" s="6" t="inlineStr">
         <is>
-          <t>OXFORD INDUSTRIES INC</t>
-        </is>
-      </c>
-      <c r="K103" s="6" t="inlineStr">
-        <is>
-          <t>Consumer Discretionary</t>
-        </is>
-      </c>
+          <t>US DOLLAR</t>
+        </is>
+      </c>
+      <c r="K103" s="6" t="inlineStr"/>
       <c r="L103" s="6" t="inlineStr"/>
       <c r="M103" s="7">
         <f>IF(H103="","",IFERROR(VLOOKUP(K103,$P$5:$Q$15,2,FALSE),"현금·선물"))</f>
@@ -29352,18 +29348,22 @@
     <row r="104">
       <c r="H104" s="6" t="inlineStr">
         <is>
-          <t>USD</t>
+          <t>OXM</t>
         </is>
       </c>
       <c r="I104" s="61" t="n">
-        <v>9.174e-05</v>
+        <v>9.129e-05</v>
       </c>
       <c r="J104" s="6" t="inlineStr">
         <is>
-          <t>US DOLLAR</t>
-        </is>
-      </c>
-      <c r="K104" s="6" t="inlineStr"/>
+          <t>OXFORD INDUSTRIES INC</t>
+        </is>
+      </c>
+      <c r="K104" s="6" t="inlineStr">
+        <is>
+          <t>Consumer Discretionary</t>
+        </is>
+      </c>
       <c r="L104" s="6" t="inlineStr"/>
       <c r="M104" s="7">
         <f>IF(H104="","",IFERROR(VLOOKUP(K104,$P$5:$Q$15,2,FALSE),"현금·선물"))</f>

</xml_diff>

<commit_message>
데이터 갱신: holdings (2026-10-28)
</commit_message>
<xml_diff>
--- a/downloads/schd_dividend_tracker.xlsx
+++ b/downloads/schd_dividend_tracker.xlsx
@@ -1724,7 +1724,7 @@
     <row r="3">
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>최종 갱신: 2026-10-27 · 반영 범위: 2012년 1분기 ~ 2026년 3분기 (배당락 2026-09-23) · GitHub Actions 자동 생성</t>
+          <t>최종 갱신: 2026-10-28 · 반영 범위: 2012년 1분기 ~ 2026년 3분기 (배당락 2026-09-23) · GitHub Actions 자동 생성</t>
         </is>
       </c>
     </row>
@@ -26257,11 +26257,11 @@
         </is>
       </c>
       <c r="B2" s="49" t="n">
-        <v>46321</v>
+        <v>46322</v>
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>← 이 날 종가로 계산한 비중. 그날 공식 파일을 못 받아 Schwab 공식 보유종목 CSV(2026-10-23)의 보유 주식 수 × 종가로 계산했습니다.</t>
+          <t>← 이 날 종가로 계산한 비중. 그날 공식 파일을 못 받아 Schwab 공식 보유종목 CSV(2026-10-26)의 보유 주식 수 × 종가로 계산했습니다.</t>
         </is>
       </c>
     </row>
@@ -26358,7 +26358,7 @@
         </is>
       </c>
       <c r="I5" s="61" t="n">
-        <v>0.046169</v>
+        <v>0.04804111</v>
       </c>
       <c r="J5" s="6" t="inlineStr">
         <is>
@@ -26412,25 +26412,25 @@
       </c>
       <c r="H6" s="6" t="inlineStr">
         <is>
-          <t>COP</t>
+          <t>QCOM</t>
         </is>
       </c>
       <c r="I6" s="61" t="n">
-        <v>0.04348015</v>
+        <v>0.04293930999999999</v>
       </c>
       <c r="J6" s="6" t="inlineStr">
         <is>
-          <t>CONOCOPHILLIPS</t>
+          <t>QUALCOMM</t>
         </is>
       </c>
       <c r="K6" s="6" t="inlineStr">
         <is>
-          <t>Energy</t>
+          <t>Information Technology</t>
         </is>
       </c>
       <c r="L6" s="6" t="inlineStr">
         <is>
-          <t>코노코필립스</t>
+          <t>퀄컴</t>
         </is>
       </c>
       <c r="M6" s="7">
@@ -26470,25 +26470,25 @@
       </c>
       <c r="H7" s="6" t="inlineStr">
         <is>
-          <t>CVX</t>
+          <t>PG</t>
         </is>
       </c>
       <c r="I7" s="61" t="n">
-        <v>0.04322924</v>
+        <v>0.04273715</v>
       </c>
       <c r="J7" s="6" t="inlineStr">
         <is>
-          <t>CHEVRON</t>
+          <t>PROCTER &amp; GAMBLE</t>
         </is>
       </c>
       <c r="K7" s="6" t="inlineStr">
         <is>
-          <t>Energy</t>
+          <t>Consumer Staples</t>
         </is>
       </c>
       <c r="L7" s="6" t="inlineStr">
         <is>
-          <t>셰브론</t>
+          <t>프록터앤드갬블</t>
         </is>
       </c>
       <c r="M7" s="7">
@@ -26528,25 +26528,25 @@
       </c>
       <c r="H8" s="6" t="inlineStr">
         <is>
-          <t>PG</t>
+          <t>CVX</t>
         </is>
       </c>
       <c r="I8" s="61" t="n">
-        <v>0.04274261</v>
+        <v>0.04270364</v>
       </c>
       <c r="J8" s="6" t="inlineStr">
         <is>
-          <t>PROCTER &amp; GAMBLE</t>
+          <t>CHEVRON</t>
         </is>
       </c>
       <c r="K8" s="6" t="inlineStr">
         <is>
-          <t>Consumer Staples</t>
+          <t>Energy</t>
         </is>
       </c>
       <c r="L8" s="6" t="inlineStr">
         <is>
-          <t>프록터앤드갬블</t>
+          <t>셰브론</t>
         </is>
       </c>
       <c r="M8" s="7">
@@ -26586,25 +26586,25 @@
       </c>
       <c r="H9" s="6" t="inlineStr">
         <is>
-          <t>QCOM</t>
+          <t>COP</t>
         </is>
       </c>
       <c r="I9" s="61" t="n">
-        <v>0.04169852</v>
+        <v>0.04267935</v>
       </c>
       <c r="J9" s="6" t="inlineStr">
         <is>
-          <t>QUALCOMM</t>
+          <t>CONOCOPHILLIPS</t>
         </is>
       </c>
       <c r="K9" s="6" t="inlineStr">
         <is>
-          <t>Information Technology</t>
+          <t>Energy</t>
         </is>
       </c>
       <c r="L9" s="6" t="inlineStr">
         <is>
-          <t>퀄컴</t>
+          <t>코노코필립스</t>
         </is>
       </c>
       <c r="M9" s="7">
@@ -26648,7 +26648,7 @@
         </is>
       </c>
       <c r="I10" s="61" t="n">
-        <v>0.04145483</v>
+        <v>0.04094653</v>
       </c>
       <c r="J10" s="6" t="inlineStr">
         <is>
@@ -26706,7 +26706,7 @@
         </is>
       </c>
       <c r="I11" s="61" t="n">
-        <v>0.04054933</v>
+        <v>0.04068892</v>
       </c>
       <c r="J11" s="6" t="inlineStr">
         <is>
@@ -26764,7 +26764,7 @@
         </is>
       </c>
       <c r="I12" s="61" t="n">
-        <v>0.03961854</v>
+        <v>0.04008198</v>
       </c>
       <c r="J12" s="6" t="inlineStr">
         <is>
@@ -26822,7 +26822,7 @@
         </is>
       </c>
       <c r="I13" s="61" t="n">
-        <v>0.03956699</v>
+        <v>0.03962369</v>
       </c>
       <c r="J13" s="6" t="inlineStr">
         <is>
@@ -26880,7 +26880,7 @@
         </is>
       </c>
       <c r="I14" s="61" t="n">
-        <v>0.03803909</v>
+        <v>0.03764625</v>
       </c>
       <c r="J14" s="6" t="inlineStr">
         <is>
@@ -26924,15 +26924,15 @@
       </c>
       <c r="H15" s="6" t="inlineStr">
         <is>
-          <t>ABT</t>
+          <t>MRK</t>
         </is>
       </c>
       <c r="I15" s="61" t="n">
-        <v>0.03746365</v>
+        <v>0.03705987</v>
       </c>
       <c r="J15" s="6" t="inlineStr">
         <is>
-          <t>ABBOTT LABORATORIES</t>
+          <t>MERCK &amp; CO INC</t>
         </is>
       </c>
       <c r="K15" s="6" t="inlineStr">
@@ -26942,7 +26942,7 @@
       </c>
       <c r="L15" s="6" t="inlineStr">
         <is>
-          <t>애보트</t>
+          <t>머크</t>
         </is>
       </c>
       <c r="M15" s="7">
@@ -26972,15 +26972,15 @@
       </c>
       <c r="H16" s="6" t="inlineStr">
         <is>
-          <t>MRK</t>
+          <t>ABT</t>
         </is>
       </c>
       <c r="I16" s="61" t="n">
-        <v>0.03658987</v>
+        <v>0.03698267</v>
       </c>
       <c r="J16" s="6" t="inlineStr">
         <is>
-          <t>MERCK &amp; CO INC</t>
+          <t>ABBOTT LABORATORIES</t>
         </is>
       </c>
       <c r="K16" s="6" t="inlineStr">
@@ -26990,7 +26990,7 @@
       </c>
       <c r="L16" s="6" t="inlineStr">
         <is>
-          <t>머크</t>
+          <t>애보트</t>
         </is>
       </c>
       <c r="M16" s="7">
@@ -27010,25 +27010,25 @@
       </c>
       <c r="H17" s="6" t="inlineStr">
         <is>
-          <t>ACN</t>
+          <t>VZ</t>
         </is>
       </c>
       <c r="I17" s="61" t="n">
-        <v>0.0361739</v>
+        <v>0.03466334</v>
       </c>
       <c r="J17" s="6" t="inlineStr">
         <is>
-          <t>ACCENTURE PLC CLASS A</t>
+          <t>VERIZON COMMUNICATIONS INC</t>
         </is>
       </c>
       <c r="K17" s="6" t="inlineStr">
         <is>
-          <t>Information Technology</t>
+          <t>Communication Services</t>
         </is>
       </c>
       <c r="L17" s="6" t="inlineStr">
         <is>
-          <t>액센츄어</t>
+          <t>버라이즌</t>
         </is>
       </c>
       <c r="M17" s="7">
@@ -27048,25 +27048,25 @@
       </c>
       <c r="H18" s="6" t="inlineStr">
         <is>
-          <t>VZ</t>
+          <t>ACN</t>
         </is>
       </c>
       <c r="I18" s="61" t="n">
-        <v>0.03386601</v>
+        <v>0.03455249</v>
       </c>
       <c r="J18" s="6" t="inlineStr">
         <is>
-          <t>VERIZON COMMUNICATIONS INC</t>
+          <t>ACCENTURE PLC CLASS A</t>
         </is>
       </c>
       <c r="K18" s="6" t="inlineStr">
         <is>
-          <t>Communication Services</t>
+          <t>Information Technology</t>
         </is>
       </c>
       <c r="L18" s="6" t="inlineStr">
         <is>
-          <t>버라이즌</t>
+          <t>액센츄어</t>
         </is>
       </c>
       <c r="M18" s="7">
@@ -27081,7 +27081,7 @@
         </is>
       </c>
       <c r="I19" s="61" t="n">
-        <v>0.03084485</v>
+        <v>0.03037897</v>
       </c>
       <c r="J19" s="6" t="inlineStr">
         <is>
@@ -27115,7 +27115,7 @@
         </is>
       </c>
       <c r="I20" s="61" t="n">
-        <v>0.03009173</v>
+        <v>0.03018884</v>
       </c>
       <c r="J20" s="6" t="inlineStr">
         <is>
@@ -27154,7 +27154,7 @@
         </is>
       </c>
       <c r="I21" s="61" t="n">
-        <v>0.02939226</v>
+        <v>0.02946372</v>
       </c>
       <c r="J21" s="6" t="inlineStr">
         <is>
@@ -27192,7 +27192,7 @@
         </is>
       </c>
       <c r="I22" s="61" t="n">
-        <v>0.02860236</v>
+        <v>0.02795858</v>
       </c>
       <c r="J22" s="6" t="inlineStr">
         <is>
@@ -27230,7 +27230,7 @@
         </is>
       </c>
       <c r="I23" s="61" t="n">
-        <v>0.02136829</v>
+        <v>0.02103275</v>
       </c>
       <c r="J23" s="6" t="inlineStr">
         <is>
@@ -27268,7 +27268,7 @@
         </is>
       </c>
       <c r="I24" s="61" t="n">
-        <v>0.02052788</v>
+        <v>0.0202892</v>
       </c>
       <c r="J24" s="6" t="inlineStr">
         <is>
@@ -27306,7 +27306,7 @@
         </is>
       </c>
       <c r="I25" s="61" t="n">
-        <v>0.01883623</v>
+        <v>0.01927179</v>
       </c>
       <c r="J25" s="6" t="inlineStr">
         <is>
@@ -27340,25 +27340,25 @@
       </c>
       <c r="H26" s="6" t="inlineStr">
         <is>
-          <t>CMCSA</t>
+          <t>UPS</t>
         </is>
       </c>
       <c r="I26" s="61" t="n">
-        <v>0.01865952</v>
+        <v>0.01908826</v>
       </c>
       <c r="J26" s="6" t="inlineStr">
         <is>
-          <t>COMCAST CLASS A</t>
+          <t>UNITED PARCEL SERVICE INC CLASS B</t>
         </is>
       </c>
       <c r="K26" s="6" t="inlineStr">
         <is>
-          <t>Communication Services</t>
+          <t>Industrials</t>
         </is>
       </c>
       <c r="L26" s="6" t="inlineStr">
         <is>
-          <t>컴캐스트</t>
+          <t>UPS</t>
         </is>
       </c>
       <c r="M26" s="7">
@@ -27378,25 +27378,25 @@
       </c>
       <c r="H27" s="6" t="inlineStr">
         <is>
-          <t>UPS</t>
+          <t>CMCSA</t>
         </is>
       </c>
       <c r="I27" s="61" t="n">
-        <v>0.01797452</v>
+        <v>0.01855952</v>
       </c>
       <c r="J27" s="6" t="inlineStr">
         <is>
-          <t>UNITED PARCEL SERVICE INC CLASS B</t>
+          <t>COMCAST CLASS A</t>
         </is>
       </c>
       <c r="K27" s="6" t="inlineStr">
         <is>
-          <t>Industrials</t>
+          <t>Communication Services</t>
         </is>
       </c>
       <c r="L27" s="6" t="inlineStr">
         <is>
-          <t>UPS</t>
+          <t>컴캐스트</t>
         </is>
       </c>
       <c r="M27" s="7">
@@ -27420,7 +27420,7 @@
         </is>
       </c>
       <c r="I28" s="61" t="n">
-        <v>0.01613016</v>
+        <v>0.01614128</v>
       </c>
       <c r="J28" s="6" t="inlineStr">
         <is>
@@ -27458,7 +27458,7 @@
         </is>
       </c>
       <c r="I29" s="61" t="n">
-        <v>0.01452372</v>
+        <v>0.01453181</v>
       </c>
       <c r="J29" s="6" t="inlineStr">
         <is>
@@ -27492,7 +27492,7 @@
         </is>
       </c>
       <c r="I30" s="61" t="n">
-        <v>0.01439619</v>
+        <v>0.01420322</v>
       </c>
       <c r="J30" s="6" t="inlineStr">
         <is>
@@ -27530,7 +27530,7 @@
         </is>
       </c>
       <c r="I31" s="61" t="n">
-        <v>0.01358198</v>
+        <v>0.01353078</v>
       </c>
       <c r="J31" s="6" t="inlineStr">
         <is>
@@ -27555,7 +27555,7 @@
         </is>
       </c>
       <c r="I32" s="61" t="n">
-        <v>0.01151425</v>
+        <v>0.01166936</v>
       </c>
       <c r="J32" s="6" t="inlineStr">
         <is>
@@ -27585,7 +27585,7 @@
         </is>
       </c>
       <c r="I33" s="61" t="n">
-        <v>0.01084481</v>
+        <v>0.01101267</v>
       </c>
       <c r="J33" s="6" t="inlineStr">
         <is>
@@ -27610,7 +27610,7 @@
         </is>
       </c>
       <c r="I34" s="61" t="n">
-        <v>0.00910477</v>
+        <v>0.00904929</v>
       </c>
       <c r="J34" s="6" t="inlineStr">
         <is>
@@ -27631,20 +27631,20 @@
     <row r="35">
       <c r="H35" s="6" t="inlineStr">
         <is>
-          <t>PAYX</t>
+          <t>KMB</t>
         </is>
       </c>
       <c r="I35" s="61" t="n">
-        <v>0.008855439999999999</v>
+        <v>0.008711719999999999</v>
       </c>
       <c r="J35" s="6" t="inlineStr">
         <is>
-          <t>PAYCHEX</t>
+          <t>KIMBERLY CLARK</t>
         </is>
       </c>
       <c r="K35" s="6" t="inlineStr">
         <is>
-          <t>Industrials</t>
+          <t>Consumer Staples</t>
         </is>
       </c>
       <c r="L35" s="6" t="inlineStr"/>
@@ -27656,20 +27656,20 @@
     <row r="36">
       <c r="H36" s="6" t="inlineStr">
         <is>
-          <t>KMB</t>
+          <t>PAYX</t>
         </is>
       </c>
       <c r="I36" s="61" t="n">
-        <v>0.00871745</v>
+        <v>0.008397659999999999</v>
       </c>
       <c r="J36" s="6" t="inlineStr">
         <is>
-          <t>KIMBERLY CLARK</t>
+          <t>PAYCHEX</t>
         </is>
       </c>
       <c r="K36" s="6" t="inlineStr">
         <is>
-          <t>Consumer Staples</t>
+          <t>Industrials</t>
         </is>
       </c>
       <c r="L36" s="6" t="inlineStr"/>
@@ -27681,15 +27681,15 @@
     <row r="37">
       <c r="H37" s="6" t="inlineStr">
         <is>
-          <t>ARES</t>
+          <t>CINF</t>
         </is>
       </c>
       <c r="I37" s="61" t="n">
-        <v>0.006526499999999999</v>
+        <v>0.00668471</v>
       </c>
       <c r="J37" s="6" t="inlineStr">
         <is>
-          <t>ARES MANAGEMENT CLASS A</t>
+          <t>CINCINNATI FINANCIAL</t>
         </is>
       </c>
       <c r="K37" s="6" t="inlineStr">
@@ -27706,15 +27706,15 @@
     <row r="38">
       <c r="H38" s="6" t="inlineStr">
         <is>
-          <t>CINF</t>
+          <t>ARES</t>
         </is>
       </c>
       <c r="I38" s="61" t="n">
-        <v>0.00650634</v>
+        <v>0.006570599999999999</v>
       </c>
       <c r="J38" s="6" t="inlineStr">
         <is>
-          <t>CINCINNATI FINANCIAL</t>
+          <t>ARES MANAGEMENT CLASS A</t>
         </is>
       </c>
       <c r="K38" s="6" t="inlineStr">
@@ -27731,20 +27731,20 @@
     <row r="39">
       <c r="H39" s="6" t="inlineStr">
         <is>
-          <t>HSY</t>
+          <t>DRI</t>
         </is>
       </c>
       <c r="I39" s="61" t="n">
-        <v>0.005884899999999999</v>
+        <v>0.00583219</v>
       </c>
       <c r="J39" s="6" t="inlineStr">
         <is>
-          <t>HERSHEY FOODS</t>
+          <t>DARDEN RESTAURANTS INC</t>
         </is>
       </c>
       <c r="K39" s="6" t="inlineStr">
         <is>
-          <t>Consumer Staples</t>
+          <t>Consumer Discretionary</t>
         </is>
       </c>
       <c r="L39" s="6" t="inlineStr"/>
@@ -27760,7 +27760,7 @@
         </is>
       </c>
       <c r="I40" s="61" t="n">
-        <v>0.00582788</v>
+        <v>0.005829879999999999</v>
       </c>
       <c r="J40" s="6" t="inlineStr">
         <is>
@@ -27781,20 +27781,20 @@
     <row r="41">
       <c r="H41" s="6" t="inlineStr">
         <is>
-          <t>DRI</t>
+          <t>HSY</t>
         </is>
       </c>
       <c r="I41" s="61" t="n">
-        <v>0.00578861</v>
+        <v>0.005778910000000001</v>
       </c>
       <c r="J41" s="6" t="inlineStr">
         <is>
-          <t>DARDEN RESTAURANTS INC</t>
+          <t>HERSHEY FOODS</t>
         </is>
       </c>
       <c r="K41" s="6" t="inlineStr">
         <is>
-          <t>Consumer Discretionary</t>
+          <t>Consumer Staples</t>
         </is>
       </c>
       <c r="L41" s="6" t="inlineStr"/>
@@ -27810,7 +27810,7 @@
         </is>
       </c>
       <c r="I42" s="61" t="n">
-        <v>0.00527821</v>
+        <v>0.00530752</v>
       </c>
       <c r="J42" s="6" t="inlineStr">
         <is>
@@ -27835,7 +27835,7 @@
         </is>
       </c>
       <c r="I43" s="61" t="n">
-        <v>0.00513027</v>
+        <v>0.00523831</v>
       </c>
       <c r="J43" s="6" t="inlineStr">
         <is>
@@ -27860,7 +27860,7 @@
         </is>
       </c>
       <c r="I44" s="61" t="n">
-        <v>0.00493773</v>
+        <v>0.00484885</v>
       </c>
       <c r="J44" s="6" t="inlineStr">
         <is>
@@ -27885,7 +27885,7 @@
         </is>
       </c>
       <c r="I45" s="61" t="n">
-        <v>0.00463751</v>
+        <v>0.00468315</v>
       </c>
       <c r="J45" s="6" t="inlineStr">
         <is>
@@ -27906,20 +27906,20 @@
     <row r="46">
       <c r="H46" s="6" t="inlineStr">
         <is>
-          <t>DINO</t>
+          <t>SNA</t>
         </is>
       </c>
       <c r="I46" s="61" t="n">
-        <v>0.00463001</v>
+        <v>0.00443953</v>
       </c>
       <c r="J46" s="6" t="inlineStr">
         <is>
-          <t>HF SINCLAIR</t>
+          <t>SNAP ON INC</t>
         </is>
       </c>
       <c r="K46" s="6" t="inlineStr">
         <is>
-          <t>Energy</t>
+          <t>Industrials</t>
         </is>
       </c>
       <c r="L46" s="6" t="inlineStr"/>
@@ -27931,20 +27931,20 @@
     <row r="47">
       <c r="H47" s="6" t="inlineStr">
         <is>
-          <t>SNA</t>
+          <t>EWBC</t>
         </is>
       </c>
       <c r="I47" s="61" t="n">
-        <v>0.00442571</v>
+        <v>0.00432334</v>
       </c>
       <c r="J47" s="6" t="inlineStr">
         <is>
-          <t>SNAP ON INC</t>
+          <t>EAST WEST BANCORP</t>
         </is>
       </c>
       <c r="K47" s="6" t="inlineStr">
         <is>
-          <t>Industrials</t>
+          <t>Financials</t>
         </is>
       </c>
       <c r="L47" s="6" t="inlineStr"/>
@@ -27956,20 +27956,20 @@
     <row r="48">
       <c r="H48" s="6" t="inlineStr">
         <is>
-          <t>APA</t>
+          <t>GIS</t>
         </is>
       </c>
       <c r="I48" s="61" t="n">
-        <v>0.00432752</v>
+        <v>0.0042973</v>
       </c>
       <c r="J48" s="6" t="inlineStr">
         <is>
-          <t>APA</t>
+          <t>GENERAL MILLS INC</t>
         </is>
       </c>
       <c r="K48" s="6" t="inlineStr">
         <is>
-          <t>Energy</t>
+          <t>Consumer Staples</t>
         </is>
       </c>
       <c r="L48" s="6" t="inlineStr"/>
@@ -27981,20 +27981,20 @@
     <row r="49">
       <c r="H49" s="6" t="inlineStr">
         <is>
-          <t>EWBC</t>
+          <t>APA</t>
         </is>
       </c>
       <c r="I49" s="61" t="n">
-        <v>0.00431709</v>
+        <v>0.00427252</v>
       </c>
       <c r="J49" s="6" t="inlineStr">
         <is>
-          <t>EAST WEST BANCORP</t>
+          <t>APA</t>
         </is>
       </c>
       <c r="K49" s="6" t="inlineStr">
         <is>
-          <t>Financials</t>
+          <t>Energy</t>
         </is>
       </c>
       <c r="L49" s="6" t="inlineStr"/>
@@ -28006,20 +28006,20 @@
     <row r="50">
       <c r="H50" s="6" t="inlineStr">
         <is>
-          <t>GIS</t>
+          <t>DINO</t>
         </is>
       </c>
       <c r="I50" s="61" t="n">
-        <v>0.00430873</v>
+        <v>0.00423965</v>
       </c>
       <c r="J50" s="6" t="inlineStr">
         <is>
-          <t>GENERAL MILLS INC</t>
+          <t>HF SINCLAIR</t>
         </is>
       </c>
       <c r="K50" s="6" t="inlineStr">
         <is>
-          <t>Consumer Staples</t>
+          <t>Energy</t>
         </is>
       </c>
       <c r="L50" s="6" t="inlineStr"/>
@@ -28035,7 +28035,7 @@
         </is>
       </c>
       <c r="I51" s="61" t="n">
-        <v>0.0025973</v>
+        <v>0.00257137</v>
       </c>
       <c r="J51" s="6" t="inlineStr">
         <is>
@@ -28060,7 +28060,7 @@
         </is>
       </c>
       <c r="I52" s="61" t="n">
-        <v>0.00247497</v>
+        <v>0.00249799</v>
       </c>
       <c r="J52" s="6" t="inlineStr">
         <is>
@@ -28085,7 +28085,7 @@
         </is>
       </c>
       <c r="I53" s="61" t="n">
-        <v>0.00243118</v>
+        <v>0.00241145</v>
       </c>
       <c r="J53" s="6" t="inlineStr">
         <is>
@@ -28110,7 +28110,7 @@
         </is>
       </c>
       <c r="I54" s="61" t="n">
-        <v>0.00239598</v>
+        <v>0.00240717</v>
       </c>
       <c r="J54" s="6" t="inlineStr">
         <is>
@@ -28135,7 +28135,7 @@
         </is>
       </c>
       <c r="I55" s="61" t="n">
-        <v>0.00209885</v>
+        <v>0.0021063</v>
       </c>
       <c r="J55" s="6" t="inlineStr">
         <is>
@@ -28160,7 +28160,7 @@
         </is>
       </c>
       <c r="I56" s="61" t="n">
-        <v>0.00204011</v>
+        <v>0.00203109</v>
       </c>
       <c r="J56" s="6" t="inlineStr">
         <is>
@@ -28185,7 +28185,7 @@
         </is>
       </c>
       <c r="I57" s="61" t="n">
-        <v>0.00183693</v>
+        <v>0.00185553</v>
       </c>
       <c r="J57" s="6" t="inlineStr">
         <is>
@@ -28210,7 +28210,7 @@
         </is>
       </c>
       <c r="I58" s="61" t="n">
-        <v>0.00155222</v>
+        <v>0.00153118</v>
       </c>
       <c r="J58" s="6" t="inlineStr">
         <is>
@@ -28235,7 +28235,7 @@
         </is>
       </c>
       <c r="I59" s="61" t="n">
-        <v>0.00148222</v>
+        <v>0.00150548</v>
       </c>
       <c r="J59" s="6" t="inlineStr">
         <is>
@@ -28260,7 +28260,7 @@
         </is>
       </c>
       <c r="I60" s="61" t="n">
-        <v>0.00142633</v>
+        <v>0.00139764</v>
       </c>
       <c r="J60" s="6" t="inlineStr">
         <is>
@@ -28285,7 +28285,7 @@
         </is>
       </c>
       <c r="I61" s="61" t="n">
-        <v>0.00130045</v>
+        <v>0.00130215</v>
       </c>
       <c r="J61" s="6" t="inlineStr">
         <is>
@@ -28310,7 +28310,7 @@
         </is>
       </c>
       <c r="I62" s="61" t="n">
-        <v>0.00127277</v>
+        <v>0.00129564</v>
       </c>
       <c r="J62" s="6" t="inlineStr">
         <is>
@@ -28335,7 +28335,7 @@
         </is>
       </c>
       <c r="I63" s="61" t="n">
-        <v>0.0012227</v>
+        <v>0.00123781</v>
       </c>
       <c r="J63" s="6" t="inlineStr">
         <is>
@@ -28360,7 +28360,7 @@
         </is>
       </c>
       <c r="I64" s="61" t="n">
-        <v>0.00114217</v>
+        <v>0.00115746</v>
       </c>
       <c r="J64" s="6" t="inlineStr">
         <is>
@@ -28385,7 +28385,7 @@
         </is>
       </c>
       <c r="I65" s="61" t="n">
-        <v>0.00107896</v>
+        <v>0.00101075</v>
       </c>
       <c r="J65" s="6" t="inlineStr">
         <is>
@@ -28410,7 +28410,7 @@
         </is>
       </c>
       <c r="I66" s="61" t="n">
-        <v>0.00097594</v>
+        <v>0.00099121</v>
       </c>
       <c r="J66" s="6" t="inlineStr">
         <is>
@@ -28435,7 +28435,7 @@
         </is>
       </c>
       <c r="I67" s="61" t="n">
-        <v>0.0009702900000000001</v>
+        <v>0.0009637199999999999</v>
       </c>
       <c r="J67" s="6" t="inlineStr">
         <is>
@@ -28456,20 +28456,20 @@
     <row r="68">
       <c r="H68" s="6" t="inlineStr">
         <is>
-          <t>KFY</t>
+          <t>CWEN</t>
         </is>
       </c>
       <c r="I68" s="61" t="n">
-        <v>0.0009701600000000001</v>
+        <v>0.00094911</v>
       </c>
       <c r="J68" s="6" t="inlineStr">
         <is>
-          <t>KORN FERRY</t>
+          <t>CLEARWAY ENERGY INC CLASS C</t>
         </is>
       </c>
       <c r="K68" s="6" t="inlineStr">
         <is>
-          <t>Industrials</t>
+          <t>Utilities</t>
         </is>
       </c>
       <c r="L68" s="6" t="inlineStr"/>
@@ -28481,20 +28481,20 @@
     <row r="69">
       <c r="H69" s="6" t="inlineStr">
         <is>
-          <t>CVBF</t>
+          <t>KFY</t>
         </is>
       </c>
       <c r="I69" s="61" t="n">
-        <v>0.00091338</v>
+        <v>0.00093986</v>
       </c>
       <c r="J69" s="6" t="inlineStr">
         <is>
-          <t>CVB FINANCIAL CORP</t>
+          <t>KORN FERRY</t>
         </is>
       </c>
       <c r="K69" s="6" t="inlineStr">
         <is>
-          <t>Financials</t>
+          <t>Industrials</t>
         </is>
       </c>
       <c r="L69" s="6" t="inlineStr"/>
@@ -28506,20 +28506,20 @@
     <row r="70">
       <c r="H70" s="6" t="inlineStr">
         <is>
-          <t>CWEN</t>
+          <t>CVBF</t>
         </is>
       </c>
       <c r="I70" s="61" t="n">
-        <v>0.00090731</v>
+        <v>0.00091322</v>
       </c>
       <c r="J70" s="6" t="inlineStr">
         <is>
-          <t>CLEARWAY ENERGY INC CLASS C</t>
+          <t>CVB FINANCIAL CORP</t>
         </is>
       </c>
       <c r="K70" s="6" t="inlineStr">
         <is>
-          <t>Utilities</t>
+          <t>Financials</t>
         </is>
       </c>
       <c r="L70" s="6" t="inlineStr"/>
@@ -28535,7 +28535,7 @@
         </is>
       </c>
       <c r="I71" s="61" t="n">
-        <v>0.00090034</v>
+        <v>0.00090431</v>
       </c>
       <c r="J71" s="6" t="inlineStr">
         <is>
@@ -28556,15 +28556,15 @@
     <row r="72">
       <c r="H72" s="6" t="inlineStr">
         <is>
-          <t>BANR</t>
+          <t>APAM</t>
         </is>
       </c>
       <c r="I72" s="61" t="n">
-        <v>0.00056977</v>
+        <v>0.00056335</v>
       </c>
       <c r="J72" s="6" t="inlineStr">
         <is>
-          <t>BANNER CORP</t>
+          <t>ARTISAN PARTNERS ASSET MANAGEMENT</t>
         </is>
       </c>
       <c r="K72" s="6" t="inlineStr">
@@ -28581,15 +28581,15 @@
     <row r="73">
       <c r="H73" s="6" t="inlineStr">
         <is>
-          <t>APAM</t>
+          <t>BANR</t>
         </is>
       </c>
       <c r="I73" s="61" t="n">
-        <v>0.00056338</v>
+        <v>0.0005627399999999999</v>
       </c>
       <c r="J73" s="6" t="inlineStr">
         <is>
-          <t>ARTISAN PARTNERS ASSET MANAGEMENT</t>
+          <t>BANNER CORP</t>
         </is>
       </c>
       <c r="K73" s="6" t="inlineStr">
@@ -28610,7 +28610,7 @@
         </is>
       </c>
       <c r="I74" s="61" t="n">
-        <v>0.00052084</v>
+        <v>0.00051742</v>
       </c>
       <c r="J74" s="6" t="inlineStr">
         <is>
@@ -28631,15 +28631,15 @@
     <row r="75">
       <c r="H75" s="6" t="inlineStr">
         <is>
-          <t>MZTI</t>
+          <t>IPAR</t>
         </is>
       </c>
       <c r="I75" s="61" t="n">
-        <v>0.00050793</v>
+        <v>0.0005049200000000001</v>
       </c>
       <c r="J75" s="6" t="inlineStr">
         <is>
-          <t>MARZETTI</t>
+          <t>INTERPARFUMS INC</t>
         </is>
       </c>
       <c r="K75" s="6" t="inlineStr">
@@ -28656,15 +28656,15 @@
     <row r="76">
       <c r="H76" s="6" t="inlineStr">
         <is>
-          <t>IPAR</t>
+          <t>MZTI</t>
         </is>
       </c>
       <c r="I76" s="61" t="n">
-        <v>0.0005036</v>
+        <v>0.00050434</v>
       </c>
       <c r="J76" s="6" t="inlineStr">
         <is>
-          <t>INTERPARFUMS INC</t>
+          <t>MARZETTI</t>
         </is>
       </c>
       <c r="K76" s="6" t="inlineStr">
@@ -28685,7 +28685,7 @@
         </is>
       </c>
       <c r="I77" s="61" t="n">
-        <v>0.00048119</v>
+        <v>0.00048079</v>
       </c>
       <c r="J77" s="6" t="inlineStr">
         <is>
@@ -28710,7 +28710,7 @@
         </is>
       </c>
       <c r="I78" s="61" t="n">
-        <v>0.00047939</v>
+        <v>0.00047747</v>
       </c>
       <c r="J78" s="6" t="inlineStr">
         <is>
@@ -28731,18 +28731,22 @@
     <row r="79">
       <c r="H79" s="6" t="inlineStr">
         <is>
-          <t>GVMXX</t>
+          <t>AGM</t>
         </is>
       </c>
       <c r="I79" s="61" t="n">
-        <v>0.00047706</v>
+        <v>0.00045739</v>
       </c>
       <c r="J79" s="6" t="inlineStr">
         <is>
-          <t>SSC GOVERNMENT MM GVMXX</t>
-        </is>
-      </c>
-      <c r="K79" s="6" t="inlineStr"/>
+          <t>FEDERAL AGRICULTURAL MORTGAGE NON</t>
+        </is>
+      </c>
+      <c r="K79" s="6" t="inlineStr">
+        <is>
+          <t>Financials</t>
+        </is>
+      </c>
       <c r="L79" s="6" t="inlineStr"/>
       <c r="M79" s="7">
         <f>IF(H79="","",IFERROR(VLOOKUP(K79,$P$5:$Q$15,2,FALSE),"현금·선물"))</f>
@@ -28756,7 +28760,7 @@
         </is>
       </c>
       <c r="I80" s="61" t="n">
-        <v>0.00046433</v>
+        <v>0.00044976</v>
       </c>
       <c r="J80" s="6" t="inlineStr">
         <is>
@@ -28781,7 +28785,7 @@
         </is>
       </c>
       <c r="I81" s="61" t="n">
-        <v>0.00046177</v>
+        <v>0.00044523</v>
       </c>
       <c r="J81" s="6" t="inlineStr">
         <is>
@@ -28806,7 +28810,7 @@
         </is>
       </c>
       <c r="I82" s="61" t="n">
-        <v>0.00046028</v>
+        <v>0.00044491</v>
       </c>
       <c r="J82" s="6" t="inlineStr">
         <is>
@@ -28827,22 +28831,18 @@
     <row r="83">
       <c r="H83" s="6" t="inlineStr">
         <is>
-          <t>AGM</t>
+          <t>GVMXX</t>
         </is>
       </c>
       <c r="I83" s="61" t="n">
-        <v>0.00044801</v>
+        <v>0.00043978</v>
       </c>
       <c r="J83" s="6" t="inlineStr">
         <is>
-          <t>FEDERAL AGRICULTURAL MORTGAGE NON</t>
-        </is>
-      </c>
-      <c r="K83" s="6" t="inlineStr">
-        <is>
-          <t>Financials</t>
-        </is>
-      </c>
+          <t>SSC GOVERNMENT MM GVMXX</t>
+        </is>
+      </c>
+      <c r="K83" s="6" t="inlineStr"/>
       <c r="L83" s="6" t="inlineStr"/>
       <c r="M83" s="7">
         <f>IF(H83="","",IFERROR(VLOOKUP(K83,$P$5:$Q$15,2,FALSE),"현금·선물"))</f>
@@ -28856,7 +28856,7 @@
         </is>
       </c>
       <c r="I84" s="61" t="n">
-        <v>0.00043115</v>
+        <v>0.00042928</v>
       </c>
       <c r="J84" s="6" t="inlineStr">
         <is>
@@ -28881,7 +28881,7 @@
         </is>
       </c>
       <c r="I85" s="61" t="n">
-        <v>0.00041527</v>
+        <v>0.00041625</v>
       </c>
       <c r="J85" s="6" t="inlineStr">
         <is>
@@ -28906,7 +28906,7 @@
         </is>
       </c>
       <c r="I86" s="61" t="n">
-        <v>0.00037503</v>
+        <v>0.00037696</v>
       </c>
       <c r="J86" s="6" t="inlineStr">
         <is>
@@ -28931,7 +28931,7 @@
         </is>
       </c>
       <c r="I87" s="61" t="n">
-        <v>0.0003644399999999999</v>
+        <v>0.0003632</v>
       </c>
       <c r="J87" s="6" t="inlineStr">
         <is>
@@ -28956,7 +28956,7 @@
         </is>
       </c>
       <c r="I88" s="61" t="n">
-        <v>0.00034244</v>
+        <v>0.00034245</v>
       </c>
       <c r="J88" s="6" t="inlineStr">
         <is>
@@ -28981,7 +28981,7 @@
         </is>
       </c>
       <c r="I89" s="61" t="n">
-        <v>0.00031166</v>
+        <v>0.00031602</v>
       </c>
       <c r="J89" s="6" t="inlineStr">
         <is>
@@ -29006,7 +29006,7 @@
         </is>
       </c>
       <c r="I90" s="61" t="n">
-        <v>0.00027665</v>
+        <v>0.00027826</v>
       </c>
       <c r="J90" s="6" t="inlineStr">
         <is>
@@ -29031,7 +29031,7 @@
         </is>
       </c>
       <c r="I91" s="61" t="n">
-        <v>0.00025171</v>
+        <v>0.00025073</v>
       </c>
       <c r="J91" s="6" t="inlineStr">
         <is>
@@ -29056,7 +29056,7 @@
         </is>
       </c>
       <c r="I92" s="61" t="n">
-        <v>0.00023786</v>
+        <v>0.00023693</v>
       </c>
       <c r="J92" s="6" t="inlineStr">
         <is>
@@ -29081,7 +29081,7 @@
         </is>
       </c>
       <c r="I93" s="61" t="n">
-        <v>0.00023164</v>
+        <v>0.00023314</v>
       </c>
       <c r="J93" s="6" t="inlineStr">
         <is>
@@ -29106,7 +29106,7 @@
         </is>
       </c>
       <c r="I94" s="61" t="n">
-        <v>0.00022693</v>
+        <v>0.00022957</v>
       </c>
       <c r="J94" s="6" t="inlineStr">
         <is>
@@ -29131,7 +29131,7 @@
         </is>
       </c>
       <c r="I95" s="61" t="n">
-        <v>0.00021275</v>
+        <v>0.00021191</v>
       </c>
       <c r="J95" s="6" t="inlineStr">
         <is>
@@ -29152,15 +29152,15 @@
     <row r="96">
       <c r="H96" s="6" t="inlineStr">
         <is>
-          <t>IBCP</t>
+          <t>THFF</t>
         </is>
       </c>
       <c r="I96" s="61" t="n">
-        <v>0.00019693</v>
+        <v>0.0001993</v>
       </c>
       <c r="J96" s="6" t="inlineStr">
         <is>
-          <t>INDEPENDENT BANK CORP</t>
+          <t>FIRST FINANCIAL CORPORATION CORP</t>
         </is>
       </c>
       <c r="K96" s="6" t="inlineStr">
@@ -29177,15 +29177,15 @@
     <row r="97">
       <c r="H97" s="6" t="inlineStr">
         <is>
-          <t>THFF</t>
+          <t>IBCP</t>
         </is>
       </c>
       <c r="I97" s="61" t="n">
-        <v>0.00019513</v>
+        <v>0.00019839</v>
       </c>
       <c r="J97" s="6" t="inlineStr">
         <is>
-          <t>FIRST FINANCIAL CORPORATION CORP</t>
+          <t>INDEPENDENT BANK CORP</t>
         </is>
       </c>
       <c r="K97" s="6" t="inlineStr">
@@ -29206,7 +29206,7 @@
         </is>
       </c>
       <c r="I98" s="61" t="n">
-        <v>0.00017381</v>
+        <v>0.0001776</v>
       </c>
       <c r="J98" s="6" t="inlineStr">
         <is>
@@ -29231,7 +29231,7 @@
         </is>
       </c>
       <c r="I99" s="61" t="n">
-        <v>0.00016662</v>
+        <v>0.00016834</v>
       </c>
       <c r="J99" s="6" t="inlineStr">
         <is>
@@ -29252,22 +29252,18 @@
     <row r="100">
       <c r="H100" s="6" t="inlineStr">
         <is>
-          <t>EBF</t>
+          <t>USD</t>
         </is>
       </c>
       <c r="I100" s="61" t="n">
-        <v>0.00012907</v>
+        <v>0.00014105</v>
       </c>
       <c r="J100" s="6" t="inlineStr">
         <is>
-          <t>ENNIS INC</t>
-        </is>
-      </c>
-      <c r="K100" s="6" t="inlineStr">
-        <is>
-          <t>Industrials</t>
-        </is>
-      </c>
+          <t>US DOLLAR</t>
+        </is>
+      </c>
+      <c r="K100" s="6" t="inlineStr"/>
       <c r="L100" s="6" t="inlineStr"/>
       <c r="M100" s="7">
         <f>IF(H100="","",IFERROR(VLOOKUP(K100,$P$5:$Q$15,2,FALSE),"현금·선물"))</f>
@@ -29277,20 +29273,20 @@
     <row r="101">
       <c r="H101" s="6" t="inlineStr">
         <is>
-          <t>AMSF</t>
+          <t>EBF</t>
         </is>
       </c>
       <c r="I101" s="61" t="n">
-        <v>0.00011629</v>
+        <v>0.00012949</v>
       </c>
       <c r="J101" s="6" t="inlineStr">
         <is>
-          <t>AMERISAFE INC</t>
+          <t>ENNIS INC</t>
         </is>
       </c>
       <c r="K101" s="6" t="inlineStr">
         <is>
-          <t>Financials</t>
+          <t>Industrials</t>
         </is>
       </c>
       <c r="L101" s="6" t="inlineStr"/>
@@ -29302,20 +29298,20 @@
     <row r="102">
       <c r="H102" s="6" t="inlineStr">
         <is>
-          <t>ETD</t>
+          <t>AMSF</t>
         </is>
       </c>
       <c r="I102" s="61" t="n">
-        <v>9.601999999999999e-05</v>
+        <v>0.00011334</v>
       </c>
       <c r="J102" s="6" t="inlineStr">
         <is>
-          <t>ETHAN ALLEN INTERIORS</t>
+          <t>AMERISAFE INC</t>
         </is>
       </c>
       <c r="K102" s="6" t="inlineStr">
         <is>
-          <t>Consumer Discretionary</t>
+          <t>Financials</t>
         </is>
       </c>
       <c r="L102" s="6" t="inlineStr"/>
@@ -29327,18 +29323,22 @@
     <row r="103">
       <c r="H103" s="6" t="inlineStr">
         <is>
-          <t>USD</t>
+          <t>ETD</t>
         </is>
       </c>
       <c r="I103" s="61" t="n">
-        <v>9.407999999999999e-05</v>
+        <v>9.565000000000001e-05</v>
       </c>
       <c r="J103" s="6" t="inlineStr">
         <is>
-          <t>US DOLLAR</t>
-        </is>
-      </c>
-      <c r="K103" s="6" t="inlineStr"/>
+          <t>ETHAN ALLEN INTERIORS</t>
+        </is>
+      </c>
+      <c r="K103" s="6" t="inlineStr">
+        <is>
+          <t>Consumer Discretionary</t>
+        </is>
+      </c>
       <c r="L103" s="6" t="inlineStr"/>
       <c r="M103" s="7">
         <f>IF(H103="","",IFERROR(VLOOKUP(K103,$P$5:$Q$15,2,FALSE),"현금·선물"))</f>
@@ -29352,7 +29352,7 @@
         </is>
       </c>
       <c r="I104" s="61" t="n">
-        <v>9.129e-05</v>
+        <v>9.143e-05</v>
       </c>
       <c r="J104" s="6" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
데이터 갱신: holdings,kr_etf,official (2026-10-29)
</commit_message>
<xml_diff>
--- a/downloads/schd_dividend_tracker.xlsx
+++ b/downloads/schd_dividend_tracker.xlsx
@@ -1724,7 +1724,7 @@
     <row r="3">
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>최종 갱신: 2026-10-28 · 반영 범위: 2012년 1분기 ~ 2026년 3분기 (배당락 2026-09-23) · GitHub Actions 자동 생성</t>
+          <t>최종 갱신: 2026-10-29 · 반영 범위: 2012년 1분기 ~ 2026년 3분기 (배당락 2026-09-23) · GitHub Actions 자동 생성</t>
         </is>
       </c>
     </row>
@@ -11996,11 +11996,11 @@
         </is>
       </c>
       <c r="B34" s="19" t="n">
-        <v>0.0318</v>
+        <v>0.0314</v>
       </c>
       <c r="C34" s="2" t="inlineStr">
         <is>
-          <t>2026-10-20 기준 · 최근 30일 순투자수익(보수 차감) 연 환산</t>
+          <t>2026-10-27 기준 · 최근 30일 순투자수익(보수 차감) 연 환산</t>
         </is>
       </c>
     </row>
@@ -20053,7 +20053,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F357"/>
+  <dimension ref="A1:F359"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -20918,22 +20918,22 @@
     <row r="41">
       <c r="A41" s="46" t="inlineStr">
         <is>
-          <t>446720</t>
+          <t>458730</t>
         </is>
       </c>
       <c r="B41" s="33" t="inlineStr">
         <is>
-          <t>SOL 미국배당다우존스</t>
+          <t>TIGER 미국배당다우존스</t>
         </is>
       </c>
       <c r="C41" s="26" t="n">
-        <v>44923</v>
+        <v>46324</v>
       </c>
       <c r="D41" s="47" t="n">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="E41" s="48" t="n">
-        <v>0.003779</v>
+        <v>0.002362</v>
       </c>
     </row>
     <row r="42">
@@ -20948,13 +20948,13 @@
         </is>
       </c>
       <c r="C42" s="26" t="n">
-        <v>44956</v>
+        <v>44923</v>
       </c>
       <c r="D42" s="47" t="n">
-        <v>18</v>
+        <v>36</v>
       </c>
       <c r="E42" s="48" t="n">
-        <v>0.001938</v>
+        <v>0.003779</v>
       </c>
     </row>
     <row r="43">
@@ -20969,13 +20969,13 @@
         </is>
       </c>
       <c r="C43" s="26" t="n">
-        <v>44984</v>
+        <v>44956</v>
       </c>
       <c r="D43" s="47" t="n">
-        <v>30</v>
+        <v>18</v>
       </c>
       <c r="E43" s="48" t="n">
-        <v>0.003103</v>
+        <v>0.001938</v>
       </c>
     </row>
     <row r="44">
@@ -20990,13 +20990,13 @@
         </is>
       </c>
       <c r="C44" s="26" t="n">
-        <v>45015</v>
+        <v>44984</v>
       </c>
       <c r="D44" s="47" t="n">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="E44" s="48" t="n">
-        <v>0.003162</v>
+        <v>0.003103</v>
       </c>
     </row>
     <row r="45">
@@ -21011,13 +21011,13 @@
         </is>
       </c>
       <c r="C45" s="26" t="n">
-        <v>45043</v>
+        <v>45015</v>
       </c>
       <c r="D45" s="47" t="n">
-        <v>20</v>
+        <v>29</v>
       </c>
       <c r="E45" s="48" t="n">
-        <v>0.002106</v>
+        <v>0.003162</v>
       </c>
     </row>
     <row r="46">
@@ -21032,13 +21032,13 @@
         </is>
       </c>
       <c r="C46" s="26" t="n">
-        <v>45076</v>
+        <v>45043</v>
       </c>
       <c r="D46" s="47" t="n">
-        <v>33</v>
+        <v>20</v>
       </c>
       <c r="E46" s="48" t="n">
-        <v>0.003642</v>
+        <v>0.002106</v>
       </c>
     </row>
     <row r="47">
@@ -21053,13 +21053,13 @@
         </is>
       </c>
       <c r="C47" s="26" t="n">
-        <v>45106</v>
+        <v>45076</v>
       </c>
       <c r="D47" s="47" t="n">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="E47" s="48" t="n">
-        <v>0.003458</v>
+        <v>0.003642</v>
       </c>
     </row>
     <row r="48">
@@ -21074,13 +21074,13 @@
         </is>
       </c>
       <c r="C48" s="26" t="n">
-        <v>45135</v>
+        <v>45106</v>
       </c>
       <c r="D48" s="47" t="n">
-        <v>26</v>
+        <v>32</v>
       </c>
       <c r="E48" s="48" t="n">
-        <v>0.00274</v>
+        <v>0.003458</v>
       </c>
     </row>
     <row r="49">
@@ -21095,13 +21095,13 @@
         </is>
       </c>
       <c r="C49" s="26" t="n">
-        <v>45168</v>
+        <v>45135</v>
       </c>
       <c r="D49" s="47" t="n">
-        <v>32</v>
+        <v>26</v>
       </c>
       <c r="E49" s="48" t="n">
-        <v>0.003346</v>
+        <v>0.00274</v>
       </c>
     </row>
     <row r="50">
@@ -21116,13 +21116,13 @@
         </is>
       </c>
       <c r="C50" s="26" t="n">
-        <v>45195</v>
+        <v>45168</v>
       </c>
       <c r="D50" s="47" t="n">
-        <v>27</v>
+        <v>32</v>
       </c>
       <c r="E50" s="48" t="n">
-        <v>0.002873</v>
+        <v>0.003346</v>
       </c>
     </row>
     <row r="51">
@@ -21137,13 +21137,13 @@
         </is>
       </c>
       <c r="C51" s="26" t="n">
-        <v>45229</v>
+        <v>45195</v>
       </c>
       <c r="D51" s="47" t="n">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="E51" s="48" t="n">
-        <v>0.002864</v>
+        <v>0.002873</v>
       </c>
     </row>
     <row r="52">
@@ -21158,13 +21158,13 @@
         </is>
       </c>
       <c r="C52" s="26" t="n">
-        <v>45259</v>
+        <v>45229</v>
       </c>
       <c r="D52" s="47" t="n">
-        <v>38</v>
+        <v>26</v>
       </c>
       <c r="E52" s="48" t="n">
-        <v>0.004202</v>
+        <v>0.002864</v>
       </c>
     </row>
     <row r="53">
@@ -21179,13 +21179,13 @@
         </is>
       </c>
       <c r="C53" s="26" t="n">
-        <v>45287</v>
+        <v>45259</v>
       </c>
       <c r="D53" s="47" t="n">
-        <v>30</v>
+        <v>38</v>
       </c>
       <c r="E53" s="48" t="n">
-        <v>0.0031</v>
+        <v>0.004202</v>
       </c>
     </row>
     <row r="54">
@@ -21200,13 +21200,13 @@
         </is>
       </c>
       <c r="C54" s="26" t="n">
-        <v>45321</v>
+        <v>45287</v>
       </c>
       <c r="D54" s="47" t="n">
-        <v>27</v>
+        <v>30</v>
       </c>
       <c r="E54" s="48" t="n">
-        <v>0.00267</v>
+        <v>0.0031</v>
       </c>
     </row>
     <row r="55">
@@ -21221,13 +21221,13 @@
         </is>
       </c>
       <c r="C55" s="26" t="n">
-        <v>45350</v>
+        <v>45321</v>
       </c>
       <c r="D55" s="47" t="n">
-        <v>30</v>
+        <v>27</v>
       </c>
       <c r="E55" s="48" t="n">
-        <v>0.002969</v>
+        <v>0.00267</v>
       </c>
     </row>
     <row r="56">
@@ -21242,13 +21242,13 @@
         </is>
       </c>
       <c r="C56" s="26" t="n">
-        <v>45379</v>
+        <v>45350</v>
       </c>
       <c r="D56" s="47" t="n">
-        <v>24</v>
+        <v>30</v>
       </c>
       <c r="E56" s="48" t="n">
-        <v>0.002293</v>
+        <v>0.002969</v>
       </c>
     </row>
     <row r="57">
@@ -21263,13 +21263,13 @@
         </is>
       </c>
       <c r="C57" s="26" t="n">
-        <v>45411</v>
+        <v>45379</v>
       </c>
       <c r="D57" s="47" t="n">
-        <v>33</v>
+        <v>24</v>
       </c>
       <c r="E57" s="48" t="n">
-        <v>0.003152</v>
+        <v>0.002293</v>
       </c>
     </row>
     <row r="58">
@@ -21284,13 +21284,13 @@
         </is>
       </c>
       <c r="C58" s="26" t="n">
-        <v>45442</v>
+        <v>45411</v>
       </c>
       <c r="D58" s="47" t="n">
-        <v>39</v>
+        <v>33</v>
       </c>
       <c r="E58" s="48" t="n">
-        <v>0.003771</v>
+        <v>0.003152</v>
       </c>
     </row>
     <row r="59">
@@ -21305,13 +21305,13 @@
         </is>
       </c>
       <c r="C59" s="26" t="n">
-        <v>45470</v>
+        <v>45442</v>
       </c>
       <c r="D59" s="47" t="n">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="E59" s="48" t="n">
-        <v>0.003575</v>
+        <v>0.003771</v>
       </c>
     </row>
     <row r="60">
@@ -21326,13 +21326,13 @@
         </is>
       </c>
       <c r="C60" s="26" t="n">
-        <v>45503</v>
+        <v>45470</v>
       </c>
       <c r="D60" s="47" t="n">
-        <v>35</v>
+        <v>38</v>
       </c>
       <c r="E60" s="48" t="n">
-        <v>0.003132</v>
+        <v>0.003575</v>
       </c>
     </row>
     <row r="61">
@@ -21347,13 +21347,13 @@
         </is>
       </c>
       <c r="C61" s="26" t="n">
-        <v>45533</v>
+        <v>45503</v>
       </c>
       <c r="D61" s="47" t="n">
         <v>35</v>
       </c>
       <c r="E61" s="48" t="n">
-        <v>0.003204</v>
+        <v>0.003132</v>
       </c>
     </row>
     <row r="62">
@@ -21368,13 +21368,13 @@
         </is>
       </c>
       <c r="C62" s="26" t="n">
-        <v>45562</v>
+        <v>45533</v>
       </c>
       <c r="D62" s="47" t="n">
-        <v>30</v>
+        <v>35</v>
       </c>
       <c r="E62" s="48" t="n">
-        <v>0.002759</v>
+        <v>0.003204</v>
       </c>
     </row>
     <row r="63">
@@ -21389,13 +21389,13 @@
         </is>
       </c>
       <c r="C63" s="26" t="n">
-        <v>45595</v>
+        <v>45562</v>
       </c>
       <c r="D63" s="47" t="n">
-        <v>32</v>
+        <v>30</v>
       </c>
       <c r="E63" s="48" t="n">
-        <v>0.002775</v>
+        <v>0.002759</v>
       </c>
     </row>
     <row r="64">
@@ -21410,13 +21410,13 @@
         </is>
       </c>
       <c r="C64" s="26" t="n">
-        <v>45624</v>
+        <v>45595</v>
       </c>
       <c r="D64" s="47" t="n">
-        <v>46</v>
+        <v>32</v>
       </c>
       <c r="E64" s="48" t="n">
-        <v>0.003817</v>
+        <v>0.002775</v>
       </c>
     </row>
     <row r="65">
@@ -21431,13 +21431,13 @@
         </is>
       </c>
       <c r="C65" s="26" t="n">
-        <v>45653</v>
+        <v>45624</v>
       </c>
       <c r="D65" s="47" t="n">
-        <v>35</v>
+        <v>46</v>
       </c>
       <c r="E65" s="48" t="n">
-        <v>0.002942</v>
+        <v>0.003817</v>
       </c>
     </row>
     <row r="66">
@@ -21452,13 +21452,13 @@
         </is>
       </c>
       <c r="C66" s="26" t="n">
-        <v>45681</v>
+        <v>45653</v>
       </c>
       <c r="D66" s="47" t="n">
-        <v>42</v>
+        <v>35</v>
       </c>
       <c r="E66" s="48" t="n">
-        <v>0.003564</v>
+        <v>0.002942</v>
       </c>
     </row>
     <row r="67">
@@ -21473,13 +21473,13 @@
         </is>
       </c>
       <c r="C67" s="26" t="n">
-        <v>45715</v>
+        <v>45681</v>
       </c>
       <c r="D67" s="47" t="n">
-        <v>32</v>
+        <v>42</v>
       </c>
       <c r="E67" s="48" t="n">
-        <v>0.002692</v>
+        <v>0.003564</v>
       </c>
     </row>
     <row r="68">
@@ -21494,13 +21494,13 @@
         </is>
       </c>
       <c r="C68" s="26" t="n">
-        <v>45744</v>
+        <v>45715</v>
       </c>
       <c r="D68" s="47" t="n">
-        <v>38</v>
+        <v>32</v>
       </c>
       <c r="E68" s="48" t="n">
-        <v>0.003181</v>
+        <v>0.002692</v>
       </c>
     </row>
     <row r="69">
@@ -21515,13 +21515,13 @@
         </is>
       </c>
       <c r="C69" s="26" t="n">
-        <v>45776</v>
+        <v>45744</v>
       </c>
       <c r="D69" s="47" t="n">
-        <v>26</v>
+        <v>38</v>
       </c>
       <c r="E69" s="48" t="n">
-        <v>0.002409</v>
+        <v>0.003181</v>
       </c>
     </row>
     <row r="70">
@@ -21536,13 +21536,13 @@
         </is>
       </c>
       <c r="C70" s="26" t="n">
-        <v>45806</v>
+        <v>45776</v>
       </c>
       <c r="D70" s="47" t="n">
-        <v>30</v>
+        <v>26</v>
       </c>
       <c r="E70" s="48" t="n">
-        <v>0.002857</v>
+        <v>0.002409</v>
       </c>
     </row>
     <row r="71">
@@ -21557,13 +21557,13 @@
         </is>
       </c>
       <c r="C71" s="26" t="n">
-        <v>45835</v>
+        <v>45806</v>
       </c>
       <c r="D71" s="47" t="n">
-        <v>33</v>
+        <v>30</v>
       </c>
       <c r="E71" s="48" t="n">
-        <v>0.00315</v>
+        <v>0.002857</v>
       </c>
     </row>
     <row r="72">
@@ -21578,13 +21578,13 @@
         </is>
       </c>
       <c r="C72" s="26" t="n">
-        <v>45868</v>
+        <v>45835</v>
       </c>
       <c r="D72" s="47" t="n">
-        <v>28</v>
+        <v>33</v>
       </c>
       <c r="E72" s="48" t="n">
-        <v>0.002532</v>
+        <v>0.00315</v>
       </c>
     </row>
     <row r="73">
@@ -21599,13 +21599,13 @@
         </is>
       </c>
       <c r="C73" s="26" t="n">
-        <v>45897</v>
+        <v>45868</v>
       </c>
       <c r="D73" s="47" t="n">
-        <v>32</v>
+        <v>28</v>
       </c>
       <c r="E73" s="48" t="n">
-        <v>0.002839</v>
+        <v>0.002532</v>
       </c>
     </row>
     <row r="74">
@@ -21620,13 +21620,13 @@
         </is>
       </c>
       <c r="C74" s="26" t="n">
-        <v>45929</v>
+        <v>45897</v>
       </c>
       <c r="D74" s="47" t="n">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="E74" s="48" t="n">
-        <v>0.00314</v>
+        <v>0.002839</v>
       </c>
     </row>
     <row r="75">
@@ -21641,13 +21641,13 @@
         </is>
       </c>
       <c r="C75" s="26" t="n">
-        <v>45960</v>
+        <v>45929</v>
       </c>
       <c r="D75" s="47" t="n">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="E75" s="48" t="n">
-        <v>0.003026</v>
+        <v>0.00314</v>
       </c>
     </row>
     <row r="76">
@@ -21662,13 +21662,13 @@
         </is>
       </c>
       <c r="C76" s="26" t="n">
-        <v>45988</v>
+        <v>45960</v>
       </c>
       <c r="D76" s="47" t="n">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="E76" s="48" t="n">
-        <v>0.003017</v>
+        <v>0.003026</v>
       </c>
     </row>
     <row r="77">
@@ -21683,13 +21683,13 @@
         </is>
       </c>
       <c r="C77" s="26" t="n">
-        <v>46020</v>
+        <v>45988</v>
       </c>
       <c r="D77" s="47" t="n">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="E77" s="48" t="n">
-        <v>0.003141</v>
+        <v>0.003017</v>
       </c>
     </row>
     <row r="78">
@@ -21704,13 +21704,13 @@
         </is>
       </c>
       <c r="C78" s="26" t="n">
-        <v>46051</v>
+        <v>46020</v>
       </c>
       <c r="D78" s="47" t="n">
-        <v>30</v>
+        <v>37</v>
       </c>
       <c r="E78" s="48" t="n">
-        <v>0.002463</v>
+        <v>0.003141</v>
       </c>
     </row>
     <row r="79">
@@ -21725,13 +21725,13 @@
         </is>
       </c>
       <c r="C79" s="26" t="n">
-        <v>46079</v>
+        <v>46051</v>
       </c>
       <c r="D79" s="47" t="n">
-        <v>35</v>
+        <v>30</v>
       </c>
       <c r="E79" s="48" t="n">
-        <v>0.00266</v>
+        <v>0.002463</v>
       </c>
     </row>
     <row r="80">
@@ -21746,13 +21746,13 @@
         </is>
       </c>
       <c r="C80" s="26" t="n">
-        <v>46111</v>
+        <v>46079</v>
       </c>
       <c r="D80" s="47" t="n">
-        <v>33</v>
+        <v>35</v>
       </c>
       <c r="E80" s="48" t="n">
-        <v>0.00244</v>
+        <v>0.00266</v>
       </c>
     </row>
     <row r="81">
@@ -21767,13 +21767,13 @@
         </is>
       </c>
       <c r="C81" s="26" t="n">
-        <v>46141</v>
+        <v>46111</v>
       </c>
       <c r="D81" s="47" t="n">
-        <v>30</v>
+        <v>33</v>
       </c>
       <c r="E81" s="48" t="n">
-        <v>0.002241</v>
+        <v>0.00244</v>
       </c>
     </row>
     <row r="82">
@@ -21788,13 +21788,13 @@
         </is>
       </c>
       <c r="C82" s="26" t="n">
-        <v>46170</v>
+        <v>46141</v>
       </c>
       <c r="D82" s="47" t="n">
-        <v>33</v>
+        <v>30</v>
       </c>
       <c r="E82" s="48" t="n">
-        <v>0.002313</v>
+        <v>0.002241</v>
       </c>
     </row>
     <row r="83">
@@ -21809,13 +21809,13 @@
         </is>
       </c>
       <c r="C83" s="26" t="n">
-        <v>46202</v>
+        <v>46170</v>
       </c>
       <c r="D83" s="47" t="n">
-        <v>42</v>
+        <v>33</v>
       </c>
       <c r="E83" s="48" t="n">
-        <v>0.002932</v>
+        <v>0.002313</v>
       </c>
     </row>
     <row r="84">
@@ -21830,13 +21830,13 @@
         </is>
       </c>
       <c r="C84" s="26" t="n">
-        <v>46233</v>
+        <v>46202</v>
       </c>
       <c r="D84" s="47" t="n">
-        <v>35</v>
+        <v>42</v>
       </c>
       <c r="E84" s="48" t="n">
-        <v>0.00245</v>
+        <v>0.002932</v>
       </c>
     </row>
     <row r="85">
@@ -21851,13 +21851,13 @@
         </is>
       </c>
       <c r="C85" s="26" t="n">
-        <v>46262</v>
+        <v>46233</v>
       </c>
       <c r="D85" s="47" t="n">
-        <v>27</v>
+        <v>35</v>
       </c>
       <c r="E85" s="48" t="n">
-        <v>0.001926</v>
+        <v>0.00245</v>
       </c>
     </row>
     <row r="86">
@@ -21872,55 +21872,55 @@
         </is>
       </c>
       <c r="C86" s="26" t="n">
-        <v>46294</v>
+        <v>46262</v>
       </c>
       <c r="D86" s="47" t="n">
-        <v>37</v>
+        <v>27</v>
       </c>
       <c r="E86" s="48" t="n">
-        <v>0.0028</v>
+        <v>0.001926</v>
       </c>
     </row>
     <row r="87">
       <c r="A87" s="46" t="inlineStr">
         <is>
-          <t>402970</t>
+          <t>446720</t>
         </is>
       </c>
       <c r="B87" s="33" t="inlineStr">
         <is>
-          <t>ACE 미국배당다우존스</t>
+          <t>SOL 미국배당다우존스</t>
         </is>
       </c>
       <c r="C87" s="26" t="n">
-        <v>44588</v>
+        <v>46294</v>
       </c>
       <c r="D87" s="47" t="n">
-        <v>55</v>
+        <v>37</v>
       </c>
       <c r="E87" s="48" t="n">
-        <v>0.005337</v>
+        <v>0.0028</v>
       </c>
     </row>
     <row r="88">
       <c r="A88" s="46" t="inlineStr">
         <is>
-          <t>402970</t>
+          <t>446720</t>
         </is>
       </c>
       <c r="B88" s="33" t="inlineStr">
         <is>
-          <t>ACE 미국배당다우존스</t>
+          <t>SOL 미국배당다우존스</t>
         </is>
       </c>
       <c r="C88" s="26" t="n">
-        <v>44679</v>
+        <v>46324</v>
       </c>
       <c r="D88" s="47" t="n">
-        <v>65</v>
+        <v>32</v>
       </c>
       <c r="E88" s="48" t="n">
-        <v>0.006095000000000001</v>
+        <v>0.002357</v>
       </c>
     </row>
     <row r="89">
@@ -21935,13 +21935,13 @@
         </is>
       </c>
       <c r="C89" s="26" t="n">
-        <v>44770</v>
+        <v>44588</v>
       </c>
       <c r="D89" s="47" t="n">
-        <v>65</v>
+        <v>55</v>
       </c>
       <c r="E89" s="48" t="n">
-        <v>0.006222</v>
+        <v>0.005337</v>
       </c>
     </row>
     <row r="90">
@@ -21956,13 +21956,13 @@
         </is>
       </c>
       <c r="C90" s="26" t="n">
-        <v>44862</v>
+        <v>44679</v>
       </c>
       <c r="D90" s="47" t="n">
-        <v>105</v>
+        <v>65</v>
       </c>
       <c r="E90" s="48" t="n">
-        <v>0.009284000000000001</v>
+        <v>0.006095000000000001</v>
       </c>
     </row>
     <row r="91">
@@ -21977,13 +21977,13 @@
         </is>
       </c>
       <c r="C91" s="26" t="n">
-        <v>44956</v>
+        <v>44770</v>
       </c>
       <c r="D91" s="47" t="n">
-        <v>85</v>
+        <v>65</v>
       </c>
       <c r="E91" s="48" t="n">
-        <v>0.008215</v>
+        <v>0.006222</v>
       </c>
     </row>
     <row r="92">
@@ -21998,13 +21998,13 @@
         </is>
       </c>
       <c r="C92" s="26" t="n">
-        <v>45043</v>
+        <v>44862</v>
       </c>
       <c r="D92" s="47" t="n">
-        <v>100</v>
+        <v>105</v>
       </c>
       <c r="E92" s="48" t="n">
-        <v>0.009443</v>
+        <v>0.009284000000000001</v>
       </c>
     </row>
     <row r="93">
@@ -22019,13 +22019,13 @@
         </is>
       </c>
       <c r="C93" s="26" t="n">
-        <v>45135</v>
+        <v>44956</v>
       </c>
       <c r="D93" s="47" t="n">
-        <v>80</v>
+        <v>85</v>
       </c>
       <c r="E93" s="48" t="n">
-        <v>0.007578000000000001</v>
+        <v>0.008215</v>
       </c>
     </row>
     <row r="94">
@@ -22040,13 +22040,13 @@
         </is>
       </c>
       <c r="C94" s="26" t="n">
-        <v>45168</v>
+        <v>45043</v>
       </c>
       <c r="D94" s="47" t="n">
-        <v>35</v>
+        <v>100</v>
       </c>
       <c r="E94" s="48" t="n">
-        <v>0.003306</v>
+        <v>0.009443</v>
       </c>
     </row>
     <row r="95">
@@ -22061,13 +22061,13 @@
         </is>
       </c>
       <c r="C95" s="26" t="n">
-        <v>45195</v>
+        <v>45135</v>
       </c>
       <c r="D95" s="47" t="n">
-        <v>45</v>
+        <v>80</v>
       </c>
       <c r="E95" s="48" t="n">
-        <v>0.004327</v>
+        <v>0.007578000000000001</v>
       </c>
     </row>
     <row r="96">
@@ -22082,13 +22082,13 @@
         </is>
       </c>
       <c r="C96" s="26" t="n">
-        <v>45229</v>
+        <v>45168</v>
       </c>
       <c r="D96" s="47" t="n">
-        <v>25</v>
+        <v>35</v>
       </c>
       <c r="E96" s="48" t="n">
-        <v>0.002493</v>
+        <v>0.003306</v>
       </c>
     </row>
     <row r="97">
@@ -22103,13 +22103,13 @@
         </is>
       </c>
       <c r="C97" s="26" t="n">
-        <v>45259</v>
+        <v>45195</v>
       </c>
       <c r="D97" s="47" t="n">
-        <v>37</v>
+        <v>45</v>
       </c>
       <c r="E97" s="48" t="n">
-        <v>0.0037</v>
+        <v>0.004327</v>
       </c>
     </row>
     <row r="98">
@@ -22124,13 +22124,13 @@
         </is>
       </c>
       <c r="C98" s="26" t="n">
-        <v>45287</v>
+        <v>45229</v>
       </c>
       <c r="D98" s="47" t="n">
-        <v>45</v>
+        <v>25</v>
       </c>
       <c r="E98" s="48" t="n">
-        <v>0.004204</v>
+        <v>0.002493</v>
       </c>
     </row>
     <row r="99">
@@ -22145,13 +22145,13 @@
         </is>
       </c>
       <c r="C99" s="26" t="n">
-        <v>45321</v>
+        <v>45259</v>
       </c>
       <c r="D99" s="47" t="n">
-        <v>30</v>
+        <v>37</v>
       </c>
       <c r="E99" s="48" t="n">
-        <v>0.002685</v>
+        <v>0.0037</v>
       </c>
     </row>
     <row r="100">
@@ -22166,13 +22166,13 @@
         </is>
       </c>
       <c r="C100" s="26" t="n">
-        <v>45350</v>
+        <v>45287</v>
       </c>
       <c r="D100" s="47" t="n">
-        <v>34</v>
+        <v>45</v>
       </c>
       <c r="E100" s="48" t="n">
-        <v>0.003045</v>
+        <v>0.004204</v>
       </c>
     </row>
     <row r="101">
@@ -22187,13 +22187,13 @@
         </is>
       </c>
       <c r="C101" s="26" t="n">
-        <v>45379</v>
+        <v>45321</v>
       </c>
       <c r="D101" s="47" t="n">
-        <v>44</v>
+        <v>30</v>
       </c>
       <c r="E101" s="48" t="n">
-        <v>0.003805</v>
+        <v>0.002685</v>
       </c>
     </row>
     <row r="102">
@@ -22208,13 +22208,13 @@
         </is>
       </c>
       <c r="C102" s="26" t="n">
-        <v>45411</v>
+        <v>45350</v>
       </c>
       <c r="D102" s="47" t="n">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="E102" s="48" t="n">
-        <v>0.002771</v>
+        <v>0.003045</v>
       </c>
     </row>
     <row r="103">
@@ -22229,13 +22229,13 @@
         </is>
       </c>
       <c r="C103" s="26" t="n">
-        <v>45442</v>
+        <v>45379</v>
       </c>
       <c r="D103" s="47" t="n">
-        <v>39</v>
+        <v>44</v>
       </c>
       <c r="E103" s="48" t="n">
-        <v>0.003413</v>
+        <v>0.003805</v>
       </c>
     </row>
     <row r="104">
@@ -22250,13 +22250,13 @@
         </is>
       </c>
       <c r="C104" s="26" t="n">
-        <v>45470</v>
+        <v>45411</v>
       </c>
       <c r="D104" s="47" t="n">
-        <v>44</v>
+        <v>32</v>
       </c>
       <c r="E104" s="48" t="n">
-        <v>0.003742</v>
+        <v>0.002771</v>
       </c>
     </row>
     <row r="105">
@@ -22271,13 +22271,13 @@
         </is>
       </c>
       <c r="C105" s="26" t="n">
-        <v>45503</v>
+        <v>45442</v>
       </c>
       <c r="D105" s="47" t="n">
-        <v>44</v>
+        <v>39</v>
       </c>
       <c r="E105" s="48" t="n">
-        <v>0.00356</v>
+        <v>0.003413</v>
       </c>
     </row>
     <row r="106">
@@ -22292,13 +22292,13 @@
         </is>
       </c>
       <c r="C106" s="26" t="n">
-        <v>45547</v>
+        <v>45470</v>
       </c>
       <c r="D106" s="47" t="n">
-        <v>56</v>
+        <v>44</v>
       </c>
       <c r="E106" s="48" t="n">
-        <v>0.00466</v>
+        <v>0.003742</v>
       </c>
     </row>
     <row r="107">
@@ -22313,13 +22313,13 @@
         </is>
       </c>
       <c r="C107" s="26" t="n">
-        <v>45579</v>
+        <v>45503</v>
       </c>
       <c r="D107" s="47" t="n">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="E107" s="48" t="n">
-        <v>0.003633</v>
+        <v>0.00356</v>
       </c>
     </row>
     <row r="108">
@@ -22334,13 +22334,13 @@
         </is>
       </c>
       <c r="C108" s="26" t="n">
-        <v>45610</v>
+        <v>45547</v>
       </c>
       <c r="D108" s="47" t="n">
-        <v>30</v>
+        <v>56</v>
       </c>
       <c r="E108" s="48" t="n">
-        <v>0.002276</v>
+        <v>0.00466</v>
       </c>
     </row>
     <row r="109">
@@ -22355,13 +22355,13 @@
         </is>
       </c>
       <c r="C109" s="26" t="n">
-        <v>45638</v>
+        <v>45579</v>
       </c>
       <c r="D109" s="47" t="n">
-        <v>68</v>
+        <v>45</v>
       </c>
       <c r="E109" s="48" t="n">
-        <v>0.005121</v>
+        <v>0.003633</v>
       </c>
     </row>
     <row r="110">
@@ -22376,13 +22376,13 @@
         </is>
       </c>
       <c r="C110" s="26" t="n">
-        <v>45671</v>
+        <v>45610</v>
       </c>
       <c r="D110" s="47" t="n">
-        <v>39</v>
+        <v>30</v>
       </c>
       <c r="E110" s="48" t="n">
-        <v>0.003025</v>
+        <v>0.002276</v>
       </c>
     </row>
     <row r="111">
@@ -22397,13 +22397,13 @@
         </is>
       </c>
       <c r="C111" s="26" t="n">
-        <v>45701</v>
+        <v>45638</v>
       </c>
       <c r="D111" s="47" t="n">
-        <v>28</v>
+        <v>68</v>
       </c>
       <c r="E111" s="48" t="n">
-        <v>0.002142</v>
+        <v>0.005121</v>
       </c>
     </row>
     <row r="112">
@@ -22418,13 +22418,13 @@
         </is>
       </c>
       <c r="C112" s="26" t="n">
-        <v>45729</v>
+        <v>45671</v>
       </c>
       <c r="D112" s="47" t="n">
-        <v>46</v>
+        <v>39</v>
       </c>
       <c r="E112" s="48" t="n">
-        <v>0.003543</v>
+        <v>0.003025</v>
       </c>
     </row>
     <row r="113">
@@ -22439,13 +22439,13 @@
         </is>
       </c>
       <c r="C113" s="26" t="n">
-        <v>45761</v>
+        <v>45701</v>
       </c>
       <c r="D113" s="47" t="n">
-        <v>35</v>
+        <v>28</v>
       </c>
       <c r="E113" s="48" t="n">
-        <v>0.002925</v>
+        <v>0.002142</v>
       </c>
     </row>
     <row r="114">
@@ -22460,13 +22460,13 @@
         </is>
       </c>
       <c r="C114" s="26" t="n">
-        <v>45791</v>
+        <v>45729</v>
       </c>
       <c r="D114" s="47" t="n">
-        <v>21</v>
+        <v>46</v>
       </c>
       <c r="E114" s="48" t="n">
-        <v>0.001743</v>
+        <v>0.003543</v>
       </c>
     </row>
     <row r="115">
@@ -22481,13 +22481,13 @@
         </is>
       </c>
       <c r="C115" s="26" t="n">
-        <v>45820</v>
+        <v>45761</v>
       </c>
       <c r="D115" s="47" t="n">
-        <v>45</v>
+        <v>35</v>
       </c>
       <c r="E115" s="48" t="n">
-        <v>0.003794</v>
+        <v>0.002925</v>
       </c>
     </row>
     <row r="116">
@@ -22502,13 +22502,13 @@
         </is>
       </c>
       <c r="C116" s="26" t="n">
-        <v>45852</v>
+        <v>45791</v>
       </c>
       <c r="D116" s="47" t="n">
-        <v>38</v>
+        <v>21</v>
       </c>
       <c r="E116" s="48" t="n">
-        <v>0.003116</v>
+        <v>0.001743</v>
       </c>
     </row>
     <row r="117">
@@ -22523,13 +22523,13 @@
         </is>
       </c>
       <c r="C117" s="26" t="n">
-        <v>45882</v>
+        <v>45820</v>
       </c>
       <c r="D117" s="47" t="n">
-        <v>20</v>
+        <v>45</v>
       </c>
       <c r="E117" s="48" t="n">
-        <v>0.001665</v>
+        <v>0.003794</v>
       </c>
     </row>
     <row r="118">
@@ -22544,13 +22544,13 @@
         </is>
       </c>
       <c r="C118" s="26" t="n">
-        <v>45912</v>
+        <v>45852</v>
       </c>
       <c r="D118" s="47" t="n">
-        <v>44</v>
+        <v>38</v>
       </c>
       <c r="E118" s="48" t="n">
-        <v>0.003577</v>
+        <v>0.003116</v>
       </c>
     </row>
     <row r="119">
@@ -22565,13 +22565,13 @@
         </is>
       </c>
       <c r="C119" s="26" t="n">
-        <v>45944</v>
+        <v>45882</v>
       </c>
       <c r="D119" s="47" t="n">
-        <v>37</v>
+        <v>20</v>
       </c>
       <c r="E119" s="48" t="n">
-        <v>0.003019</v>
+        <v>0.001665</v>
       </c>
     </row>
     <row r="120">
@@ -22586,13 +22586,13 @@
         </is>
       </c>
       <c r="C120" s="26" t="n">
-        <v>45974</v>
+        <v>45912</v>
       </c>
       <c r="D120" s="47" t="n">
-        <v>21</v>
+        <v>44</v>
       </c>
       <c r="E120" s="48" t="n">
-        <v>0.001641</v>
+        <v>0.003577</v>
       </c>
     </row>
     <row r="121">
@@ -22607,13 +22607,13 @@
         </is>
       </c>
       <c r="C121" s="26" t="n">
-        <v>46003</v>
+        <v>45944</v>
       </c>
       <c r="D121" s="47" t="n">
-        <v>53</v>
+        <v>37</v>
       </c>
       <c r="E121" s="48" t="n">
-        <v>0.00404</v>
+        <v>0.003019</v>
       </c>
     </row>
     <row r="122">
@@ -22628,13 +22628,13 @@
         </is>
       </c>
       <c r="C122" s="26" t="n">
-        <v>46036</v>
+        <v>45974</v>
       </c>
       <c r="D122" s="47" t="n">
-        <v>39</v>
+        <v>21</v>
       </c>
       <c r="E122" s="48" t="n">
-        <v>0.002885</v>
+        <v>0.001641</v>
       </c>
     </row>
     <row r="123">
@@ -22649,13 +22649,13 @@
         </is>
       </c>
       <c r="C123" s="26" t="n">
-        <v>46065</v>
+        <v>46003</v>
       </c>
       <c r="D123" s="47" t="n">
-        <v>24</v>
+        <v>53</v>
       </c>
       <c r="E123" s="48" t="n">
-        <v>0.00163</v>
+        <v>0.00404</v>
       </c>
     </row>
     <row r="124">
@@ -22670,13 +22670,13 @@
         </is>
       </c>
       <c r="C124" s="26" t="n">
-        <v>46093</v>
+        <v>46036</v>
       </c>
       <c r="D124" s="47" t="n">
-        <v>46</v>
+        <v>39</v>
       </c>
       <c r="E124" s="48" t="n">
-        <v>0.003151</v>
+        <v>0.002885</v>
       </c>
     </row>
     <row r="125">
@@ -22691,13 +22691,13 @@
         </is>
       </c>
       <c r="C125" s="26" t="n">
-        <v>46126</v>
+        <v>46065</v>
       </c>
       <c r="D125" s="47" t="n">
-        <v>44</v>
+        <v>24</v>
       </c>
       <c r="E125" s="48" t="n">
-        <v>0.002994</v>
+        <v>0.00163</v>
       </c>
     </row>
     <row r="126">
@@ -22712,13 +22712,13 @@
         </is>
       </c>
       <c r="C126" s="26" t="n">
-        <v>46156</v>
+        <v>46093</v>
       </c>
       <c r="D126" s="47" t="n">
-        <v>27</v>
+        <v>46</v>
       </c>
       <c r="E126" s="48" t="n">
-        <v>0.001774</v>
+        <v>0.003151</v>
       </c>
     </row>
     <row r="127">
@@ -22733,13 +22733,13 @@
         </is>
       </c>
       <c r="C127" s="26" t="n">
-        <v>46185</v>
+        <v>46126</v>
       </c>
       <c r="D127" s="47" t="n">
-        <v>40</v>
+        <v>44</v>
       </c>
       <c r="E127" s="48" t="n">
-        <v>0.002525</v>
+        <v>0.002994</v>
       </c>
     </row>
     <row r="128">
@@ -22754,13 +22754,13 @@
         </is>
       </c>
       <c r="C128" s="26" t="n">
-        <v>46217</v>
+        <v>46156</v>
       </c>
       <c r="D128" s="47" t="n">
-        <v>50</v>
+        <v>27</v>
       </c>
       <c r="E128" s="48" t="n">
-        <v>0.003178</v>
+        <v>0.001774</v>
       </c>
     </row>
     <row r="129">
@@ -22775,13 +22775,13 @@
         </is>
       </c>
       <c r="C129" s="26" t="n">
-        <v>46247</v>
+        <v>46185</v>
       </c>
       <c r="D129" s="47" t="n">
-        <v>25</v>
+        <v>40</v>
       </c>
       <c r="E129" s="48" t="n">
-        <v>0.001604</v>
+        <v>0.002525</v>
       </c>
     </row>
     <row r="130">
@@ -22796,13 +22796,13 @@
         </is>
       </c>
       <c r="C130" s="26" t="n">
-        <v>46279</v>
+        <v>46217</v>
       </c>
       <c r="D130" s="47" t="n">
-        <v>35</v>
+        <v>50</v>
       </c>
       <c r="E130" s="48" t="n">
-        <v>0.002377</v>
+        <v>0.003178</v>
       </c>
     </row>
     <row r="131">
@@ -22817,55 +22817,55 @@
         </is>
       </c>
       <c r="C131" s="26" t="n">
-        <v>46309</v>
+        <v>46247</v>
       </c>
       <c r="D131" s="47" t="n">
-        <v>38</v>
+        <v>25</v>
       </c>
       <c r="E131" s="48" t="n">
-        <v>0.002624</v>
+        <v>0.001604</v>
       </c>
     </row>
     <row r="132">
       <c r="A132" s="46" t="inlineStr">
         <is>
-          <t>489250</t>
+          <t>402970</t>
         </is>
       </c>
       <c r="B132" s="33" t="inlineStr">
         <is>
-          <t>KODEX 미국배당다우존스</t>
+          <t>ACE 미국배당다우존스</t>
         </is>
       </c>
       <c r="C132" s="26" t="n">
-        <v>45547</v>
+        <v>46279</v>
       </c>
       <c r="D132" s="47" t="n">
-        <v>30</v>
+        <v>35</v>
       </c>
       <c r="E132" s="48" t="n">
-        <v>0.002954</v>
+        <v>0.002377</v>
       </c>
     </row>
     <row r="133">
       <c r="A133" s="46" t="inlineStr">
         <is>
-          <t>489250</t>
+          <t>402970</t>
         </is>
       </c>
       <c r="B133" s="33" t="inlineStr">
         <is>
-          <t>KODEX 미국배당다우존스</t>
+          <t>ACE 미국배당다우존스</t>
         </is>
       </c>
       <c r="C133" s="26" t="n">
-        <v>45579</v>
+        <v>46309</v>
       </c>
       <c r="D133" s="47" t="n">
-        <v>33</v>
+        <v>38</v>
       </c>
       <c r="E133" s="48" t="n">
-        <v>0.003148</v>
+        <v>0.002624</v>
       </c>
     </row>
     <row r="134">
@@ -22880,13 +22880,13 @@
         </is>
       </c>
       <c r="C134" s="26" t="n">
-        <v>45610</v>
+        <v>45547</v>
       </c>
       <c r="D134" s="47" t="n">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="E134" s="48" t="n">
-        <v>0.002509</v>
+        <v>0.002954</v>
       </c>
     </row>
     <row r="135">
@@ -22901,13 +22901,13 @@
         </is>
       </c>
       <c r="C135" s="26" t="n">
-        <v>45638</v>
+        <v>45579</v>
       </c>
       <c r="D135" s="47" t="n">
-        <v>41</v>
+        <v>33</v>
       </c>
       <c r="E135" s="48" t="n">
-        <v>0.003647</v>
+        <v>0.003148</v>
       </c>
     </row>
     <row r="136">
@@ -22922,13 +22922,13 @@
         </is>
       </c>
       <c r="C136" s="26" t="n">
-        <v>45671</v>
+        <v>45610</v>
       </c>
       <c r="D136" s="47" t="n">
-        <v>40</v>
+        <v>28</v>
       </c>
       <c r="E136" s="48" t="n">
-        <v>0.003659</v>
+        <v>0.002509</v>
       </c>
     </row>
     <row r="137">
@@ -22943,13 +22943,13 @@
         </is>
       </c>
       <c r="C137" s="26" t="n">
-        <v>45701</v>
+        <v>45638</v>
       </c>
       <c r="D137" s="47" t="n">
-        <v>32</v>
+        <v>41</v>
       </c>
       <c r="E137" s="48" t="n">
-        <v>0.002909</v>
+        <v>0.003647</v>
       </c>
     </row>
     <row r="138">
@@ -22964,13 +22964,13 @@
         </is>
       </c>
       <c r="C138" s="26" t="n">
-        <v>45729</v>
+        <v>45671</v>
       </c>
       <c r="D138" s="47" t="n">
-        <v>29</v>
+        <v>40</v>
       </c>
       <c r="E138" s="48" t="n">
-        <v>0.002634</v>
+        <v>0.003659</v>
       </c>
     </row>
     <row r="139">
@@ -22985,13 +22985,13 @@
         </is>
       </c>
       <c r="C139" s="26" t="n">
-        <v>45761</v>
+        <v>45701</v>
       </c>
       <c r="D139" s="47" t="n">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="E139" s="48" t="n">
-        <v>0.003378</v>
+        <v>0.002909</v>
       </c>
     </row>
     <row r="140">
@@ -23006,13 +23006,13 @@
         </is>
       </c>
       <c r="C140" s="26" t="n">
-        <v>45791</v>
+        <v>45729</v>
       </c>
       <c r="D140" s="47" t="n">
-        <v>24</v>
+        <v>29</v>
       </c>
       <c r="E140" s="48" t="n">
-        <v>0.002356</v>
+        <v>0.002634</v>
       </c>
     </row>
     <row r="141">
@@ -23027,13 +23027,13 @@
         </is>
       </c>
       <c r="C141" s="26" t="n">
-        <v>45820</v>
+        <v>45761</v>
       </c>
       <c r="D141" s="47" t="n">
-        <v>30</v>
+        <v>34</v>
       </c>
       <c r="E141" s="48" t="n">
-        <v>0.00299</v>
+        <v>0.003378</v>
       </c>
     </row>
     <row r="142">
@@ -23048,13 +23048,13 @@
         </is>
       </c>
       <c r="C142" s="26" t="n">
-        <v>45852</v>
+        <v>45791</v>
       </c>
       <c r="D142" s="47" t="n">
-        <v>31</v>
+        <v>24</v>
       </c>
       <c r="E142" s="48" t="n">
-        <v>0.003007</v>
+        <v>0.002356</v>
       </c>
     </row>
     <row r="143">
@@ -23069,13 +23069,13 @@
         </is>
       </c>
       <c r="C143" s="26" t="n">
-        <v>45882</v>
+        <v>45820</v>
       </c>
       <c r="D143" s="47" t="n">
-        <v>22</v>
+        <v>30</v>
       </c>
       <c r="E143" s="48" t="n">
-        <v>0.002165</v>
+        <v>0.00299</v>
       </c>
     </row>
     <row r="144">
@@ -23090,13 +23090,13 @@
         </is>
       </c>
       <c r="C144" s="26" t="n">
-        <v>45912</v>
+        <v>45852</v>
       </c>
       <c r="D144" s="47" t="n">
-        <v>28</v>
+        <v>31</v>
       </c>
       <c r="E144" s="48" t="n">
-        <v>0.002688</v>
+        <v>0.003007</v>
       </c>
     </row>
     <row r="145">
@@ -23111,13 +23111,13 @@
         </is>
       </c>
       <c r="C145" s="26" t="n">
-        <v>45944</v>
+        <v>45882</v>
       </c>
       <c r="D145" s="47" t="n">
-        <v>31</v>
+        <v>22</v>
       </c>
       <c r="E145" s="48" t="n">
-        <v>0.002989</v>
+        <v>0.002165</v>
       </c>
     </row>
     <row r="146">
@@ -23132,13 +23132,13 @@
         </is>
       </c>
       <c r="C146" s="26" t="n">
-        <v>45974</v>
+        <v>45912</v>
       </c>
       <c r="D146" s="47" t="n">
-        <v>21</v>
+        <v>28</v>
       </c>
       <c r="E146" s="48" t="n">
-        <v>0.001939</v>
+        <v>0.002688</v>
       </c>
     </row>
     <row r="147">
@@ -23153,13 +23153,13 @@
         </is>
       </c>
       <c r="C147" s="26" t="n">
-        <v>46003</v>
+        <v>45944</v>
       </c>
       <c r="D147" s="47" t="n">
-        <v>33</v>
+        <v>31</v>
       </c>
       <c r="E147" s="48" t="n">
-        <v>0.002966</v>
+        <v>0.002989</v>
       </c>
     </row>
     <row r="148">
@@ -23174,13 +23174,13 @@
         </is>
       </c>
       <c r="C148" s="26" t="n">
-        <v>46036</v>
+        <v>45974</v>
       </c>
       <c r="D148" s="47" t="n">
-        <v>34</v>
+        <v>21</v>
       </c>
       <c r="E148" s="48" t="n">
-        <v>0.002964</v>
+        <v>0.001939</v>
       </c>
     </row>
     <row r="149">
@@ -23195,13 +23195,13 @@
         </is>
       </c>
       <c r="C149" s="26" t="n">
-        <v>46065</v>
+        <v>46003</v>
       </c>
       <c r="D149" s="47" t="n">
-        <v>28</v>
+        <v>33</v>
       </c>
       <c r="E149" s="48" t="n">
-        <v>0.00224</v>
+        <v>0.002966</v>
       </c>
     </row>
     <row r="150">
@@ -23216,13 +23216,13 @@
         </is>
       </c>
       <c r="C150" s="26" t="n">
-        <v>46093</v>
+        <v>46036</v>
       </c>
       <c r="D150" s="47" t="n">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="E150" s="48" t="n">
-        <v>0.002589</v>
+        <v>0.002964</v>
       </c>
     </row>
     <row r="151">
@@ -23237,13 +23237,13 @@
         </is>
       </c>
       <c r="C151" s="26" t="n">
-        <v>46126</v>
+        <v>46065</v>
       </c>
       <c r="D151" s="47" t="n">
-        <v>33</v>
+        <v>28</v>
       </c>
       <c r="E151" s="48" t="n">
-        <v>0.002645</v>
+        <v>0.00224</v>
       </c>
     </row>
     <row r="152">
@@ -23258,13 +23258,13 @@
         </is>
       </c>
       <c r="C152" s="26" t="n">
-        <v>46156</v>
+        <v>46093</v>
       </c>
       <c r="D152" s="47" t="n">
-        <v>26</v>
+        <v>32</v>
       </c>
       <c r="E152" s="48" t="n">
-        <v>0.002016</v>
+        <v>0.002589</v>
       </c>
     </row>
     <row r="153">
@@ -23279,13 +23279,13 @@
         </is>
       </c>
       <c r="C153" s="26" t="n">
-        <v>46185</v>
+        <v>46126</v>
       </c>
       <c r="D153" s="47" t="n">
-        <v>29</v>
+        <v>33</v>
       </c>
       <c r="E153" s="48" t="n">
-        <v>0.002161</v>
+        <v>0.002645</v>
       </c>
     </row>
     <row r="154">
@@ -23300,13 +23300,13 @@
         </is>
       </c>
       <c r="C154" s="26" t="n">
-        <v>46217</v>
+        <v>46156</v>
       </c>
       <c r="D154" s="47" t="n">
-        <v>40</v>
+        <v>26</v>
       </c>
       <c r="E154" s="48" t="n">
-        <v>0.003001</v>
+        <v>0.002016</v>
       </c>
     </row>
     <row r="155">
@@ -23321,13 +23321,13 @@
         </is>
       </c>
       <c r="C155" s="26" t="n">
-        <v>46247</v>
+        <v>46185</v>
       </c>
       <c r="D155" s="47" t="n">
-        <v>37</v>
+        <v>29</v>
       </c>
       <c r="E155" s="48" t="n">
-        <v>0.0028</v>
+        <v>0.002161</v>
       </c>
     </row>
     <row r="156">
@@ -23342,13 +23342,13 @@
         </is>
       </c>
       <c r="C156" s="26" t="n">
-        <v>46279</v>
+        <v>46217</v>
       </c>
       <c r="D156" s="47" t="n">
-        <v>24</v>
+        <v>40</v>
       </c>
       <c r="E156" s="48" t="n">
-        <v>0.001924</v>
+        <v>0.003001</v>
       </c>
     </row>
     <row r="157">
@@ -23363,28 +23363,56 @@
         </is>
       </c>
       <c r="C157" s="26" t="n">
-        <v>46309</v>
+        <v>46247</v>
       </c>
       <c r="D157" s="47" t="n">
         <v>37</v>
       </c>
       <c r="E157" s="48" t="n">
+        <v>0.0028</v>
+      </c>
+    </row>
+    <row r="158">
+      <c r="A158" s="46" t="inlineStr">
+        <is>
+          <t>489250</t>
+        </is>
+      </c>
+      <c r="B158" s="33" t="inlineStr">
+        <is>
+          <t>KODEX 미국배당다우존스</t>
+        </is>
+      </c>
+      <c r="C158" s="26" t="n">
+        <v>46279</v>
+      </c>
+      <c r="D158" s="47" t="n">
+        <v>24</v>
+      </c>
+      <c r="E158" s="48" t="n">
+        <v>0.001924</v>
+      </c>
+    </row>
+    <row r="159">
+      <c r="A159" s="46" t="inlineStr">
+        <is>
+          <t>489250</t>
+        </is>
+      </c>
+      <c r="B159" s="33" t="inlineStr">
+        <is>
+          <t>KODEX 미국배당다우존스</t>
+        </is>
+      </c>
+      <c r="C159" s="26" t="n">
+        <v>46309</v>
+      </c>
+      <c r="D159" s="47" t="n">
+        <v>37</v>
+      </c>
+      <c r="E159" s="48" t="n">
         <v>0.003019</v>
       </c>
-    </row>
-    <row r="158">
-      <c r="A158" s="46" t="n"/>
-      <c r="B158" s="33" t="n"/>
-      <c r="C158" s="26" t="n"/>
-      <c r="D158" s="47" t="n"/>
-      <c r="E158" s="48" t="n"/>
-    </row>
-    <row r="159">
-      <c r="A159" s="46" t="n"/>
-      <c r="B159" s="33" t="n"/>
-      <c r="C159" s="26" t="n"/>
-      <c r="D159" s="47" t="n"/>
-      <c r="E159" s="48" t="n"/>
     </row>
     <row r="160">
       <c r="A160" s="46" t="n"/>
@@ -24771,6 +24799,20 @@
       <c r="C357" s="26" t="n"/>
       <c r="D357" s="47" t="n"/>
       <c r="E357" s="48" t="n"/>
+    </row>
+    <row r="358">
+      <c r="A358" s="46" t="n"/>
+      <c r="B358" s="33" t="n"/>
+      <c r="C358" s="26" t="n"/>
+      <c r="D358" s="47" t="n"/>
+      <c r="E358" s="48" t="n"/>
+    </row>
+    <row r="359">
+      <c r="A359" s="46" t="n"/>
+      <c r="B359" s="33" t="n"/>
+      <c r="C359" s="26" t="n"/>
+      <c r="D359" s="47" t="n"/>
+      <c r="E359" s="48" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -24892,23 +24934,23 @@
         </is>
       </c>
       <c r="E6" s="52">
-        <f>_xlfn.MAXIFS(국내SCHD형_분배!$C$2:$C$357,국내SCHD형_분배!$A$2:$A$357,$B6,국내SCHD형_분배!$C$2:$C$357,"&lt;="&amp;$B$3)</f>
+        <f>_xlfn.MAXIFS(국내SCHD형_분배!$C$2:$C$359,국내SCHD형_분배!$A$2:$A$359,$B6,국내SCHD형_분배!$C$2:$C$359,"&lt;="&amp;$B$3)</f>
         <v/>
       </c>
       <c r="F6" s="53">
-        <f>SUMIFS(국내SCHD형_분배!$D$2:$D$357,국내SCHD형_분배!$A$2:$A$357,$B6,국내SCHD형_분배!$C$2:$C$357,E6)</f>
+        <f>SUMIFS(국내SCHD형_분배!$D$2:$D$359,국내SCHD형_분배!$A$2:$A$359,$B6,국내SCHD형_분배!$C$2:$C$359,E6)</f>
         <v/>
       </c>
       <c r="G6" s="45">
-        <f>COUNTIFS(국내SCHD형_분배!$A$2:$A$357,$B6,국내SCHD형_분배!$C$2:$C$357,"&gt;"&amp;EDATE($B$3,-12),국내SCHD형_분배!$C$2:$C$357,"&lt;="&amp;$B$3)</f>
+        <f>COUNTIFS(국내SCHD형_분배!$A$2:$A$359,$B6,국내SCHD형_분배!$C$2:$C$359,"&gt;"&amp;EDATE($B$3,-12),국내SCHD형_분배!$C$2:$C$359,"&lt;="&amp;$B$3)</f>
         <v/>
       </c>
       <c r="H6" s="53">
-        <f>SUMIFS(국내SCHD형_분배!$D$2:$D$357,국내SCHD형_분배!$A$2:$A$357,$B6,국내SCHD형_분배!$C$2:$C$357,"&gt;"&amp;EDATE($B$3,-12),국내SCHD형_분배!$C$2:$C$357,"&lt;="&amp;$B$3)</f>
+        <f>SUMIFS(국내SCHD형_분배!$D$2:$D$359,국내SCHD형_분배!$A$2:$A$359,$B6,국내SCHD형_분배!$C$2:$C$359,"&gt;"&amp;EDATE($B$3,-12),국내SCHD형_분배!$C$2:$C$359,"&lt;="&amp;$B$3)</f>
         <v/>
       </c>
       <c r="I6" s="29">
-        <f>SUMIFS(국내SCHD형_분배!$E$2:$E$357,국내SCHD형_분배!$A$2:$A$357,$B6,국내SCHD형_분배!$C$2:$C$357,"&gt;"&amp;EDATE($B$3,-12),국내SCHD형_분배!$C$2:$C$357,"&lt;="&amp;$B$3)</f>
+        <f>SUMIFS(국내SCHD형_분배!$E$2:$E$359,국내SCHD형_분배!$A$2:$A$359,$B6,국내SCHD형_분배!$C$2:$C$359,"&gt;"&amp;EDATE($B$3,-12),국내SCHD형_분배!$C$2:$C$359,"&lt;="&amp;$B$3)</f>
         <v/>
       </c>
     </row>
@@ -24932,23 +24974,23 @@
         </is>
       </c>
       <c r="E7" s="52">
-        <f>_xlfn.MAXIFS(국내SCHD형_분배!$C$2:$C$357,국내SCHD형_분배!$A$2:$A$357,$B7,국내SCHD형_분배!$C$2:$C$357,"&lt;="&amp;$B$3)</f>
+        <f>_xlfn.MAXIFS(국내SCHD형_분배!$C$2:$C$359,국내SCHD형_분배!$A$2:$A$359,$B7,국내SCHD형_분배!$C$2:$C$359,"&lt;="&amp;$B$3)</f>
         <v/>
       </c>
       <c r="F7" s="53">
-        <f>SUMIFS(국내SCHD형_분배!$D$2:$D$357,국내SCHD형_분배!$A$2:$A$357,$B7,국내SCHD형_분배!$C$2:$C$357,E7)</f>
+        <f>SUMIFS(국내SCHD형_분배!$D$2:$D$359,국내SCHD형_분배!$A$2:$A$359,$B7,국내SCHD형_분배!$C$2:$C$359,E7)</f>
         <v/>
       </c>
       <c r="G7" s="45">
-        <f>COUNTIFS(국내SCHD형_분배!$A$2:$A$357,$B7,국내SCHD형_분배!$C$2:$C$357,"&gt;"&amp;EDATE($B$3,-12),국내SCHD형_분배!$C$2:$C$357,"&lt;="&amp;$B$3)</f>
+        <f>COUNTIFS(국내SCHD형_분배!$A$2:$A$359,$B7,국내SCHD형_분배!$C$2:$C$359,"&gt;"&amp;EDATE($B$3,-12),국내SCHD형_분배!$C$2:$C$359,"&lt;="&amp;$B$3)</f>
         <v/>
       </c>
       <c r="H7" s="53">
-        <f>SUMIFS(국내SCHD형_분배!$D$2:$D$357,국내SCHD형_분배!$A$2:$A$357,$B7,국내SCHD형_분배!$C$2:$C$357,"&gt;"&amp;EDATE($B$3,-12),국내SCHD형_분배!$C$2:$C$357,"&lt;="&amp;$B$3)</f>
+        <f>SUMIFS(국내SCHD형_분배!$D$2:$D$359,국내SCHD형_분배!$A$2:$A$359,$B7,국내SCHD형_분배!$C$2:$C$359,"&gt;"&amp;EDATE($B$3,-12),국내SCHD형_분배!$C$2:$C$359,"&lt;="&amp;$B$3)</f>
         <v/>
       </c>
       <c r="I7" s="29">
-        <f>SUMIFS(국내SCHD형_분배!$E$2:$E$357,국내SCHD형_분배!$A$2:$A$357,$B7,국내SCHD형_분배!$C$2:$C$357,"&gt;"&amp;EDATE($B$3,-12),국내SCHD형_분배!$C$2:$C$357,"&lt;="&amp;$B$3)</f>
+        <f>SUMIFS(국내SCHD형_분배!$E$2:$E$359,국내SCHD형_분배!$A$2:$A$359,$B7,국내SCHD형_분배!$C$2:$C$359,"&gt;"&amp;EDATE($B$3,-12),국내SCHD형_분배!$C$2:$C$359,"&lt;="&amp;$B$3)</f>
         <v/>
       </c>
     </row>
@@ -24972,23 +25014,23 @@
         </is>
       </c>
       <c r="E8" s="52">
-        <f>_xlfn.MAXIFS(국내SCHD형_분배!$C$2:$C$357,국내SCHD형_분배!$A$2:$A$357,$B8,국내SCHD형_분배!$C$2:$C$357,"&lt;="&amp;$B$3)</f>
+        <f>_xlfn.MAXIFS(국내SCHD형_분배!$C$2:$C$359,국내SCHD형_분배!$A$2:$A$359,$B8,국내SCHD형_분배!$C$2:$C$359,"&lt;="&amp;$B$3)</f>
         <v/>
       </c>
       <c r="F8" s="53">
-        <f>SUMIFS(국내SCHD형_분배!$D$2:$D$357,국내SCHD형_분배!$A$2:$A$357,$B8,국내SCHD형_분배!$C$2:$C$357,E8)</f>
+        <f>SUMIFS(국내SCHD형_분배!$D$2:$D$359,국내SCHD형_분배!$A$2:$A$359,$B8,국내SCHD형_분배!$C$2:$C$359,E8)</f>
         <v/>
       </c>
       <c r="G8" s="45">
-        <f>COUNTIFS(국내SCHD형_분배!$A$2:$A$357,$B8,국내SCHD형_분배!$C$2:$C$357,"&gt;"&amp;EDATE($B$3,-12),국내SCHD형_분배!$C$2:$C$357,"&lt;="&amp;$B$3)</f>
+        <f>COUNTIFS(국내SCHD형_분배!$A$2:$A$359,$B8,국내SCHD형_분배!$C$2:$C$359,"&gt;"&amp;EDATE($B$3,-12),국내SCHD형_분배!$C$2:$C$359,"&lt;="&amp;$B$3)</f>
         <v/>
       </c>
       <c r="H8" s="53">
-        <f>SUMIFS(국내SCHD형_분배!$D$2:$D$357,국내SCHD형_분배!$A$2:$A$357,$B8,국내SCHD형_분배!$C$2:$C$357,"&gt;"&amp;EDATE($B$3,-12),국내SCHD형_분배!$C$2:$C$357,"&lt;="&amp;$B$3)</f>
+        <f>SUMIFS(국내SCHD형_분배!$D$2:$D$359,국내SCHD형_분배!$A$2:$A$359,$B8,국내SCHD형_분배!$C$2:$C$359,"&gt;"&amp;EDATE($B$3,-12),국내SCHD형_분배!$C$2:$C$359,"&lt;="&amp;$B$3)</f>
         <v/>
       </c>
       <c r="I8" s="29">
-        <f>SUMIFS(국내SCHD형_분배!$E$2:$E$357,국내SCHD형_분배!$A$2:$A$357,$B8,국내SCHD형_분배!$C$2:$C$357,"&gt;"&amp;EDATE($B$3,-12),국내SCHD형_분배!$C$2:$C$357,"&lt;="&amp;$B$3)</f>
+        <f>SUMIFS(국내SCHD형_분배!$E$2:$E$359,국내SCHD형_분배!$A$2:$A$359,$B8,국내SCHD형_분배!$C$2:$C$359,"&gt;"&amp;EDATE($B$3,-12),국내SCHD형_분배!$C$2:$C$359,"&lt;="&amp;$B$3)</f>
         <v/>
       </c>
     </row>
@@ -25012,23 +25054,23 @@
         </is>
       </c>
       <c r="E9" s="52">
-        <f>_xlfn.MAXIFS(국내SCHD형_분배!$C$2:$C$357,국내SCHD형_분배!$A$2:$A$357,$B9,국내SCHD형_분배!$C$2:$C$357,"&lt;="&amp;$B$3)</f>
+        <f>_xlfn.MAXIFS(국내SCHD형_분배!$C$2:$C$359,국내SCHD형_분배!$A$2:$A$359,$B9,국내SCHD형_분배!$C$2:$C$359,"&lt;="&amp;$B$3)</f>
         <v/>
       </c>
       <c r="F9" s="53">
-        <f>SUMIFS(국내SCHD형_분배!$D$2:$D$357,국내SCHD형_분배!$A$2:$A$357,$B9,국내SCHD형_분배!$C$2:$C$357,E9)</f>
+        <f>SUMIFS(국내SCHD형_분배!$D$2:$D$359,국내SCHD형_분배!$A$2:$A$359,$B9,국내SCHD형_분배!$C$2:$C$359,E9)</f>
         <v/>
       </c>
       <c r="G9" s="45">
-        <f>COUNTIFS(국내SCHD형_분배!$A$2:$A$357,$B9,국내SCHD형_분배!$C$2:$C$357,"&gt;"&amp;EDATE($B$3,-12),국내SCHD형_분배!$C$2:$C$357,"&lt;="&amp;$B$3)</f>
+        <f>COUNTIFS(국내SCHD형_분배!$A$2:$A$359,$B9,국내SCHD형_분배!$C$2:$C$359,"&gt;"&amp;EDATE($B$3,-12),국내SCHD형_분배!$C$2:$C$359,"&lt;="&amp;$B$3)</f>
         <v/>
       </c>
       <c r="H9" s="53">
-        <f>SUMIFS(국내SCHD형_분배!$D$2:$D$357,국내SCHD형_분배!$A$2:$A$357,$B9,국내SCHD형_분배!$C$2:$C$357,"&gt;"&amp;EDATE($B$3,-12),국내SCHD형_분배!$C$2:$C$357,"&lt;="&amp;$B$3)</f>
+        <f>SUMIFS(국내SCHD형_분배!$D$2:$D$359,국내SCHD형_분배!$A$2:$A$359,$B9,국내SCHD형_분배!$C$2:$C$359,"&gt;"&amp;EDATE($B$3,-12),국내SCHD형_분배!$C$2:$C$359,"&lt;="&amp;$B$3)</f>
         <v/>
       </c>
       <c r="I9" s="29">
-        <f>SUMIFS(국내SCHD형_분배!$E$2:$E$357,국내SCHD형_분배!$A$2:$A$357,$B9,국내SCHD형_분배!$C$2:$C$357,"&gt;"&amp;EDATE($B$3,-12),국내SCHD형_분배!$C$2:$C$357,"&lt;="&amp;$B$3)</f>
+        <f>SUMIFS(국내SCHD형_분배!$E$2:$E$359,국내SCHD형_분배!$A$2:$A$359,$B9,국내SCHD형_분배!$C$2:$C$359,"&gt;"&amp;EDATE($B$3,-12),국내SCHD형_분배!$C$2:$C$359,"&lt;="&amp;$B$3)</f>
         <v/>
       </c>
     </row>
@@ -25163,19 +25205,19 @@
         <v/>
       </c>
       <c r="D17" s="53">
-        <f>IF(COUNTIFS(국내SCHD형_분배!$A$2:$A$357,"458730",국내SCHD형_분배!$C$2:$C$357,"&gt;="&amp;$B17,국내SCHD형_분배!$C$2:$C$357,"&lt;="&amp;$C17)=0,"",SUMIFS(국내SCHD형_분배!$D$2:$D$357,국내SCHD형_분배!$A$2:$A$357,"458730",국내SCHD형_분배!$C$2:$C$357,"&gt;="&amp;$B17,국내SCHD형_분배!$C$2:$C$357,"&lt;="&amp;$C17))</f>
+        <f>IF(COUNTIFS(국내SCHD형_분배!$A$2:$A$359,"458730",국내SCHD형_분배!$C$2:$C$359,"&gt;="&amp;$B17,국내SCHD형_분배!$C$2:$C$359,"&lt;="&amp;$C17)=0,"",SUMIFS(국내SCHD형_분배!$D$2:$D$359,국내SCHD형_분배!$A$2:$A$359,"458730",국내SCHD형_분배!$C$2:$C$359,"&gt;="&amp;$B17,국내SCHD형_분배!$C$2:$C$359,"&lt;="&amp;$C17))</f>
         <v/>
       </c>
       <c r="E17" s="53">
-        <f>IF(COUNTIFS(국내SCHD형_분배!$A$2:$A$357,"446720",국내SCHD형_분배!$C$2:$C$357,"&gt;="&amp;$B17,국내SCHD형_분배!$C$2:$C$357,"&lt;="&amp;$C17)=0,"",SUMIFS(국내SCHD형_분배!$D$2:$D$357,국내SCHD형_분배!$A$2:$A$357,"446720",국내SCHD형_분배!$C$2:$C$357,"&gt;="&amp;$B17,국내SCHD형_분배!$C$2:$C$357,"&lt;="&amp;$C17))</f>
+        <f>IF(COUNTIFS(국내SCHD형_분배!$A$2:$A$359,"446720",국내SCHD형_분배!$C$2:$C$359,"&gt;="&amp;$B17,국내SCHD형_분배!$C$2:$C$359,"&lt;="&amp;$C17)=0,"",SUMIFS(국내SCHD형_분배!$D$2:$D$359,국내SCHD형_분배!$A$2:$A$359,"446720",국내SCHD형_분배!$C$2:$C$359,"&gt;="&amp;$B17,국내SCHD형_분배!$C$2:$C$359,"&lt;="&amp;$C17))</f>
         <v/>
       </c>
       <c r="F17" s="53">
-        <f>IF(COUNTIFS(국내SCHD형_분배!$A$2:$A$357,"402970",국내SCHD형_분배!$C$2:$C$357,"&gt;="&amp;$B17,국내SCHD형_분배!$C$2:$C$357,"&lt;="&amp;$C17)=0,"",SUMIFS(국내SCHD형_분배!$D$2:$D$357,국내SCHD형_분배!$A$2:$A$357,"402970",국내SCHD형_분배!$C$2:$C$357,"&gt;="&amp;$B17,국내SCHD형_분배!$C$2:$C$357,"&lt;="&amp;$C17))</f>
+        <f>IF(COUNTIFS(국내SCHD형_분배!$A$2:$A$359,"402970",국내SCHD형_분배!$C$2:$C$359,"&gt;="&amp;$B17,국내SCHD형_분배!$C$2:$C$359,"&lt;="&amp;$C17)=0,"",SUMIFS(국내SCHD형_분배!$D$2:$D$359,국내SCHD형_분배!$A$2:$A$359,"402970",국내SCHD형_분배!$C$2:$C$359,"&gt;="&amp;$B17,국내SCHD형_분배!$C$2:$C$359,"&lt;="&amp;$C17))</f>
         <v/>
       </c>
       <c r="G17" s="53">
-        <f>IF(COUNTIFS(국내SCHD형_분배!$A$2:$A$357,"489250",국내SCHD형_분배!$C$2:$C$357,"&gt;="&amp;$B17,국내SCHD형_분배!$C$2:$C$357,"&lt;="&amp;$C17)=0,"",SUMIFS(국내SCHD형_분배!$D$2:$D$357,국내SCHD형_분배!$A$2:$A$357,"489250",국내SCHD형_분배!$C$2:$C$357,"&gt;="&amp;$B17,국내SCHD형_분배!$C$2:$C$357,"&lt;="&amp;$C17))</f>
+        <f>IF(COUNTIFS(국내SCHD형_분배!$A$2:$A$359,"489250",국내SCHD형_분배!$C$2:$C$359,"&gt;="&amp;$B17,국내SCHD형_분배!$C$2:$C$359,"&lt;="&amp;$C17)=0,"",SUMIFS(국내SCHD형_분배!$D$2:$D$359,국내SCHD형_분배!$A$2:$A$359,"489250",국내SCHD형_분배!$C$2:$C$359,"&gt;="&amp;$B17,국내SCHD형_분배!$C$2:$C$359,"&lt;="&amp;$C17))</f>
         <v/>
       </c>
       <c r="H17" s="28">
@@ -25201,19 +25243,19 @@
         <v/>
       </c>
       <c r="D18" s="53">
-        <f>IF(COUNTIFS(국내SCHD형_분배!$A$2:$A$357,"458730",국내SCHD형_분배!$C$2:$C$357,"&gt;="&amp;$B18,국내SCHD형_분배!$C$2:$C$357,"&lt;="&amp;$C18)=0,"",SUMIFS(국내SCHD형_분배!$D$2:$D$357,국내SCHD형_분배!$A$2:$A$357,"458730",국내SCHD형_분배!$C$2:$C$357,"&gt;="&amp;$B18,국내SCHD형_분배!$C$2:$C$357,"&lt;="&amp;$C18))</f>
+        <f>IF(COUNTIFS(국내SCHD형_분배!$A$2:$A$359,"458730",국내SCHD형_분배!$C$2:$C$359,"&gt;="&amp;$B18,국내SCHD형_분배!$C$2:$C$359,"&lt;="&amp;$C18)=0,"",SUMIFS(국내SCHD형_분배!$D$2:$D$359,국내SCHD형_분배!$A$2:$A$359,"458730",국내SCHD형_분배!$C$2:$C$359,"&gt;="&amp;$B18,국내SCHD형_분배!$C$2:$C$359,"&lt;="&amp;$C18))</f>
         <v/>
       </c>
       <c r="E18" s="53">
-        <f>IF(COUNTIFS(국내SCHD형_분배!$A$2:$A$357,"446720",국내SCHD형_분배!$C$2:$C$357,"&gt;="&amp;$B18,국내SCHD형_분배!$C$2:$C$357,"&lt;="&amp;$C18)=0,"",SUMIFS(국내SCHD형_분배!$D$2:$D$357,국내SCHD형_분배!$A$2:$A$357,"446720",국내SCHD형_분배!$C$2:$C$357,"&gt;="&amp;$B18,국내SCHD형_분배!$C$2:$C$357,"&lt;="&amp;$C18))</f>
+        <f>IF(COUNTIFS(국내SCHD형_분배!$A$2:$A$359,"446720",국내SCHD형_분배!$C$2:$C$359,"&gt;="&amp;$B18,국내SCHD형_분배!$C$2:$C$359,"&lt;="&amp;$C18)=0,"",SUMIFS(국내SCHD형_분배!$D$2:$D$359,국내SCHD형_분배!$A$2:$A$359,"446720",국내SCHD형_분배!$C$2:$C$359,"&gt;="&amp;$B18,국내SCHD형_분배!$C$2:$C$359,"&lt;="&amp;$C18))</f>
         <v/>
       </c>
       <c r="F18" s="53">
-        <f>IF(COUNTIFS(국내SCHD형_분배!$A$2:$A$357,"402970",국내SCHD형_분배!$C$2:$C$357,"&gt;="&amp;$B18,국내SCHD형_분배!$C$2:$C$357,"&lt;="&amp;$C18)=0,"",SUMIFS(국내SCHD형_분배!$D$2:$D$357,국내SCHD형_분배!$A$2:$A$357,"402970",국내SCHD형_분배!$C$2:$C$357,"&gt;="&amp;$B18,국내SCHD형_분배!$C$2:$C$357,"&lt;="&amp;$C18))</f>
+        <f>IF(COUNTIFS(국내SCHD형_분배!$A$2:$A$359,"402970",국내SCHD형_분배!$C$2:$C$359,"&gt;="&amp;$B18,국내SCHD형_분배!$C$2:$C$359,"&lt;="&amp;$C18)=0,"",SUMIFS(국내SCHD형_분배!$D$2:$D$359,국내SCHD형_분배!$A$2:$A$359,"402970",국내SCHD형_분배!$C$2:$C$359,"&gt;="&amp;$B18,국내SCHD형_분배!$C$2:$C$359,"&lt;="&amp;$C18))</f>
         <v/>
       </c>
       <c r="G18" s="53">
-        <f>IF(COUNTIFS(국내SCHD형_분배!$A$2:$A$357,"489250",국내SCHD형_분배!$C$2:$C$357,"&gt;="&amp;$B18,국내SCHD형_분배!$C$2:$C$357,"&lt;="&amp;$C18)=0,"",SUMIFS(국내SCHD형_분배!$D$2:$D$357,국내SCHD형_분배!$A$2:$A$357,"489250",국내SCHD형_분배!$C$2:$C$357,"&gt;="&amp;$B18,국내SCHD형_분배!$C$2:$C$357,"&lt;="&amp;$C18))</f>
+        <f>IF(COUNTIFS(국내SCHD형_분배!$A$2:$A$359,"489250",국내SCHD형_분배!$C$2:$C$359,"&gt;="&amp;$B18,국내SCHD형_분배!$C$2:$C$359,"&lt;="&amp;$C18)=0,"",SUMIFS(국내SCHD형_분배!$D$2:$D$359,국내SCHD형_분배!$A$2:$A$359,"489250",국내SCHD형_분배!$C$2:$C$359,"&gt;="&amp;$B18,국내SCHD형_분배!$C$2:$C$359,"&lt;="&amp;$C18))</f>
         <v/>
       </c>
       <c r="H18" s="28">
@@ -25239,19 +25281,19 @@
         <v/>
       </c>
       <c r="D19" s="53">
-        <f>IF(COUNTIFS(국내SCHD형_분배!$A$2:$A$357,"458730",국내SCHD형_분배!$C$2:$C$357,"&gt;="&amp;$B19,국내SCHD형_분배!$C$2:$C$357,"&lt;="&amp;$C19)=0,"",SUMIFS(국내SCHD형_분배!$D$2:$D$357,국내SCHD형_분배!$A$2:$A$357,"458730",국내SCHD형_분배!$C$2:$C$357,"&gt;="&amp;$B19,국내SCHD형_분배!$C$2:$C$357,"&lt;="&amp;$C19))</f>
+        <f>IF(COUNTIFS(국내SCHD형_분배!$A$2:$A$359,"458730",국내SCHD형_분배!$C$2:$C$359,"&gt;="&amp;$B19,국내SCHD형_분배!$C$2:$C$359,"&lt;="&amp;$C19)=0,"",SUMIFS(국내SCHD형_분배!$D$2:$D$359,국내SCHD형_분배!$A$2:$A$359,"458730",국내SCHD형_분배!$C$2:$C$359,"&gt;="&amp;$B19,국내SCHD형_분배!$C$2:$C$359,"&lt;="&amp;$C19))</f>
         <v/>
       </c>
       <c r="E19" s="53">
-        <f>IF(COUNTIFS(국내SCHD형_분배!$A$2:$A$357,"446720",국내SCHD형_분배!$C$2:$C$357,"&gt;="&amp;$B19,국내SCHD형_분배!$C$2:$C$357,"&lt;="&amp;$C19)=0,"",SUMIFS(국내SCHD형_분배!$D$2:$D$357,국내SCHD형_분배!$A$2:$A$357,"446720",국내SCHD형_분배!$C$2:$C$357,"&gt;="&amp;$B19,국내SCHD형_분배!$C$2:$C$357,"&lt;="&amp;$C19))</f>
+        <f>IF(COUNTIFS(국내SCHD형_분배!$A$2:$A$359,"446720",국내SCHD형_분배!$C$2:$C$359,"&gt;="&amp;$B19,국내SCHD형_분배!$C$2:$C$359,"&lt;="&amp;$C19)=0,"",SUMIFS(국내SCHD형_분배!$D$2:$D$359,국내SCHD형_분배!$A$2:$A$359,"446720",국내SCHD형_분배!$C$2:$C$359,"&gt;="&amp;$B19,국내SCHD형_분배!$C$2:$C$359,"&lt;="&amp;$C19))</f>
         <v/>
       </c>
       <c r="F19" s="53">
-        <f>IF(COUNTIFS(국내SCHD형_분배!$A$2:$A$357,"402970",국내SCHD형_분배!$C$2:$C$357,"&gt;="&amp;$B19,국내SCHD형_분배!$C$2:$C$357,"&lt;="&amp;$C19)=0,"",SUMIFS(국내SCHD형_분배!$D$2:$D$357,국내SCHD형_분배!$A$2:$A$357,"402970",국내SCHD형_분배!$C$2:$C$357,"&gt;="&amp;$B19,국내SCHD형_분배!$C$2:$C$357,"&lt;="&amp;$C19))</f>
+        <f>IF(COUNTIFS(국내SCHD형_분배!$A$2:$A$359,"402970",국내SCHD형_분배!$C$2:$C$359,"&gt;="&amp;$B19,국내SCHD형_분배!$C$2:$C$359,"&lt;="&amp;$C19)=0,"",SUMIFS(국내SCHD형_분배!$D$2:$D$359,국내SCHD형_분배!$A$2:$A$359,"402970",국내SCHD형_분배!$C$2:$C$359,"&gt;="&amp;$B19,국내SCHD형_분배!$C$2:$C$359,"&lt;="&amp;$C19))</f>
         <v/>
       </c>
       <c r="G19" s="53">
-        <f>IF(COUNTIFS(국내SCHD형_분배!$A$2:$A$357,"489250",국내SCHD형_분배!$C$2:$C$357,"&gt;="&amp;$B19,국내SCHD형_분배!$C$2:$C$357,"&lt;="&amp;$C19)=0,"",SUMIFS(국내SCHD형_분배!$D$2:$D$357,국내SCHD형_분배!$A$2:$A$357,"489250",국내SCHD형_분배!$C$2:$C$357,"&gt;="&amp;$B19,국내SCHD형_분배!$C$2:$C$357,"&lt;="&amp;$C19))</f>
+        <f>IF(COUNTIFS(국내SCHD형_분배!$A$2:$A$359,"489250",국내SCHD형_분배!$C$2:$C$359,"&gt;="&amp;$B19,국내SCHD형_분배!$C$2:$C$359,"&lt;="&amp;$C19)=0,"",SUMIFS(국내SCHD형_분배!$D$2:$D$359,국내SCHD형_분배!$A$2:$A$359,"489250",국내SCHD형_분배!$C$2:$C$359,"&gt;="&amp;$B19,국내SCHD형_분배!$C$2:$C$359,"&lt;="&amp;$C19))</f>
         <v/>
       </c>
       <c r="H19" s="28">
@@ -25277,19 +25319,19 @@
         <v/>
       </c>
       <c r="D20" s="53">
-        <f>IF(COUNTIFS(국내SCHD형_분배!$A$2:$A$357,"458730",국내SCHD형_분배!$C$2:$C$357,"&gt;="&amp;$B20,국내SCHD형_분배!$C$2:$C$357,"&lt;="&amp;$C20)=0,"",SUMIFS(국내SCHD형_분배!$D$2:$D$357,국내SCHD형_분배!$A$2:$A$357,"458730",국내SCHD형_분배!$C$2:$C$357,"&gt;="&amp;$B20,국내SCHD형_분배!$C$2:$C$357,"&lt;="&amp;$C20))</f>
+        <f>IF(COUNTIFS(국내SCHD형_분배!$A$2:$A$359,"458730",국내SCHD형_분배!$C$2:$C$359,"&gt;="&amp;$B20,국내SCHD형_분배!$C$2:$C$359,"&lt;="&amp;$C20)=0,"",SUMIFS(국내SCHD형_분배!$D$2:$D$359,국내SCHD형_분배!$A$2:$A$359,"458730",국내SCHD형_분배!$C$2:$C$359,"&gt;="&amp;$B20,국내SCHD형_분배!$C$2:$C$359,"&lt;="&amp;$C20))</f>
         <v/>
       </c>
       <c r="E20" s="53">
-        <f>IF(COUNTIFS(국내SCHD형_분배!$A$2:$A$357,"446720",국내SCHD형_분배!$C$2:$C$357,"&gt;="&amp;$B20,국내SCHD형_분배!$C$2:$C$357,"&lt;="&amp;$C20)=0,"",SUMIFS(국내SCHD형_분배!$D$2:$D$357,국내SCHD형_분배!$A$2:$A$357,"446720",국내SCHD형_분배!$C$2:$C$357,"&gt;="&amp;$B20,국내SCHD형_분배!$C$2:$C$357,"&lt;="&amp;$C20))</f>
+        <f>IF(COUNTIFS(국내SCHD형_분배!$A$2:$A$359,"446720",국내SCHD형_분배!$C$2:$C$359,"&gt;="&amp;$B20,국내SCHD형_분배!$C$2:$C$359,"&lt;="&amp;$C20)=0,"",SUMIFS(국내SCHD형_분배!$D$2:$D$359,국내SCHD형_분배!$A$2:$A$359,"446720",국내SCHD형_분배!$C$2:$C$359,"&gt;="&amp;$B20,국내SCHD형_분배!$C$2:$C$359,"&lt;="&amp;$C20))</f>
         <v/>
       </c>
       <c r="F20" s="53">
-        <f>IF(COUNTIFS(국내SCHD형_분배!$A$2:$A$357,"402970",국내SCHD형_분배!$C$2:$C$357,"&gt;="&amp;$B20,국내SCHD형_분배!$C$2:$C$357,"&lt;="&amp;$C20)=0,"",SUMIFS(국내SCHD형_분배!$D$2:$D$357,국내SCHD형_분배!$A$2:$A$357,"402970",국내SCHD형_분배!$C$2:$C$357,"&gt;="&amp;$B20,국내SCHD형_분배!$C$2:$C$357,"&lt;="&amp;$C20))</f>
+        <f>IF(COUNTIFS(국내SCHD형_분배!$A$2:$A$359,"402970",국내SCHD형_분배!$C$2:$C$359,"&gt;="&amp;$B20,국내SCHD형_분배!$C$2:$C$359,"&lt;="&amp;$C20)=0,"",SUMIFS(국내SCHD형_분배!$D$2:$D$359,국내SCHD형_분배!$A$2:$A$359,"402970",국내SCHD형_분배!$C$2:$C$359,"&gt;="&amp;$B20,국내SCHD형_분배!$C$2:$C$359,"&lt;="&amp;$C20))</f>
         <v/>
       </c>
       <c r="G20" s="53">
-        <f>IF(COUNTIFS(국내SCHD형_분배!$A$2:$A$357,"489250",국내SCHD형_분배!$C$2:$C$357,"&gt;="&amp;$B20,국내SCHD형_분배!$C$2:$C$357,"&lt;="&amp;$C20)=0,"",SUMIFS(국내SCHD형_분배!$D$2:$D$357,국내SCHD형_분배!$A$2:$A$357,"489250",국내SCHD형_분배!$C$2:$C$357,"&gt;="&amp;$B20,국내SCHD형_분배!$C$2:$C$357,"&lt;="&amp;$C20))</f>
+        <f>IF(COUNTIFS(국내SCHD형_분배!$A$2:$A$359,"489250",국내SCHD형_분배!$C$2:$C$359,"&gt;="&amp;$B20,국내SCHD형_분배!$C$2:$C$359,"&lt;="&amp;$C20)=0,"",SUMIFS(국내SCHD형_분배!$D$2:$D$359,국내SCHD형_분배!$A$2:$A$359,"489250",국내SCHD형_분배!$C$2:$C$359,"&gt;="&amp;$B20,국내SCHD형_분배!$C$2:$C$359,"&lt;="&amp;$C20))</f>
         <v/>
       </c>
       <c r="H20" s="28">
@@ -25315,19 +25357,19 @@
         <v/>
       </c>
       <c r="D21" s="53">
-        <f>IF(COUNTIFS(국내SCHD형_분배!$A$2:$A$357,"458730",국내SCHD형_분배!$C$2:$C$357,"&gt;="&amp;$B21,국내SCHD형_분배!$C$2:$C$357,"&lt;="&amp;$C21)=0,"",SUMIFS(국내SCHD형_분배!$D$2:$D$357,국내SCHD형_분배!$A$2:$A$357,"458730",국내SCHD형_분배!$C$2:$C$357,"&gt;="&amp;$B21,국내SCHD형_분배!$C$2:$C$357,"&lt;="&amp;$C21))</f>
+        <f>IF(COUNTIFS(국내SCHD형_분배!$A$2:$A$359,"458730",국내SCHD형_분배!$C$2:$C$359,"&gt;="&amp;$B21,국내SCHD형_분배!$C$2:$C$359,"&lt;="&amp;$C21)=0,"",SUMIFS(국내SCHD형_분배!$D$2:$D$359,국내SCHD형_분배!$A$2:$A$359,"458730",국내SCHD형_분배!$C$2:$C$359,"&gt;="&amp;$B21,국내SCHD형_분배!$C$2:$C$359,"&lt;="&amp;$C21))</f>
         <v/>
       </c>
       <c r="E21" s="53">
-        <f>IF(COUNTIFS(국내SCHD형_분배!$A$2:$A$357,"446720",국내SCHD형_분배!$C$2:$C$357,"&gt;="&amp;$B21,국내SCHD형_분배!$C$2:$C$357,"&lt;="&amp;$C21)=0,"",SUMIFS(국내SCHD형_분배!$D$2:$D$357,국내SCHD형_분배!$A$2:$A$357,"446720",국내SCHD형_분배!$C$2:$C$357,"&gt;="&amp;$B21,국내SCHD형_분배!$C$2:$C$357,"&lt;="&amp;$C21))</f>
+        <f>IF(COUNTIFS(국내SCHD형_분배!$A$2:$A$359,"446720",국내SCHD형_분배!$C$2:$C$359,"&gt;="&amp;$B21,국내SCHD형_분배!$C$2:$C$359,"&lt;="&amp;$C21)=0,"",SUMIFS(국내SCHD형_분배!$D$2:$D$359,국내SCHD형_분배!$A$2:$A$359,"446720",국내SCHD형_분배!$C$2:$C$359,"&gt;="&amp;$B21,국내SCHD형_분배!$C$2:$C$359,"&lt;="&amp;$C21))</f>
         <v/>
       </c>
       <c r="F21" s="53">
-        <f>IF(COUNTIFS(국내SCHD형_분배!$A$2:$A$357,"402970",국내SCHD형_분배!$C$2:$C$357,"&gt;="&amp;$B21,국내SCHD형_분배!$C$2:$C$357,"&lt;="&amp;$C21)=0,"",SUMIFS(국내SCHD형_분배!$D$2:$D$357,국내SCHD형_분배!$A$2:$A$357,"402970",국내SCHD형_분배!$C$2:$C$357,"&gt;="&amp;$B21,국내SCHD형_분배!$C$2:$C$357,"&lt;="&amp;$C21))</f>
+        <f>IF(COUNTIFS(국내SCHD형_분배!$A$2:$A$359,"402970",국내SCHD형_분배!$C$2:$C$359,"&gt;="&amp;$B21,국내SCHD형_분배!$C$2:$C$359,"&lt;="&amp;$C21)=0,"",SUMIFS(국내SCHD형_분배!$D$2:$D$359,국내SCHD형_분배!$A$2:$A$359,"402970",국내SCHD형_분배!$C$2:$C$359,"&gt;="&amp;$B21,국내SCHD형_분배!$C$2:$C$359,"&lt;="&amp;$C21))</f>
         <v/>
       </c>
       <c r="G21" s="53">
-        <f>IF(COUNTIFS(국내SCHD형_분배!$A$2:$A$357,"489250",국내SCHD형_분배!$C$2:$C$357,"&gt;="&amp;$B21,국내SCHD형_분배!$C$2:$C$357,"&lt;="&amp;$C21)=0,"",SUMIFS(국내SCHD형_분배!$D$2:$D$357,국내SCHD형_분배!$A$2:$A$357,"489250",국내SCHD형_분배!$C$2:$C$357,"&gt;="&amp;$B21,국내SCHD형_분배!$C$2:$C$357,"&lt;="&amp;$C21))</f>
+        <f>IF(COUNTIFS(국내SCHD형_분배!$A$2:$A$359,"489250",국내SCHD형_분배!$C$2:$C$359,"&gt;="&amp;$B21,국내SCHD형_분배!$C$2:$C$359,"&lt;="&amp;$C21)=0,"",SUMIFS(국내SCHD형_분배!$D$2:$D$359,국내SCHD형_분배!$A$2:$A$359,"489250",국내SCHD형_분배!$C$2:$C$359,"&gt;="&amp;$B21,국내SCHD형_분배!$C$2:$C$359,"&lt;="&amp;$C21))</f>
         <v/>
       </c>
       <c r="H21" s="28">
@@ -25353,19 +25395,19 @@
         <v/>
       </c>
       <c r="D22" s="53">
-        <f>IF(COUNTIFS(국내SCHD형_분배!$A$2:$A$357,"458730",국내SCHD형_분배!$C$2:$C$357,"&gt;="&amp;$B22,국내SCHD형_분배!$C$2:$C$357,"&lt;="&amp;$C22)=0,"",SUMIFS(국내SCHD형_분배!$D$2:$D$357,국내SCHD형_분배!$A$2:$A$357,"458730",국내SCHD형_분배!$C$2:$C$357,"&gt;="&amp;$B22,국내SCHD형_분배!$C$2:$C$357,"&lt;="&amp;$C22))</f>
+        <f>IF(COUNTIFS(국내SCHD형_분배!$A$2:$A$359,"458730",국내SCHD형_분배!$C$2:$C$359,"&gt;="&amp;$B22,국내SCHD형_분배!$C$2:$C$359,"&lt;="&amp;$C22)=0,"",SUMIFS(국내SCHD형_분배!$D$2:$D$359,국내SCHD형_분배!$A$2:$A$359,"458730",국내SCHD형_분배!$C$2:$C$359,"&gt;="&amp;$B22,국내SCHD형_분배!$C$2:$C$359,"&lt;="&amp;$C22))</f>
         <v/>
       </c>
       <c r="E22" s="53">
-        <f>IF(COUNTIFS(국내SCHD형_분배!$A$2:$A$357,"446720",국내SCHD형_분배!$C$2:$C$357,"&gt;="&amp;$B22,국내SCHD형_분배!$C$2:$C$357,"&lt;="&amp;$C22)=0,"",SUMIFS(국내SCHD형_분배!$D$2:$D$357,국내SCHD형_분배!$A$2:$A$357,"446720",국내SCHD형_분배!$C$2:$C$357,"&gt;="&amp;$B22,국내SCHD형_분배!$C$2:$C$357,"&lt;="&amp;$C22))</f>
+        <f>IF(COUNTIFS(국내SCHD형_분배!$A$2:$A$359,"446720",국내SCHD형_분배!$C$2:$C$359,"&gt;="&amp;$B22,국내SCHD형_분배!$C$2:$C$359,"&lt;="&amp;$C22)=0,"",SUMIFS(국내SCHD형_분배!$D$2:$D$359,국내SCHD형_분배!$A$2:$A$359,"446720",국내SCHD형_분배!$C$2:$C$359,"&gt;="&amp;$B22,국내SCHD형_분배!$C$2:$C$359,"&lt;="&amp;$C22))</f>
         <v/>
       </c>
       <c r="F22" s="53">
-        <f>IF(COUNTIFS(국내SCHD형_분배!$A$2:$A$357,"402970",국내SCHD형_분배!$C$2:$C$357,"&gt;="&amp;$B22,국내SCHD형_분배!$C$2:$C$357,"&lt;="&amp;$C22)=0,"",SUMIFS(국내SCHD형_분배!$D$2:$D$357,국내SCHD형_분배!$A$2:$A$357,"402970",국내SCHD형_분배!$C$2:$C$357,"&gt;="&amp;$B22,국내SCHD형_분배!$C$2:$C$357,"&lt;="&amp;$C22))</f>
+        <f>IF(COUNTIFS(국내SCHD형_분배!$A$2:$A$359,"402970",국내SCHD형_분배!$C$2:$C$359,"&gt;="&amp;$B22,국내SCHD형_분배!$C$2:$C$359,"&lt;="&amp;$C22)=0,"",SUMIFS(국내SCHD형_분배!$D$2:$D$359,국내SCHD형_분배!$A$2:$A$359,"402970",국내SCHD형_분배!$C$2:$C$359,"&gt;="&amp;$B22,국내SCHD형_분배!$C$2:$C$359,"&lt;="&amp;$C22))</f>
         <v/>
       </c>
       <c r="G22" s="53">
-        <f>IF(COUNTIFS(국내SCHD형_분배!$A$2:$A$357,"489250",국내SCHD형_분배!$C$2:$C$357,"&gt;="&amp;$B22,국내SCHD형_분배!$C$2:$C$357,"&lt;="&amp;$C22)=0,"",SUMIFS(국내SCHD형_분배!$D$2:$D$357,국내SCHD형_분배!$A$2:$A$357,"489250",국내SCHD형_분배!$C$2:$C$357,"&gt;="&amp;$B22,국내SCHD형_분배!$C$2:$C$357,"&lt;="&amp;$C22))</f>
+        <f>IF(COUNTIFS(국내SCHD형_분배!$A$2:$A$359,"489250",국내SCHD형_분배!$C$2:$C$359,"&gt;="&amp;$B22,국내SCHD형_분배!$C$2:$C$359,"&lt;="&amp;$C22)=0,"",SUMIFS(국내SCHD형_분배!$D$2:$D$359,국내SCHD형_분배!$A$2:$A$359,"489250",국내SCHD형_분배!$C$2:$C$359,"&gt;="&amp;$B22,국내SCHD형_분배!$C$2:$C$359,"&lt;="&amp;$C22))</f>
         <v/>
       </c>
       <c r="H22" s="28">
@@ -25391,19 +25433,19 @@
         <v/>
       </c>
       <c r="D23" s="53">
-        <f>IF(COUNTIFS(국내SCHD형_분배!$A$2:$A$357,"458730",국내SCHD형_분배!$C$2:$C$357,"&gt;="&amp;$B23,국내SCHD형_분배!$C$2:$C$357,"&lt;="&amp;$C23)=0,"",SUMIFS(국내SCHD형_분배!$D$2:$D$357,국내SCHD형_분배!$A$2:$A$357,"458730",국내SCHD형_분배!$C$2:$C$357,"&gt;="&amp;$B23,국내SCHD형_분배!$C$2:$C$357,"&lt;="&amp;$C23))</f>
+        <f>IF(COUNTIFS(국내SCHD형_분배!$A$2:$A$359,"458730",국내SCHD형_분배!$C$2:$C$359,"&gt;="&amp;$B23,국내SCHD형_분배!$C$2:$C$359,"&lt;="&amp;$C23)=0,"",SUMIFS(국내SCHD형_분배!$D$2:$D$359,국내SCHD형_분배!$A$2:$A$359,"458730",국내SCHD형_분배!$C$2:$C$359,"&gt;="&amp;$B23,국내SCHD형_분배!$C$2:$C$359,"&lt;="&amp;$C23))</f>
         <v/>
       </c>
       <c r="E23" s="53">
-        <f>IF(COUNTIFS(국내SCHD형_분배!$A$2:$A$357,"446720",국내SCHD형_분배!$C$2:$C$357,"&gt;="&amp;$B23,국내SCHD형_분배!$C$2:$C$357,"&lt;="&amp;$C23)=0,"",SUMIFS(국내SCHD형_분배!$D$2:$D$357,국내SCHD형_분배!$A$2:$A$357,"446720",국내SCHD형_분배!$C$2:$C$357,"&gt;="&amp;$B23,국내SCHD형_분배!$C$2:$C$357,"&lt;="&amp;$C23))</f>
+        <f>IF(COUNTIFS(국내SCHD형_분배!$A$2:$A$359,"446720",국내SCHD형_분배!$C$2:$C$359,"&gt;="&amp;$B23,국내SCHD형_분배!$C$2:$C$359,"&lt;="&amp;$C23)=0,"",SUMIFS(국내SCHD형_분배!$D$2:$D$359,국내SCHD형_분배!$A$2:$A$359,"446720",국내SCHD형_분배!$C$2:$C$359,"&gt;="&amp;$B23,국내SCHD형_분배!$C$2:$C$359,"&lt;="&amp;$C23))</f>
         <v/>
       </c>
       <c r="F23" s="53">
-        <f>IF(COUNTIFS(국내SCHD형_분배!$A$2:$A$357,"402970",국내SCHD형_분배!$C$2:$C$357,"&gt;="&amp;$B23,국내SCHD형_분배!$C$2:$C$357,"&lt;="&amp;$C23)=0,"",SUMIFS(국내SCHD형_분배!$D$2:$D$357,국내SCHD형_분배!$A$2:$A$357,"402970",국내SCHD형_분배!$C$2:$C$357,"&gt;="&amp;$B23,국내SCHD형_분배!$C$2:$C$357,"&lt;="&amp;$C23))</f>
+        <f>IF(COUNTIFS(국내SCHD형_분배!$A$2:$A$359,"402970",국내SCHD형_분배!$C$2:$C$359,"&gt;="&amp;$B23,국내SCHD형_분배!$C$2:$C$359,"&lt;="&amp;$C23)=0,"",SUMIFS(국내SCHD형_분배!$D$2:$D$359,국내SCHD형_분배!$A$2:$A$359,"402970",국내SCHD형_분배!$C$2:$C$359,"&gt;="&amp;$B23,국내SCHD형_분배!$C$2:$C$359,"&lt;="&amp;$C23))</f>
         <v/>
       </c>
       <c r="G23" s="53">
-        <f>IF(COUNTIFS(국내SCHD형_분배!$A$2:$A$357,"489250",국내SCHD형_분배!$C$2:$C$357,"&gt;="&amp;$B23,국내SCHD형_분배!$C$2:$C$357,"&lt;="&amp;$C23)=0,"",SUMIFS(국내SCHD형_분배!$D$2:$D$357,국내SCHD형_분배!$A$2:$A$357,"489250",국내SCHD형_분배!$C$2:$C$357,"&gt;="&amp;$B23,국내SCHD형_분배!$C$2:$C$357,"&lt;="&amp;$C23))</f>
+        <f>IF(COUNTIFS(국내SCHD형_분배!$A$2:$A$359,"489250",국내SCHD형_분배!$C$2:$C$359,"&gt;="&amp;$B23,국내SCHD형_분배!$C$2:$C$359,"&lt;="&amp;$C23)=0,"",SUMIFS(국내SCHD형_분배!$D$2:$D$359,국내SCHD형_분배!$A$2:$A$359,"489250",국내SCHD형_분배!$C$2:$C$359,"&gt;="&amp;$B23,국내SCHD형_분배!$C$2:$C$359,"&lt;="&amp;$C23))</f>
         <v/>
       </c>
       <c r="H23" s="28">
@@ -25429,19 +25471,19 @@
         <v/>
       </c>
       <c r="D24" s="53">
-        <f>IF(COUNTIFS(국내SCHD형_분배!$A$2:$A$357,"458730",국내SCHD형_분배!$C$2:$C$357,"&gt;="&amp;$B24,국내SCHD형_분배!$C$2:$C$357,"&lt;="&amp;$C24)=0,"",SUMIFS(국내SCHD형_분배!$D$2:$D$357,국내SCHD형_분배!$A$2:$A$357,"458730",국내SCHD형_분배!$C$2:$C$357,"&gt;="&amp;$B24,국내SCHD형_분배!$C$2:$C$357,"&lt;="&amp;$C24))</f>
+        <f>IF(COUNTIFS(국내SCHD형_분배!$A$2:$A$359,"458730",국내SCHD형_분배!$C$2:$C$359,"&gt;="&amp;$B24,국내SCHD형_분배!$C$2:$C$359,"&lt;="&amp;$C24)=0,"",SUMIFS(국내SCHD형_분배!$D$2:$D$359,국내SCHD형_분배!$A$2:$A$359,"458730",국내SCHD형_분배!$C$2:$C$359,"&gt;="&amp;$B24,국내SCHD형_분배!$C$2:$C$359,"&lt;="&amp;$C24))</f>
         <v/>
       </c>
       <c r="E24" s="53">
-        <f>IF(COUNTIFS(국내SCHD형_분배!$A$2:$A$357,"446720",국내SCHD형_분배!$C$2:$C$357,"&gt;="&amp;$B24,국내SCHD형_분배!$C$2:$C$357,"&lt;="&amp;$C24)=0,"",SUMIFS(국내SCHD형_분배!$D$2:$D$357,국내SCHD형_분배!$A$2:$A$357,"446720",국내SCHD형_분배!$C$2:$C$357,"&gt;="&amp;$B24,국내SCHD형_분배!$C$2:$C$357,"&lt;="&amp;$C24))</f>
+        <f>IF(COUNTIFS(국내SCHD형_분배!$A$2:$A$359,"446720",국내SCHD형_분배!$C$2:$C$359,"&gt;="&amp;$B24,국내SCHD형_분배!$C$2:$C$359,"&lt;="&amp;$C24)=0,"",SUMIFS(국내SCHD형_분배!$D$2:$D$359,국내SCHD형_분배!$A$2:$A$359,"446720",국내SCHD형_분배!$C$2:$C$359,"&gt;="&amp;$B24,국내SCHD형_분배!$C$2:$C$359,"&lt;="&amp;$C24))</f>
         <v/>
       </c>
       <c r="F24" s="53">
-        <f>IF(COUNTIFS(국내SCHD형_분배!$A$2:$A$357,"402970",국내SCHD형_분배!$C$2:$C$357,"&gt;="&amp;$B24,국내SCHD형_분배!$C$2:$C$357,"&lt;="&amp;$C24)=0,"",SUMIFS(국내SCHD형_분배!$D$2:$D$357,국내SCHD형_분배!$A$2:$A$357,"402970",국내SCHD형_분배!$C$2:$C$357,"&gt;="&amp;$B24,국내SCHD형_분배!$C$2:$C$357,"&lt;="&amp;$C24))</f>
+        <f>IF(COUNTIFS(국내SCHD형_분배!$A$2:$A$359,"402970",국내SCHD형_분배!$C$2:$C$359,"&gt;="&amp;$B24,국내SCHD형_분배!$C$2:$C$359,"&lt;="&amp;$C24)=0,"",SUMIFS(국내SCHD형_분배!$D$2:$D$359,국내SCHD형_분배!$A$2:$A$359,"402970",국내SCHD형_분배!$C$2:$C$359,"&gt;="&amp;$B24,국내SCHD형_분배!$C$2:$C$359,"&lt;="&amp;$C24))</f>
         <v/>
       </c>
       <c r="G24" s="53">
-        <f>IF(COUNTIFS(국내SCHD형_분배!$A$2:$A$357,"489250",국내SCHD형_분배!$C$2:$C$357,"&gt;="&amp;$B24,국내SCHD형_분배!$C$2:$C$357,"&lt;="&amp;$C24)=0,"",SUMIFS(국내SCHD형_분배!$D$2:$D$357,국내SCHD형_분배!$A$2:$A$357,"489250",국내SCHD형_분배!$C$2:$C$357,"&gt;="&amp;$B24,국내SCHD형_분배!$C$2:$C$357,"&lt;="&amp;$C24))</f>
+        <f>IF(COUNTIFS(국내SCHD형_분배!$A$2:$A$359,"489250",국내SCHD형_분배!$C$2:$C$359,"&gt;="&amp;$B24,국내SCHD형_분배!$C$2:$C$359,"&lt;="&amp;$C24)=0,"",SUMIFS(국내SCHD형_분배!$D$2:$D$359,국내SCHD형_분배!$A$2:$A$359,"489250",국내SCHD형_분배!$C$2:$C$359,"&gt;="&amp;$B24,국내SCHD형_분배!$C$2:$C$359,"&lt;="&amp;$C24))</f>
         <v/>
       </c>
       <c r="H24" s="28">
@@ -25467,19 +25509,19 @@
         <v/>
       </c>
       <c r="D25" s="53">
-        <f>IF(COUNTIFS(국내SCHD형_분배!$A$2:$A$357,"458730",국내SCHD형_분배!$C$2:$C$357,"&gt;="&amp;$B25,국내SCHD형_분배!$C$2:$C$357,"&lt;="&amp;$C25)=0,"",SUMIFS(국내SCHD형_분배!$D$2:$D$357,국내SCHD형_분배!$A$2:$A$357,"458730",국내SCHD형_분배!$C$2:$C$357,"&gt;="&amp;$B25,국내SCHD형_분배!$C$2:$C$357,"&lt;="&amp;$C25))</f>
+        <f>IF(COUNTIFS(국내SCHD형_분배!$A$2:$A$359,"458730",국내SCHD형_분배!$C$2:$C$359,"&gt;="&amp;$B25,국내SCHD형_분배!$C$2:$C$359,"&lt;="&amp;$C25)=0,"",SUMIFS(국내SCHD형_분배!$D$2:$D$359,국내SCHD형_분배!$A$2:$A$359,"458730",국내SCHD형_분배!$C$2:$C$359,"&gt;="&amp;$B25,국내SCHD형_분배!$C$2:$C$359,"&lt;="&amp;$C25))</f>
         <v/>
       </c>
       <c r="E25" s="53">
-        <f>IF(COUNTIFS(국내SCHD형_분배!$A$2:$A$357,"446720",국내SCHD형_분배!$C$2:$C$357,"&gt;="&amp;$B25,국내SCHD형_분배!$C$2:$C$357,"&lt;="&amp;$C25)=0,"",SUMIFS(국내SCHD형_분배!$D$2:$D$357,국내SCHD형_분배!$A$2:$A$357,"446720",국내SCHD형_분배!$C$2:$C$357,"&gt;="&amp;$B25,국내SCHD형_분배!$C$2:$C$357,"&lt;="&amp;$C25))</f>
+        <f>IF(COUNTIFS(국내SCHD형_분배!$A$2:$A$359,"446720",국내SCHD형_분배!$C$2:$C$359,"&gt;="&amp;$B25,국내SCHD형_분배!$C$2:$C$359,"&lt;="&amp;$C25)=0,"",SUMIFS(국내SCHD형_분배!$D$2:$D$359,국내SCHD형_분배!$A$2:$A$359,"446720",국내SCHD형_분배!$C$2:$C$359,"&gt;="&amp;$B25,국내SCHD형_분배!$C$2:$C$359,"&lt;="&amp;$C25))</f>
         <v/>
       </c>
       <c r="F25" s="53">
-        <f>IF(COUNTIFS(국내SCHD형_분배!$A$2:$A$357,"402970",국내SCHD형_분배!$C$2:$C$357,"&gt;="&amp;$B25,국내SCHD형_분배!$C$2:$C$357,"&lt;="&amp;$C25)=0,"",SUMIFS(국내SCHD형_분배!$D$2:$D$357,국내SCHD형_분배!$A$2:$A$357,"402970",국내SCHD형_분배!$C$2:$C$357,"&gt;="&amp;$B25,국내SCHD형_분배!$C$2:$C$357,"&lt;="&amp;$C25))</f>
+        <f>IF(COUNTIFS(국내SCHD형_분배!$A$2:$A$359,"402970",국내SCHD형_분배!$C$2:$C$359,"&gt;="&amp;$B25,국내SCHD형_분배!$C$2:$C$359,"&lt;="&amp;$C25)=0,"",SUMIFS(국내SCHD형_분배!$D$2:$D$359,국내SCHD형_분배!$A$2:$A$359,"402970",국내SCHD형_분배!$C$2:$C$359,"&gt;="&amp;$B25,국내SCHD형_분배!$C$2:$C$359,"&lt;="&amp;$C25))</f>
         <v/>
       </c>
       <c r="G25" s="53">
-        <f>IF(COUNTIFS(국내SCHD형_분배!$A$2:$A$357,"489250",국내SCHD형_분배!$C$2:$C$357,"&gt;="&amp;$B25,국내SCHD형_분배!$C$2:$C$357,"&lt;="&amp;$C25)=0,"",SUMIFS(국내SCHD형_분배!$D$2:$D$357,국내SCHD형_분배!$A$2:$A$357,"489250",국내SCHD형_분배!$C$2:$C$357,"&gt;="&amp;$B25,국내SCHD형_분배!$C$2:$C$357,"&lt;="&amp;$C25))</f>
+        <f>IF(COUNTIFS(국내SCHD형_분배!$A$2:$A$359,"489250",국내SCHD형_분배!$C$2:$C$359,"&gt;="&amp;$B25,국내SCHD형_분배!$C$2:$C$359,"&lt;="&amp;$C25)=0,"",SUMIFS(국내SCHD형_분배!$D$2:$D$359,국내SCHD형_분배!$A$2:$A$359,"489250",국내SCHD형_분배!$C$2:$C$359,"&gt;="&amp;$B25,국내SCHD형_분배!$C$2:$C$359,"&lt;="&amp;$C25))</f>
         <v/>
       </c>
       <c r="H25" s="28">
@@ -25505,19 +25547,19 @@
         <v/>
       </c>
       <c r="D26" s="53">
-        <f>IF(COUNTIFS(국내SCHD형_분배!$A$2:$A$357,"458730",국내SCHD형_분배!$C$2:$C$357,"&gt;="&amp;$B26,국내SCHD형_분배!$C$2:$C$357,"&lt;="&amp;$C26)=0,"",SUMIFS(국내SCHD형_분배!$D$2:$D$357,국내SCHD형_분배!$A$2:$A$357,"458730",국내SCHD형_분배!$C$2:$C$357,"&gt;="&amp;$B26,국내SCHD형_분배!$C$2:$C$357,"&lt;="&amp;$C26))</f>
+        <f>IF(COUNTIFS(국내SCHD형_분배!$A$2:$A$359,"458730",국내SCHD형_분배!$C$2:$C$359,"&gt;="&amp;$B26,국내SCHD형_분배!$C$2:$C$359,"&lt;="&amp;$C26)=0,"",SUMIFS(국내SCHD형_분배!$D$2:$D$359,국내SCHD형_분배!$A$2:$A$359,"458730",국내SCHD형_분배!$C$2:$C$359,"&gt;="&amp;$B26,국내SCHD형_분배!$C$2:$C$359,"&lt;="&amp;$C26))</f>
         <v/>
       </c>
       <c r="E26" s="53">
-        <f>IF(COUNTIFS(국내SCHD형_분배!$A$2:$A$357,"446720",국내SCHD형_분배!$C$2:$C$357,"&gt;="&amp;$B26,국내SCHD형_분배!$C$2:$C$357,"&lt;="&amp;$C26)=0,"",SUMIFS(국내SCHD형_분배!$D$2:$D$357,국내SCHD형_분배!$A$2:$A$357,"446720",국내SCHD형_분배!$C$2:$C$357,"&gt;="&amp;$B26,국내SCHD형_분배!$C$2:$C$357,"&lt;="&amp;$C26))</f>
+        <f>IF(COUNTIFS(국내SCHD형_분배!$A$2:$A$359,"446720",국내SCHD형_분배!$C$2:$C$359,"&gt;="&amp;$B26,국내SCHD형_분배!$C$2:$C$359,"&lt;="&amp;$C26)=0,"",SUMIFS(국내SCHD형_분배!$D$2:$D$359,국내SCHD형_분배!$A$2:$A$359,"446720",국내SCHD형_분배!$C$2:$C$359,"&gt;="&amp;$B26,국내SCHD형_분배!$C$2:$C$359,"&lt;="&amp;$C26))</f>
         <v/>
       </c>
       <c r="F26" s="53">
-        <f>IF(COUNTIFS(국내SCHD형_분배!$A$2:$A$357,"402970",국내SCHD형_분배!$C$2:$C$357,"&gt;="&amp;$B26,국내SCHD형_분배!$C$2:$C$357,"&lt;="&amp;$C26)=0,"",SUMIFS(국내SCHD형_분배!$D$2:$D$357,국내SCHD형_분배!$A$2:$A$357,"402970",국내SCHD형_분배!$C$2:$C$357,"&gt;="&amp;$B26,국내SCHD형_분배!$C$2:$C$357,"&lt;="&amp;$C26))</f>
+        <f>IF(COUNTIFS(국내SCHD형_분배!$A$2:$A$359,"402970",국내SCHD형_분배!$C$2:$C$359,"&gt;="&amp;$B26,국내SCHD형_분배!$C$2:$C$359,"&lt;="&amp;$C26)=0,"",SUMIFS(국내SCHD형_분배!$D$2:$D$359,국내SCHD형_분배!$A$2:$A$359,"402970",국내SCHD형_분배!$C$2:$C$359,"&gt;="&amp;$B26,국내SCHD형_분배!$C$2:$C$359,"&lt;="&amp;$C26))</f>
         <v/>
       </c>
       <c r="G26" s="53">
-        <f>IF(COUNTIFS(국내SCHD형_분배!$A$2:$A$357,"489250",국내SCHD형_분배!$C$2:$C$357,"&gt;="&amp;$B26,국내SCHD형_분배!$C$2:$C$357,"&lt;="&amp;$C26)=0,"",SUMIFS(국내SCHD형_분배!$D$2:$D$357,국내SCHD형_분배!$A$2:$A$357,"489250",국내SCHD형_분배!$C$2:$C$357,"&gt;="&amp;$B26,국내SCHD형_분배!$C$2:$C$357,"&lt;="&amp;$C26))</f>
+        <f>IF(COUNTIFS(국내SCHD형_분배!$A$2:$A$359,"489250",국내SCHD형_분배!$C$2:$C$359,"&gt;="&amp;$B26,국내SCHD형_분배!$C$2:$C$359,"&lt;="&amp;$C26)=0,"",SUMIFS(국내SCHD형_분배!$D$2:$D$359,국내SCHD형_분배!$A$2:$A$359,"489250",국내SCHD형_분배!$C$2:$C$359,"&gt;="&amp;$B26,국내SCHD형_분배!$C$2:$C$359,"&lt;="&amp;$C26))</f>
         <v/>
       </c>
       <c r="H26" s="28">
@@ -25543,19 +25585,19 @@
         <v/>
       </c>
       <c r="D27" s="53">
-        <f>IF(COUNTIFS(국내SCHD형_분배!$A$2:$A$357,"458730",국내SCHD형_분배!$C$2:$C$357,"&gt;="&amp;$B27,국내SCHD형_분배!$C$2:$C$357,"&lt;="&amp;$C27)=0,"",SUMIFS(국내SCHD형_분배!$D$2:$D$357,국내SCHD형_분배!$A$2:$A$357,"458730",국내SCHD형_분배!$C$2:$C$357,"&gt;="&amp;$B27,국내SCHD형_분배!$C$2:$C$357,"&lt;="&amp;$C27))</f>
+        <f>IF(COUNTIFS(국내SCHD형_분배!$A$2:$A$359,"458730",국내SCHD형_분배!$C$2:$C$359,"&gt;="&amp;$B27,국내SCHD형_분배!$C$2:$C$359,"&lt;="&amp;$C27)=0,"",SUMIFS(국내SCHD형_분배!$D$2:$D$359,국내SCHD형_분배!$A$2:$A$359,"458730",국내SCHD형_분배!$C$2:$C$359,"&gt;="&amp;$B27,국내SCHD형_분배!$C$2:$C$359,"&lt;="&amp;$C27))</f>
         <v/>
       </c>
       <c r="E27" s="53">
-        <f>IF(COUNTIFS(국내SCHD형_분배!$A$2:$A$357,"446720",국내SCHD형_분배!$C$2:$C$357,"&gt;="&amp;$B27,국내SCHD형_분배!$C$2:$C$357,"&lt;="&amp;$C27)=0,"",SUMIFS(국내SCHD형_분배!$D$2:$D$357,국내SCHD형_분배!$A$2:$A$357,"446720",국내SCHD형_분배!$C$2:$C$357,"&gt;="&amp;$B27,국내SCHD형_분배!$C$2:$C$357,"&lt;="&amp;$C27))</f>
+        <f>IF(COUNTIFS(국내SCHD형_분배!$A$2:$A$359,"446720",국내SCHD형_분배!$C$2:$C$359,"&gt;="&amp;$B27,국내SCHD형_분배!$C$2:$C$359,"&lt;="&amp;$C27)=0,"",SUMIFS(국내SCHD형_분배!$D$2:$D$359,국내SCHD형_분배!$A$2:$A$359,"446720",국내SCHD형_분배!$C$2:$C$359,"&gt;="&amp;$B27,국내SCHD형_분배!$C$2:$C$359,"&lt;="&amp;$C27))</f>
         <v/>
       </c>
       <c r="F27" s="53">
-        <f>IF(COUNTIFS(국내SCHD형_분배!$A$2:$A$357,"402970",국내SCHD형_분배!$C$2:$C$357,"&gt;="&amp;$B27,국내SCHD형_분배!$C$2:$C$357,"&lt;="&amp;$C27)=0,"",SUMIFS(국내SCHD형_분배!$D$2:$D$357,국내SCHD형_분배!$A$2:$A$357,"402970",국내SCHD형_분배!$C$2:$C$357,"&gt;="&amp;$B27,국내SCHD형_분배!$C$2:$C$357,"&lt;="&amp;$C27))</f>
+        <f>IF(COUNTIFS(국내SCHD형_분배!$A$2:$A$359,"402970",국내SCHD형_분배!$C$2:$C$359,"&gt;="&amp;$B27,국내SCHD형_분배!$C$2:$C$359,"&lt;="&amp;$C27)=0,"",SUMIFS(국내SCHD형_분배!$D$2:$D$359,국내SCHD형_분배!$A$2:$A$359,"402970",국내SCHD형_분배!$C$2:$C$359,"&gt;="&amp;$B27,국내SCHD형_분배!$C$2:$C$359,"&lt;="&amp;$C27))</f>
         <v/>
       </c>
       <c r="G27" s="53">
-        <f>IF(COUNTIFS(국내SCHD형_분배!$A$2:$A$357,"489250",국내SCHD형_분배!$C$2:$C$357,"&gt;="&amp;$B27,국내SCHD형_분배!$C$2:$C$357,"&lt;="&amp;$C27)=0,"",SUMIFS(국내SCHD형_분배!$D$2:$D$357,국내SCHD형_분배!$A$2:$A$357,"489250",국내SCHD형_분배!$C$2:$C$357,"&gt;="&amp;$B27,국내SCHD형_분배!$C$2:$C$357,"&lt;="&amp;$C27))</f>
+        <f>IF(COUNTIFS(국내SCHD형_분배!$A$2:$A$359,"489250",국내SCHD형_분배!$C$2:$C$359,"&gt;="&amp;$B27,국내SCHD형_분배!$C$2:$C$359,"&lt;="&amp;$C27)=0,"",SUMIFS(국내SCHD형_분배!$D$2:$D$359,국내SCHD형_분배!$A$2:$A$359,"489250",국내SCHD형_분배!$C$2:$C$359,"&gt;="&amp;$B27,국내SCHD형_분배!$C$2:$C$359,"&lt;="&amp;$C27))</f>
         <v/>
       </c>
       <c r="H27" s="28">
@@ -25581,19 +25623,19 @@
         <v/>
       </c>
       <c r="D28" s="53">
-        <f>IF(COUNTIFS(국내SCHD형_분배!$A$2:$A$357,"458730",국내SCHD형_분배!$C$2:$C$357,"&gt;="&amp;$B28,국내SCHD형_분배!$C$2:$C$357,"&lt;="&amp;$C28)=0,"",SUMIFS(국내SCHD형_분배!$D$2:$D$357,국내SCHD형_분배!$A$2:$A$357,"458730",국내SCHD형_분배!$C$2:$C$357,"&gt;="&amp;$B28,국내SCHD형_분배!$C$2:$C$357,"&lt;="&amp;$C28))</f>
+        <f>IF(COUNTIFS(국내SCHD형_분배!$A$2:$A$359,"458730",국내SCHD형_분배!$C$2:$C$359,"&gt;="&amp;$B28,국내SCHD형_분배!$C$2:$C$359,"&lt;="&amp;$C28)=0,"",SUMIFS(국내SCHD형_분배!$D$2:$D$359,국내SCHD형_분배!$A$2:$A$359,"458730",국내SCHD형_분배!$C$2:$C$359,"&gt;="&amp;$B28,국내SCHD형_분배!$C$2:$C$359,"&lt;="&amp;$C28))</f>
         <v/>
       </c>
       <c r="E28" s="53">
-        <f>IF(COUNTIFS(국내SCHD형_분배!$A$2:$A$357,"446720",국내SCHD형_분배!$C$2:$C$357,"&gt;="&amp;$B28,국내SCHD형_분배!$C$2:$C$357,"&lt;="&amp;$C28)=0,"",SUMIFS(국내SCHD형_분배!$D$2:$D$357,국내SCHD형_분배!$A$2:$A$357,"446720",국내SCHD형_분배!$C$2:$C$357,"&gt;="&amp;$B28,국내SCHD형_분배!$C$2:$C$357,"&lt;="&amp;$C28))</f>
+        <f>IF(COUNTIFS(국내SCHD형_분배!$A$2:$A$359,"446720",국내SCHD형_분배!$C$2:$C$359,"&gt;="&amp;$B28,국내SCHD형_분배!$C$2:$C$359,"&lt;="&amp;$C28)=0,"",SUMIFS(국내SCHD형_분배!$D$2:$D$359,국내SCHD형_분배!$A$2:$A$359,"446720",국내SCHD형_분배!$C$2:$C$359,"&gt;="&amp;$B28,국내SCHD형_분배!$C$2:$C$359,"&lt;="&amp;$C28))</f>
         <v/>
       </c>
       <c r="F28" s="53">
-        <f>IF(COUNTIFS(국내SCHD형_분배!$A$2:$A$357,"402970",국내SCHD형_분배!$C$2:$C$357,"&gt;="&amp;$B28,국내SCHD형_분배!$C$2:$C$357,"&lt;="&amp;$C28)=0,"",SUMIFS(국내SCHD형_분배!$D$2:$D$357,국내SCHD형_분배!$A$2:$A$357,"402970",국내SCHD형_분배!$C$2:$C$357,"&gt;="&amp;$B28,국내SCHD형_분배!$C$2:$C$357,"&lt;="&amp;$C28))</f>
+        <f>IF(COUNTIFS(국내SCHD형_분배!$A$2:$A$359,"402970",국내SCHD형_분배!$C$2:$C$359,"&gt;="&amp;$B28,국내SCHD형_분배!$C$2:$C$359,"&lt;="&amp;$C28)=0,"",SUMIFS(국내SCHD형_분배!$D$2:$D$359,국내SCHD형_분배!$A$2:$A$359,"402970",국내SCHD형_분배!$C$2:$C$359,"&gt;="&amp;$B28,국내SCHD형_분배!$C$2:$C$359,"&lt;="&amp;$C28))</f>
         <v/>
       </c>
       <c r="G28" s="53">
-        <f>IF(COUNTIFS(국내SCHD형_분배!$A$2:$A$357,"489250",국내SCHD형_분배!$C$2:$C$357,"&gt;="&amp;$B28,국내SCHD형_분배!$C$2:$C$357,"&lt;="&amp;$C28)=0,"",SUMIFS(국내SCHD형_분배!$D$2:$D$357,국내SCHD형_분배!$A$2:$A$357,"489250",국내SCHD형_분배!$C$2:$C$357,"&gt;="&amp;$B28,국내SCHD형_분배!$C$2:$C$357,"&lt;="&amp;$C28))</f>
+        <f>IF(COUNTIFS(국내SCHD형_분배!$A$2:$A$359,"489250",국내SCHD형_분배!$C$2:$C$359,"&gt;="&amp;$B28,국내SCHD형_분배!$C$2:$C$359,"&lt;="&amp;$C28)=0,"",SUMIFS(국내SCHD형_분배!$D$2:$D$359,국내SCHD형_분배!$A$2:$A$359,"489250",국내SCHD형_분배!$C$2:$C$359,"&gt;="&amp;$B28,국내SCHD형_분배!$C$2:$C$359,"&lt;="&amp;$C28))</f>
         <v/>
       </c>
       <c r="H28" s="28">
@@ -25619,19 +25661,19 @@
         <v/>
       </c>
       <c r="D29" s="53">
-        <f>IF(COUNTIFS(국내SCHD형_분배!$A$2:$A$357,"458730",국내SCHD형_분배!$C$2:$C$357,"&gt;="&amp;$B29,국내SCHD형_분배!$C$2:$C$357,"&lt;="&amp;$C29)=0,"",SUMIFS(국내SCHD형_분배!$D$2:$D$357,국내SCHD형_분배!$A$2:$A$357,"458730",국내SCHD형_분배!$C$2:$C$357,"&gt;="&amp;$B29,국내SCHD형_분배!$C$2:$C$357,"&lt;="&amp;$C29))</f>
+        <f>IF(COUNTIFS(국내SCHD형_분배!$A$2:$A$359,"458730",국내SCHD형_분배!$C$2:$C$359,"&gt;="&amp;$B29,국내SCHD형_분배!$C$2:$C$359,"&lt;="&amp;$C29)=0,"",SUMIFS(국내SCHD형_분배!$D$2:$D$359,국내SCHD형_분배!$A$2:$A$359,"458730",국내SCHD형_분배!$C$2:$C$359,"&gt;="&amp;$B29,국내SCHD형_분배!$C$2:$C$359,"&lt;="&amp;$C29))</f>
         <v/>
       </c>
       <c r="E29" s="53">
-        <f>IF(COUNTIFS(국내SCHD형_분배!$A$2:$A$357,"446720",국내SCHD형_분배!$C$2:$C$357,"&gt;="&amp;$B29,국내SCHD형_분배!$C$2:$C$357,"&lt;="&amp;$C29)=0,"",SUMIFS(국내SCHD형_분배!$D$2:$D$357,국내SCHD형_분배!$A$2:$A$357,"446720",국내SCHD형_분배!$C$2:$C$357,"&gt;="&amp;$B29,국내SCHD형_분배!$C$2:$C$357,"&lt;="&amp;$C29))</f>
+        <f>IF(COUNTIFS(국내SCHD형_분배!$A$2:$A$359,"446720",국내SCHD형_분배!$C$2:$C$359,"&gt;="&amp;$B29,국내SCHD형_분배!$C$2:$C$359,"&lt;="&amp;$C29)=0,"",SUMIFS(국내SCHD형_분배!$D$2:$D$359,국내SCHD형_분배!$A$2:$A$359,"446720",국내SCHD형_분배!$C$2:$C$359,"&gt;="&amp;$B29,국내SCHD형_분배!$C$2:$C$359,"&lt;="&amp;$C29))</f>
         <v/>
       </c>
       <c r="F29" s="53">
-        <f>IF(COUNTIFS(국내SCHD형_분배!$A$2:$A$357,"402970",국내SCHD형_분배!$C$2:$C$357,"&gt;="&amp;$B29,국내SCHD형_분배!$C$2:$C$357,"&lt;="&amp;$C29)=0,"",SUMIFS(국내SCHD형_분배!$D$2:$D$357,국내SCHD형_분배!$A$2:$A$357,"402970",국내SCHD형_분배!$C$2:$C$357,"&gt;="&amp;$B29,국내SCHD형_분배!$C$2:$C$357,"&lt;="&amp;$C29))</f>
+        <f>IF(COUNTIFS(국내SCHD형_분배!$A$2:$A$359,"402970",국내SCHD형_분배!$C$2:$C$359,"&gt;="&amp;$B29,국내SCHD형_분배!$C$2:$C$359,"&lt;="&amp;$C29)=0,"",SUMIFS(국내SCHD형_분배!$D$2:$D$359,국내SCHD형_분배!$A$2:$A$359,"402970",국내SCHD형_분배!$C$2:$C$359,"&gt;="&amp;$B29,국내SCHD형_분배!$C$2:$C$359,"&lt;="&amp;$C29))</f>
         <v/>
       </c>
       <c r="G29" s="53">
-        <f>IF(COUNTIFS(국내SCHD형_분배!$A$2:$A$357,"489250",국내SCHD형_분배!$C$2:$C$357,"&gt;="&amp;$B29,국내SCHD형_분배!$C$2:$C$357,"&lt;="&amp;$C29)=0,"",SUMIFS(국내SCHD형_분배!$D$2:$D$357,국내SCHD형_분배!$A$2:$A$357,"489250",국내SCHD형_분배!$C$2:$C$357,"&gt;="&amp;$B29,국내SCHD형_분배!$C$2:$C$357,"&lt;="&amp;$C29))</f>
+        <f>IF(COUNTIFS(국내SCHD형_분배!$A$2:$A$359,"489250",국내SCHD형_분배!$C$2:$C$359,"&gt;="&amp;$B29,국내SCHD형_분배!$C$2:$C$359,"&lt;="&amp;$C29)=0,"",SUMIFS(국내SCHD형_분배!$D$2:$D$359,국내SCHD형_분배!$A$2:$A$359,"489250",국내SCHD형_분배!$C$2:$C$359,"&gt;="&amp;$B29,국내SCHD형_분배!$C$2:$C$359,"&lt;="&amp;$C29))</f>
         <v/>
       </c>
       <c r="H29" s="28">
@@ -25657,19 +25699,19 @@
         <v/>
       </c>
       <c r="D30" s="53">
-        <f>IF(COUNTIFS(국내SCHD형_분배!$A$2:$A$357,"458730",국내SCHD형_분배!$C$2:$C$357,"&gt;="&amp;$B30,국내SCHD형_분배!$C$2:$C$357,"&lt;="&amp;$C30)=0,"",SUMIFS(국내SCHD형_분배!$D$2:$D$357,국내SCHD형_분배!$A$2:$A$357,"458730",국내SCHD형_분배!$C$2:$C$357,"&gt;="&amp;$B30,국내SCHD형_분배!$C$2:$C$357,"&lt;="&amp;$C30))</f>
+        <f>IF(COUNTIFS(국내SCHD형_분배!$A$2:$A$359,"458730",국내SCHD형_분배!$C$2:$C$359,"&gt;="&amp;$B30,국내SCHD형_분배!$C$2:$C$359,"&lt;="&amp;$C30)=0,"",SUMIFS(국내SCHD형_분배!$D$2:$D$359,국내SCHD형_분배!$A$2:$A$359,"458730",국내SCHD형_분배!$C$2:$C$359,"&gt;="&amp;$B30,국내SCHD형_분배!$C$2:$C$359,"&lt;="&amp;$C30))</f>
         <v/>
       </c>
       <c r="E30" s="53">
-        <f>IF(COUNTIFS(국내SCHD형_분배!$A$2:$A$357,"446720",국내SCHD형_분배!$C$2:$C$357,"&gt;="&amp;$B30,국내SCHD형_분배!$C$2:$C$357,"&lt;="&amp;$C30)=0,"",SUMIFS(국내SCHD형_분배!$D$2:$D$357,국내SCHD형_분배!$A$2:$A$357,"446720",국내SCHD형_분배!$C$2:$C$357,"&gt;="&amp;$B30,국내SCHD형_분배!$C$2:$C$357,"&lt;="&amp;$C30))</f>
+        <f>IF(COUNTIFS(국내SCHD형_분배!$A$2:$A$359,"446720",국내SCHD형_분배!$C$2:$C$359,"&gt;="&amp;$B30,국내SCHD형_분배!$C$2:$C$359,"&lt;="&amp;$C30)=0,"",SUMIFS(국내SCHD형_분배!$D$2:$D$359,국내SCHD형_분배!$A$2:$A$359,"446720",국내SCHD형_분배!$C$2:$C$359,"&gt;="&amp;$B30,국내SCHD형_분배!$C$2:$C$359,"&lt;="&amp;$C30))</f>
         <v/>
       </c>
       <c r="F30" s="53">
-        <f>IF(COUNTIFS(국내SCHD형_분배!$A$2:$A$357,"402970",국내SCHD형_분배!$C$2:$C$357,"&gt;="&amp;$B30,국내SCHD형_분배!$C$2:$C$357,"&lt;="&amp;$C30)=0,"",SUMIFS(국내SCHD형_분배!$D$2:$D$357,국내SCHD형_분배!$A$2:$A$357,"402970",국내SCHD형_분배!$C$2:$C$357,"&gt;="&amp;$B30,국내SCHD형_분배!$C$2:$C$357,"&lt;="&amp;$C30))</f>
+        <f>IF(COUNTIFS(국내SCHD형_분배!$A$2:$A$359,"402970",국내SCHD형_분배!$C$2:$C$359,"&gt;="&amp;$B30,국내SCHD형_분배!$C$2:$C$359,"&lt;="&amp;$C30)=0,"",SUMIFS(국내SCHD형_분배!$D$2:$D$359,국내SCHD형_분배!$A$2:$A$359,"402970",국내SCHD형_분배!$C$2:$C$359,"&gt;="&amp;$B30,국내SCHD형_분배!$C$2:$C$359,"&lt;="&amp;$C30))</f>
         <v/>
       </c>
       <c r="G30" s="53">
-        <f>IF(COUNTIFS(국내SCHD형_분배!$A$2:$A$357,"489250",국내SCHD형_분배!$C$2:$C$357,"&gt;="&amp;$B30,국내SCHD형_분배!$C$2:$C$357,"&lt;="&amp;$C30)=0,"",SUMIFS(국내SCHD형_분배!$D$2:$D$357,국내SCHD형_분배!$A$2:$A$357,"489250",국내SCHD형_분배!$C$2:$C$357,"&gt;="&amp;$B30,국내SCHD형_분배!$C$2:$C$357,"&lt;="&amp;$C30))</f>
+        <f>IF(COUNTIFS(국내SCHD형_분배!$A$2:$A$359,"489250",국내SCHD형_분배!$C$2:$C$359,"&gt;="&amp;$B30,국내SCHD형_분배!$C$2:$C$359,"&lt;="&amp;$C30)=0,"",SUMIFS(국내SCHD형_분배!$D$2:$D$359,국내SCHD형_분배!$A$2:$A$359,"489250",국내SCHD형_분배!$C$2:$C$359,"&gt;="&amp;$B30,국내SCHD형_분배!$C$2:$C$359,"&lt;="&amp;$C30))</f>
         <v/>
       </c>
       <c r="H30" s="28">
@@ -25695,19 +25737,19 @@
         <v/>
       </c>
       <c r="D31" s="53">
-        <f>IF(COUNTIFS(국내SCHD형_분배!$A$2:$A$357,"458730",국내SCHD형_분배!$C$2:$C$357,"&gt;="&amp;$B31,국내SCHD형_분배!$C$2:$C$357,"&lt;="&amp;$C31)=0,"",SUMIFS(국내SCHD형_분배!$D$2:$D$357,국내SCHD형_분배!$A$2:$A$357,"458730",국내SCHD형_분배!$C$2:$C$357,"&gt;="&amp;$B31,국내SCHD형_분배!$C$2:$C$357,"&lt;="&amp;$C31))</f>
+        <f>IF(COUNTIFS(국내SCHD형_분배!$A$2:$A$359,"458730",국내SCHD형_분배!$C$2:$C$359,"&gt;="&amp;$B31,국내SCHD형_분배!$C$2:$C$359,"&lt;="&amp;$C31)=0,"",SUMIFS(국내SCHD형_분배!$D$2:$D$359,국내SCHD형_분배!$A$2:$A$359,"458730",국내SCHD형_분배!$C$2:$C$359,"&gt;="&amp;$B31,국내SCHD형_분배!$C$2:$C$359,"&lt;="&amp;$C31))</f>
         <v/>
       </c>
       <c r="E31" s="53">
-        <f>IF(COUNTIFS(국내SCHD형_분배!$A$2:$A$357,"446720",국내SCHD형_분배!$C$2:$C$357,"&gt;="&amp;$B31,국내SCHD형_분배!$C$2:$C$357,"&lt;="&amp;$C31)=0,"",SUMIFS(국내SCHD형_분배!$D$2:$D$357,국내SCHD형_분배!$A$2:$A$357,"446720",국내SCHD형_분배!$C$2:$C$357,"&gt;="&amp;$B31,국내SCHD형_분배!$C$2:$C$357,"&lt;="&amp;$C31))</f>
+        <f>IF(COUNTIFS(국내SCHD형_분배!$A$2:$A$359,"446720",국내SCHD형_분배!$C$2:$C$359,"&gt;="&amp;$B31,국내SCHD형_분배!$C$2:$C$359,"&lt;="&amp;$C31)=0,"",SUMIFS(국내SCHD형_분배!$D$2:$D$359,국내SCHD형_분배!$A$2:$A$359,"446720",국내SCHD형_분배!$C$2:$C$359,"&gt;="&amp;$B31,국내SCHD형_분배!$C$2:$C$359,"&lt;="&amp;$C31))</f>
         <v/>
       </c>
       <c r="F31" s="53">
-        <f>IF(COUNTIFS(국내SCHD형_분배!$A$2:$A$357,"402970",국내SCHD형_분배!$C$2:$C$357,"&gt;="&amp;$B31,국내SCHD형_분배!$C$2:$C$357,"&lt;="&amp;$C31)=0,"",SUMIFS(국내SCHD형_분배!$D$2:$D$357,국내SCHD형_분배!$A$2:$A$357,"402970",국내SCHD형_분배!$C$2:$C$357,"&gt;="&amp;$B31,국내SCHD형_분배!$C$2:$C$357,"&lt;="&amp;$C31))</f>
+        <f>IF(COUNTIFS(국내SCHD형_분배!$A$2:$A$359,"402970",국내SCHD형_분배!$C$2:$C$359,"&gt;="&amp;$B31,국내SCHD형_분배!$C$2:$C$359,"&lt;="&amp;$C31)=0,"",SUMIFS(국내SCHD형_분배!$D$2:$D$359,국내SCHD형_분배!$A$2:$A$359,"402970",국내SCHD형_분배!$C$2:$C$359,"&gt;="&amp;$B31,국내SCHD형_분배!$C$2:$C$359,"&lt;="&amp;$C31))</f>
         <v/>
       </c>
       <c r="G31" s="53">
-        <f>IF(COUNTIFS(국내SCHD형_분배!$A$2:$A$357,"489250",국내SCHD형_분배!$C$2:$C$357,"&gt;="&amp;$B31,국내SCHD형_분배!$C$2:$C$357,"&lt;="&amp;$C31)=0,"",SUMIFS(국내SCHD형_분배!$D$2:$D$357,국내SCHD형_분배!$A$2:$A$357,"489250",국내SCHD형_분배!$C$2:$C$357,"&gt;="&amp;$B31,국내SCHD형_분배!$C$2:$C$357,"&lt;="&amp;$C31))</f>
+        <f>IF(COUNTIFS(국내SCHD형_분배!$A$2:$A$359,"489250",국내SCHD형_분배!$C$2:$C$359,"&gt;="&amp;$B31,국내SCHD형_분배!$C$2:$C$359,"&lt;="&amp;$C31)=0,"",SUMIFS(국내SCHD형_분배!$D$2:$D$359,국내SCHD형_분배!$A$2:$A$359,"489250",국내SCHD형_분배!$C$2:$C$359,"&gt;="&amp;$B31,국내SCHD형_분배!$C$2:$C$359,"&lt;="&amp;$C31))</f>
         <v/>
       </c>
       <c r="H31" s="28">
@@ -25733,19 +25775,19 @@
         <v/>
       </c>
       <c r="D32" s="53">
-        <f>IF(COUNTIFS(국내SCHD형_분배!$A$2:$A$357,"458730",국내SCHD형_분배!$C$2:$C$357,"&gt;="&amp;$B32,국내SCHD형_분배!$C$2:$C$357,"&lt;="&amp;$C32)=0,"",SUMIFS(국내SCHD형_분배!$D$2:$D$357,국내SCHD형_분배!$A$2:$A$357,"458730",국내SCHD형_분배!$C$2:$C$357,"&gt;="&amp;$B32,국내SCHD형_분배!$C$2:$C$357,"&lt;="&amp;$C32))</f>
+        <f>IF(COUNTIFS(국내SCHD형_분배!$A$2:$A$359,"458730",국내SCHD형_분배!$C$2:$C$359,"&gt;="&amp;$B32,국내SCHD형_분배!$C$2:$C$359,"&lt;="&amp;$C32)=0,"",SUMIFS(국내SCHD형_분배!$D$2:$D$359,국내SCHD형_분배!$A$2:$A$359,"458730",국내SCHD형_분배!$C$2:$C$359,"&gt;="&amp;$B32,국내SCHD형_분배!$C$2:$C$359,"&lt;="&amp;$C32))</f>
         <v/>
       </c>
       <c r="E32" s="53">
-        <f>IF(COUNTIFS(국내SCHD형_분배!$A$2:$A$357,"446720",국내SCHD형_분배!$C$2:$C$357,"&gt;="&amp;$B32,국내SCHD형_분배!$C$2:$C$357,"&lt;="&amp;$C32)=0,"",SUMIFS(국내SCHD형_분배!$D$2:$D$357,국내SCHD형_분배!$A$2:$A$357,"446720",국내SCHD형_분배!$C$2:$C$357,"&gt;="&amp;$B32,국내SCHD형_분배!$C$2:$C$357,"&lt;="&amp;$C32))</f>
+        <f>IF(COUNTIFS(국내SCHD형_분배!$A$2:$A$359,"446720",국내SCHD형_분배!$C$2:$C$359,"&gt;="&amp;$B32,국내SCHD형_분배!$C$2:$C$359,"&lt;="&amp;$C32)=0,"",SUMIFS(국내SCHD형_분배!$D$2:$D$359,국내SCHD형_분배!$A$2:$A$359,"446720",국내SCHD형_분배!$C$2:$C$359,"&gt;="&amp;$B32,국내SCHD형_분배!$C$2:$C$359,"&lt;="&amp;$C32))</f>
         <v/>
       </c>
       <c r="F32" s="53">
-        <f>IF(COUNTIFS(국내SCHD형_분배!$A$2:$A$357,"402970",국내SCHD형_분배!$C$2:$C$357,"&gt;="&amp;$B32,국내SCHD형_분배!$C$2:$C$357,"&lt;="&amp;$C32)=0,"",SUMIFS(국내SCHD형_분배!$D$2:$D$357,국내SCHD형_분배!$A$2:$A$357,"402970",국내SCHD형_분배!$C$2:$C$357,"&gt;="&amp;$B32,국내SCHD형_분배!$C$2:$C$357,"&lt;="&amp;$C32))</f>
+        <f>IF(COUNTIFS(국내SCHD형_분배!$A$2:$A$359,"402970",국내SCHD형_분배!$C$2:$C$359,"&gt;="&amp;$B32,국내SCHD형_분배!$C$2:$C$359,"&lt;="&amp;$C32)=0,"",SUMIFS(국내SCHD형_분배!$D$2:$D$359,국내SCHD형_분배!$A$2:$A$359,"402970",국내SCHD형_분배!$C$2:$C$359,"&gt;="&amp;$B32,국내SCHD형_분배!$C$2:$C$359,"&lt;="&amp;$C32))</f>
         <v/>
       </c>
       <c r="G32" s="53">
-        <f>IF(COUNTIFS(국내SCHD형_분배!$A$2:$A$357,"489250",국내SCHD형_분배!$C$2:$C$357,"&gt;="&amp;$B32,국내SCHD형_분배!$C$2:$C$357,"&lt;="&amp;$C32)=0,"",SUMIFS(국내SCHD형_분배!$D$2:$D$357,국내SCHD형_분배!$A$2:$A$357,"489250",국내SCHD형_분배!$C$2:$C$357,"&gt;="&amp;$B32,국내SCHD형_분배!$C$2:$C$357,"&lt;="&amp;$C32))</f>
+        <f>IF(COUNTIFS(국내SCHD형_분배!$A$2:$A$359,"489250",국내SCHD형_분배!$C$2:$C$359,"&gt;="&amp;$B32,국내SCHD형_분배!$C$2:$C$359,"&lt;="&amp;$C32)=0,"",SUMIFS(국내SCHD형_분배!$D$2:$D$359,국내SCHD형_분배!$A$2:$A$359,"489250",국내SCHD형_분배!$C$2:$C$359,"&gt;="&amp;$B32,국내SCHD형_분배!$C$2:$C$359,"&lt;="&amp;$C32))</f>
         <v/>
       </c>
       <c r="H32" s="28">
@@ -25771,19 +25813,19 @@
         <v/>
       </c>
       <c r="D33" s="53">
-        <f>IF(COUNTIFS(국내SCHD형_분배!$A$2:$A$357,"458730",국내SCHD형_분배!$C$2:$C$357,"&gt;="&amp;$B33,국내SCHD형_분배!$C$2:$C$357,"&lt;="&amp;$C33)=0,"",SUMIFS(국내SCHD형_분배!$D$2:$D$357,국내SCHD형_분배!$A$2:$A$357,"458730",국내SCHD형_분배!$C$2:$C$357,"&gt;="&amp;$B33,국내SCHD형_분배!$C$2:$C$357,"&lt;="&amp;$C33))</f>
+        <f>IF(COUNTIFS(국내SCHD형_분배!$A$2:$A$359,"458730",국내SCHD형_분배!$C$2:$C$359,"&gt;="&amp;$B33,국내SCHD형_분배!$C$2:$C$359,"&lt;="&amp;$C33)=0,"",SUMIFS(국내SCHD형_분배!$D$2:$D$359,국내SCHD형_분배!$A$2:$A$359,"458730",국내SCHD형_분배!$C$2:$C$359,"&gt;="&amp;$B33,국내SCHD형_분배!$C$2:$C$359,"&lt;="&amp;$C33))</f>
         <v/>
       </c>
       <c r="E33" s="53">
-        <f>IF(COUNTIFS(국내SCHD형_분배!$A$2:$A$357,"446720",국내SCHD형_분배!$C$2:$C$357,"&gt;="&amp;$B33,국내SCHD형_분배!$C$2:$C$357,"&lt;="&amp;$C33)=0,"",SUMIFS(국내SCHD형_분배!$D$2:$D$357,국내SCHD형_분배!$A$2:$A$357,"446720",국내SCHD형_분배!$C$2:$C$357,"&gt;="&amp;$B33,국내SCHD형_분배!$C$2:$C$357,"&lt;="&amp;$C33))</f>
+        <f>IF(COUNTIFS(국내SCHD형_분배!$A$2:$A$359,"446720",국내SCHD형_분배!$C$2:$C$359,"&gt;="&amp;$B33,국내SCHD형_분배!$C$2:$C$359,"&lt;="&amp;$C33)=0,"",SUMIFS(국내SCHD형_분배!$D$2:$D$359,국내SCHD형_분배!$A$2:$A$359,"446720",국내SCHD형_분배!$C$2:$C$359,"&gt;="&amp;$B33,국내SCHD형_분배!$C$2:$C$359,"&lt;="&amp;$C33))</f>
         <v/>
       </c>
       <c r="F33" s="53">
-        <f>IF(COUNTIFS(국내SCHD형_분배!$A$2:$A$357,"402970",국내SCHD형_분배!$C$2:$C$357,"&gt;="&amp;$B33,국내SCHD형_분배!$C$2:$C$357,"&lt;="&amp;$C33)=0,"",SUMIFS(국내SCHD형_분배!$D$2:$D$357,국내SCHD형_분배!$A$2:$A$357,"402970",국내SCHD형_분배!$C$2:$C$357,"&gt;="&amp;$B33,국내SCHD형_분배!$C$2:$C$357,"&lt;="&amp;$C33))</f>
+        <f>IF(COUNTIFS(국내SCHD형_분배!$A$2:$A$359,"402970",국내SCHD형_분배!$C$2:$C$359,"&gt;="&amp;$B33,국내SCHD형_분배!$C$2:$C$359,"&lt;="&amp;$C33)=0,"",SUMIFS(국내SCHD형_분배!$D$2:$D$359,국내SCHD형_분배!$A$2:$A$359,"402970",국내SCHD형_분배!$C$2:$C$359,"&gt;="&amp;$B33,국내SCHD형_분배!$C$2:$C$359,"&lt;="&amp;$C33))</f>
         <v/>
       </c>
       <c r="G33" s="53">
-        <f>IF(COUNTIFS(국내SCHD형_분배!$A$2:$A$357,"489250",국내SCHD형_분배!$C$2:$C$357,"&gt;="&amp;$B33,국내SCHD형_분배!$C$2:$C$357,"&lt;="&amp;$C33)=0,"",SUMIFS(국내SCHD형_분배!$D$2:$D$357,국내SCHD형_분배!$A$2:$A$357,"489250",국내SCHD형_분배!$C$2:$C$357,"&gt;="&amp;$B33,국내SCHD형_분배!$C$2:$C$357,"&lt;="&amp;$C33))</f>
+        <f>IF(COUNTIFS(국내SCHD형_분배!$A$2:$A$359,"489250",국내SCHD형_분배!$C$2:$C$359,"&gt;="&amp;$B33,국내SCHD형_분배!$C$2:$C$359,"&lt;="&amp;$C33)=0,"",SUMIFS(국내SCHD형_분배!$D$2:$D$359,국내SCHD형_분배!$A$2:$A$359,"489250",국내SCHD형_분배!$C$2:$C$359,"&gt;="&amp;$B33,국내SCHD형_분배!$C$2:$C$359,"&lt;="&amp;$C33))</f>
         <v/>
       </c>
       <c r="H33" s="28">
@@ -25809,19 +25851,19 @@
         <v/>
       </c>
       <c r="D34" s="53">
-        <f>IF(COUNTIFS(국내SCHD형_분배!$A$2:$A$357,"458730",국내SCHD형_분배!$C$2:$C$357,"&gt;="&amp;$B34,국내SCHD형_분배!$C$2:$C$357,"&lt;="&amp;$C34)=0,"",SUMIFS(국내SCHD형_분배!$D$2:$D$357,국내SCHD형_분배!$A$2:$A$357,"458730",국내SCHD형_분배!$C$2:$C$357,"&gt;="&amp;$B34,국내SCHD형_분배!$C$2:$C$357,"&lt;="&amp;$C34))</f>
+        <f>IF(COUNTIFS(국내SCHD형_분배!$A$2:$A$359,"458730",국내SCHD형_분배!$C$2:$C$359,"&gt;="&amp;$B34,국내SCHD형_분배!$C$2:$C$359,"&lt;="&amp;$C34)=0,"",SUMIFS(국내SCHD형_분배!$D$2:$D$359,국내SCHD형_분배!$A$2:$A$359,"458730",국내SCHD형_분배!$C$2:$C$359,"&gt;="&amp;$B34,국내SCHD형_분배!$C$2:$C$359,"&lt;="&amp;$C34))</f>
         <v/>
       </c>
       <c r="E34" s="53">
-        <f>IF(COUNTIFS(국내SCHD형_분배!$A$2:$A$357,"446720",국내SCHD형_분배!$C$2:$C$357,"&gt;="&amp;$B34,국내SCHD형_분배!$C$2:$C$357,"&lt;="&amp;$C34)=0,"",SUMIFS(국내SCHD형_분배!$D$2:$D$357,국내SCHD형_분배!$A$2:$A$357,"446720",국내SCHD형_분배!$C$2:$C$357,"&gt;="&amp;$B34,국내SCHD형_분배!$C$2:$C$357,"&lt;="&amp;$C34))</f>
+        <f>IF(COUNTIFS(국내SCHD형_분배!$A$2:$A$359,"446720",국내SCHD형_분배!$C$2:$C$359,"&gt;="&amp;$B34,국내SCHD형_분배!$C$2:$C$359,"&lt;="&amp;$C34)=0,"",SUMIFS(국내SCHD형_분배!$D$2:$D$359,국내SCHD형_분배!$A$2:$A$359,"446720",국내SCHD형_분배!$C$2:$C$359,"&gt;="&amp;$B34,국내SCHD형_분배!$C$2:$C$359,"&lt;="&amp;$C34))</f>
         <v/>
       </c>
       <c r="F34" s="53">
-        <f>IF(COUNTIFS(국내SCHD형_분배!$A$2:$A$357,"402970",국내SCHD형_분배!$C$2:$C$357,"&gt;="&amp;$B34,국내SCHD형_분배!$C$2:$C$357,"&lt;="&amp;$C34)=0,"",SUMIFS(국내SCHD형_분배!$D$2:$D$357,국내SCHD형_분배!$A$2:$A$357,"402970",국내SCHD형_분배!$C$2:$C$357,"&gt;="&amp;$B34,국내SCHD형_분배!$C$2:$C$357,"&lt;="&amp;$C34))</f>
+        <f>IF(COUNTIFS(국내SCHD형_분배!$A$2:$A$359,"402970",국내SCHD형_분배!$C$2:$C$359,"&gt;="&amp;$B34,국내SCHD형_분배!$C$2:$C$359,"&lt;="&amp;$C34)=0,"",SUMIFS(국내SCHD형_분배!$D$2:$D$359,국내SCHD형_분배!$A$2:$A$359,"402970",국내SCHD형_분배!$C$2:$C$359,"&gt;="&amp;$B34,국내SCHD형_분배!$C$2:$C$359,"&lt;="&amp;$C34))</f>
         <v/>
       </c>
       <c r="G34" s="53">
-        <f>IF(COUNTIFS(국내SCHD형_분배!$A$2:$A$357,"489250",국내SCHD형_분배!$C$2:$C$357,"&gt;="&amp;$B34,국내SCHD형_분배!$C$2:$C$357,"&lt;="&amp;$C34)=0,"",SUMIFS(국내SCHD형_분배!$D$2:$D$357,국내SCHD형_분배!$A$2:$A$357,"489250",국내SCHD형_분배!$C$2:$C$357,"&gt;="&amp;$B34,국내SCHD형_분배!$C$2:$C$357,"&lt;="&amp;$C34))</f>
+        <f>IF(COUNTIFS(국내SCHD형_분배!$A$2:$A$359,"489250",국내SCHD형_분배!$C$2:$C$359,"&gt;="&amp;$B34,국내SCHD형_분배!$C$2:$C$359,"&lt;="&amp;$C34)=0,"",SUMIFS(국내SCHD형_분배!$D$2:$D$359,국내SCHD형_분배!$A$2:$A$359,"489250",국내SCHD형_분배!$C$2:$C$359,"&gt;="&amp;$B34,국내SCHD형_분배!$C$2:$C$359,"&lt;="&amp;$C34))</f>
         <v/>
       </c>
       <c r="H34" s="28">
@@ -25847,19 +25889,19 @@
         <v/>
       </c>
       <c r="D35" s="53">
-        <f>IF(COUNTIFS(국내SCHD형_분배!$A$2:$A$357,"458730",국내SCHD형_분배!$C$2:$C$357,"&gt;="&amp;$B35,국내SCHD형_분배!$C$2:$C$357,"&lt;="&amp;$C35)=0,"",SUMIFS(국내SCHD형_분배!$D$2:$D$357,국내SCHD형_분배!$A$2:$A$357,"458730",국내SCHD형_분배!$C$2:$C$357,"&gt;="&amp;$B35,국내SCHD형_분배!$C$2:$C$357,"&lt;="&amp;$C35))</f>
+        <f>IF(COUNTIFS(국내SCHD형_분배!$A$2:$A$359,"458730",국내SCHD형_분배!$C$2:$C$359,"&gt;="&amp;$B35,국내SCHD형_분배!$C$2:$C$359,"&lt;="&amp;$C35)=0,"",SUMIFS(국내SCHD형_분배!$D$2:$D$359,국내SCHD형_분배!$A$2:$A$359,"458730",국내SCHD형_분배!$C$2:$C$359,"&gt;="&amp;$B35,국내SCHD형_분배!$C$2:$C$359,"&lt;="&amp;$C35))</f>
         <v/>
       </c>
       <c r="E35" s="53">
-        <f>IF(COUNTIFS(국내SCHD형_분배!$A$2:$A$357,"446720",국내SCHD형_분배!$C$2:$C$357,"&gt;="&amp;$B35,국내SCHD형_분배!$C$2:$C$357,"&lt;="&amp;$C35)=0,"",SUMIFS(국내SCHD형_분배!$D$2:$D$357,국내SCHD형_분배!$A$2:$A$357,"446720",국내SCHD형_분배!$C$2:$C$357,"&gt;="&amp;$B35,국내SCHD형_분배!$C$2:$C$357,"&lt;="&amp;$C35))</f>
+        <f>IF(COUNTIFS(국내SCHD형_분배!$A$2:$A$359,"446720",국내SCHD형_분배!$C$2:$C$359,"&gt;="&amp;$B35,국내SCHD형_분배!$C$2:$C$359,"&lt;="&amp;$C35)=0,"",SUMIFS(국내SCHD형_분배!$D$2:$D$359,국내SCHD형_분배!$A$2:$A$359,"446720",국내SCHD형_분배!$C$2:$C$359,"&gt;="&amp;$B35,국내SCHD형_분배!$C$2:$C$359,"&lt;="&amp;$C35))</f>
         <v/>
       </c>
       <c r="F35" s="53">
-        <f>IF(COUNTIFS(국내SCHD형_분배!$A$2:$A$357,"402970",국내SCHD형_분배!$C$2:$C$357,"&gt;="&amp;$B35,국내SCHD형_분배!$C$2:$C$357,"&lt;="&amp;$C35)=0,"",SUMIFS(국내SCHD형_분배!$D$2:$D$357,국내SCHD형_분배!$A$2:$A$357,"402970",국내SCHD형_분배!$C$2:$C$357,"&gt;="&amp;$B35,국내SCHD형_분배!$C$2:$C$357,"&lt;="&amp;$C35))</f>
+        <f>IF(COUNTIFS(국내SCHD형_분배!$A$2:$A$359,"402970",국내SCHD형_분배!$C$2:$C$359,"&gt;="&amp;$B35,국내SCHD형_분배!$C$2:$C$359,"&lt;="&amp;$C35)=0,"",SUMIFS(국내SCHD형_분배!$D$2:$D$359,국내SCHD형_분배!$A$2:$A$359,"402970",국내SCHD형_분배!$C$2:$C$359,"&gt;="&amp;$B35,국내SCHD형_분배!$C$2:$C$359,"&lt;="&amp;$C35))</f>
         <v/>
       </c>
       <c r="G35" s="53">
-        <f>IF(COUNTIFS(국내SCHD형_분배!$A$2:$A$357,"489250",국내SCHD형_분배!$C$2:$C$357,"&gt;="&amp;$B35,국내SCHD형_분배!$C$2:$C$357,"&lt;="&amp;$C35)=0,"",SUMIFS(국내SCHD형_분배!$D$2:$D$357,국내SCHD형_분배!$A$2:$A$357,"489250",국내SCHD형_분배!$C$2:$C$357,"&gt;="&amp;$B35,국내SCHD형_분배!$C$2:$C$357,"&lt;="&amp;$C35))</f>
+        <f>IF(COUNTIFS(국내SCHD형_분배!$A$2:$A$359,"489250",국내SCHD형_분배!$C$2:$C$359,"&gt;="&amp;$B35,국내SCHD형_분배!$C$2:$C$359,"&lt;="&amp;$C35)=0,"",SUMIFS(국내SCHD형_분배!$D$2:$D$359,국내SCHD형_분배!$A$2:$A$359,"489250",국내SCHD형_분배!$C$2:$C$359,"&gt;="&amp;$B35,국내SCHD형_분배!$C$2:$C$359,"&lt;="&amp;$C35))</f>
         <v/>
       </c>
       <c r="H35" s="28">
@@ -25885,19 +25927,19 @@
         <v/>
       </c>
       <c r="D36" s="53">
-        <f>IF(COUNTIFS(국내SCHD형_분배!$A$2:$A$357,"458730",국내SCHD형_분배!$C$2:$C$357,"&gt;="&amp;$B36,국내SCHD형_분배!$C$2:$C$357,"&lt;="&amp;$C36)=0,"",SUMIFS(국내SCHD형_분배!$D$2:$D$357,국내SCHD형_분배!$A$2:$A$357,"458730",국내SCHD형_분배!$C$2:$C$357,"&gt;="&amp;$B36,국내SCHD형_분배!$C$2:$C$357,"&lt;="&amp;$C36))</f>
+        <f>IF(COUNTIFS(국내SCHD형_분배!$A$2:$A$359,"458730",국내SCHD형_분배!$C$2:$C$359,"&gt;="&amp;$B36,국내SCHD형_분배!$C$2:$C$359,"&lt;="&amp;$C36)=0,"",SUMIFS(국내SCHD형_분배!$D$2:$D$359,국내SCHD형_분배!$A$2:$A$359,"458730",국내SCHD형_분배!$C$2:$C$359,"&gt;="&amp;$B36,국내SCHD형_분배!$C$2:$C$359,"&lt;="&amp;$C36))</f>
         <v/>
       </c>
       <c r="E36" s="53">
-        <f>IF(COUNTIFS(국내SCHD형_분배!$A$2:$A$357,"446720",국내SCHD형_분배!$C$2:$C$357,"&gt;="&amp;$B36,국내SCHD형_분배!$C$2:$C$357,"&lt;="&amp;$C36)=0,"",SUMIFS(국내SCHD형_분배!$D$2:$D$357,국내SCHD형_분배!$A$2:$A$357,"446720",국내SCHD형_분배!$C$2:$C$357,"&gt;="&amp;$B36,국내SCHD형_분배!$C$2:$C$357,"&lt;="&amp;$C36))</f>
+        <f>IF(COUNTIFS(국내SCHD형_분배!$A$2:$A$359,"446720",국내SCHD형_분배!$C$2:$C$359,"&gt;="&amp;$B36,국내SCHD형_분배!$C$2:$C$359,"&lt;="&amp;$C36)=0,"",SUMIFS(국내SCHD형_분배!$D$2:$D$359,국내SCHD형_분배!$A$2:$A$359,"446720",국내SCHD형_분배!$C$2:$C$359,"&gt;="&amp;$B36,국내SCHD형_분배!$C$2:$C$359,"&lt;="&amp;$C36))</f>
         <v/>
       </c>
       <c r="F36" s="53">
-        <f>IF(COUNTIFS(국내SCHD형_분배!$A$2:$A$357,"402970",국내SCHD형_분배!$C$2:$C$357,"&gt;="&amp;$B36,국내SCHD형_분배!$C$2:$C$357,"&lt;="&amp;$C36)=0,"",SUMIFS(국내SCHD형_분배!$D$2:$D$357,국내SCHD형_분배!$A$2:$A$357,"402970",국내SCHD형_분배!$C$2:$C$357,"&gt;="&amp;$B36,국내SCHD형_분배!$C$2:$C$357,"&lt;="&amp;$C36))</f>
+        <f>IF(COUNTIFS(국내SCHD형_분배!$A$2:$A$359,"402970",국내SCHD형_분배!$C$2:$C$359,"&gt;="&amp;$B36,국내SCHD형_분배!$C$2:$C$359,"&lt;="&amp;$C36)=0,"",SUMIFS(국내SCHD형_분배!$D$2:$D$359,국내SCHD형_분배!$A$2:$A$359,"402970",국내SCHD형_분배!$C$2:$C$359,"&gt;="&amp;$B36,국내SCHD형_분배!$C$2:$C$359,"&lt;="&amp;$C36))</f>
         <v/>
       </c>
       <c r="G36" s="53">
-        <f>IF(COUNTIFS(국내SCHD형_분배!$A$2:$A$357,"489250",국내SCHD형_분배!$C$2:$C$357,"&gt;="&amp;$B36,국내SCHD형_분배!$C$2:$C$357,"&lt;="&amp;$C36)=0,"",SUMIFS(국내SCHD형_분배!$D$2:$D$357,국내SCHD형_분배!$A$2:$A$357,"489250",국내SCHD형_분배!$C$2:$C$357,"&gt;="&amp;$B36,국내SCHD형_분배!$C$2:$C$357,"&lt;="&amp;$C36))</f>
+        <f>IF(COUNTIFS(국내SCHD형_분배!$A$2:$A$359,"489250",국내SCHD형_분배!$C$2:$C$359,"&gt;="&amp;$B36,국내SCHD형_분배!$C$2:$C$359,"&lt;="&amp;$C36)=0,"",SUMIFS(국내SCHD형_분배!$D$2:$D$359,국내SCHD형_분배!$A$2:$A$359,"489250",국내SCHD형_분배!$C$2:$C$359,"&gt;="&amp;$B36,국내SCHD형_분배!$C$2:$C$359,"&lt;="&amp;$C36))</f>
         <v/>
       </c>
       <c r="H36" s="28">
@@ -25923,19 +25965,19 @@
         <v/>
       </c>
       <c r="D37" s="53">
-        <f>IF(COUNTIFS(국내SCHD형_분배!$A$2:$A$357,"458730",국내SCHD형_분배!$C$2:$C$357,"&gt;="&amp;$B37,국내SCHD형_분배!$C$2:$C$357,"&lt;="&amp;$C37)=0,"",SUMIFS(국내SCHD형_분배!$D$2:$D$357,국내SCHD형_분배!$A$2:$A$357,"458730",국내SCHD형_분배!$C$2:$C$357,"&gt;="&amp;$B37,국내SCHD형_분배!$C$2:$C$357,"&lt;="&amp;$C37))</f>
+        <f>IF(COUNTIFS(국내SCHD형_분배!$A$2:$A$359,"458730",국내SCHD형_분배!$C$2:$C$359,"&gt;="&amp;$B37,국내SCHD형_분배!$C$2:$C$359,"&lt;="&amp;$C37)=0,"",SUMIFS(국내SCHD형_분배!$D$2:$D$359,국내SCHD형_분배!$A$2:$A$359,"458730",국내SCHD형_분배!$C$2:$C$359,"&gt;="&amp;$B37,국내SCHD형_분배!$C$2:$C$359,"&lt;="&amp;$C37))</f>
         <v/>
       </c>
       <c r="E37" s="53">
-        <f>IF(COUNTIFS(국내SCHD형_분배!$A$2:$A$357,"446720",국내SCHD형_분배!$C$2:$C$357,"&gt;="&amp;$B37,국내SCHD형_분배!$C$2:$C$357,"&lt;="&amp;$C37)=0,"",SUMIFS(국내SCHD형_분배!$D$2:$D$357,국내SCHD형_분배!$A$2:$A$357,"446720",국내SCHD형_분배!$C$2:$C$357,"&gt;="&amp;$B37,국내SCHD형_분배!$C$2:$C$357,"&lt;="&amp;$C37))</f>
+        <f>IF(COUNTIFS(국내SCHD형_분배!$A$2:$A$359,"446720",국내SCHD형_분배!$C$2:$C$359,"&gt;="&amp;$B37,국내SCHD형_분배!$C$2:$C$359,"&lt;="&amp;$C37)=0,"",SUMIFS(국내SCHD형_분배!$D$2:$D$359,국내SCHD형_분배!$A$2:$A$359,"446720",국내SCHD형_분배!$C$2:$C$359,"&gt;="&amp;$B37,국내SCHD형_분배!$C$2:$C$359,"&lt;="&amp;$C37))</f>
         <v/>
       </c>
       <c r="F37" s="53">
-        <f>IF(COUNTIFS(국내SCHD형_분배!$A$2:$A$357,"402970",국내SCHD형_분배!$C$2:$C$357,"&gt;="&amp;$B37,국내SCHD형_분배!$C$2:$C$357,"&lt;="&amp;$C37)=0,"",SUMIFS(국내SCHD형_분배!$D$2:$D$357,국내SCHD형_분배!$A$2:$A$357,"402970",국내SCHD형_분배!$C$2:$C$357,"&gt;="&amp;$B37,국내SCHD형_분배!$C$2:$C$357,"&lt;="&amp;$C37))</f>
+        <f>IF(COUNTIFS(국내SCHD형_분배!$A$2:$A$359,"402970",국내SCHD형_분배!$C$2:$C$359,"&gt;="&amp;$B37,국내SCHD형_분배!$C$2:$C$359,"&lt;="&amp;$C37)=0,"",SUMIFS(국내SCHD형_분배!$D$2:$D$359,국내SCHD형_분배!$A$2:$A$359,"402970",국내SCHD형_분배!$C$2:$C$359,"&gt;="&amp;$B37,국내SCHD형_분배!$C$2:$C$359,"&lt;="&amp;$C37))</f>
         <v/>
       </c>
       <c r="G37" s="53">
-        <f>IF(COUNTIFS(국내SCHD형_분배!$A$2:$A$357,"489250",국내SCHD형_분배!$C$2:$C$357,"&gt;="&amp;$B37,국내SCHD형_분배!$C$2:$C$357,"&lt;="&amp;$C37)=0,"",SUMIFS(국내SCHD형_분배!$D$2:$D$357,국내SCHD형_분배!$A$2:$A$357,"489250",국내SCHD형_분배!$C$2:$C$357,"&gt;="&amp;$B37,국내SCHD형_분배!$C$2:$C$357,"&lt;="&amp;$C37))</f>
+        <f>IF(COUNTIFS(국내SCHD형_분배!$A$2:$A$359,"489250",국내SCHD형_분배!$C$2:$C$359,"&gt;="&amp;$B37,국내SCHD형_분배!$C$2:$C$359,"&lt;="&amp;$C37)=0,"",SUMIFS(국내SCHD형_분배!$D$2:$D$359,국내SCHD형_분배!$A$2:$A$359,"489250",국내SCHD형_분배!$C$2:$C$359,"&gt;="&amp;$B37,국내SCHD형_분배!$C$2:$C$359,"&lt;="&amp;$C37))</f>
         <v/>
       </c>
       <c r="H37" s="28">
@@ -25961,19 +26003,19 @@
         <v/>
       </c>
       <c r="D38" s="53">
-        <f>IF(COUNTIFS(국내SCHD형_분배!$A$2:$A$357,"458730",국내SCHD형_분배!$C$2:$C$357,"&gt;="&amp;$B38,국내SCHD형_분배!$C$2:$C$357,"&lt;="&amp;$C38)=0,"",SUMIFS(국내SCHD형_분배!$D$2:$D$357,국내SCHD형_분배!$A$2:$A$357,"458730",국내SCHD형_분배!$C$2:$C$357,"&gt;="&amp;$B38,국내SCHD형_분배!$C$2:$C$357,"&lt;="&amp;$C38))</f>
+        <f>IF(COUNTIFS(국내SCHD형_분배!$A$2:$A$359,"458730",국내SCHD형_분배!$C$2:$C$359,"&gt;="&amp;$B38,국내SCHD형_분배!$C$2:$C$359,"&lt;="&amp;$C38)=0,"",SUMIFS(국내SCHD형_분배!$D$2:$D$359,국내SCHD형_분배!$A$2:$A$359,"458730",국내SCHD형_분배!$C$2:$C$359,"&gt;="&amp;$B38,국내SCHD형_분배!$C$2:$C$359,"&lt;="&amp;$C38))</f>
         <v/>
       </c>
       <c r="E38" s="53">
-        <f>IF(COUNTIFS(국내SCHD형_분배!$A$2:$A$357,"446720",국내SCHD형_분배!$C$2:$C$357,"&gt;="&amp;$B38,국내SCHD형_분배!$C$2:$C$357,"&lt;="&amp;$C38)=0,"",SUMIFS(국내SCHD형_분배!$D$2:$D$357,국내SCHD형_분배!$A$2:$A$357,"446720",국내SCHD형_분배!$C$2:$C$357,"&gt;="&amp;$B38,국내SCHD형_분배!$C$2:$C$357,"&lt;="&amp;$C38))</f>
+        <f>IF(COUNTIFS(국내SCHD형_분배!$A$2:$A$359,"446720",국내SCHD형_분배!$C$2:$C$359,"&gt;="&amp;$B38,국내SCHD형_분배!$C$2:$C$359,"&lt;="&amp;$C38)=0,"",SUMIFS(국내SCHD형_분배!$D$2:$D$359,국내SCHD형_분배!$A$2:$A$359,"446720",국내SCHD형_분배!$C$2:$C$359,"&gt;="&amp;$B38,국내SCHD형_분배!$C$2:$C$359,"&lt;="&amp;$C38))</f>
         <v/>
       </c>
       <c r="F38" s="53">
-        <f>IF(COUNTIFS(국내SCHD형_분배!$A$2:$A$357,"402970",국내SCHD형_분배!$C$2:$C$357,"&gt;="&amp;$B38,국내SCHD형_분배!$C$2:$C$357,"&lt;="&amp;$C38)=0,"",SUMIFS(국내SCHD형_분배!$D$2:$D$357,국내SCHD형_분배!$A$2:$A$357,"402970",국내SCHD형_분배!$C$2:$C$357,"&gt;="&amp;$B38,국내SCHD형_분배!$C$2:$C$357,"&lt;="&amp;$C38))</f>
+        <f>IF(COUNTIFS(국내SCHD형_분배!$A$2:$A$359,"402970",국내SCHD형_분배!$C$2:$C$359,"&gt;="&amp;$B38,국내SCHD형_분배!$C$2:$C$359,"&lt;="&amp;$C38)=0,"",SUMIFS(국내SCHD형_분배!$D$2:$D$359,국내SCHD형_분배!$A$2:$A$359,"402970",국내SCHD형_분배!$C$2:$C$359,"&gt;="&amp;$B38,국내SCHD형_분배!$C$2:$C$359,"&lt;="&amp;$C38))</f>
         <v/>
       </c>
       <c r="G38" s="53">
-        <f>IF(COUNTIFS(국내SCHD형_분배!$A$2:$A$357,"489250",국내SCHD형_분배!$C$2:$C$357,"&gt;="&amp;$B38,국내SCHD형_분배!$C$2:$C$357,"&lt;="&amp;$C38)=0,"",SUMIFS(국내SCHD형_분배!$D$2:$D$357,국내SCHD형_분배!$A$2:$A$357,"489250",국내SCHD형_분배!$C$2:$C$357,"&gt;="&amp;$B38,국내SCHD형_분배!$C$2:$C$357,"&lt;="&amp;$C38))</f>
+        <f>IF(COUNTIFS(국내SCHD형_분배!$A$2:$A$359,"489250",국내SCHD형_분배!$C$2:$C$359,"&gt;="&amp;$B38,국내SCHD형_분배!$C$2:$C$359,"&lt;="&amp;$C38)=0,"",SUMIFS(국내SCHD형_분배!$D$2:$D$359,국내SCHD형_분배!$A$2:$A$359,"489250",국내SCHD형_분배!$C$2:$C$359,"&gt;="&amp;$B38,국내SCHD형_분배!$C$2:$C$359,"&lt;="&amp;$C38))</f>
         <v/>
       </c>
       <c r="H38" s="28">
@@ -25999,19 +26041,19 @@
         <v/>
       </c>
       <c r="D39" s="53">
-        <f>IF(COUNTIFS(국내SCHD형_분배!$A$2:$A$357,"458730",국내SCHD형_분배!$C$2:$C$357,"&gt;="&amp;$B39,국내SCHD형_분배!$C$2:$C$357,"&lt;="&amp;$C39)=0,"",SUMIFS(국내SCHD형_분배!$D$2:$D$357,국내SCHD형_분배!$A$2:$A$357,"458730",국내SCHD형_분배!$C$2:$C$357,"&gt;="&amp;$B39,국내SCHD형_분배!$C$2:$C$357,"&lt;="&amp;$C39))</f>
+        <f>IF(COUNTIFS(국내SCHD형_분배!$A$2:$A$359,"458730",국내SCHD형_분배!$C$2:$C$359,"&gt;="&amp;$B39,국내SCHD형_분배!$C$2:$C$359,"&lt;="&amp;$C39)=0,"",SUMIFS(국내SCHD형_분배!$D$2:$D$359,국내SCHD형_분배!$A$2:$A$359,"458730",국내SCHD형_분배!$C$2:$C$359,"&gt;="&amp;$B39,국내SCHD형_분배!$C$2:$C$359,"&lt;="&amp;$C39))</f>
         <v/>
       </c>
       <c r="E39" s="53">
-        <f>IF(COUNTIFS(국내SCHD형_분배!$A$2:$A$357,"446720",국내SCHD형_분배!$C$2:$C$357,"&gt;="&amp;$B39,국내SCHD형_분배!$C$2:$C$357,"&lt;="&amp;$C39)=0,"",SUMIFS(국내SCHD형_분배!$D$2:$D$357,국내SCHD형_분배!$A$2:$A$357,"446720",국내SCHD형_분배!$C$2:$C$357,"&gt;="&amp;$B39,국내SCHD형_분배!$C$2:$C$357,"&lt;="&amp;$C39))</f>
+        <f>IF(COUNTIFS(국내SCHD형_분배!$A$2:$A$359,"446720",국내SCHD형_분배!$C$2:$C$359,"&gt;="&amp;$B39,국내SCHD형_분배!$C$2:$C$359,"&lt;="&amp;$C39)=0,"",SUMIFS(국내SCHD형_분배!$D$2:$D$359,국내SCHD형_분배!$A$2:$A$359,"446720",국내SCHD형_분배!$C$2:$C$359,"&gt;="&amp;$B39,국내SCHD형_분배!$C$2:$C$359,"&lt;="&amp;$C39))</f>
         <v/>
       </c>
       <c r="F39" s="53">
-        <f>IF(COUNTIFS(국내SCHD형_분배!$A$2:$A$357,"402970",국내SCHD형_분배!$C$2:$C$357,"&gt;="&amp;$B39,국내SCHD형_분배!$C$2:$C$357,"&lt;="&amp;$C39)=0,"",SUMIFS(국내SCHD형_분배!$D$2:$D$357,국내SCHD형_분배!$A$2:$A$357,"402970",국내SCHD형_분배!$C$2:$C$357,"&gt;="&amp;$B39,국내SCHD형_분배!$C$2:$C$357,"&lt;="&amp;$C39))</f>
+        <f>IF(COUNTIFS(국내SCHD형_분배!$A$2:$A$359,"402970",국내SCHD형_분배!$C$2:$C$359,"&gt;="&amp;$B39,국내SCHD형_분배!$C$2:$C$359,"&lt;="&amp;$C39)=0,"",SUMIFS(국내SCHD형_분배!$D$2:$D$359,국내SCHD형_분배!$A$2:$A$359,"402970",국내SCHD형_분배!$C$2:$C$359,"&gt;="&amp;$B39,국내SCHD형_분배!$C$2:$C$359,"&lt;="&amp;$C39))</f>
         <v/>
       </c>
       <c r="G39" s="53">
-        <f>IF(COUNTIFS(국내SCHD형_분배!$A$2:$A$357,"489250",국내SCHD형_분배!$C$2:$C$357,"&gt;="&amp;$B39,국내SCHD형_분배!$C$2:$C$357,"&lt;="&amp;$C39)=0,"",SUMIFS(국내SCHD형_분배!$D$2:$D$357,국내SCHD형_분배!$A$2:$A$357,"489250",국내SCHD형_분배!$C$2:$C$357,"&gt;="&amp;$B39,국내SCHD형_분배!$C$2:$C$357,"&lt;="&amp;$C39))</f>
+        <f>IF(COUNTIFS(국내SCHD형_분배!$A$2:$A$359,"489250",국내SCHD형_분배!$C$2:$C$359,"&gt;="&amp;$B39,국내SCHD형_분배!$C$2:$C$359,"&lt;="&amp;$C39)=0,"",SUMIFS(국내SCHD형_분배!$D$2:$D$359,국내SCHD형_분배!$A$2:$A$359,"489250",국내SCHD형_분배!$C$2:$C$359,"&gt;="&amp;$B39,국내SCHD형_분배!$C$2:$C$359,"&lt;="&amp;$C39))</f>
         <v/>
       </c>
       <c r="H39" s="28">
@@ -26037,19 +26079,19 @@
         <v/>
       </c>
       <c r="D40" s="53">
-        <f>IF(COUNTIFS(국내SCHD형_분배!$A$2:$A$357,"458730",국내SCHD형_분배!$C$2:$C$357,"&gt;="&amp;$B40,국내SCHD형_분배!$C$2:$C$357,"&lt;="&amp;$C40)=0,"",SUMIFS(국내SCHD형_분배!$D$2:$D$357,국내SCHD형_분배!$A$2:$A$357,"458730",국내SCHD형_분배!$C$2:$C$357,"&gt;="&amp;$B40,국내SCHD형_분배!$C$2:$C$357,"&lt;="&amp;$C40))</f>
+        <f>IF(COUNTIFS(국내SCHD형_분배!$A$2:$A$359,"458730",국내SCHD형_분배!$C$2:$C$359,"&gt;="&amp;$B40,국내SCHD형_분배!$C$2:$C$359,"&lt;="&amp;$C40)=0,"",SUMIFS(국내SCHD형_분배!$D$2:$D$359,국내SCHD형_분배!$A$2:$A$359,"458730",국내SCHD형_분배!$C$2:$C$359,"&gt;="&amp;$B40,국내SCHD형_분배!$C$2:$C$359,"&lt;="&amp;$C40))</f>
         <v/>
       </c>
       <c r="E40" s="53">
-        <f>IF(COUNTIFS(국내SCHD형_분배!$A$2:$A$357,"446720",국내SCHD형_분배!$C$2:$C$357,"&gt;="&amp;$B40,국내SCHD형_분배!$C$2:$C$357,"&lt;="&amp;$C40)=0,"",SUMIFS(국내SCHD형_분배!$D$2:$D$357,국내SCHD형_분배!$A$2:$A$357,"446720",국내SCHD형_분배!$C$2:$C$357,"&gt;="&amp;$B40,국내SCHD형_분배!$C$2:$C$357,"&lt;="&amp;$C40))</f>
+        <f>IF(COUNTIFS(국내SCHD형_분배!$A$2:$A$359,"446720",국내SCHD형_분배!$C$2:$C$359,"&gt;="&amp;$B40,국내SCHD형_분배!$C$2:$C$359,"&lt;="&amp;$C40)=0,"",SUMIFS(국내SCHD형_분배!$D$2:$D$359,국내SCHD형_분배!$A$2:$A$359,"446720",국내SCHD형_분배!$C$2:$C$359,"&gt;="&amp;$B40,국내SCHD형_분배!$C$2:$C$359,"&lt;="&amp;$C40))</f>
         <v/>
       </c>
       <c r="F40" s="53">
-        <f>IF(COUNTIFS(국내SCHD형_분배!$A$2:$A$357,"402970",국내SCHD형_분배!$C$2:$C$357,"&gt;="&amp;$B40,국내SCHD형_분배!$C$2:$C$357,"&lt;="&amp;$C40)=0,"",SUMIFS(국내SCHD형_분배!$D$2:$D$357,국내SCHD형_분배!$A$2:$A$357,"402970",국내SCHD형_분배!$C$2:$C$357,"&gt;="&amp;$B40,국내SCHD형_분배!$C$2:$C$357,"&lt;="&amp;$C40))</f>
+        <f>IF(COUNTIFS(국내SCHD형_분배!$A$2:$A$359,"402970",국내SCHD형_분배!$C$2:$C$359,"&gt;="&amp;$B40,국내SCHD형_분배!$C$2:$C$359,"&lt;="&amp;$C40)=0,"",SUMIFS(국내SCHD형_분배!$D$2:$D$359,국내SCHD형_분배!$A$2:$A$359,"402970",국내SCHD형_분배!$C$2:$C$359,"&gt;="&amp;$B40,국내SCHD형_분배!$C$2:$C$359,"&lt;="&amp;$C40))</f>
         <v/>
       </c>
       <c r="G40" s="53">
-        <f>IF(COUNTIFS(국내SCHD형_분배!$A$2:$A$357,"489250",국내SCHD형_분배!$C$2:$C$357,"&gt;="&amp;$B40,국내SCHD형_분배!$C$2:$C$357,"&lt;="&amp;$C40)=0,"",SUMIFS(국내SCHD형_분배!$D$2:$D$357,국내SCHD형_분배!$A$2:$A$357,"489250",국내SCHD형_분배!$C$2:$C$357,"&gt;="&amp;$B40,국내SCHD형_분배!$C$2:$C$357,"&lt;="&amp;$C40))</f>
+        <f>IF(COUNTIFS(국내SCHD형_분배!$A$2:$A$359,"489250",국내SCHD형_분배!$C$2:$C$359,"&gt;="&amp;$B40,국내SCHD형_분배!$C$2:$C$359,"&lt;="&amp;$C40)=0,"",SUMIFS(국내SCHD형_분배!$D$2:$D$359,국내SCHD형_분배!$A$2:$A$359,"489250",국내SCHD형_분배!$C$2:$C$359,"&gt;="&amp;$B40,국내SCHD형_분배!$C$2:$C$359,"&lt;="&amp;$C40))</f>
         <v/>
       </c>
       <c r="H40" s="28">
@@ -26075,19 +26117,19 @@
         <v/>
       </c>
       <c r="D41" s="53">
-        <f>IF(COUNTIFS(국내SCHD형_분배!$A$2:$A$357,"458730",국내SCHD형_분배!$C$2:$C$357,"&gt;="&amp;$B41,국내SCHD형_분배!$C$2:$C$357,"&lt;="&amp;$C41)=0,"",SUMIFS(국내SCHD형_분배!$D$2:$D$357,국내SCHD형_분배!$A$2:$A$357,"458730",국내SCHD형_분배!$C$2:$C$357,"&gt;="&amp;$B41,국내SCHD형_분배!$C$2:$C$357,"&lt;="&amp;$C41))</f>
+        <f>IF(COUNTIFS(국내SCHD형_분배!$A$2:$A$359,"458730",국내SCHD형_분배!$C$2:$C$359,"&gt;="&amp;$B41,국내SCHD형_분배!$C$2:$C$359,"&lt;="&amp;$C41)=0,"",SUMIFS(국내SCHD형_분배!$D$2:$D$359,국내SCHD형_분배!$A$2:$A$359,"458730",국내SCHD형_분배!$C$2:$C$359,"&gt;="&amp;$B41,국내SCHD형_분배!$C$2:$C$359,"&lt;="&amp;$C41))</f>
         <v/>
       </c>
       <c r="E41" s="53">
-        <f>IF(COUNTIFS(국내SCHD형_분배!$A$2:$A$357,"446720",국내SCHD형_분배!$C$2:$C$357,"&gt;="&amp;$B41,국내SCHD형_분배!$C$2:$C$357,"&lt;="&amp;$C41)=0,"",SUMIFS(국내SCHD형_분배!$D$2:$D$357,국내SCHD형_분배!$A$2:$A$357,"446720",국내SCHD형_분배!$C$2:$C$357,"&gt;="&amp;$B41,국내SCHD형_분배!$C$2:$C$357,"&lt;="&amp;$C41))</f>
+        <f>IF(COUNTIFS(국내SCHD형_분배!$A$2:$A$359,"446720",국내SCHD형_분배!$C$2:$C$359,"&gt;="&amp;$B41,국내SCHD형_분배!$C$2:$C$359,"&lt;="&amp;$C41)=0,"",SUMIFS(국내SCHD형_분배!$D$2:$D$359,국내SCHD형_분배!$A$2:$A$359,"446720",국내SCHD형_분배!$C$2:$C$359,"&gt;="&amp;$B41,국내SCHD형_분배!$C$2:$C$359,"&lt;="&amp;$C41))</f>
         <v/>
       </c>
       <c r="F41" s="53">
-        <f>IF(COUNTIFS(국내SCHD형_분배!$A$2:$A$357,"402970",국내SCHD형_분배!$C$2:$C$357,"&gt;="&amp;$B41,국내SCHD형_분배!$C$2:$C$357,"&lt;="&amp;$C41)=0,"",SUMIFS(국내SCHD형_분배!$D$2:$D$357,국내SCHD형_분배!$A$2:$A$357,"402970",국내SCHD형_분배!$C$2:$C$357,"&gt;="&amp;$B41,국내SCHD형_분배!$C$2:$C$357,"&lt;="&amp;$C41))</f>
+        <f>IF(COUNTIFS(국내SCHD형_분배!$A$2:$A$359,"402970",국내SCHD형_분배!$C$2:$C$359,"&gt;="&amp;$B41,국내SCHD형_분배!$C$2:$C$359,"&lt;="&amp;$C41)=0,"",SUMIFS(국내SCHD형_분배!$D$2:$D$359,국내SCHD형_분배!$A$2:$A$359,"402970",국내SCHD형_분배!$C$2:$C$359,"&gt;="&amp;$B41,국내SCHD형_분배!$C$2:$C$359,"&lt;="&amp;$C41))</f>
         <v/>
       </c>
       <c r="G41" s="53">
-        <f>IF(COUNTIFS(국내SCHD형_분배!$A$2:$A$357,"489250",국내SCHD형_분배!$C$2:$C$357,"&gt;="&amp;$B41,국내SCHD형_분배!$C$2:$C$357,"&lt;="&amp;$C41)=0,"",SUMIFS(국내SCHD형_분배!$D$2:$D$357,국내SCHD형_분배!$A$2:$A$357,"489250",국내SCHD형_분배!$C$2:$C$357,"&gt;="&amp;$B41,국내SCHD형_분배!$C$2:$C$357,"&lt;="&amp;$C41))</f>
+        <f>IF(COUNTIFS(국내SCHD형_분배!$A$2:$A$359,"489250",국내SCHD형_분배!$C$2:$C$359,"&gt;="&amp;$B41,국내SCHD형_분배!$C$2:$C$359,"&lt;="&amp;$C41)=0,"",SUMIFS(국내SCHD형_분배!$D$2:$D$359,국내SCHD형_분배!$A$2:$A$359,"489250",국내SCHD형_분배!$C$2:$C$359,"&gt;="&amp;$B41,국내SCHD형_분배!$C$2:$C$359,"&lt;="&amp;$C41))</f>
         <v/>
       </c>
       <c r="H41" s="28">
@@ -26113,19 +26155,19 @@
         <v/>
       </c>
       <c r="D42" s="53">
-        <f>IF(COUNTIFS(국내SCHD형_분배!$A$2:$A$357,"458730",국내SCHD형_분배!$C$2:$C$357,"&gt;="&amp;$B42,국내SCHD형_분배!$C$2:$C$357,"&lt;="&amp;$C42)=0,"",SUMIFS(국내SCHD형_분배!$D$2:$D$357,국내SCHD형_분배!$A$2:$A$357,"458730",국내SCHD형_분배!$C$2:$C$357,"&gt;="&amp;$B42,국내SCHD형_분배!$C$2:$C$357,"&lt;="&amp;$C42))</f>
+        <f>IF(COUNTIFS(국내SCHD형_분배!$A$2:$A$359,"458730",국내SCHD형_분배!$C$2:$C$359,"&gt;="&amp;$B42,국내SCHD형_분배!$C$2:$C$359,"&lt;="&amp;$C42)=0,"",SUMIFS(국내SCHD형_분배!$D$2:$D$359,국내SCHD형_분배!$A$2:$A$359,"458730",국내SCHD형_분배!$C$2:$C$359,"&gt;="&amp;$B42,국내SCHD형_분배!$C$2:$C$359,"&lt;="&amp;$C42))</f>
         <v/>
       </c>
       <c r="E42" s="53">
-        <f>IF(COUNTIFS(국내SCHD형_분배!$A$2:$A$357,"446720",국내SCHD형_분배!$C$2:$C$357,"&gt;="&amp;$B42,국내SCHD형_분배!$C$2:$C$357,"&lt;="&amp;$C42)=0,"",SUMIFS(국내SCHD형_분배!$D$2:$D$357,국내SCHD형_분배!$A$2:$A$357,"446720",국내SCHD형_분배!$C$2:$C$357,"&gt;="&amp;$B42,국내SCHD형_분배!$C$2:$C$357,"&lt;="&amp;$C42))</f>
+        <f>IF(COUNTIFS(국내SCHD형_분배!$A$2:$A$359,"446720",국내SCHD형_분배!$C$2:$C$359,"&gt;="&amp;$B42,국내SCHD형_분배!$C$2:$C$359,"&lt;="&amp;$C42)=0,"",SUMIFS(국내SCHD형_분배!$D$2:$D$359,국내SCHD형_분배!$A$2:$A$359,"446720",국내SCHD형_분배!$C$2:$C$359,"&gt;="&amp;$B42,국내SCHD형_분배!$C$2:$C$359,"&lt;="&amp;$C42))</f>
         <v/>
       </c>
       <c r="F42" s="53">
-        <f>IF(COUNTIFS(국내SCHD형_분배!$A$2:$A$357,"402970",국내SCHD형_분배!$C$2:$C$357,"&gt;="&amp;$B42,국내SCHD형_분배!$C$2:$C$357,"&lt;="&amp;$C42)=0,"",SUMIFS(국내SCHD형_분배!$D$2:$D$357,국내SCHD형_분배!$A$2:$A$357,"402970",국내SCHD형_분배!$C$2:$C$357,"&gt;="&amp;$B42,국내SCHD형_분배!$C$2:$C$357,"&lt;="&amp;$C42))</f>
+        <f>IF(COUNTIFS(국내SCHD형_분배!$A$2:$A$359,"402970",국내SCHD형_분배!$C$2:$C$359,"&gt;="&amp;$B42,국내SCHD형_분배!$C$2:$C$359,"&lt;="&amp;$C42)=0,"",SUMIFS(국내SCHD형_분배!$D$2:$D$359,국내SCHD형_분배!$A$2:$A$359,"402970",국내SCHD형_분배!$C$2:$C$359,"&gt;="&amp;$B42,국내SCHD형_분배!$C$2:$C$359,"&lt;="&amp;$C42))</f>
         <v/>
       </c>
       <c r="G42" s="53">
-        <f>IF(COUNTIFS(국내SCHD형_분배!$A$2:$A$357,"489250",국내SCHD형_분배!$C$2:$C$357,"&gt;="&amp;$B42,국내SCHD형_분배!$C$2:$C$357,"&lt;="&amp;$C42)=0,"",SUMIFS(국내SCHD형_분배!$D$2:$D$357,국내SCHD형_분배!$A$2:$A$357,"489250",국내SCHD형_분배!$C$2:$C$357,"&gt;="&amp;$B42,국내SCHD형_분배!$C$2:$C$357,"&lt;="&amp;$C42))</f>
+        <f>IF(COUNTIFS(국내SCHD형_분배!$A$2:$A$359,"489250",국내SCHD형_분배!$C$2:$C$359,"&gt;="&amp;$B42,국내SCHD형_분배!$C$2:$C$359,"&lt;="&amp;$C42)=0,"",SUMIFS(국내SCHD형_분배!$D$2:$D$359,국내SCHD형_분배!$A$2:$A$359,"489250",국내SCHD형_분배!$C$2:$C$359,"&gt;="&amp;$B42,국내SCHD형_분배!$C$2:$C$359,"&lt;="&amp;$C42))</f>
         <v/>
       </c>
       <c r="H42" s="28">
@@ -26151,19 +26193,19 @@
         <v/>
       </c>
       <c r="D43" s="53">
-        <f>IF(COUNTIFS(국내SCHD형_분배!$A$2:$A$357,"458730",국내SCHD형_분배!$C$2:$C$357,"&gt;="&amp;$B43,국내SCHD형_분배!$C$2:$C$357,"&lt;="&amp;$C43)=0,"",SUMIFS(국내SCHD형_분배!$D$2:$D$357,국내SCHD형_분배!$A$2:$A$357,"458730",국내SCHD형_분배!$C$2:$C$357,"&gt;="&amp;$B43,국내SCHD형_분배!$C$2:$C$357,"&lt;="&amp;$C43))</f>
+        <f>IF(COUNTIFS(국내SCHD형_분배!$A$2:$A$359,"458730",국내SCHD형_분배!$C$2:$C$359,"&gt;="&amp;$B43,국내SCHD형_분배!$C$2:$C$359,"&lt;="&amp;$C43)=0,"",SUMIFS(국내SCHD형_분배!$D$2:$D$359,국내SCHD형_분배!$A$2:$A$359,"458730",국내SCHD형_분배!$C$2:$C$359,"&gt;="&amp;$B43,국내SCHD형_분배!$C$2:$C$359,"&lt;="&amp;$C43))</f>
         <v/>
       </c>
       <c r="E43" s="53">
-        <f>IF(COUNTIFS(국내SCHD형_분배!$A$2:$A$357,"446720",국내SCHD형_분배!$C$2:$C$357,"&gt;="&amp;$B43,국내SCHD형_분배!$C$2:$C$357,"&lt;="&amp;$C43)=0,"",SUMIFS(국내SCHD형_분배!$D$2:$D$357,국내SCHD형_분배!$A$2:$A$357,"446720",국내SCHD형_분배!$C$2:$C$357,"&gt;="&amp;$B43,국내SCHD형_분배!$C$2:$C$357,"&lt;="&amp;$C43))</f>
+        <f>IF(COUNTIFS(국내SCHD형_분배!$A$2:$A$359,"446720",국내SCHD형_분배!$C$2:$C$359,"&gt;="&amp;$B43,국내SCHD형_분배!$C$2:$C$359,"&lt;="&amp;$C43)=0,"",SUMIFS(국내SCHD형_분배!$D$2:$D$359,국내SCHD형_분배!$A$2:$A$359,"446720",국내SCHD형_분배!$C$2:$C$359,"&gt;="&amp;$B43,국내SCHD형_분배!$C$2:$C$359,"&lt;="&amp;$C43))</f>
         <v/>
       </c>
       <c r="F43" s="53">
-        <f>IF(COUNTIFS(국내SCHD형_분배!$A$2:$A$357,"402970",국내SCHD형_분배!$C$2:$C$357,"&gt;="&amp;$B43,국내SCHD형_분배!$C$2:$C$357,"&lt;="&amp;$C43)=0,"",SUMIFS(국내SCHD형_분배!$D$2:$D$357,국내SCHD형_분배!$A$2:$A$357,"402970",국내SCHD형_분배!$C$2:$C$357,"&gt;="&amp;$B43,국내SCHD형_분배!$C$2:$C$357,"&lt;="&amp;$C43))</f>
+        <f>IF(COUNTIFS(국내SCHD형_분배!$A$2:$A$359,"402970",국내SCHD형_분배!$C$2:$C$359,"&gt;="&amp;$B43,국내SCHD형_분배!$C$2:$C$359,"&lt;="&amp;$C43)=0,"",SUMIFS(국내SCHD형_분배!$D$2:$D$359,국내SCHD형_분배!$A$2:$A$359,"402970",국내SCHD형_분배!$C$2:$C$359,"&gt;="&amp;$B43,국내SCHD형_분배!$C$2:$C$359,"&lt;="&amp;$C43))</f>
         <v/>
       </c>
       <c r="G43" s="53">
-        <f>IF(COUNTIFS(국내SCHD형_분배!$A$2:$A$357,"489250",국내SCHD형_분배!$C$2:$C$357,"&gt;="&amp;$B43,국내SCHD형_분배!$C$2:$C$357,"&lt;="&amp;$C43)=0,"",SUMIFS(국내SCHD형_분배!$D$2:$D$357,국내SCHD형_분배!$A$2:$A$357,"489250",국내SCHD형_분배!$C$2:$C$357,"&gt;="&amp;$B43,국내SCHD형_분배!$C$2:$C$357,"&lt;="&amp;$C43))</f>
+        <f>IF(COUNTIFS(국내SCHD형_분배!$A$2:$A$359,"489250",국내SCHD형_분배!$C$2:$C$359,"&gt;="&amp;$B43,국내SCHD형_분배!$C$2:$C$359,"&lt;="&amp;$C43)=0,"",SUMIFS(국내SCHD형_분배!$D$2:$D$359,국내SCHD형_분배!$A$2:$A$359,"489250",국내SCHD형_분배!$C$2:$C$359,"&gt;="&amp;$B43,국내SCHD형_분배!$C$2:$C$359,"&lt;="&amp;$C43))</f>
         <v/>
       </c>
       <c r="H43" s="28">
@@ -26189,19 +26231,19 @@
         <v/>
       </c>
       <c r="D44" s="53">
-        <f>IF(COUNTIFS(국내SCHD형_분배!$A$2:$A$357,"458730",국내SCHD형_분배!$C$2:$C$357,"&gt;="&amp;$B44,국내SCHD형_분배!$C$2:$C$357,"&lt;="&amp;$C44)=0,"",SUMIFS(국내SCHD형_분배!$D$2:$D$357,국내SCHD형_분배!$A$2:$A$357,"458730",국내SCHD형_분배!$C$2:$C$357,"&gt;="&amp;$B44,국내SCHD형_분배!$C$2:$C$357,"&lt;="&amp;$C44))</f>
+        <f>IF(COUNTIFS(국내SCHD형_분배!$A$2:$A$359,"458730",국내SCHD형_분배!$C$2:$C$359,"&gt;="&amp;$B44,국내SCHD형_분배!$C$2:$C$359,"&lt;="&amp;$C44)=0,"",SUMIFS(국내SCHD형_분배!$D$2:$D$359,국내SCHD형_분배!$A$2:$A$359,"458730",국내SCHD형_분배!$C$2:$C$359,"&gt;="&amp;$B44,국내SCHD형_분배!$C$2:$C$359,"&lt;="&amp;$C44))</f>
         <v/>
       </c>
       <c r="E44" s="53">
-        <f>IF(COUNTIFS(국내SCHD형_분배!$A$2:$A$357,"446720",국내SCHD형_분배!$C$2:$C$357,"&gt;="&amp;$B44,국내SCHD형_분배!$C$2:$C$357,"&lt;="&amp;$C44)=0,"",SUMIFS(국내SCHD형_분배!$D$2:$D$357,국내SCHD형_분배!$A$2:$A$357,"446720",국내SCHD형_분배!$C$2:$C$357,"&gt;="&amp;$B44,국내SCHD형_분배!$C$2:$C$357,"&lt;="&amp;$C44))</f>
+        <f>IF(COUNTIFS(국내SCHD형_분배!$A$2:$A$359,"446720",국내SCHD형_분배!$C$2:$C$359,"&gt;="&amp;$B44,국내SCHD형_분배!$C$2:$C$359,"&lt;="&amp;$C44)=0,"",SUMIFS(국내SCHD형_분배!$D$2:$D$359,국내SCHD형_분배!$A$2:$A$359,"446720",국내SCHD형_분배!$C$2:$C$359,"&gt;="&amp;$B44,국내SCHD형_분배!$C$2:$C$359,"&lt;="&amp;$C44))</f>
         <v/>
       </c>
       <c r="F44" s="53">
-        <f>IF(COUNTIFS(국내SCHD형_분배!$A$2:$A$357,"402970",국내SCHD형_분배!$C$2:$C$357,"&gt;="&amp;$B44,국내SCHD형_분배!$C$2:$C$357,"&lt;="&amp;$C44)=0,"",SUMIFS(국내SCHD형_분배!$D$2:$D$357,국내SCHD형_분배!$A$2:$A$357,"402970",국내SCHD형_분배!$C$2:$C$357,"&gt;="&amp;$B44,국내SCHD형_분배!$C$2:$C$357,"&lt;="&amp;$C44))</f>
+        <f>IF(COUNTIFS(국내SCHD형_분배!$A$2:$A$359,"402970",국내SCHD형_분배!$C$2:$C$359,"&gt;="&amp;$B44,국내SCHD형_분배!$C$2:$C$359,"&lt;="&amp;$C44)=0,"",SUMIFS(국내SCHD형_분배!$D$2:$D$359,국내SCHD형_분배!$A$2:$A$359,"402970",국내SCHD형_분배!$C$2:$C$359,"&gt;="&amp;$B44,국내SCHD형_분배!$C$2:$C$359,"&lt;="&amp;$C44))</f>
         <v/>
       </c>
       <c r="G44" s="53">
-        <f>IF(COUNTIFS(국내SCHD형_분배!$A$2:$A$357,"489250",국내SCHD형_분배!$C$2:$C$357,"&gt;="&amp;$B44,국내SCHD형_분배!$C$2:$C$357,"&lt;="&amp;$C44)=0,"",SUMIFS(국내SCHD형_분배!$D$2:$D$357,국내SCHD형_분배!$A$2:$A$357,"489250",국내SCHD형_분배!$C$2:$C$357,"&gt;="&amp;$B44,국내SCHD형_분배!$C$2:$C$357,"&lt;="&amp;$C44))</f>
+        <f>IF(COUNTIFS(국내SCHD형_분배!$A$2:$A$359,"489250",국내SCHD형_분배!$C$2:$C$359,"&gt;="&amp;$B44,국내SCHD형_분배!$C$2:$C$359,"&lt;="&amp;$C44)=0,"",SUMIFS(국내SCHD형_분배!$D$2:$D$359,국내SCHD형_분배!$A$2:$A$359,"489250",국내SCHD형_분배!$C$2:$C$359,"&gt;="&amp;$B44,국내SCHD형_분배!$C$2:$C$359,"&lt;="&amp;$C44))</f>
         <v/>
       </c>
       <c r="H44" s="28">
@@ -26257,11 +26299,11 @@
         </is>
       </c>
       <c r="B2" s="49" t="n">
-        <v>46322</v>
+        <v>46323</v>
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>← 이 날 종가로 계산한 비중. 그날 공식 파일을 못 받아 Schwab 공식 보유종목 CSV(2026-10-26)의 보유 주식 수 × 종가로 계산했습니다.</t>
+          <t>← 이 날 종가로 계산한 비중. 그날 공식 파일을 못 받아 Schwab 공식 보유종목 CSV(2026-10-27)의 보유 주식 수 × 종가로 계산했습니다.</t>
         </is>
       </c>
     </row>
@@ -26358,7 +26400,7 @@
         </is>
       </c>
       <c r="I5" s="61" t="n">
-        <v>0.04804111</v>
+        <v>0.048266</v>
       </c>
       <c r="J5" s="6" t="inlineStr">
         <is>
@@ -26412,25 +26454,25 @@
       </c>
       <c r="H6" s="6" t="inlineStr">
         <is>
-          <t>QCOM</t>
+          <t>COP</t>
         </is>
       </c>
       <c r="I6" s="61" t="n">
-        <v>0.04293930999999999</v>
+        <v>0.04306968999999999</v>
       </c>
       <c r="J6" s="6" t="inlineStr">
         <is>
-          <t>QUALCOMM</t>
+          <t>CONOCOPHILLIPS</t>
         </is>
       </c>
       <c r="K6" s="6" t="inlineStr">
         <is>
-          <t>Information Technology</t>
+          <t>Energy</t>
         </is>
       </c>
       <c r="L6" s="6" t="inlineStr">
         <is>
-          <t>퀄컴</t>
+          <t>코노코필립스</t>
         </is>
       </c>
       <c r="M6" s="7">
@@ -26470,25 +26512,25 @@
       </c>
       <c r="H7" s="6" t="inlineStr">
         <is>
-          <t>PG</t>
+          <t>CVX</t>
         </is>
       </c>
       <c r="I7" s="61" t="n">
-        <v>0.04273715</v>
+        <v>0.04295792</v>
       </c>
       <c r="J7" s="6" t="inlineStr">
         <is>
-          <t>PROCTER &amp; GAMBLE</t>
+          <t>CHEVRON</t>
         </is>
       </c>
       <c r="K7" s="6" t="inlineStr">
         <is>
-          <t>Consumer Staples</t>
+          <t>Energy</t>
         </is>
       </c>
       <c r="L7" s="6" t="inlineStr">
         <is>
-          <t>프록터앤드갬블</t>
+          <t>셰브론</t>
         </is>
       </c>
       <c r="M7" s="7">
@@ -26528,25 +26570,25 @@
       </c>
       <c r="H8" s="6" t="inlineStr">
         <is>
-          <t>CVX</t>
+          <t>QCOM</t>
         </is>
       </c>
       <c r="I8" s="61" t="n">
-        <v>0.04270364</v>
+        <v>0.04273199</v>
       </c>
       <c r="J8" s="6" t="inlineStr">
         <is>
-          <t>CHEVRON</t>
+          <t>QUALCOMM</t>
         </is>
       </c>
       <c r="K8" s="6" t="inlineStr">
         <is>
-          <t>Energy</t>
+          <t>Information Technology</t>
         </is>
       </c>
       <c r="L8" s="6" t="inlineStr">
         <is>
-          <t>셰브론</t>
+          <t>퀄컴</t>
         </is>
       </c>
       <c r="M8" s="7">
@@ -26586,25 +26628,25 @@
       </c>
       <c r="H9" s="6" t="inlineStr">
         <is>
-          <t>COP</t>
+          <t>PG</t>
         </is>
       </c>
       <c r="I9" s="61" t="n">
-        <v>0.04267935</v>
+        <v>0.04254898</v>
       </c>
       <c r="J9" s="6" t="inlineStr">
         <is>
-          <t>CONOCOPHILLIPS</t>
+          <t>PROCTER &amp; GAMBLE</t>
         </is>
       </c>
       <c r="K9" s="6" t="inlineStr">
         <is>
-          <t>Energy</t>
+          <t>Consumer Staples</t>
         </is>
       </c>
       <c r="L9" s="6" t="inlineStr">
         <is>
-          <t>코노코필립스</t>
+          <t>프록터앤드갬블</t>
         </is>
       </c>
       <c r="M9" s="7">
@@ -26648,7 +26690,7 @@
         </is>
       </c>
       <c r="I10" s="61" t="n">
-        <v>0.04094653</v>
+        <v>0.0412635</v>
       </c>
       <c r="J10" s="6" t="inlineStr">
         <is>
@@ -26702,15 +26744,15 @@
       </c>
       <c r="H11" s="6" t="inlineStr">
         <is>
-          <t>UNH</t>
+          <t>AMGN</t>
         </is>
       </c>
       <c r="I11" s="61" t="n">
-        <v>0.04068892</v>
+        <v>0.04049768</v>
       </c>
       <c r="J11" s="6" t="inlineStr">
         <is>
-          <t>UNITEDHEALTH GROUP</t>
+          <t>AMGEN INC</t>
         </is>
       </c>
       <c r="K11" s="6" t="inlineStr">
@@ -26720,7 +26762,7 @@
       </c>
       <c r="L11" s="6" t="inlineStr">
         <is>
-          <t>유나이티드헬스</t>
+          <t>암젠</t>
         </is>
       </c>
       <c r="M11" s="7">
@@ -26760,15 +26802,15 @@
       </c>
       <c r="H12" s="6" t="inlineStr">
         <is>
-          <t>AMGN</t>
+          <t>UNH</t>
         </is>
       </c>
       <c r="I12" s="61" t="n">
-        <v>0.04008198</v>
+        <v>0.04043118</v>
       </c>
       <c r="J12" s="6" t="inlineStr">
         <is>
-          <t>AMGEN INC</t>
+          <t>UNITEDHEALTH GROUP</t>
         </is>
       </c>
       <c r="K12" s="6" t="inlineStr">
@@ -26778,7 +26820,7 @@
       </c>
       <c r="L12" s="6" t="inlineStr">
         <is>
-          <t>암젠</t>
+          <t>유나이티드헬스</t>
         </is>
       </c>
       <c r="M12" s="7">
@@ -26822,7 +26864,7 @@
         </is>
       </c>
       <c r="I13" s="61" t="n">
-        <v>0.03962369</v>
+        <v>0.03957373</v>
       </c>
       <c r="J13" s="6" t="inlineStr">
         <is>
@@ -26880,7 +26922,7 @@
         </is>
       </c>
       <c r="I14" s="61" t="n">
-        <v>0.03764625</v>
+        <v>0.03746441</v>
       </c>
       <c r="J14" s="6" t="inlineStr">
         <is>
@@ -26928,7 +26970,7 @@
         </is>
       </c>
       <c r="I15" s="61" t="n">
-        <v>0.03705987</v>
+        <v>0.03688982</v>
       </c>
       <c r="J15" s="6" t="inlineStr">
         <is>
@@ -26976,7 +27018,7 @@
         </is>
       </c>
       <c r="I16" s="61" t="n">
-        <v>0.03698267</v>
+        <v>0.03688022</v>
       </c>
       <c r="J16" s="6" t="inlineStr">
         <is>
@@ -27010,25 +27052,25 @@
       </c>
       <c r="H17" s="6" t="inlineStr">
         <is>
-          <t>VZ</t>
+          <t>ACN</t>
         </is>
       </c>
       <c r="I17" s="61" t="n">
-        <v>0.03466334</v>
+        <v>0.03582394</v>
       </c>
       <c r="J17" s="6" t="inlineStr">
         <is>
-          <t>VERIZON COMMUNICATIONS INC</t>
+          <t>ACCENTURE PLC CLASS A</t>
         </is>
       </c>
       <c r="K17" s="6" t="inlineStr">
         <is>
-          <t>Communication Services</t>
+          <t>Information Technology</t>
         </is>
       </c>
       <c r="L17" s="6" t="inlineStr">
         <is>
-          <t>버라이즌</t>
+          <t>액센츄어</t>
         </is>
       </c>
       <c r="M17" s="7">
@@ -27048,25 +27090,25 @@
       </c>
       <c r="H18" s="6" t="inlineStr">
         <is>
-          <t>ACN</t>
+          <t>VZ</t>
         </is>
       </c>
       <c r="I18" s="61" t="n">
-        <v>0.03455249</v>
+        <v>0.03412945</v>
       </c>
       <c r="J18" s="6" t="inlineStr">
         <is>
-          <t>ACCENTURE PLC CLASS A</t>
+          <t>VERIZON COMMUNICATIONS INC</t>
         </is>
       </c>
       <c r="K18" s="6" t="inlineStr">
         <is>
-          <t>Information Technology</t>
+          <t>Communication Services</t>
         </is>
       </c>
       <c r="L18" s="6" t="inlineStr">
         <is>
-          <t>액센츄어</t>
+          <t>버라이즌</t>
         </is>
       </c>
       <c r="M18" s="7">
@@ -27081,7 +27123,7 @@
         </is>
       </c>
       <c r="I19" s="61" t="n">
-        <v>0.03037897</v>
+        <v>0.03076066</v>
       </c>
       <c r="J19" s="6" t="inlineStr">
         <is>
@@ -27115,7 +27157,7 @@
         </is>
       </c>
       <c r="I20" s="61" t="n">
-        <v>0.03018884</v>
+        <v>0.02975866</v>
       </c>
       <c r="J20" s="6" t="inlineStr">
         <is>
@@ -27154,7 +27196,7 @@
         </is>
       </c>
       <c r="I21" s="61" t="n">
-        <v>0.02946372</v>
+        <v>0.02931298</v>
       </c>
       <c r="J21" s="6" t="inlineStr">
         <is>
@@ -27192,7 +27234,7 @@
         </is>
       </c>
       <c r="I22" s="61" t="n">
-        <v>0.02795858</v>
+        <v>0.02726654</v>
       </c>
       <c r="J22" s="6" t="inlineStr">
         <is>
@@ -27230,7 +27272,7 @@
         </is>
       </c>
       <c r="I23" s="61" t="n">
-        <v>0.02103275</v>
+        <v>0.02113345</v>
       </c>
       <c r="J23" s="6" t="inlineStr">
         <is>
@@ -27268,7 +27310,7 @@
         </is>
       </c>
       <c r="I24" s="61" t="n">
-        <v>0.0202892</v>
+        <v>0.02030092</v>
       </c>
       <c r="J24" s="6" t="inlineStr">
         <is>
@@ -27306,7 +27348,7 @@
         </is>
       </c>
       <c r="I25" s="61" t="n">
-        <v>0.01927179</v>
+        <v>0.01918674</v>
       </c>
       <c r="J25" s="6" t="inlineStr">
         <is>
@@ -27344,7 +27386,7 @@
         </is>
       </c>
       <c r="I26" s="61" t="n">
-        <v>0.01908826</v>
+        <v>0.01903599</v>
       </c>
       <c r="J26" s="6" t="inlineStr">
         <is>
@@ -27382,7 +27424,7 @@
         </is>
       </c>
       <c r="I27" s="61" t="n">
-        <v>0.01855952</v>
+        <v>0.01836122</v>
       </c>
       <c r="J27" s="6" t="inlineStr">
         <is>
@@ -27420,7 +27462,7 @@
         </is>
       </c>
       <c r="I28" s="61" t="n">
-        <v>0.01614128</v>
+        <v>0.01627249</v>
       </c>
       <c r="J28" s="6" t="inlineStr">
         <is>
@@ -27458,7 +27500,7 @@
         </is>
       </c>
       <c r="I29" s="61" t="n">
-        <v>0.01453181</v>
+        <v>0.01433363</v>
       </c>
       <c r="J29" s="6" t="inlineStr">
         <is>
@@ -27492,7 +27534,7 @@
         </is>
       </c>
       <c r="I30" s="61" t="n">
-        <v>0.01420322</v>
+        <v>0.01419975</v>
       </c>
       <c r="J30" s="6" t="inlineStr">
         <is>
@@ -27530,7 +27572,7 @@
         </is>
       </c>
       <c r="I31" s="61" t="n">
-        <v>0.01353078</v>
+        <v>0.01356434</v>
       </c>
       <c r="J31" s="6" t="inlineStr">
         <is>
@@ -27555,7 +27597,7 @@
         </is>
       </c>
       <c r="I32" s="61" t="n">
-        <v>0.01166936</v>
+        <v>0.011663</v>
       </c>
       <c r="J32" s="6" t="inlineStr">
         <is>
@@ -27585,7 +27627,7 @@
         </is>
       </c>
       <c r="I33" s="61" t="n">
-        <v>0.01101267</v>
+        <v>0.01125747</v>
       </c>
       <c r="J33" s="6" t="inlineStr">
         <is>
@@ -27610,7 +27652,7 @@
         </is>
       </c>
       <c r="I34" s="61" t="n">
-        <v>0.00904929</v>
+        <v>0.0089522</v>
       </c>
       <c r="J34" s="6" t="inlineStr">
         <is>
@@ -27635,7 +27677,7 @@
         </is>
       </c>
       <c r="I35" s="61" t="n">
-        <v>0.008711719999999999</v>
+        <v>0.008670489999999999</v>
       </c>
       <c r="J35" s="6" t="inlineStr">
         <is>
@@ -27660,7 +27702,7 @@
         </is>
       </c>
       <c r="I36" s="61" t="n">
-        <v>0.008397659999999999</v>
+        <v>0.00833105</v>
       </c>
       <c r="J36" s="6" t="inlineStr">
         <is>
@@ -27681,15 +27723,15 @@
     <row r="37">
       <c r="H37" s="6" t="inlineStr">
         <is>
-          <t>CINF</t>
+          <t>ARES</t>
         </is>
       </c>
       <c r="I37" s="61" t="n">
-        <v>0.00668471</v>
+        <v>0.00666956</v>
       </c>
       <c r="J37" s="6" t="inlineStr">
         <is>
-          <t>CINCINNATI FINANCIAL</t>
+          <t>ARES MANAGEMENT CLASS A</t>
         </is>
       </c>
       <c r="K37" s="6" t="inlineStr">
@@ -27706,15 +27748,15 @@
     <row r="38">
       <c r="H38" s="6" t="inlineStr">
         <is>
-          <t>ARES</t>
+          <t>CINF</t>
         </is>
       </c>
       <c r="I38" s="61" t="n">
-        <v>0.006570599999999999</v>
+        <v>0.00662146</v>
       </c>
       <c r="J38" s="6" t="inlineStr">
         <is>
-          <t>ARES MANAGEMENT CLASS A</t>
+          <t>CINCINNATI FINANCIAL</t>
         </is>
       </c>
       <c r="K38" s="6" t="inlineStr">
@@ -27735,7 +27777,7 @@
         </is>
       </c>
       <c r="I39" s="61" t="n">
-        <v>0.00583219</v>
+        <v>0.00591301</v>
       </c>
       <c r="J39" s="6" t="inlineStr">
         <is>
@@ -27760,7 +27802,7 @@
         </is>
       </c>
       <c r="I40" s="61" t="n">
-        <v>0.005829879999999999</v>
+        <v>0.00581724</v>
       </c>
       <c r="J40" s="6" t="inlineStr">
         <is>
@@ -27785,7 +27827,7 @@
         </is>
       </c>
       <c r="I41" s="61" t="n">
-        <v>0.005778910000000001</v>
+        <v>0.00576264</v>
       </c>
       <c r="J41" s="6" t="inlineStr">
         <is>
@@ -27810,7 +27852,7 @@
         </is>
       </c>
       <c r="I42" s="61" t="n">
-        <v>0.00530752</v>
+        <v>0.005335490000000001</v>
       </c>
       <c r="J42" s="6" t="inlineStr">
         <is>
@@ -27835,7 +27877,7 @@
         </is>
       </c>
       <c r="I43" s="61" t="n">
-        <v>0.00523831</v>
+        <v>0.005240590000000001</v>
       </c>
       <c r="J43" s="6" t="inlineStr">
         <is>
@@ -27860,7 +27902,7 @@
         </is>
       </c>
       <c r="I44" s="61" t="n">
-        <v>0.00484885</v>
+        <v>0.00485371</v>
       </c>
       <c r="J44" s="6" t="inlineStr">
         <is>
@@ -27885,7 +27927,7 @@
         </is>
       </c>
       <c r="I45" s="61" t="n">
-        <v>0.00468315</v>
+        <v>0.00461775</v>
       </c>
       <c r="J45" s="6" t="inlineStr">
         <is>
@@ -27910,7 +27952,7 @@
         </is>
       </c>
       <c r="I46" s="61" t="n">
-        <v>0.00443953</v>
+        <v>0.00442342</v>
       </c>
       <c r="J46" s="6" t="inlineStr">
         <is>
@@ -27935,7 +27977,7 @@
         </is>
       </c>
       <c r="I47" s="61" t="n">
-        <v>0.00432334</v>
+        <v>0.00432635</v>
       </c>
       <c r="J47" s="6" t="inlineStr">
         <is>
@@ -27956,20 +27998,20 @@
     <row r="48">
       <c r="H48" s="6" t="inlineStr">
         <is>
-          <t>GIS</t>
+          <t>APA</t>
         </is>
       </c>
       <c r="I48" s="61" t="n">
-        <v>0.0042973</v>
+        <v>0.00430674</v>
       </c>
       <c r="J48" s="6" t="inlineStr">
         <is>
-          <t>GENERAL MILLS INC</t>
+          <t>APA</t>
         </is>
       </c>
       <c r="K48" s="6" t="inlineStr">
         <is>
-          <t>Consumer Staples</t>
+          <t>Energy</t>
         </is>
       </c>
       <c r="L48" s="6" t="inlineStr"/>
@@ -27981,20 +28023,20 @@
     <row r="49">
       <c r="H49" s="6" t="inlineStr">
         <is>
-          <t>APA</t>
+          <t>GIS</t>
         </is>
       </c>
       <c r="I49" s="61" t="n">
-        <v>0.00427252</v>
+        <v>0.00425057</v>
       </c>
       <c r="J49" s="6" t="inlineStr">
         <is>
-          <t>APA</t>
+          <t>GENERAL MILLS INC</t>
         </is>
       </c>
       <c r="K49" s="6" t="inlineStr">
         <is>
-          <t>Energy</t>
+          <t>Consumer Staples</t>
         </is>
       </c>
       <c r="L49" s="6" t="inlineStr"/>
@@ -28010,7 +28052,7 @@
         </is>
       </c>
       <c r="I50" s="61" t="n">
-        <v>0.00423965</v>
+        <v>0.00416319</v>
       </c>
       <c r="J50" s="6" t="inlineStr">
         <is>
@@ -28035,7 +28077,7 @@
         </is>
       </c>
       <c r="I51" s="61" t="n">
-        <v>0.00257137</v>
+        <v>0.00248823</v>
       </c>
       <c r="J51" s="6" t="inlineStr">
         <is>
@@ -28060,7 +28102,7 @@
         </is>
       </c>
       <c r="I52" s="61" t="n">
-        <v>0.00249799</v>
+        <v>0.00248447</v>
       </c>
       <c r="J52" s="6" t="inlineStr">
         <is>
@@ -28081,20 +28123,20 @@
     <row r="53">
       <c r="H53" s="6" t="inlineStr">
         <is>
-          <t>FNF</t>
+          <t>BAH</t>
         </is>
       </c>
       <c r="I53" s="61" t="n">
-        <v>0.00241145</v>
+        <v>0.00241355</v>
       </c>
       <c r="J53" s="6" t="inlineStr">
         <is>
-          <t>FIDELITY NATIONAL FINANCIAL INC</t>
+          <t>BOOZ ALLEN HAMILTON HOLDING CLASS</t>
         </is>
       </c>
       <c r="K53" s="6" t="inlineStr">
         <is>
-          <t>Financials</t>
+          <t>Industrials</t>
         </is>
       </c>
       <c r="L53" s="6" t="inlineStr"/>
@@ -28106,20 +28148,20 @@
     <row r="54">
       <c r="H54" s="6" t="inlineStr">
         <is>
-          <t>BAH</t>
+          <t>FNF</t>
         </is>
       </c>
       <c r="I54" s="61" t="n">
-        <v>0.00240717</v>
+        <v>0.00240637</v>
       </c>
       <c r="J54" s="6" t="inlineStr">
         <is>
-          <t>BOOZ ALLEN HAMILTON HOLDING CLASS</t>
+          <t>FIDELITY NATIONAL FINANCIAL INC</t>
         </is>
       </c>
       <c r="K54" s="6" t="inlineStr">
         <is>
-          <t>Industrials</t>
+          <t>Financials</t>
         </is>
       </c>
       <c r="L54" s="6" t="inlineStr"/>
@@ -28135,7 +28177,7 @@
         </is>
       </c>
       <c r="I55" s="61" t="n">
-        <v>0.0021063</v>
+        <v>0.00208811</v>
       </c>
       <c r="J55" s="6" t="inlineStr">
         <is>
@@ -28160,7 +28202,7 @@
         </is>
       </c>
       <c r="I56" s="61" t="n">
-        <v>0.00203109</v>
+        <v>0.00201477</v>
       </c>
       <c r="J56" s="6" t="inlineStr">
         <is>
@@ -28185,7 +28227,7 @@
         </is>
       </c>
       <c r="I57" s="61" t="n">
-        <v>0.00185553</v>
+        <v>0.00185147</v>
       </c>
       <c r="J57" s="6" t="inlineStr">
         <is>
@@ -28210,7 +28252,7 @@
         </is>
       </c>
       <c r="I58" s="61" t="n">
-        <v>0.00153118</v>
+        <v>0.00153062</v>
       </c>
       <c r="J58" s="6" t="inlineStr">
         <is>
@@ -28235,7 +28277,7 @@
         </is>
       </c>
       <c r="I59" s="61" t="n">
-        <v>0.00150548</v>
+        <v>0.00150044</v>
       </c>
       <c r="J59" s="6" t="inlineStr">
         <is>
@@ -28260,7 +28302,7 @@
         </is>
       </c>
       <c r="I60" s="61" t="n">
-        <v>0.00139764</v>
+        <v>0.00139481</v>
       </c>
       <c r="J60" s="6" t="inlineStr">
         <is>
@@ -28285,7 +28327,7 @@
         </is>
       </c>
       <c r="I61" s="61" t="n">
-        <v>0.00130215</v>
+        <v>0.00135074</v>
       </c>
       <c r="J61" s="6" t="inlineStr">
         <is>
@@ -28310,7 +28352,7 @@
         </is>
       </c>
       <c r="I62" s="61" t="n">
-        <v>0.00129564</v>
+        <v>0.00130196</v>
       </c>
       <c r="J62" s="6" t="inlineStr">
         <is>
@@ -28335,7 +28377,7 @@
         </is>
       </c>
       <c r="I63" s="61" t="n">
-        <v>0.00123781</v>
+        <v>0.00123355</v>
       </c>
       <c r="J63" s="6" t="inlineStr">
         <is>
@@ -28360,7 +28402,7 @@
         </is>
       </c>
       <c r="I64" s="61" t="n">
-        <v>0.00115746</v>
+        <v>0.00114714</v>
       </c>
       <c r="J64" s="6" t="inlineStr">
         <is>
@@ -28381,20 +28423,20 @@
     <row r="65">
       <c r="H65" s="6" t="inlineStr">
         <is>
-          <t>RHI</t>
+          <t>MC</t>
         </is>
       </c>
       <c r="I65" s="61" t="n">
-        <v>0.00101075</v>
+        <v>0.00103589</v>
       </c>
       <c r="J65" s="6" t="inlineStr">
         <is>
-          <t>ROBERT HALF INC</t>
+          <t>MOELIS CLASS A</t>
         </is>
       </c>
       <c r="K65" s="6" t="inlineStr">
         <is>
-          <t>Industrials</t>
+          <t>Financials</t>
         </is>
       </c>
       <c r="L65" s="6" t="inlineStr"/>
@@ -28406,20 +28448,20 @@
     <row r="66">
       <c r="H66" s="6" t="inlineStr">
         <is>
-          <t>MC</t>
+          <t>RHI</t>
         </is>
       </c>
       <c r="I66" s="61" t="n">
-        <v>0.00099121</v>
+        <v>0.00101029</v>
       </c>
       <c r="J66" s="6" t="inlineStr">
         <is>
-          <t>MOELIS CLASS A</t>
+          <t>ROBERT HALF INC</t>
         </is>
       </c>
       <c r="K66" s="6" t="inlineStr">
         <is>
-          <t>Financials</t>
+          <t>Industrials</t>
         </is>
       </c>
       <c r="L66" s="6" t="inlineStr"/>
@@ -28435,7 +28477,7 @@
         </is>
       </c>
       <c r="I67" s="61" t="n">
-        <v>0.0009637199999999999</v>
+        <v>0.00097339</v>
       </c>
       <c r="J67" s="6" t="inlineStr">
         <is>
@@ -28460,7 +28502,7 @@
         </is>
       </c>
       <c r="I68" s="61" t="n">
-        <v>0.00094911</v>
+        <v>0.00095216</v>
       </c>
       <c r="J68" s="6" t="inlineStr">
         <is>
@@ -28485,7 +28527,7 @@
         </is>
       </c>
       <c r="I69" s="61" t="n">
-        <v>0.00093986</v>
+        <v>0.00093041</v>
       </c>
       <c r="J69" s="6" t="inlineStr">
         <is>
@@ -28506,20 +28548,20 @@
     <row r="70">
       <c r="H70" s="6" t="inlineStr">
         <is>
-          <t>CVBF</t>
+          <t>PAG</t>
         </is>
       </c>
       <c r="I70" s="61" t="n">
-        <v>0.00091322</v>
+        <v>0.00090494</v>
       </c>
       <c r="J70" s="6" t="inlineStr">
         <is>
-          <t>CVB FINANCIAL CORP</t>
+          <t>PENSKE AUTOMOTIVE GROUP VOTING INC</t>
         </is>
       </c>
       <c r="K70" s="6" t="inlineStr">
         <is>
-          <t>Financials</t>
+          <t>Consumer Discretionary</t>
         </is>
       </c>
       <c r="L70" s="6" t="inlineStr"/>
@@ -28531,20 +28573,20 @@
     <row r="71">
       <c r="H71" s="6" t="inlineStr">
         <is>
-          <t>PAG</t>
+          <t>CVBF</t>
         </is>
       </c>
       <c r="I71" s="61" t="n">
-        <v>0.00090431</v>
+        <v>0.0009031400000000001</v>
       </c>
       <c r="J71" s="6" t="inlineStr">
         <is>
-          <t>PENSKE AUTOMOTIVE GROUP VOTING INC</t>
+          <t>CVB FINANCIAL CORP</t>
         </is>
       </c>
       <c r="K71" s="6" t="inlineStr">
         <is>
-          <t>Consumer Discretionary</t>
+          <t>Financials</t>
         </is>
       </c>
       <c r="L71" s="6" t="inlineStr"/>
@@ -28560,7 +28602,7 @@
         </is>
       </c>
       <c r="I72" s="61" t="n">
-        <v>0.00056335</v>
+        <v>0.0005903</v>
       </c>
       <c r="J72" s="6" t="inlineStr">
         <is>
@@ -28585,7 +28627,7 @@
         </is>
       </c>
       <c r="I73" s="61" t="n">
-        <v>0.0005627399999999999</v>
+        <v>0.00055848</v>
       </c>
       <c r="J73" s="6" t="inlineStr">
         <is>
@@ -28610,7 +28652,7 @@
         </is>
       </c>
       <c r="I74" s="61" t="n">
-        <v>0.00051742</v>
+        <v>0.00051614</v>
       </c>
       <c r="J74" s="6" t="inlineStr">
         <is>
@@ -28631,15 +28673,15 @@
     <row r="75">
       <c r="H75" s="6" t="inlineStr">
         <is>
-          <t>IPAR</t>
+          <t>MZTI</t>
         </is>
       </c>
       <c r="I75" s="61" t="n">
-        <v>0.0005049200000000001</v>
+        <v>0.00050795</v>
       </c>
       <c r="J75" s="6" t="inlineStr">
         <is>
-          <t>INTERPARFUMS INC</t>
+          <t>MARZETTI</t>
         </is>
       </c>
       <c r="K75" s="6" t="inlineStr">
@@ -28656,15 +28698,15 @@
     <row r="76">
       <c r="H76" s="6" t="inlineStr">
         <is>
-          <t>MZTI</t>
+          <t>IPAR</t>
         </is>
       </c>
       <c r="I76" s="61" t="n">
-        <v>0.00050434</v>
+        <v>0.00050156</v>
       </c>
       <c r="J76" s="6" t="inlineStr">
         <is>
-          <t>MARZETTI</t>
+          <t>INTERPARFUMS INC</t>
         </is>
       </c>
       <c r="K76" s="6" t="inlineStr">
@@ -28681,15 +28723,15 @@
     <row r="77">
       <c r="H77" s="6" t="inlineStr">
         <is>
-          <t>CNS</t>
+          <t>CHCO</t>
         </is>
       </c>
       <c r="I77" s="61" t="n">
-        <v>0.00048079</v>
+        <v>0.00048047</v>
       </c>
       <c r="J77" s="6" t="inlineStr">
         <is>
-          <t>COHEN &amp; STEERS INC</t>
+          <t>CITY HOLDING</t>
         </is>
       </c>
       <c r="K77" s="6" t="inlineStr">
@@ -28706,15 +28748,15 @@
     <row r="78">
       <c r="H78" s="6" t="inlineStr">
         <is>
-          <t>CHCO</t>
+          <t>CNS</t>
         </is>
       </c>
       <c r="I78" s="61" t="n">
-        <v>0.00047747</v>
+        <v>0.00047654</v>
       </c>
       <c r="J78" s="6" t="inlineStr">
         <is>
-          <t>CITY HOLDING</t>
+          <t>COHEN &amp; STEERS INC</t>
         </is>
       </c>
       <c r="K78" s="6" t="inlineStr">
@@ -28735,7 +28777,7 @@
         </is>
       </c>
       <c r="I79" s="61" t="n">
-        <v>0.00045739</v>
+        <v>0.00045831</v>
       </c>
       <c r="J79" s="6" t="inlineStr">
         <is>
@@ -28760,7 +28802,7 @@
         </is>
       </c>
       <c r="I80" s="61" t="n">
-        <v>0.00044976</v>
+        <v>0.00045805</v>
       </c>
       <c r="J80" s="6" t="inlineStr">
         <is>
@@ -28781,22 +28823,18 @@
     <row r="81">
       <c r="H81" s="6" t="inlineStr">
         <is>
-          <t>NSP</t>
+          <t>GVMXX</t>
         </is>
       </c>
       <c r="I81" s="61" t="n">
-        <v>0.00044523</v>
+        <v>0.00045189</v>
       </c>
       <c r="J81" s="6" t="inlineStr">
         <is>
-          <t>INSPERITY</t>
-        </is>
-      </c>
-      <c r="K81" s="6" t="inlineStr">
-        <is>
-          <t>Industrials</t>
-        </is>
-      </c>
+          <t>SSC GOVERNMENT MM GVMXX</t>
+        </is>
+      </c>
+      <c r="K81" s="6" t="inlineStr"/>
       <c r="L81" s="6" t="inlineStr"/>
       <c r="M81" s="7">
         <f>IF(H81="","",IFERROR(VLOOKUP(K81,$P$5:$Q$15,2,FALSE),"현금·선물"))</f>
@@ -28806,20 +28844,20 @@
     <row r="82">
       <c r="H82" s="6" t="inlineStr">
         <is>
-          <t>GABC</t>
+          <t>NSP</t>
         </is>
       </c>
       <c r="I82" s="61" t="n">
-        <v>0.00044491</v>
+        <v>0.00044478</v>
       </c>
       <c r="J82" s="6" t="inlineStr">
         <is>
-          <t>GERMAN AMERICAN BANCORP INC</t>
+          <t>INSPERITY</t>
         </is>
       </c>
       <c r="K82" s="6" t="inlineStr">
         <is>
-          <t>Financials</t>
+          <t>Industrials</t>
         </is>
       </c>
       <c r="L82" s="6" t="inlineStr"/>
@@ -28831,18 +28869,22 @@
     <row r="83">
       <c r="H83" s="6" t="inlineStr">
         <is>
-          <t>GVMXX</t>
+          <t>GABC</t>
         </is>
       </c>
       <c r="I83" s="61" t="n">
-        <v>0.00043978</v>
+        <v>0.00044338</v>
       </c>
       <c r="J83" s="6" t="inlineStr">
         <is>
-          <t>SSC GOVERNMENT MM GVMXX</t>
-        </is>
-      </c>
-      <c r="K83" s="6" t="inlineStr"/>
+          <t>GERMAN AMERICAN BANCORP INC</t>
+        </is>
+      </c>
+      <c r="K83" s="6" t="inlineStr">
+        <is>
+          <t>Financials</t>
+        </is>
+      </c>
       <c r="L83" s="6" t="inlineStr"/>
       <c r="M83" s="7">
         <f>IF(H83="","",IFERROR(VLOOKUP(K83,$P$5:$Q$15,2,FALSE),"현금·선물"))</f>
@@ -28856,7 +28898,7 @@
         </is>
       </c>
       <c r="I84" s="61" t="n">
-        <v>0.00042928</v>
+        <v>0.00042906</v>
       </c>
       <c r="J84" s="6" t="inlineStr">
         <is>
@@ -28881,7 +28923,7 @@
         </is>
       </c>
       <c r="I85" s="61" t="n">
-        <v>0.00041625</v>
+        <v>0.00040089</v>
       </c>
       <c r="J85" s="6" t="inlineStr">
         <is>
@@ -28906,7 +28948,7 @@
         </is>
       </c>
       <c r="I86" s="61" t="n">
-        <v>0.00037696</v>
+        <v>0.00037513</v>
       </c>
       <c r="J86" s="6" t="inlineStr">
         <is>
@@ -28931,7 +28973,7 @@
         </is>
       </c>
       <c r="I87" s="61" t="n">
-        <v>0.0003632</v>
+        <v>0.00036194</v>
       </c>
       <c r="J87" s="6" t="inlineStr">
         <is>
@@ -28956,7 +28998,7 @@
         </is>
       </c>
       <c r="I88" s="61" t="n">
-        <v>0.00034245</v>
+        <v>0.00033613</v>
       </c>
       <c r="J88" s="6" t="inlineStr">
         <is>
@@ -28981,7 +29023,7 @@
         </is>
       </c>
       <c r="I89" s="61" t="n">
-        <v>0.00031602</v>
+        <v>0.0003135</v>
       </c>
       <c r="J89" s="6" t="inlineStr">
         <is>
@@ -29006,7 +29048,7 @@
         </is>
       </c>
       <c r="I90" s="61" t="n">
-        <v>0.00027826</v>
+        <v>0.0002808</v>
       </c>
       <c r="J90" s="6" t="inlineStr">
         <is>
@@ -29027,20 +29069,20 @@
     <row r="91">
       <c r="H91" s="6" t="inlineStr">
         <is>
-          <t>CNA</t>
+          <t>WEN</t>
         </is>
       </c>
       <c r="I91" s="61" t="n">
-        <v>0.00025073</v>
+        <v>0.00027328</v>
       </c>
       <c r="J91" s="6" t="inlineStr">
         <is>
-          <t>CNA FINANCIAL CORP</t>
+          <t>WENDYS</t>
         </is>
       </c>
       <c r="K91" s="6" t="inlineStr">
         <is>
-          <t>Financials</t>
+          <t>Consumer Discretionary</t>
         </is>
       </c>
       <c r="L91" s="6" t="inlineStr"/>
@@ -29052,20 +29094,20 @@
     <row r="92">
       <c r="H92" s="6" t="inlineStr">
         <is>
-          <t>WEN</t>
+          <t>CNA</t>
         </is>
       </c>
       <c r="I92" s="61" t="n">
-        <v>0.00023693</v>
+        <v>0.00025016</v>
       </c>
       <c r="J92" s="6" t="inlineStr">
         <is>
-          <t>WENDYS</t>
+          <t>CNA FINANCIAL CORP</t>
         </is>
       </c>
       <c r="K92" s="6" t="inlineStr">
         <is>
-          <t>Consumer Discretionary</t>
+          <t>Financials</t>
         </is>
       </c>
       <c r="L92" s="6" t="inlineStr"/>
@@ -29081,7 +29123,7 @@
         </is>
       </c>
       <c r="I93" s="61" t="n">
-        <v>0.00023314</v>
+        <v>0.00023396</v>
       </c>
       <c r="J93" s="6" t="inlineStr">
         <is>
@@ -29106,7 +29148,7 @@
         </is>
       </c>
       <c r="I94" s="61" t="n">
-        <v>0.00022957</v>
+        <v>0.00023201</v>
       </c>
       <c r="J94" s="6" t="inlineStr">
         <is>
@@ -29131,7 +29173,7 @@
         </is>
       </c>
       <c r="I95" s="61" t="n">
-        <v>0.00021191</v>
+        <v>0.00021154</v>
       </c>
       <c r="J95" s="6" t="inlineStr">
         <is>
@@ -29152,15 +29194,15 @@
     <row r="96">
       <c r="H96" s="6" t="inlineStr">
         <is>
-          <t>THFF</t>
+          <t>IBCP</t>
         </is>
       </c>
       <c r="I96" s="61" t="n">
-        <v>0.0001993</v>
+        <v>0.00019759</v>
       </c>
       <c r="J96" s="6" t="inlineStr">
         <is>
-          <t>FIRST FINANCIAL CORPORATION CORP</t>
+          <t>INDEPENDENT BANK CORP</t>
         </is>
       </c>
       <c r="K96" s="6" t="inlineStr">
@@ -29177,15 +29219,15 @@
     <row r="97">
       <c r="H97" s="6" t="inlineStr">
         <is>
-          <t>IBCP</t>
+          <t>THFF</t>
         </is>
       </c>
       <c r="I97" s="61" t="n">
-        <v>0.00019839</v>
+        <v>0.00019718</v>
       </c>
       <c r="J97" s="6" t="inlineStr">
         <is>
-          <t>INDEPENDENT BANK CORP</t>
+          <t>FIRST FINANCIAL CORPORATION CORP</t>
         </is>
       </c>
       <c r="K97" s="6" t="inlineStr">
@@ -29206,7 +29248,7 @@
         </is>
       </c>
       <c r="I98" s="61" t="n">
-        <v>0.0001776</v>
+        <v>0.00018082</v>
       </c>
       <c r="J98" s="6" t="inlineStr">
         <is>
@@ -29231,7 +29273,7 @@
         </is>
       </c>
       <c r="I99" s="61" t="n">
-        <v>0.00016834</v>
+        <v>0.00016726</v>
       </c>
       <c r="J99" s="6" t="inlineStr">
         <is>
@@ -29256,7 +29298,7 @@
         </is>
       </c>
       <c r="I100" s="61" t="n">
-        <v>0.00014105</v>
+        <v>0.00013781</v>
       </c>
       <c r="J100" s="6" t="inlineStr">
         <is>
@@ -29277,7 +29319,7 @@
         </is>
       </c>
       <c r="I101" s="61" t="n">
-        <v>0.00012949</v>
+        <v>0.00012793</v>
       </c>
       <c r="J101" s="6" t="inlineStr">
         <is>
@@ -29302,7 +29344,7 @@
         </is>
       </c>
       <c r="I102" s="61" t="n">
-        <v>0.00011334</v>
+        <v>0.0001128</v>
       </c>
       <c r="J102" s="6" t="inlineStr">
         <is>
@@ -29327,7 +29369,7 @@
         </is>
       </c>
       <c r="I103" s="61" t="n">
-        <v>9.565000000000001e-05</v>
+        <v>9.331000000000001e-05</v>
       </c>
       <c r="J103" s="6" t="inlineStr">
         <is>
@@ -29352,7 +29394,7 @@
         </is>
       </c>
       <c r="I104" s="61" t="n">
-        <v>9.143e-05</v>
+        <v>9.083000000000001e-05</v>
       </c>
       <c r="J104" s="6" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
데이터 갱신: holdings (2026-10-30)
</commit_message>
<xml_diff>
--- a/downloads/schd_dividend_tracker.xlsx
+++ b/downloads/schd_dividend_tracker.xlsx
@@ -1724,7 +1724,7 @@
     <row r="3">
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>최종 갱신: 2026-10-29 · 반영 범위: 2012년 1분기 ~ 2026년 3분기 (배당락 2026-09-23) · GitHub Actions 자동 생성</t>
+          <t>최종 갱신: 2026-10-30 · 반영 범위: 2012년 1분기 ~ 2026년 3분기 (배당락 2026-09-23) · GitHub Actions 자동 생성</t>
         </is>
       </c>
     </row>
@@ -26299,11 +26299,11 @@
         </is>
       </c>
       <c r="B2" s="49" t="n">
-        <v>46323</v>
+        <v>46324</v>
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>← 이 날 종가로 계산한 비중. 그날 공식 파일을 못 받아 Schwab 공식 보유종목 CSV(2026-10-27)의 보유 주식 수 × 종가로 계산했습니다.</t>
+          <t>← 이 날 종가로 계산한 비중. 그날 공식 파일을 못 받아 Schwab 공식 보유종목 CSV(2026-10-28)의 보유 주식 수 × 종가로 계산했습니다.</t>
         </is>
       </c>
     </row>
@@ -26400,7 +26400,7 @@
         </is>
       </c>
       <c r="I5" s="61" t="n">
-        <v>0.048266</v>
+        <v>0.04795357</v>
       </c>
       <c r="J5" s="6" t="inlineStr">
         <is>
@@ -26454,15 +26454,15 @@
       </c>
       <c r="H6" s="6" t="inlineStr">
         <is>
-          <t>COP</t>
+          <t>CVX</t>
         </is>
       </c>
       <c r="I6" s="61" t="n">
-        <v>0.04306968999999999</v>
+        <v>0.04267233</v>
       </c>
       <c r="J6" s="6" t="inlineStr">
         <is>
-          <t>CONOCOPHILLIPS</t>
+          <t>CHEVRON</t>
         </is>
       </c>
       <c r="K6" s="6" t="inlineStr">
@@ -26472,7 +26472,7 @@
       </c>
       <c r="L6" s="6" t="inlineStr">
         <is>
-          <t>코노코필립스</t>
+          <t>셰브론</t>
         </is>
       </c>
       <c r="M6" s="7">
@@ -26512,15 +26512,15 @@
       </c>
       <c r="H7" s="6" t="inlineStr">
         <is>
-          <t>CVX</t>
+          <t>COP</t>
         </is>
       </c>
       <c r="I7" s="61" t="n">
-        <v>0.04295792</v>
+        <v>0.04264136</v>
       </c>
       <c r="J7" s="6" t="inlineStr">
         <is>
-          <t>CHEVRON</t>
+          <t>CONOCOPHILLIPS</t>
         </is>
       </c>
       <c r="K7" s="6" t="inlineStr">
@@ -26530,7 +26530,7 @@
       </c>
       <c r="L7" s="6" t="inlineStr">
         <is>
-          <t>셰브론</t>
+          <t>코노코필립스</t>
         </is>
       </c>
       <c r="M7" s="7">
@@ -26574,7 +26574,7 @@
         </is>
       </c>
       <c r="I8" s="61" t="n">
-        <v>0.04273199</v>
+        <v>0.04259401</v>
       </c>
       <c r="J8" s="6" t="inlineStr">
         <is>
@@ -26632,7 +26632,7 @@
         </is>
       </c>
       <c r="I9" s="61" t="n">
-        <v>0.04254898</v>
+        <v>0.04246965999999999</v>
       </c>
       <c r="J9" s="6" t="inlineStr">
         <is>
@@ -26690,7 +26690,7 @@
         </is>
       </c>
       <c r="I10" s="61" t="n">
-        <v>0.0412635</v>
+        <v>0.0410713</v>
       </c>
       <c r="J10" s="6" t="inlineStr">
         <is>
@@ -26748,7 +26748,7 @@
         </is>
       </c>
       <c r="I11" s="61" t="n">
-        <v>0.04049768</v>
+        <v>0.04062024</v>
       </c>
       <c r="J11" s="6" t="inlineStr">
         <is>
@@ -26802,25 +26802,25 @@
       </c>
       <c r="H12" s="6" t="inlineStr">
         <is>
-          <t>UNH</t>
+          <t>HD</t>
         </is>
       </c>
       <c r="I12" s="61" t="n">
-        <v>0.04043118</v>
+        <v>0.04032661</v>
       </c>
       <c r="J12" s="6" t="inlineStr">
         <is>
-          <t>UNITEDHEALTH GROUP</t>
+          <t>HOME DEPOT</t>
         </is>
       </c>
       <c r="K12" s="6" t="inlineStr">
         <is>
-          <t>Health Care</t>
+          <t>Consumer Discretionary</t>
         </is>
       </c>
       <c r="L12" s="6" t="inlineStr">
         <is>
-          <t>유나이티드헬스</t>
+          <t>홈디포</t>
         </is>
       </c>
       <c r="M12" s="7">
@@ -26860,25 +26860,25 @@
       </c>
       <c r="H13" s="6" t="inlineStr">
         <is>
-          <t>HD</t>
+          <t>UNH</t>
         </is>
       </c>
       <c r="I13" s="61" t="n">
-        <v>0.03957373</v>
+        <v>0.04014238</v>
       </c>
       <c r="J13" s="6" t="inlineStr">
         <is>
-          <t>HOME DEPOT</t>
+          <t>UNITEDHEALTH GROUP</t>
         </is>
       </c>
       <c r="K13" s="6" t="inlineStr">
         <is>
-          <t>Consumer Discretionary</t>
+          <t>Health Care</t>
         </is>
       </c>
       <c r="L13" s="6" t="inlineStr">
         <is>
-          <t>홈디포</t>
+          <t>유나이티드헬스</t>
         </is>
       </c>
       <c r="M13" s="7">
@@ -26918,25 +26918,25 @@
       </c>
       <c r="H14" s="6" t="inlineStr">
         <is>
-          <t>PEP</t>
+          <t>MRK</t>
         </is>
       </c>
       <c r="I14" s="61" t="n">
-        <v>0.03746441</v>
+        <v>0.03767718</v>
       </c>
       <c r="J14" s="6" t="inlineStr">
         <is>
-          <t>PEPSICO</t>
+          <t>MERCK &amp; CO INC</t>
         </is>
       </c>
       <c r="K14" s="6" t="inlineStr">
         <is>
-          <t>Consumer Staples</t>
+          <t>Health Care</t>
         </is>
       </c>
       <c r="L14" s="6" t="inlineStr">
         <is>
-          <t>펩시코</t>
+          <t>머크</t>
         </is>
       </c>
       <c r="M14" s="7">
@@ -26966,25 +26966,25 @@
       </c>
       <c r="H15" s="6" t="inlineStr">
         <is>
-          <t>MRK</t>
+          <t>PEP</t>
         </is>
       </c>
       <c r="I15" s="61" t="n">
-        <v>0.03688982</v>
+        <v>0.03717428</v>
       </c>
       <c r="J15" s="6" t="inlineStr">
         <is>
-          <t>MERCK &amp; CO INC</t>
+          <t>PEPSICO</t>
         </is>
       </c>
       <c r="K15" s="6" t="inlineStr">
         <is>
-          <t>Health Care</t>
+          <t>Consumer Staples</t>
         </is>
       </c>
       <c r="L15" s="6" t="inlineStr">
         <is>
-          <t>머크</t>
+          <t>펩시코</t>
         </is>
       </c>
       <c r="M15" s="7">
@@ -27018,7 +27018,7 @@
         </is>
       </c>
       <c r="I16" s="61" t="n">
-        <v>0.03688022</v>
+        <v>0.03695951</v>
       </c>
       <c r="J16" s="6" t="inlineStr">
         <is>
@@ -27056,7 +27056,7 @@
         </is>
       </c>
       <c r="I17" s="61" t="n">
-        <v>0.03582394</v>
+        <v>0.03579137</v>
       </c>
       <c r="J17" s="6" t="inlineStr">
         <is>
@@ -27094,7 +27094,7 @@
         </is>
       </c>
       <c r="I18" s="61" t="n">
-        <v>0.03412945</v>
+        <v>0.03394476</v>
       </c>
       <c r="J18" s="6" t="inlineStr">
         <is>
@@ -27123,7 +27123,7 @@
         </is>
       </c>
       <c r="I19" s="61" t="n">
-        <v>0.03076066</v>
+        <v>0.03092271</v>
       </c>
       <c r="J19" s="6" t="inlineStr">
         <is>
@@ -27153,25 +27153,25 @@
       </c>
       <c r="H20" s="6" t="inlineStr">
         <is>
-          <t>BMY</t>
+          <t>MO</t>
         </is>
       </c>
       <c r="I20" s="61" t="n">
-        <v>0.02975866</v>
+        <v>0.03031918</v>
       </c>
       <c r="J20" s="6" t="inlineStr">
         <is>
-          <t>BRISTOL MYERS SQUIBB</t>
+          <t>ALTRIA GROUP INC</t>
         </is>
       </c>
       <c r="K20" s="6" t="inlineStr">
         <is>
-          <t>Health Care</t>
+          <t>Consumer Staples</t>
         </is>
       </c>
       <c r="L20" s="6" t="inlineStr">
         <is>
-          <t>브리스톨마이어스스퀴브</t>
+          <t>알트리아</t>
         </is>
       </c>
       <c r="M20" s="7">
@@ -27192,25 +27192,25 @@
       </c>
       <c r="H21" s="6" t="inlineStr">
         <is>
-          <t>MO</t>
+          <t>BMY</t>
         </is>
       </c>
       <c r="I21" s="61" t="n">
-        <v>0.02931298</v>
+        <v>0.02966852</v>
       </c>
       <c r="J21" s="6" t="inlineStr">
         <is>
-          <t>ALTRIA GROUP INC</t>
+          <t>BRISTOL MYERS SQUIBB</t>
         </is>
       </c>
       <c r="K21" s="6" t="inlineStr">
         <is>
-          <t>Consumer Staples</t>
+          <t>Health Care</t>
         </is>
       </c>
       <c r="L21" s="6" t="inlineStr">
         <is>
-          <t>알트리아</t>
+          <t>브리스톨마이어스스퀴브</t>
         </is>
       </c>
       <c r="M21" s="7">
@@ -27234,7 +27234,7 @@
         </is>
       </c>
       <c r="I22" s="61" t="n">
-        <v>0.02726654</v>
+        <v>0.02688757</v>
       </c>
       <c r="J22" s="6" t="inlineStr">
         <is>
@@ -27272,7 +27272,7 @@
         </is>
       </c>
       <c r="I23" s="61" t="n">
-        <v>0.02113345</v>
+        <v>0.02141662</v>
       </c>
       <c r="J23" s="6" t="inlineStr">
         <is>
@@ -27310,7 +27310,7 @@
         </is>
       </c>
       <c r="I24" s="61" t="n">
-        <v>0.02030092</v>
+        <v>0.02013037</v>
       </c>
       <c r="J24" s="6" t="inlineStr">
         <is>
@@ -27344,25 +27344,25 @@
       </c>
       <c r="H25" s="6" t="inlineStr">
         <is>
-          <t>SLB</t>
+          <t>UPS</t>
         </is>
       </c>
       <c r="I25" s="61" t="n">
-        <v>0.01918674</v>
+        <v>0.01902798</v>
       </c>
       <c r="J25" s="6" t="inlineStr">
         <is>
-          <t>SLB</t>
+          <t>UNITED PARCEL SERVICE INC CLASS B</t>
         </is>
       </c>
       <c r="K25" s="6" t="inlineStr">
         <is>
-          <t>Energy</t>
+          <t>Industrials</t>
         </is>
       </c>
       <c r="L25" s="6" t="inlineStr">
         <is>
-          <t>SLB</t>
+          <t>UPS</t>
         </is>
       </c>
       <c r="M25" s="7">
@@ -27382,25 +27382,25 @@
       </c>
       <c r="H26" s="6" t="inlineStr">
         <is>
-          <t>UPS</t>
+          <t>SLB</t>
         </is>
       </c>
       <c r="I26" s="61" t="n">
-        <v>0.01903599</v>
+        <v>0.01889418</v>
       </c>
       <c r="J26" s="6" t="inlineStr">
         <is>
-          <t>UNITED PARCEL SERVICE INC CLASS B</t>
+          <t>SLB</t>
         </is>
       </c>
       <c r="K26" s="6" t="inlineStr">
         <is>
-          <t>Industrials</t>
+          <t>Energy</t>
         </is>
       </c>
       <c r="L26" s="6" t="inlineStr">
         <is>
-          <t>UPS</t>
+          <t>SLB</t>
         </is>
       </c>
       <c r="M26" s="7">
@@ -27424,7 +27424,7 @@
         </is>
       </c>
       <c r="I27" s="61" t="n">
-        <v>0.01836122</v>
+        <v>0.01864722</v>
       </c>
       <c r="J27" s="6" t="inlineStr">
         <is>
@@ -27462,7 +27462,7 @@
         </is>
       </c>
       <c r="I28" s="61" t="n">
-        <v>0.01627249</v>
+        <v>0.01631382</v>
       </c>
       <c r="J28" s="6" t="inlineStr">
         <is>
@@ -27500,7 +27500,7 @@
         </is>
       </c>
       <c r="I29" s="61" t="n">
-        <v>0.01433363</v>
+        <v>0.01429022</v>
       </c>
       <c r="J29" s="6" t="inlineStr">
         <is>
@@ -27534,7 +27534,7 @@
         </is>
       </c>
       <c r="I30" s="61" t="n">
-        <v>0.01419975</v>
+        <v>0.01426625</v>
       </c>
       <c r="J30" s="6" t="inlineStr">
         <is>
@@ -27572,7 +27572,7 @@
         </is>
       </c>
       <c r="I31" s="61" t="n">
-        <v>0.01356434</v>
+        <v>0.01331659</v>
       </c>
       <c r="J31" s="6" t="inlineStr">
         <is>
@@ -27597,7 +27597,7 @@
         </is>
       </c>
       <c r="I32" s="61" t="n">
-        <v>0.011663</v>
+        <v>0.01168047</v>
       </c>
       <c r="J32" s="6" t="inlineStr">
         <is>
@@ -27627,7 +27627,7 @@
         </is>
       </c>
       <c r="I33" s="61" t="n">
-        <v>0.01125747</v>
+        <v>0.01145338</v>
       </c>
       <c r="J33" s="6" t="inlineStr">
         <is>
@@ -27652,7 +27652,7 @@
         </is>
       </c>
       <c r="I34" s="61" t="n">
-        <v>0.0089522</v>
+        <v>0.008688399999999999</v>
       </c>
       <c r="J34" s="6" t="inlineStr">
         <is>
@@ -27677,7 +27677,7 @@
         </is>
       </c>
       <c r="I35" s="61" t="n">
-        <v>0.008670489999999999</v>
+        <v>0.008656179999999999</v>
       </c>
       <c r="J35" s="6" t="inlineStr">
         <is>
@@ -27702,7 +27702,7 @@
         </is>
       </c>
       <c r="I36" s="61" t="n">
-        <v>0.00833105</v>
+        <v>0.008282690000000001</v>
       </c>
       <c r="J36" s="6" t="inlineStr">
         <is>
@@ -27727,7 +27727,7 @@
         </is>
       </c>
       <c r="I37" s="61" t="n">
-        <v>0.00666956</v>
+        <v>0.00675392</v>
       </c>
       <c r="J37" s="6" t="inlineStr">
         <is>
@@ -27752,7 +27752,7 @@
         </is>
       </c>
       <c r="I38" s="61" t="n">
-        <v>0.00662146</v>
+        <v>0.00660323</v>
       </c>
       <c r="J38" s="6" t="inlineStr">
         <is>
@@ -27777,7 +27777,7 @@
         </is>
       </c>
       <c r="I39" s="61" t="n">
-        <v>0.00591301</v>
+        <v>0.00592157</v>
       </c>
       <c r="J39" s="6" t="inlineStr">
         <is>
@@ -27802,7 +27802,7 @@
         </is>
       </c>
       <c r="I40" s="61" t="n">
-        <v>0.00581724</v>
+        <v>0.00582091</v>
       </c>
       <c r="J40" s="6" t="inlineStr">
         <is>
@@ -27827,7 +27827,7 @@
         </is>
       </c>
       <c r="I41" s="61" t="n">
-        <v>0.00576264</v>
+        <v>0.00554762</v>
       </c>
       <c r="J41" s="6" t="inlineStr">
         <is>
@@ -27852,7 +27852,7 @@
         </is>
       </c>
       <c r="I42" s="61" t="n">
-        <v>0.005335490000000001</v>
+        <v>0.005380960000000001</v>
       </c>
       <c r="J42" s="6" t="inlineStr">
         <is>
@@ -27877,7 +27877,7 @@
         </is>
       </c>
       <c r="I43" s="61" t="n">
-        <v>0.005240590000000001</v>
+        <v>0.00523831</v>
       </c>
       <c r="J43" s="6" t="inlineStr">
         <is>
@@ -27902,7 +27902,7 @@
         </is>
       </c>
       <c r="I44" s="61" t="n">
-        <v>0.00485371</v>
+        <v>0.00480586</v>
       </c>
       <c r="J44" s="6" t="inlineStr">
         <is>
@@ -27927,7 +27927,7 @@
         </is>
       </c>
       <c r="I45" s="61" t="n">
-        <v>0.00461775</v>
+        <v>0.00470294</v>
       </c>
       <c r="J45" s="6" t="inlineStr">
         <is>
@@ -27952,7 +27952,7 @@
         </is>
       </c>
       <c r="I46" s="61" t="n">
-        <v>0.00442342</v>
+        <v>0.00438746</v>
       </c>
       <c r="J46" s="6" t="inlineStr">
         <is>
@@ -27977,7 +27977,7 @@
         </is>
       </c>
       <c r="I47" s="61" t="n">
-        <v>0.00432635</v>
+        <v>0.00430974</v>
       </c>
       <c r="J47" s="6" t="inlineStr">
         <is>
@@ -28002,7 +28002,7 @@
         </is>
       </c>
       <c r="I48" s="61" t="n">
-        <v>0.00430674</v>
+        <v>0.00426949</v>
       </c>
       <c r="J48" s="6" t="inlineStr">
         <is>
@@ -28027,7 +28027,7 @@
         </is>
       </c>
       <c r="I49" s="61" t="n">
-        <v>0.00425057</v>
+        <v>0.004215229999999999</v>
       </c>
       <c r="J49" s="6" t="inlineStr">
         <is>
@@ -28052,7 +28052,7 @@
         </is>
       </c>
       <c r="I50" s="61" t="n">
-        <v>0.00416319</v>
+        <v>0.00409258</v>
       </c>
       <c r="J50" s="6" t="inlineStr">
         <is>
@@ -28077,7 +28077,7 @@
         </is>
       </c>
       <c r="I51" s="61" t="n">
-        <v>0.00248823</v>
+        <v>0.00254985</v>
       </c>
       <c r="J51" s="6" t="inlineStr">
         <is>
@@ -28102,7 +28102,7 @@
         </is>
       </c>
       <c r="I52" s="61" t="n">
-        <v>0.00248447</v>
+        <v>0.00248949</v>
       </c>
       <c r="J52" s="6" t="inlineStr">
         <is>
@@ -28123,20 +28123,20 @@
     <row r="53">
       <c r="H53" s="6" t="inlineStr">
         <is>
-          <t>BAH</t>
+          <t>FNF</t>
         </is>
       </c>
       <c r="I53" s="61" t="n">
-        <v>0.00241355</v>
+        <v>0.00242606</v>
       </c>
       <c r="J53" s="6" t="inlineStr">
         <is>
-          <t>BOOZ ALLEN HAMILTON HOLDING CLASS</t>
+          <t>FIDELITY NATIONAL FINANCIAL INC</t>
         </is>
       </c>
       <c r="K53" s="6" t="inlineStr">
         <is>
-          <t>Industrials</t>
+          <t>Financials</t>
         </is>
       </c>
       <c r="L53" s="6" t="inlineStr"/>
@@ -28148,20 +28148,20 @@
     <row r="54">
       <c r="H54" s="6" t="inlineStr">
         <is>
-          <t>FNF</t>
+          <t>BAH</t>
         </is>
       </c>
       <c r="I54" s="61" t="n">
-        <v>0.00240637</v>
+        <v>0.00239541</v>
       </c>
       <c r="J54" s="6" t="inlineStr">
         <is>
-          <t>FIDELITY NATIONAL FINANCIAL INC</t>
+          <t>BOOZ ALLEN HAMILTON HOLDING CLASS</t>
         </is>
       </c>
       <c r="K54" s="6" t="inlineStr">
         <is>
-          <t>Financials</t>
+          <t>Industrials</t>
         </is>
       </c>
       <c r="L54" s="6" t="inlineStr"/>
@@ -28177,7 +28177,7 @@
         </is>
       </c>
       <c r="I55" s="61" t="n">
-        <v>0.00208811</v>
+        <v>0.00207336</v>
       </c>
       <c r="J55" s="6" t="inlineStr">
         <is>
@@ -28202,7 +28202,7 @@
         </is>
       </c>
       <c r="I56" s="61" t="n">
-        <v>0.00201477</v>
+        <v>0.00201913</v>
       </c>
       <c r="J56" s="6" t="inlineStr">
         <is>
@@ -28227,7 +28227,7 @@
         </is>
       </c>
       <c r="I57" s="61" t="n">
-        <v>0.00185147</v>
+        <v>0.00184327</v>
       </c>
       <c r="J57" s="6" t="inlineStr">
         <is>
@@ -28248,20 +28248,20 @@
     <row r="58">
       <c r="H58" s="6" t="inlineStr">
         <is>
-          <t>ERIE</t>
+          <t>M</t>
         </is>
       </c>
       <c r="I58" s="61" t="n">
-        <v>0.00153062</v>
+        <v>0.00153684</v>
       </c>
       <c r="J58" s="6" t="inlineStr">
         <is>
-          <t>ERIE INDEMNITY CLASS A</t>
+          <t>MACYS</t>
         </is>
       </c>
       <c r="K58" s="6" t="inlineStr">
         <is>
-          <t>Financials</t>
+          <t>Consumer Discretionary</t>
         </is>
       </c>
       <c r="L58" s="6" t="inlineStr"/>
@@ -28273,20 +28273,20 @@
     <row r="59">
       <c r="H59" s="6" t="inlineStr">
         <is>
-          <t>M</t>
+          <t>ERIE</t>
         </is>
       </c>
       <c r="I59" s="61" t="n">
-        <v>0.00150044</v>
+        <v>0.0015324</v>
       </c>
       <c r="J59" s="6" t="inlineStr">
         <is>
-          <t>MACYS</t>
+          <t>ERIE INDEMNITY CLASS A</t>
         </is>
       </c>
       <c r="K59" s="6" t="inlineStr">
         <is>
-          <t>Consumer Discretionary</t>
+          <t>Financials</t>
         </is>
       </c>
       <c r="L59" s="6" t="inlineStr"/>
@@ -28302,7 +28302,7 @@
         </is>
       </c>
       <c r="I60" s="61" t="n">
-        <v>0.00139481</v>
+        <v>0.00136721</v>
       </c>
       <c r="J60" s="6" t="inlineStr">
         <is>
@@ -28327,7 +28327,7 @@
         </is>
       </c>
       <c r="I61" s="61" t="n">
-        <v>0.00135074</v>
+        <v>0.00133222</v>
       </c>
       <c r="J61" s="6" t="inlineStr">
         <is>
@@ -28352,7 +28352,7 @@
         </is>
       </c>
       <c r="I62" s="61" t="n">
-        <v>0.00130196</v>
+        <v>0.00130236</v>
       </c>
       <c r="J62" s="6" t="inlineStr">
         <is>
@@ -28377,7 +28377,7 @@
         </is>
       </c>
       <c r="I63" s="61" t="n">
-        <v>0.00123355</v>
+        <v>0.00123259</v>
       </c>
       <c r="J63" s="6" t="inlineStr">
         <is>
@@ -28402,7 +28402,7 @@
         </is>
       </c>
       <c r="I64" s="61" t="n">
-        <v>0.00114714</v>
+        <v>0.00116678</v>
       </c>
       <c r="J64" s="6" t="inlineStr">
         <is>
@@ -28427,7 +28427,7 @@
         </is>
       </c>
       <c r="I65" s="61" t="n">
-        <v>0.00103589</v>
+        <v>0.00104832</v>
       </c>
       <c r="J65" s="6" t="inlineStr">
         <is>
@@ -28452,7 +28452,7 @@
         </is>
       </c>
       <c r="I66" s="61" t="n">
-        <v>0.00101029</v>
+        <v>0.00101585</v>
       </c>
       <c r="J66" s="6" t="inlineStr">
         <is>
@@ -28477,7 +28477,7 @@
         </is>
       </c>
       <c r="I67" s="61" t="n">
-        <v>0.00097339</v>
+        <v>0.0009781900000000001</v>
       </c>
       <c r="J67" s="6" t="inlineStr">
         <is>
@@ -28502,7 +28502,7 @@
         </is>
       </c>
       <c r="I68" s="61" t="n">
-        <v>0.00095216</v>
+        <v>0.0009397300000000001</v>
       </c>
       <c r="J68" s="6" t="inlineStr">
         <is>
@@ -28527,7 +28527,7 @@
         </is>
       </c>
       <c r="I69" s="61" t="n">
-        <v>0.00093041</v>
+        <v>0.00092419</v>
       </c>
       <c r="J69" s="6" t="inlineStr">
         <is>
@@ -28548,20 +28548,20 @@
     <row r="70">
       <c r="H70" s="6" t="inlineStr">
         <is>
-          <t>PAG</t>
+          <t>CVBF</t>
         </is>
       </c>
       <c r="I70" s="61" t="n">
-        <v>0.00090494</v>
+        <v>0.00089745</v>
       </c>
       <c r="J70" s="6" t="inlineStr">
         <is>
-          <t>PENSKE AUTOMOTIVE GROUP VOTING INC</t>
+          <t>CVB FINANCIAL CORP</t>
         </is>
       </c>
       <c r="K70" s="6" t="inlineStr">
         <is>
-          <t>Consumer Discretionary</t>
+          <t>Financials</t>
         </is>
       </c>
       <c r="L70" s="6" t="inlineStr"/>
@@ -28573,20 +28573,20 @@
     <row r="71">
       <c r="H71" s="6" t="inlineStr">
         <is>
-          <t>CVBF</t>
+          <t>PAG</t>
         </is>
       </c>
       <c r="I71" s="61" t="n">
-        <v>0.0009031400000000001</v>
+        <v>0.0008917500000000001</v>
       </c>
       <c r="J71" s="6" t="inlineStr">
         <is>
-          <t>CVB FINANCIAL CORP</t>
+          <t>PENSKE AUTOMOTIVE GROUP VOTING INC</t>
         </is>
       </c>
       <c r="K71" s="6" t="inlineStr">
         <is>
-          <t>Financials</t>
+          <t>Consumer Discretionary</t>
         </is>
       </c>
       <c r="L71" s="6" t="inlineStr"/>
@@ -28598,22 +28598,18 @@
     <row r="72">
       <c r="H72" s="6" t="inlineStr">
         <is>
-          <t>APAM</t>
+          <t>GVMXX</t>
         </is>
       </c>
       <c r="I72" s="61" t="n">
-        <v>0.0005903</v>
+        <v>0.0007404</v>
       </c>
       <c r="J72" s="6" t="inlineStr">
         <is>
-          <t>ARTISAN PARTNERS ASSET MANAGEMENT</t>
-        </is>
-      </c>
-      <c r="K72" s="6" t="inlineStr">
-        <is>
-          <t>Financials</t>
-        </is>
-      </c>
+          <t>SSC GOVERNMENT MM GVMXX</t>
+        </is>
+      </c>
+      <c r="K72" s="6" t="inlineStr"/>
       <c r="L72" s="6" t="inlineStr"/>
       <c r="M72" s="7">
         <f>IF(H72="","",IFERROR(VLOOKUP(K72,$P$5:$Q$15,2,FALSE),"현금·선물"))</f>
@@ -28623,15 +28619,15 @@
     <row r="73">
       <c r="H73" s="6" t="inlineStr">
         <is>
-          <t>BANR</t>
+          <t>APAM</t>
         </is>
       </c>
       <c r="I73" s="61" t="n">
-        <v>0.00055848</v>
+        <v>0.0006083999999999999</v>
       </c>
       <c r="J73" s="6" t="inlineStr">
         <is>
-          <t>BANNER CORP</t>
+          <t>ARTISAN PARTNERS ASSET MANAGEMENT</t>
         </is>
       </c>
       <c r="K73" s="6" t="inlineStr">
@@ -28648,15 +28644,15 @@
     <row r="74">
       <c r="H74" s="6" t="inlineStr">
         <is>
-          <t>OFG</t>
+          <t>BANR</t>
         </is>
       </c>
       <c r="I74" s="61" t="n">
-        <v>0.00051614</v>
+        <v>0.00055446</v>
       </c>
       <c r="J74" s="6" t="inlineStr">
         <is>
-          <t>OFG BANCORP</t>
+          <t>BANNER CORP</t>
         </is>
       </c>
       <c r="K74" s="6" t="inlineStr">
@@ -28673,20 +28669,20 @@
     <row r="75">
       <c r="H75" s="6" t="inlineStr">
         <is>
-          <t>MZTI</t>
+          <t>OFG</t>
         </is>
       </c>
       <c r="I75" s="61" t="n">
-        <v>0.00050795</v>
+        <v>0.00050899</v>
       </c>
       <c r="J75" s="6" t="inlineStr">
         <is>
-          <t>MARZETTI</t>
+          <t>OFG BANCORP</t>
         </is>
       </c>
       <c r="K75" s="6" t="inlineStr">
         <is>
-          <t>Consumer Staples</t>
+          <t>Financials</t>
         </is>
       </c>
       <c r="L75" s="6" t="inlineStr"/>
@@ -28698,15 +28694,15 @@
     <row r="76">
       <c r="H76" s="6" t="inlineStr">
         <is>
-          <t>IPAR</t>
+          <t>MZTI</t>
         </is>
       </c>
       <c r="I76" s="61" t="n">
-        <v>0.00050156</v>
+        <v>0.00050296</v>
       </c>
       <c r="J76" s="6" t="inlineStr">
         <is>
-          <t>INTERPARFUMS INC</t>
+          <t>MARZETTI</t>
         </is>
       </c>
       <c r="K76" s="6" t="inlineStr">
@@ -28723,20 +28719,20 @@
     <row r="77">
       <c r="H77" s="6" t="inlineStr">
         <is>
-          <t>CHCO</t>
+          <t>IPAR</t>
         </is>
       </c>
       <c r="I77" s="61" t="n">
-        <v>0.00048047</v>
+        <v>0.0004987699999999999</v>
       </c>
       <c r="J77" s="6" t="inlineStr">
         <is>
-          <t>CITY HOLDING</t>
+          <t>INTERPARFUMS INC</t>
         </is>
       </c>
       <c r="K77" s="6" t="inlineStr">
         <is>
-          <t>Financials</t>
+          <t>Consumer Staples</t>
         </is>
       </c>
       <c r="L77" s="6" t="inlineStr"/>
@@ -28752,7 +28748,7 @@
         </is>
       </c>
       <c r="I78" s="61" t="n">
-        <v>0.00047654</v>
+        <v>0.00048786</v>
       </c>
       <c r="J78" s="6" t="inlineStr">
         <is>
@@ -28773,15 +28769,15 @@
     <row r="79">
       <c r="H79" s="6" t="inlineStr">
         <is>
-          <t>AGM</t>
+          <t>CHCO</t>
         </is>
       </c>
       <c r="I79" s="61" t="n">
-        <v>0.00045831</v>
+        <v>0.00047741</v>
       </c>
       <c r="J79" s="6" t="inlineStr">
         <is>
-          <t>FEDERAL AGRICULTURAL MORTGAGE NON</t>
+          <t>CITY HOLDING</t>
         </is>
       </c>
       <c r="K79" s="6" t="inlineStr">
@@ -28802,7 +28798,7 @@
         </is>
       </c>
       <c r="I80" s="61" t="n">
-        <v>0.00045805</v>
+        <v>0.00045943</v>
       </c>
       <c r="J80" s="6" t="inlineStr">
         <is>
@@ -28823,18 +28819,22 @@
     <row r="81">
       <c r="H81" s="6" t="inlineStr">
         <is>
-          <t>GVMXX</t>
+          <t>AGM</t>
         </is>
       </c>
       <c r="I81" s="61" t="n">
-        <v>0.00045189</v>
+        <v>0.00045034</v>
       </c>
       <c r="J81" s="6" t="inlineStr">
         <is>
-          <t>SSC GOVERNMENT MM GVMXX</t>
-        </is>
-      </c>
-      <c r="K81" s="6" t="inlineStr"/>
+          <t>FEDERAL AGRICULTURAL MORTGAGE NON</t>
+        </is>
+      </c>
+      <c r="K81" s="6" t="inlineStr">
+        <is>
+          <t>Financials</t>
+        </is>
+      </c>
       <c r="L81" s="6" t="inlineStr"/>
       <c r="M81" s="7">
         <f>IF(H81="","",IFERROR(VLOOKUP(K81,$P$5:$Q$15,2,FALSE),"현금·선물"))</f>
@@ -28844,20 +28844,20 @@
     <row r="82">
       <c r="H82" s="6" t="inlineStr">
         <is>
-          <t>NSP</t>
+          <t>GABC</t>
         </is>
       </c>
       <c r="I82" s="61" t="n">
-        <v>0.00044478</v>
+        <v>0.00044021</v>
       </c>
       <c r="J82" s="6" t="inlineStr">
         <is>
-          <t>INSPERITY</t>
+          <t>GERMAN AMERICAN BANCORP INC</t>
         </is>
       </c>
       <c r="K82" s="6" t="inlineStr">
         <is>
-          <t>Industrials</t>
+          <t>Financials</t>
         </is>
       </c>
       <c r="L82" s="6" t="inlineStr"/>
@@ -28869,15 +28869,15 @@
     <row r="83">
       <c r="H83" s="6" t="inlineStr">
         <is>
-          <t>GABC</t>
+          <t>STBA</t>
         </is>
       </c>
       <c r="I83" s="61" t="n">
-        <v>0.00044338</v>
+        <v>0.00042712</v>
       </c>
       <c r="J83" s="6" t="inlineStr">
         <is>
-          <t>GERMAN AMERICAN BANCORP INC</t>
+          <t>S AND T BANCORP INC</t>
         </is>
       </c>
       <c r="K83" s="6" t="inlineStr">
@@ -28894,15 +28894,15 @@
     <row r="84">
       <c r="H84" s="6" t="inlineStr">
         <is>
-          <t>STBA</t>
+          <t>NBHC</t>
         </is>
       </c>
       <c r="I84" s="61" t="n">
-        <v>0.00042906</v>
+        <v>0.00039517</v>
       </c>
       <c r="J84" s="6" t="inlineStr">
         <is>
-          <t>S AND T BANCORP INC</t>
+          <t>NATIONAL BANK HOLDINGS CORP CLASS</t>
         </is>
       </c>
       <c r="K84" s="6" t="inlineStr">
@@ -28919,20 +28919,20 @@
     <row r="85">
       <c r="H85" s="6" t="inlineStr">
         <is>
-          <t>NBHC</t>
+          <t>NSP</t>
         </is>
       </c>
       <c r="I85" s="61" t="n">
-        <v>0.00040089</v>
+        <v>0.0003921</v>
       </c>
       <c r="J85" s="6" t="inlineStr">
         <is>
-          <t>NATIONAL BANK HOLDINGS CORP CLASS</t>
+          <t>INSPERITY</t>
         </is>
       </c>
       <c r="K85" s="6" t="inlineStr">
         <is>
-          <t>Financials</t>
+          <t>Industrials</t>
         </is>
       </c>
       <c r="L85" s="6" t="inlineStr"/>
@@ -28948,7 +28948,7 @@
         </is>
       </c>
       <c r="I86" s="61" t="n">
-        <v>0.00037513</v>
+        <v>0.00037257</v>
       </c>
       <c r="J86" s="6" t="inlineStr">
         <is>
@@ -28973,7 +28973,7 @@
         </is>
       </c>
       <c r="I87" s="61" t="n">
-        <v>0.00036194</v>
+        <v>0.00035967</v>
       </c>
       <c r="J87" s="6" t="inlineStr">
         <is>
@@ -28998,7 +28998,7 @@
         </is>
       </c>
       <c r="I88" s="61" t="n">
-        <v>0.00033613</v>
+        <v>0.0003416</v>
       </c>
       <c r="J88" s="6" t="inlineStr">
         <is>
@@ -29023,7 +29023,7 @@
         </is>
       </c>
       <c r="I89" s="61" t="n">
-        <v>0.0003135</v>
+        <v>0.00031038</v>
       </c>
       <c r="J89" s="6" t="inlineStr">
         <is>
@@ -29048,7 +29048,7 @@
         </is>
       </c>
       <c r="I90" s="61" t="n">
-        <v>0.0002808</v>
+        <v>0.00027592</v>
       </c>
       <c r="J90" s="6" t="inlineStr">
         <is>
@@ -29073,7 +29073,7 @@
         </is>
       </c>
       <c r="I91" s="61" t="n">
-        <v>0.00027328</v>
+        <v>0.00027261</v>
       </c>
       <c r="J91" s="6" t="inlineStr">
         <is>
@@ -29098,7 +29098,7 @@
         </is>
       </c>
       <c r="I92" s="61" t="n">
-        <v>0.00025016</v>
+        <v>0.0002511</v>
       </c>
       <c r="J92" s="6" t="inlineStr">
         <is>
@@ -29123,7 +29123,7 @@
         </is>
       </c>
       <c r="I93" s="61" t="n">
-        <v>0.00023396</v>
+        <v>0.00023498</v>
       </c>
       <c r="J93" s="6" t="inlineStr">
         <is>
@@ -29148,7 +29148,7 @@
         </is>
       </c>
       <c r="I94" s="61" t="n">
-        <v>0.00023201</v>
+        <v>0.00023121</v>
       </c>
       <c r="J94" s="6" t="inlineStr">
         <is>
@@ -29173,7 +29173,7 @@
         </is>
       </c>
       <c r="I95" s="61" t="n">
-        <v>0.00021154</v>
+        <v>0.00020949</v>
       </c>
       <c r="J95" s="6" t="inlineStr">
         <is>
@@ -29194,15 +29194,15 @@
     <row r="96">
       <c r="H96" s="6" t="inlineStr">
         <is>
-          <t>IBCP</t>
+          <t>THFF</t>
         </is>
       </c>
       <c r="I96" s="61" t="n">
-        <v>0.00019759</v>
+        <v>0.00019564</v>
       </c>
       <c r="J96" s="6" t="inlineStr">
         <is>
-          <t>INDEPENDENT BANK CORP</t>
+          <t>FIRST FINANCIAL CORPORATION CORP</t>
         </is>
       </c>
       <c r="K96" s="6" t="inlineStr">
@@ -29219,15 +29219,15 @@
     <row r="97">
       <c r="H97" s="6" t="inlineStr">
         <is>
-          <t>THFF</t>
+          <t>IBCP</t>
         </is>
       </c>
       <c r="I97" s="61" t="n">
-        <v>0.00019718</v>
+        <v>0.0001953</v>
       </c>
       <c r="J97" s="6" t="inlineStr">
         <is>
-          <t>FIRST FINANCIAL CORPORATION CORP</t>
+          <t>INDEPENDENT BANK CORP</t>
         </is>
       </c>
       <c r="K97" s="6" t="inlineStr">
@@ -29248,7 +29248,7 @@
         </is>
       </c>
       <c r="I98" s="61" t="n">
-        <v>0.00018082</v>
+        <v>0.00018058</v>
       </c>
       <c r="J98" s="6" t="inlineStr">
         <is>
@@ -29273,7 +29273,7 @@
         </is>
       </c>
       <c r="I99" s="61" t="n">
-        <v>0.00016726</v>
+        <v>0.0001657</v>
       </c>
       <c r="J99" s="6" t="inlineStr">
         <is>
@@ -29298,7 +29298,7 @@
         </is>
       </c>
       <c r="I100" s="61" t="n">
-        <v>0.00013781</v>
+        <v>0.00013253</v>
       </c>
       <c r="J100" s="6" t="inlineStr">
         <is>
@@ -29319,7 +29319,7 @@
         </is>
       </c>
       <c r="I101" s="61" t="n">
-        <v>0.00012793</v>
+        <v>0.00012318</v>
       </c>
       <c r="J101" s="6" t="inlineStr">
         <is>
@@ -29344,7 +29344,7 @@
         </is>
       </c>
       <c r="I102" s="61" t="n">
-        <v>0.0001128</v>
+        <v>0.00010126</v>
       </c>
       <c r="J102" s="6" t="inlineStr">
         <is>
@@ -29369,7 +29369,7 @@
         </is>
       </c>
       <c r="I103" s="61" t="n">
-        <v>9.331000000000001e-05</v>
+        <v>9.547000000000001e-05</v>
       </c>
       <c r="J103" s="6" t="inlineStr">
         <is>
@@ -29394,7 +29394,7 @@
         </is>
       </c>
       <c r="I104" s="61" t="n">
-        <v>9.083000000000001e-05</v>
+        <v>9.400000000000001e-05</v>
       </c>
       <c r="J104" s="6" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
데이터 갱신: holdings (2026-10-31)
</commit_message>
<xml_diff>
--- a/downloads/schd_dividend_tracker.xlsx
+++ b/downloads/schd_dividend_tracker.xlsx
@@ -1724,7 +1724,7 @@
     <row r="3">
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>최종 갱신: 2026-10-30 · 반영 범위: 2012년 1분기 ~ 2026년 3분기 (배당락 2026-09-23) · GitHub Actions 자동 생성</t>
+          <t>최종 갱신: 2026-10-31 · 반영 범위: 2012년 1분기 ~ 2026년 3분기 (배당락 2026-09-23) · GitHub Actions 자동 생성</t>
         </is>
       </c>
     </row>
@@ -26299,11 +26299,11 @@
         </is>
       </c>
       <c r="B2" s="49" t="n">
-        <v>46324</v>
+        <v>46325</v>
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>← 이 날 종가로 계산한 비중. 그날 공식 파일을 못 받아 Schwab 공식 보유종목 CSV(2026-10-28)의 보유 주식 수 × 종가로 계산했습니다.</t>
+          <t>← 이 날 종가로 계산한 비중. 그날 공식 파일을 못 받아 Schwab 공식 보유종목 CSV(2026-10-29)의 보유 주식 수 × 종가로 계산했습니다.</t>
         </is>
       </c>
     </row>
@@ -26400,7 +26400,7 @@
         </is>
       </c>
       <c r="I5" s="61" t="n">
-        <v>0.04795357</v>
+        <v>0.04591873</v>
       </c>
       <c r="J5" s="6" t="inlineStr">
         <is>
@@ -26454,15 +26454,15 @@
       </c>
       <c r="H6" s="6" t="inlineStr">
         <is>
-          <t>CVX</t>
+          <t>COP</t>
         </is>
       </c>
       <c r="I6" s="61" t="n">
-        <v>0.04267233</v>
+        <v>0.04360672</v>
       </c>
       <c r="J6" s="6" t="inlineStr">
         <is>
-          <t>CHEVRON</t>
+          <t>CONOCOPHILLIPS</t>
         </is>
       </c>
       <c r="K6" s="6" t="inlineStr">
@@ -26472,7 +26472,7 @@
       </c>
       <c r="L6" s="6" t="inlineStr">
         <is>
-          <t>셰브론</t>
+          <t>코노코필립스</t>
         </is>
       </c>
       <c r="M6" s="7">
@@ -26512,15 +26512,15 @@
       </c>
       <c r="H7" s="6" t="inlineStr">
         <is>
-          <t>COP</t>
+          <t>CVX</t>
         </is>
       </c>
       <c r="I7" s="61" t="n">
-        <v>0.04264136</v>
+        <v>0.04325059000000001</v>
       </c>
       <c r="J7" s="6" t="inlineStr">
         <is>
-          <t>CONOCOPHILLIPS</t>
+          <t>CHEVRON</t>
         </is>
       </c>
       <c r="K7" s="6" t="inlineStr">
@@ -26530,7 +26530,7 @@
       </c>
       <c r="L7" s="6" t="inlineStr">
         <is>
-          <t>코노코필립스</t>
+          <t>셰브론</t>
         </is>
       </c>
       <c r="M7" s="7">
@@ -26570,25 +26570,25 @@
       </c>
       <c r="H8" s="6" t="inlineStr">
         <is>
-          <t>QCOM</t>
+          <t>PG</t>
         </is>
       </c>
       <c r="I8" s="61" t="n">
-        <v>0.04259401</v>
+        <v>0.04256144</v>
       </c>
       <c r="J8" s="6" t="inlineStr">
         <is>
-          <t>QUALCOMM</t>
+          <t>PROCTER &amp; GAMBLE</t>
         </is>
       </c>
       <c r="K8" s="6" t="inlineStr">
         <is>
-          <t>Information Technology</t>
+          <t>Consumer Staples</t>
         </is>
       </c>
       <c r="L8" s="6" t="inlineStr">
         <is>
-          <t>퀄컴</t>
+          <t>프록터앤드갬블</t>
         </is>
       </c>
       <c r="M8" s="7">
@@ -26628,15 +26628,15 @@
       </c>
       <c r="H9" s="6" t="inlineStr">
         <is>
-          <t>PG</t>
+          <t>KO</t>
         </is>
       </c>
       <c r="I9" s="61" t="n">
-        <v>0.04246965999999999</v>
+        <v>0.04146571</v>
       </c>
       <c r="J9" s="6" t="inlineStr">
         <is>
-          <t>PROCTER &amp; GAMBLE</t>
+          <t>COCA-COLA</t>
         </is>
       </c>
       <c r="K9" s="6" t="inlineStr">
@@ -26646,7 +26646,7 @@
       </c>
       <c r="L9" s="6" t="inlineStr">
         <is>
-          <t>프록터앤드갬블</t>
+          <t>코카콜라</t>
         </is>
       </c>
       <c r="M9" s="7">
@@ -26686,25 +26686,25 @@
       </c>
       <c r="H10" s="6" t="inlineStr">
         <is>
-          <t>KO</t>
+          <t>AMGN</t>
         </is>
       </c>
       <c r="I10" s="61" t="n">
-        <v>0.0410713</v>
+        <v>0.0409245</v>
       </c>
       <c r="J10" s="6" t="inlineStr">
         <is>
-          <t>COCA-COLA</t>
+          <t>AMGEN INC</t>
         </is>
       </c>
       <c r="K10" s="6" t="inlineStr">
         <is>
-          <t>Consumer Staples</t>
+          <t>Health Care</t>
         </is>
       </c>
       <c r="L10" s="6" t="inlineStr">
         <is>
-          <t>코카콜라</t>
+          <t>암젠</t>
         </is>
       </c>
       <c r="M10" s="7">
@@ -26744,25 +26744,25 @@
       </c>
       <c r="H11" s="6" t="inlineStr">
         <is>
-          <t>AMGN</t>
+          <t>HD</t>
         </is>
       </c>
       <c r="I11" s="61" t="n">
-        <v>0.04062024</v>
+        <v>0.04019523999999999</v>
       </c>
       <c r="J11" s="6" t="inlineStr">
         <is>
-          <t>AMGEN INC</t>
+          <t>HOME DEPOT</t>
         </is>
       </c>
       <c r="K11" s="6" t="inlineStr">
         <is>
-          <t>Health Care</t>
+          <t>Consumer Discretionary</t>
         </is>
       </c>
       <c r="L11" s="6" t="inlineStr">
         <is>
-          <t>암젠</t>
+          <t>홈디포</t>
         </is>
       </c>
       <c r="M11" s="7">
@@ -26802,25 +26802,25 @@
       </c>
       <c r="H12" s="6" t="inlineStr">
         <is>
-          <t>HD</t>
+          <t>UNH</t>
         </is>
       </c>
       <c r="I12" s="61" t="n">
-        <v>0.04032661</v>
+        <v>0.0396015</v>
       </c>
       <c r="J12" s="6" t="inlineStr">
         <is>
-          <t>HOME DEPOT</t>
+          <t>UNITEDHEALTH GROUP</t>
         </is>
       </c>
       <c r="K12" s="6" t="inlineStr">
         <is>
-          <t>Consumer Discretionary</t>
+          <t>Health Care</t>
         </is>
       </c>
       <c r="L12" s="6" t="inlineStr">
         <is>
-          <t>홈디포</t>
+          <t>유나이티드헬스</t>
         </is>
       </c>
       <c r="M12" s="7">
@@ -26860,15 +26860,15 @@
       </c>
       <c r="H13" s="6" t="inlineStr">
         <is>
-          <t>UNH</t>
+          <t>MRK</t>
         </is>
       </c>
       <c r="I13" s="61" t="n">
-        <v>0.04014238</v>
+        <v>0.03834765</v>
       </c>
       <c r="J13" s="6" t="inlineStr">
         <is>
-          <t>UNITEDHEALTH GROUP</t>
+          <t>MERCK &amp; CO INC</t>
         </is>
       </c>
       <c r="K13" s="6" t="inlineStr">
@@ -26878,7 +26878,7 @@
       </c>
       <c r="L13" s="6" t="inlineStr">
         <is>
-          <t>유나이티드헬스</t>
+          <t>머크</t>
         </is>
       </c>
       <c r="M13" s="7">
@@ -26918,25 +26918,25 @@
       </c>
       <c r="H14" s="6" t="inlineStr">
         <is>
-          <t>MRK</t>
+          <t>PEP</t>
         </is>
       </c>
       <c r="I14" s="61" t="n">
-        <v>0.03767718</v>
+        <v>0.03801107</v>
       </c>
       <c r="J14" s="6" t="inlineStr">
         <is>
-          <t>MERCK &amp; CO INC</t>
+          <t>PEPSICO</t>
         </is>
       </c>
       <c r="K14" s="6" t="inlineStr">
         <is>
-          <t>Health Care</t>
+          <t>Consumer Staples</t>
         </is>
       </c>
       <c r="L14" s="6" t="inlineStr">
         <is>
-          <t>머크</t>
+          <t>펩시코</t>
         </is>
       </c>
       <c r="M14" s="7">
@@ -26966,25 +26966,25 @@
       </c>
       <c r="H15" s="6" t="inlineStr">
         <is>
-          <t>PEP</t>
+          <t>QCOM</t>
         </is>
       </c>
       <c r="I15" s="61" t="n">
-        <v>0.03717428</v>
+        <v>0.03770865</v>
       </c>
       <c r="J15" s="6" t="inlineStr">
         <is>
-          <t>PEPSICO</t>
+          <t>QUALCOMM</t>
         </is>
       </c>
       <c r="K15" s="6" t="inlineStr">
         <is>
-          <t>Consumer Staples</t>
+          <t>Information Technology</t>
         </is>
       </c>
       <c r="L15" s="6" t="inlineStr">
         <is>
-          <t>펩시코</t>
+          <t>퀄컴</t>
         </is>
       </c>
       <c r="M15" s="7">
@@ -27018,7 +27018,7 @@
         </is>
       </c>
       <c r="I16" s="61" t="n">
-        <v>0.03695951</v>
+        <v>0.03738856</v>
       </c>
       <c r="J16" s="6" t="inlineStr">
         <is>
@@ -27056,7 +27056,7 @@
         </is>
       </c>
       <c r="I17" s="61" t="n">
-        <v>0.03579137</v>
+        <v>0.03724026</v>
       </c>
       <c r="J17" s="6" t="inlineStr">
         <is>
@@ -27094,7 +27094,7 @@
         </is>
       </c>
       <c r="I18" s="61" t="n">
-        <v>0.03394476</v>
+        <v>0.03464044</v>
       </c>
       <c r="J18" s="6" t="inlineStr">
         <is>
@@ -27119,25 +27119,25 @@
     <row r="19">
       <c r="H19" s="6" t="inlineStr">
         <is>
-          <t>LMT</t>
+          <t>MO</t>
         </is>
       </c>
       <c r="I19" s="61" t="n">
-        <v>0.03092271</v>
+        <v>0.03070406</v>
       </c>
       <c r="J19" s="6" t="inlineStr">
         <is>
-          <t>LOCKHEED MARTIN</t>
+          <t>ALTRIA GROUP INC</t>
         </is>
       </c>
       <c r="K19" s="6" t="inlineStr">
         <is>
-          <t>Industrials</t>
+          <t>Consumer Staples</t>
         </is>
       </c>
       <c r="L19" s="6" t="inlineStr">
         <is>
-          <t>록히드마틴</t>
+          <t>알트리아</t>
         </is>
       </c>
       <c r="M19" s="7">
@@ -27153,25 +27153,25 @@
       </c>
       <c r="H20" s="6" t="inlineStr">
         <is>
-          <t>MO</t>
+          <t>LMT</t>
         </is>
       </c>
       <c r="I20" s="61" t="n">
-        <v>0.03031918</v>
+        <v>0.03048356</v>
       </c>
       <c r="J20" s="6" t="inlineStr">
         <is>
-          <t>ALTRIA GROUP INC</t>
+          <t>LOCKHEED MARTIN</t>
         </is>
       </c>
       <c r="K20" s="6" t="inlineStr">
         <is>
-          <t>Consumer Staples</t>
+          <t>Industrials</t>
         </is>
       </c>
       <c r="L20" s="6" t="inlineStr">
         <is>
-          <t>알트리아</t>
+          <t>록히드마틴</t>
         </is>
       </c>
       <c r="M20" s="7">
@@ -27196,7 +27196,7 @@
         </is>
       </c>
       <c r="I21" s="61" t="n">
-        <v>0.02966852</v>
+        <v>0.03007701</v>
       </c>
       <c r="J21" s="6" t="inlineStr">
         <is>
@@ -27234,7 +27234,7 @@
         </is>
       </c>
       <c r="I22" s="61" t="n">
-        <v>0.02688757</v>
+        <v>0.0275087</v>
       </c>
       <c r="J22" s="6" t="inlineStr">
         <is>
@@ -27272,7 +27272,7 @@
         </is>
       </c>
       <c r="I23" s="61" t="n">
-        <v>0.02141662</v>
+        <v>0.02096295</v>
       </c>
       <c r="J23" s="6" t="inlineStr">
         <is>
@@ -27310,7 +27310,7 @@
         </is>
       </c>
       <c r="I24" s="61" t="n">
-        <v>0.02013037</v>
+        <v>0.0204618</v>
       </c>
       <c r="J24" s="6" t="inlineStr">
         <is>
@@ -27344,25 +27344,25 @@
       </c>
       <c r="H25" s="6" t="inlineStr">
         <is>
-          <t>UPS</t>
+          <t>CMCSA</t>
         </is>
       </c>
       <c r="I25" s="61" t="n">
-        <v>0.01902798</v>
+        <v>0.01936651</v>
       </c>
       <c r="J25" s="6" t="inlineStr">
         <is>
-          <t>UNITED PARCEL SERVICE INC CLASS B</t>
+          <t>COMCAST CLASS A</t>
         </is>
       </c>
       <c r="K25" s="6" t="inlineStr">
         <is>
-          <t>Industrials</t>
+          <t>Communication Services</t>
         </is>
       </c>
       <c r="L25" s="6" t="inlineStr">
         <is>
-          <t>UPS</t>
+          <t>컴캐스트</t>
         </is>
       </c>
       <c r="M25" s="7">
@@ -27382,25 +27382,25 @@
       </c>
       <c r="H26" s="6" t="inlineStr">
         <is>
-          <t>SLB</t>
+          <t>UPS</t>
         </is>
       </c>
       <c r="I26" s="61" t="n">
-        <v>0.01889418</v>
+        <v>0.01911589</v>
       </c>
       <c r="J26" s="6" t="inlineStr">
         <is>
-          <t>SLB</t>
+          <t>UNITED PARCEL SERVICE INC CLASS B</t>
         </is>
       </c>
       <c r="K26" s="6" t="inlineStr">
         <is>
-          <t>Energy</t>
+          <t>Industrials</t>
         </is>
       </c>
       <c r="L26" s="6" t="inlineStr">
         <is>
-          <t>SLB</t>
+          <t>UPS</t>
         </is>
       </c>
       <c r="M26" s="7">
@@ -27420,25 +27420,25 @@
       </c>
       <c r="H27" s="6" t="inlineStr">
         <is>
-          <t>CMCSA</t>
+          <t>SLB</t>
         </is>
       </c>
       <c r="I27" s="61" t="n">
-        <v>0.01864722</v>
+        <v>0.01879568</v>
       </c>
       <c r="J27" s="6" t="inlineStr">
         <is>
-          <t>COMCAST CLASS A</t>
+          <t>SLB</t>
         </is>
       </c>
       <c r="K27" s="6" t="inlineStr">
         <is>
-          <t>Communication Services</t>
+          <t>Energy</t>
         </is>
       </c>
       <c r="L27" s="6" t="inlineStr">
         <is>
-          <t>컴캐스트</t>
+          <t>SLB</t>
         </is>
       </c>
       <c r="M27" s="7">
@@ -27462,7 +27462,7 @@
         </is>
       </c>
       <c r="I28" s="61" t="n">
-        <v>0.01631382</v>
+        <v>0.01652392</v>
       </c>
       <c r="J28" s="6" t="inlineStr">
         <is>
@@ -27500,7 +27500,7 @@
         </is>
       </c>
       <c r="I29" s="61" t="n">
-        <v>0.01429022</v>
+        <v>0.01441993</v>
       </c>
       <c r="J29" s="6" t="inlineStr">
         <is>
@@ -27534,7 +27534,7 @@
         </is>
       </c>
       <c r="I30" s="61" t="n">
-        <v>0.01426625</v>
+        <v>0.01403728</v>
       </c>
       <c r="J30" s="6" t="inlineStr">
         <is>
@@ -27572,7 +27572,7 @@
         </is>
       </c>
       <c r="I31" s="61" t="n">
-        <v>0.01331659</v>
+        <v>0.01351843</v>
       </c>
       <c r="J31" s="6" t="inlineStr">
         <is>
@@ -27597,7 +27597,7 @@
         </is>
       </c>
       <c r="I32" s="61" t="n">
-        <v>0.01168047</v>
+        <v>0.01151288</v>
       </c>
       <c r="J32" s="6" t="inlineStr">
         <is>
@@ -27627,7 +27627,7 @@
         </is>
       </c>
       <c r="I33" s="61" t="n">
-        <v>0.01145338</v>
+        <v>0.01130699</v>
       </c>
       <c r="J33" s="6" t="inlineStr">
         <is>
@@ -27652,7 +27652,7 @@
         </is>
       </c>
       <c r="I34" s="61" t="n">
-        <v>0.008688399999999999</v>
+        <v>0.00873496</v>
       </c>
       <c r="J34" s="6" t="inlineStr">
         <is>
@@ -27677,7 +27677,7 @@
         </is>
       </c>
       <c r="I35" s="61" t="n">
-        <v>0.008656179999999999</v>
+        <v>0.00845918</v>
       </c>
       <c r="J35" s="6" t="inlineStr">
         <is>
@@ -27702,7 +27702,7 @@
         </is>
       </c>
       <c r="I36" s="61" t="n">
-        <v>0.008282690000000001</v>
+        <v>0.008457630000000001</v>
       </c>
       <c r="J36" s="6" t="inlineStr">
         <is>
@@ -27727,7 +27727,7 @@
         </is>
       </c>
       <c r="I37" s="61" t="n">
-        <v>0.00675392</v>
+        <v>0.00676333</v>
       </c>
       <c r="J37" s="6" t="inlineStr">
         <is>
@@ -27752,7 +27752,7 @@
         </is>
       </c>
       <c r="I38" s="61" t="n">
-        <v>0.00660323</v>
+        <v>0.00655268</v>
       </c>
       <c r="J38" s="6" t="inlineStr">
         <is>
@@ -27777,7 +27777,7 @@
         </is>
       </c>
       <c r="I39" s="61" t="n">
-        <v>0.00592157</v>
+        <v>0.00588993</v>
       </c>
       <c r="J39" s="6" t="inlineStr">
         <is>
@@ -27802,7 +27802,7 @@
         </is>
       </c>
       <c r="I40" s="61" t="n">
-        <v>0.00582091</v>
+        <v>0.005735860000000001</v>
       </c>
       <c r="J40" s="6" t="inlineStr">
         <is>
@@ -27827,7 +27827,7 @@
         </is>
       </c>
       <c r="I41" s="61" t="n">
-        <v>0.00554762</v>
+        <v>0.00570956</v>
       </c>
       <c r="J41" s="6" t="inlineStr">
         <is>
@@ -27852,7 +27852,7 @@
         </is>
       </c>
       <c r="I42" s="61" t="n">
-        <v>0.005380960000000001</v>
+        <v>0.00522259</v>
       </c>
       <c r="J42" s="6" t="inlineStr">
         <is>
@@ -27877,7 +27877,7 @@
         </is>
       </c>
       <c r="I43" s="61" t="n">
-        <v>0.00523831</v>
+        <v>0.005124950000000001</v>
       </c>
       <c r="J43" s="6" t="inlineStr">
         <is>
@@ -27902,7 +27902,7 @@
         </is>
       </c>
       <c r="I44" s="61" t="n">
-        <v>0.00480586</v>
+        <v>0.00480515</v>
       </c>
       <c r="J44" s="6" t="inlineStr">
         <is>
@@ -27927,7 +27927,7 @@
         </is>
       </c>
       <c r="I45" s="61" t="n">
-        <v>0.00470294</v>
+        <v>0.00446331</v>
       </c>
       <c r="J45" s="6" t="inlineStr">
         <is>
@@ -27948,20 +27948,20 @@
     <row r="46">
       <c r="H46" s="6" t="inlineStr">
         <is>
-          <t>SNA</t>
+          <t>APA</t>
         </is>
       </c>
       <c r="I46" s="61" t="n">
-        <v>0.00438746</v>
+        <v>0.0043609</v>
       </c>
       <c r="J46" s="6" t="inlineStr">
         <is>
-          <t>SNAP ON INC</t>
+          <t>APA</t>
         </is>
       </c>
       <c r="K46" s="6" t="inlineStr">
         <is>
-          <t>Industrials</t>
+          <t>Energy</t>
         </is>
       </c>
       <c r="L46" s="6" t="inlineStr"/>
@@ -27973,20 +27973,20 @@
     <row r="47">
       <c r="H47" s="6" t="inlineStr">
         <is>
-          <t>EWBC</t>
+          <t>SNA</t>
         </is>
       </c>
       <c r="I47" s="61" t="n">
-        <v>0.00430974</v>
+        <v>0.0043342</v>
       </c>
       <c r="J47" s="6" t="inlineStr">
         <is>
-          <t>EAST WEST BANCORP</t>
+          <t>SNAP ON INC</t>
         </is>
       </c>
       <c r="K47" s="6" t="inlineStr">
         <is>
-          <t>Financials</t>
+          <t>Industrials</t>
         </is>
       </c>
       <c r="L47" s="6" t="inlineStr"/>
@@ -27998,20 +27998,20 @@
     <row r="48">
       <c r="H48" s="6" t="inlineStr">
         <is>
-          <t>APA</t>
+          <t>GIS</t>
         </is>
       </c>
       <c r="I48" s="61" t="n">
-        <v>0.00426949</v>
+        <v>0.00432092</v>
       </c>
       <c r="J48" s="6" t="inlineStr">
         <is>
-          <t>APA</t>
+          <t>GENERAL MILLS INC</t>
         </is>
       </c>
       <c r="K48" s="6" t="inlineStr">
         <is>
-          <t>Energy</t>
+          <t>Consumer Staples</t>
         </is>
       </c>
       <c r="L48" s="6" t="inlineStr"/>
@@ -28023,20 +28023,20 @@
     <row r="49">
       <c r="H49" s="6" t="inlineStr">
         <is>
-          <t>GIS</t>
+          <t>EWBC</t>
         </is>
       </c>
       <c r="I49" s="61" t="n">
-        <v>0.004215229999999999</v>
+        <v>0.00422368</v>
       </c>
       <c r="J49" s="6" t="inlineStr">
         <is>
-          <t>GENERAL MILLS INC</t>
+          <t>EAST WEST BANCORP</t>
         </is>
       </c>
       <c r="K49" s="6" t="inlineStr">
         <is>
-          <t>Consumer Staples</t>
+          <t>Financials</t>
         </is>
       </c>
       <c r="L49" s="6" t="inlineStr"/>
@@ -28052,7 +28052,7 @@
         </is>
       </c>
       <c r="I50" s="61" t="n">
-        <v>0.00409258</v>
+        <v>0.00418986</v>
       </c>
       <c r="J50" s="6" t="inlineStr">
         <is>
@@ -28077,7 +28077,7 @@
         </is>
       </c>
       <c r="I51" s="61" t="n">
-        <v>0.00254985</v>
+        <v>0.00254429</v>
       </c>
       <c r="J51" s="6" t="inlineStr">
         <is>
@@ -28098,20 +28098,20 @@
     <row r="52">
       <c r="H52" s="6" t="inlineStr">
         <is>
-          <t>AFG</t>
+          <t>BAH</t>
         </is>
       </c>
       <c r="I52" s="61" t="n">
-        <v>0.00248949</v>
+        <v>0.00250666</v>
       </c>
       <c r="J52" s="6" t="inlineStr">
         <is>
-          <t>AMERICAN FINANCIAL GROUP</t>
+          <t>BOOZ ALLEN HAMILTON HOLDING CLASS</t>
         </is>
       </c>
       <c r="K52" s="6" t="inlineStr">
         <is>
-          <t>Financials</t>
+          <t>Industrials</t>
         </is>
       </c>
       <c r="L52" s="6" t="inlineStr"/>
@@ -28123,15 +28123,15 @@
     <row r="53">
       <c r="H53" s="6" t="inlineStr">
         <is>
-          <t>FNF</t>
+          <t>AFG</t>
         </is>
       </c>
       <c r="I53" s="61" t="n">
-        <v>0.00242606</v>
+        <v>0.00249208</v>
       </c>
       <c r="J53" s="6" t="inlineStr">
         <is>
-          <t>FIDELITY NATIONAL FINANCIAL INC</t>
+          <t>AMERICAN FINANCIAL GROUP</t>
         </is>
       </c>
       <c r="K53" s="6" t="inlineStr">
@@ -28148,20 +28148,20 @@
     <row r="54">
       <c r="H54" s="6" t="inlineStr">
         <is>
-          <t>BAH</t>
+          <t>FNF</t>
         </is>
       </c>
       <c r="I54" s="61" t="n">
-        <v>0.00239541</v>
+        <v>0.00243035</v>
       </c>
       <c r="J54" s="6" t="inlineStr">
         <is>
-          <t>BOOZ ALLEN HAMILTON HOLDING CLASS</t>
+          <t>FIDELITY NATIONAL FINANCIAL INC</t>
         </is>
       </c>
       <c r="K54" s="6" t="inlineStr">
         <is>
-          <t>Industrials</t>
+          <t>Financials</t>
         </is>
       </c>
       <c r="L54" s="6" t="inlineStr"/>
@@ -28177,7 +28177,7 @@
         </is>
       </c>
       <c r="I55" s="61" t="n">
-        <v>0.00207336</v>
+        <v>0.00204457</v>
       </c>
       <c r="J55" s="6" t="inlineStr">
         <is>
@@ -28202,7 +28202,7 @@
         </is>
       </c>
       <c r="I56" s="61" t="n">
-        <v>0.00201913</v>
+        <v>0.00201539</v>
       </c>
       <c r="J56" s="6" t="inlineStr">
         <is>
@@ -28227,7 +28227,7 @@
         </is>
       </c>
       <c r="I57" s="61" t="n">
-        <v>0.00184327</v>
+        <v>0.00184531</v>
       </c>
       <c r="J57" s="6" t="inlineStr">
         <is>
@@ -28248,20 +28248,20 @@
     <row r="58">
       <c r="H58" s="6" t="inlineStr">
         <is>
-          <t>M</t>
+          <t>ERIE</t>
         </is>
       </c>
       <c r="I58" s="61" t="n">
-        <v>0.00153684</v>
+        <v>0.0015907</v>
       </c>
       <c r="J58" s="6" t="inlineStr">
         <is>
-          <t>MACYS</t>
+          <t>ERIE INDEMNITY CLASS A</t>
         </is>
       </c>
       <c r="K58" s="6" t="inlineStr">
         <is>
-          <t>Consumer Discretionary</t>
+          <t>Financials</t>
         </is>
       </c>
       <c r="L58" s="6" t="inlineStr"/>
@@ -28273,20 +28273,20 @@
     <row r="59">
       <c r="H59" s="6" t="inlineStr">
         <is>
-          <t>ERIE</t>
+          <t>M</t>
         </is>
       </c>
       <c r="I59" s="61" t="n">
-        <v>0.0015324</v>
+        <v>0.00149303</v>
       </c>
       <c r="J59" s="6" t="inlineStr">
         <is>
-          <t>ERIE INDEMNITY CLASS A</t>
+          <t>MACYS</t>
         </is>
       </c>
       <c r="K59" s="6" t="inlineStr">
         <is>
-          <t>Financials</t>
+          <t>Consumer Discretionary</t>
         </is>
       </c>
       <c r="L59" s="6" t="inlineStr"/>
@@ -28302,7 +28302,7 @@
         </is>
       </c>
       <c r="I60" s="61" t="n">
-        <v>0.00136721</v>
+        <v>0.00139711</v>
       </c>
       <c r="J60" s="6" t="inlineStr">
         <is>
@@ -28327,7 +28327,7 @@
         </is>
       </c>
       <c r="I61" s="61" t="n">
-        <v>0.00133222</v>
+        <v>0.00130646</v>
       </c>
       <c r="J61" s="6" t="inlineStr">
         <is>
@@ -28352,7 +28352,7 @@
         </is>
       </c>
       <c r="I62" s="61" t="n">
-        <v>0.00130236</v>
+        <v>0.00127445</v>
       </c>
       <c r="J62" s="6" t="inlineStr">
         <is>
@@ -28377,7 +28377,7 @@
         </is>
       </c>
       <c r="I63" s="61" t="n">
-        <v>0.00123259</v>
+        <v>0.00123254</v>
       </c>
       <c r="J63" s="6" t="inlineStr">
         <is>
@@ -28402,7 +28402,7 @@
         </is>
       </c>
       <c r="I64" s="61" t="n">
-        <v>0.00116678</v>
+        <v>0.00117134</v>
       </c>
       <c r="J64" s="6" t="inlineStr">
         <is>
@@ -28423,20 +28423,20 @@
     <row r="65">
       <c r="H65" s="6" t="inlineStr">
         <is>
-          <t>MC</t>
+          <t>RHI</t>
         </is>
       </c>
       <c r="I65" s="61" t="n">
-        <v>0.00104832</v>
+        <v>0.00103385</v>
       </c>
       <c r="J65" s="6" t="inlineStr">
         <is>
-          <t>MOELIS CLASS A</t>
+          <t>ROBERT HALF INC</t>
         </is>
       </c>
       <c r="K65" s="6" t="inlineStr">
         <is>
-          <t>Financials</t>
+          <t>Industrials</t>
         </is>
       </c>
       <c r="L65" s="6" t="inlineStr"/>
@@ -28448,20 +28448,20 @@
     <row r="66">
       <c r="H66" s="6" t="inlineStr">
         <is>
-          <t>RHI</t>
+          <t>MC</t>
         </is>
       </c>
       <c r="I66" s="61" t="n">
-        <v>0.00101585</v>
+        <v>0.00102001</v>
       </c>
       <c r="J66" s="6" t="inlineStr">
         <is>
-          <t>ROBERT HALF INC</t>
+          <t>MOELIS CLASS A</t>
         </is>
       </c>
       <c r="K66" s="6" t="inlineStr">
         <is>
-          <t>Industrials</t>
+          <t>Financials</t>
         </is>
       </c>
       <c r="L66" s="6" t="inlineStr"/>
@@ -28477,7 +28477,7 @@
         </is>
       </c>
       <c r="I67" s="61" t="n">
-        <v>0.0009781900000000001</v>
+        <v>0.0009821999999999999</v>
       </c>
       <c r="J67" s="6" t="inlineStr">
         <is>
@@ -28498,20 +28498,20 @@
     <row r="68">
       <c r="H68" s="6" t="inlineStr">
         <is>
-          <t>CWEN</t>
+          <t>KFY</t>
         </is>
       </c>
       <c r="I68" s="61" t="n">
-        <v>0.0009397300000000001</v>
+        <v>0.00092817</v>
       </c>
       <c r="J68" s="6" t="inlineStr">
         <is>
-          <t>CLEARWAY ENERGY INC CLASS C</t>
+          <t>KORN FERRY</t>
         </is>
       </c>
       <c r="K68" s="6" t="inlineStr">
         <is>
-          <t>Utilities</t>
+          <t>Industrials</t>
         </is>
       </c>
       <c r="L68" s="6" t="inlineStr"/>
@@ -28523,20 +28523,20 @@
     <row r="69">
       <c r="H69" s="6" t="inlineStr">
         <is>
-          <t>KFY</t>
+          <t>CWEN</t>
         </is>
       </c>
       <c r="I69" s="61" t="n">
-        <v>0.00092419</v>
+        <v>0.00091182</v>
       </c>
       <c r="J69" s="6" t="inlineStr">
         <is>
-          <t>KORN FERRY</t>
+          <t>CLEARWAY ENERGY INC CLASS C</t>
         </is>
       </c>
       <c r="K69" s="6" t="inlineStr">
         <is>
-          <t>Industrials</t>
+          <t>Utilities</t>
         </is>
       </c>
       <c r="L69" s="6" t="inlineStr"/>
@@ -28552,7 +28552,7 @@
         </is>
       </c>
       <c r="I70" s="61" t="n">
-        <v>0.00089745</v>
+        <v>0.00088725</v>
       </c>
       <c r="J70" s="6" t="inlineStr">
         <is>
@@ -28577,7 +28577,7 @@
         </is>
       </c>
       <c r="I71" s="61" t="n">
-        <v>0.0008917500000000001</v>
+        <v>0.00088724</v>
       </c>
       <c r="J71" s="6" t="inlineStr">
         <is>
@@ -28602,7 +28602,7 @@
         </is>
       </c>
       <c r="I72" s="61" t="n">
-        <v>0.0007404</v>
+        <v>0.00074929</v>
       </c>
       <c r="J72" s="6" t="inlineStr">
         <is>
@@ -28623,7 +28623,7 @@
         </is>
       </c>
       <c r="I73" s="61" t="n">
-        <v>0.0006083999999999999</v>
+        <v>0.0006091499999999999</v>
       </c>
       <c r="J73" s="6" t="inlineStr">
         <is>
@@ -28648,7 +28648,7 @@
         </is>
       </c>
       <c r="I74" s="61" t="n">
-        <v>0.00055446</v>
+        <v>0.0005514000000000001</v>
       </c>
       <c r="J74" s="6" t="inlineStr">
         <is>
@@ -28669,20 +28669,20 @@
     <row r="75">
       <c r="H75" s="6" t="inlineStr">
         <is>
-          <t>OFG</t>
+          <t>MZTI</t>
         </is>
       </c>
       <c r="I75" s="61" t="n">
-        <v>0.00050899</v>
+        <v>0.00050382</v>
       </c>
       <c r="J75" s="6" t="inlineStr">
         <is>
-          <t>OFG BANCORP</t>
+          <t>MARZETTI</t>
         </is>
       </c>
       <c r="K75" s="6" t="inlineStr">
         <is>
-          <t>Financials</t>
+          <t>Consumer Staples</t>
         </is>
       </c>
       <c r="L75" s="6" t="inlineStr"/>
@@ -28694,15 +28694,15 @@
     <row r="76">
       <c r="H76" s="6" t="inlineStr">
         <is>
-          <t>MZTI</t>
+          <t>IPAR</t>
         </is>
       </c>
       <c r="I76" s="61" t="n">
-        <v>0.00050296</v>
+        <v>0.00050049</v>
       </c>
       <c r="J76" s="6" t="inlineStr">
         <is>
-          <t>MARZETTI</t>
+          <t>INTERPARFUMS INC</t>
         </is>
       </c>
       <c r="K76" s="6" t="inlineStr">
@@ -28719,20 +28719,20 @@
     <row r="77">
       <c r="H77" s="6" t="inlineStr">
         <is>
-          <t>IPAR</t>
+          <t>OFG</t>
         </is>
       </c>
       <c r="I77" s="61" t="n">
-        <v>0.0004987699999999999</v>
+        <v>0.00049829</v>
       </c>
       <c r="J77" s="6" t="inlineStr">
         <is>
-          <t>INTERPARFUMS INC</t>
+          <t>OFG BANCORP</t>
         </is>
       </c>
       <c r="K77" s="6" t="inlineStr">
         <is>
-          <t>Consumer Staples</t>
+          <t>Financials</t>
         </is>
       </c>
       <c r="L77" s="6" t="inlineStr"/>
@@ -28748,7 +28748,7 @@
         </is>
       </c>
       <c r="I78" s="61" t="n">
-        <v>0.00048786</v>
+        <v>0.00048302</v>
       </c>
       <c r="J78" s="6" t="inlineStr">
         <is>
@@ -28773,7 +28773,7 @@
         </is>
       </c>
       <c r="I79" s="61" t="n">
-        <v>0.00047741</v>
+        <v>0.00047175</v>
       </c>
       <c r="J79" s="6" t="inlineStr">
         <is>
@@ -28798,7 +28798,7 @@
         </is>
       </c>
       <c r="I80" s="61" t="n">
-        <v>0.00045943</v>
+        <v>0.00045395</v>
       </c>
       <c r="J80" s="6" t="inlineStr">
         <is>
@@ -28823,7 +28823,7 @@
         </is>
       </c>
       <c r="I81" s="61" t="n">
-        <v>0.00045034</v>
+        <v>0.00044446</v>
       </c>
       <c r="J81" s="6" t="inlineStr">
         <is>
@@ -28848,7 +28848,7 @@
         </is>
       </c>
       <c r="I82" s="61" t="n">
-        <v>0.00044021</v>
+        <v>0.0004343700000000001</v>
       </c>
       <c r="J82" s="6" t="inlineStr">
         <is>
@@ -28873,7 +28873,7 @@
         </is>
       </c>
       <c r="I83" s="61" t="n">
-        <v>0.00042712</v>
+        <v>0.00042091</v>
       </c>
       <c r="J83" s="6" t="inlineStr">
         <is>
@@ -28894,20 +28894,20 @@
     <row r="84">
       <c r="H84" s="6" t="inlineStr">
         <is>
-          <t>NBHC</t>
+          <t>NSP</t>
         </is>
       </c>
       <c r="I84" s="61" t="n">
-        <v>0.00039517</v>
+        <v>0.00041073</v>
       </c>
       <c r="J84" s="6" t="inlineStr">
         <is>
-          <t>NATIONAL BANK HOLDINGS CORP CLASS</t>
+          <t>INSPERITY</t>
         </is>
       </c>
       <c r="K84" s="6" t="inlineStr">
         <is>
-          <t>Financials</t>
+          <t>Industrials</t>
         </is>
       </c>
       <c r="L84" s="6" t="inlineStr"/>
@@ -28919,20 +28919,20 @@
     <row r="85">
       <c r="H85" s="6" t="inlineStr">
         <is>
-          <t>NSP</t>
+          <t>NBHC</t>
         </is>
       </c>
       <c r="I85" s="61" t="n">
-        <v>0.0003921</v>
+        <v>0.00039224</v>
       </c>
       <c r="J85" s="6" t="inlineStr">
         <is>
-          <t>INSPERITY</t>
+          <t>NATIONAL BANK HOLDINGS CORP CLASS</t>
         </is>
       </c>
       <c r="K85" s="6" t="inlineStr">
         <is>
-          <t>Industrials</t>
+          <t>Financials</t>
         </is>
       </c>
       <c r="L85" s="6" t="inlineStr"/>
@@ -28948,7 +28948,7 @@
         </is>
       </c>
       <c r="I86" s="61" t="n">
-        <v>0.00037257</v>
+        <v>0.00036766</v>
       </c>
       <c r="J86" s="6" t="inlineStr">
         <is>
@@ -28973,7 +28973,7 @@
         </is>
       </c>
       <c r="I87" s="61" t="n">
-        <v>0.00035967</v>
+        <v>0.00035277</v>
       </c>
       <c r="J87" s="6" t="inlineStr">
         <is>
@@ -28998,7 +28998,7 @@
         </is>
       </c>
       <c r="I88" s="61" t="n">
-        <v>0.0003416</v>
+        <v>0.00033595</v>
       </c>
       <c r="J88" s="6" t="inlineStr">
         <is>
@@ -29023,7 +29023,7 @@
         </is>
       </c>
       <c r="I89" s="61" t="n">
-        <v>0.00031038</v>
+        <v>0.00031367</v>
       </c>
       <c r="J89" s="6" t="inlineStr">
         <is>
@@ -29044,20 +29044,20 @@
     <row r="90">
       <c r="H90" s="6" t="inlineStr">
         <is>
-          <t>PFBC</t>
+          <t>WEN</t>
         </is>
       </c>
       <c r="I90" s="61" t="n">
-        <v>0.00027592</v>
+        <v>0.00027305</v>
       </c>
       <c r="J90" s="6" t="inlineStr">
         <is>
-          <t>PREFERRED BANK</t>
+          <t>WENDYS</t>
         </is>
       </c>
       <c r="K90" s="6" t="inlineStr">
         <is>
-          <t>Financials</t>
+          <t>Consumer Discretionary</t>
         </is>
       </c>
       <c r="L90" s="6" t="inlineStr"/>
@@ -29069,20 +29069,20 @@
     <row r="91">
       <c r="H91" s="6" t="inlineStr">
         <is>
-          <t>WEN</t>
+          <t>PFBC</t>
         </is>
       </c>
       <c r="I91" s="61" t="n">
-        <v>0.00027261</v>
+        <v>0.00027137</v>
       </c>
       <c r="J91" s="6" t="inlineStr">
         <is>
-          <t>WENDYS</t>
+          <t>PREFERRED BANK</t>
         </is>
       </c>
       <c r="K91" s="6" t="inlineStr">
         <is>
-          <t>Consumer Discretionary</t>
+          <t>Financials</t>
         </is>
       </c>
       <c r="L91" s="6" t="inlineStr"/>
@@ -29098,7 +29098,7 @@
         </is>
       </c>
       <c r="I92" s="61" t="n">
-        <v>0.0002511</v>
+        <v>0.00024914</v>
       </c>
       <c r="J92" s="6" t="inlineStr">
         <is>
@@ -29123,7 +29123,7 @@
         </is>
       </c>
       <c r="I93" s="61" t="n">
-        <v>0.00023498</v>
+        <v>0.00022973</v>
       </c>
       <c r="J93" s="6" t="inlineStr">
         <is>
@@ -29148,7 +29148,7 @@
         </is>
       </c>
       <c r="I94" s="61" t="n">
-        <v>0.00023121</v>
+        <v>0.00022626</v>
       </c>
       <c r="J94" s="6" t="inlineStr">
         <is>
@@ -29173,7 +29173,7 @@
         </is>
       </c>
       <c r="I95" s="61" t="n">
-        <v>0.00020949</v>
+        <v>0.00020621</v>
       </c>
       <c r="J95" s="6" t="inlineStr">
         <is>
@@ -29198,7 +29198,7 @@
         </is>
       </c>
       <c r="I96" s="61" t="n">
-        <v>0.00019564</v>
+        <v>0.00019245</v>
       </c>
       <c r="J96" s="6" t="inlineStr">
         <is>
@@ -29223,7 +29223,7 @@
         </is>
       </c>
       <c r="I97" s="61" t="n">
-        <v>0.0001953</v>
+        <v>0.00019175</v>
       </c>
       <c r="J97" s="6" t="inlineStr">
         <is>
@@ -29248,7 +29248,7 @@
         </is>
       </c>
       <c r="I98" s="61" t="n">
-        <v>0.00018058</v>
+        <v>0.00017011</v>
       </c>
       <c r="J98" s="6" t="inlineStr">
         <is>
@@ -29273,7 +29273,7 @@
         </is>
       </c>
       <c r="I99" s="61" t="n">
-        <v>0.0001657</v>
+        <v>0.00016399</v>
       </c>
       <c r="J99" s="6" t="inlineStr">
         <is>
@@ -29298,7 +29298,7 @@
         </is>
       </c>
       <c r="I100" s="61" t="n">
-        <v>0.00013253</v>
+        <v>0.00013187</v>
       </c>
       <c r="J100" s="6" t="inlineStr">
         <is>
@@ -29319,7 +29319,7 @@
         </is>
       </c>
       <c r="I101" s="61" t="n">
-        <v>0.00012318</v>
+        <v>0.00012055</v>
       </c>
       <c r="J101" s="6" t="inlineStr">
         <is>
@@ -29340,20 +29340,20 @@
     <row r="102">
       <c r="H102" s="6" t="inlineStr">
         <is>
-          <t>AMSF</t>
+          <t>ETD</t>
         </is>
       </c>
       <c r="I102" s="61" t="n">
-        <v>0.00010126</v>
+        <v>9.593000000000001e-05</v>
       </c>
       <c r="J102" s="6" t="inlineStr">
         <is>
-          <t>AMERISAFE INC</t>
+          <t>ETHAN ALLEN INTERIORS</t>
         </is>
       </c>
       <c r="K102" s="6" t="inlineStr">
         <is>
-          <t>Financials</t>
+          <t>Consumer Discretionary</t>
         </is>
       </c>
       <c r="L102" s="6" t="inlineStr"/>
@@ -29365,15 +29365,15 @@
     <row r="103">
       <c r="H103" s="6" t="inlineStr">
         <is>
-          <t>ETD</t>
+          <t>OXM</t>
         </is>
       </c>
       <c r="I103" s="61" t="n">
-        <v>9.547000000000001e-05</v>
+        <v>9.221e-05</v>
       </c>
       <c r="J103" s="6" t="inlineStr">
         <is>
-          <t>ETHAN ALLEN INTERIORS</t>
+          <t>OXFORD INDUSTRIES INC</t>
         </is>
       </c>
       <c r="K103" s="6" t="inlineStr">
@@ -29390,20 +29390,20 @@
     <row r="104">
       <c r="H104" s="6" t="inlineStr">
         <is>
-          <t>OXM</t>
+          <t>AMSF</t>
         </is>
       </c>
       <c r="I104" s="61" t="n">
-        <v>9.400000000000001e-05</v>
+        <v>9.132e-05</v>
       </c>
       <c r="J104" s="6" t="inlineStr">
         <is>
-          <t>OXFORD INDUSTRIES INC</t>
+          <t>AMERISAFE INC</t>
         </is>
       </c>
       <c r="K104" s="6" t="inlineStr">
         <is>
-          <t>Consumer Discretionary</t>
+          <t>Financials</t>
         </is>
       </c>
       <c r="L104" s="6" t="inlineStr"/>

</xml_diff>